<commit_message>
feat: add Solana DeFi positions via Jupiter page scrape
- scrape_sol_defi_positions() uses Playwright to open jup.ag/portfolio
  and parse Loopscale + Kamino positions from page text
- _parse_jupiter_text() regex parser handles mixed-case token names,
  health %, net worth, and Kamino claimable rewards
- Grand total combines Rabby EVM reported total + Jupiter sol net worth
- Health shown as "X% to liq" (not raw ratio) for Loopscale positions
- GitHub Actions workflow installs playwright chromium before refresh
- launch.json updated to serve from docs/ (GitHub Pages source)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O106"/>
+  <dimension ref="A1:O120"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -7644,6 +7644,948 @@
       <c r="O106" s="15" t="inlineStr">
         <is>
           <t>Rabby API (api.rabby.io/v1/user/complex_protocol_list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:29:17</t>
+        </is>
+      </c>
+      <c r="B107" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C107" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D107" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E107" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F107" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G107" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H107" s="16" t="n">
+        <v>1.0481</v>
+      </c>
+      <c r="I107" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J107" s="17" t="n">
+        <v>140902.2704240698</v>
+      </c>
+      <c r="K107" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,017.2084</t>
+        </is>
+      </c>
+      <c r="L107" s="17" t="n">
+        <v>120988.1643189722</v>
+      </c>
+      <c r="M107" s="17">
+        <f>J107-L107</f>
+        <v/>
+      </c>
+      <c r="N107" s="18">
+        <f>IF(J107=0,"",L107/J107)</f>
+        <v/>
+      </c>
+      <c r="O107" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:29:17</t>
+        </is>
+      </c>
+      <c r="B108" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C108" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D108" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E108" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F108" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G108" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H108" s="16" t="n">
+        <v>1.0451</v>
+      </c>
+      <c r="I108" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J108" s="17" t="n">
+        <v>328667.8726651539</v>
+      </c>
+      <c r="K108" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,366.2953</t>
+        </is>
+      </c>
+      <c r="L108" s="17" t="n">
+        <v>306390.58393976</v>
+      </c>
+      <c r="M108" s="17">
+        <f>J108-L108</f>
+        <v/>
+      </c>
+      <c r="N108" s="18">
+        <f>IF(J108=0,"",L108/J108)</f>
+        <v/>
+      </c>
+      <c r="O108" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:29:17</t>
+        </is>
+      </c>
+      <c r="B109" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C109" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D109" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E109" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F109" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G109" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H109" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I109" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J109" s="17" t="n">
+        <v>385882.1286604155</v>
+      </c>
+      <c r="K109" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,577.8899</t>
+        </is>
+      </c>
+      <c r="L109" s="17" t="n">
+        <v>349605.6043233544</v>
+      </c>
+      <c r="M109" s="17">
+        <f>J109-L109</f>
+        <v/>
+      </c>
+      <c r="N109" s="18">
+        <f>IF(J109=0,"",L109/J109)</f>
+        <v/>
+      </c>
+      <c r="O109" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:29:17</t>
+        </is>
+      </c>
+      <c r="B110" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C110" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D110" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E110" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F110" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G110" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H110" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I110" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7815</t>
+        </is>
+      </c>
+      <c r="J110" s="17" t="n">
+        <v>77796.16806942438</v>
+      </c>
+      <c r="K110" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,020.1544; USDC 0.0775</t>
+        </is>
+      </c>
+      <c r="L110" s="17" t="n">
+        <v>68003.90714193678</v>
+      </c>
+      <c r="M110" s="17">
+        <f>J110-L110</f>
+        <v/>
+      </c>
+      <c r="N110" s="18">
+        <f>IF(J110=0,"",L110/J110)</f>
+        <v/>
+      </c>
+      <c r="O110" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:29:17</t>
+        </is>
+      </c>
+      <c r="B111" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C111" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D111" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E111" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F111" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G111" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H111" s="16" t="n">
+        <v>1.1282</v>
+      </c>
+      <c r="I111" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J111" s="17" t="n">
+        <v>196966.0787510267</v>
+      </c>
+      <c r="K111" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,217.1999</t>
+        </is>
+      </c>
+      <c r="L111" s="17" t="n">
+        <v>150217.1998588595</v>
+      </c>
+      <c r="M111" s="17">
+        <f>J111-L111</f>
+        <v/>
+      </c>
+      <c r="N111" s="18">
+        <f>IF(J111=0,"",L111/J111)</f>
+        <v/>
+      </c>
+      <c r="O111" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:29:17</t>
+        </is>
+      </c>
+      <c r="B112" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C112" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D112" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E112" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F112" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G112" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H112" s="16" t="n">
+        <v>1.0528</v>
+      </c>
+      <c r="I112" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J112" s="17" t="n">
+        <v>186095.5217336493</v>
+      </c>
+      <c r="K112" s="15" t="inlineStr">
+        <is>
+          <t>USDC 161,824.1564</t>
+        </is>
+      </c>
+      <c r="L112" s="17" t="n">
+        <v>161824.1563839606</v>
+      </c>
+      <c r="M112" s="17">
+        <f>J112-L112</f>
+        <v/>
+      </c>
+      <c r="N112" s="18">
+        <f>IF(J112=0,"",L112/J112)</f>
+        <v/>
+      </c>
+      <c r="O112" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:29:17</t>
+        </is>
+      </c>
+      <c r="B113" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C113" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D113" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E113" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F113" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G113" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H113" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I113" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J113" s="17" t="n">
+        <v>327483.1065447227</v>
+      </c>
+      <c r="K113" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L113" s="17" t="n">
+        <v>280184.6947195007</v>
+      </c>
+      <c r="M113" s="17">
+        <f>J113-L113</f>
+        <v/>
+      </c>
+      <c r="N113" s="18">
+        <f>IF(J113=0,"",L113/J113)</f>
+        <v/>
+      </c>
+      <c r="O113" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:29:17</t>
+        </is>
+      </c>
+      <c r="B114" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C114" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D114" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E114" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F114" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G114" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H114" s="16" t="n">
+        <v>1.1297</v>
+      </c>
+      <c r="I114" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J114" s="17" t="n">
+        <v>159924.3452</v>
+      </c>
+      <c r="K114" s="15" t="inlineStr">
+        <is>
+          <t>USDC 119,558.7697</t>
+        </is>
+      </c>
+      <c r="L114" s="17" t="n">
+        <v>119558.7696910311</v>
+      </c>
+      <c r="M114" s="17">
+        <f>J114-L114</f>
+        <v/>
+      </c>
+      <c r="N114" s="18">
+        <f>IF(J114=0,"",L114/J114)</f>
+        <v/>
+      </c>
+      <c r="O114" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:29:17</t>
+        </is>
+      </c>
+      <c r="B115" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C115" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D115" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E115" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F115" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G115" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H115" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I115" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J115" s="17" t="n">
+        <v>160092.0534906599</v>
+      </c>
+      <c r="K115" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,509.0058</t>
+        </is>
+      </c>
+      <c r="L115" s="17" t="n">
+        <v>138481.3039849279</v>
+      </c>
+      <c r="M115" s="17">
+        <f>J115-L115</f>
+        <v/>
+      </c>
+      <c r="N115" s="18">
+        <f>IF(J115=0,"",L115/J115)</f>
+        <v/>
+      </c>
+      <c r="O115" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:29:17</t>
+        </is>
+      </c>
+      <c r="B116" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C116" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D116" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E116" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F116" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeef003c</t>
+        </is>
+      </c>
+      <c r="G116" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H116" s="16" t="inlineStr"/>
+      <c r="I116" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,800.0745</t>
+        </is>
+      </c>
+      <c r="J116" s="17" t="n">
+        <v>50787.88245012768</v>
+      </c>
+      <c r="K116" s="15" t="inlineStr"/>
+      <c r="L116" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M116" s="17">
+        <f>J116-L116</f>
+        <v/>
+      </c>
+      <c r="N116" s="18">
+        <f>IF(J116=0,"",L116/J116)</f>
+        <v/>
+      </c>
+      <c r="O116" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:29:17</t>
+        </is>
+      </c>
+      <c r="B117" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C117" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D117" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E117" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F117" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G117" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H117" s="16" t="inlineStr"/>
+      <c r="I117" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J117" s="17" t="n">
+        <v>95911.90540587669</v>
+      </c>
+      <c r="K117" s="15" t="inlineStr"/>
+      <c r="L117" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M117" s="17">
+        <f>J117-L117</f>
+        <v/>
+      </c>
+      <c r="N117" s="18">
+        <f>IF(J117=0,"",L117/J117)</f>
+        <v/>
+      </c>
+      <c r="O117" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:29:17</t>
+        </is>
+      </c>
+      <c r="B118" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C118" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D118" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E118" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F118" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G118" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H118" s="16" t="inlineStr"/>
+      <c r="I118" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J118" s="17" t="n">
+        <v>34339.01569920389</v>
+      </c>
+      <c r="K118" s="15" t="inlineStr"/>
+      <c r="L118" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M118" s="17">
+        <f>J118-L118</f>
+        <v/>
+      </c>
+      <c r="N118" s="18">
+        <f>IF(J118=0,"",L118/J118)</f>
+        <v/>
+      </c>
+      <c r="O118" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:29:17</t>
+        </is>
+      </c>
+      <c r="B119" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C119" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D119" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E119" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F119" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G119" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H119" s="16" t="n">
+        <v>1.0419</v>
+      </c>
+      <c r="I119" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J119" s="17" t="n">
+        <v>269662.1813443768</v>
+      </c>
+      <c r="K119" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,002.3970</t>
+        </is>
+      </c>
+      <c r="L119" s="17" t="n">
+        <v>232946.4764227205</v>
+      </c>
+      <c r="M119" s="17">
+        <f>J119-L119</f>
+        <v/>
+      </c>
+      <c r="N119" s="18">
+        <f>IF(J119=0,"",L119/J119)</f>
+        <v/>
+      </c>
+      <c r="O119" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:29:17</t>
+        </is>
+      </c>
+      <c r="B120" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C120" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D120" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E120" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F120" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G120" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H120" s="16" t="inlineStr"/>
+      <c r="I120" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,500.3087</t>
+        </is>
+      </c>
+      <c r="J120" s="17" t="n">
+        <v>15496.58862373629</v>
+      </c>
+      <c r="K120" s="15" t="inlineStr"/>
+      <c r="L120" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M120" s="17">
+        <f>J120-L120</f>
+        <v/>
+      </c>
+      <c r="N120" s="18">
+        <f>IF(J120=0,"",L120/J120)</f>
+        <v/>
+      </c>
+      <c r="O120" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
         </is>
       </c>
     </row>
@@ -7672,7 +8614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -8005,6 +8947,41 @@
       <c r="I9" s="15" t="inlineStr">
         <is>
           <t>Rabby API (api.rabby.io/v1/user/complex_protocol_list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:29:17</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="n">
+        <v>553069.6462611336</v>
+      </c>
+      <c r="D10" s="17" t="n">
+        <v>501806.2582774202</v>
+      </c>
+      <c r="E10" s="17" t="n">
+        <v>2430007.119062444</v>
+      </c>
+      <c r="F10" s="17" t="n">
+        <v>1928200.860785024</v>
+      </c>
+      <c r="G10" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="H10" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I10" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: final day-0 snapshot + filter AICC scam token
- Saved day0.json as permanent baseline reference
- Blocked AICC (0x66a3c2fa...) airdrop scam token from wallet display
- Total equity: $654,814 (EVM $553k + Solana $101k)
- 15 EVM positions + 2 Loopscale + 1 Kamino

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O120"/>
+  <dimension ref="A1:O149"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -8584,6 +8584,1953 @@
         <v/>
       </c>
       <c r="O120" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:41:20</t>
+        </is>
+      </c>
+      <c r="B121" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C121" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D121" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E121" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F121" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G121" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H121" s="16" t="n">
+        <v>1.0479</v>
+      </c>
+      <c r="I121" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J121" s="17" t="n">
+        <v>140874.4736785287</v>
+      </c>
+      <c r="K121" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,017.2084</t>
+        </is>
+      </c>
+      <c r="L121" s="17" t="n">
+        <v>120988.1643189722</v>
+      </c>
+      <c r="M121" s="17">
+        <f>J121-L121</f>
+        <v/>
+      </c>
+      <c r="N121" s="18">
+        <f>IF(J121=0,"",L121/J121)</f>
+        <v/>
+      </c>
+      <c r="O121" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:41:20</t>
+        </is>
+      </c>
+      <c r="B122" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C122" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D122" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E122" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F122" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G122" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H122" s="16" t="n">
+        <v>1.0451</v>
+      </c>
+      <c r="I122" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J122" s="17" t="n">
+        <v>328667.8726651539</v>
+      </c>
+      <c r="K122" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,366.2953</t>
+        </is>
+      </c>
+      <c r="L122" s="17" t="n">
+        <v>306390.5826091492</v>
+      </c>
+      <c r="M122" s="17">
+        <f>J122-L122</f>
+        <v/>
+      </c>
+      <c r="N122" s="18">
+        <f>IF(J122=0,"",L122/J122)</f>
+        <v/>
+      </c>
+      <c r="O122" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:41:20</t>
+        </is>
+      </c>
+      <c r="B123" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C123" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D123" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E123" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F123" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G123" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H123" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I123" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J123" s="17" t="n">
+        <v>385882.1286604155</v>
+      </c>
+      <c r="K123" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,577.8899</t>
+        </is>
+      </c>
+      <c r="L123" s="17" t="n">
+        <v>349605.6028050669</v>
+      </c>
+      <c r="M123" s="17">
+        <f>J123-L123</f>
+        <v/>
+      </c>
+      <c r="N123" s="18">
+        <f>IF(J123=0,"",L123/J123)</f>
+        <v/>
+      </c>
+      <c r="O123" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:41:20</t>
+        </is>
+      </c>
+      <c r="B124" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C124" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D124" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E124" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F124" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G124" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H124" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I124" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7815</t>
+        </is>
+      </c>
+      <c r="J124" s="17" t="n">
+        <v>77796.19687370764</v>
+      </c>
+      <c r="K124" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,020.1544; USDC 0.0775</t>
+        </is>
+      </c>
+      <c r="L124" s="17" t="n">
+        <v>68001.86654505957</v>
+      </c>
+      <c r="M124" s="17">
+        <f>J124-L124</f>
+        <v/>
+      </c>
+      <c r="N124" s="18">
+        <f>IF(J124=0,"",L124/J124)</f>
+        <v/>
+      </c>
+      <c r="O124" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:41:20</t>
+        </is>
+      </c>
+      <c r="B125" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C125" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D125" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E125" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F125" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G125" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H125" s="16" t="n">
+        <v>1.1282</v>
+      </c>
+      <c r="I125" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J125" s="17" t="n">
+        <v>197021.5867003927</v>
+      </c>
+      <c r="K125" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,217.1999</t>
+        </is>
+      </c>
+      <c r="L125" s="17" t="n">
+        <v>150232.2230811676</v>
+      </c>
+      <c r="M125" s="17">
+        <f>J125-L125</f>
+        <v/>
+      </c>
+      <c r="N125" s="18">
+        <f>IF(J125=0,"",L125/J125)</f>
+        <v/>
+      </c>
+      <c r="O125" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:41:20</t>
+        </is>
+      </c>
+      <c r="B126" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C126" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D126" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E126" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F126" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G126" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H126" s="16" t="n">
+        <v>1.0528</v>
+      </c>
+      <c r="I126" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J126" s="17" t="n">
+        <v>186096.1049750841</v>
+      </c>
+      <c r="K126" s="15" t="inlineStr">
+        <is>
+          <t>USDC 161,824.1564</t>
+        </is>
+      </c>
+      <c r="L126" s="17" t="n">
+        <v>161840.3404180024</v>
+      </c>
+      <c r="M126" s="17">
+        <f>J126-L126</f>
+        <v/>
+      </c>
+      <c r="N126" s="18">
+        <f>IF(J126=0,"",L126/J126)</f>
+        <v/>
+      </c>
+      <c r="O126" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:41:20</t>
+        </is>
+      </c>
+      <c r="B127" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C127" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D127" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E127" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F127" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G127" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H127" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I127" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J127" s="17" t="n">
+        <v>327483.0881365995</v>
+      </c>
+      <c r="K127" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L127" s="17" t="n">
+        <v>280184.6617515259</v>
+      </c>
+      <c r="M127" s="17">
+        <f>J127-L127</f>
+        <v/>
+      </c>
+      <c r="N127" s="18">
+        <f>IF(J127=0,"",L127/J127)</f>
+        <v/>
+      </c>
+      <c r="O127" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:41:20</t>
+        </is>
+      </c>
+      <c r="B128" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C128" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D128" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E128" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F128" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G128" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H128" s="16" t="n">
+        <v>1.1297</v>
+      </c>
+      <c r="I128" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J128" s="17" t="n">
+        <v>159924.3452</v>
+      </c>
+      <c r="K128" s="15" t="inlineStr">
+        <is>
+          <t>USDC 119,558.7697</t>
+        </is>
+      </c>
+      <c r="L128" s="17" t="n">
+        <v>119570.7267637075</v>
+      </c>
+      <c r="M128" s="17">
+        <f>J128-L128</f>
+        <v/>
+      </c>
+      <c r="N128" s="18">
+        <f>IF(J128=0,"",L128/J128)</f>
+        <v/>
+      </c>
+      <c r="O128" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:41:20</t>
+        </is>
+      </c>
+      <c r="B129" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C129" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D129" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E129" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F129" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G129" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H129" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I129" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J129" s="17" t="n">
+        <v>160092.0534906599</v>
+      </c>
+      <c r="K129" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,509.0058</t>
+        </is>
+      </c>
+      <c r="L129" s="17" t="n">
+        <v>138481.3039849279</v>
+      </c>
+      <c r="M129" s="17">
+        <f>J129-L129</f>
+        <v/>
+      </c>
+      <c r="N129" s="18">
+        <f>IF(J129=0,"",L129/J129)</f>
+        <v/>
+      </c>
+      <c r="O129" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:41:20</t>
+        </is>
+      </c>
+      <c r="B130" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C130" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D130" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E130" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F130" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeef003c</t>
+        </is>
+      </c>
+      <c r="G130" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H130" s="16" t="inlineStr"/>
+      <c r="I130" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,800.0745</t>
+        </is>
+      </c>
+      <c r="J130" s="17" t="n">
+        <v>50787.88245012768</v>
+      </c>
+      <c r="K130" s="15" t="inlineStr"/>
+      <c r="L130" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M130" s="17">
+        <f>J130-L130</f>
+        <v/>
+      </c>
+      <c r="N130" s="18">
+        <f>IF(J130=0,"",L130/J130)</f>
+        <v/>
+      </c>
+      <c r="O130" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:41:20</t>
+        </is>
+      </c>
+      <c r="B131" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C131" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D131" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E131" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F131" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G131" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H131" s="16" t="inlineStr"/>
+      <c r="I131" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J131" s="17" t="n">
+        <v>95911.90540587669</v>
+      </c>
+      <c r="K131" s="15" t="inlineStr"/>
+      <c r="L131" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M131" s="17">
+        <f>J131-L131</f>
+        <v/>
+      </c>
+      <c r="N131" s="18">
+        <f>IF(J131=0,"",L131/J131)</f>
+        <v/>
+      </c>
+      <c r="O131" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:41:20</t>
+        </is>
+      </c>
+      <c r="B132" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C132" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D132" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E132" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F132" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G132" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H132" s="16" t="inlineStr"/>
+      <c r="I132" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J132" s="17" t="n">
+        <v>34339.20546328334</v>
+      </c>
+      <c r="K132" s="15" t="inlineStr"/>
+      <c r="L132" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M132" s="17">
+        <f>J132-L132</f>
+        <v/>
+      </c>
+      <c r="N132" s="18">
+        <f>IF(J132=0,"",L132/J132)</f>
+        <v/>
+      </c>
+      <c r="O132" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:41:20</t>
+        </is>
+      </c>
+      <c r="B133" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C133" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D133" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E133" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F133" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G133" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H133" s="16" t="n">
+        <v>1.042</v>
+      </c>
+      <c r="I133" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J133" s="17" t="n">
+        <v>269689.1502594027</v>
+      </c>
+      <c r="K133" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,002.3970</t>
+        </is>
+      </c>
+      <c r="L133" s="17" t="n">
+        <v>232946.4764227205</v>
+      </c>
+      <c r="M133" s="17">
+        <f>J133-L133</f>
+        <v/>
+      </c>
+      <c r="N133" s="18">
+        <f>IF(J133=0,"",L133/J133)</f>
+        <v/>
+      </c>
+      <c r="O133" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:41:20</t>
+        </is>
+      </c>
+      <c r="B134" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C134" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D134" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E134" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F134" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G134" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H134" s="16" t="inlineStr"/>
+      <c r="I134" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,500.3087</t>
+        </is>
+      </c>
+      <c r="J134" s="17" t="n">
+        <v>15496.58862373629</v>
+      </c>
+      <c r="K134" s="15" t="inlineStr"/>
+      <c r="L134" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M134" s="17">
+        <f>J134-L134</f>
+        <v/>
+      </c>
+      <c r="N134" s="18">
+        <f>IF(J134=0,"",L134/J134)</f>
+        <v/>
+      </c>
+      <c r="O134" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:48:04</t>
+        </is>
+      </c>
+      <c r="B135" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C135" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D135" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E135" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F135" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G135" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H135" s="16" t="n">
+        <v>1.0478</v>
+      </c>
+      <c r="I135" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J135" s="17" t="n">
+        <v>140874.4736785287</v>
+      </c>
+      <c r="K135" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,018.0445</t>
+        </is>
+      </c>
+      <c r="L135" s="17" t="n">
+        <v>120998.6815998821</v>
+      </c>
+      <c r="M135" s="17">
+        <f>J135-L135</f>
+        <v/>
+      </c>
+      <c r="N135" s="18">
+        <f>IF(J135=0,"",L135/J135)</f>
+        <v/>
+      </c>
+      <c r="O135" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:48:04</t>
+        </is>
+      </c>
+      <c r="B136" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C136" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D136" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E136" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F136" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G136" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H136" s="16" t="n">
+        <v>1.0451</v>
+      </c>
+      <c r="I136" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J136" s="17" t="n">
+        <v>328668.3463586073</v>
+      </c>
+      <c r="K136" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,367.2077</t>
+        </is>
+      </c>
+      <c r="L136" s="17" t="n">
+        <v>306391.4951144939</v>
+      </c>
+      <c r="M136" s="17">
+        <f>J136-L136</f>
+        <v/>
+      </c>
+      <c r="N136" s="18">
+        <f>IF(J136=0,"",L136/J136)</f>
+        <v/>
+      </c>
+      <c r="O136" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:48:04</t>
+        </is>
+      </c>
+      <c r="B137" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C137" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D137" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E137" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F137" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G137" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H137" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I137" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J137" s="17" t="n">
+        <v>385882.8757830351</v>
+      </c>
+      <c r="K137" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,579.2903</t>
+        </is>
+      </c>
+      <c r="L137" s="17" t="n">
+        <v>349607.0033187549</v>
+      </c>
+      <c r="M137" s="17">
+        <f>J137-L137</f>
+        <v/>
+      </c>
+      <c r="N137" s="18">
+        <f>IF(J137=0,"",L137/J137)</f>
+        <v/>
+      </c>
+      <c r="O137" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:48:04</t>
+        </is>
+      </c>
+      <c r="B138" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C138" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D138" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E138" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F138" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G138" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H138" s="16" t="n">
+        <v>1.0541</v>
+      </c>
+      <c r="I138" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7817</t>
+        </is>
+      </c>
+      <c r="J138" s="17" t="n">
+        <v>77796.19074829285</v>
+      </c>
+      <c r="K138" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,020.5213; USDC 0.0775</t>
+        </is>
+      </c>
+      <c r="L138" s="17" t="n">
+        <v>68009.71556859167</v>
+      </c>
+      <c r="M138" s="17">
+        <f>J138-L138</f>
+        <v/>
+      </c>
+      <c r="N138" s="18">
+        <f>IF(J138=0,"",L138/J138)</f>
+        <v/>
+      </c>
+      <c r="O138" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:48:04</t>
+        </is>
+      </c>
+      <c r="B139" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C139" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D139" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E139" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F139" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G139" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H139" s="16" t="n">
+        <v>1.1282</v>
+      </c>
+      <c r="I139" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J139" s="17" t="n">
+        <v>197021.5867003927</v>
+      </c>
+      <c r="K139" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,218.4491</t>
+        </is>
+      </c>
+      <c r="L139" s="17" t="n">
+        <v>150218.4490685559</v>
+      </c>
+      <c r="M139" s="17">
+        <f>J139-L139</f>
+        <v/>
+      </c>
+      <c r="N139" s="18">
+        <f>IF(J139=0,"",L139/J139)</f>
+        <v/>
+      </c>
+      <c r="O139" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:48:04</t>
+        </is>
+      </c>
+      <c r="B140" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C140" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D140" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E140" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F140" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G140" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H140" s="16" t="n">
+        <v>1.0527</v>
+      </c>
+      <c r="I140" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J140" s="17" t="n">
+        <v>186096.1049750841</v>
+      </c>
+      <c r="K140" s="15" t="inlineStr">
+        <is>
+          <t>USDC 161,827.5551</t>
+        </is>
+      </c>
+      <c r="L140" s="17" t="n">
+        <v>161827.5551410827</v>
+      </c>
+      <c r="M140" s="17">
+        <f>J140-L140</f>
+        <v/>
+      </c>
+      <c r="N140" s="18">
+        <f>IF(J140=0,"",L140/J140)</f>
+        <v/>
+      </c>
+      <c r="O140" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:48:04</t>
+        </is>
+      </c>
+      <c r="B141" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C141" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D141" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E141" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F141" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G141" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H141" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I141" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J141" s="17" t="n">
+        <v>327483.0881365995</v>
+      </c>
+      <c r="K141" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L141" s="17" t="n">
+        <v>280184.6617515259</v>
+      </c>
+      <c r="M141" s="17">
+        <f>J141-L141</f>
+        <v/>
+      </c>
+      <c r="N141" s="18">
+        <f>IF(J141=0,"",L141/J141)</f>
+        <v/>
+      </c>
+      <c r="O141" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:48:04</t>
+        </is>
+      </c>
+      <c r="B142" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C142" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D142" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E142" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F142" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G142" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H142" s="16" t="n">
+        <v>1.1297</v>
+      </c>
+      <c r="I142" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J142" s="17" t="n">
+        <v>159924.3452</v>
+      </c>
+      <c r="K142" s="15" t="inlineStr">
+        <is>
+          <t>USDC 119,560.3956</t>
+        </is>
+      </c>
+      <c r="L142" s="17" t="n">
+        <v>119560.3956380491</v>
+      </c>
+      <c r="M142" s="17">
+        <f>J142-L142</f>
+        <v/>
+      </c>
+      <c r="N142" s="18">
+        <f>IF(J142=0,"",L142/J142)</f>
+        <v/>
+      </c>
+      <c r="O142" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:48:04</t>
+        </is>
+      </c>
+      <c r="B143" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C143" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D143" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E143" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F143" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G143" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H143" s="16" t="n">
+        <v>1.0575</v>
+      </c>
+      <c r="I143" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J143" s="17" t="n">
+        <v>160092.3634516182</v>
+      </c>
+      <c r="K143" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,509.0058</t>
+        </is>
+      </c>
+      <c r="L143" s="17" t="n">
+        <v>138481.3039849279</v>
+      </c>
+      <c r="M143" s="17">
+        <f>J143-L143</f>
+        <v/>
+      </c>
+      <c r="N143" s="18">
+        <f>IF(J143=0,"",L143/J143)</f>
+        <v/>
+      </c>
+      <c r="O143" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:48:04</t>
+        </is>
+      </c>
+      <c r="B144" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C144" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D144" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E144" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F144" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeef003c</t>
+        </is>
+      </c>
+      <c r="G144" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H144" s="16" t="inlineStr"/>
+      <c r="I144" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,800.3108</t>
+        </is>
+      </c>
+      <c r="J144" s="17" t="n">
+        <v>50792.18277926736</v>
+      </c>
+      <c r="K144" s="15" t="inlineStr"/>
+      <c r="L144" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M144" s="17">
+        <f>J144-L144</f>
+        <v/>
+      </c>
+      <c r="N144" s="18">
+        <f>IF(J144=0,"",L144/J144)</f>
+        <v/>
+      </c>
+      <c r="O144" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:48:04</t>
+        </is>
+      </c>
+      <c r="B145" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C145" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D145" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E145" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F145" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeeff047</t>
+        </is>
+      </c>
+      <c r="G145" s="15" t="inlineStr">
+        <is>
+          <t>USDC vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H145" s="16" t="inlineStr"/>
+      <c r="I145" s="15" t="inlineStr">
+        <is>
+          <t>USDC 48,646.1854</t>
+        </is>
+      </c>
+      <c r="J145" s="17" t="n">
+        <v>48646.185411</v>
+      </c>
+      <c r="K145" s="15" t="inlineStr"/>
+      <c r="L145" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M145" s="17">
+        <f>J145-L145</f>
+        <v/>
+      </c>
+      <c r="N145" s="18">
+        <f>IF(J145=0,"",L145/J145)</f>
+        <v/>
+      </c>
+      <c r="O145" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:48:04</t>
+        </is>
+      </c>
+      <c r="B146" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C146" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D146" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E146" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F146" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G146" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H146" s="16" t="inlineStr"/>
+      <c r="I146" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J146" s="17" t="n">
+        <v>95911.90540587669</v>
+      </c>
+      <c r="K146" s="15" t="inlineStr"/>
+      <c r="L146" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M146" s="17">
+        <f>J146-L146</f>
+        <v/>
+      </c>
+      <c r="N146" s="18">
+        <f>IF(J146=0,"",L146/J146)</f>
+        <v/>
+      </c>
+      <c r="O146" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:48:04</t>
+        </is>
+      </c>
+      <c r="B147" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C147" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D147" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E147" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F147" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G147" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H147" s="16" t="inlineStr"/>
+      <c r="I147" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J147" s="17" t="n">
+        <v>34339.20546328334</v>
+      </c>
+      <c r="K147" s="15" t="inlineStr"/>
+      <c r="L147" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M147" s="17">
+        <f>J147-L147</f>
+        <v/>
+      </c>
+      <c r="N147" s="18">
+        <f>IF(J147=0,"",L147/J147)</f>
+        <v/>
+      </c>
+      <c r="O147" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:48:04</t>
+        </is>
+      </c>
+      <c r="B148" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C148" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D148" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E148" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F148" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G148" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H148" s="16" t="n">
+        <v>1.0419</v>
+      </c>
+      <c r="I148" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J148" s="17" t="n">
+        <v>269689.1502594027</v>
+      </c>
+      <c r="K148" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,004.2248</t>
+        </is>
+      </c>
+      <c r="L148" s="17" t="n">
+        <v>232966.9441700246</v>
+      </c>
+      <c r="M148" s="17">
+        <f>J148-L148</f>
+        <v/>
+      </c>
+      <c r="N148" s="18">
+        <f>IF(J148=0,"",L148/J148)</f>
+        <v/>
+      </c>
+      <c r="O148" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:48:04</t>
+        </is>
+      </c>
+      <c r="B149" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C149" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D149" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E149" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F149" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G149" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H149" s="16" t="inlineStr"/>
+      <c r="I149" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,500.5029</t>
+        </is>
+      </c>
+      <c r="J149" s="17" t="n">
+        <v>15498.02281787477</v>
+      </c>
+      <c r="K149" s="15" t="inlineStr"/>
+      <c r="L149" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M149" s="17">
+        <f>J149-L149</f>
+        <v/>
+      </c>
+      <c r="N149" s="18">
+        <f>IF(J149=0,"",L149/J149)</f>
+        <v/>
+      </c>
+      <c r="O149" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -8614,7 +10561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -8980,6 +10927,76 @@
         <v>1.0375</v>
       </c>
       <c r="I10" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:41:20</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="n">
+        <v>553089.0820788638</v>
+      </c>
+      <c r="D11" s="17" t="n">
+        <v>501820.6338826688</v>
+      </c>
+      <c r="E11" s="17" t="n">
+        <v>2430062.582582969</v>
+      </c>
+      <c r="F11" s="17" t="n">
+        <v>1928241.9487003</v>
+      </c>
+      <c r="G11" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="H11" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I11" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 10:48:04</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="n">
+        <v>553085.8928705006</v>
+      </c>
+      <c r="D12" s="17" t="n">
+        <v>550469.8218129736</v>
+      </c>
+      <c r="E12" s="17" t="n">
+        <v>2478716.027168863</v>
+      </c>
+      <c r="F12" s="17" t="n">
+        <v>1928246.205355889</v>
+      </c>
+      <c r="G12" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="H12" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I12" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-28 17:13 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O149"/>
+  <dimension ref="A1:O164"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -10531,6 +10531,1011 @@
         <v/>
       </c>
       <c r="O149" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:13:37</t>
+        </is>
+      </c>
+      <c r="B150" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C150" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D150" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E150" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F150" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G150" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H150" s="16" t="n">
+        <v>1.0479</v>
+      </c>
+      <c r="I150" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J150" s="17" t="n">
+        <v>140876.8652683409</v>
+      </c>
+      <c r="K150" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,021.5606</t>
+        </is>
+      </c>
+      <c r="L150" s="17" t="n">
+        <v>120994.9358076788</v>
+      </c>
+      <c r="M150" s="17">
+        <f>J150-L150</f>
+        <v/>
+      </c>
+      <c r="N150" s="18">
+        <f>IF(J150=0,"",L150/J150)</f>
+        <v/>
+      </c>
+      <c r="O150" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:13:37</t>
+        </is>
+      </c>
+      <c r="B151" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C151" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D151" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E151" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F151" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G151" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H151" s="16" t="n">
+        <v>1.0451</v>
+      </c>
+      <c r="I151" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J151" s="17" t="n">
+        <v>328676.7198404301</v>
+      </c>
+      <c r="K151" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,371.3254</t>
+        </is>
+      </c>
+      <c r="L151" s="17" t="n">
+        <v>306415.1971347085</v>
+      </c>
+      <c r="M151" s="17">
+        <f>J151-L151</f>
+        <v/>
+      </c>
+      <c r="N151" s="18">
+        <f>IF(J151=0,"",L151/J151)</f>
+        <v/>
+      </c>
+      <c r="O151" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:13:37</t>
+        </is>
+      </c>
+      <c r="B152" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C152" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D152" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E152" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F152" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G152" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H152" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I152" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J152" s="17" t="n">
+        <v>385897.0076295341</v>
+      </c>
+      <c r="K152" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,585.6100</t>
+        </is>
+      </c>
+      <c r="L152" s="17" t="n">
+        <v>349635.6700018566</v>
+      </c>
+      <c r="M152" s="17">
+        <f>J152-L152</f>
+        <v/>
+      </c>
+      <c r="N152" s="18">
+        <f>IF(J152=0,"",L152/J152)</f>
+        <v/>
+      </c>
+      <c r="O152" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:13:37</t>
+        </is>
+      </c>
+      <c r="B153" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C153" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D153" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E153" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F153" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G153" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H153" s="16" t="n">
+        <v>1.0541</v>
+      </c>
+      <c r="I153" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7823</t>
+        </is>
+      </c>
+      <c r="J153" s="17" t="n">
+        <v>77797.75026982719</v>
+      </c>
+      <c r="K153" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,022.0527; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L153" s="17" t="n">
+        <v>68007.16545715183</v>
+      </c>
+      <c r="M153" s="17">
+        <f>J153-L153</f>
+        <v/>
+      </c>
+      <c r="N153" s="18">
+        <f>IF(J153=0,"",L153/J153)</f>
+        <v/>
+      </c>
+      <c r="O153" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:13:37</t>
+        </is>
+      </c>
+      <c r="B154" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C154" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D154" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E154" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F154" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G154" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H154" s="16" t="n">
+        <v>1.1285</v>
+      </c>
+      <c r="I154" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J154" s="17" t="n">
+        <v>197081.3128413185</v>
+      </c>
+      <c r="K154" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,225.0296</t>
+        </is>
+      </c>
+      <c r="L154" s="17" t="n">
+        <v>150240.0536008047</v>
+      </c>
+      <c r="M154" s="17">
+        <f>J154-L154</f>
+        <v/>
+      </c>
+      <c r="N154" s="18">
+        <f>IF(J154=0,"",L154/J154)</f>
+        <v/>
+      </c>
+      <c r="O154" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:13:37</t>
+        </is>
+      </c>
+      <c r="B155" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C155" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D155" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E155" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F155" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G155" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H155" s="16" t="n">
+        <v>1.0528</v>
+      </c>
+      <c r="I155" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J155" s="17" t="n">
+        <v>186079.7945419633</v>
+      </c>
+      <c r="K155" s="15" t="inlineStr">
+        <is>
+          <t>USDC 161,827.6712</t>
+        </is>
+      </c>
+      <c r="L155" s="17" t="n">
+        <v>161843.8556121311</v>
+      </c>
+      <c r="M155" s="17">
+        <f>J155-L155</f>
+        <v/>
+      </c>
+      <c r="N155" s="18">
+        <f>IF(J155=0,"",L155/J155)</f>
+        <v/>
+      </c>
+      <c r="O155" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:13:37</t>
+        </is>
+      </c>
+      <c r="B156" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C156" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D156" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E156" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F156" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G156" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H156" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I156" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J156" s="17" t="n">
+        <v>327484.2985285849</v>
+      </c>
+      <c r="K156" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L156" s="17" t="n">
+        <v>280151.2075648866</v>
+      </c>
+      <c r="M156" s="17">
+        <f>J156-L156</f>
+        <v/>
+      </c>
+      <c r="N156" s="18">
+        <f>IF(J156=0,"",L156/J156)</f>
+        <v/>
+      </c>
+      <c r="O156" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:13:37</t>
+        </is>
+      </c>
+      <c r="B157" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C157" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D157" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E157" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F157" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G157" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H157" s="16" t="n">
+        <v>1.1296</v>
+      </c>
+      <c r="I157" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J157" s="17" t="n">
+        <v>159908.3543645635</v>
+      </c>
+      <c r="K157" s="15" t="inlineStr">
+        <is>
+          <t>USDC 119,565.5188</t>
+        </is>
+      </c>
+      <c r="L157" s="17" t="n">
+        <v>119577.4765555012</v>
+      </c>
+      <c r="M157" s="17">
+        <f>J157-L157</f>
+        <v/>
+      </c>
+      <c r="N157" s="18">
+        <f>IF(J157=0,"",L157/J157)</f>
+        <v/>
+      </c>
+      <c r="O157" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:13:37</t>
+        </is>
+      </c>
+      <c r="B158" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C158" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D158" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E158" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F158" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G158" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H158" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I158" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J158" s="17" t="n">
+        <v>160098.2263723331</v>
+      </c>
+      <c r="K158" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,513.6478</t>
+        </is>
+      </c>
+      <c r="L158" s="17" t="n">
+        <v>138485.9450208691</v>
+      </c>
+      <c r="M158" s="17">
+        <f>J158-L158</f>
+        <v/>
+      </c>
+      <c r="N158" s="18">
+        <f>IF(J158=0,"",L158/J158)</f>
+        <v/>
+      </c>
+      <c r="O158" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:13:37</t>
+        </is>
+      </c>
+      <c r="B159" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C159" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D159" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E159" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F159" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeef003c</t>
+        </is>
+      </c>
+      <c r="G159" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H159" s="16" t="inlineStr"/>
+      <c r="I159" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,801.2199</t>
+        </is>
+      </c>
+      <c r="J159" s="17" t="n">
+        <v>50790.04360362816</v>
+      </c>
+      <c r="K159" s="15" t="inlineStr"/>
+      <c r="L159" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M159" s="17">
+        <f>J159-L159</f>
+        <v/>
+      </c>
+      <c r="N159" s="18">
+        <f>IF(J159=0,"",L159/J159)</f>
+        <v/>
+      </c>
+      <c r="O159" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:13:37</t>
+        </is>
+      </c>
+      <c r="B160" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C160" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D160" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E160" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F160" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeeff047</t>
+        </is>
+      </c>
+      <c r="G160" s="15" t="inlineStr">
+        <is>
+          <t>USDC vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H160" s="16" t="inlineStr"/>
+      <c r="I160" s="15" t="inlineStr">
+        <is>
+          <t>USDC 48,647.0829</t>
+        </is>
+      </c>
+      <c r="J160" s="17" t="n">
+        <v>48651.94808880887</v>
+      </c>
+      <c r="K160" s="15" t="inlineStr"/>
+      <c r="L160" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M160" s="17">
+        <f>J160-L160</f>
+        <v/>
+      </c>
+      <c r="N160" s="18">
+        <f>IF(J160=0,"",L160/J160)</f>
+        <v/>
+      </c>
+      <c r="O160" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:13:37</t>
+        </is>
+      </c>
+      <c r="B161" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C161" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D161" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E161" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F161" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G161" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H161" s="16" t="inlineStr"/>
+      <c r="I161" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J161" s="17" t="n">
+        <v>95898.34722895516</v>
+      </c>
+      <c r="K161" s="15" t="inlineStr"/>
+      <c r="L161" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M161" s="17">
+        <f>J161-L161</f>
+        <v/>
+      </c>
+      <c r="N161" s="18">
+        <f>IF(J161=0,"",L161/J161)</f>
+        <v/>
+      </c>
+      <c r="O161" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:13:37</t>
+        </is>
+      </c>
+      <c r="B162" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C162" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D162" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E162" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F162" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G162" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H162" s="16" t="inlineStr"/>
+      <c r="I162" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J162" s="17" t="n">
+        <v>34342.73872267789</v>
+      </c>
+      <c r="K162" s="15" t="inlineStr"/>
+      <c r="L162" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M162" s="17">
+        <f>J162-L162</f>
+        <v/>
+      </c>
+      <c r="N162" s="18">
+        <f>IF(J162=0,"",L162/J162)</f>
+        <v/>
+      </c>
+      <c r="O162" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:13:37</t>
+        </is>
+      </c>
+      <c r="B163" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C163" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D163" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E163" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F163" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G163" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H163" s="16" t="n">
+        <v>1.0419</v>
+      </c>
+      <c r="I163" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J163" s="17" t="n">
+        <v>269695.4896114625</v>
+      </c>
+      <c r="K163" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,011.8464</t>
+        </is>
+      </c>
+      <c r="L163" s="17" t="n">
+        <v>232960.5837448028</v>
+      </c>
+      <c r="M163" s="17">
+        <f>J163-L163</f>
+        <v/>
+      </c>
+      <c r="N163" s="18">
+        <f>IF(J163=0,"",L163/J163)</f>
+        <v/>
+      </c>
+      <c r="O163" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:13:37</t>
+        </is>
+      </c>
+      <c r="B164" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C164" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D164" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E164" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F164" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G164" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H164" s="16" t="inlineStr"/>
+      <c r="I164" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,502.9223</t>
+        </is>
+      </c>
+      <c r="J164" s="17" t="n">
+        <v>15499.51164260171</v>
+      </c>
+      <c r="K164" s="15" t="inlineStr"/>
+      <c r="L164" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M164" s="17">
+        <f>J164-L164</f>
+        <v/>
+      </c>
+      <c r="N164" s="18">
+        <f>IF(J164=0,"",L164/J164)</f>
+        <v/>
+      </c>
+      <c r="O164" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -10561,7 +11566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -10997,6 +12002,41 @@
         <v>1.0375</v>
       </c>
       <c r="I12" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:13:37</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="n">
+        <v>553081.6586247215</v>
+      </c>
+      <c r="D13" s="17" t="n">
+        <v>550466.3180546388</v>
+      </c>
+      <c r="E13" s="17" t="n">
+        <v>2478778.40855503</v>
+      </c>
+      <c r="F13" s="17" t="n">
+        <v>1928312.090500392</v>
+      </c>
+      <c r="G13" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="H13" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I13" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-28 17:14 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O164"/>
+  <dimension ref="A1:O179"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -11536,6 +11536,1011 @@
         <v/>
       </c>
       <c r="O164" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:14:01</t>
+        </is>
+      </c>
+      <c r="B165" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C165" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D165" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E165" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F165" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G165" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H165" s="16" t="n">
+        <v>1.0479</v>
+      </c>
+      <c r="I165" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J165" s="17" t="n">
+        <v>140876.8652683409</v>
+      </c>
+      <c r="K165" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,021.5606</t>
+        </is>
+      </c>
+      <c r="L165" s="17" t="n">
+        <v>120994.9358076788</v>
+      </c>
+      <c r="M165" s="17">
+        <f>J165-L165</f>
+        <v/>
+      </c>
+      <c r="N165" s="18">
+        <f>IF(J165=0,"",L165/J165)</f>
+        <v/>
+      </c>
+      <c r="O165" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:14:01</t>
+        </is>
+      </c>
+      <c r="B166" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C166" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D166" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E166" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F166" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G166" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H166" s="16" t="n">
+        <v>1.0451</v>
+      </c>
+      <c r="I166" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J166" s="17" t="n">
+        <v>328676.7198404301</v>
+      </c>
+      <c r="K166" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,371.3254</t>
+        </is>
+      </c>
+      <c r="L166" s="17" t="n">
+        <v>306415.1971347085</v>
+      </c>
+      <c r="M166" s="17">
+        <f>J166-L166</f>
+        <v/>
+      </c>
+      <c r="N166" s="18">
+        <f>IF(J166=0,"",L166/J166)</f>
+        <v/>
+      </c>
+      <c r="O166" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:14:01</t>
+        </is>
+      </c>
+      <c r="B167" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C167" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D167" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E167" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F167" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G167" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H167" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I167" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J167" s="17" t="n">
+        <v>385897.0076295341</v>
+      </c>
+      <c r="K167" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,585.6100</t>
+        </is>
+      </c>
+      <c r="L167" s="17" t="n">
+        <v>349635.6700018566</v>
+      </c>
+      <c r="M167" s="17">
+        <f>J167-L167</f>
+        <v/>
+      </c>
+      <c r="N167" s="18">
+        <f>IF(J167=0,"",L167/J167)</f>
+        <v/>
+      </c>
+      <c r="O167" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:14:01</t>
+        </is>
+      </c>
+      <c r="B168" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C168" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D168" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E168" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F168" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G168" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H168" s="16" t="n">
+        <v>1.0541</v>
+      </c>
+      <c r="I168" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7823</t>
+        </is>
+      </c>
+      <c r="J168" s="17" t="n">
+        <v>77797.74763674867</v>
+      </c>
+      <c r="K168" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,022.0527; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L168" s="17" t="n">
+        <v>68007.16545715183</v>
+      </c>
+      <c r="M168" s="17">
+        <f>J168-L168</f>
+        <v/>
+      </c>
+      <c r="N168" s="18">
+        <f>IF(J168=0,"",L168/J168)</f>
+        <v/>
+      </c>
+      <c r="O168" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:14:01</t>
+        </is>
+      </c>
+      <c r="B169" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C169" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D169" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E169" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F169" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G169" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H169" s="16" t="n">
+        <v>1.1285</v>
+      </c>
+      <c r="I169" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J169" s="17" t="n">
+        <v>197081.3128413185</v>
+      </c>
+      <c r="K169" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,225.0296</t>
+        </is>
+      </c>
+      <c r="L169" s="17" t="n">
+        <v>150240.0536008047</v>
+      </c>
+      <c r="M169" s="17">
+        <f>J169-L169</f>
+        <v/>
+      </c>
+      <c r="N169" s="18">
+        <f>IF(J169=0,"",L169/J169)</f>
+        <v/>
+      </c>
+      <c r="O169" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:14:01</t>
+        </is>
+      </c>
+      <c r="B170" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C170" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D170" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E170" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F170" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G170" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H170" s="16" t="n">
+        <v>1.0528</v>
+      </c>
+      <c r="I170" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J170" s="17" t="n">
+        <v>186079.7945419633</v>
+      </c>
+      <c r="K170" s="15" t="inlineStr">
+        <is>
+          <t>USDC 161,827.6712</t>
+        </is>
+      </c>
+      <c r="L170" s="17" t="n">
+        <v>161843.8556121311</v>
+      </c>
+      <c r="M170" s="17">
+        <f>J170-L170</f>
+        <v/>
+      </c>
+      <c r="N170" s="18">
+        <f>IF(J170=0,"",L170/J170)</f>
+        <v/>
+      </c>
+      <c r="O170" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:14:01</t>
+        </is>
+      </c>
+      <c r="B171" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C171" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D171" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E171" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F171" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G171" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H171" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I171" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J171" s="17" t="n">
+        <v>327484.2985285849</v>
+      </c>
+      <c r="K171" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L171" s="17" t="n">
+        <v>280151.2075648866</v>
+      </c>
+      <c r="M171" s="17">
+        <f>J171-L171</f>
+        <v/>
+      </c>
+      <c r="N171" s="18">
+        <f>IF(J171=0,"",L171/J171)</f>
+        <v/>
+      </c>
+      <c r="O171" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:14:01</t>
+        </is>
+      </c>
+      <c r="B172" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C172" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D172" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E172" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F172" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G172" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H172" s="16" t="n">
+        <v>1.1296</v>
+      </c>
+      <c r="I172" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J172" s="17" t="n">
+        <v>159908.3543645635</v>
+      </c>
+      <c r="K172" s="15" t="inlineStr">
+        <is>
+          <t>USDC 119,565.5188</t>
+        </is>
+      </c>
+      <c r="L172" s="17" t="n">
+        <v>119577.4765555012</v>
+      </c>
+      <c r="M172" s="17">
+        <f>J172-L172</f>
+        <v/>
+      </c>
+      <c r="N172" s="18">
+        <f>IF(J172=0,"",L172/J172)</f>
+        <v/>
+      </c>
+      <c r="O172" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:14:01</t>
+        </is>
+      </c>
+      <c r="B173" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C173" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D173" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E173" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F173" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G173" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H173" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I173" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J173" s="17" t="n">
+        <v>160098.2263723331</v>
+      </c>
+      <c r="K173" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,513.6478</t>
+        </is>
+      </c>
+      <c r="L173" s="17" t="n">
+        <v>138485.9450208691</v>
+      </c>
+      <c r="M173" s="17">
+        <f>J173-L173</f>
+        <v/>
+      </c>
+      <c r="N173" s="18">
+        <f>IF(J173=0,"",L173/J173)</f>
+        <v/>
+      </c>
+      <c r="O173" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:14:01</t>
+        </is>
+      </c>
+      <c r="B174" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C174" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D174" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E174" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F174" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeef003c</t>
+        </is>
+      </c>
+      <c r="G174" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H174" s="16" t="inlineStr"/>
+      <c r="I174" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,801.2199</t>
+        </is>
+      </c>
+      <c r="J174" s="17" t="n">
+        <v>50790.04360362816</v>
+      </c>
+      <c r="K174" s="15" t="inlineStr"/>
+      <c r="L174" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M174" s="17">
+        <f>J174-L174</f>
+        <v/>
+      </c>
+      <c r="N174" s="18">
+        <f>IF(J174=0,"",L174/J174)</f>
+        <v/>
+      </c>
+      <c r="O174" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:14:01</t>
+        </is>
+      </c>
+      <c r="B175" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C175" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D175" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E175" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F175" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeeff047</t>
+        </is>
+      </c>
+      <c r="G175" s="15" t="inlineStr">
+        <is>
+          <t>USDC vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H175" s="16" t="inlineStr"/>
+      <c r="I175" s="15" t="inlineStr">
+        <is>
+          <t>USDC 48,647.0829</t>
+        </is>
+      </c>
+      <c r="J175" s="17" t="n">
+        <v>48651.94808880887</v>
+      </c>
+      <c r="K175" s="15" t="inlineStr"/>
+      <c r="L175" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M175" s="17">
+        <f>J175-L175</f>
+        <v/>
+      </c>
+      <c r="N175" s="18">
+        <f>IF(J175=0,"",L175/J175)</f>
+        <v/>
+      </c>
+      <c r="O175" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:14:01</t>
+        </is>
+      </c>
+      <c r="B176" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C176" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D176" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E176" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F176" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G176" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H176" s="16" t="inlineStr"/>
+      <c r="I176" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J176" s="17" t="n">
+        <v>95898.34722895516</v>
+      </c>
+      <c r="K176" s="15" t="inlineStr"/>
+      <c r="L176" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M176" s="17">
+        <f>J176-L176</f>
+        <v/>
+      </c>
+      <c r="N176" s="18">
+        <f>IF(J176=0,"",L176/J176)</f>
+        <v/>
+      </c>
+      <c r="O176" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:14:01</t>
+        </is>
+      </c>
+      <c r="B177" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C177" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D177" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E177" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F177" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G177" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H177" s="16" t="inlineStr"/>
+      <c r="I177" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J177" s="17" t="n">
+        <v>34342.73872267789</v>
+      </c>
+      <c r="K177" s="15" t="inlineStr"/>
+      <c r="L177" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M177" s="17">
+        <f>J177-L177</f>
+        <v/>
+      </c>
+      <c r="N177" s="18">
+        <f>IF(J177=0,"",L177/J177)</f>
+        <v/>
+      </c>
+      <c r="O177" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:14:01</t>
+        </is>
+      </c>
+      <c r="B178" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C178" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D178" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E178" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F178" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G178" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H178" s="16" t="n">
+        <v>1.0419</v>
+      </c>
+      <c r="I178" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J178" s="17" t="n">
+        <v>269695.4896114625</v>
+      </c>
+      <c r="K178" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,011.8464</t>
+        </is>
+      </c>
+      <c r="L178" s="17" t="n">
+        <v>232960.5837448028</v>
+      </c>
+      <c r="M178" s="17">
+        <f>J178-L178</f>
+        <v/>
+      </c>
+      <c r="N178" s="18">
+        <f>IF(J178=0,"",L178/J178)</f>
+        <v/>
+      </c>
+      <c r="O178" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:14:01</t>
+        </is>
+      </c>
+      <c r="B179" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C179" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D179" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E179" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F179" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G179" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H179" s="16" t="inlineStr"/>
+      <c r="I179" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,502.9223</t>
+        </is>
+      </c>
+      <c r="J179" s="17" t="n">
+        <v>15499.51164260171</v>
+      </c>
+      <c r="K179" s="15" t="inlineStr"/>
+      <c r="L179" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M179" s="17">
+        <f>J179-L179</f>
+        <v/>
+      </c>
+      <c r="N179" s="18">
+        <f>IF(J179=0,"",L179/J179)</f>
+        <v/>
+      </c>
+      <c r="O179" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -11566,7 +12571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -12037,6 +13042,41 @@
         <v>1.0375</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 17:14:01</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="n">
+        <v>553081.6123284872</v>
+      </c>
+      <c r="D14" s="17" t="n">
+        <v>550466.3154215603</v>
+      </c>
+      <c r="E14" s="17" t="n">
+        <v>2478778.405921952</v>
+      </c>
+      <c r="F14" s="17" t="n">
+        <v>1928312.090500392</v>
+      </c>
+      <c r="G14" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="H14" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I14" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-28 19:13 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O179"/>
+  <dimension ref="A1:O194"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -12541,6 +12541,1011 @@
         <v/>
       </c>
       <c r="O179" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 19:12:28</t>
+        </is>
+      </c>
+      <c r="B180" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C180" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D180" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E180" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F180" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G180" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H180" s="16" t="n">
+        <v>1.0478</v>
+      </c>
+      <c r="I180" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J180" s="17" t="n">
+        <v>140874.26130531</v>
+      </c>
+      <c r="K180" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,022.8377</t>
+        </is>
+      </c>
+      <c r="L180" s="17" t="n">
+        <v>121004.6842883429</v>
+      </c>
+      <c r="M180" s="17">
+        <f>J180-L180</f>
+        <v/>
+      </c>
+      <c r="N180" s="18">
+        <f>IF(J180=0,"",L180/J180)</f>
+        <v/>
+      </c>
+      <c r="O180" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 19:12:28</t>
+        </is>
+      </c>
+      <c r="B181" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C181" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D181" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E181" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F181" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G181" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H181" s="16" t="n">
+        <v>1.0451</v>
+      </c>
+      <c r="I181" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J181" s="17" t="n">
+        <v>328679.4807437729</v>
+      </c>
+      <c r="K181" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,372.4926</t>
+        </is>
+      </c>
+      <c r="L181" s="17" t="n">
+        <v>306414.6357528478</v>
+      </c>
+      <c r="M181" s="17">
+        <f>J181-L181</f>
+        <v/>
+      </c>
+      <c r="N181" s="18">
+        <f>IF(J181=0,"",L181/J181)</f>
+        <v/>
+      </c>
+      <c r="O181" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 19:12:28</t>
+        </is>
+      </c>
+      <c r="B182" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C182" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D182" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E182" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F182" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G182" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H182" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I182" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J182" s="17" t="n">
+        <v>385940.2051645985</v>
+      </c>
+      <c r="K182" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,587.4014</t>
+        </is>
+      </c>
+      <c r="L182" s="17" t="n">
+        <v>349635.4890771247</v>
+      </c>
+      <c r="M182" s="17">
+        <f>J182-L182</f>
+        <v/>
+      </c>
+      <c r="N182" s="18">
+        <f>IF(J182=0,"",L182/J182)</f>
+        <v/>
+      </c>
+      <c r="O182" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 19:12:28</t>
+        </is>
+      </c>
+      <c r="B183" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C183" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D183" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E183" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F183" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G183" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H183" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I183" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7826</t>
+        </is>
+      </c>
+      <c r="J183" s="17" t="n">
+        <v>77786.95059201948</v>
+      </c>
+      <c r="K183" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,022.6150; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L183" s="17" t="n">
+        <v>68012.48912251322</v>
+      </c>
+      <c r="M183" s="17">
+        <f>J183-L183</f>
+        <v/>
+      </c>
+      <c r="N183" s="18">
+        <f>IF(J183=0,"",L183/J183)</f>
+        <v/>
+      </c>
+      <c r="O183" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 19:12:28</t>
+        </is>
+      </c>
+      <c r="B184" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C184" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D184" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E184" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F184" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G184" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H184" s="16" t="n">
+        <v>1.1285</v>
+      </c>
+      <c r="I184" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J184" s="17" t="n">
+        <v>197088.6958399535</v>
+      </c>
+      <c r="K184" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,228.5848</t>
+        </is>
+      </c>
+      <c r="L184" s="17" t="n">
+        <v>150243.6091312141</v>
+      </c>
+      <c r="M184" s="17">
+        <f>J184-L184</f>
+        <v/>
+      </c>
+      <c r="N184" s="18">
+        <f>IF(J184=0,"",L184/J184)</f>
+        <v/>
+      </c>
+      <c r="O184" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 19:12:28</t>
+        </is>
+      </c>
+      <c r="B185" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C185" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D185" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E185" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F185" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G185" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H185" s="16" t="n">
+        <v>1.0528</v>
+      </c>
+      <c r="I185" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J185" s="17" t="n">
+        <v>186079.019978838</v>
+      </c>
+      <c r="K185" s="15" t="inlineStr">
+        <is>
+          <t>USDC 161,827.6712</t>
+        </is>
+      </c>
+      <c r="L185" s="17" t="n">
+        <v>161843.8556121311</v>
+      </c>
+      <c r="M185" s="17">
+        <f>J185-L185</f>
+        <v/>
+      </c>
+      <c r="N185" s="18">
+        <f>IF(J185=0,"",L185/J185)</f>
+        <v/>
+      </c>
+      <c r="O185" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 19:12:28</t>
+        </is>
+      </c>
+      <c r="B186" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C186" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D186" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E186" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F186" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G186" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H186" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I186" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J186" s="17" t="n">
+        <v>327466.9850072496</v>
+      </c>
+      <c r="K186" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L186" s="17" t="n">
+        <v>280151.2992174175</v>
+      </c>
+      <c r="M186" s="17">
+        <f>J186-L186</f>
+        <v/>
+      </c>
+      <c r="N186" s="18">
+        <f>IF(J186=0,"",L186/J186)</f>
+        <v/>
+      </c>
+      <c r="O186" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 19:12:28</t>
+        </is>
+      </c>
+      <c r="B187" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C187" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D187" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E187" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F187" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G187" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H187" s="16" t="n">
+        <v>1.1296</v>
+      </c>
+      <c r="I187" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J187" s="17" t="n">
+        <v>159924.3452</v>
+      </c>
+      <c r="K187" s="15" t="inlineStr">
+        <is>
+          <t>USDC 119,566.4850</t>
+        </is>
+      </c>
+      <c r="L187" s="17" t="n">
+        <v>119578.4428387121</v>
+      </c>
+      <c r="M187" s="17">
+        <f>J187-L187</f>
+        <v/>
+      </c>
+      <c r="N187" s="18">
+        <f>IF(J187=0,"",L187/J187)</f>
+        <v/>
+      </c>
+      <c r="O187" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 19:12:28</t>
+        </is>
+      </c>
+      <c r="B188" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C188" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D188" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E188" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F188" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G188" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H188" s="16" t="n">
+        <v>1.0575</v>
+      </c>
+      <c r="I188" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J188" s="17" t="n">
+        <v>160116.1478607374</v>
+      </c>
+      <c r="K188" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,514.6077</t>
+        </is>
+      </c>
+      <c r="L188" s="17" t="n">
+        <v>138486.9047712727</v>
+      </c>
+      <c r="M188" s="17">
+        <f>J188-L188</f>
+        <v/>
+      </c>
+      <c r="N188" s="18">
+        <f>IF(J188=0,"",L188/J188)</f>
+        <v/>
+      </c>
+      <c r="O188" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 19:12:28</t>
+        </is>
+      </c>
+      <c r="B189" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C189" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D189" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E189" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F189" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeef003c</t>
+        </is>
+      </c>
+      <c r="G189" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H189" s="16" t="inlineStr"/>
+      <c r="I189" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,801.5319</t>
+        </is>
+      </c>
+      <c r="J189" s="17" t="n">
+        <v>50793.9116842129</v>
+      </c>
+      <c r="K189" s="15" t="inlineStr"/>
+      <c r="L189" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M189" s="17">
+        <f>J189-L189</f>
+        <v/>
+      </c>
+      <c r="N189" s="18">
+        <f>IF(J189=0,"",L189/J189)</f>
+        <v/>
+      </c>
+      <c r="O189" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 19:12:28</t>
+        </is>
+      </c>
+      <c r="B190" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C190" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D190" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E190" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F190" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeeff047</t>
+        </is>
+      </c>
+      <c r="G190" s="15" t="inlineStr">
+        <is>
+          <t>USDC vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H190" s="16" t="inlineStr"/>
+      <c r="I190" s="15" t="inlineStr">
+        <is>
+          <t>USDC 48,647.3916</t>
+        </is>
+      </c>
+      <c r="J190" s="17" t="n">
+        <v>48652.25680268027</v>
+      </c>
+      <c r="K190" s="15" t="inlineStr"/>
+      <c r="L190" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M190" s="17">
+        <f>J190-L190</f>
+        <v/>
+      </c>
+      <c r="N190" s="18">
+        <f>IF(J190=0,"",L190/J190)</f>
+        <v/>
+      </c>
+      <c r="O190" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 19:12:28</t>
+        </is>
+      </c>
+      <c r="B191" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C191" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D191" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E191" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F191" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G191" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H191" s="16" t="inlineStr"/>
+      <c r="I191" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J191" s="17" t="n">
+        <v>95907.28669653094</v>
+      </c>
+      <c r="K191" s="15" t="inlineStr"/>
+      <c r="L191" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M191" s="17">
+        <f>J191-L191</f>
+        <v/>
+      </c>
+      <c r="N191" s="18">
+        <f>IF(J191=0,"",L191/J191)</f>
+        <v/>
+      </c>
+      <c r="O191" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 19:12:28</t>
+        </is>
+      </c>
+      <c r="B192" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C192" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D192" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E192" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F192" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G192" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H192" s="16" t="inlineStr"/>
+      <c r="I192" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J192" s="17" t="n">
+        <v>34343.77163866379</v>
+      </c>
+      <c r="K192" s="15" t="inlineStr"/>
+      <c r="L192" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M192" s="17">
+        <f>J192-L192</f>
+        <v/>
+      </c>
+      <c r="N192" s="18">
+        <f>IF(J192=0,"",L192/J192)</f>
+        <v/>
+      </c>
+      <c r="O192" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 19:12:28</t>
+        </is>
+      </c>
+      <c r="B193" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C193" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D193" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E193" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F193" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G193" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H193" s="16" t="n">
+        <v>1.0418</v>
+      </c>
+      <c r="I193" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J193" s="17" t="n">
+        <v>269695.4896114625</v>
+      </c>
+      <c r="K193" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,014.6260</t>
+        </is>
+      </c>
+      <c r="L193" s="17" t="n">
+        <v>232979.6737821036</v>
+      </c>
+      <c r="M193" s="17">
+        <f>J193-L193</f>
+        <v/>
+      </c>
+      <c r="N193" s="18">
+        <f>IF(J193=0,"",L193/J193)</f>
+        <v/>
+      </c>
+      <c r="O193" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 19:12:28</t>
+        </is>
+      </c>
+      <c r="B194" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C194" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D194" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E194" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F194" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G194" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H194" s="16" t="inlineStr"/>
+      <c r="I194" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,503.8448</t>
+        </is>
+      </c>
+      <c r="J194" s="17" t="n">
+        <v>15501.51926213774</v>
+      </c>
+      <c r="K194" s="15" t="inlineStr"/>
+      <c r="L194" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M194" s="17">
+        <f>J194-L194</f>
+        <v/>
+      </c>
+      <c r="N194" s="18">
+        <f>IF(J194=0,"",L194/J194)</f>
+        <v/>
+      </c>
+      <c r="O194" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -12571,7 +13576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -13077,6 +14082,41 @@
         <v>1.0375</v>
       </c>
       <c r="I14" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 19:12:28</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="n">
+        <v>553114.9149874265</v>
+      </c>
+      <c r="D15" s="17" t="n">
+        <v>550499.2437944878</v>
+      </c>
+      <c r="E15" s="17" t="n">
+        <v>2478850.327388168</v>
+      </c>
+      <c r="F15" s="17" t="n">
+        <v>1928351.08359368</v>
+      </c>
+      <c r="G15" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="H15" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I15" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-28 21:23 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O179"/>
+  <dimension ref="A1:O194"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -12541,6 +12541,1011 @@
         <v/>
       </c>
       <c r="O179" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:23:42</t>
+        </is>
+      </c>
+      <c r="B180" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C180" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D180" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E180" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F180" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G180" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H180" s="16" t="n">
+        <v>1.0477</v>
+      </c>
+      <c r="I180" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J180" s="17" t="n">
+        <v>140890.1677259687</v>
+      </c>
+      <c r="K180" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,022.8377</t>
+        </is>
+      </c>
+      <c r="L180" s="17" t="n">
+        <v>121027.6786275086</v>
+      </c>
+      <c r="M180" s="17">
+        <f>J180-L180</f>
+        <v/>
+      </c>
+      <c r="N180" s="18">
+        <f>IF(J180=0,"",L180/J180)</f>
+        <v/>
+      </c>
+      <c r="O180" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:23:42</t>
+        </is>
+      </c>
+      <c r="B181" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C181" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D181" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E181" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F181" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G181" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H181" s="16" t="n">
+        <v>1.0451</v>
+      </c>
+      <c r="I181" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J181" s="17" t="n">
+        <v>328692.6042976156</v>
+      </c>
+      <c r="K181" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,372.4926</t>
+        </is>
+      </c>
+      <c r="L181" s="17" t="n">
+        <v>306403.0893439293</v>
+      </c>
+      <c r="M181" s="17">
+        <f>J181-L181</f>
+        <v/>
+      </c>
+      <c r="N181" s="18">
+        <f>IF(J181=0,"",L181/J181)</f>
+        <v/>
+      </c>
+      <c r="O181" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:23:42</t>
+        </is>
+      </c>
+      <c r="B182" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C182" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D182" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E182" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F182" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G182" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H182" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I182" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J182" s="17" t="n">
+        <v>385944.8325625386</v>
+      </c>
+      <c r="K182" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,587.4014</t>
+        </is>
+      </c>
+      <c r="L182" s="17" t="n">
+        <v>349622.3140069479</v>
+      </c>
+      <c r="M182" s="17">
+        <f>J182-L182</f>
+        <v/>
+      </c>
+      <c r="N182" s="18">
+        <f>IF(J182=0,"",L182/J182)</f>
+        <v/>
+      </c>
+      <c r="O182" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:23:42</t>
+        </is>
+      </c>
+      <c r="B183" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C183" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D183" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E183" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F183" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G183" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H183" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I183" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7826</t>
+        </is>
+      </c>
+      <c r="J183" s="17" t="n">
+        <v>77792.29965331552</v>
+      </c>
+      <c r="K183" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,022.6150; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L183" s="17" t="n">
+        <v>68025.4134193543</v>
+      </c>
+      <c r="M183" s="17">
+        <f>J183-L183</f>
+        <v/>
+      </c>
+      <c r="N183" s="18">
+        <f>IF(J183=0,"",L183/J183)</f>
+        <v/>
+      </c>
+      <c r="O183" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:23:42</t>
+        </is>
+      </c>
+      <c r="B184" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C184" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D184" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E184" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F184" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G184" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H184" s="16" t="n">
+        <v>1.1285</v>
+      </c>
+      <c r="I184" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J184" s="17" t="n">
+        <v>197083.7555060171</v>
+      </c>
+      <c r="K184" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,228.5848</t>
+        </is>
+      </c>
+      <c r="L184" s="17" t="n">
+        <v>150243.6091312141</v>
+      </c>
+      <c r="M184" s="17">
+        <f>J184-L184</f>
+        <v/>
+      </c>
+      <c r="N184" s="18">
+        <f>IF(J184=0,"",L184/J184)</f>
+        <v/>
+      </c>
+      <c r="O184" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:23:42</t>
+        </is>
+      </c>
+      <c r="B185" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C185" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D185" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E185" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F185" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G185" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H185" s="16" t="n">
+        <v>1.0528</v>
+      </c>
+      <c r="I185" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J185" s="17" t="n">
+        <v>186061.45173414</v>
+      </c>
+      <c r="K185" s="15" t="inlineStr">
+        <is>
+          <t>USDC 161,827.6712</t>
+        </is>
+      </c>
+      <c r="L185" s="17" t="n">
+        <v>161843.8556121311</v>
+      </c>
+      <c r="M185" s="17">
+        <f>J185-L185</f>
+        <v/>
+      </c>
+      <c r="N185" s="18">
+        <f>IF(J185=0,"",L185/J185)</f>
+        <v/>
+      </c>
+      <c r="O185" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:23:42</t>
+        </is>
+      </c>
+      <c r="B186" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C186" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D186" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E186" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F186" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G186" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H186" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I186" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J186" s="17" t="n">
+        <v>327526.9068972116</v>
+      </c>
+      <c r="K186" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L186" s="17" t="n">
+        <v>280201.6701739081</v>
+      </c>
+      <c r="M186" s="17">
+        <f>J186-L186</f>
+        <v/>
+      </c>
+      <c r="N186" s="18">
+        <f>IF(J186=0,"",L186/J186)</f>
+        <v/>
+      </c>
+      <c r="O186" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:23:42</t>
+        </is>
+      </c>
+      <c r="B187" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C187" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D187" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E187" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F187" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G187" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H187" s="16" t="n">
+        <v>1.1296</v>
+      </c>
+      <c r="I187" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J187" s="17" t="n">
+        <v>159940.3392339234</v>
+      </c>
+      <c r="K187" s="15" t="inlineStr">
+        <is>
+          <t>USDC 119,566.4850</t>
+        </is>
+      </c>
+      <c r="L187" s="17" t="n">
+        <v>119578.4428387121</v>
+      </c>
+      <c r="M187" s="17">
+        <f>J187-L187</f>
+        <v/>
+      </c>
+      <c r="N187" s="18">
+        <f>IF(J187=0,"",L187/J187)</f>
+        <v/>
+      </c>
+      <c r="O187" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:23:42</t>
+        </is>
+      </c>
+      <c r="B188" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C188" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D188" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E188" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F188" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G188" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H188" s="16" t="n">
+        <v>1.0575</v>
+      </c>
+      <c r="I188" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J188" s="17" t="n">
+        <v>160118.0676429287</v>
+      </c>
+      <c r="K188" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,514.6077</t>
+        </is>
+      </c>
+      <c r="L188" s="17" t="n">
+        <v>138500.756232042</v>
+      </c>
+      <c r="M188" s="17">
+        <f>J188-L188</f>
+        <v/>
+      </c>
+      <c r="N188" s="18">
+        <f>IF(J188=0,"",L188/J188)</f>
+        <v/>
+      </c>
+      <c r="O188" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:23:42</t>
+        </is>
+      </c>
+      <c r="B189" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C189" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D189" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E189" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F189" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeef003c</t>
+        </is>
+      </c>
+      <c r="G189" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H189" s="16" t="inlineStr"/>
+      <c r="I189" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,801.5319</t>
+        </is>
+      </c>
+      <c r="J189" s="17" t="n">
+        <v>50803.56397527656</v>
+      </c>
+      <c r="K189" s="15" t="inlineStr"/>
+      <c r="L189" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M189" s="17">
+        <f>J189-L189</f>
+        <v/>
+      </c>
+      <c r="N189" s="18">
+        <f>IF(J189=0,"",L189/J189)</f>
+        <v/>
+      </c>
+      <c r="O189" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:23:42</t>
+        </is>
+      </c>
+      <c r="B190" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C190" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D190" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E190" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F190" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeeff047</t>
+        </is>
+      </c>
+      <c r="G190" s="15" t="inlineStr">
+        <is>
+          <t>USDC vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H190" s="16" t="inlineStr"/>
+      <c r="I190" s="15" t="inlineStr">
+        <is>
+          <t>USDC 48,647.3916</t>
+        </is>
+      </c>
+      <c r="J190" s="17" t="n">
+        <v>48652.25680268027</v>
+      </c>
+      <c r="K190" s="15" t="inlineStr"/>
+      <c r="L190" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M190" s="17">
+        <f>J190-L190</f>
+        <v/>
+      </c>
+      <c r="N190" s="18">
+        <f>IF(J190=0,"",L190/J190)</f>
+        <v/>
+      </c>
+      <c r="O190" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:23:42</t>
+        </is>
+      </c>
+      <c r="B191" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C191" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D191" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E191" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F191" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G191" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H191" s="16" t="inlineStr"/>
+      <c r="I191" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J191" s="17" t="n">
+        <v>95894.71003258934</v>
+      </c>
+      <c r="K191" s="15" t="inlineStr"/>
+      <c r="L191" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M191" s="17">
+        <f>J191-L191</f>
+        <v/>
+      </c>
+      <c r="N191" s="18">
+        <f>IF(J191=0,"",L191/J191)</f>
+        <v/>
+      </c>
+      <c r="O191" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:23:42</t>
+        </is>
+      </c>
+      <c r="B192" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C192" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D192" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E192" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F192" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G192" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H192" s="16" t="inlineStr"/>
+      <c r="I192" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J192" s="17" t="n">
+        <v>34344.9049620861</v>
+      </c>
+      <c r="K192" s="15" t="inlineStr"/>
+      <c r="L192" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M192" s="17">
+        <f>J192-L192</f>
+        <v/>
+      </c>
+      <c r="N192" s="18">
+        <f>IF(J192=0,"",L192/J192)</f>
+        <v/>
+      </c>
+      <c r="O192" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:23:42</t>
+        </is>
+      </c>
+      <c r="B193" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C193" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D193" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E193" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F193" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G193" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H193" s="16" t="n">
+        <v>1.0415</v>
+      </c>
+      <c r="I193" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J193" s="17" t="n">
+        <v>269668.5200625014</v>
+      </c>
+      <c r="K193" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,014.6260</t>
+        </is>
+      </c>
+      <c r="L193" s="17" t="n">
+        <v>233023.946561039</v>
+      </c>
+      <c r="M193" s="17">
+        <f>J193-L193</f>
+        <v/>
+      </c>
+      <c r="N193" s="18">
+        <f>IF(J193=0,"",L193/J193)</f>
+        <v/>
+      </c>
+      <c r="O193" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:23:42</t>
+        </is>
+      </c>
+      <c r="B194" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C194" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D194" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E194" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F194" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G194" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H194" s="16" t="inlineStr"/>
+      <c r="I194" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,504.7434</t>
+        </is>
+      </c>
+      <c r="J194" s="17" t="n">
+        <v>15505.36354952781</v>
+      </c>
+      <c r="K194" s="15" t="inlineStr"/>
+      <c r="L194" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M194" s="17">
+        <f>J194-L194</f>
+        <v/>
+      </c>
+      <c r="N194" s="18">
+        <f>IF(J194=0,"",L194/J194)</f>
+        <v/>
+      </c>
+      <c r="O194" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -12571,7 +13576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -13077,6 +14082,41 @@
         <v>1.0375</v>
       </c>
       <c r="I14" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:23:42</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="n">
+        <v>553064.8934978675</v>
+      </c>
+      <c r="D15" s="17" t="n">
+        <v>550448.9686915346</v>
+      </c>
+      <c r="E15" s="17" t="n">
+        <v>2478919.744638321</v>
+      </c>
+      <c r="F15" s="17" t="n">
+        <v>1928470.775946786</v>
+      </c>
+      <c r="G15" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="H15" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I15" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-28 21:54 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O194"/>
+  <dimension ref="A1:O209"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -13546,6 +13546,1011 @@
         <v/>
       </c>
       <c r="O194" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:54:03</t>
+        </is>
+      </c>
+      <c r="B195" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C195" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D195" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E195" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F195" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G195" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H195" s="16" t="n">
+        <v>1.0479</v>
+      </c>
+      <c r="I195" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J195" s="17" t="n">
+        <v>140890.5803555972</v>
+      </c>
+      <c r="K195" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,022.8377</t>
+        </is>
+      </c>
+      <c r="L195" s="17" t="n">
+        <v>121009.5252018514</v>
+      </c>
+      <c r="M195" s="17">
+        <f>J195-L195</f>
+        <v/>
+      </c>
+      <c r="N195" s="18">
+        <f>IF(J195=0,"",L195/J195)</f>
+        <v/>
+      </c>
+      <c r="O195" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:54:03</t>
+        </is>
+      </c>
+      <c r="B196" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C196" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D196" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E196" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F196" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G196" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H196" s="16" t="n">
+        <v>1.0451</v>
+      </c>
+      <c r="I196" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J196" s="17" t="n">
+        <v>328693.2885731984</v>
+      </c>
+      <c r="K196" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,372.4926</t>
+        </is>
+      </c>
+      <c r="L196" s="17" t="n">
+        <v>306402.9640295008</v>
+      </c>
+      <c r="M196" s="17">
+        <f>J196-L196</f>
+        <v/>
+      </c>
+      <c r="N196" s="18">
+        <f>IF(J196=0,"",L196/J196)</f>
+        <v/>
+      </c>
+      <c r="O196" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:54:03</t>
+        </is>
+      </c>
+      <c r="B197" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C197" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D197" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E197" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F197" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G197" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H197" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I197" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J197" s="17" t="n">
+        <v>385907.3145752501</v>
+      </c>
+      <c r="K197" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,587.4014</t>
+        </is>
+      </c>
+      <c r="L197" s="17" t="n">
+        <v>349622.171016482</v>
+      </c>
+      <c r="M197" s="17">
+        <f>J197-L197</f>
+        <v/>
+      </c>
+      <c r="N197" s="18">
+        <f>IF(J197=0,"",L197/J197)</f>
+        <v/>
+      </c>
+      <c r="O197" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:54:03</t>
+        </is>
+      </c>
+      <c r="B198" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C198" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D198" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E198" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F198" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G198" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H198" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I198" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7826</t>
+        </is>
+      </c>
+      <c r="J198" s="17" t="n">
+        <v>77820.23676692478</v>
+      </c>
+      <c r="K198" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,022.6150; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L198" s="17" t="n">
+        <v>68017.25069780376</v>
+      </c>
+      <c r="M198" s="17">
+        <f>J198-L198</f>
+        <v/>
+      </c>
+      <c r="N198" s="18">
+        <f>IF(J198=0,"",L198/J198)</f>
+        <v/>
+      </c>
+      <c r="O198" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:54:03</t>
+        </is>
+      </c>
+      <c r="B199" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C199" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D199" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E199" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F199" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G199" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H199" s="16" t="n">
+        <v>1.1285</v>
+      </c>
+      <c r="I199" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J199" s="17" t="n">
+        <v>197085.8646484622</v>
+      </c>
+      <c r="K199" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,228.5848</t>
+        </is>
+      </c>
+      <c r="L199" s="17" t="n">
+        <v>150228.584770301</v>
+      </c>
+      <c r="M199" s="17">
+        <f>J199-L199</f>
+        <v/>
+      </c>
+      <c r="N199" s="18">
+        <f>IF(J199=0,"",L199/J199)</f>
+        <v/>
+      </c>
+      <c r="O199" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:54:03</t>
+        </is>
+      </c>
+      <c r="B200" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C200" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D200" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E200" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F200" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G200" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H200" s="16" t="n">
+        <v>1.0528</v>
+      </c>
+      <c r="I200" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J200" s="17" t="n">
+        <v>186062.5474745291</v>
+      </c>
+      <c r="K200" s="15" t="inlineStr">
+        <is>
+          <t>USDC 161,827.6712</t>
+        </is>
+      </c>
+      <c r="L200" s="17" t="n">
+        <v>161827.6712265699</v>
+      </c>
+      <c r="M200" s="17">
+        <f>J200-L200</f>
+        <v/>
+      </c>
+      <c r="N200" s="18">
+        <f>IF(J200=0,"",L200/J200)</f>
+        <v/>
+      </c>
+      <c r="O200" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:54:03</t>
+        </is>
+      </c>
+      <c r="B201" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C201" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D201" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E201" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F201" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G201" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H201" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I201" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J201" s="17" t="n">
+        <v>327501.2343689038</v>
+      </c>
+      <c r="K201" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L201" s="17" t="n">
+        <v>280176.6788984244</v>
+      </c>
+      <c r="M201" s="17">
+        <f>J201-L201</f>
+        <v/>
+      </c>
+      <c r="N201" s="18">
+        <f>IF(J201=0,"",L201/J201)</f>
+        <v/>
+      </c>
+      <c r="O201" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:54:03</t>
+        </is>
+      </c>
+      <c r="B202" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C202" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D202" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E202" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F202" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G202" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H202" s="16" t="n">
+        <v>1.1296</v>
+      </c>
+      <c r="I202" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J202" s="17" t="n">
+        <v>159940.3392339234</v>
+      </c>
+      <c r="K202" s="15" t="inlineStr">
+        <is>
+          <t>USDC 119,566.4850</t>
+        </is>
+      </c>
+      <c r="L202" s="17" t="n">
+        <v>119566.4849944282</v>
+      </c>
+      <c r="M202" s="17">
+        <f>J202-L202</f>
+        <v/>
+      </c>
+      <c r="N202" s="18">
+        <f>IF(J202=0,"",L202/J202)</f>
+        <v/>
+      </c>
+      <c r="O202" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:54:03</t>
+        </is>
+      </c>
+      <c r="B203" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C203" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D203" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E203" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F203" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G203" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H203" s="16" t="n">
+        <v>1.0575</v>
+      </c>
+      <c r="I203" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J203" s="17" t="n">
+        <v>160102.5024452122</v>
+      </c>
+      <c r="K203" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,514.6077</t>
+        </is>
+      </c>
+      <c r="L203" s="17" t="n">
+        <v>138500.756232042</v>
+      </c>
+      <c r="M203" s="17">
+        <f>J203-L203</f>
+        <v/>
+      </c>
+      <c r="N203" s="18">
+        <f>IF(J203=0,"",L203/J203)</f>
+        <v/>
+      </c>
+      <c r="O203" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:54:03</t>
+        </is>
+      </c>
+      <c r="B204" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C204" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D204" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E204" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F204" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeef003c</t>
+        </is>
+      </c>
+      <c r="G204" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H204" s="16" t="inlineStr"/>
+      <c r="I204" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,801.5319</t>
+        </is>
+      </c>
+      <c r="J204" s="17" t="n">
+        <v>50795.94374548946</v>
+      </c>
+      <c r="K204" s="15" t="inlineStr"/>
+      <c r="L204" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M204" s="17">
+        <f>J204-L204</f>
+        <v/>
+      </c>
+      <c r="N204" s="18">
+        <f>IF(J204=0,"",L204/J204)</f>
+        <v/>
+      </c>
+      <c r="O204" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:54:03</t>
+        </is>
+      </c>
+      <c r="B205" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C205" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D205" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E205" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F205" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeeff047</t>
+        </is>
+      </c>
+      <c r="G205" s="15" t="inlineStr">
+        <is>
+          <t>USDC vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H205" s="16" t="inlineStr"/>
+      <c r="I205" s="15" t="inlineStr">
+        <is>
+          <t>USDC 48,647.3916</t>
+        </is>
+      </c>
+      <c r="J205" s="17" t="n">
+        <v>48647.391577</v>
+      </c>
+      <c r="K205" s="15" t="inlineStr"/>
+      <c r="L205" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M205" s="17">
+        <f>J205-L205</f>
+        <v/>
+      </c>
+      <c r="N205" s="18">
+        <f>IF(J205=0,"",L205/J205)</f>
+        <v/>
+      </c>
+      <c r="O205" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:54:03</t>
+        </is>
+      </c>
+      <c r="B206" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C206" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D206" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E206" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F206" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G206" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H206" s="16" t="inlineStr"/>
+      <c r="I206" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J206" s="17" t="n">
+        <v>95894.71003258934</v>
+      </c>
+      <c r="K206" s="15" t="inlineStr"/>
+      <c r="L206" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M206" s="17">
+        <f>J206-L206</f>
+        <v/>
+      </c>
+      <c r="N206" s="18">
+        <f>IF(J206=0,"",L206/J206)</f>
+        <v/>
+      </c>
+      <c r="O206" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:54:03</t>
+        </is>
+      </c>
+      <c r="B207" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C207" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D207" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E207" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F207" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G207" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H207" s="16" t="inlineStr"/>
+      <c r="I207" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J207" s="17" t="n">
+        <v>34345.51860602789</v>
+      </c>
+      <c r="K207" s="15" t="inlineStr"/>
+      <c r="L207" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M207" s="17">
+        <f>J207-L207</f>
+        <v/>
+      </c>
+      <c r="N207" s="18">
+        <f>IF(J207=0,"",L207/J207)</f>
+        <v/>
+      </c>
+      <c r="O207" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:54:03</t>
+        </is>
+      </c>
+      <c r="B208" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C208" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D208" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E208" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F208" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G208" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H208" s="16" t="n">
+        <v>1.0417</v>
+      </c>
+      <c r="I208" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J208" s="17" t="n">
+        <v>269668.5200625014</v>
+      </c>
+      <c r="K208" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,014.6260</t>
+        </is>
+      </c>
+      <c r="L208" s="17" t="n">
+        <v>232995.9848059219</v>
+      </c>
+      <c r="M208" s="17">
+        <f>J208-L208</f>
+        <v/>
+      </c>
+      <c r="N208" s="18">
+        <f>IF(J208=0,"",L208/J208)</f>
+        <v/>
+      </c>
+      <c r="O208" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:54:03</t>
+        </is>
+      </c>
+      <c r="B209" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C209" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D209" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E209" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F209" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G209" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H209" s="16" t="inlineStr"/>
+      <c r="I209" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,504.9471</t>
+        </is>
+      </c>
+      <c r="J209" s="17" t="n">
+        <v>15503.70667818198</v>
+      </c>
+      <c r="K209" s="15" t="inlineStr"/>
+      <c r="L209" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M209" s="17">
+        <f>J209-L209</f>
+        <v/>
+      </c>
+      <c r="N209" s="18">
+        <f>IF(J209=0,"",L209/J209)</f>
+        <v/>
+      </c>
+      <c r="O209" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -13576,7 +14581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -14117,6 +15122,41 @@
         <v>1.0375</v>
       </c>
       <c r="I15" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 21:54:03</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="n">
+        <v>553127.3843637337</v>
+      </c>
+      <c r="D16" s="17" t="n">
+        <v>550511.6272704662</v>
+      </c>
+      <c r="E16" s="17" t="n">
+        <v>2478859.699143792</v>
+      </c>
+      <c r="F16" s="17" t="n">
+        <v>1928348.071873325</v>
+      </c>
+      <c r="G16" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="H16" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I16" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-28 22:41 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O194"/>
+  <dimension ref="A1:O209"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -13546,6 +13546,1011 @@
         <v/>
       </c>
       <c r="O194" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 22:40:57</t>
+        </is>
+      </c>
+      <c r="B195" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C195" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D195" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E195" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F195" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G195" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H195" s="16" t="n">
+        <v>1.0479</v>
+      </c>
+      <c r="I195" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J195" s="17" t="n">
+        <v>140891.2830733743</v>
+      </c>
+      <c r="K195" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,022.8377</t>
+        </is>
+      </c>
+      <c r="L195" s="17" t="n">
+        <v>121008.3149734743</v>
+      </c>
+      <c r="M195" s="17">
+        <f>J195-L195</f>
+        <v/>
+      </c>
+      <c r="N195" s="18">
+        <f>IF(J195=0,"",L195/J195)</f>
+        <v/>
+      </c>
+      <c r="O195" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 22:40:57</t>
+        </is>
+      </c>
+      <c r="B196" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C196" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D196" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E196" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F196" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G196" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H196" s="16" t="n">
+        <v>1.0451</v>
+      </c>
+      <c r="I196" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J196" s="17" t="n">
+        <v>328694.0063463195</v>
+      </c>
+      <c r="K196" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,372.4926</t>
+        </is>
+      </c>
+      <c r="L196" s="17" t="n">
+        <v>306433.619412939</v>
+      </c>
+      <c r="M196" s="17">
+        <f>J196-L196</f>
+        <v/>
+      </c>
+      <c r="N196" s="18">
+        <f>IF(J196=0,"",L196/J196)</f>
+        <v/>
+      </c>
+      <c r="O196" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 22:40:57</t>
+        </is>
+      </c>
+      <c r="B197" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C197" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D197" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E197" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F197" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G197" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H197" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I197" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J197" s="17" t="n">
+        <v>385948.2162738222</v>
+      </c>
+      <c r="K197" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,587.4014</t>
+        </is>
+      </c>
+      <c r="L197" s="17" t="n">
+        <v>349657.1504486979</v>
+      </c>
+      <c r="M197" s="17">
+        <f>J197-L197</f>
+        <v/>
+      </c>
+      <c r="N197" s="18">
+        <f>IF(J197=0,"",L197/J197)</f>
+        <v/>
+      </c>
+      <c r="O197" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 22:40:57</t>
+        </is>
+      </c>
+      <c r="B198" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C198" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D198" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E198" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F198" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G198" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H198" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I198" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7826</t>
+        </is>
+      </c>
+      <c r="J198" s="17" t="n">
+        <v>77799.95475562754</v>
+      </c>
+      <c r="K198" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,022.6150; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L198" s="17" t="n">
+        <v>68014.52979320564</v>
+      </c>
+      <c r="M198" s="17">
+        <f>J198-L198</f>
+        <v/>
+      </c>
+      <c r="N198" s="18">
+        <f>IF(J198=0,"",L198/J198)</f>
+        <v/>
+      </c>
+      <c r="O198" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 22:40:57</t>
+        </is>
+      </c>
+      <c r="B199" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C199" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D199" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E199" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F199" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G199" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H199" s="16" t="n">
+        <v>1.1285</v>
+      </c>
+      <c r="I199" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J199" s="17" t="n">
+        <v>197085.4745971195</v>
+      </c>
+      <c r="K199" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,228.5848</t>
+        </is>
+      </c>
+      <c r="L199" s="17" t="n">
+        <v>150228.584770301</v>
+      </c>
+      <c r="M199" s="17">
+        <f>J199-L199</f>
+        <v/>
+      </c>
+      <c r="N199" s="18">
+        <f>IF(J199=0,"",L199/J199)</f>
+        <v/>
+      </c>
+      <c r="O199" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 22:40:57</t>
+        </is>
+      </c>
+      <c r="B200" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C200" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D200" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E200" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F200" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G200" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H200" s="16" t="n">
+        <v>1.0528</v>
+      </c>
+      <c r="I200" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J200" s="17" t="n">
+        <v>186063.9830996562</v>
+      </c>
+      <c r="K200" s="15" t="inlineStr">
+        <is>
+          <t>USDC 161,827.6712</t>
+        </is>
+      </c>
+      <c r="L200" s="17" t="n">
+        <v>161827.6712265699</v>
+      </c>
+      <c r="M200" s="17">
+        <f>J200-L200</f>
+        <v/>
+      </c>
+      <c r="N200" s="18">
+        <f>IF(J200=0,"",L200/J200)</f>
+        <v/>
+      </c>
+      <c r="O200" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 22:40:57</t>
+        </is>
+      </c>
+      <c r="B201" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C201" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D201" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E201" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F201" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G201" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H201" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I201" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J201" s="17" t="n">
+        <v>327500.5275613879</v>
+      </c>
+      <c r="K201" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L201" s="17" t="n">
+        <v>280204.7156862481</v>
+      </c>
+      <c r="M201" s="17">
+        <f>J201-L201</f>
+        <v/>
+      </c>
+      <c r="N201" s="18">
+        <f>IF(J201=0,"",L201/J201)</f>
+        <v/>
+      </c>
+      <c r="O201" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 22:40:57</t>
+        </is>
+      </c>
+      <c r="B202" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C202" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D202" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E202" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F202" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G202" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H202" s="16" t="n">
+        <v>1.1296</v>
+      </c>
+      <c r="I202" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J202" s="17" t="n">
+        <v>159940.3392339234</v>
+      </c>
+      <c r="K202" s="15" t="inlineStr">
+        <is>
+          <t>USDC 119,566.4850</t>
+        </is>
+      </c>
+      <c r="L202" s="17" t="n">
+        <v>119566.4849944282</v>
+      </c>
+      <c r="M202" s="17">
+        <f>J202-L202</f>
+        <v/>
+      </c>
+      <c r="N202" s="18">
+        <f>IF(J202=0,"",L202/J202)</f>
+        <v/>
+      </c>
+      <c r="O202" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 22:40:57</t>
+        </is>
+      </c>
+      <c r="B203" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C203" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D203" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E203" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F203" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G203" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H203" s="16" t="n">
+        <v>1.0575</v>
+      </c>
+      <c r="I203" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J203" s="17" t="n">
+        <v>160119.4714531795</v>
+      </c>
+      <c r="K203" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,514.6077</t>
+        </is>
+      </c>
+      <c r="L203" s="17" t="n">
+        <v>138500.756232042</v>
+      </c>
+      <c r="M203" s="17">
+        <f>J203-L203</f>
+        <v/>
+      </c>
+      <c r="N203" s="18">
+        <f>IF(J203=0,"",L203/J203)</f>
+        <v/>
+      </c>
+      <c r="O203" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 22:40:57</t>
+        </is>
+      </c>
+      <c r="B204" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C204" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D204" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E204" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F204" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeef003c</t>
+        </is>
+      </c>
+      <c r="G204" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H204" s="16" t="inlineStr"/>
+      <c r="I204" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,801.5319</t>
+        </is>
+      </c>
+      <c r="J204" s="17" t="n">
+        <v>50795.43573017032</v>
+      </c>
+      <c r="K204" s="15" t="inlineStr"/>
+      <c r="L204" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M204" s="17">
+        <f>J204-L204</f>
+        <v/>
+      </c>
+      <c r="N204" s="18">
+        <f>IF(J204=0,"",L204/J204)</f>
+        <v/>
+      </c>
+      <c r="O204" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 22:40:57</t>
+        </is>
+      </c>
+      <c r="B205" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C205" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D205" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E205" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F205" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeeff047</t>
+        </is>
+      </c>
+      <c r="G205" s="15" t="inlineStr">
+        <is>
+          <t>USDC vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H205" s="16" t="inlineStr"/>
+      <c r="I205" s="15" t="inlineStr">
+        <is>
+          <t>USDC 48,647.3916</t>
+        </is>
+      </c>
+      <c r="J205" s="17" t="n">
+        <v>48647.391577</v>
+      </c>
+      <c r="K205" s="15" t="inlineStr"/>
+      <c r="L205" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M205" s="17">
+        <f>J205-L205</f>
+        <v/>
+      </c>
+      <c r="N205" s="18">
+        <f>IF(J205=0,"",L205/J205)</f>
+        <v/>
+      </c>
+      <c r="O205" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 22:40:57</t>
+        </is>
+      </c>
+      <c r="B206" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C206" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D206" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E206" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F206" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G206" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H206" s="16" t="inlineStr"/>
+      <c r="I206" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J206" s="17" t="n">
+        <v>95894.71003258934</v>
+      </c>
+      <c r="K206" s="15" t="inlineStr"/>
+      <c r="L206" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M206" s="17">
+        <f>J206-L206</f>
+        <v/>
+      </c>
+      <c r="N206" s="18">
+        <f>IF(J206=0,"",L206/J206)</f>
+        <v/>
+      </c>
+      <c r="O206" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 22:40:57</t>
+        </is>
+      </c>
+      <c r="B207" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C207" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D207" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E207" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F207" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G207" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H207" s="16" t="inlineStr"/>
+      <c r="I207" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J207" s="17" t="n">
+        <v>34345.98566635666</v>
+      </c>
+      <c r="K207" s="15" t="inlineStr"/>
+      <c r="L207" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M207" s="17">
+        <f>J207-L207</f>
+        <v/>
+      </c>
+      <c r="N207" s="18">
+        <f>IF(J207=0,"",L207/J207)</f>
+        <v/>
+      </c>
+      <c r="O207" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 22:40:57</t>
+        </is>
+      </c>
+      <c r="B208" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C208" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D208" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E208" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F208" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G208" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H208" s="16" t="n">
+        <v>1.0417</v>
+      </c>
+      <c r="I208" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J208" s="17" t="n">
+        <v>269668.5200625014</v>
+      </c>
+      <c r="K208" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,014.6260</t>
+        </is>
+      </c>
+      <c r="L208" s="17" t="n">
+        <v>232986.6642208829</v>
+      </c>
+      <c r="M208" s="17">
+        <f>J208-L208</f>
+        <v/>
+      </c>
+      <c r="N208" s="18">
+        <f>IF(J208=0,"",L208/J208)</f>
+        <v/>
+      </c>
+      <c r="O208" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 22:40:57</t>
+        </is>
+      </c>
+      <c r="B209" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C209" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D209" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E209" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F209" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G209" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H209" s="16" t="inlineStr"/>
+      <c r="I209" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,505.1502</t>
+        </is>
+      </c>
+      <c r="J209" s="17" t="n">
+        <v>15503.28960857206</v>
+      </c>
+      <c r="K209" s="15" t="inlineStr"/>
+      <c r="L209" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M209" s="17">
+        <f>J209-L209</f>
+        <v/>
+      </c>
+      <c r="N209" s="18">
+        <f>IF(J209=0,"",L209/J209)</f>
+        <v/>
+      </c>
+      <c r="O209" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -13576,7 +14581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -14117,6 +15122,41 @@
         <v>1.0375</v>
       </c>
       <c r="I15" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 22:40:57</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="n">
+        <v>553085.7774437794</v>
+      </c>
+      <c r="D16" s="17" t="n">
+        <v>550470.0973128111</v>
+      </c>
+      <c r="E16" s="17" t="n">
+        <v>2478898.5890716</v>
+      </c>
+      <c r="F16" s="17" t="n">
+        <v>1928428.491758789</v>
+      </c>
+      <c r="G16" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="H16" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I16" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-28 23:41 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O209"/>
+  <dimension ref="A1:O224"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -14551,6 +14551,1011 @@
         <v/>
       </c>
       <c r="O209" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 23:41:01</t>
+        </is>
+      </c>
+      <c r="B210" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C210" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D210" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E210" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F210" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G210" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H210" s="16" t="n">
+        <v>1.0481</v>
+      </c>
+      <c r="I210" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J210" s="17" t="n">
+        <v>140891.7013707673</v>
+      </c>
+      <c r="K210" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,022.8377</t>
+        </is>
+      </c>
+      <c r="L210" s="17" t="n">
+        <v>120984.1104059315</v>
+      </c>
+      <c r="M210" s="17">
+        <f>J210-L210</f>
+        <v/>
+      </c>
+      <c r="N210" s="18">
+        <f>IF(J210=0,"",L210/J210)</f>
+        <v/>
+      </c>
+      <c r="O210" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 23:41:01</t>
+        </is>
+      </c>
+      <c r="B211" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C211" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D211" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E211" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F211" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G211" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H211" s="16" t="n">
+        <v>1.0451</v>
+      </c>
+      <c r="I211" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J211" s="17" t="n">
+        <v>328695.4610379857</v>
+      </c>
+      <c r="K211" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,372.4926</t>
+        </is>
+      </c>
+      <c r="L211" s="17" t="n">
+        <v>306433.6395884262</v>
+      </c>
+      <c r="M211" s="17">
+        <f>J211-L211</f>
+        <v/>
+      </c>
+      <c r="N211" s="18">
+        <f>IF(J211=0,"",L211/J211)</f>
+        <v/>
+      </c>
+      <c r="O211" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 23:41:01</t>
+        </is>
+      </c>
+      <c r="B212" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C212" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D212" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E212" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F212" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G212" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H212" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I212" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J212" s="17" t="n">
+        <v>385911.9203470302</v>
+      </c>
+      <c r="K212" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,587.4014</t>
+        </is>
+      </c>
+      <c r="L212" s="17" t="n">
+        <v>349657.1734700078</v>
+      </c>
+      <c r="M212" s="17">
+        <f>J212-L212</f>
+        <v/>
+      </c>
+      <c r="N212" s="18">
+        <f>IF(J212=0,"",L212/J212)</f>
+        <v/>
+      </c>
+      <c r="O212" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 23:41:01</t>
+        </is>
+      </c>
+      <c r="B213" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C213" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D213" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E213" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F213" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G213" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H213" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I213" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7826</t>
+        </is>
+      </c>
+      <c r="J213" s="17" t="n">
+        <v>77789.10192055572</v>
+      </c>
+      <c r="K213" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,022.6150; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L213" s="17" t="n">
+        <v>68000.92527797121</v>
+      </c>
+      <c r="M213" s="17">
+        <f>J213-L213</f>
+        <v/>
+      </c>
+      <c r="N213" s="18">
+        <f>IF(J213=0,"",L213/J213)</f>
+        <v/>
+      </c>
+      <c r="O213" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 23:41:01</t>
+        </is>
+      </c>
+      <c r="B214" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C214" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D214" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E214" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F214" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G214" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H214" s="16" t="n">
+        <v>1.1285</v>
+      </c>
+      <c r="I214" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J214" s="17" t="n">
+        <v>197087.958589618</v>
+      </c>
+      <c r="K214" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,228.5848</t>
+        </is>
+      </c>
+      <c r="L214" s="17" t="n">
+        <v>150243.6091312141</v>
+      </c>
+      <c r="M214" s="17">
+        <f>J214-L214</f>
+        <v/>
+      </c>
+      <c r="N214" s="18">
+        <f>IF(J214=0,"",L214/J214)</f>
+        <v/>
+      </c>
+      <c r="O214" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 23:41:01</t>
+        </is>
+      </c>
+      <c r="B215" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C215" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D215" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E215" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F215" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G215" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H215" s="16" t="n">
+        <v>1.0528</v>
+      </c>
+      <c r="I215" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J215" s="17" t="n">
+        <v>186065.1898534056</v>
+      </c>
+      <c r="K215" s="15" t="inlineStr">
+        <is>
+          <t>USDC 161,827.6712</t>
+        </is>
+      </c>
+      <c r="L215" s="17" t="n">
+        <v>161843.8556121311</v>
+      </c>
+      <c r="M215" s="17">
+        <f>J215-L215</f>
+        <v/>
+      </c>
+      <c r="N215" s="18">
+        <f>IF(J215=0,"",L215/J215)</f>
+        <v/>
+      </c>
+      <c r="O215" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 23:41:01</t>
+        </is>
+      </c>
+      <c r="B216" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C216" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D216" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E216" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F216" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G216" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H216" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I216" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J216" s="17" t="n">
+        <v>327529.809485435</v>
+      </c>
+      <c r="K216" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L216" s="17" t="n">
+        <v>280204.706780643</v>
+      </c>
+      <c r="M216" s="17">
+        <f>J216-L216</f>
+        <v/>
+      </c>
+      <c r="N216" s="18">
+        <f>IF(J216=0,"",L216/J216)</f>
+        <v/>
+      </c>
+      <c r="O216" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 23:41:01</t>
+        </is>
+      </c>
+      <c r="B217" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C217" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D217" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E217" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F217" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G217" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H217" s="16" t="n">
+        <v>1.1296</v>
+      </c>
+      <c r="I217" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J217" s="17" t="n">
+        <v>159924.3452</v>
+      </c>
+      <c r="K217" s="15" t="inlineStr">
+        <is>
+          <t>USDC 119,566.4850</t>
+        </is>
+      </c>
+      <c r="L217" s="17" t="n">
+        <v>119578.4428387121</v>
+      </c>
+      <c r="M217" s="17">
+        <f>J217-L217</f>
+        <v/>
+      </c>
+      <c r="N217" s="18">
+        <f>IF(J217=0,"",L217/J217)</f>
+        <v/>
+      </c>
+      <c r="O217" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 23:41:01</t>
+        </is>
+      </c>
+      <c r="B218" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C218" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D218" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E218" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F218" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G218" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H218" s="16" t="n">
+        <v>1.0575</v>
+      </c>
+      <c r="I218" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J218" s="17" t="n">
+        <v>160104.4132552949</v>
+      </c>
+      <c r="K218" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,514.6077</t>
+        </is>
+      </c>
+      <c r="L218" s="17" t="n">
+        <v>138514.6076928112</v>
+      </c>
+      <c r="M218" s="17">
+        <f>J218-L218</f>
+        <v/>
+      </c>
+      <c r="N218" s="18">
+        <f>IF(J218=0,"",L218/J218)</f>
+        <v/>
+      </c>
+      <c r="O218" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 23:41:01</t>
+        </is>
+      </c>
+      <c r="B219" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C219" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D219" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E219" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F219" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeef003c</t>
+        </is>
+      </c>
+      <c r="G219" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H219" s="16" t="inlineStr"/>
+      <c r="I219" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,801.5319</t>
+        </is>
+      </c>
+      <c r="J219" s="17" t="n">
+        <v>50785.27542378752</v>
+      </c>
+      <c r="K219" s="15" t="inlineStr"/>
+      <c r="L219" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M219" s="17">
+        <f>J219-L219</f>
+        <v/>
+      </c>
+      <c r="N219" s="18">
+        <f>IF(J219=0,"",L219/J219)</f>
+        <v/>
+      </c>
+      <c r="O219" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 23:41:01</t>
+        </is>
+      </c>
+      <c r="B220" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C220" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D220" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E220" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F220" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeeff047</t>
+        </is>
+      </c>
+      <c r="G220" s="15" t="inlineStr">
+        <is>
+          <t>USDC vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H220" s="16" t="inlineStr"/>
+      <c r="I220" s="15" t="inlineStr">
+        <is>
+          <t>USDC 48,647.3916</t>
+        </is>
+      </c>
+      <c r="J220" s="17" t="n">
+        <v>48652.25680268027</v>
+      </c>
+      <c r="K220" s="15" t="inlineStr"/>
+      <c r="L220" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M220" s="17">
+        <f>J220-L220</f>
+        <v/>
+      </c>
+      <c r="N220" s="18">
+        <f>IF(J220=0,"",L220/J220)</f>
+        <v/>
+      </c>
+      <c r="O220" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 23:41:01</t>
+        </is>
+      </c>
+      <c r="B221" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C221" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D221" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E221" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F221" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G221" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H221" s="16" t="inlineStr"/>
+      <c r="I221" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J221" s="17" t="n">
+        <v>95894.57893567815</v>
+      </c>
+      <c r="K221" s="15" t="inlineStr"/>
+      <c r="L221" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M221" s="17">
+        <f>J221-L221</f>
+        <v/>
+      </c>
+      <c r="N221" s="18">
+        <f>IF(J221=0,"",L221/J221)</f>
+        <v/>
+      </c>
+      <c r="O221" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 23:41:01</t>
+        </is>
+      </c>
+      <c r="B222" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C222" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D222" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E222" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F222" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G222" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H222" s="16" t="inlineStr"/>
+      <c r="I222" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J222" s="17" t="n">
+        <v>34346.44178608892</v>
+      </c>
+      <c r="K222" s="15" t="inlineStr"/>
+      <c r="L222" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M222" s="17">
+        <f>J222-L222</f>
+        <v/>
+      </c>
+      <c r="N222" s="18">
+        <f>IF(J222=0,"",L222/J222)</f>
+        <v/>
+      </c>
+      <c r="O222" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 23:41:01</t>
+        </is>
+      </c>
+      <c r="B223" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C223" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D223" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E223" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F223" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G223" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H223" s="16" t="n">
+        <v>1.0425</v>
+      </c>
+      <c r="I223" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J223" s="17" t="n">
+        <v>269822.0475770817</v>
+      </c>
+      <c r="K223" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,014.6260</t>
+        </is>
+      </c>
+      <c r="L223" s="17" t="n">
+        <v>232940.0612956877</v>
+      </c>
+      <c r="M223" s="17">
+        <f>J223-L223</f>
+        <v/>
+      </c>
+      <c r="N223" s="18">
+        <f>IF(J223=0,"",L223/J223)</f>
+        <v/>
+      </c>
+      <c r="O223" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 23:41:01</t>
+        </is>
+      </c>
+      <c r="B224" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C224" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D224" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E224" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F224" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G224" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H224" s="16" t="inlineStr"/>
+      <c r="I224" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,505.5564</t>
+        </is>
+      </c>
+      <c r="J224" s="17" t="n">
+        <v>15500.59464154897</v>
+      </c>
+      <c r="K224" s="15" t="inlineStr"/>
+      <c r="L224" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M224" s="17">
+        <f>J224-L224</f>
+        <v/>
+      </c>
+      <c r="N224" s="18">
+        <f>IF(J224=0,"",L224/J224)</f>
+        <v/>
+      </c>
+      <c r="O224" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -14581,7 +15586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -15157,6 +16162,41 @@
         <v>1.0375</v>
       </c>
       <c r="I16" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-28 23:41:01</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="n">
+        <v>553215.8988364545</v>
+      </c>
+      <c r="D17" s="17" t="n">
+        <v>550599.9641334221</v>
+      </c>
+      <c r="E17" s="17" t="n">
+        <v>2479001.096226958</v>
+      </c>
+      <c r="F17" s="17" t="n">
+        <v>1928401.132093536</v>
+      </c>
+      <c r="G17" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="H17" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I17" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 00:11 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O224"/>
+  <dimension ref="A1:O239"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -15556,6 +15556,1011 @@
         <v/>
       </c>
       <c r="O224" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:11:08</t>
+        </is>
+      </c>
+      <c r="B225" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C225" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D225" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E225" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F225" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G225" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H225" s="16" t="n">
+        <v>1.048</v>
+      </c>
+      <c r="I225" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J225" s="17" t="n">
+        <v>140878.0331619084</v>
+      </c>
+      <c r="K225" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,022.8377</t>
+        </is>
+      </c>
+      <c r="L225" s="17" t="n">
+        <v>120982.9001775544</v>
+      </c>
+      <c r="M225" s="17">
+        <f>J225-L225</f>
+        <v/>
+      </c>
+      <c r="N225" s="18">
+        <f>IF(J225=0,"",L225/J225)</f>
+        <v/>
+      </c>
+      <c r="O225" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:11:08</t>
+        </is>
+      </c>
+      <c r="B226" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C226" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D226" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E226" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F226" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G226" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H226" s="16" t="n">
+        <v>1.0451</v>
+      </c>
+      <c r="I226" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J226" s="17" t="n">
+        <v>328696.1548898968</v>
+      </c>
+      <c r="K226" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,372.4926</t>
+        </is>
+      </c>
+      <c r="L226" s="17" t="n">
+        <v>306433.6393306822</v>
+      </c>
+      <c r="M226" s="17">
+        <f>J226-L226</f>
+        <v/>
+      </c>
+      <c r="N226" s="18">
+        <f>IF(J226=0,"",L226/J226)</f>
+        <v/>
+      </c>
+      <c r="O226" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:11:08</t>
+        </is>
+      </c>
+      <c r="B227" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C227" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D227" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E227" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F227" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G227" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H227" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I227" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J227" s="17" t="n">
+        <v>385913.0279260208</v>
+      </c>
+      <c r="K227" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,587.4014</t>
+        </is>
+      </c>
+      <c r="L227" s="17" t="n">
+        <v>349657.1731759082</v>
+      </c>
+      <c r="M227" s="17">
+        <f>J227-L227</f>
+        <v/>
+      </c>
+      <c r="N227" s="18">
+        <f>IF(J227=0,"",L227/J227)</f>
+        <v/>
+      </c>
+      <c r="O227" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:11:08</t>
+        </is>
+      </c>
+      <c r="B228" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C228" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D228" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E228" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F228" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G228" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H228" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I228" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7826</t>
+        </is>
+      </c>
+      <c r="J228" s="17" t="n">
+        <v>77801.59546440652</v>
+      </c>
+      <c r="K228" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,022.6150; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L228" s="17" t="n">
+        <v>68000.24505182168</v>
+      </c>
+      <c r="M228" s="17">
+        <f>J228-L228</f>
+        <v/>
+      </c>
+      <c r="N228" s="18">
+        <f>IF(J228=0,"",L228/J228)</f>
+        <v/>
+      </c>
+      <c r="O228" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:11:08</t>
+        </is>
+      </c>
+      <c r="B229" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C229" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D229" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E229" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F229" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G229" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H229" s="16" t="n">
+        <v>1.1285</v>
+      </c>
+      <c r="I229" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J229" s="17" t="n">
+        <v>197091.2460699542</v>
+      </c>
+      <c r="K229" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,228.5848</t>
+        </is>
+      </c>
+      <c r="L229" s="17" t="n">
+        <v>150243.6091312141</v>
+      </c>
+      <c r="M229" s="17">
+        <f>J229-L229</f>
+        <v/>
+      </c>
+      <c r="N229" s="18">
+        <f>IF(J229=0,"",L229/J229)</f>
+        <v/>
+      </c>
+      <c r="O229" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:11:08</t>
+        </is>
+      </c>
+      <c r="B230" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C230" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D230" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E230" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F230" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G230" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H230" s="16" t="n">
+        <v>1.0528</v>
+      </c>
+      <c r="I230" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J230" s="17" t="n">
+        <v>186066.0294054695</v>
+      </c>
+      <c r="K230" s="15" t="inlineStr">
+        <is>
+          <t>USDC 161,827.6712</t>
+        </is>
+      </c>
+      <c r="L230" s="17" t="n">
+        <v>161843.8556121311</v>
+      </c>
+      <c r="M230" s="17">
+        <f>J230-L230</f>
+        <v/>
+      </c>
+      <c r="N230" s="18">
+        <f>IF(J230=0,"",L230/J230)</f>
+        <v/>
+      </c>
+      <c r="O230" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:11:08</t>
+        </is>
+      </c>
+      <c r="B231" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C231" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D231" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E231" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F231" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G231" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H231" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I231" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J231" s="17" t="n">
+        <v>327535.5753168139</v>
+      </c>
+      <c r="K231" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L231" s="17" t="n">
+        <v>280179.7165889733</v>
+      </c>
+      <c r="M231" s="17">
+        <f>J231-L231</f>
+        <v/>
+      </c>
+      <c r="N231" s="18">
+        <f>IF(J231=0,"",L231/J231)</f>
+        <v/>
+      </c>
+      <c r="O231" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:11:08</t>
+        </is>
+      </c>
+      <c r="B232" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C232" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D232" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E232" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F232" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G232" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H232" s="16" t="n">
+        <v>1.1296</v>
+      </c>
+      <c r="I232" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J232" s="17" t="n">
+        <v>159924.3452</v>
+      </c>
+      <c r="K232" s="15" t="inlineStr">
+        <is>
+          <t>USDC 119,566.4850</t>
+        </is>
+      </c>
+      <c r="L232" s="17" t="n">
+        <v>119578.4428387121</v>
+      </c>
+      <c r="M232" s="17">
+        <f>J232-L232</f>
+        <v/>
+      </c>
+      <c r="N232" s="18">
+        <f>IF(J232=0,"",L232/J232)</f>
+        <v/>
+      </c>
+      <c r="O232" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:11:08</t>
+        </is>
+      </c>
+      <c r="B233" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C233" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D233" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E233" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F233" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G233" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H233" s="16" t="n">
+        <v>1.0575</v>
+      </c>
+      <c r="I233" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J233" s="17" t="n">
+        <v>160104.8727598479</v>
+      </c>
+      <c r="K233" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,514.6077</t>
+        </is>
+      </c>
+      <c r="L233" s="17" t="n">
+        <v>138514.6076928112</v>
+      </c>
+      <c r="M233" s="17">
+        <f>J233-L233</f>
+        <v/>
+      </c>
+      <c r="N233" s="18">
+        <f>IF(J233=0,"",L233/J233)</f>
+        <v/>
+      </c>
+      <c r="O233" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:11:08</t>
+        </is>
+      </c>
+      <c r="B234" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C234" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D234" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E234" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F234" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeef003c</t>
+        </is>
+      </c>
+      <c r="G234" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H234" s="16" t="inlineStr"/>
+      <c r="I234" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,801.5319</t>
+        </is>
+      </c>
+      <c r="J234" s="17" t="n">
+        <v>50784.76740846837</v>
+      </c>
+      <c r="K234" s="15" t="inlineStr"/>
+      <c r="L234" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M234" s="17">
+        <f>J234-L234</f>
+        <v/>
+      </c>
+      <c r="N234" s="18">
+        <f>IF(J234=0,"",L234/J234)</f>
+        <v/>
+      </c>
+      <c r="O234" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:11:08</t>
+        </is>
+      </c>
+      <c r="B235" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C235" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D235" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E235" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F235" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeeff047</t>
+        </is>
+      </c>
+      <c r="G235" s="15" t="inlineStr">
+        <is>
+          <t>USDC vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H235" s="16" t="inlineStr"/>
+      <c r="I235" s="15" t="inlineStr">
+        <is>
+          <t>USDC 48,647.3916</t>
+        </is>
+      </c>
+      <c r="J235" s="17" t="n">
+        <v>48652.25680268027</v>
+      </c>
+      <c r="K235" s="15" t="inlineStr"/>
+      <c r="L235" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M235" s="17">
+        <f>J235-L235</f>
+        <v/>
+      </c>
+      <c r="N235" s="18">
+        <f>IF(J235=0,"",L235/J235)</f>
+        <v/>
+      </c>
+      <c r="O235" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:11:08</t>
+        </is>
+      </c>
+      <c r="B236" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C236" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D236" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E236" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F236" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G236" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H236" s="16" t="inlineStr"/>
+      <c r="I236" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J236" s="17" t="n">
+        <v>95894.57893567815</v>
+      </c>
+      <c r="K236" s="15" t="inlineStr"/>
+      <c r="L236" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M236" s="17">
+        <f>J236-L236</f>
+        <v/>
+      </c>
+      <c r="N236" s="18">
+        <f>IF(J236=0,"",L236/J236)</f>
+        <v/>
+      </c>
+      <c r="O236" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:11:08</t>
+        </is>
+      </c>
+      <c r="B237" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C237" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D237" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E237" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F237" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G237" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H237" s="16" t="inlineStr"/>
+      <c r="I237" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J237" s="17" t="n">
+        <v>34346.71910984715</v>
+      </c>
+      <c r="K237" s="15" t="inlineStr"/>
+      <c r="L237" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M237" s="17">
+        <f>J237-L237</f>
+        <v/>
+      </c>
+      <c r="N237" s="18">
+        <f>IF(J237=0,"",L237/J237)</f>
+        <v/>
+      </c>
+      <c r="O237" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:11:08</t>
+        </is>
+      </c>
+      <c r="B238" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C238" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D238" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E238" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F238" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G238" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H238" s="16" t="n">
+        <v>1.0425</v>
+      </c>
+      <c r="I238" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J238" s="17" t="n">
+        <v>269822.0475770817</v>
+      </c>
+      <c r="K238" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,014.6260</t>
+        </is>
+      </c>
+      <c r="L238" s="17" t="n">
+        <v>232937.7311494279</v>
+      </c>
+      <c r="M238" s="17">
+        <f>J238-L238</f>
+        <v/>
+      </c>
+      <c r="N238" s="18">
+        <f>IF(J238=0,"",L238/J238)</f>
+        <v/>
+      </c>
+      <c r="O238" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:11:08</t>
+        </is>
+      </c>
+      <c r="B239" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C239" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D239" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E239" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F239" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G239" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H239" s="16" t="inlineStr"/>
+      <c r="I239" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,505.7542</t>
+        </is>
+      </c>
+      <c r="J239" s="17" t="n">
+        <v>15500.63728291745</v>
+      </c>
+      <c r="K239" s="15" t="inlineStr"/>
+      <c r="L239" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M239" s="17">
+        <f>J239-L239</f>
+        <v/>
+      </c>
+      <c r="N239" s="18">
+        <f>IF(J239=0,"",L239/J239)</f>
+        <v/>
+      </c>
+      <c r="O239" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -15586,7 +16591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -16197,6 +17202,41 @@
         <v>1.0375</v>
       </c>
       <c r="I17" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:11:08</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C18" s="17" t="n">
+        <v>553255.9692622912</v>
+      </c>
+      <c r="D18" s="17" t="n">
+        <v>550639.9665617549</v>
+      </c>
+      <c r="E18" s="17" t="n">
+        <v>2479011.887310991</v>
+      </c>
+      <c r="F18" s="17" t="n">
+        <v>1928371.920749236</v>
+      </c>
+      <c r="G18" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="H18" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I18" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 00:41 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O239"/>
+  <dimension ref="A1:O254"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -16561,6 +16561,1011 @@
         <v/>
       </c>
       <c r="O239" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:41:15</t>
+        </is>
+      </c>
+      <c r="B240" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C240" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D240" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E240" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F240" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G240" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H240" s="16" t="n">
+        <v>1.0481</v>
+      </c>
+      <c r="I240" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J240" s="17" t="n">
+        <v>140892.5351983107</v>
+      </c>
+      <c r="K240" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,022.8377</t>
+        </is>
+      </c>
+      <c r="L240" s="17" t="n">
+        <v>120984.1104059315</v>
+      </c>
+      <c r="M240" s="17">
+        <f>J240-L240</f>
+        <v/>
+      </c>
+      <c r="N240" s="18">
+        <f>IF(J240=0,"",L240/J240)</f>
+        <v/>
+      </c>
+      <c r="O240" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:41:15</t>
+        </is>
+      </c>
+      <c r="B241" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C241" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D241" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E241" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F241" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G241" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H241" s="16" t="n">
+        <v>1.0451</v>
+      </c>
+      <c r="I241" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J241" s="17" t="n">
+        <v>328697.7148657488</v>
+      </c>
+      <c r="K241" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,372.4926</t>
+        </is>
+      </c>
+      <c r="L241" s="17" t="n">
+        <v>306433.5416267464</v>
+      </c>
+      <c r="M241" s="17">
+        <f>J241-L241</f>
+        <v/>
+      </c>
+      <c r="N241" s="18">
+        <f>IF(J241=0,"",L241/J241)</f>
+        <v/>
+      </c>
+      <c r="O241" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:41:15</t>
+        </is>
+      </c>
+      <c r="B242" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C242" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D242" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E242" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F242" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G242" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H242" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I242" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J242" s="17" t="n">
+        <v>385952.7845084352</v>
+      </c>
+      <c r="K242" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,587.4014</t>
+        </is>
+      </c>
+      <c r="L242" s="17" t="n">
+        <v>349657.0616904913</v>
+      </c>
+      <c r="M242" s="17">
+        <f>J242-L242</f>
+        <v/>
+      </c>
+      <c r="N242" s="18">
+        <f>IF(J242=0,"",L242/J242)</f>
+        <v/>
+      </c>
+      <c r="O242" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:41:15</t>
+        </is>
+      </c>
+      <c r="B243" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C243" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D243" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E243" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F243" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G243" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H243" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I243" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7826</t>
+        </is>
+      </c>
+      <c r="J243" s="17" t="n">
+        <v>77793.00642127056</v>
+      </c>
+      <c r="K243" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,022.6150; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L243" s="17" t="n">
+        <v>68000.92527797121</v>
+      </c>
+      <c r="M243" s="17">
+        <f>J243-L243</f>
+        <v/>
+      </c>
+      <c r="N243" s="18">
+        <f>IF(J243=0,"",L243/J243)</f>
+        <v/>
+      </c>
+      <c r="O243" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:41:15</t>
+        </is>
+      </c>
+      <c r="B244" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C244" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D244" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E244" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F244" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G244" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H244" s="16" t="n">
+        <v>1.1285</v>
+      </c>
+      <c r="I244" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J244" s="17" t="n">
+        <v>197112.8506198896</v>
+      </c>
+      <c r="K244" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,228.5848</t>
+        </is>
+      </c>
+      <c r="L244" s="17" t="n">
+        <v>150243.6091312141</v>
+      </c>
+      <c r="M244" s="17">
+        <f>J244-L244</f>
+        <v/>
+      </c>
+      <c r="N244" s="18">
+        <f>IF(J244=0,"",L244/J244)</f>
+        <v/>
+      </c>
+      <c r="O244" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:41:15</t>
+        </is>
+      </c>
+      <c r="B245" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C245" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D245" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E245" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F245" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G245" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H245" s="16" t="n">
+        <v>1.0528</v>
+      </c>
+      <c r="I245" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J245" s="17" t="n">
+        <v>186067.1716366149</v>
+      </c>
+      <c r="K245" s="15" t="inlineStr">
+        <is>
+          <t>USDC 161,827.6712</t>
+        </is>
+      </c>
+      <c r="L245" s="17" t="n">
+        <v>161843.8556121311</v>
+      </c>
+      <c r="M245" s="17">
+        <f>J245-L245</f>
+        <v/>
+      </c>
+      <c r="N245" s="18">
+        <f>IF(J245=0,"",L245/J245)</f>
+        <v/>
+      </c>
+      <c r="O245" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:41:15</t>
+        </is>
+      </c>
+      <c r="B246" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C246" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D246" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E246" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F246" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G246" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H246" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I246" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J246" s="17" t="n">
+        <v>327504.1902147376</v>
+      </c>
+      <c r="K246" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L246" s="17" t="n">
+        <v>280176.6841163451</v>
+      </c>
+      <c r="M246" s="17">
+        <f>J246-L246</f>
+        <v/>
+      </c>
+      <c r="N246" s="18">
+        <f>IF(J246=0,"",L246/J246)</f>
+        <v/>
+      </c>
+      <c r="O246" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:41:15</t>
+        </is>
+      </c>
+      <c r="B247" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C247" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D247" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E247" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F247" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G247" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H247" s="16" t="n">
+        <v>1.1296</v>
+      </c>
+      <c r="I247" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J247" s="17" t="n">
+        <v>159924.3452</v>
+      </c>
+      <c r="K247" s="15" t="inlineStr">
+        <is>
+          <t>USDC 119,566.4850</t>
+        </is>
+      </c>
+      <c r="L247" s="17" t="n">
+        <v>119578.4428387121</v>
+      </c>
+      <c r="M247" s="17">
+        <f>J247-L247</f>
+        <v/>
+      </c>
+      <c r="N247" s="18">
+        <f>IF(J247=0,"",L247/J247)</f>
+        <v/>
+      </c>
+      <c r="O247" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:41:15</t>
+        </is>
+      </c>
+      <c r="B248" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C248" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D248" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E248" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F248" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G248" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H248" s="16" t="n">
+        <v>1.0575</v>
+      </c>
+      <c r="I248" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J248" s="17" t="n">
+        <v>160121.3666901073</v>
+      </c>
+      <c r="K248" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,514.6077</t>
+        </is>
+      </c>
+      <c r="L248" s="17" t="n">
+        <v>138473.0533105034</v>
+      </c>
+      <c r="M248" s="17">
+        <f>J248-L248</f>
+        <v/>
+      </c>
+      <c r="N248" s="18">
+        <f>IF(J248=0,"",L248/J248)</f>
+        <v/>
+      </c>
+      <c r="O248" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:41:15</t>
+        </is>
+      </c>
+      <c r="B249" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C249" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D249" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E249" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F249" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeef003c</t>
+        </is>
+      </c>
+      <c r="G249" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H249" s="16" t="inlineStr"/>
+      <c r="I249" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,801.5319</t>
+        </is>
+      </c>
+      <c r="J249" s="17" t="n">
+        <v>50785.27542378752</v>
+      </c>
+      <c r="K249" s="15" t="inlineStr"/>
+      <c r="L249" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M249" s="17">
+        <f>J249-L249</f>
+        <v/>
+      </c>
+      <c r="N249" s="18">
+        <f>IF(J249=0,"",L249/J249)</f>
+        <v/>
+      </c>
+      <c r="O249" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:41:15</t>
+        </is>
+      </c>
+      <c r="B250" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C250" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D250" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E250" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F250" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeeff047</t>
+        </is>
+      </c>
+      <c r="G250" s="15" t="inlineStr">
+        <is>
+          <t>USDC vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H250" s="16" t="inlineStr"/>
+      <c r="I250" s="15" t="inlineStr">
+        <is>
+          <t>USDC 48,647.3916</t>
+        </is>
+      </c>
+      <c r="J250" s="17" t="n">
+        <v>48652.25680268027</v>
+      </c>
+      <c r="K250" s="15" t="inlineStr"/>
+      <c r="L250" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M250" s="17">
+        <f>J250-L250</f>
+        <v/>
+      </c>
+      <c r="N250" s="18">
+        <f>IF(J250=0,"",L250/J250)</f>
+        <v/>
+      </c>
+      <c r="O250" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:41:15</t>
+        </is>
+      </c>
+      <c r="B251" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C251" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D251" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E251" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F251" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G251" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H251" s="16" t="inlineStr"/>
+      <c r="I251" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J251" s="17" t="n">
+        <v>95894.57893567815</v>
+      </c>
+      <c r="K251" s="15" t="inlineStr"/>
+      <c r="L251" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M251" s="17">
+        <f>J251-L251</f>
+        <v/>
+      </c>
+      <c r="N251" s="18">
+        <f>IF(J251=0,"",L251/J251)</f>
+        <v/>
+      </c>
+      <c r="O251" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:41:15</t>
+        </is>
+      </c>
+      <c r="B252" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C252" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D252" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E252" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F252" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G252" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H252" s="16" t="inlineStr"/>
+      <c r="I252" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J252" s="17" t="n">
+        <v>34347.09313556756</v>
+      </c>
+      <c r="K252" s="15" t="inlineStr"/>
+      <c r="L252" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M252" s="17">
+        <f>J252-L252</f>
+        <v/>
+      </c>
+      <c r="N252" s="18">
+        <f>IF(J252=0,"",L252/J252)</f>
+        <v/>
+      </c>
+      <c r="O252" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:41:15</t>
+        </is>
+      </c>
+      <c r="B253" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C253" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D253" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E253" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F253" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G253" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H253" s="16" t="n">
+        <v>1.0425</v>
+      </c>
+      <c r="I253" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J253" s="17" t="n">
+        <v>269822.0475770817</v>
+      </c>
+      <c r="K253" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,014.6260</t>
+        </is>
+      </c>
+      <c r="L253" s="17" t="n">
+        <v>232940.0612956877</v>
+      </c>
+      <c r="M253" s="17">
+        <f>J253-L253</f>
+        <v/>
+      </c>
+      <c r="N253" s="18">
+        <f>IF(J253=0,"",L253/J253)</f>
+        <v/>
+      </c>
+      <c r="O253" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:41:15</t>
+        </is>
+      </c>
+      <c r="B254" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C254" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D254" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E254" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F254" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G254" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H254" s="16" t="inlineStr"/>
+      <c r="I254" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,505.9560</t>
+        </is>
+      </c>
+      <c r="J254" s="17" t="n">
+        <v>15500.9940809246</v>
+      </c>
+      <c r="K254" s="15" t="inlineStr"/>
+      <c r="L254" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M254" s="17">
+        <f>J254-L254</f>
+        <v/>
+      </c>
+      <c r="N254" s="18">
+        <f>IF(J254=0,"",L254/J254)</f>
+        <v/>
+      </c>
+      <c r="O254" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -16591,7 +17596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -17237,6 +18242,41 @@
         <v>1.0375</v>
       </c>
       <c r="I18" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 00:41:15</t>
+        </is>
+      </c>
+      <c r="B19" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C19" s="17" t="n">
+        <v>553352.1049741694</v>
+      </c>
+      <c r="D19" s="17" t="n">
+        <v>550736.8660051001</v>
+      </c>
+      <c r="E19" s="17" t="n">
+        <v>2479068.211310834</v>
+      </c>
+      <c r="F19" s="17" t="n">
+        <v>1928331.345305734</v>
+      </c>
+      <c r="G19" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="H19" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I19" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 01:11 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O254"/>
+  <dimension ref="A1:O269"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -17566,6 +17566,1011 @@
         <v/>
       </c>
       <c r="O254" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:11:23</t>
+        </is>
+      </c>
+      <c r="B255" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C255" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D255" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E255" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F255" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G255" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H255" s="16" t="n">
+        <v>1.0482</v>
+      </c>
+      <c r="I255" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J255" s="17" t="n">
+        <v>140902.0030288818</v>
+      </c>
+      <c r="K255" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,022.8377</t>
+        </is>
+      </c>
+      <c r="L255" s="17" t="n">
+        <v>120985.3206343086</v>
+      </c>
+      <c r="M255" s="17">
+        <f>J255-L255</f>
+        <v/>
+      </c>
+      <c r="N255" s="18">
+        <f>IF(J255=0,"",L255/J255)</f>
+        <v/>
+      </c>
+      <c r="O255" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:11:23</t>
+        </is>
+      </c>
+      <c r="B256" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C256" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D256" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E256" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F256" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G256" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H256" s="16" t="n">
+        <v>1.0451</v>
+      </c>
+      <c r="I256" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J256" s="17" t="n">
+        <v>328698.1933874324</v>
+      </c>
+      <c r="K256" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,372.4926</t>
+        </is>
+      </c>
+      <c r="L256" s="17" t="n">
+        <v>306433.8982430834</v>
+      </c>
+      <c r="M256" s="17">
+        <f>J256-L256</f>
+        <v/>
+      </c>
+      <c r="N256" s="18">
+        <f>IF(J256=0,"",L256/J256)</f>
+        <v/>
+      </c>
+      <c r="O256" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:11:23</t>
+        </is>
+      </c>
+      <c r="B257" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C257" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D257" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E257" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F257" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G257" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H257" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I257" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J257" s="17" t="n">
+        <v>385953.9227552288</v>
+      </c>
+      <c r="K257" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,587.4014</t>
+        </is>
+      </c>
+      <c r="L257" s="17" t="n">
+        <v>349657.4686088068</v>
+      </c>
+      <c r="M257" s="17">
+        <f>J257-L257</f>
+        <v/>
+      </c>
+      <c r="N257" s="18">
+        <f>IF(J257=0,"",L257/J257)</f>
+        <v/>
+      </c>
+      <c r="O257" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:11:23</t>
+        </is>
+      </c>
+      <c r="B258" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C258" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D258" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E258" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F258" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G258" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H258" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I258" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7826</t>
+        </is>
+      </c>
+      <c r="J258" s="17" t="n">
+        <v>77790.70877617823</v>
+      </c>
+      <c r="K258" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,022.6150; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L258" s="17" t="n">
+        <v>68001.60550412074</v>
+      </c>
+      <c r="M258" s="17">
+        <f>J258-L258</f>
+        <v/>
+      </c>
+      <c r="N258" s="18">
+        <f>IF(J258=0,"",L258/J258)</f>
+        <v/>
+      </c>
+      <c r="O258" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:11:23</t>
+        </is>
+      </c>
+      <c r="B259" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C259" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D259" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E259" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F259" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G259" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H259" s="16" t="n">
+        <v>1.1285</v>
+      </c>
+      <c r="I259" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J259" s="17" t="n">
+        <v>197082.7910068016</v>
+      </c>
+      <c r="K259" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,228.5848</t>
+        </is>
+      </c>
+      <c r="L259" s="17" t="n">
+        <v>150243.6091312141</v>
+      </c>
+      <c r="M259" s="17">
+        <f>J259-L259</f>
+        <v/>
+      </c>
+      <c r="N259" s="18">
+        <f>IF(J259=0,"",L259/J259)</f>
+        <v/>
+      </c>
+      <c r="O259" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:11:23</t>
+        </is>
+      </c>
+      <c r="B260" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C260" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D260" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E260" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F260" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G260" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H260" s="16" t="n">
+        <v>1.0528</v>
+      </c>
+      <c r="I260" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J260" s="17" t="n">
+        <v>186067.7529068127</v>
+      </c>
+      <c r="K260" s="15" t="inlineStr">
+        <is>
+          <t>USDC 161,827.6712</t>
+        </is>
+      </c>
+      <c r="L260" s="17" t="n">
+        <v>161843.8556121311</v>
+      </c>
+      <c r="M260" s="17">
+        <f>J260-L260</f>
+        <v/>
+      </c>
+      <c r="N260" s="18">
+        <f>IF(J260=0,"",L260/J260)</f>
+        <v/>
+      </c>
+      <c r="O260" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:11:23</t>
+        </is>
+      </c>
+      <c r="B261" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C261" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D261" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E261" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F261" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G261" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H261" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I261" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J261" s="17" t="n">
+        <v>327507.7401785134</v>
+      </c>
+      <c r="K261" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L261" s="17" t="n">
+        <v>280204.7178768861</v>
+      </c>
+      <c r="M261" s="17">
+        <f>J261-L261</f>
+        <v/>
+      </c>
+      <c r="N261" s="18">
+        <f>IF(J261=0,"",L261/J261)</f>
+        <v/>
+      </c>
+      <c r="O261" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:11:23</t>
+        </is>
+      </c>
+      <c r="B262" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C262" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D262" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E262" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F262" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G262" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H262" s="16" t="n">
+        <v>1.1296</v>
+      </c>
+      <c r="I262" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J262" s="17" t="n">
+        <v>159924.3452</v>
+      </c>
+      <c r="K262" s="15" t="inlineStr">
+        <is>
+          <t>USDC 119,566.4850</t>
+        </is>
+      </c>
+      <c r="L262" s="17" t="n">
+        <v>119578.4428387121</v>
+      </c>
+      <c r="M262" s="17">
+        <f>J262-L262</f>
+        <v/>
+      </c>
+      <c r="N262" s="18">
+        <f>IF(J262=0,"",L262/J262)</f>
+        <v/>
+      </c>
+      <c r="O262" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:11:23</t>
+        </is>
+      </c>
+      <c r="B263" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C263" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D263" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E263" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F263" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G263" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H263" s="16" t="n">
+        <v>1.0575</v>
+      </c>
+      <c r="I263" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J263" s="17" t="n">
+        <v>160121.8389179019</v>
+      </c>
+      <c r="K263" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,514.6077</t>
+        </is>
+      </c>
+      <c r="L263" s="17" t="n">
+        <v>138473.0533105034</v>
+      </c>
+      <c r="M263" s="17">
+        <f>J263-L263</f>
+        <v/>
+      </c>
+      <c r="N263" s="18">
+        <f>IF(J263=0,"",L263/J263)</f>
+        <v/>
+      </c>
+      <c r="O263" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:11:23</t>
+        </is>
+      </c>
+      <c r="B264" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C264" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D264" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E264" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F264" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeef003c</t>
+        </is>
+      </c>
+      <c r="G264" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H264" s="16" t="inlineStr"/>
+      <c r="I264" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,801.5319</t>
+        </is>
+      </c>
+      <c r="J264" s="17" t="n">
+        <v>50785.78343910666</v>
+      </c>
+      <c r="K264" s="15" t="inlineStr"/>
+      <c r="L264" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M264" s="17">
+        <f>J264-L264</f>
+        <v/>
+      </c>
+      <c r="N264" s="18">
+        <f>IF(J264=0,"",L264/J264)</f>
+        <v/>
+      </c>
+      <c r="O264" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:11:23</t>
+        </is>
+      </c>
+      <c r="B265" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C265" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D265" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E265" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F265" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeeff047</t>
+        </is>
+      </c>
+      <c r="G265" s="15" t="inlineStr">
+        <is>
+          <t>USDC vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H265" s="16" t="inlineStr"/>
+      <c r="I265" s="15" t="inlineStr">
+        <is>
+          <t>USDC 48,647.3916</t>
+        </is>
+      </c>
+      <c r="J265" s="17" t="n">
+        <v>48652.25680268027</v>
+      </c>
+      <c r="K265" s="15" t="inlineStr"/>
+      <c r="L265" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M265" s="17">
+        <f>J265-L265</f>
+        <v/>
+      </c>
+      <c r="N265" s="18">
+        <f>IF(J265=0,"",L265/J265)</f>
+        <v/>
+      </c>
+      <c r="O265" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:11:23</t>
+        </is>
+      </c>
+      <c r="B266" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C266" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D266" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E266" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F266" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G266" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H266" s="16" t="inlineStr"/>
+      <c r="I266" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J266" s="17" t="n">
+        <v>95894.57893567815</v>
+      </c>
+      <c r="K266" s="15" t="inlineStr"/>
+      <c r="L266" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M266" s="17">
+        <f>J266-L266</f>
+        <v/>
+      </c>
+      <c r="N266" s="18">
+        <f>IF(J266=0,"",L266/J266)</f>
+        <v/>
+      </c>
+      <c r="O266" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:11:23</t>
+        </is>
+      </c>
+      <c r="B267" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C267" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D267" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E267" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F267" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G267" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H267" s="16" t="inlineStr"/>
+      <c r="I267" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J267" s="17" t="n">
+        <v>34347.28106222296</v>
+      </c>
+      <c r="K267" s="15" t="inlineStr"/>
+      <c r="L267" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M267" s="17">
+        <f>J267-L267</f>
+        <v/>
+      </c>
+      <c r="N267" s="18">
+        <f>IF(J267=0,"",L267/J267)</f>
+        <v/>
+      </c>
+      <c r="O267" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:11:23</t>
+        </is>
+      </c>
+      <c r="B268" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C268" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D268" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E268" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F268" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G268" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H268" s="16" t="n">
+        <v>1.0425</v>
+      </c>
+      <c r="I268" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J268" s="17" t="n">
+        <v>269822.0475770817</v>
+      </c>
+      <c r="K268" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,014.6260</t>
+        </is>
+      </c>
+      <c r="L268" s="17" t="n">
+        <v>232942.3914419474</v>
+      </c>
+      <c r="M268" s="17">
+        <f>J268-L268</f>
+        <v/>
+      </c>
+      <c r="N268" s="18">
+        <f>IF(J268=0,"",L268/J268)</f>
+        <v/>
+      </c>
+      <c r="O268" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:11:23</t>
+        </is>
+      </c>
+      <c r="B269" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C269" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D269" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E269" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F269" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G269" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H269" s="16" t="inlineStr"/>
+      <c r="I269" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,506.1659</t>
+        </is>
+      </c>
+      <c r="J269" s="17" t="n">
+        <v>15501.35896613529</v>
+      </c>
+      <c r="K269" s="15" t="inlineStr"/>
+      <c r="L269" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M269" s="17">
+        <f>J269-L269</f>
+        <v/>
+      </c>
+      <c r="N269" s="18">
+        <f>IF(J269=0,"",L269/J269)</f>
+        <v/>
+      </c>
+      <c r="O269" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -17596,7 +18601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -18277,6 +19282,41 @@
         <v>1.0375</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:11:23</t>
+        </is>
+      </c>
+      <c r="B20" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C20" s="17" t="n">
+        <v>553303.3604767559</v>
+      </c>
+      <c r="D20" s="17" t="n">
+        <v>550688.2397389426</v>
+      </c>
+      <c r="E20" s="17" t="n">
+        <v>2479052.602940656</v>
+      </c>
+      <c r="F20" s="17" t="n">
+        <v>1928364.363201714</v>
+      </c>
+      <c r="G20" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="H20" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I20" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 01:41 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O269"/>
+  <dimension ref="A1:O284"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -18571,6 +18571,1011 @@
         <v/>
       </c>
       <c r="O269" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:41:29</t>
+        </is>
+      </c>
+      <c r="B270" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C270" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D270" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E270" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F270" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G270" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H270" s="16" t="n">
+        <v>1.0481</v>
+      </c>
+      <c r="I270" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J270" s="17" t="n">
+        <v>140902.694676422</v>
+      </c>
+      <c r="K270" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,022.8377</t>
+        </is>
+      </c>
+      <c r="L270" s="17" t="n">
+        <v>120996.2126897029</v>
+      </c>
+      <c r="M270" s="17">
+        <f>J270-L270</f>
+        <v/>
+      </c>
+      <c r="N270" s="18">
+        <f>IF(J270=0,"",L270/J270)</f>
+        <v/>
+      </c>
+      <c r="O270" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:41:29</t>
+        </is>
+      </c>
+      <c r="B271" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C271" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D271" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E271" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F271" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G271" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H271" s="16" t="n">
+        <v>1.0451</v>
+      </c>
+      <c r="I271" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J271" s="17" t="n">
+        <v>328698.3178031844</v>
+      </c>
+      <c r="K271" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,372.4926</t>
+        </is>
+      </c>
+      <c r="L271" s="17" t="n">
+        <v>306433.8934959499</v>
+      </c>
+      <c r="M271" s="17">
+        <f>J271-L271</f>
+        <v/>
+      </c>
+      <c r="N271" s="18">
+        <f>IF(J271=0,"",L271/J271)</f>
+        <v/>
+      </c>
+      <c r="O271" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:41:29</t>
+        </is>
+      </c>
+      <c r="B272" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C272" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D272" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E272" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F272" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G272" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H272" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I272" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J272" s="17" t="n">
+        <v>385916.4423246147</v>
+      </c>
+      <c r="K272" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,587.4014</t>
+        </is>
+      </c>
+      <c r="L272" s="17" t="n">
+        <v>349657.4631920736</v>
+      </c>
+      <c r="M272" s="17">
+        <f>J272-L272</f>
+        <v/>
+      </c>
+      <c r="N272" s="18">
+        <f>IF(J272=0,"",L272/J272)</f>
+        <v/>
+      </c>
+      <c r="O272" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:41:29</t>
+        </is>
+      </c>
+      <c r="B273" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C273" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D273" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E273" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F273" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G273" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H273" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I273" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7826</t>
+        </is>
+      </c>
+      <c r="J273" s="17" t="n">
+        <v>77792.25535709324</v>
+      </c>
+      <c r="K273" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,022.6150; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L273" s="17" t="n">
+        <v>68007.7275394665</v>
+      </c>
+      <c r="M273" s="17">
+        <f>J273-L273</f>
+        <v/>
+      </c>
+      <c r="N273" s="18">
+        <f>IF(J273=0,"",L273/J273)</f>
+        <v/>
+      </c>
+      <c r="O273" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:41:29</t>
+        </is>
+      </c>
+      <c r="B274" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C274" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D274" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E274" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F274" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G274" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H274" s="16" t="n">
+        <v>1.1285</v>
+      </c>
+      <c r="I274" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J274" s="17" t="n">
+        <v>197058.9565966042</v>
+      </c>
+      <c r="K274" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,228.5848</t>
+        </is>
+      </c>
+      <c r="L274" s="17" t="n">
+        <v>150243.6091312141</v>
+      </c>
+      <c r="M274" s="17">
+        <f>J274-L274</f>
+        <v/>
+      </c>
+      <c r="N274" s="18">
+        <f>IF(J274=0,"",L274/J274)</f>
+        <v/>
+      </c>
+      <c r="O274" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:41:29</t>
+        </is>
+      </c>
+      <c r="B275" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C275" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D275" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E275" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F275" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G275" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H275" s="16" t="n">
+        <v>1.0528</v>
+      </c>
+      <c r="I275" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J275" s="17" t="n">
+        <v>186044.2974512673</v>
+      </c>
+      <c r="K275" s="15" t="inlineStr">
+        <is>
+          <t>USDC 161,827.6712</t>
+        </is>
+      </c>
+      <c r="L275" s="17" t="n">
+        <v>161843.8556121311</v>
+      </c>
+      <c r="M275" s="17">
+        <f>J275-L275</f>
+        <v/>
+      </c>
+      <c r="N275" s="18">
+        <f>IF(J275=0,"",L275/J275)</f>
+        <v/>
+      </c>
+      <c r="O275" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:41:29</t>
+        </is>
+      </c>
+      <c r="B276" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C276" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D276" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E276" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F276" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G276" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H276" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I276" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J276" s="17" t="n">
+        <v>327509.3107886366</v>
+      </c>
+      <c r="K276" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L276" s="17" t="n">
+        <v>280179.2207224844</v>
+      </c>
+      <c r="M276" s="17">
+        <f>J276-L276</f>
+        <v/>
+      </c>
+      <c r="N276" s="18">
+        <f>IF(J276=0,"",L276/J276)</f>
+        <v/>
+      </c>
+      <c r="O276" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:41:29</t>
+        </is>
+      </c>
+      <c r="B277" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C277" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D277" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E277" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F277" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G277" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H277" s="16" t="n">
+        <v>1.1296</v>
+      </c>
+      <c r="I277" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J277" s="17" t="n">
+        <v>159924.3452</v>
+      </c>
+      <c r="K277" s="15" t="inlineStr">
+        <is>
+          <t>USDC 119,566.4850</t>
+        </is>
+      </c>
+      <c r="L277" s="17" t="n">
+        <v>119578.4428387121</v>
+      </c>
+      <c r="M277" s="17">
+        <f>J277-L277</f>
+        <v/>
+      </c>
+      <c r="N277" s="18">
+        <f>IF(J277=0,"",L277/J277)</f>
+        <v/>
+      </c>
+      <c r="O277" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:41:29</t>
+        </is>
+      </c>
+      <c r="B278" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C278" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D278" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E278" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F278" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G278" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H278" s="16" t="n">
+        <v>1.0575</v>
+      </c>
+      <c r="I278" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J278" s="17" t="n">
+        <v>160106.2893014333</v>
+      </c>
+      <c r="K278" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,514.6077</t>
+        </is>
+      </c>
+      <c r="L278" s="17" t="n">
+        <v>138486.9047712727</v>
+      </c>
+      <c r="M278" s="17">
+        <f>J278-L278</f>
+        <v/>
+      </c>
+      <c r="N278" s="18">
+        <f>IF(J278=0,"",L278/J278)</f>
+        <v/>
+      </c>
+      <c r="O278" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:41:29</t>
+        </is>
+      </c>
+      <c r="B279" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C279" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D279" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E279" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F279" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeef003c</t>
+        </is>
+      </c>
+      <c r="G279" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H279" s="16" t="inlineStr"/>
+      <c r="I279" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,801.5319</t>
+        </is>
+      </c>
+      <c r="J279" s="17" t="n">
+        <v>50790.35557697892</v>
+      </c>
+      <c r="K279" s="15" t="inlineStr"/>
+      <c r="L279" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M279" s="17">
+        <f>J279-L279</f>
+        <v/>
+      </c>
+      <c r="N279" s="18">
+        <f>IF(J279=0,"",L279/J279)</f>
+        <v/>
+      </c>
+      <c r="O279" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:41:29</t>
+        </is>
+      </c>
+      <c r="B280" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C280" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D280" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E280" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F280" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeeff047</t>
+        </is>
+      </c>
+      <c r="G280" s="15" t="inlineStr">
+        <is>
+          <t>USDC vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H280" s="16" t="inlineStr"/>
+      <c r="I280" s="15" t="inlineStr">
+        <is>
+          <t>USDC 48,647.3916</t>
+        </is>
+      </c>
+      <c r="J280" s="17" t="n">
+        <v>48652.25680268027</v>
+      </c>
+      <c r="K280" s="15" t="inlineStr"/>
+      <c r="L280" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M280" s="17">
+        <f>J280-L280</f>
+        <v/>
+      </c>
+      <c r="N280" s="18">
+        <f>IF(J280=0,"",L280/J280)</f>
+        <v/>
+      </c>
+      <c r="O280" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:41:29</t>
+        </is>
+      </c>
+      <c r="B281" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C281" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D281" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E281" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F281" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G281" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H281" s="16" t="inlineStr"/>
+      <c r="I281" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J281" s="17" t="n">
+        <v>95894.57893567815</v>
+      </c>
+      <c r="K281" s="15" t="inlineStr"/>
+      <c r="L281" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M281" s="17">
+        <f>J281-L281</f>
+        <v/>
+      </c>
+      <c r="N281" s="18">
+        <f>IF(J281=0,"",L281/J281)</f>
+        <v/>
+      </c>
+      <c r="O281" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:41:29</t>
+        </is>
+      </c>
+      <c r="B282" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C282" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D282" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E282" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F282" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G282" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H282" s="16" t="inlineStr"/>
+      <c r="I282" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J282" s="17" t="n">
+        <v>34347.57663826618</v>
+      </c>
+      <c r="K282" s="15" t="inlineStr"/>
+      <c r="L282" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M282" s="17">
+        <f>J282-L282</f>
+        <v/>
+      </c>
+      <c r="N282" s="18">
+        <f>IF(J282=0,"",L282/J282)</f>
+        <v/>
+      </c>
+      <c r="O282" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:41:29</t>
+        </is>
+      </c>
+      <c r="B283" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C283" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D283" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E283" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F283" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G283" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H283" s="16" t="n">
+        <v>1.043</v>
+      </c>
+      <c r="I283" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J283" s="17" t="n">
+        <v>269988.2546126188</v>
+      </c>
+      <c r="K283" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,014.6260</t>
+        </is>
+      </c>
+      <c r="L283" s="17" t="n">
+        <v>232963.3627582853</v>
+      </c>
+      <c r="M283" s="17">
+        <f>J283-L283</f>
+        <v/>
+      </c>
+      <c r="N283" s="18">
+        <f>IF(J283=0,"",L283/J283)</f>
+        <v/>
+      </c>
+      <c r="O283" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:41:29</t>
+        </is>
+      </c>
+      <c r="B284" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C284" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D284" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E284" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F284" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G284" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H284" s="16" t="inlineStr"/>
+      <c r="I284" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,506.3609</t>
+        </is>
+      </c>
+      <c r="J284" s="17" t="n">
+        <v>15502.94954512221</v>
+      </c>
+      <c r="K284" s="15" t="inlineStr"/>
+      <c r="L284" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M284" s="17">
+        <f>J284-L284</f>
+        <v/>
+      </c>
+      <c r="N284" s="18">
+        <f>IF(J284=0,"",L284/J284)</f>
+        <v/>
+      </c>
+      <c r="O284" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -18601,7 +19606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -19317,6 +20322,41 @@
         <v>1.0375</v>
       </c>
       <c r="I20" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 01:41:29</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C21" s="17" t="n">
+        <v>553353.5248996333</v>
+      </c>
+      <c r="D21" s="17" t="n">
+        <v>550738.1888593072</v>
+      </c>
+      <c r="E21" s="17" t="n">
+        <v>2479128.8816106</v>
+      </c>
+      <c r="F21" s="17" t="n">
+        <v>1928390.692751293</v>
+      </c>
+      <c r="G21" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="H21" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I21" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 02:11 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O284"/>
+  <dimension ref="A1:O299"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -19576,6 +19576,1011 @@
         <v/>
       </c>
       <c r="O284" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:11:36</t>
+        </is>
+      </c>
+      <c r="B285" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C285" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D285" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E285" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F285" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G285" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H285" s="16" t="n">
+        <v>1.0481</v>
+      </c>
+      <c r="I285" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J285" s="17" t="n">
+        <v>140889.0337609608</v>
+      </c>
+      <c r="K285" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,022.8377</t>
+        </is>
+      </c>
+      <c r="L285" s="17" t="n">
+        <v>120986.5308626858</v>
+      </c>
+      <c r="M285" s="17">
+        <f>J285-L285</f>
+        <v/>
+      </c>
+      <c r="N285" s="18">
+        <f>IF(J285=0,"",L285/J285)</f>
+        <v/>
+      </c>
+      <c r="O285" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:11:36</t>
+        </is>
+      </c>
+      <c r="B286" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C286" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D286" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E286" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F286" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G286" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H286" s="16" t="n">
+        <v>1.0451</v>
+      </c>
+      <c r="I286" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J286" s="17" t="n">
+        <v>328699.8730040566</v>
+      </c>
+      <c r="K286" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,372.4926</t>
+        </is>
+      </c>
+      <c r="L286" s="17" t="n">
+        <v>306436.5451914429</v>
+      </c>
+      <c r="M286" s="17">
+        <f>J286-L286</f>
+        <v/>
+      </c>
+      <c r="N286" s="18">
+        <f>IF(J286=0,"",L286/J286)</f>
+        <v/>
+      </c>
+      <c r="O286" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:11:36</t>
+        </is>
+      </c>
+      <c r="B287" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C287" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D287" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E287" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F287" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G287" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H287" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I287" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J287" s="17" t="n">
+        <v>385956.2068854743</v>
+      </c>
+      <c r="K287" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,587.4014</t>
+        </is>
+      </c>
+      <c r="L287" s="17" t="n">
+        <v>349660.4889184666</v>
+      </c>
+      <c r="M287" s="17">
+        <f>J287-L287</f>
+        <v/>
+      </c>
+      <c r="N287" s="18">
+        <f>IF(J287=0,"",L287/J287)</f>
+        <v/>
+      </c>
+      <c r="O287" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:11:36</t>
+        </is>
+      </c>
+      <c r="B288" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C288" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D288" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E288" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F288" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G288" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H288" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I288" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7826</t>
+        </is>
+      </c>
+      <c r="J288" s="17" t="n">
+        <v>77792.33871755133</v>
+      </c>
+      <c r="K288" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,022.6150; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L288" s="17" t="n">
+        <v>68002.28573027028</v>
+      </c>
+      <c r="M288" s="17">
+        <f>J288-L288</f>
+        <v/>
+      </c>
+      <c r="N288" s="18">
+        <f>IF(J288=0,"",L288/J288)</f>
+        <v/>
+      </c>
+      <c r="O288" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:11:36</t>
+        </is>
+      </c>
+      <c r="B289" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C289" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D289" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E289" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F289" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G289" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H289" s="16" t="n">
+        <v>1.1285</v>
+      </c>
+      <c r="I289" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J289" s="17" t="n">
+        <v>197062.7640894585</v>
+      </c>
+      <c r="K289" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,228.5848</t>
+        </is>
+      </c>
+      <c r="L289" s="17" t="n">
+        <v>150243.6091312141</v>
+      </c>
+      <c r="M289" s="17">
+        <f>J289-L289</f>
+        <v/>
+      </c>
+      <c r="N289" s="18">
+        <f>IF(J289=0,"",L289/J289)</f>
+        <v/>
+      </c>
+      <c r="O289" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:11:36</t>
+        </is>
+      </c>
+      <c r="B290" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C290" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D290" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E290" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F290" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G290" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H290" s="16" t="n">
+        <v>1.0528</v>
+      </c>
+      <c r="I290" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J290" s="17" t="n">
+        <v>186037.9001008217</v>
+      </c>
+      <c r="K290" s="15" t="inlineStr">
+        <is>
+          <t>USDC 161,827.6712</t>
+        </is>
+      </c>
+      <c r="L290" s="17" t="n">
+        <v>161843.8556121311</v>
+      </c>
+      <c r="M290" s="17">
+        <f>J290-L290</f>
+        <v/>
+      </c>
+      <c r="N290" s="18">
+        <f>IF(J290=0,"",L290/J290)</f>
+        <v/>
+      </c>
+      <c r="O290" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:11:36</t>
+        </is>
+      </c>
+      <c r="B291" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C291" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D291" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E291" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F291" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G291" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H291" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I291" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J291" s="17" t="n">
+        <v>327509.9768799879</v>
+      </c>
+      <c r="K291" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L291" s="17" t="n">
+        <v>280179.2309369973</v>
+      </c>
+      <c r="M291" s="17">
+        <f>J291-L291</f>
+        <v/>
+      </c>
+      <c r="N291" s="18">
+        <f>IF(J291=0,"",L291/J291)</f>
+        <v/>
+      </c>
+      <c r="O291" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:11:36</t>
+        </is>
+      </c>
+      <c r="B292" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C292" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D292" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E292" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F292" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G292" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H292" s="16" t="n">
+        <v>1.1296</v>
+      </c>
+      <c r="I292" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J292" s="17" t="n">
+        <v>159989.8916291629</v>
+      </c>
+      <c r="K292" s="15" t="inlineStr">
+        <is>
+          <t>USDC 119,566.4850</t>
+        </is>
+      </c>
+      <c r="L292" s="17" t="n">
+        <v>119578.4428387121</v>
+      </c>
+      <c r="M292" s="17">
+        <f>J292-L292</f>
+        <v/>
+      </c>
+      <c r="N292" s="18">
+        <f>IF(J292=0,"",L292/J292)</f>
+        <v/>
+      </c>
+      <c r="O292" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:11:36</t>
+        </is>
+      </c>
+      <c r="B293" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C293" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D293" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E293" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F293" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G293" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H293" s="16" t="n">
+        <v>1.0575</v>
+      </c>
+      <c r="I293" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J293" s="17" t="n">
+        <v>160122.7865417338</v>
+      </c>
+      <c r="K293" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,514.6077</t>
+        </is>
+      </c>
+      <c r="L293" s="17" t="n">
+        <v>138486.9047712727</v>
+      </c>
+      <c r="M293" s="17">
+        <f>J293-L293</f>
+        <v/>
+      </c>
+      <c r="N293" s="18">
+        <f>IF(J293=0,"",L293/J293)</f>
+        <v/>
+      </c>
+      <c r="O293" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:11:36</t>
+        </is>
+      </c>
+      <c r="B294" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C294" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D294" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E294" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F294" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeef003c</t>
+        </is>
+      </c>
+      <c r="G294" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H294" s="16" t="inlineStr"/>
+      <c r="I294" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,801.5319</t>
+        </is>
+      </c>
+      <c r="J294" s="17" t="n">
+        <v>50786.2914544258</v>
+      </c>
+      <c r="K294" s="15" t="inlineStr"/>
+      <c r="L294" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M294" s="17">
+        <f>J294-L294</f>
+        <v/>
+      </c>
+      <c r="N294" s="18">
+        <f>IF(J294=0,"",L294/J294)</f>
+        <v/>
+      </c>
+      <c r="O294" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:11:36</t>
+        </is>
+      </c>
+      <c r="B295" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C295" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D295" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E295" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F295" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeeff047</t>
+        </is>
+      </c>
+      <c r="G295" s="15" t="inlineStr">
+        <is>
+          <t>USDC vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H295" s="16" t="inlineStr"/>
+      <c r="I295" s="15" t="inlineStr">
+        <is>
+          <t>USDC 48,647.3916</t>
+        </is>
+      </c>
+      <c r="J295" s="17" t="n">
+        <v>48652.25680268027</v>
+      </c>
+      <c r="K295" s="15" t="inlineStr"/>
+      <c r="L295" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M295" s="17">
+        <f>J295-L295</f>
+        <v/>
+      </c>
+      <c r="N295" s="18">
+        <f>IF(J295=0,"",L295/J295)</f>
+        <v/>
+      </c>
+      <c r="O295" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:11:36</t>
+        </is>
+      </c>
+      <c r="B296" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C296" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D296" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E296" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F296" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G296" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H296" s="16" t="inlineStr"/>
+      <c r="I296" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J296" s="17" t="n">
+        <v>95890.87931367986</v>
+      </c>
+      <c r="K296" s="15" t="inlineStr"/>
+      <c r="L296" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M296" s="17">
+        <f>J296-L296</f>
+        <v/>
+      </c>
+      <c r="N296" s="18">
+        <f>IF(J296=0,"",L296/J296)</f>
+        <v/>
+      </c>
+      <c r="O296" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:11:36</t>
+        </is>
+      </c>
+      <c r="B297" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C297" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D297" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E297" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F297" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G297" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H297" s="16" t="inlineStr"/>
+      <c r="I297" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J297" s="17" t="n">
+        <v>34341.04517868713</v>
+      </c>
+      <c r="K297" s="15" t="inlineStr"/>
+      <c r="L297" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M297" s="17">
+        <f>J297-L297</f>
+        <v/>
+      </c>
+      <c r="N297" s="18">
+        <f>IF(J297=0,"",L297/J297)</f>
+        <v/>
+      </c>
+      <c r="O297" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:11:36</t>
+        </is>
+      </c>
+      <c r="B298" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C298" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D298" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E298" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F298" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G298" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H298" s="16" t="n">
+        <v>1.0432</v>
+      </c>
+      <c r="I298" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J298" s="17" t="n">
+        <v>270016.4372794854</v>
+      </c>
+      <c r="K298" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,014.6260</t>
+        </is>
+      </c>
+      <c r="L298" s="17" t="n">
+        <v>232944.7215882072</v>
+      </c>
+      <c r="M298" s="17">
+        <f>J298-L298</f>
+        <v/>
+      </c>
+      <c r="N298" s="18">
+        <f>IF(J298=0,"",L298/J298)</f>
+        <v/>
+      </c>
+      <c r="O298" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:11:36</t>
+        </is>
+      </c>
+      <c r="B299" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C299" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D299" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E299" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F299" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G299" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H299" s="16" t="inlineStr"/>
+      <c r="I299" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,506.5666</t>
+        </is>
+      </c>
+      <c r="J299" s="17" t="n">
+        <v>15501.91459783038</v>
+      </c>
+      <c r="K299" s="15" t="inlineStr"/>
+      <c r="L299" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M299" s="17">
+        <f>J299-L299</f>
+        <v/>
+      </c>
+      <c r="N299" s="18">
+        <f>IF(J299=0,"",L299/J299)</f>
+        <v/>
+      </c>
+      <c r="O299" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -19606,7 +20611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -20357,6 +21362,41 @@
         <v>1.0375</v>
       </c>
       <c r="I21" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:11:36</t>
+        </is>
+      </c>
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="n">
+        <v>553502.5867893468</v>
+      </c>
+      <c r="D22" s="17" t="n">
+        <v>550886.9806545966</v>
+      </c>
+      <c r="E22" s="17" t="n">
+        <v>2479249.596235997</v>
+      </c>
+      <c r="F22" s="17" t="n">
+        <v>1928362.6155814</v>
+      </c>
+      <c r="G22" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="H22" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I22" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 02:41 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O299"/>
+  <dimension ref="A1:O314"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -20581,6 +20581,1011 @@
         <v/>
       </c>
       <c r="O299" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:41:41</t>
+        </is>
+      </c>
+      <c r="B300" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C300" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D300" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E300" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F300" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G300" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H300" s="16" t="n">
+        <v>1.0481</v>
+      </c>
+      <c r="I300" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J300" s="17" t="n">
+        <v>140889.446524815</v>
+      </c>
+      <c r="K300" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,022.8377</t>
+        </is>
+      </c>
+      <c r="L300" s="17" t="n">
+        <v>120978.0592640458</v>
+      </c>
+      <c r="M300" s="17">
+        <f>J300-L300</f>
+        <v/>
+      </c>
+      <c r="N300" s="18">
+        <f>IF(J300=0,"",L300/J300)</f>
+        <v/>
+      </c>
+      <c r="O300" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:41:41</t>
+        </is>
+      </c>
+      <c r="B301" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C301" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D301" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E301" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F301" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G301" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H301" s="16" t="n">
+        <v>1.0451</v>
+      </c>
+      <c r="I301" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J301" s="17" t="n">
+        <v>328700.3467436305</v>
+      </c>
+      <c r="K301" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,372.4926</t>
+        </is>
+      </c>
+      <c r="L301" s="17" t="n">
+        <v>306436.5437402071</v>
+      </c>
+      <c r="M301" s="17">
+        <f>J301-L301</f>
+        <v/>
+      </c>
+      <c r="N301" s="18">
+        <f>IF(J301=0,"",L301/J301)</f>
+        <v/>
+      </c>
+      <c r="O301" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:41:41</t>
+        </is>
+      </c>
+      <c r="B302" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C302" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D302" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E302" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F302" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G302" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H302" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I302" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J302" s="17" t="n">
+        <v>385957.3529691919</v>
+      </c>
+      <c r="K302" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,587.4014</t>
+        </is>
+      </c>
+      <c r="L302" s="17" t="n">
+        <v>349660.4872625289</v>
+      </c>
+      <c r="M302" s="17">
+        <f>J302-L302</f>
+        <v/>
+      </c>
+      <c r="N302" s="18">
+        <f>IF(J302=0,"",L302/J302)</f>
+        <v/>
+      </c>
+      <c r="O302" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:41:41</t>
+        </is>
+      </c>
+      <c r="B303" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C303" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D303" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E303" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F303" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G303" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H303" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I303" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7826</t>
+        </is>
+      </c>
+      <c r="J303" s="17" t="n">
+        <v>77787.66045226256</v>
+      </c>
+      <c r="K303" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,022.6150; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L303" s="17" t="n">
+        <v>67997.52414722356</v>
+      </c>
+      <c r="M303" s="17">
+        <f>J303-L303</f>
+        <v/>
+      </c>
+      <c r="N303" s="18">
+        <f>IF(J303=0,"",L303/J303)</f>
+        <v/>
+      </c>
+      <c r="O303" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:41:41</t>
+        </is>
+      </c>
+      <c r="B304" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C304" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D304" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E304" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F304" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G304" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H304" s="16" t="n">
+        <v>1.1285</v>
+      </c>
+      <c r="I304" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J304" s="17" t="n">
+        <v>197063.7394283608</v>
+      </c>
+      <c r="K304" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,228.5848</t>
+        </is>
+      </c>
+      <c r="L304" s="17" t="n">
+        <v>150243.6091312141</v>
+      </c>
+      <c r="M304" s="17">
+        <f>J304-L304</f>
+        <v/>
+      </c>
+      <c r="N304" s="18">
+        <f>IF(J304=0,"",L304/J304)</f>
+        <v/>
+      </c>
+      <c r="O304" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:41:41</t>
+        </is>
+      </c>
+      <c r="B305" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C305" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D305" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E305" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F305" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G305" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H305" s="16" t="n">
+        <v>1.0528</v>
+      </c>
+      <c r="I305" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J305" s="17" t="n">
+        <v>186038.4553128569</v>
+      </c>
+      <c r="K305" s="15" t="inlineStr">
+        <is>
+          <t>USDC 161,827.6712</t>
+        </is>
+      </c>
+      <c r="L305" s="17" t="n">
+        <v>161843.8556121311</v>
+      </c>
+      <c r="M305" s="17">
+        <f>J305-L305</f>
+        <v/>
+      </c>
+      <c r="N305" s="18">
+        <f>IF(J305=0,"",L305/J305)</f>
+        <v/>
+      </c>
+      <c r="O305" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:41:41</t>
+        </is>
+      </c>
+      <c r="B306" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C306" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D306" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E306" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F306" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G306" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H306" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I306" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J306" s="17" t="n">
+        <v>327510.8530358593</v>
+      </c>
+      <c r="K306" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L306" s="17" t="n">
+        <v>280179.3866731562</v>
+      </c>
+      <c r="M306" s="17">
+        <f>J306-L306</f>
+        <v/>
+      </c>
+      <c r="N306" s="18">
+        <f>IF(J306=0,"",L306/J306)</f>
+        <v/>
+      </c>
+      <c r="O306" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:41:41</t>
+        </is>
+      </c>
+      <c r="B307" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C307" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D307" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E307" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F307" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G307" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H307" s="16" t="n">
+        <v>1.1296</v>
+      </c>
+      <c r="I307" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J307" s="17" t="n">
+        <v>159989.8916291629</v>
+      </c>
+      <c r="K307" s="15" t="inlineStr">
+        <is>
+          <t>USDC 119,566.4850</t>
+        </is>
+      </c>
+      <c r="L307" s="17" t="n">
+        <v>119578.4428387121</v>
+      </c>
+      <c r="M307" s="17">
+        <f>J307-L307</f>
+        <v/>
+      </c>
+      <c r="N307" s="18">
+        <f>IF(J307=0,"",L307/J307)</f>
+        <v/>
+      </c>
+      <c r="O307" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:41:41</t>
+        </is>
+      </c>
+      <c r="B308" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C308" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D308" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E308" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F308" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G308" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H308" s="16" t="n">
+        <v>1.0575</v>
+      </c>
+      <c r="I308" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J308" s="17" t="n">
+        <v>160123.262020856</v>
+      </c>
+      <c r="K308" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,514.6077</t>
+        </is>
+      </c>
+      <c r="L308" s="17" t="n">
+        <v>138500.756232042</v>
+      </c>
+      <c r="M308" s="17">
+        <f>J308-L308</f>
+        <v/>
+      </c>
+      <c r="N308" s="18">
+        <f>IF(J308=0,"",L308/J308)</f>
+        <v/>
+      </c>
+      <c r="O308" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:41:41</t>
+        </is>
+      </c>
+      <c r="B309" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C309" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D309" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E309" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F309" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeef003c</t>
+        </is>
+      </c>
+      <c r="G309" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H309" s="16" t="inlineStr"/>
+      <c r="I309" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,801.5319</t>
+        </is>
+      </c>
+      <c r="J309" s="17" t="n">
+        <v>50782.73534719182</v>
+      </c>
+      <c r="K309" s="15" t="inlineStr"/>
+      <c r="L309" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M309" s="17">
+        <f>J309-L309</f>
+        <v/>
+      </c>
+      <c r="N309" s="18">
+        <f>IF(J309=0,"",L309/J309)</f>
+        <v/>
+      </c>
+      <c r="O309" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:41:41</t>
+        </is>
+      </c>
+      <c r="B310" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C310" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D310" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E310" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F310" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeeff047</t>
+        </is>
+      </c>
+      <c r="G310" s="15" t="inlineStr">
+        <is>
+          <t>USDC vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H310" s="16" t="inlineStr"/>
+      <c r="I310" s="15" t="inlineStr">
+        <is>
+          <t>USDC 48,647.3916</t>
+        </is>
+      </c>
+      <c r="J310" s="17" t="n">
+        <v>48652.25680268027</v>
+      </c>
+      <c r="K310" s="15" t="inlineStr"/>
+      <c r="L310" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M310" s="17">
+        <f>J310-L310</f>
+        <v/>
+      </c>
+      <c r="N310" s="18">
+        <f>IF(J310=0,"",L310/J310)</f>
+        <v/>
+      </c>
+      <c r="O310" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:41:41</t>
+        </is>
+      </c>
+      <c r="B311" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C311" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D311" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E311" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F311" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G311" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H311" s="16" t="inlineStr"/>
+      <c r="I311" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J311" s="17" t="n">
+        <v>95890.87931367986</v>
+      </c>
+      <c r="K311" s="15" t="inlineStr"/>
+      <c r="L311" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M311" s="17">
+        <f>J311-L311</f>
+        <v/>
+      </c>
+      <c r="N311" s="18">
+        <f>IF(J311=0,"",L311/J311)</f>
+        <v/>
+      </c>
+      <c r="O311" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:41:41</t>
+        </is>
+      </c>
+      <c r="B312" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C312" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D312" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E312" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F312" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G312" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H312" s="16" t="inlineStr"/>
+      <c r="I312" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J312" s="17" t="n">
+        <v>34341.22577539509</v>
+      </c>
+      <c r="K312" s="15" t="inlineStr"/>
+      <c r="L312" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M312" s="17">
+        <f>J312-L312</f>
+        <v/>
+      </c>
+      <c r="N312" s="18">
+        <f>IF(J312=0,"",L312/J312)</f>
+        <v/>
+      </c>
+      <c r="O312" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:41:41</t>
+        </is>
+      </c>
+      <c r="B313" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C313" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D313" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E313" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F313" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G313" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H313" s="16" t="n">
+        <v>1.0433</v>
+      </c>
+      <c r="I313" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J313" s="17" t="n">
+        <v>270015.2563153427</v>
+      </c>
+      <c r="K313" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,014.6260</t>
+        </is>
+      </c>
+      <c r="L313" s="17" t="n">
+        <v>232928.4105643889</v>
+      </c>
+      <c r="M313" s="17">
+        <f>J313-L313</f>
+        <v/>
+      </c>
+      <c r="N313" s="18">
+        <f>IF(J313=0,"",L313/J313)</f>
+        <v/>
+      </c>
+      <c r="O313" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:41:41</t>
+        </is>
+      </c>
+      <c r="B314" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C314" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D314" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E314" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F314" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G314" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H314" s="16" t="inlineStr"/>
+      <c r="I314" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,506.7642</t>
+        </is>
+      </c>
+      <c r="J314" s="17" t="n">
+        <v>15501.02671494033</v>
+      </c>
+      <c r="K314" s="15" t="inlineStr"/>
+      <c r="L314" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M314" s="17">
+        <f>J314-L314</f>
+        <v/>
+      </c>
+      <c r="N314" s="18">
+        <f>IF(J314=0,"",L314/J314)</f>
+        <v/>
+      </c>
+      <c r="O314" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -20611,7 +21616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -21397,6 +22402,41 @@
         <v>1.0375</v>
       </c>
       <c r="I22" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 02:41:41</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C23" s="17" t="n">
+        <v>553512.7777375347</v>
+      </c>
+      <c r="D23" s="17" t="n">
+        <v>550897.3129205762</v>
+      </c>
+      <c r="E23" s="17" t="n">
+        <v>2479244.388386226</v>
+      </c>
+      <c r="F23" s="17" t="n">
+        <v>1928347.07546565</v>
+      </c>
+      <c r="G23" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="H23" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I23" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 03:11 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O314"/>
+  <dimension ref="A1:O329"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -21586,6 +21586,1011 @@
         <v/>
       </c>
       <c r="O314" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:11:49</t>
+        </is>
+      </c>
+      <c r="B315" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C315" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D315" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E315" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F315" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G315" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H315" s="16" t="n">
+        <v>1.0481</v>
+      </c>
+      <c r="I315" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J315" s="17" t="n">
+        <v>140912.7611625717</v>
+      </c>
+      <c r="K315" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,022.8377</t>
+        </is>
+      </c>
+      <c r="L315" s="17" t="n">
+        <v>120998.6331464572</v>
+      </c>
+      <c r="M315" s="17">
+        <f>J315-L315</f>
+        <v/>
+      </c>
+      <c r="N315" s="18">
+        <f>IF(J315=0,"",L315/J315)</f>
+        <v/>
+      </c>
+      <c r="O315" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:11:49</t>
+        </is>
+      </c>
+      <c r="B316" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C316" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D316" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E316" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F316" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G316" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H316" s="16" t="n">
+        <v>1.0451</v>
+      </c>
+      <c r="I316" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J316" s="17" t="n">
+        <v>328701.0741026891</v>
+      </c>
+      <c r="K316" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,372.4926</t>
+        </is>
+      </c>
+      <c r="L316" s="17" t="n">
+        <v>306405.6160133582</v>
+      </c>
+      <c r="M316" s="17">
+        <f>J316-L316</f>
+        <v/>
+      </c>
+      <c r="N316" s="18">
+        <f>IF(J316=0,"",L316/J316)</f>
+        <v/>
+      </c>
+      <c r="O316" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:11:49</t>
+        </is>
+      </c>
+      <c r="B317" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C317" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D317" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E317" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F317" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G317" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H317" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I317" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J317" s="17" t="n">
+        <v>385958.5143551041</v>
+      </c>
+      <c r="K317" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,587.4014</t>
+        </is>
+      </c>
+      <c r="L317" s="17" t="n">
+        <v>349625.1970719141</v>
+      </c>
+      <c r="M317" s="17">
+        <f>J317-L317</f>
+        <v/>
+      </c>
+      <c r="N317" s="18">
+        <f>IF(J317=0,"",L317/J317)</f>
+        <v/>
+      </c>
+      <c r="O317" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:11:49</t>
+        </is>
+      </c>
+      <c r="B318" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C318" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D318" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E318" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F318" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G318" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H318" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I318" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7826</t>
+        </is>
+      </c>
+      <c r="J318" s="17" t="n">
+        <v>77797.84344090558</v>
+      </c>
+      <c r="K318" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,022.6150; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L318" s="17" t="n">
+        <v>68009.0879840094</v>
+      </c>
+      <c r="M318" s="17">
+        <f>J318-L318</f>
+        <v/>
+      </c>
+      <c r="N318" s="18">
+        <f>IF(J318=0,"",L318/J318)</f>
+        <v/>
+      </c>
+      <c r="O318" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:11:49</t>
+        </is>
+      </c>
+      <c r="B319" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C319" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D319" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E319" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F319" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G319" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H319" s="16" t="n">
+        <v>1.1285</v>
+      </c>
+      <c r="I319" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J319" s="17" t="n">
+        <v>197059.5137517813</v>
+      </c>
+      <c r="K319" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,228.5848</t>
+        </is>
+      </c>
+      <c r="L319" s="17" t="n">
+        <v>150228.584770301</v>
+      </c>
+      <c r="M319" s="17">
+        <f>J319-L319</f>
+        <v/>
+      </c>
+      <c r="N319" s="18">
+        <f>IF(J319=0,"",L319/J319)</f>
+        <v/>
+      </c>
+      <c r="O319" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:11:49</t>
+        </is>
+      </c>
+      <c r="B320" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C320" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D320" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E320" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F320" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G320" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H320" s="16" t="n">
+        <v>1.0528</v>
+      </c>
+      <c r="I320" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J320" s="17" t="n">
+        <v>186039.6196589177</v>
+      </c>
+      <c r="K320" s="15" t="inlineStr">
+        <is>
+          <t>USDC 161,827.6712</t>
+        </is>
+      </c>
+      <c r="L320" s="17" t="n">
+        <v>161827.6712265699</v>
+      </c>
+      <c r="M320" s="17">
+        <f>J320-L320</f>
+        <v/>
+      </c>
+      <c r="N320" s="18">
+        <f>IF(J320=0,"",L320/J320)</f>
+        <v/>
+      </c>
+      <c r="O320" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:11:49</t>
+        </is>
+      </c>
+      <c r="B321" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C321" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D321" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E321" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F321" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G321" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H321" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I321" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J321" s="17" t="n">
+        <v>327536.508782132</v>
+      </c>
+      <c r="K321" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L321" s="17" t="n">
+        <v>280201.3346824776</v>
+      </c>
+      <c r="M321" s="17">
+        <f>J321-L321</f>
+        <v/>
+      </c>
+      <c r="N321" s="18">
+        <f>IF(J321=0,"",L321/J321)</f>
+        <v/>
+      </c>
+      <c r="O321" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:11:49</t>
+        </is>
+      </c>
+      <c r="B322" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C322" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D322" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E322" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F322" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G322" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H322" s="16" t="n">
+        <v>1.1296</v>
+      </c>
+      <c r="I322" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J322" s="17" t="n">
+        <v>159989.8916291629</v>
+      </c>
+      <c r="K322" s="15" t="inlineStr">
+        <is>
+          <t>USDC 119,566.4850</t>
+        </is>
+      </c>
+      <c r="L322" s="17" t="n">
+        <v>119566.4849944282</v>
+      </c>
+      <c r="M322" s="17">
+        <f>J322-L322</f>
+        <v/>
+      </c>
+      <c r="N322" s="18">
+        <f>IF(J322=0,"",L322/J322)</f>
+        <v/>
+      </c>
+      <c r="O322" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:11:49</t>
+        </is>
+      </c>
+      <c r="B323" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C323" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D323" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E323" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F323" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G323" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H323" s="16" t="n">
+        <v>1.0575</v>
+      </c>
+      <c r="I323" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J323" s="17" t="n">
+        <v>160123.7438484447</v>
+      </c>
+      <c r="K323" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,514.6077</t>
+        </is>
+      </c>
+      <c r="L323" s="17" t="n">
+        <v>138500.756232042</v>
+      </c>
+      <c r="M323" s="17">
+        <f>J323-L323</f>
+        <v/>
+      </c>
+      <c r="N323" s="18">
+        <f>IF(J323=0,"",L323/J323)</f>
+        <v/>
+      </c>
+      <c r="O323" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:11:49</t>
+        </is>
+      </c>
+      <c r="B324" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C324" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D324" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E324" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F324" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeef003c</t>
+        </is>
+      </c>
+      <c r="G324" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H324" s="16" t="inlineStr"/>
+      <c r="I324" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,801.5319</t>
+        </is>
+      </c>
+      <c r="J324" s="17" t="n">
+        <v>50791.3716076172</v>
+      </c>
+      <c r="K324" s="15" t="inlineStr"/>
+      <c r="L324" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M324" s="17">
+        <f>J324-L324</f>
+        <v/>
+      </c>
+      <c r="N324" s="18">
+        <f>IF(J324=0,"",L324/J324)</f>
+        <v/>
+      </c>
+      <c r="O324" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:11:49</t>
+        </is>
+      </c>
+      <c r="B325" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C325" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D325" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E325" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F325" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeeff047</t>
+        </is>
+      </c>
+      <c r="G325" s="15" t="inlineStr">
+        <is>
+          <t>USDC vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H325" s="16" t="inlineStr"/>
+      <c r="I325" s="15" t="inlineStr">
+        <is>
+          <t>USDC 48,647.3916</t>
+        </is>
+      </c>
+      <c r="J325" s="17" t="n">
+        <v>48647.391577</v>
+      </c>
+      <c r="K325" s="15" t="inlineStr"/>
+      <c r="L325" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M325" s="17">
+        <f>J325-L325</f>
+        <v/>
+      </c>
+      <c r="N325" s="18">
+        <f>IF(J325=0,"",L325/J325)</f>
+        <v/>
+      </c>
+      <c r="O325" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:11:49</t>
+        </is>
+      </c>
+      <c r="B326" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C326" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D326" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E326" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F326" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G326" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H326" s="16" t="inlineStr"/>
+      <c r="I326" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J326" s="17" t="n">
+        <v>95881.27646034981</v>
+      </c>
+      <c r="K326" s="15" t="inlineStr"/>
+      <c r="L326" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M326" s="17">
+        <f>J326-L326</f>
+        <v/>
+      </c>
+      <c r="N326" s="18">
+        <f>IF(J326=0,"",L326/J326)</f>
+        <v/>
+      </c>
+      <c r="O326" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:11:49</t>
+        </is>
+      </c>
+      <c r="B327" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C327" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D327" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E327" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F327" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G327" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H327" s="16" t="inlineStr"/>
+      <c r="I327" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J327" s="17" t="n">
+        <v>34341.6070382308</v>
+      </c>
+      <c r="K327" s="15" t="inlineStr"/>
+      <c r="L327" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M327" s="17">
+        <f>J327-L327</f>
+        <v/>
+      </c>
+      <c r="N327" s="18">
+        <f>IF(J327=0,"",L327/J327)</f>
+        <v/>
+      </c>
+      <c r="O327" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:11:49</t>
+        </is>
+      </c>
+      <c r="B328" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C328" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D328" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E328" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F328" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G328" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H328" s="16" t="n">
+        <v>1.0431</v>
+      </c>
+      <c r="I328" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J328" s="17" t="n">
+        <v>270015.2563153427</v>
+      </c>
+      <c r="K328" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,014.6260</t>
+        </is>
+      </c>
+      <c r="L328" s="17" t="n">
+        <v>232968.0230508048</v>
+      </c>
+      <c r="M328" s="17">
+        <f>J328-L328</f>
+        <v/>
+      </c>
+      <c r="N328" s="18">
+        <f>IF(J328=0,"",L328/J328)</f>
+        <v/>
+      </c>
+      <c r="O328" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:11:49</t>
+        </is>
+      </c>
+      <c r="B329" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C329" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D329" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E329" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F329" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G329" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H329" s="16" t="inlineStr"/>
+      <c r="I329" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,506.9751</t>
+        </is>
+      </c>
+      <c r="J329" s="17" t="n">
+        <v>15503.87372410148</v>
+      </c>
+      <c r="K329" s="15" t="inlineStr"/>
+      <c r="L329" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M329" s="17">
+        <f>J329-L329</f>
+        <v/>
+      </c>
+      <c r="N329" s="18">
+        <f>IF(J329=0,"",L329/J329)</f>
+        <v/>
+      </c>
+      <c r="O329" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -21616,7 +22621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -22437,6 +23442,41 @@
         <v>1.0375</v>
       </c>
       <c r="I23" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:11:49</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C24" s="17" t="n">
+        <v>553584.6026243781</v>
+      </c>
+      <c r="D24" s="17" t="n">
+        <v>550968.8582819884</v>
+      </c>
+      <c r="E24" s="17" t="n">
+        <v>2479300.247454351</v>
+      </c>
+      <c r="F24" s="17" t="n">
+        <v>1928331.389172362</v>
+      </c>
+      <c r="G24" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="H24" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I24" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 03:42 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O329"/>
+  <dimension ref="A1:O344"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -22591,6 +22591,1011 @@
         <v/>
       </c>
       <c r="O329" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:41:56</t>
+        </is>
+      </c>
+      <c r="B330" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C330" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D330" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E330" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F330" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G330" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H330" s="16" t="n">
+        <v>1.0483</v>
+      </c>
+      <c r="I330" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J330" s="17" t="n">
+        <v>140913.1684460175</v>
+      </c>
+      <c r="K330" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,022.8377</t>
+        </is>
+      </c>
+      <c r="L330" s="17" t="n">
+        <v>120984.1104059315</v>
+      </c>
+      <c r="M330" s="17">
+        <f>J330-L330</f>
+        <v/>
+      </c>
+      <c r="N330" s="18">
+        <f>IF(J330=0,"",L330/J330)</f>
+        <v/>
+      </c>
+      <c r="O330" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:41:56</t>
+        </is>
+      </c>
+      <c r="B331" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C331" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D331" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E331" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F331" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G331" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H331" s="16" t="n">
+        <v>1.0451</v>
+      </c>
+      <c r="I331" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J331" s="17" t="n">
+        <v>328701.1937342673</v>
+      </c>
+      <c r="K331" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,372.4926</t>
+        </is>
+      </c>
+      <c r="L331" s="17" t="n">
+        <v>306440.8072102179</v>
+      </c>
+      <c r="M331" s="17">
+        <f>J331-L331</f>
+        <v/>
+      </c>
+      <c r="N331" s="18">
+        <f>IF(J331=0,"",L331/J331)</f>
+        <v/>
+      </c>
+      <c r="O331" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:41:56</t>
+        </is>
+      </c>
+      <c r="B332" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C332" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D332" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E332" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F332" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G332" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H332" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I332" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J332" s="17" t="n">
+        <v>385959.6472838931</v>
+      </c>
+      <c r="K332" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,587.4014</t>
+        </is>
+      </c>
+      <c r="L332" s="17" t="n">
+        <v>349665.3521098581</v>
+      </c>
+      <c r="M332" s="17">
+        <f>J332-L332</f>
+        <v/>
+      </c>
+      <c r="N332" s="18">
+        <f>IF(J332=0,"",L332/J332)</f>
+        <v/>
+      </c>
+      <c r="O332" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:41:56</t>
+        </is>
+      </c>
+      <c r="B333" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C333" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D333" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E333" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F333" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G333" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H333" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I333" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7826</t>
+        </is>
+      </c>
+      <c r="J333" s="17" t="n">
+        <v>77790.1089121126</v>
+      </c>
+      <c r="K333" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,022.6150; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L333" s="17" t="n">
+        <v>68000.92527797121</v>
+      </c>
+      <c r="M333" s="17">
+        <f>J333-L333</f>
+        <v/>
+      </c>
+      <c r="N333" s="18">
+        <f>IF(J333=0,"",L333/J333)</f>
+        <v/>
+      </c>
+      <c r="O333" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:41:56</t>
+        </is>
+      </c>
+      <c r="B334" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C334" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D334" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E334" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F334" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G334" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H334" s="16" t="n">
+        <v>1.1285</v>
+      </c>
+      <c r="I334" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J334" s="17" t="n">
+        <v>197046.3526243202</v>
+      </c>
+      <c r="K334" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,228.5848</t>
+        </is>
+      </c>
+      <c r="L334" s="17" t="n">
+        <v>150243.6091312141</v>
+      </c>
+      <c r="M334" s="17">
+        <f>J334-L334</f>
+        <v/>
+      </c>
+      <c r="N334" s="18">
+        <f>IF(J334=0,"",L334/J334)</f>
+        <v/>
+      </c>
+      <c r="O334" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:41:56</t>
+        </is>
+      </c>
+      <c r="B335" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C335" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D335" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E335" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F335" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G335" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H335" s="16" t="n">
+        <v>1.0528</v>
+      </c>
+      <c r="I335" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J335" s="17" t="n">
+        <v>186040.5091404216</v>
+      </c>
+      <c r="K335" s="15" t="inlineStr">
+        <is>
+          <t>USDC 161,827.6712</t>
+        </is>
+      </c>
+      <c r="L335" s="17" t="n">
+        <v>161843.8556121311</v>
+      </c>
+      <c r="M335" s="17">
+        <f>J335-L335</f>
+        <v/>
+      </c>
+      <c r="N335" s="18">
+        <f>IF(J335=0,"",L335/J335)</f>
+        <v/>
+      </c>
+      <c r="O335" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:41:56</t>
+        </is>
+      </c>
+      <c r="B336" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C336" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D336" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E336" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F336" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G336" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H336" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I336" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J336" s="17" t="n">
+        <v>327538.6267114204</v>
+      </c>
+      <c r="K336" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L336" s="17" t="n">
+        <v>280204.2961223047</v>
+      </c>
+      <c r="M336" s="17">
+        <f>J336-L336</f>
+        <v/>
+      </c>
+      <c r="N336" s="18">
+        <f>IF(J336=0,"",L336/J336)</f>
+        <v/>
+      </c>
+      <c r="O336" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:41:56</t>
+        </is>
+      </c>
+      <c r="B337" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C337" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D337" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E337" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F337" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G337" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H337" s="16" t="n">
+        <v>1.1296</v>
+      </c>
+      <c r="I337" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J337" s="17" t="n">
+        <v>159989.8916291629</v>
+      </c>
+      <c r="K337" s="15" t="inlineStr">
+        <is>
+          <t>USDC 119,566.4850</t>
+        </is>
+      </c>
+      <c r="L337" s="17" t="n">
+        <v>119578.4428387121</v>
+      </c>
+      <c r="M337" s="17">
+        <f>J337-L337</f>
+        <v/>
+      </c>
+      <c r="N337" s="18">
+        <f>IF(J337=0,"",L337/J337)</f>
+        <v/>
+      </c>
+      <c r="O337" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:41:56</t>
+        </is>
+      </c>
+      <c r="B338" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C338" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D338" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E338" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F338" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G338" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H338" s="16" t="n">
+        <v>1.0575</v>
+      </c>
+      <c r="I338" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J338" s="17" t="n">
+        <v>160124.2138699431</v>
+      </c>
+      <c r="K338" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,514.6077</t>
+        </is>
+      </c>
+      <c r="L338" s="17" t="n">
+        <v>138500.756232042</v>
+      </c>
+      <c r="M338" s="17">
+        <f>J338-L338</f>
+        <v/>
+      </c>
+      <c r="N338" s="18">
+        <f>IF(J338=0,"",L338/J338)</f>
+        <v/>
+      </c>
+      <c r="O338" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:41:56</t>
+        </is>
+      </c>
+      <c r="B339" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C339" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D339" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E339" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F339" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeef003c</t>
+        </is>
+      </c>
+      <c r="G339" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H339" s="16" t="inlineStr"/>
+      <c r="I339" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,801.5319</t>
+        </is>
+      </c>
+      <c r="J339" s="17" t="n">
+        <v>50785.27542378752</v>
+      </c>
+      <c r="K339" s="15" t="inlineStr"/>
+      <c r="L339" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M339" s="17">
+        <f>J339-L339</f>
+        <v/>
+      </c>
+      <c r="N339" s="18">
+        <f>IF(J339=0,"",L339/J339)</f>
+        <v/>
+      </c>
+      <c r="O339" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:41:56</t>
+        </is>
+      </c>
+      <c r="B340" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C340" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D340" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E340" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F340" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeeff047</t>
+        </is>
+      </c>
+      <c r="G340" s="15" t="inlineStr">
+        <is>
+          <t>USDC vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H340" s="16" t="inlineStr"/>
+      <c r="I340" s="15" t="inlineStr">
+        <is>
+          <t>USDC 48,647.3916</t>
+        </is>
+      </c>
+      <c r="J340" s="17" t="n">
+        <v>48652.25680268027</v>
+      </c>
+      <c r="K340" s="15" t="inlineStr"/>
+      <c r="L340" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M340" s="17">
+        <f>J340-L340</f>
+        <v/>
+      </c>
+      <c r="N340" s="18">
+        <f>IF(J340=0,"",L340/J340)</f>
+        <v/>
+      </c>
+      <c r="O340" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:41:56</t>
+        </is>
+      </c>
+      <c r="B341" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C341" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D341" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E341" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F341" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G341" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H341" s="16" t="inlineStr"/>
+      <c r="I341" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J341" s="17" t="n">
+        <v>95890.83836192379</v>
+      </c>
+      <c r="K341" s="15" t="inlineStr"/>
+      <c r="L341" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M341" s="17">
+        <f>J341-L341</f>
+        <v/>
+      </c>
+      <c r="N341" s="18">
+        <f>IF(J341=0,"",L341/J341)</f>
+        <v/>
+      </c>
+      <c r="O341" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:41:56</t>
+        </is>
+      </c>
+      <c r="B342" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C342" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D342" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E342" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F342" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G342" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H342" s="16" t="inlineStr"/>
+      <c r="I342" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J342" s="17" t="n">
+        <v>34341.89709269682</v>
+      </c>
+      <c r="K342" s="15" t="inlineStr"/>
+      <c r="L342" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M342" s="17">
+        <f>J342-L342</f>
+        <v/>
+      </c>
+      <c r="N342" s="18">
+        <f>IF(J342=0,"",L342/J342)</f>
+        <v/>
+      </c>
+      <c r="O342" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:41:56</t>
+        </is>
+      </c>
+      <c r="B343" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C343" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D343" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E343" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F343" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G343" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H343" s="16" t="n">
+        <v>1.0432</v>
+      </c>
+      <c r="I343" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J343" s="17" t="n">
+        <v>270015.2563153427</v>
+      </c>
+      <c r="K343" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,014.6260</t>
+        </is>
+      </c>
+      <c r="L343" s="17" t="n">
+        <v>232940.0612956877</v>
+      </c>
+      <c r="M343" s="17">
+        <f>J343-L343</f>
+        <v/>
+      </c>
+      <c r="N343" s="18">
+        <f>IF(J343=0,"",L343/J343)</f>
+        <v/>
+      </c>
+      <c r="O343" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:41:56</t>
+        </is>
+      </c>
+      <c r="B344" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C344" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D344" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E344" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F344" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G344" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H344" s="16" t="inlineStr"/>
+      <c r="I344" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,507.1774</t>
+        </is>
+      </c>
+      <c r="J344" s="17" t="n">
+        <v>15502.21507660845</v>
+      </c>
+      <c r="K344" s="15" t="inlineStr"/>
+      <c r="L344" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M344" s="17">
+        <f>J344-L344</f>
+        <v/>
+      </c>
+      <c r="N344" s="18">
+        <f>IF(J344=0,"",L344/J344)</f>
+        <v/>
+      </c>
+      <c r="O344" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -22621,7 +23626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -23477,6 +24482,41 @@
         <v>1.0375</v>
       </c>
       <c r="I24" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 03:41:56</t>
+        </is>
+      </c>
+      <c r="B25" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C25" s="17" t="n">
+        <v>553505.6052593027</v>
+      </c>
+      <c r="D25" s="17" t="n">
+        <v>550889.235188528</v>
+      </c>
+      <c r="E25" s="17" t="n">
+        <v>2479291.451424598</v>
+      </c>
+      <c r="F25" s="17" t="n">
+        <v>1928402.21623607</v>
+      </c>
+      <c r="G25" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="H25" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I25" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 04:12 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O344"/>
+  <dimension ref="A1:O359"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -23596,6 +23596,1011 @@
         <v/>
       </c>
       <c r="O344" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:12:02</t>
+        </is>
+      </c>
+      <c r="B345" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C345" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D345" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E345" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F345" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G345" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H345" s="16" t="n">
+        <v>1.0481</v>
+      </c>
+      <c r="I345" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J345" s="17" t="n">
+        <v>140913.5877088107</v>
+      </c>
+      <c r="K345" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,022.8377</t>
+        </is>
+      </c>
+      <c r="L345" s="17" t="n">
+        <v>121004.6842883429</v>
+      </c>
+      <c r="M345" s="17">
+        <f>J345-L345</f>
+        <v/>
+      </c>
+      <c r="N345" s="18">
+        <f>IF(J345=0,"",L345/J345)</f>
+        <v/>
+      </c>
+      <c r="O345" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:12:02</t>
+        </is>
+      </c>
+      <c r="B346" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C346" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D346" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E346" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F346" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G346" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H346" s="16" t="n">
+        <v>1.0451</v>
+      </c>
+      <c r="I346" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J346" s="17" t="n">
+        <v>328701.911524651</v>
+      </c>
+      <c r="K346" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,372.4926</t>
+        </is>
+      </c>
+      <c r="L346" s="17" t="n">
+        <v>306418.8931989584</v>
+      </c>
+      <c r="M346" s="17">
+        <f>J346-L346</f>
+        <v/>
+      </c>
+      <c r="N346" s="18">
+        <f>IF(J346=0,"",L346/J346)</f>
+        <v/>
+      </c>
+      <c r="O346" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:12:02</t>
+        </is>
+      </c>
+      <c r="B347" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C347" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D347" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E347" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F347" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G347" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H347" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I347" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J347" s="17" t="n">
+        <v>385922.1794903676</v>
+      </c>
+      <c r="K347" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,587.4014</t>
+        </is>
+      </c>
+      <c r="L347" s="17" t="n">
+        <v>349640.3470508617</v>
+      </c>
+      <c r="M347" s="17">
+        <f>J347-L347</f>
+        <v/>
+      </c>
+      <c r="N347" s="18">
+        <f>IF(J347=0,"",L347/J347)</f>
+        <v/>
+      </c>
+      <c r="O347" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:12:02</t>
+        </is>
+      </c>
+      <c r="B348" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C348" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D348" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E348" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F348" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G348" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H348" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I348" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7826</t>
+        </is>
+      </c>
+      <c r="J348" s="17" t="n">
+        <v>77804.07477953077</v>
+      </c>
+      <c r="K348" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,022.6150; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L348" s="17" t="n">
+        <v>68012.48911475705</v>
+      </c>
+      <c r="M348" s="17">
+        <f>J348-L348</f>
+        <v/>
+      </c>
+      <c r="N348" s="18">
+        <f>IF(J348=0,"",L348/J348)</f>
+        <v/>
+      </c>
+      <c r="O348" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:12:02</t>
+        </is>
+      </c>
+      <c r="B349" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C349" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D349" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E349" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F349" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G349" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H349" s="16" t="n">
+        <v>1.1285</v>
+      </c>
+      <c r="I349" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J349" s="17" t="n">
+        <v>197049.5244567003</v>
+      </c>
+      <c r="K349" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,228.5848</t>
+        </is>
+      </c>
+      <c r="L349" s="17" t="n">
+        <v>150228.584770301</v>
+      </c>
+      <c r="M349" s="17">
+        <f>J349-L349</f>
+        <v/>
+      </c>
+      <c r="N349" s="18">
+        <f>IF(J349=0,"",L349/J349)</f>
+        <v/>
+      </c>
+      <c r="O349" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:12:02</t>
+        </is>
+      </c>
+      <c r="B350" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C350" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D350" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E350" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F350" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G350" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H350" s="16" t="n">
+        <v>1.0528</v>
+      </c>
+      <c r="I350" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J350" s="17" t="n">
+        <v>186036.3792231292</v>
+      </c>
+      <c r="K350" s="15" t="inlineStr">
+        <is>
+          <t>USDC 161,827.6712</t>
+        </is>
+      </c>
+      <c r="L350" s="17" t="n">
+        <v>161827.6712265699</v>
+      </c>
+      <c r="M350" s="17">
+        <f>J350-L350</f>
+        <v/>
+      </c>
+      <c r="N350" s="18">
+        <f>IF(J350=0,"",L350/J350)</f>
+        <v/>
+      </c>
+      <c r="O350" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:12:02</t>
+        </is>
+      </c>
+      <c r="B351" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C351" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D351" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E351" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F351" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G351" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H351" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I351" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J351" s="17" t="n">
+        <v>327542.0884577219</v>
+      </c>
+      <c r="K351" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L351" s="17" t="n">
+        <v>280201.265999979</v>
+      </c>
+      <c r="M351" s="17">
+        <f>J351-L351</f>
+        <v/>
+      </c>
+      <c r="N351" s="18">
+        <f>IF(J351=0,"",L351/J351)</f>
+        <v/>
+      </c>
+      <c r="O351" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:12:02</t>
+        </is>
+      </c>
+      <c r="B352" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C352" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D352" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E352" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F352" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G352" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H352" s="16" t="n">
+        <v>1.1296</v>
+      </c>
+      <c r="I352" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J352" s="17" t="n">
+        <v>159989.8916291629</v>
+      </c>
+      <c r="K352" s="15" t="inlineStr">
+        <is>
+          <t>USDC 119,566.4850</t>
+        </is>
+      </c>
+      <c r="L352" s="17" t="n">
+        <v>119566.4849944282</v>
+      </c>
+      <c r="M352" s="17">
+        <f>J352-L352</f>
+        <v/>
+      </c>
+      <c r="N352" s="18">
+        <f>IF(J352=0,"",L352/J352)</f>
+        <v/>
+      </c>
+      <c r="O352" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:12:02</t>
+        </is>
+      </c>
+      <c r="B353" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C353" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D353" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E353" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F353" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G353" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H353" s="16" t="n">
+        <v>1.0575</v>
+      </c>
+      <c r="I353" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J353" s="17" t="n">
+        <v>160108.6694962607</v>
+      </c>
+      <c r="K353" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,514.6077</t>
+        </is>
+      </c>
+      <c r="L353" s="17" t="n">
+        <v>138473.0533105034</v>
+      </c>
+      <c r="M353" s="17">
+        <f>J353-L353</f>
+        <v/>
+      </c>
+      <c r="N353" s="18">
+        <f>IF(J353=0,"",L353/J353)</f>
+        <v/>
+      </c>
+      <c r="O353" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:12:02</t>
+        </is>
+      </c>
+      <c r="B354" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C354" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D354" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E354" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F354" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeef003c</t>
+        </is>
+      </c>
+      <c r="G354" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H354" s="16" t="inlineStr"/>
+      <c r="I354" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,801.5319</t>
+        </is>
+      </c>
+      <c r="J354" s="17" t="n">
+        <v>50793.9116842129</v>
+      </c>
+      <c r="K354" s="15" t="inlineStr"/>
+      <c r="L354" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M354" s="17">
+        <f>J354-L354</f>
+        <v/>
+      </c>
+      <c r="N354" s="18">
+        <f>IF(J354=0,"",L354/J354)</f>
+        <v/>
+      </c>
+      <c r="O354" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:12:02</t>
+        </is>
+      </c>
+      <c r="B355" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C355" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D355" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E355" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F355" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeeff047</t>
+        </is>
+      </c>
+      <c r="G355" s="15" t="inlineStr">
+        <is>
+          <t>USDC vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H355" s="16" t="inlineStr"/>
+      <c r="I355" s="15" t="inlineStr">
+        <is>
+          <t>USDC 48,647.3916</t>
+        </is>
+      </c>
+      <c r="J355" s="17" t="n">
+        <v>48647.391577</v>
+      </c>
+      <c r="K355" s="15" t="inlineStr"/>
+      <c r="L355" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M355" s="17">
+        <f>J355-L355</f>
+        <v/>
+      </c>
+      <c r="N355" s="18">
+        <f>IF(J355=0,"",L355/J355)</f>
+        <v/>
+      </c>
+      <c r="O355" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:12:02</t>
+        </is>
+      </c>
+      <c r="B356" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C356" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D356" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E356" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F356" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G356" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H356" s="16" t="inlineStr"/>
+      <c r="I356" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J356" s="17" t="n">
+        <v>95890.83836192379</v>
+      </c>
+      <c r="K356" s="15" t="inlineStr"/>
+      <c r="L356" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M356" s="17">
+        <f>J356-L356</f>
+        <v/>
+      </c>
+      <c r="N356" s="18">
+        <f>IF(J356=0,"",L356/J356)</f>
+        <v/>
+      </c>
+      <c r="O356" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:12:02</t>
+        </is>
+      </c>
+      <c r="B357" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C357" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D357" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E357" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F357" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G357" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H357" s="16" t="inlineStr"/>
+      <c r="I357" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J357" s="17" t="n">
+        <v>34342.19079814294</v>
+      </c>
+      <c r="K357" s="15" t="inlineStr"/>
+      <c r="L357" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M357" s="17">
+        <f>J357-L357</f>
+        <v/>
+      </c>
+      <c r="N357" s="18">
+        <f>IF(J357=0,"",L357/J357)</f>
+        <v/>
+      </c>
+      <c r="O357" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:12:02</t>
+        </is>
+      </c>
+      <c r="B358" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C358" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D358" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E358" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F358" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G358" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H358" s="16" t="n">
+        <v>1.043</v>
+      </c>
+      <c r="I358" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J358" s="17" t="n">
+        <v>269988.2547897112</v>
+      </c>
+      <c r="K358" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,014.6260</t>
+        </is>
+      </c>
+      <c r="L358" s="17" t="n">
+        <v>232979.6737821036</v>
+      </c>
+      <c r="M358" s="17">
+        <f>J358-L358</f>
+        <v/>
+      </c>
+      <c r="N358" s="18">
+        <f>IF(J358=0,"",L358/J358)</f>
+        <v/>
+      </c>
+      <c r="O358" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:12:02</t>
+        </is>
+      </c>
+      <c r="B359" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C359" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D359" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E359" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F359" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G359" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H359" s="16" t="inlineStr"/>
+      <c r="I359" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,507.3711</t>
+        </is>
+      </c>
+      <c r="J359" s="17" t="n">
+        <v>15505.04498706357</v>
+      </c>
+      <c r="K359" s="15" t="inlineStr"/>
+      <c r="L359" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M359" s="17">
+        <f>J359-L359</f>
+        <v/>
+      </c>
+      <c r="N359" s="18">
+        <f>IF(J359=0,"",L359/J359)</f>
+        <v/>
+      </c>
+      <c r="O359" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -23626,7 +24631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -24517,6 +25522,41 @@
         <v>1.0375</v>
       </c>
       <c r="I25" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:12:02</t>
+        </is>
+      </c>
+      <c r="B26" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C26" s="17" t="n">
+        <v>553498.7573523375</v>
+      </c>
+      <c r="D26" s="17" t="n">
+        <v>550882.791227584</v>
+      </c>
+      <c r="E26" s="17" t="n">
+        <v>2479235.938964389</v>
+      </c>
+      <c r="F26" s="17" t="n">
+        <v>1928353.147736805</v>
+      </c>
+      <c r="G26" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="H26" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I26" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 04:42 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O359"/>
+  <dimension ref="A1:O374"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -24601,6 +24601,1011 @@
         <v/>
       </c>
       <c r="O359" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:42:09</t>
+        </is>
+      </c>
+      <c r="B360" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C360" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D360" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E360" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F360" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G360" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H360" s="16" t="n">
+        <v>1.0481</v>
+      </c>
+      <c r="I360" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J360" s="17" t="n">
+        <v>140900.0427578861</v>
+      </c>
+      <c r="K360" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,022.8377</t>
+        </is>
+      </c>
+      <c r="L360" s="17" t="n">
+        <v>120986.5308626858</v>
+      </c>
+      <c r="M360" s="17">
+        <f>J360-L360</f>
+        <v/>
+      </c>
+      <c r="N360" s="18">
+        <f>IF(J360=0,"",L360/J360)</f>
+        <v/>
+      </c>
+      <c r="O360" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:42:09</t>
+        </is>
+      </c>
+      <c r="B361" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C361" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D361" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E361" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F361" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G361" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H361" s="16" t="n">
+        <v>1.0451</v>
+      </c>
+      <c r="I361" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J361" s="17" t="n">
+        <v>328703.4571719325</v>
+      </c>
+      <c r="K361" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,372.4926</t>
+        </is>
+      </c>
+      <c r="L361" s="17" t="n">
+        <v>306423.8413238105</v>
+      </c>
+      <c r="M361" s="17">
+        <f>J361-L361</f>
+        <v/>
+      </c>
+      <c r="N361" s="18">
+        <f>IF(J361=0,"",L361/J361)</f>
+        <v/>
+      </c>
+      <c r="O361" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:42:09</t>
+        </is>
+      </c>
+      <c r="B362" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C362" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D362" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E362" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F362" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G362" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H362" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I362" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J362" s="17" t="n">
+        <v>385961.950199689</v>
+      </c>
+      <c r="K362" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,587.4014</t>
+        </is>
+      </c>
+      <c r="L362" s="17" t="n">
+        <v>349645.9931259861</v>
+      </c>
+      <c r="M362" s="17">
+        <f>J362-L362</f>
+        <v/>
+      </c>
+      <c r="N362" s="18">
+        <f>IF(J362=0,"",L362/J362)</f>
+        <v/>
+      </c>
+      <c r="O362" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:42:09</t>
+        </is>
+      </c>
+      <c r="B363" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C363" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D363" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E363" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F363" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G363" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H363" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I363" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7826</t>
+        </is>
+      </c>
+      <c r="J363" s="17" t="n">
+        <v>77792.52687121146</v>
+      </c>
+      <c r="K363" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,022.6150; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L363" s="17" t="n">
+        <v>68002.28572251411</v>
+      </c>
+      <c r="M363" s="17">
+        <f>J363-L363</f>
+        <v/>
+      </c>
+      <c r="N363" s="18">
+        <f>IF(J363=0,"",L363/J363)</f>
+        <v/>
+      </c>
+      <c r="O363" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:42:09</t>
+        </is>
+      </c>
+      <c r="B364" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C364" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D364" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E364" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F364" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G364" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H364" s="16" t="n">
+        <v>1.1285</v>
+      </c>
+      <c r="I364" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J364" s="17" t="n">
+        <v>197092.8123921969</v>
+      </c>
+      <c r="K364" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,228.5848</t>
+        </is>
+      </c>
+      <c r="L364" s="17" t="n">
+        <v>150228.584770301</v>
+      </c>
+      <c r="M364" s="17">
+        <f>J364-L364</f>
+        <v/>
+      </c>
+      <c r="N364" s="18">
+        <f>IF(J364=0,"",L364/J364)</f>
+        <v/>
+      </c>
+      <c r="O364" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:42:09</t>
+        </is>
+      </c>
+      <c r="B365" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C365" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D365" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E365" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F365" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G365" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H365" s="16" t="n">
+        <v>1.0528</v>
+      </c>
+      <c r="I365" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J365" s="17" t="n">
+        <v>186028.5062595782</v>
+      </c>
+      <c r="K365" s="15" t="inlineStr">
+        <is>
+          <t>USDC 161,827.6712</t>
+        </is>
+      </c>
+      <c r="L365" s="17" t="n">
+        <v>161827.6712265699</v>
+      </c>
+      <c r="M365" s="17">
+        <f>J365-L365</f>
+        <v/>
+      </c>
+      <c r="N365" s="18">
+        <f>IF(J365=0,"",L365/J365)</f>
+        <v/>
+      </c>
+      <c r="O365" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:42:09</t>
+        </is>
+      </c>
+      <c r="B366" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C366" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D366" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E366" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F366" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G366" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H366" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I366" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J366" s="17" t="n">
+        <v>327539.9886961927</v>
+      </c>
+      <c r="K366" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L366" s="17" t="n">
+        <v>280229.8296761051</v>
+      </c>
+      <c r="M366" s="17">
+        <f>J366-L366</f>
+        <v/>
+      </c>
+      <c r="N366" s="18">
+        <f>IF(J366=0,"",L366/J366)</f>
+        <v/>
+      </c>
+      <c r="O366" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:42:09</t>
+        </is>
+      </c>
+      <c r="B367" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C367" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D367" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E367" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F367" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G367" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H367" s="16" t="n">
+        <v>1.1296</v>
+      </c>
+      <c r="I367" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J367" s="17" t="n">
+        <v>160005.8938187637</v>
+      </c>
+      <c r="K367" s="15" t="inlineStr">
+        <is>
+          <t>USDC 119,566.4850</t>
+        </is>
+      </c>
+      <c r="L367" s="17" t="n">
+        <v>119566.4849944282</v>
+      </c>
+      <c r="M367" s="17">
+        <f>J367-L367</f>
+        <v/>
+      </c>
+      <c r="N367" s="18">
+        <f>IF(J367=0,"",L367/J367)</f>
+        <v/>
+      </c>
+      <c r="O367" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:42:09</t>
+        </is>
+      </c>
+      <c r="B368" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C368" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D368" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E368" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F368" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G368" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H368" s="16" t="n">
+        <v>1.0575</v>
+      </c>
+      <c r="I368" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J368" s="17" t="n">
+        <v>160125.1692873915</v>
+      </c>
+      <c r="K368" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,514.6077</t>
+        </is>
+      </c>
+      <c r="L368" s="17" t="n">
+        <v>138486.9047712727</v>
+      </c>
+      <c r="M368" s="17">
+        <f>J368-L368</f>
+        <v/>
+      </c>
+      <c r="N368" s="18">
+        <f>IF(J368=0,"",L368/J368)</f>
+        <v/>
+      </c>
+      <c r="O368" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:42:09</t>
+        </is>
+      </c>
+      <c r="B369" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C369" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D369" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E369" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F369" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeef003c</t>
+        </is>
+      </c>
+      <c r="G369" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H369" s="16" t="inlineStr"/>
+      <c r="I369" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,801.5319</t>
+        </is>
+      </c>
+      <c r="J369" s="17" t="n">
+        <v>50786.2914544258</v>
+      </c>
+      <c r="K369" s="15" t="inlineStr"/>
+      <c r="L369" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M369" s="17">
+        <f>J369-L369</f>
+        <v/>
+      </c>
+      <c r="N369" s="18">
+        <f>IF(J369=0,"",L369/J369)</f>
+        <v/>
+      </c>
+      <c r="O369" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:42:09</t>
+        </is>
+      </c>
+      <c r="B370" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C370" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D370" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E370" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F370" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeeff047</t>
+        </is>
+      </c>
+      <c r="G370" s="15" t="inlineStr">
+        <is>
+          <t>USDC vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H370" s="16" t="inlineStr"/>
+      <c r="I370" s="15" t="inlineStr">
+        <is>
+          <t>USDC 48,647.3916</t>
+        </is>
+      </c>
+      <c r="J370" s="17" t="n">
+        <v>48647.391577</v>
+      </c>
+      <c r="K370" s="15" t="inlineStr"/>
+      <c r="L370" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M370" s="17">
+        <f>J370-L370</f>
+        <v/>
+      </c>
+      <c r="N370" s="18">
+        <f>IF(J370=0,"",L370/J370)</f>
+        <v/>
+      </c>
+      <c r="O370" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:42:09</t>
+        </is>
+      </c>
+      <c r="B371" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C371" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D371" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E371" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F371" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G371" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H371" s="16" t="inlineStr"/>
+      <c r="I371" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J371" s="17" t="n">
+        <v>95878.67937969997</v>
+      </c>
+      <c r="K371" s="15" t="inlineStr"/>
+      <c r="L371" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M371" s="17">
+        <f>J371-L371</f>
+        <v/>
+      </c>
+      <c r="N371" s="18">
+        <f>IF(J371=0,"",L371/J371)</f>
+        <v/>
+      </c>
+      <c r="O371" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:42:09</t>
+        </is>
+      </c>
+      <c r="B372" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C372" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D372" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E372" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F372" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G372" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H372" s="16" t="inlineStr"/>
+      <c r="I372" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J372" s="17" t="n">
+        <v>34342.35863095422</v>
+      </c>
+      <c r="K372" s="15" t="inlineStr"/>
+      <c r="L372" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M372" s="17">
+        <f>J372-L372</f>
+        <v/>
+      </c>
+      <c r="N372" s="18">
+        <f>IF(J372=0,"",L372/J372)</f>
+        <v/>
+      </c>
+      <c r="O372" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:42:09</t>
+        </is>
+      </c>
+      <c r="B373" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C373" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D373" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E373" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F373" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G373" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H373" s="16" t="n">
+        <v>1.043</v>
+      </c>
+      <c r="I373" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J373" s="17" t="n">
+        <v>269988.2547897112</v>
+      </c>
+      <c r="K373" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,031.5881</t>
+        </is>
+      </c>
+      <c r="L373" s="17" t="n">
+        <v>232961.6786585595</v>
+      </c>
+      <c r="M373" s="17">
+        <f>J373-L373</f>
+        <v/>
+      </c>
+      <c r="N373" s="18">
+        <f>IF(J373=0,"",L373/J373)</f>
+        <v/>
+      </c>
+      <c r="O373" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:42:09</t>
+        </is>
+      </c>
+      <c r="B374" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C374" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D374" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E374" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F374" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G374" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H374" s="16" t="inlineStr"/>
+      <c r="I374" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,507.5765</t>
+        </is>
+      </c>
+      <c r="J374" s="17" t="n">
+        <v>15502.92421845328</v>
+      </c>
+      <c r="K374" s="15" t="inlineStr"/>
+      <c r="L374" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M374" s="17">
+        <f>J374-L374</f>
+        <v/>
+      </c>
+      <c r="N374" s="18">
+        <f>IF(J374=0,"",L374/J374)</f>
+        <v/>
+      </c>
+      <c r="O374" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -24631,7 +25636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -25557,6 +26562,41 @@
         <v>1.0375</v>
       </c>
       <c r="I26" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 04:42:09</t>
+        </is>
+      </c>
+      <c r="B27" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C27" s="17" t="n">
+        <v>553553.7627541267</v>
+      </c>
+      <c r="D27" s="17" t="n">
+        <v>550936.4423728539</v>
+      </c>
+      <c r="E27" s="17" t="n">
+        <v>2479296.247505086</v>
+      </c>
+      <c r="F27" s="17" t="n">
+        <v>1928359.805132233</v>
+      </c>
+      <c r="G27" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="H27" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I27" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 05:12 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O374"/>
+  <dimension ref="A1:O389"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -25606,6 +25606,1011 @@
         <v/>
       </c>
       <c r="O374" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:12:15</t>
+        </is>
+      </c>
+      <c r="B375" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C375" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D375" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E375" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F375" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G375" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H375" s="16" t="n">
+        <v>1.048</v>
+      </c>
+      <c r="I375" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J375" s="17" t="n">
+        <v>140900.7405533565</v>
+      </c>
+      <c r="K375" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,022.8377</t>
+        </is>
+      </c>
+      <c r="L375" s="17" t="n">
+        <v>120997.42291808</v>
+      </c>
+      <c r="M375" s="17">
+        <f>J375-L375</f>
+        <v/>
+      </c>
+      <c r="N375" s="18">
+        <f>IF(J375=0,"",L375/J375)</f>
+        <v/>
+      </c>
+      <c r="O375" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:12:15</t>
+        </is>
+      </c>
+      <c r="B376" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C376" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D376" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E376" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F376" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G376" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H376" s="16" t="n">
+        <v>1.0451</v>
+      </c>
+      <c r="I376" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J376" s="17" t="n">
+        <v>328703.7012221676</v>
+      </c>
+      <c r="K376" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,372.4926</t>
+        </is>
+      </c>
+      <c r="L376" s="17" t="n">
+        <v>306419.5537919081</v>
+      </c>
+      <c r="M376" s="17">
+        <f>J376-L376</f>
+        <v/>
+      </c>
+      <c r="N376" s="18">
+        <f>IF(J376=0,"",L376/J376)</f>
+        <v/>
+      </c>
+      <c r="O376" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:12:15</t>
+        </is>
+      </c>
+      <c r="B377" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C377" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D377" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E377" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F377" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G377" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H377" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I377" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J377" s="17" t="n">
+        <v>385924.4898712235</v>
+      </c>
+      <c r="K377" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,587.4014</t>
+        </is>
+      </c>
+      <c r="L377" s="17" t="n">
+        <v>349641.1008227516</v>
+      </c>
+      <c r="M377" s="17">
+        <f>J377-L377</f>
+        <v/>
+      </c>
+      <c r="N377" s="18">
+        <f>IF(J377=0,"",L377/J377)</f>
+        <v/>
+      </c>
+      <c r="O377" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:12:15</t>
+        </is>
+      </c>
+      <c r="B378" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C378" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D378" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E378" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F378" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G378" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H378" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I378" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7826</t>
+        </is>
+      </c>
+      <c r="J378" s="17" t="n">
+        <v>77792.50524216217</v>
+      </c>
+      <c r="K378" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,022.6150; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L378" s="17" t="n">
+        <v>68008.40775785987</v>
+      </c>
+      <c r="M378" s="17">
+        <f>J378-L378</f>
+        <v/>
+      </c>
+      <c r="N378" s="18">
+        <f>IF(J378=0,"",L378/J378)</f>
+        <v/>
+      </c>
+      <c r="O378" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:12:15</t>
+        </is>
+      </c>
+      <c r="B379" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C379" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D379" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E379" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F379" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G379" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H379" s="16" t="n">
+        <v>1.1285</v>
+      </c>
+      <c r="I379" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J379" s="17" t="n">
+        <v>197094.2816174144</v>
+      </c>
+      <c r="K379" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,228.5848</t>
+        </is>
+      </c>
+      <c r="L379" s="17" t="n">
+        <v>150228.584770301</v>
+      </c>
+      <c r="M379" s="17">
+        <f>J379-L379</f>
+        <v/>
+      </c>
+      <c r="N379" s="18">
+        <f>IF(J379=0,"",L379/J379)</f>
+        <v/>
+      </c>
+      <c r="O379" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:12:15</t>
+        </is>
+      </c>
+      <c r="B380" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C380" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D380" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E380" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F380" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G380" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H380" s="16" t="n">
+        <v>1.0528</v>
+      </c>
+      <c r="I380" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J380" s="17" t="n">
+        <v>186027.4331403626</v>
+      </c>
+      <c r="K380" s="15" t="inlineStr">
+        <is>
+          <t>USDC 161,827.6712</t>
+        </is>
+      </c>
+      <c r="L380" s="17" t="n">
+        <v>161827.6712265699</v>
+      </c>
+      <c r="M380" s="17">
+        <f>J380-L380</f>
+        <v/>
+      </c>
+      <c r="N380" s="18">
+        <f>IF(J380=0,"",L380/J380)</f>
+        <v/>
+      </c>
+      <c r="O380" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:12:15</t>
+        </is>
+      </c>
+      <c r="B381" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C381" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D381" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E381" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F381" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G381" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H381" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I381" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J381" s="17" t="n">
+        <v>327575.4900924469</v>
+      </c>
+      <c r="K381" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L381" s="17" t="n">
+        <v>280212.7973819937</v>
+      </c>
+      <c r="M381" s="17">
+        <f>J381-L381</f>
+        <v/>
+      </c>
+      <c r="N381" s="18">
+        <f>IF(J381=0,"",L381/J381)</f>
+        <v/>
+      </c>
+      <c r="O381" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:12:15</t>
+        </is>
+      </c>
+      <c r="B382" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C382" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D382" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E382" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F382" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G382" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H382" s="16" t="n">
+        <v>1.1296</v>
+      </c>
+      <c r="I382" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J382" s="17" t="n">
+        <v>160005.8938187637</v>
+      </c>
+      <c r="K382" s="15" t="inlineStr">
+        <is>
+          <t>USDC 119,566.4850</t>
+        </is>
+      </c>
+      <c r="L382" s="17" t="n">
+        <v>119566.4849944282</v>
+      </c>
+      <c r="M382" s="17">
+        <f>J382-L382</f>
+        <v/>
+      </c>
+      <c r="N382" s="18">
+        <f>IF(J382=0,"",L382/J382)</f>
+        <v/>
+      </c>
+      <c r="O382" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:12:15</t>
+        </is>
+      </c>
+      <c r="B383" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C383" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D383" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E383" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F383" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G383" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H383" s="16" t="n">
+        <v>1.0575</v>
+      </c>
+      <c r="I383" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J383" s="17" t="n">
+        <v>160109.6280107605</v>
+      </c>
+      <c r="K383" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,514.6077</t>
+        </is>
+      </c>
+      <c r="L383" s="17" t="n">
+        <v>138486.9047712727</v>
+      </c>
+      <c r="M383" s="17">
+        <f>J383-L383</f>
+        <v/>
+      </c>
+      <c r="N383" s="18">
+        <f>IF(J383=0,"",L383/J383)</f>
+        <v/>
+      </c>
+      <c r="O383" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:12:15</t>
+        </is>
+      </c>
+      <c r="B384" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C384" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D384" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E384" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F384" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeef003c</t>
+        </is>
+      </c>
+      <c r="G384" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H384" s="16" t="inlineStr"/>
+      <c r="I384" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,801.5319</t>
+        </is>
+      </c>
+      <c r="J384" s="17" t="n">
+        <v>50790.86359229805</v>
+      </c>
+      <c r="K384" s="15" t="inlineStr"/>
+      <c r="L384" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M384" s="17">
+        <f>J384-L384</f>
+        <v/>
+      </c>
+      <c r="N384" s="18">
+        <f>IF(J384=0,"",L384/J384)</f>
+        <v/>
+      </c>
+      <c r="O384" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:12:15</t>
+        </is>
+      </c>
+      <c r="B385" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C385" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D385" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E385" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F385" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeeff047</t>
+        </is>
+      </c>
+      <c r="G385" s="15" t="inlineStr">
+        <is>
+          <t>USDC vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H385" s="16" t="inlineStr"/>
+      <c r="I385" s="15" t="inlineStr">
+        <is>
+          <t>USDC 48,647.3916</t>
+        </is>
+      </c>
+      <c r="J385" s="17" t="n">
+        <v>48647.391577</v>
+      </c>
+      <c r="K385" s="15" t="inlineStr"/>
+      <c r="L385" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M385" s="17">
+        <f>J385-L385</f>
+        <v/>
+      </c>
+      <c r="N385" s="18">
+        <f>IF(J385=0,"",L385/J385)</f>
+        <v/>
+      </c>
+      <c r="O385" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:12:15</t>
+        </is>
+      </c>
+      <c r="B386" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C386" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D386" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E386" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F386" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G386" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H386" s="16" t="inlineStr"/>
+      <c r="I386" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J386" s="17" t="n">
+        <v>95873.39753982412</v>
+      </c>
+      <c r="K386" s="15" t="inlineStr"/>
+      <c r="L386" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M386" s="17">
+        <f>J386-L386</f>
+        <v/>
+      </c>
+      <c r="N386" s="18">
+        <f>IF(J386=0,"",L386/J386)</f>
+        <v/>
+      </c>
+      <c r="O386" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:12:15</t>
+        </is>
+      </c>
+      <c r="B387" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C387" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D387" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E387" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F387" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G387" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H387" s="16" t="inlineStr"/>
+      <c r="I387" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J387" s="17" t="n">
+        <v>34342.67788041355</v>
+      </c>
+      <c r="K387" s="15" t="inlineStr"/>
+      <c r="L387" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M387" s="17">
+        <f>J387-L387</f>
+        <v/>
+      </c>
+      <c r="N387" s="18">
+        <f>IF(J387=0,"",L387/J387)</f>
+        <v/>
+      </c>
+      <c r="O387" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:12:15</t>
+        </is>
+      </c>
+      <c r="B388" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C388" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D388" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E388" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F388" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G388" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H388" s="16" t="n">
+        <v>1.043</v>
+      </c>
+      <c r="I388" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J388" s="17" t="n">
+        <v>269988.2547897112</v>
+      </c>
+      <c r="K388" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,031.5881</t>
+        </is>
+      </c>
+      <c r="L388" s="17" t="n">
+        <v>232982.6515014916</v>
+      </c>
+      <c r="M388" s="17">
+        <f>J388-L388</f>
+        <v/>
+      </c>
+      <c r="N388" s="18">
+        <f>IF(J388=0,"",L388/J388)</f>
+        <v/>
+      </c>
+      <c r="O388" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:12:15</t>
+        </is>
+      </c>
+      <c r="B389" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C389" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D389" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E389" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F389" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G389" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H389" s="16" t="inlineStr"/>
+      <c r="I389" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,507.7789</t>
+        </is>
+      </c>
+      <c r="J389" s="17" t="n">
+        <v>15504.52222438191</v>
+      </c>
+      <c r="K389" s="15" t="inlineStr"/>
+      <c r="L389" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M389" s="17">
+        <f>J389-L389</f>
+        <v/>
+      </c>
+      <c r="N389" s="18">
+        <f>IF(J389=0,"",L389/J389)</f>
+        <v/>
+      </c>
+      <c r="O389" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -25636,7 +26641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -26597,6 +27602,41 @@
         <v>1.0375</v>
       </c>
       <c r="I27" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:12:15</t>
+        </is>
+      </c>
+      <c r="B28" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C28" s="17" t="n">
+        <v>553526.6663458915</v>
+      </c>
+      <c r="D28" s="17" t="n">
+        <v>550909.6912356298</v>
+      </c>
+      <c r="E28" s="17" t="n">
+        <v>2479281.271172286</v>
+      </c>
+      <c r="F28" s="17" t="n">
+        <v>1928371.579936657</v>
+      </c>
+      <c r="G28" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="H28" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I28" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 05:42 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O389"/>
+  <dimension ref="A1:O404"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -26611,6 +26611,1011 @@
         <v/>
       </c>
       <c r="O389" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:42:22</t>
+        </is>
+      </c>
+      <c r="B390" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C390" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D390" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E390" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F390" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G390" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H390" s="16" t="n">
+        <v>1.0482</v>
+      </c>
+      <c r="I390" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J390" s="17" t="n">
+        <v>140901.1581139202</v>
+      </c>
+      <c r="K390" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,022.8377</t>
+        </is>
+      </c>
+      <c r="L390" s="17" t="n">
+        <v>120984.1104059315</v>
+      </c>
+      <c r="M390" s="17">
+        <f>J390-L390</f>
+        <v/>
+      </c>
+      <c r="N390" s="18">
+        <f>IF(J390=0,"",L390/J390)</f>
+        <v/>
+      </c>
+      <c r="O390" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:42:22</t>
+        </is>
+      </c>
+      <c r="B391" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C391" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D391" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E391" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F391" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G391" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H391" s="16" t="n">
+        <v>1.0451</v>
+      </c>
+      <c r="I391" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J391" s="17" t="n">
+        <v>328704.069690513</v>
+      </c>
+      <c r="K391" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,372.4926</t>
+        </is>
+      </c>
+      <c r="L391" s="17" t="n">
+        <v>306421.3249769644</v>
+      </c>
+      <c r="M391" s="17">
+        <f>J391-L391</f>
+        <v/>
+      </c>
+      <c r="N391" s="18">
+        <f>IF(J391=0,"",L391/J391)</f>
+        <v/>
+      </c>
+      <c r="O391" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:42:22</t>
+        </is>
+      </c>
+      <c r="B392" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C392" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D392" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E392" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F392" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G392" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H392" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I392" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J392" s="17" t="n">
+        <v>385964.2531588625</v>
+      </c>
+      <c r="K392" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,587.4014</t>
+        </is>
+      </c>
+      <c r="L392" s="17" t="n">
+        <v>349643.121839639</v>
+      </c>
+      <c r="M392" s="17">
+        <f>J392-L392</f>
+        <v/>
+      </c>
+      <c r="N392" s="18">
+        <f>IF(J392=0,"",L392/J392)</f>
+        <v/>
+      </c>
+      <c r="O392" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:42:22</t>
+        </is>
+      </c>
+      <c r="B393" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C393" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D393" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E393" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F393" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G393" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H393" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I393" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7826</t>
+        </is>
+      </c>
+      <c r="J393" s="17" t="n">
+        <v>77795.63174371538</v>
+      </c>
+      <c r="K393" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,022.6150; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L393" s="17" t="n">
+        <v>68000.92527797121</v>
+      </c>
+      <c r="M393" s="17">
+        <f>J393-L393</f>
+        <v/>
+      </c>
+      <c r="N393" s="18">
+        <f>IF(J393=0,"",L393/J393)</f>
+        <v/>
+      </c>
+      <c r="O393" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:42:22</t>
+        </is>
+      </c>
+      <c r="B394" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C394" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D394" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E394" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F394" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G394" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H394" s="16" t="n">
+        <v>1.1285</v>
+      </c>
+      <c r="I394" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J394" s="17" t="n">
+        <v>197095.9588007503</v>
+      </c>
+      <c r="K394" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,228.5848</t>
+        </is>
+      </c>
+      <c r="L394" s="17" t="n">
+        <v>150243.6091312141</v>
+      </c>
+      <c r="M394" s="17">
+        <f>J394-L394</f>
+        <v/>
+      </c>
+      <c r="N394" s="18">
+        <f>IF(J394=0,"",L394/J394)</f>
+        <v/>
+      </c>
+      <c r="O394" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:42:22</t>
+        </is>
+      </c>
+      <c r="B395" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C395" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D395" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E395" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F395" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G395" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H395" s="16" t="n">
+        <v>1.0528</v>
+      </c>
+      <c r="I395" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J395" s="17" t="n">
+        <v>186028.3206748245</v>
+      </c>
+      <c r="K395" s="15" t="inlineStr">
+        <is>
+          <t>USDC 161,827.6712</t>
+        </is>
+      </c>
+      <c r="L395" s="17" t="n">
+        <v>161843.8556121311</v>
+      </c>
+      <c r="M395" s="17">
+        <f>J395-L395</f>
+        <v/>
+      </c>
+      <c r="N395" s="18">
+        <f>IF(J395=0,"",L395/J395)</f>
+        <v/>
+      </c>
+      <c r="O395" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:42:22</t>
+        </is>
+      </c>
+      <c r="B396" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C396" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D396" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E396" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F396" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G396" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H396" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I396" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J396" s="17" t="n">
+        <v>327555.5801417562</v>
+      </c>
+      <c r="K396" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L396" s="17" t="n">
+        <v>280212.7994848645</v>
+      </c>
+      <c r="M396" s="17">
+        <f>J396-L396</f>
+        <v/>
+      </c>
+      <c r="N396" s="18">
+        <f>IF(J396=0,"",L396/J396)</f>
+        <v/>
+      </c>
+      <c r="O396" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:42:22</t>
+        </is>
+      </c>
+      <c r="B397" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C397" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D397" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E397" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F397" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G397" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H397" s="16" t="n">
+        <v>1.1296</v>
+      </c>
+      <c r="I397" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J397" s="17" t="n">
+        <v>160005.8938187637</v>
+      </c>
+      <c r="K397" s="15" t="inlineStr">
+        <is>
+          <t>USDC 119,566.4850</t>
+        </is>
+      </c>
+      <c r="L397" s="17" t="n">
+        <v>119578.4428387121</v>
+      </c>
+      <c r="M397" s="17">
+        <f>J397-L397</f>
+        <v/>
+      </c>
+      <c r="N397" s="18">
+        <f>IF(J397=0,"",L397/J397)</f>
+        <v/>
+      </c>
+      <c r="O397" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:42:22</t>
+        </is>
+      </c>
+      <c r="B398" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C398" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D398" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E398" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F398" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G398" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H398" s="16" t="n">
+        <v>1.0575</v>
+      </c>
+      <c r="I398" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J398" s="17" t="n">
+        <v>160126.1247228362</v>
+      </c>
+      <c r="K398" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,514.6077</t>
+        </is>
+      </c>
+      <c r="L398" s="17" t="n">
+        <v>138473.0533105034</v>
+      </c>
+      <c r="M398" s="17">
+        <f>J398-L398</f>
+        <v/>
+      </c>
+      <c r="N398" s="18">
+        <f>IF(J398=0,"",L398/J398)</f>
+        <v/>
+      </c>
+      <c r="O398" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:42:22</t>
+        </is>
+      </c>
+      <c r="B399" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C399" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D399" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E399" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F399" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeef003c</t>
+        </is>
+      </c>
+      <c r="G399" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H399" s="16" t="inlineStr"/>
+      <c r="I399" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,801.5319</t>
+        </is>
+      </c>
+      <c r="J399" s="17" t="n">
+        <v>50785.27542378752</v>
+      </c>
+      <c r="K399" s="15" t="inlineStr"/>
+      <c r="L399" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M399" s="17">
+        <f>J399-L399</f>
+        <v/>
+      </c>
+      <c r="N399" s="18">
+        <f>IF(J399=0,"",L399/J399)</f>
+        <v/>
+      </c>
+      <c r="O399" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:42:22</t>
+        </is>
+      </c>
+      <c r="B400" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C400" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D400" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E400" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F400" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeeff047</t>
+        </is>
+      </c>
+      <c r="G400" s="15" t="inlineStr">
+        <is>
+          <t>USDC vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H400" s="16" t="inlineStr"/>
+      <c r="I400" s="15" t="inlineStr">
+        <is>
+          <t>USDC 48,647.3916</t>
+        </is>
+      </c>
+      <c r="J400" s="17" t="n">
+        <v>48652.25680268027</v>
+      </c>
+      <c r="K400" s="15" t="inlineStr"/>
+      <c r="L400" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M400" s="17">
+        <f>J400-L400</f>
+        <v/>
+      </c>
+      <c r="N400" s="18">
+        <f>IF(J400=0,"",L400/J400)</f>
+        <v/>
+      </c>
+      <c r="O400" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:42:22</t>
+        </is>
+      </c>
+      <c r="B401" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C401" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D401" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E401" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F401" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G401" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H401" s="16" t="inlineStr"/>
+      <c r="I401" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J401" s="17" t="n">
+        <v>95873.39753982412</v>
+      </c>
+      <c r="K401" s="15" t="inlineStr"/>
+      <c r="L401" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M401" s="17">
+        <f>J401-L401</f>
+        <v/>
+      </c>
+      <c r="N401" s="18">
+        <f>IF(J401=0,"",L401/J401)</f>
+        <v/>
+      </c>
+      <c r="O401" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:42:22</t>
+        </is>
+      </c>
+      <c r="B402" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C402" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D402" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E402" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F402" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G402" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H402" s="16" t="inlineStr"/>
+      <c r="I402" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J402" s="17" t="n">
+        <v>34342.65065108767</v>
+      </c>
+      <c r="K402" s="15" t="inlineStr"/>
+      <c r="L402" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M402" s="17">
+        <f>J402-L402</f>
+        <v/>
+      </c>
+      <c r="N402" s="18">
+        <f>IF(J402=0,"",L402/J402)</f>
+        <v/>
+      </c>
+      <c r="O402" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:42:22</t>
+        </is>
+      </c>
+      <c r="B403" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C403" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D403" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E403" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F403" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G403" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H403" s="16" t="n">
+        <v>1.0431</v>
+      </c>
+      <c r="I403" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J403" s="17" t="n">
+        <v>269988.2547897112</v>
+      </c>
+      <c r="K403" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,031.5881</t>
+        </is>
+      </c>
+      <c r="L403" s="17" t="n">
+        <v>232957.0180267968</v>
+      </c>
+      <c r="M403" s="17">
+        <f>J403-L403</f>
+        <v/>
+      </c>
+      <c r="N403" s="18">
+        <f>IF(J403=0,"",L403/J403)</f>
+        <v/>
+      </c>
+      <c r="O403" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:42:22</t>
+        </is>
+      </c>
+      <c r="B404" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C404" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D404" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E404" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F404" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G404" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H404" s="16" t="inlineStr"/>
+      <c r="I404" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,508.1587</t>
+        </is>
+      </c>
+      <c r="J404" s="17" t="n">
+        <v>15503.1960494156</v>
+      </c>
+      <c r="K404" s="15" t="inlineStr"/>
+      <c r="L404" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M404" s="17">
+        <f>J404-L404</f>
+        <v/>
+      </c>
+      <c r="N404" s="18">
+        <f>IF(J404=0,"",L404/J404)</f>
+        <v/>
+      </c>
+      <c r="O404" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -26641,7 +27646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -27637,6 +28642,41 @@
         <v>1.0375</v>
       </c>
       <c r="I28" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 05:42:22</t>
+        </is>
+      </c>
+      <c r="B29" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C29" s="17" t="n">
+        <v>553580.2534061192</v>
+      </c>
+      <c r="D29" s="17" t="n">
+        <v>550963.7612177199</v>
+      </c>
+      <c r="E29" s="17" t="n">
+        <v>2479322.022122448</v>
+      </c>
+      <c r="F29" s="17" t="n">
+        <v>1928358.260904728</v>
+      </c>
+      <c r="G29" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="H29" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I29" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 06:43 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O404"/>
+  <dimension ref="A1:O419"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -27616,6 +27616,1011 @@
         <v/>
       </c>
       <c r="O404" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 06:43:36</t>
+        </is>
+      </c>
+      <c r="B405" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C405" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D405" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E405" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F405" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G405" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H405" s="16" t="n">
+        <v>1.048</v>
+      </c>
+      <c r="I405" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J405" s="17" t="n">
+        <v>140923.1370848467</v>
+      </c>
+      <c r="K405" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,031.5767</t>
+        </is>
+      </c>
+      <c r="L405" s="17" t="n">
+        <v>121017.0529267941</v>
+      </c>
+      <c r="M405" s="17">
+        <f>J405-L405</f>
+        <v/>
+      </c>
+      <c r="N405" s="18">
+        <f>IF(J405=0,"",L405/J405)</f>
+        <v/>
+      </c>
+      <c r="O405" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 06:43:36</t>
+        </is>
+      </c>
+      <c r="B406" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C406" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D406" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E406" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F406" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G406" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H406" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I406" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J406" s="17" t="n">
+        <v>328705.4957147553</v>
+      </c>
+      <c r="K406" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,382.2278</t>
+        </is>
+      </c>
+      <c r="L406" s="17" t="n">
+        <v>306431.08034998</v>
+      </c>
+      <c r="M406" s="17">
+        <f>J406-L406</f>
+        <v/>
+      </c>
+      <c r="N406" s="18">
+        <f>IF(J406=0,"",L406/J406)</f>
+        <v/>
+      </c>
+      <c r="O406" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 06:43:36</t>
+        </is>
+      </c>
+      <c r="B407" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C407" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D407" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E407" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F407" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G407" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H407" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I407" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J407" s="17" t="n">
+        <v>386044.5635815085</v>
+      </c>
+      <c r="K407" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,602.3431</t>
+        </is>
+      </c>
+      <c r="L407" s="17" t="n">
+        <v>349658.0870666757</v>
+      </c>
+      <c r="M407" s="17">
+        <f>J407-L407</f>
+        <v/>
+      </c>
+      <c r="N407" s="18">
+        <f>IF(J407=0,"",L407/J407)</f>
+        <v/>
+      </c>
+      <c r="O407" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 06:43:36</t>
+        </is>
+      </c>
+      <c r="B408" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C408" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D408" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E408" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F408" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G408" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H408" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I408" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7842</t>
+        </is>
+      </c>
+      <c r="J408" s="17" t="n">
+        <v>77806.49098298652</v>
+      </c>
+      <c r="K408" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,026.6816; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L408" s="17" t="n">
+        <v>68018.59592821136</v>
+      </c>
+      <c r="M408" s="17">
+        <f>J408-L408</f>
+        <v/>
+      </c>
+      <c r="N408" s="18">
+        <f>IF(J408=0,"",L408/J408)</f>
+        <v/>
+      </c>
+      <c r="O408" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 06:43:36</t>
+        </is>
+      </c>
+      <c r="B409" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C409" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D409" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E409" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F409" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G409" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H409" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I409" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J409" s="17" t="n">
+        <v>197098.8893611626</v>
+      </c>
+      <c r="K409" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,242.8959</t>
+        </is>
+      </c>
+      <c r="L409" s="17" t="n">
+        <v>150257.9217081781</v>
+      </c>
+      <c r="M409" s="17">
+        <f>J409-L409</f>
+        <v/>
+      </c>
+      <c r="N409" s="18">
+        <f>IF(J409=0,"",L409/J409)</f>
+        <v/>
+      </c>
+      <c r="O409" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 06:43:36</t>
+        </is>
+      </c>
+      <c r="B410" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C410" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D410" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E410" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F410" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G410" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H410" s="16" t="n">
+        <v>1.0527</v>
+      </c>
+      <c r="I410" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J410" s="17" t="n">
+        <v>186104.1620661334</v>
+      </c>
+      <c r="K410" s="15" t="inlineStr">
+        <is>
+          <t>USDC 161,854.7536</t>
+        </is>
+      </c>
+      <c r="L410" s="17" t="n">
+        <v>161870.9407238165</v>
+      </c>
+      <c r="M410" s="17">
+        <f>J410-L410</f>
+        <v/>
+      </c>
+      <c r="N410" s="18">
+        <f>IF(J410=0,"",L410/J410)</f>
+        <v/>
+      </c>
+      <c r="O410" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 06:43:36</t>
+        </is>
+      </c>
+      <c r="B411" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C411" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D411" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E411" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F411" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G411" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H411" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I411" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J411" s="17" t="n">
+        <v>327616.1975722574</v>
+      </c>
+      <c r="K411" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L411" s="17" t="n">
+        <v>280262.6969285922</v>
+      </c>
+      <c r="M411" s="17">
+        <f>J411-L411</f>
+        <v/>
+      </c>
+      <c r="N411" s="18">
+        <f>IF(J411=0,"",L411/J411)</f>
+        <v/>
+      </c>
+      <c r="O411" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 06:43:36</t>
+        </is>
+      </c>
+      <c r="B412" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C412" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D412" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E412" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F412" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G412" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H412" s="16" t="n">
+        <v>1.1298</v>
+      </c>
+      <c r="I412" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J412" s="17" t="n">
+        <v>160005.8938187637</v>
+      </c>
+      <c r="K412" s="15" t="inlineStr">
+        <is>
+          <t>USDC 119,582.1396</t>
+        </is>
+      </c>
+      <c r="L412" s="17" t="n">
+        <v>119594.0990013717</v>
+      </c>
+      <c r="M412" s="17">
+        <f>J412-L412</f>
+        <v/>
+      </c>
+      <c r="N412" s="18">
+        <f>IF(J412=0,"",L412/J412)</f>
+        <v/>
+      </c>
+      <c r="O412" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 06:43:36</t>
+        </is>
+      </c>
+      <c r="B413" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C413" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D413" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E413" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F413" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G413" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H413" s="16" t="n">
+        <v>1.0575</v>
+      </c>
+      <c r="I413" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J413" s="17" t="n">
+        <v>160159.4433440502</v>
+      </c>
+      <c r="K413" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,520.1778</t>
+        </is>
+      </c>
+      <c r="L413" s="17" t="n">
+        <v>138492.4737949295</v>
+      </c>
+      <c r="M413" s="17">
+        <f>J413-L413</f>
+        <v/>
+      </c>
+      <c r="N413" s="18">
+        <f>IF(J413=0,"",L413/J413)</f>
+        <v/>
+      </c>
+      <c r="O413" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 06:43:36</t>
+        </is>
+      </c>
+      <c r="B414" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C414" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D414" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E414" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F414" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeef003c</t>
+        </is>
+      </c>
+      <c r="G414" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H414" s="16" t="inlineStr"/>
+      <c r="I414" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,803.6760</t>
+        </is>
+      </c>
+      <c r="J414" s="17" t="n">
+        <v>50797.57960287472</v>
+      </c>
+      <c r="K414" s="15" t="inlineStr"/>
+      <c r="L414" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M414" s="17">
+        <f>J414-L414</f>
+        <v/>
+      </c>
+      <c r="N414" s="18">
+        <f>IF(J414=0,"",L414/J414)</f>
+        <v/>
+      </c>
+      <c r="O414" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 06:43:36</t>
+        </is>
+      </c>
+      <c r="B415" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C415" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D415" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E415" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F415" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeeff047</t>
+        </is>
+      </c>
+      <c r="G415" s="15" t="inlineStr">
+        <is>
+          <t>USDC vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H415" s="16" t="inlineStr"/>
+      <c r="I415" s="15" t="inlineStr">
+        <is>
+          <t>USDC 48,649.8115</t>
+        </is>
+      </c>
+      <c r="J415" s="17" t="n">
+        <v>48654.67691969197</v>
+      </c>
+      <c r="K415" s="15" t="inlineStr"/>
+      <c r="L415" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M415" s="17">
+        <f>J415-L415</f>
+        <v/>
+      </c>
+      <c r="N415" s="18">
+        <f>IF(J415=0,"",L415/J415)</f>
+        <v/>
+      </c>
+      <c r="O415" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 06:43:36</t>
+        </is>
+      </c>
+      <c r="B416" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C416" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D416" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E416" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F416" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G416" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H416" s="16" t="inlineStr"/>
+      <c r="I416" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J416" s="17" t="n">
+        <v>95912.29247918157</v>
+      </c>
+      <c r="K416" s="15" t="inlineStr"/>
+      <c r="L416" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M416" s="17">
+        <f>J416-L416</f>
+        <v/>
+      </c>
+      <c r="N416" s="18">
+        <f>IF(J416=0,"",L416/J416)</f>
+        <v/>
+      </c>
+      <c r="O416" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 06:43:36</t>
+        </is>
+      </c>
+      <c r="B417" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C417" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D417" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E417" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F417" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G417" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H417" s="16" t="inlineStr"/>
+      <c r="I417" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J417" s="17" t="n">
+        <v>34343.14159613344</v>
+      </c>
+      <c r="K417" s="15" t="inlineStr"/>
+      <c r="L417" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M417" s="17">
+        <f>J417-L417</f>
+        <v/>
+      </c>
+      <c r="N417" s="18">
+        <f>IF(J417=0,"",L417/J417)</f>
+        <v/>
+      </c>
+      <c r="O417" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 06:43:36</t>
+        </is>
+      </c>
+      <c r="B418" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C418" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D418" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E418" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F418" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G418" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H418" s="16" t="n">
+        <v>1.0428</v>
+      </c>
+      <c r="I418" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J418" s="17" t="n">
+        <v>269988.2547897112</v>
+      </c>
+      <c r="K418" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,033.8811</t>
+        </is>
+      </c>
+      <c r="L418" s="17" t="n">
+        <v>233005.9170542656</v>
+      </c>
+      <c r="M418" s="17">
+        <f>J418-L418</f>
+        <v/>
+      </c>
+      <c r="N418" s="18">
+        <f>IF(J418=0,"",L418/J418)</f>
+        <v/>
+      </c>
+      <c r="O418" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 06:43:36</t>
+        </is>
+      </c>
+      <c r="B419" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C419" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D419" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E419" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F419" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G419" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H419" s="16" t="inlineStr"/>
+      <c r="I419" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,508.3816</t>
+        </is>
+      </c>
+      <c r="J419" s="17" t="n">
+        <v>15506.52057204125</v>
+      </c>
+      <c r="K419" s="15" t="inlineStr"/>
+      <c r="L419" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M419" s="17">
+        <f>J419-L419</f>
+        <v/>
+      </c>
+      <c r="N419" s="18">
+        <f>IF(J419=0,"",L419/J419)</f>
+        <v/>
+      </c>
+      <c r="O419" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -27646,7 +28651,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -28677,6 +29682,41 @@
         <v>1.0375</v>
       </c>
       <c r="I29" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 06:43:36</t>
+        </is>
+      </c>
+      <c r="B30" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C30" s="17" t="n">
+        <v>553677.1247883895</v>
+      </c>
+      <c r="D30" s="17" t="n">
+        <v>551057.8740032837</v>
+      </c>
+      <c r="E30" s="17" t="n">
+        <v>2479666.739486098</v>
+      </c>
+      <c r="F30" s="17" t="n">
+        <v>1928608.865482815</v>
+      </c>
+      <c r="G30" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="H30" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I30" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 07:13 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O419"/>
+  <dimension ref="A1:O449"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -28621,6 +28621,2016 @@
         <v/>
       </c>
       <c r="O419" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:01:12</t>
+        </is>
+      </c>
+      <c r="B420" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C420" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D420" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E420" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F420" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G420" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H420" s="16" t="n">
+        <v>1.0482</v>
+      </c>
+      <c r="I420" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J420" s="17" t="n">
+        <v>140937.5167591604</v>
+      </c>
+      <c r="K420" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,031.5767</t>
+        </is>
+      </c>
+      <c r="L420" s="17" t="n">
+        <v>121015.8426110269</v>
+      </c>
+      <c r="M420" s="17">
+        <f>J420-L420</f>
+        <v/>
+      </c>
+      <c r="N420" s="18">
+        <f>IF(J420=0,"",L420/J420)</f>
+        <v/>
+      </c>
+      <c r="O420" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:01:12</t>
+        </is>
+      </c>
+      <c r="B421" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C421" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D421" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E421" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F421" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G421" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H421" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I421" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J421" s="17" t="n">
+        <v>328706.2278705448</v>
+      </c>
+      <c r="K421" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,382.2278</t>
+        </is>
+      </c>
+      <c r="L421" s="17" t="n">
+        <v>306461.6742472709</v>
+      </c>
+      <c r="M421" s="17">
+        <f>J421-L421</f>
+        <v/>
+      </c>
+      <c r="N421" s="18">
+        <f>IF(J421=0,"",L421/J421)</f>
+        <v/>
+      </c>
+      <c r="O421" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:01:12</t>
+        </is>
+      </c>
+      <c r="B422" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C422" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D422" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E422" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F422" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G422" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H422" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I422" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J422" s="17" t="n">
+        <v>386044.5635815085</v>
+      </c>
+      <c r="K422" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,602.3431</t>
+        </is>
+      </c>
+      <c r="L422" s="17" t="n">
+        <v>349692.9967226755</v>
+      </c>
+      <c r="M422" s="17">
+        <f>J422-L422</f>
+        <v/>
+      </c>
+      <c r="N422" s="18">
+        <f>IF(J422=0,"",L422/J422)</f>
+        <v/>
+      </c>
+      <c r="O422" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:01:12</t>
+        </is>
+      </c>
+      <c r="B423" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C423" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D423" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E423" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F423" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G423" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H423" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I423" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7843</t>
+        </is>
+      </c>
+      <c r="J423" s="17" t="n">
+        <v>77806.45947632685</v>
+      </c>
+      <c r="K423" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,026.9892; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L423" s="17" t="n">
+        <v>68018.22330715432</v>
+      </c>
+      <c r="M423" s="17">
+        <f>J423-L423</f>
+        <v/>
+      </c>
+      <c r="N423" s="18">
+        <f>IF(J423=0,"",L423/J423)</f>
+        <v/>
+      </c>
+      <c r="O423" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:01:12</t>
+        </is>
+      </c>
+      <c r="B424" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C424" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D424" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E424" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F424" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G424" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H424" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I424" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J424" s="17" t="n">
+        <v>197100.6872366178</v>
+      </c>
+      <c r="K424" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,242.8959</t>
+        </is>
+      </c>
+      <c r="L424" s="17" t="n">
+        <v>150257.9217081781</v>
+      </c>
+      <c r="M424" s="17">
+        <f>J424-L424</f>
+        <v/>
+      </c>
+      <c r="N424" s="18">
+        <f>IF(J424=0,"",L424/J424)</f>
+        <v/>
+      </c>
+      <c r="O424" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:01:12</t>
+        </is>
+      </c>
+      <c r="B425" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C425" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D425" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E425" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F425" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G425" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H425" s="16" t="n">
+        <v>1.0527</v>
+      </c>
+      <c r="I425" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J425" s="17" t="n">
+        <v>186071.4879427598</v>
+      </c>
+      <c r="K425" s="15" t="inlineStr">
+        <is>
+          <t>USDC 161,854.7536</t>
+        </is>
+      </c>
+      <c r="L425" s="17" t="n">
+        <v>161870.9407238165</v>
+      </c>
+      <c r="M425" s="17">
+        <f>J425-L425</f>
+        <v/>
+      </c>
+      <c r="N425" s="18">
+        <f>IF(J425=0,"",L425/J425)</f>
+        <v/>
+      </c>
+      <c r="O425" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:01:12</t>
+        </is>
+      </c>
+      <c r="B426" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C426" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D426" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E426" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F426" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G426" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H426" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I426" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J426" s="17" t="n">
+        <v>327645.3596202203</v>
+      </c>
+      <c r="K426" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L426" s="17" t="n">
+        <v>280290.7252219897</v>
+      </c>
+      <c r="M426" s="17">
+        <f>J426-L426</f>
+        <v/>
+      </c>
+      <c r="N426" s="18">
+        <f>IF(J426=0,"",L426/J426)</f>
+        <v/>
+      </c>
+      <c r="O426" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:01:12</t>
+        </is>
+      </c>
+      <c r="B427" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C427" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D427" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E427" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F427" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G427" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H427" s="16" t="n">
+        <v>1.1298</v>
+      </c>
+      <c r="I427" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J427" s="17" t="n">
+        <v>159973.89264</v>
+      </c>
+      <c r="K427" s="15" t="inlineStr">
+        <is>
+          <t>USDC 119,582.1396</t>
+        </is>
+      </c>
+      <c r="L427" s="17" t="n">
+        <v>119594.0990013717</v>
+      </c>
+      <c r="M427" s="17">
+        <f>J427-L427</f>
+        <v/>
+      </c>
+      <c r="N427" s="18">
+        <f>IF(J427=0,"",L427/J427)</f>
+        <v/>
+      </c>
+      <c r="O427" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:01:12</t>
+        </is>
+      </c>
+      <c r="B428" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C428" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D428" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E428" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F428" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G428" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H428" s="16" t="n">
+        <v>1.0575</v>
+      </c>
+      <c r="I428" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J428" s="17" t="n">
+        <v>160159.4433440502</v>
+      </c>
+      <c r="K428" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,520.1778</t>
+        </is>
+      </c>
+      <c r="L428" s="17" t="n">
+        <v>138492.4737949295</v>
+      </c>
+      <c r="M428" s="17">
+        <f>J428-L428</f>
+        <v/>
+      </c>
+      <c r="N428" s="18">
+        <f>IF(J428=0,"",L428/J428)</f>
+        <v/>
+      </c>
+      <c r="O428" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:01:12</t>
+        </is>
+      </c>
+      <c r="B429" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C429" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D429" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E429" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F429" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeef003c</t>
+        </is>
+      </c>
+      <c r="G429" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H429" s="16" t="inlineStr"/>
+      <c r="I429" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,803.6760</t>
+        </is>
+      </c>
+      <c r="J429" s="17" t="n">
+        <v>50797.07156611428</v>
+      </c>
+      <c r="K429" s="15" t="inlineStr"/>
+      <c r="L429" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M429" s="17">
+        <f>J429-L429</f>
+        <v/>
+      </c>
+      <c r="N429" s="18">
+        <f>IF(J429=0,"",L429/J429)</f>
+        <v/>
+      </c>
+      <c r="O429" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:01:12</t>
+        </is>
+      </c>
+      <c r="B430" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C430" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D430" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E430" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F430" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeeff047</t>
+        </is>
+      </c>
+      <c r="G430" s="15" t="inlineStr">
+        <is>
+          <t>USDC vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H430" s="16" t="inlineStr"/>
+      <c r="I430" s="15" t="inlineStr">
+        <is>
+          <t>USDC 48,649.8115</t>
+        </is>
+      </c>
+      <c r="J430" s="17" t="n">
+        <v>48654.67691969197</v>
+      </c>
+      <c r="K430" s="15" t="inlineStr"/>
+      <c r="L430" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M430" s="17">
+        <f>J430-L430</f>
+        <v/>
+      </c>
+      <c r="N430" s="18">
+        <f>IF(J430=0,"",L430/J430)</f>
+        <v/>
+      </c>
+      <c r="O430" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:01:12</t>
+        </is>
+      </c>
+      <c r="B431" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C431" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D431" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E431" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F431" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G431" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H431" s="16" t="inlineStr"/>
+      <c r="I431" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J431" s="17" t="n">
+        <v>95904.64029486699</v>
+      </c>
+      <c r="K431" s="15" t="inlineStr"/>
+      <c r="L431" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M431" s="17">
+        <f>J431-L431</f>
+        <v/>
+      </c>
+      <c r="N431" s="18">
+        <f>IF(J431=0,"",L431/J431)</f>
+        <v/>
+      </c>
+      <c r="O431" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:01:12</t>
+        </is>
+      </c>
+      <c r="B432" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C432" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D432" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E432" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F432" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G432" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H432" s="16" t="inlineStr"/>
+      <c r="I432" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J432" s="17" t="n">
+        <v>34343.41718546145</v>
+      </c>
+      <c r="K432" s="15" t="inlineStr"/>
+      <c r="L432" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M432" s="17">
+        <f>J432-L432</f>
+        <v/>
+      </c>
+      <c r="N432" s="18">
+        <f>IF(J432=0,"",L432/J432)</f>
+        <v/>
+      </c>
+      <c r="O432" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:01:12</t>
+        </is>
+      </c>
+      <c r="B433" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C433" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D433" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E433" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F433" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G433" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H433" s="16" t="n">
+        <v>1.043</v>
+      </c>
+      <c r="I433" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J433" s="17" t="n">
+        <v>270015.2563153427</v>
+      </c>
+      <c r="K433" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,033.8811</t>
+        </is>
+      </c>
+      <c r="L433" s="17" t="n">
+        <v>233003.5867154544</v>
+      </c>
+      <c r="M433" s="17">
+        <f>J433-L433</f>
+        <v/>
+      </c>
+      <c r="N433" s="18">
+        <f>IF(J433=0,"",L433/J433)</f>
+        <v/>
+      </c>
+      <c r="O433" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:01:12</t>
+        </is>
+      </c>
+      <c r="B434" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C434" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D434" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E434" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F434" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G434" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H434" s="16" t="inlineStr"/>
+      <c r="I434" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,508.5828</t>
+        </is>
+      </c>
+      <c r="J434" s="17" t="n">
+        <v>15506.56670559425</v>
+      </c>
+      <c r="K434" s="15" t="inlineStr"/>
+      <c r="L434" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M434" s="17">
+        <f>J434-L434</f>
+        <v/>
+      </c>
+      <c r="N434" s="18">
+        <f>IF(J434=0,"",L434/J434)</f>
+        <v/>
+      </c>
+      <c r="O434" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:13:42</t>
+        </is>
+      </c>
+      <c r="B435" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C435" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D435" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E435" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F435" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G435" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H435" s="16" t="n">
+        <v>1.0481</v>
+      </c>
+      <c r="I435" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J435" s="17" t="n">
+        <v>140937.5167591604</v>
+      </c>
+      <c r="K435" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,031.5767</t>
+        </is>
+      </c>
+      <c r="L435" s="17" t="n">
+        <v>121017.0529267941</v>
+      </c>
+      <c r="M435" s="17">
+        <f>J435-L435</f>
+        <v/>
+      </c>
+      <c r="N435" s="18">
+        <f>IF(J435=0,"",L435/J435)</f>
+        <v/>
+      </c>
+      <c r="O435" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:13:42</t>
+        </is>
+      </c>
+      <c r="B436" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C436" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D436" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E436" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F436" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G436" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H436" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I436" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J436" s="17" t="n">
+        <v>328706.2278705448</v>
+      </c>
+      <c r="K436" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,382.2278</t>
+        </is>
+      </c>
+      <c r="L436" s="17" t="n">
+        <v>306431.0280798462</v>
+      </c>
+      <c r="M436" s="17">
+        <f>J436-L436</f>
+        <v/>
+      </c>
+      <c r="N436" s="18">
+        <f>IF(J436=0,"",L436/J436)</f>
+        <v/>
+      </c>
+      <c r="O436" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:13:42</t>
+        </is>
+      </c>
+      <c r="B437" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C437" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D437" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E437" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F437" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G437" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H437" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I437" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J437" s="17" t="n">
+        <v>386006.3275407022</v>
+      </c>
+      <c r="K437" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,602.3431</t>
+        </is>
+      </c>
+      <c r="L437" s="17" t="n">
+        <v>349658.0274230032</v>
+      </c>
+      <c r="M437" s="17">
+        <f>J437-L437</f>
+        <v/>
+      </c>
+      <c r="N437" s="18">
+        <f>IF(J437=0,"",L437/J437)</f>
+        <v/>
+      </c>
+      <c r="O437" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:13:42</t>
+        </is>
+      </c>
+      <c r="B438" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C438" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D438" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E438" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F438" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G438" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H438" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I438" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7843</t>
+        </is>
+      </c>
+      <c r="J438" s="17" t="n">
+        <v>77806.44696973043</v>
+      </c>
+      <c r="K438" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,026.9892; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L438" s="17" t="n">
+        <v>68018.90356929012</v>
+      </c>
+      <c r="M438" s="17">
+        <f>J438-L438</f>
+        <v/>
+      </c>
+      <c r="N438" s="18">
+        <f>IF(J438=0,"",L438/J438)</f>
+        <v/>
+      </c>
+      <c r="O438" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:13:42</t>
+        </is>
+      </c>
+      <c r="B439" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C439" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D439" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E439" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F439" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G439" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H439" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I439" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J439" s="17" t="n">
+        <v>197103.9649547567</v>
+      </c>
+      <c r="K439" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,242.8959</t>
+        </is>
+      </c>
+      <c r="L439" s="17" t="n">
+        <v>150242.8959160073</v>
+      </c>
+      <c r="M439" s="17">
+        <f>J439-L439</f>
+        <v/>
+      </c>
+      <c r="N439" s="18">
+        <f>IF(J439=0,"",L439/J439)</f>
+        <v/>
+      </c>
+      <c r="O439" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:13:42</t>
+        </is>
+      </c>
+      <c r="B440" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C440" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D440" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E440" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F440" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G440" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H440" s="16" t="n">
+        <v>1.0527</v>
+      </c>
+      <c r="I440" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J440" s="17" t="n">
+        <v>186071.7743648881</v>
+      </c>
+      <c r="K440" s="15" t="inlineStr">
+        <is>
+          <t>USDC 161,854.7536</t>
+        </is>
+      </c>
+      <c r="L440" s="17" t="n">
+        <v>161854.7536297442</v>
+      </c>
+      <c r="M440" s="17">
+        <f>J440-L440</f>
+        <v/>
+      </c>
+      <c r="N440" s="18">
+        <f>IF(J440=0,"",L440/J440)</f>
+        <v/>
+      </c>
+      <c r="O440" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:13:42</t>
+        </is>
+      </c>
+      <c r="B441" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C441" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D441" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E441" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F441" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G441" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H441" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I441" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J441" s="17" t="n">
+        <v>327645.3596202203</v>
+      </c>
+      <c r="K441" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L441" s="17" t="n">
+        <v>280290.7401899829</v>
+      </c>
+      <c r="M441" s="17">
+        <f>J441-L441</f>
+        <v/>
+      </c>
+      <c r="N441" s="18">
+        <f>IF(J441=0,"",L441/J441)</f>
+        <v/>
+      </c>
+      <c r="O441" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:13:42</t>
+        </is>
+      </c>
+      <c r="B442" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C442" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D442" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E442" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F442" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G442" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H442" s="16" t="n">
+        <v>1.1298</v>
+      </c>
+      <c r="I442" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J442" s="17" t="n">
+        <v>159973.89264</v>
+      </c>
+      <c r="K442" s="15" t="inlineStr">
+        <is>
+          <t>USDC 119,582.1396</t>
+        </is>
+      </c>
+      <c r="L442" s="17" t="n">
+        <v>119582.1395914716</v>
+      </c>
+      <c r="M442" s="17">
+        <f>J442-L442</f>
+        <v/>
+      </c>
+      <c r="N442" s="18">
+        <f>IF(J442=0,"",L442/J442)</f>
+        <v/>
+      </c>
+      <c r="O442" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:13:42</t>
+        </is>
+      </c>
+      <c r="B443" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C443" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D443" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E443" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F443" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G443" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H443" s="16" t="n">
+        <v>1.0575</v>
+      </c>
+      <c r="I443" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J443" s="17" t="n">
+        <v>160143.5802453593</v>
+      </c>
+      <c r="K443" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,520.1778</t>
+        </is>
+      </c>
+      <c r="L443" s="17" t="n">
+        <v>138492.4737949295</v>
+      </c>
+      <c r="M443" s="17">
+        <f>J443-L443</f>
+        <v/>
+      </c>
+      <c r="N443" s="18">
+        <f>IF(J443=0,"",L443/J443)</f>
+        <v/>
+      </c>
+      <c r="O443" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:13:42</t>
+        </is>
+      </c>
+      <c r="B444" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C444" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D444" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E444" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F444" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeef003c</t>
+        </is>
+      </c>
+      <c r="G444" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H444" s="16" t="inlineStr"/>
+      <c r="I444" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,803.6760</t>
+        </is>
+      </c>
+      <c r="J444" s="17" t="n">
+        <v>50797.57960287472</v>
+      </c>
+      <c r="K444" s="15" t="inlineStr"/>
+      <c r="L444" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M444" s="17">
+        <f>J444-L444</f>
+        <v/>
+      </c>
+      <c r="N444" s="18">
+        <f>IF(J444=0,"",L444/J444)</f>
+        <v/>
+      </c>
+      <c r="O444" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:13:42</t>
+        </is>
+      </c>
+      <c r="B445" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C445" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D445" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E445" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F445" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeeff047</t>
+        </is>
+      </c>
+      <c r="G445" s="15" t="inlineStr">
+        <is>
+          <t>USDC vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H445" s="16" t="inlineStr"/>
+      <c r="I445" s="15" t="inlineStr">
+        <is>
+          <t>USDC 48,649.8115</t>
+        </is>
+      </c>
+      <c r="J445" s="17" t="n">
+        <v>48649.811452</v>
+      </c>
+      <c r="K445" s="15" t="inlineStr"/>
+      <c r="L445" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M445" s="17">
+        <f>J445-L445</f>
+        <v/>
+      </c>
+      <c r="N445" s="18">
+        <f>IF(J445=0,"",L445/J445)</f>
+        <v/>
+      </c>
+      <c r="O445" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:13:42</t>
+        </is>
+      </c>
+      <c r="B446" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C446" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D446" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E446" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F446" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G446" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H446" s="16" t="inlineStr"/>
+      <c r="I446" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J446" s="17" t="n">
+        <v>95904.64029486699</v>
+      </c>
+      <c r="K446" s="15" t="inlineStr"/>
+      <c r="L446" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M446" s="17">
+        <f>J446-L446</f>
+        <v/>
+      </c>
+      <c r="N446" s="18">
+        <f>IF(J446=0,"",L446/J446)</f>
+        <v/>
+      </c>
+      <c r="O446" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:13:42</t>
+        </is>
+      </c>
+      <c r="B447" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C447" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D447" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E447" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F447" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G447" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H447" s="16" t="inlineStr"/>
+      <c r="I447" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J447" s="17" t="n">
+        <v>34343.5120909075</v>
+      </c>
+      <c r="K447" s="15" t="inlineStr"/>
+      <c r="L447" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M447" s="17">
+        <f>J447-L447</f>
+        <v/>
+      </c>
+      <c r="N447" s="18">
+        <f>IF(J447=0,"",L447/J447)</f>
+        <v/>
+      </c>
+      <c r="O447" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:13:42</t>
+        </is>
+      </c>
+      <c r="B448" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C448" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D448" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E448" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F448" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G448" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H448" s="16" t="n">
+        <v>1.043</v>
+      </c>
+      <c r="I448" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J448" s="17" t="n">
+        <v>270015.2563153427</v>
+      </c>
+      <c r="K448" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,033.8811</t>
+        </is>
+      </c>
+      <c r="L448" s="17" t="n">
+        <v>233005.9170542656</v>
+      </c>
+      <c r="M448" s="17">
+        <f>J448-L448</f>
+        <v/>
+      </c>
+      <c r="N448" s="18">
+        <f>IF(J448=0,"",L448/J448)</f>
+        <v/>
+      </c>
+      <c r="O448" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:13:42</t>
+        </is>
+      </c>
+      <c r="B449" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C449" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D449" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E449" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F449" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G449" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H449" s="16" t="inlineStr"/>
+      <c r="I449" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,508.5828</t>
+        </is>
+      </c>
+      <c r="J449" s="17" t="n">
+        <v>15506.72179142246</v>
+      </c>
+      <c r="K449" s="15" t="inlineStr"/>
+      <c r="L449" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M449" s="17">
+        <f>J449-L449</f>
+        <v/>
+      </c>
+      <c r="N449" s="18">
+        <f>IF(J449=0,"",L449/J449)</f>
+        <v/>
+      </c>
+      <c r="O449" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -28651,7 +30661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -29717,6 +31727,76 @@
         <v>1.0375</v>
       </c>
       <c r="I30" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:01:12</t>
+        </is>
+      </c>
+      <c r="B31" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C31" s="17" t="n">
+        <v>553587.864329559</v>
+      </c>
+      <c r="D31" s="17" t="n">
+        <v>550968.7834043929</v>
+      </c>
+      <c r="E31" s="17" t="n">
+        <v>2479667.267458261</v>
+      </c>
+      <c r="F31" s="17" t="n">
+        <v>1928698.484053868</v>
+      </c>
+      <c r="G31" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="H31" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I31" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:13:42</t>
+        </is>
+      </c>
+      <c r="B32" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C32" s="17" t="n">
+        <v>553637.7591732943</v>
+      </c>
+      <c r="D32" s="17" t="n">
+        <v>551018.6803374421</v>
+      </c>
+      <c r="E32" s="17" t="n">
+        <v>2479612.612512777</v>
+      </c>
+      <c r="F32" s="17" t="n">
+        <v>1928593.932175335</v>
+      </c>
+      <c r="G32" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="H32" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I32" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 07:38 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O209"/>
+  <dimension ref="A1:O224"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -14551,6 +14551,1011 @@
         <v/>
       </c>
       <c r="O209" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:37:42</t>
+        </is>
+      </c>
+      <c r="B210" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C210" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D210" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E210" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F210" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G210" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H210" s="16" t="n">
+        <v>1.048</v>
+      </c>
+      <c r="I210" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J210" s="17" t="n">
+        <v>140923.0871168789</v>
+      </c>
+      <c r="K210" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,032.5316</t>
+        </is>
+      </c>
+      <c r="L210" s="17" t="n">
+        <v>121019.2180375222</v>
+      </c>
+      <c r="M210" s="17">
+        <f>J210-L210</f>
+        <v/>
+      </c>
+      <c r="N210" s="18">
+        <f>IF(J210=0,"",L210/J210)</f>
+        <v/>
+      </c>
+      <c r="O210" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:37:42</t>
+        </is>
+      </c>
+      <c r="B211" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C211" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D211" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E211" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F211" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G211" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H211" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I211" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J211" s="17" t="n">
+        <v>328706.9408865741</v>
+      </c>
+      <c r="K211" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,383.3066</t>
+        </is>
+      </c>
+      <c r="L211" s="17" t="n">
+        <v>306432.7393687018</v>
+      </c>
+      <c r="M211" s="17">
+        <f>J211-L211</f>
+        <v/>
+      </c>
+      <c r="N211" s="18">
+        <f>IF(J211=0,"",L211/J211)</f>
+        <v/>
+      </c>
+      <c r="O211" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:37:42</t>
+        </is>
+      </c>
+      <c r="B212" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C212" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D212" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E212" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F212" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G212" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H212" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I212" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J212" s="17" t="n">
+        <v>386046.4830717298</v>
+      </c>
+      <c r="K212" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,603.9988</t>
+        </is>
+      </c>
+      <c r="L212" s="17" t="n">
+        <v>349660.4049468862</v>
+      </c>
+      <c r="M212" s="17">
+        <f>J212-L212</f>
+        <v/>
+      </c>
+      <c r="N212" s="18">
+        <f>IF(J212=0,"",L212/J212)</f>
+        <v/>
+      </c>
+      <c r="O212" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:37:42</t>
+        </is>
+      </c>
+      <c r="B213" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C213" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D213" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E213" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F213" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G213" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H213" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I213" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7844</t>
+        </is>
+      </c>
+      <c r="J213" s="17" t="n">
+        <v>77805.7099851872</v>
+      </c>
+      <c r="K213" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,027.1079; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L213" s="17" t="n">
+        <v>68019.70247913078</v>
+      </c>
+      <c r="M213" s="17">
+        <f>J213-L213</f>
+        <v/>
+      </c>
+      <c r="N213" s="18">
+        <f>IF(J213=0,"",L213/J213)</f>
+        <v/>
+      </c>
+      <c r="O213" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:37:42</t>
+        </is>
+      </c>
+      <c r="B214" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C214" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D214" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E214" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F214" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G214" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H214" s="16" t="n">
+        <v>1.1288</v>
+      </c>
+      <c r="I214" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J214" s="17" t="n">
+        <v>197106.8645552084</v>
+      </c>
+      <c r="K214" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,243.9962</t>
+        </is>
+      </c>
+      <c r="L214" s="17" t="n">
+        <v>150243.996246735</v>
+      </c>
+      <c r="M214" s="17">
+        <f>J214-L214</f>
+        <v/>
+      </c>
+      <c r="N214" s="18">
+        <f>IF(J214=0,"",L214/J214)</f>
+        <v/>
+      </c>
+      <c r="O214" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:37:42</t>
+        </is>
+      </c>
+      <c r="B215" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C215" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D215" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E215" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F215" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G215" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H215" s="16" t="n">
+        <v>1.0527</v>
+      </c>
+      <c r="I215" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J215" s="17" t="n">
+        <v>186072.3322242796</v>
+      </c>
+      <c r="K215" s="15" t="inlineStr">
+        <is>
+          <t>USDC 161,856.7587</t>
+        </is>
+      </c>
+      <c r="L215" s="17" t="n">
+        <v>161856.7586590647</v>
+      </c>
+      <c r="M215" s="17">
+        <f>J215-L215</f>
+        <v/>
+      </c>
+      <c r="N215" s="18">
+        <f>IF(J215=0,"",L215/J215)</f>
+        <v/>
+      </c>
+      <c r="O215" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:37:42</t>
+        </is>
+      </c>
+      <c r="B216" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C216" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D216" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E216" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F216" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G216" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H216" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I216" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J216" s="17" t="n">
+        <v>327618.1746978707</v>
+      </c>
+      <c r="K216" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L216" s="17" t="n">
+        <v>280262.6860364191</v>
+      </c>
+      <c r="M216" s="17">
+        <f>J216-L216</f>
+        <v/>
+      </c>
+      <c r="N216" s="18">
+        <f>IF(J216=0,"",L216/J216)</f>
+        <v/>
+      </c>
+      <c r="O216" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:37:42</t>
+        </is>
+      </c>
+      <c r="B217" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C217" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D217" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E217" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F217" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G217" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H217" s="16" t="n">
+        <v>1.1298</v>
+      </c>
+      <c r="I217" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J217" s="17" t="n">
+        <v>159973.89264</v>
+      </c>
+      <c r="K217" s="15" t="inlineStr">
+        <is>
+          <t>USDC 119,584.3639</t>
+        </is>
+      </c>
+      <c r="L217" s="17" t="n">
+        <v>119584.3639445559</v>
+      </c>
+      <c r="M217" s="17">
+        <f>J217-L217</f>
+        <v/>
+      </c>
+      <c r="N217" s="18">
+        <f>IF(J217=0,"",L217/J217)</f>
+        <v/>
+      </c>
+      <c r="O217" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:37:42</t>
+        </is>
+      </c>
+      <c r="B218" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C218" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D218" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E218" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F218" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G218" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H218" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I218" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J218" s="17" t="n">
+        <v>160160.2396886031</v>
+      </c>
+      <c r="K218" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,521.1458</t>
+        </is>
+      </c>
+      <c r="L218" s="17" t="n">
+        <v>138493.4415612677</v>
+      </c>
+      <c r="M218" s="17">
+        <f>J218-L218</f>
+        <v/>
+      </c>
+      <c r="N218" s="18">
+        <f>IF(J218=0,"",L218/J218)</f>
+        <v/>
+      </c>
+      <c r="O218" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:37:42</t>
+        </is>
+      </c>
+      <c r="B219" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C219" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D219" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E219" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F219" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeef003c</t>
+        </is>
+      </c>
+      <c r="G219" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H219" s="16" t="inlineStr"/>
+      <c r="I219" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,803.9136</t>
+        </is>
+      </c>
+      <c r="J219" s="17" t="n">
+        <v>50798.32513050829</v>
+      </c>
+      <c r="K219" s="15" t="inlineStr"/>
+      <c r="L219" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M219" s="17">
+        <f>J219-L219</f>
+        <v/>
+      </c>
+      <c r="N219" s="18">
+        <f>IF(J219=0,"",L219/J219)</f>
+        <v/>
+      </c>
+      <c r="O219" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:37:42</t>
+        </is>
+      </c>
+      <c r="B220" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C220" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D220" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E220" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F220" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeeff047</t>
+        </is>
+      </c>
+      <c r="G220" s="15" t="inlineStr">
+        <is>
+          <t>USDC vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H220" s="16" t="inlineStr"/>
+      <c r="I220" s="15" t="inlineStr">
+        <is>
+          <t>USDC 48,650.0864</t>
+        </is>
+      </c>
+      <c r="J220" s="17" t="n">
+        <v>48650.086392</v>
+      </c>
+      <c r="K220" s="15" t="inlineStr"/>
+      <c r="L220" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M220" s="17">
+        <f>J220-L220</f>
+        <v/>
+      </c>
+      <c r="N220" s="18">
+        <f>IF(J220=0,"",L220/J220)</f>
+        <v/>
+      </c>
+      <c r="O220" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:37:42</t>
+        </is>
+      </c>
+      <c r="B221" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C221" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D221" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E221" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F221" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G221" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H221" s="16" t="inlineStr"/>
+      <c r="I221" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J221" s="17" t="n">
+        <v>95895.0498308375</v>
+      </c>
+      <c r="K221" s="15" t="inlineStr"/>
+      <c r="L221" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M221" s="17">
+        <f>J221-L221</f>
+        <v/>
+      </c>
+      <c r="N221" s="18">
+        <f>IF(J221=0,"",L221/J221)</f>
+        <v/>
+      </c>
+      <c r="O221" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:37:42</t>
+        </is>
+      </c>
+      <c r="B222" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C222" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D222" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E222" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F222" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G222" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H222" s="16" t="inlineStr"/>
+      <c r="I222" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J222" s="17" t="n">
+        <v>34343.69460211784</v>
+      </c>
+      <c r="K222" s="15" t="inlineStr"/>
+      <c r="L222" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M222" s="17">
+        <f>J222-L222</f>
+        <v/>
+      </c>
+      <c r="N222" s="18">
+        <f>IF(J222=0,"",L222/J222)</f>
+        <v/>
+      </c>
+      <c r="O222" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:37:42</t>
+        </is>
+      </c>
+      <c r="B223" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C223" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D223" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E223" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F223" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G223" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H223" s="16" t="n">
+        <v>1.0428</v>
+      </c>
+      <c r="I223" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J223" s="17" t="n">
+        <v>269992.7871700212</v>
+      </c>
+      <c r="K223" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,036.0347</t>
+        </is>
+      </c>
+      <c r="L223" s="17" t="n">
+        <v>233010.4007731789</v>
+      </c>
+      <c r="M223" s="17">
+        <f>J223-L223</f>
+        <v/>
+      </c>
+      <c r="N223" s="18">
+        <f>IF(J223=0,"",L223/J223)</f>
+        <v/>
+      </c>
+      <c r="O223" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:37:42</t>
+        </is>
+      </c>
+      <c r="B224" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C224" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D224" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E224" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F224" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G224" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H224" s="16" t="inlineStr"/>
+      <c r="I224" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,508.7870</t>
+        </is>
+      </c>
+      <c r="J224" s="17" t="n">
+        <v>15507.08101815625</v>
+      </c>
+      <c r="K224" s="15" t="inlineStr"/>
+      <c r="L224" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M224" s="17">
+        <f>J224-L224</f>
+        <v/>
+      </c>
+      <c r="N224" s="18">
+        <f>IF(J224=0,"",L224/J224)</f>
+        <v/>
+      </c>
+      <c r="O224" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -14581,7 +15586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -15157,6 +16162,41 @@
         <v>1.0375</v>
       </c>
       <c r="I16" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:37:42</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="n">
+        <v>553636.2746545596</v>
+      </c>
+      <c r="D17" s="17" t="n">
+        <v>551017.0369565105</v>
+      </c>
+      <c r="E17" s="17" t="n">
+        <v>2479600.749009973</v>
+      </c>
+      <c r="F17" s="17" t="n">
+        <v>1928583.712053462</v>
+      </c>
+      <c r="G17" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="H17" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I17" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 07:43 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O449"/>
+  <dimension ref="A1:O467"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -30631,6 +30631,1208 @@
         <v/>
       </c>
       <c r="O449" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:43:52</t>
+        </is>
+      </c>
+      <c r="B450" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C450" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D450" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E450" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F450" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G450" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H450" s="16" t="n">
+        <v>1.048</v>
+      </c>
+      <c r="I450" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J450" s="17" t="n">
+        <v>140923.0871168789</v>
+      </c>
+      <c r="K450" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,032.5316</t>
+        </is>
+      </c>
+      <c r="L450" s="17" t="n">
+        <v>121018.0077122061</v>
+      </c>
+      <c r="M450" s="17">
+        <f>J450-L450</f>
+        <v/>
+      </c>
+      <c r="N450" s="18">
+        <f>IF(J450=0,"",L450/J450)</f>
+        <v/>
+      </c>
+      <c r="O450" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:43:52</t>
+        </is>
+      </c>
+      <c r="B451" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C451" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D451" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E451" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F451" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G451" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H451" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I451" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J451" s="17" t="n">
+        <v>328706.9408865741</v>
+      </c>
+      <c r="K451" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,383.3066</t>
+        </is>
+      </c>
+      <c r="L451" s="17" t="n">
+        <v>306432.7390860405</v>
+      </c>
+      <c r="M451" s="17">
+        <f>J451-L451</f>
+        <v/>
+      </c>
+      <c r="N451" s="18">
+        <f>IF(J451=0,"",L451/J451)</f>
+        <v/>
+      </c>
+      <c r="O451" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:43:52</t>
+        </is>
+      </c>
+      <c r="B452" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C452" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D452" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E452" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F452" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G452" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H452" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I452" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J452" s="17" t="n">
+        <v>386046.1222212454</v>
+      </c>
+      <c r="K452" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,603.9988</t>
+        </is>
+      </c>
+      <c r="L452" s="17" t="n">
+        <v>349660.4046243506</v>
+      </c>
+      <c r="M452" s="17">
+        <f>J452-L452</f>
+        <v/>
+      </c>
+      <c r="N452" s="18">
+        <f>IF(J452=0,"",L452/J452)</f>
+        <v/>
+      </c>
+      <c r="O452" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:43:52</t>
+        </is>
+      </c>
+      <c r="B453" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C453" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D453" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E453" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F453" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G453" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H453" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I453" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7844</t>
+        </is>
+      </c>
+      <c r="J453" s="17" t="n">
+        <v>77805.66673886721</v>
+      </c>
+      <c r="K453" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,027.1079; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L453" s="17" t="n">
+        <v>68019.02220805176</v>
+      </c>
+      <c r="M453" s="17">
+        <f>J453-L453</f>
+        <v/>
+      </c>
+      <c r="N453" s="18">
+        <f>IF(J453=0,"",L453/J453)</f>
+        <v/>
+      </c>
+      <c r="O453" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:43:52</t>
+        </is>
+      </c>
+      <c r="B454" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C454" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D454" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E454" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F454" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G454" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H454" s="16" t="n">
+        <v>1.1288</v>
+      </c>
+      <c r="I454" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J454" s="17" t="n">
+        <v>197105.8906091341</v>
+      </c>
+      <c r="K454" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,243.9962</t>
+        </is>
+      </c>
+      <c r="L454" s="17" t="n">
+        <v>150243.996246735</v>
+      </c>
+      <c r="M454" s="17">
+        <f>J454-L454</f>
+        <v/>
+      </c>
+      <c r="N454" s="18">
+        <f>IF(J454=0,"",L454/J454)</f>
+        <v/>
+      </c>
+      <c r="O454" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:43:52</t>
+        </is>
+      </c>
+      <c r="B455" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C455" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D455" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E455" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F455" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G455" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H455" s="16" t="n">
+        <v>1.0527</v>
+      </c>
+      <c r="I455" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J455" s="17" t="n">
+        <v>186069.2970253674</v>
+      </c>
+      <c r="K455" s="15" t="inlineStr">
+        <is>
+          <t>USDC 161,856.7587</t>
+        </is>
+      </c>
+      <c r="L455" s="17" t="n">
+        <v>161856.7586590647</v>
+      </c>
+      <c r="M455" s="17">
+        <f>J455-L455</f>
+        <v/>
+      </c>
+      <c r="N455" s="18">
+        <f>IF(J455=0,"",L455/J455)</f>
+        <v/>
+      </c>
+      <c r="O455" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:43:52</t>
+        </is>
+      </c>
+      <c r="B456" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C456" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D456" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E456" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F456" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G456" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H456" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I456" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J456" s="17" t="n">
+        <v>327618.1746978707</v>
+      </c>
+      <c r="K456" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L456" s="17" t="n">
+        <v>280262.6989204241</v>
+      </c>
+      <c r="M456" s="17">
+        <f>J456-L456</f>
+        <v/>
+      </c>
+      <c r="N456" s="18">
+        <f>IF(J456=0,"",L456/J456)</f>
+        <v/>
+      </c>
+      <c r="O456" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:43:52</t>
+        </is>
+      </c>
+      <c r="B457" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C457" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D457" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E457" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F457" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G457" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H457" s="16" t="n">
+        <v>1.1298</v>
+      </c>
+      <c r="I457" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J457" s="17" t="n">
+        <v>159973.89264</v>
+      </c>
+      <c r="K457" s="15" t="inlineStr">
+        <is>
+          <t>USDC 119,584.3639</t>
+        </is>
+      </c>
+      <c r="L457" s="17" t="n">
+        <v>119584.3639445559</v>
+      </c>
+      <c r="M457" s="17">
+        <f>J457-L457</f>
+        <v/>
+      </c>
+      <c r="N457" s="18">
+        <f>IF(J457=0,"",L457/J457)</f>
+        <v/>
+      </c>
+      <c r="O457" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:43:52</t>
+        </is>
+      </c>
+      <c r="B458" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C458" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D458" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E458" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F458" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G458" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H458" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I458" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J458" s="17" t="n">
+        <v>160160.0899815015</v>
+      </c>
+      <c r="K458" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,521.1458</t>
+        </is>
+      </c>
+      <c r="L458" s="17" t="n">
+        <v>138493.4415612677</v>
+      </c>
+      <c r="M458" s="17">
+        <f>J458-L458</f>
+        <v/>
+      </c>
+      <c r="N458" s="18">
+        <f>IF(J458=0,"",L458/J458)</f>
+        <v/>
+      </c>
+      <c r="O458" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:43:52</t>
+        </is>
+      </c>
+      <c r="B459" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C459" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D459" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E459" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F459" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeef003c</t>
+        </is>
+      </c>
+      <c r="G459" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H459" s="16" t="inlineStr"/>
+      <c r="I459" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,803.9136</t>
+        </is>
+      </c>
+      <c r="J459" s="17" t="n">
+        <v>50797.81709137268</v>
+      </c>
+      <c r="K459" s="15" t="inlineStr"/>
+      <c r="L459" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M459" s="17">
+        <f>J459-L459</f>
+        <v/>
+      </c>
+      <c r="N459" s="18">
+        <f>IF(J459=0,"",L459/J459)</f>
+        <v/>
+      </c>
+      <c r="O459" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:43:52</t>
+        </is>
+      </c>
+      <c r="B460" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C460" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D460" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E460" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F460" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeeff047</t>
+        </is>
+      </c>
+      <c r="G460" s="15" t="inlineStr">
+        <is>
+          <t>USDC vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H460" s="16" t="inlineStr"/>
+      <c r="I460" s="15" t="inlineStr">
+        <is>
+          <t>USDC 48,650.0864</t>
+        </is>
+      </c>
+      <c r="J460" s="17" t="n">
+        <v>48650.086392</v>
+      </c>
+      <c r="K460" s="15" t="inlineStr"/>
+      <c r="L460" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M460" s="17">
+        <f>J460-L460</f>
+        <v/>
+      </c>
+      <c r="N460" s="18">
+        <f>IF(J460=0,"",L460/J460)</f>
+        <v/>
+      </c>
+      <c r="O460" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:43:52</t>
+        </is>
+      </c>
+      <c r="B461" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C461" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D461" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E461" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F461" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G461" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H461" s="16" t="inlineStr"/>
+      <c r="I461" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J461" s="17" t="n">
+        <v>95895.0498308375</v>
+      </c>
+      <c r="K461" s="15" t="inlineStr"/>
+      <c r="L461" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M461" s="17">
+        <f>J461-L461</f>
+        <v/>
+      </c>
+      <c r="N461" s="18">
+        <f>IF(J461=0,"",L461/J461)</f>
+        <v/>
+      </c>
+      <c r="O461" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:43:52</t>
+        </is>
+      </c>
+      <c r="B462" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C462" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D462" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E462" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F462" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G462" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H462" s="16" t="inlineStr"/>
+      <c r="I462" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J462" s="17" t="n">
+        <v>34344.41551331289</v>
+      </c>
+      <c r="K462" s="15" t="inlineStr"/>
+      <c r="L462" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M462" s="17">
+        <f>J462-L462</f>
+        <v/>
+      </c>
+      <c r="N462" s="18">
+        <f>IF(J462=0,"",L462/J462)</f>
+        <v/>
+      </c>
+      <c r="O462" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:43:52</t>
+        </is>
+      </c>
+      <c r="B463" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C463" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D463" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E463" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F463" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G463" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H463" s="16" t="n">
+        <v>1.0429</v>
+      </c>
+      <c r="I463" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J463" s="17" t="n">
+        <v>269992.7871700212</v>
+      </c>
+      <c r="K463" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,036.0347</t>
+        </is>
+      </c>
+      <c r="L463" s="17" t="n">
+        <v>233008.0704128316</v>
+      </c>
+      <c r="M463" s="17">
+        <f>J463-L463</f>
+        <v/>
+      </c>
+      <c r="N463" s="18">
+        <f>IF(J463=0,"",L463/J463)</f>
+        <v/>
+      </c>
+      <c r="O463" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:43:52</t>
+        </is>
+      </c>
+      <c r="B464" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C464" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D464" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E464" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F464" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G464" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H464" s="16" t="inlineStr"/>
+      <c r="I464" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,508.7870</t>
+        </is>
+      </c>
+      <c r="J464" s="17" t="n">
+        <v>15506.9259302864</v>
+      </c>
+      <c r="K464" s="15" t="inlineStr"/>
+      <c r="L464" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M464" s="17">
+        <f>J464-L464</f>
+        <v/>
+      </c>
+      <c r="N464" s="18">
+        <f>IF(J464=0,"",L464/J464)</f>
+        <v/>
+      </c>
+      <c r="O464" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:43:52</t>
+        </is>
+      </c>
+      <c r="B465" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C465" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D465" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E465" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F465" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-ONyc~USDC</t>
+        </is>
+      </c>
+      <c r="G465" s="15" t="inlineStr">
+        <is>
+          <t>ONyc vs USDC</t>
+        </is>
+      </c>
+      <c r="H465" s="16" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="I465" s="15" t="inlineStr">
+        <is>
+          <t>ONyc 183,630.0000</t>
+        </is>
+      </c>
+      <c r="J465" s="17" t="n">
+        <v>201537.44</v>
+      </c>
+      <c r="K465" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,720.0000</t>
+        </is>
+      </c>
+      <c r="L465" s="17" t="n">
+        <v>148689.7</v>
+      </c>
+      <c r="M465" s="17">
+        <f>J465-L465</f>
+        <v/>
+      </c>
+      <c r="N465" s="18">
+        <f>IF(J465=0,"",L465/J465)</f>
+        <v/>
+      </c>
+      <c r="O465" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:43:52</t>
+        </is>
+      </c>
+      <c r="B466" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C466" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D466" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E466" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F466" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-PRIME~USDC</t>
+        </is>
+      </c>
+      <c r="G466" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H466" s="16" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="I466" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,234.0000</t>
+        </is>
+      </c>
+      <c r="J466" s="17" t="n">
+        <v>300953.43</v>
+      </c>
+      <c r="K466" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,976.0000</t>
+        </is>
+      </c>
+      <c r="L466" s="17" t="n">
+        <v>251924.41</v>
+      </c>
+      <c r="M466" s="17">
+        <f>J466-L466</f>
+        <v/>
+      </c>
+      <c r="N466" s="18">
+        <f>IF(J466=0,"",L466/J466)</f>
+        <v/>
+      </c>
+      <c r="O466" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:43:52</t>
+        </is>
+      </c>
+      <c r="B467" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C467" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D467" s="15" t="inlineStr">
+        <is>
+          <t>Kamino</t>
+        </is>
+      </c>
+      <c r="E467" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F467" s="15" t="inlineStr">
+        <is>
+          <t>Kamino-sol-none~none</t>
+        </is>
+      </c>
+      <c r="G467" s="15" t="inlineStr">
+        <is>
+          <t>— vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H467" s="16" t="inlineStr"/>
+      <c r="I467" s="15" t="inlineStr"/>
+      <c r="J467" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K467" s="15" t="inlineStr"/>
+      <c r="L467" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M467" s="17">
+        <f>J467-L467</f>
+        <v/>
+      </c>
+      <c r="N467" s="18">
+        <f>IF(J467=0,"",L467/J467)</f>
+        <v/>
+      </c>
+      <c r="O467" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -30661,7 +31863,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -31797,6 +32999,41 @@
         <v>1.0375</v>
       </c>
       <c r="I32" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:43:52</t>
+        </is>
+      </c>
+      <c r="B33" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C33" s="17" t="n">
+        <v>655513.2303052403</v>
+      </c>
+      <c r="D33" s="17" t="n">
+        <v>652893.5004697423</v>
+      </c>
+      <c r="E33" s="17" t="n">
+        <v>2982087.11384527</v>
+      </c>
+      <c r="F33" s="17" t="n">
+        <v>2329193.613375528</v>
+      </c>
+      <c r="G33" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="H33" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I33" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 08:14 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O467"/>
+  <dimension ref="A1:O485"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -31833,6 +31833,1208 @@
         <v/>
       </c>
       <c r="O467" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:14:00</t>
+        </is>
+      </c>
+      <c r="B468" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C468" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D468" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E468" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F468" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G468" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H468" s="16" t="n">
+        <v>1.048</v>
+      </c>
+      <c r="I468" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J468" s="17" t="n">
+        <v>140923.5047151899</v>
+      </c>
+      <c r="K468" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,032.5316</t>
+        </is>
+      </c>
+      <c r="L468" s="17" t="n">
+        <v>121019.2180375222</v>
+      </c>
+      <c r="M468" s="17">
+        <f>J468-L468</f>
+        <v/>
+      </c>
+      <c r="N468" s="18">
+        <f>IF(J468=0,"",L468/J468)</f>
+        <v/>
+      </c>
+      <c r="O468" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:14:00</t>
+        </is>
+      </c>
+      <c r="B469" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C469" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D469" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E469" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F469" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G469" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H469" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I469" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J469" s="17" t="n">
+        <v>328707.6826162995</v>
+      </c>
+      <c r="K469" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,383.3066</t>
+        </is>
+      </c>
+      <c r="L469" s="17" t="n">
+        <v>306463.2142467774</v>
+      </c>
+      <c r="M469" s="17">
+        <f>J469-L469</f>
+        <v/>
+      </c>
+      <c r="N469" s="18">
+        <f>IF(J469=0,"",L469/J469)</f>
+        <v/>
+      </c>
+      <c r="O469" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:14:00</t>
+        </is>
+      </c>
+      <c r="B470" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C470" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D470" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E470" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F470" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G470" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H470" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I470" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J470" s="17" t="n">
+        <v>386008.6306273799</v>
+      </c>
+      <c r="K470" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,603.9988</t>
+        </is>
+      </c>
+      <c r="L470" s="17" t="n">
+        <v>349695.1788363555</v>
+      </c>
+      <c r="M470" s="17">
+        <f>J470-L470</f>
+        <v/>
+      </c>
+      <c r="N470" s="18">
+        <f>IF(J470=0,"",L470/J470)</f>
+        <v/>
+      </c>
+      <c r="O470" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:14:00</t>
+        </is>
+      </c>
+      <c r="B471" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C471" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D471" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E471" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F471" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G471" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H471" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I471" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7844</t>
+        </is>
+      </c>
+      <c r="J471" s="17" t="n">
+        <v>77806.45158506812</v>
+      </c>
+      <c r="K471" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,027.1079; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L471" s="17" t="n">
+        <v>68019.70248688746</v>
+      </c>
+      <c r="M471" s="17">
+        <f>J471-L471</f>
+        <v/>
+      </c>
+      <c r="N471" s="18">
+        <f>IF(J471=0,"",L471/J471)</f>
+        <v/>
+      </c>
+      <c r="O471" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:14:00</t>
+        </is>
+      </c>
+      <c r="B472" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C472" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D472" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E472" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F472" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G472" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H472" s="16" t="n">
+        <v>1.1288</v>
+      </c>
+      <c r="I472" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J472" s="17" t="n">
+        <v>197108.2858129336</v>
+      </c>
+      <c r="K472" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,243.9962</t>
+        </is>
+      </c>
+      <c r="L472" s="17" t="n">
+        <v>150259.0221489499</v>
+      </c>
+      <c r="M472" s="17">
+        <f>J472-L472</f>
+        <v/>
+      </c>
+      <c r="N472" s="18">
+        <f>IF(J472=0,"",L472/J472)</f>
+        <v/>
+      </c>
+      <c r="O472" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:14:00</t>
+        </is>
+      </c>
+      <c r="B473" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C473" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D473" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E473" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F473" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G473" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H473" s="16" t="n">
+        <v>1.0527</v>
+      </c>
+      <c r="I473" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J473" s="17" t="n">
+        <v>186070.1394367595</v>
+      </c>
+      <c r="K473" s="15" t="inlineStr">
+        <is>
+          <t>USDC 161,856.7587</t>
+        </is>
+      </c>
+      <c r="L473" s="17" t="n">
+        <v>161872.9459536601</v>
+      </c>
+      <c r="M473" s="17">
+        <f>J473-L473</f>
+        <v/>
+      </c>
+      <c r="N473" s="18">
+        <f>IF(J473=0,"",L473/J473)</f>
+        <v/>
+      </c>
+      <c r="O473" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:14:00</t>
+        </is>
+      </c>
+      <c r="B474" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C474" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D474" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E474" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F474" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G474" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H474" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I474" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J474" s="17" t="n">
+        <v>327619.0135601666</v>
+      </c>
+      <c r="K474" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L474" s="17" t="n">
+        <v>280287.6624865407</v>
+      </c>
+      <c r="M474" s="17">
+        <f>J474-L474</f>
+        <v/>
+      </c>
+      <c r="N474" s="18">
+        <f>IF(J474=0,"",L474/J474)</f>
+        <v/>
+      </c>
+      <c r="O474" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:14:00</t>
+        </is>
+      </c>
+      <c r="B475" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C475" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D475" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E475" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F475" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G475" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H475" s="16" t="n">
+        <v>1.1298</v>
+      </c>
+      <c r="I475" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J475" s="17" t="n">
+        <v>159973.89264</v>
+      </c>
+      <c r="K475" s="15" t="inlineStr">
+        <is>
+          <t>USDC 119,584.3639</t>
+        </is>
+      </c>
+      <c r="L475" s="17" t="n">
+        <v>119596.3235769136</v>
+      </c>
+      <c r="M475" s="17">
+        <f>J475-L475</f>
+        <v/>
+      </c>
+      <c r="N475" s="18">
+        <f>IF(J475=0,"",L475/J475)</f>
+        <v/>
+      </c>
+      <c r="O475" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:14:00</t>
+        </is>
+      </c>
+      <c r="B476" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C476" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D476" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E476" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F476" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G476" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H476" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I476" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J476" s="17" t="n">
+        <v>160144.535733702</v>
+      </c>
+      <c r="K476" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,521.1458</t>
+        </is>
+      </c>
+      <c r="L476" s="17" t="n">
+        <v>138493.4415612677</v>
+      </c>
+      <c r="M476" s="17">
+        <f>J476-L476</f>
+        <v/>
+      </c>
+      <c r="N476" s="18">
+        <f>IF(J476=0,"",L476/J476)</f>
+        <v/>
+      </c>
+      <c r="O476" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:14:00</t>
+        </is>
+      </c>
+      <c r="B477" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C477" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D477" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E477" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F477" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeef003c</t>
+        </is>
+      </c>
+      <c r="G477" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H477" s="16" t="inlineStr"/>
+      <c r="I477" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,803.9136</t>
+        </is>
+      </c>
+      <c r="J477" s="17" t="n">
+        <v>50798.32513050829</v>
+      </c>
+      <c r="K477" s="15" t="inlineStr"/>
+      <c r="L477" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M477" s="17">
+        <f>J477-L477</f>
+        <v/>
+      </c>
+      <c r="N477" s="18">
+        <f>IF(J477=0,"",L477/J477)</f>
+        <v/>
+      </c>
+      <c r="O477" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:14:00</t>
+        </is>
+      </c>
+      <c r="B478" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C478" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D478" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E478" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F478" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeeff047</t>
+        </is>
+      </c>
+      <c r="G478" s="15" t="inlineStr">
+        <is>
+          <t>USDC vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H478" s="16" t="inlineStr"/>
+      <c r="I478" s="15" t="inlineStr">
+        <is>
+          <t>USDC 48,650.0864</t>
+        </is>
+      </c>
+      <c r="J478" s="17" t="n">
+        <v>48654.95188718871</v>
+      </c>
+      <c r="K478" s="15" t="inlineStr"/>
+      <c r="L478" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M478" s="17">
+        <f>J478-L478</f>
+        <v/>
+      </c>
+      <c r="N478" s="18">
+        <f>IF(J478=0,"",L478/J478)</f>
+        <v/>
+      </c>
+      <c r="O478" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:14:00</t>
+        </is>
+      </c>
+      <c r="B479" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C479" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D479" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E479" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F479" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G479" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H479" s="16" t="inlineStr"/>
+      <c r="I479" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J479" s="17" t="n">
+        <v>95893.35382679763</v>
+      </c>
+      <c r="K479" s="15" t="inlineStr"/>
+      <c r="L479" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M479" s="17">
+        <f>J479-L479</f>
+        <v/>
+      </c>
+      <c r="N479" s="18">
+        <f>IF(J479=0,"",L479/J479)</f>
+        <v/>
+      </c>
+      <c r="O479" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:14:00</t>
+        </is>
+      </c>
+      <c r="B480" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C480" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D480" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E480" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F480" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G480" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H480" s="16" t="inlineStr"/>
+      <c r="I480" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J480" s="17" t="n">
+        <v>34344.69088393729</v>
+      </c>
+      <c r="K480" s="15" t="inlineStr"/>
+      <c r="L480" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M480" s="17">
+        <f>J480-L480</f>
+        <v/>
+      </c>
+      <c r="N480" s="18">
+        <f>IF(J480=0,"",L480/J480)</f>
+        <v/>
+      </c>
+      <c r="O480" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:14:00</t>
+        </is>
+      </c>
+      <c r="B481" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C481" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D481" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E481" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F481" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G481" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H481" s="16" t="n">
+        <v>1.0429</v>
+      </c>
+      <c r="I481" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J481" s="17" t="n">
+        <v>269996.1113129806</v>
+      </c>
+      <c r="K481" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,036.0347</t>
+        </is>
+      </c>
+      <c r="L481" s="17" t="n">
+        <v>233010.4007731789</v>
+      </c>
+      <c r="M481" s="17">
+        <f>J481-L481</f>
+        <v/>
+      </c>
+      <c r="N481" s="18">
+        <f>IF(J481=0,"",L481/J481)</f>
+        <v/>
+      </c>
+      <c r="O481" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:14:00</t>
+        </is>
+      </c>
+      <c r="B482" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C482" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D482" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E482" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F482" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G482" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H482" s="16" t="inlineStr"/>
+      <c r="I482" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,508.9882</t>
+        </is>
+      </c>
+      <c r="J482" s="17" t="n">
+        <v>15507.2822395499</v>
+      </c>
+      <c r="K482" s="15" t="inlineStr"/>
+      <c r="L482" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M482" s="17">
+        <f>J482-L482</f>
+        <v/>
+      </c>
+      <c r="N482" s="18">
+        <f>IF(J482=0,"",L482/J482)</f>
+        <v/>
+      </c>
+      <c r="O482" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:14:00</t>
+        </is>
+      </c>
+      <c r="B483" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C483" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D483" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E483" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F483" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-ONyc~USDC</t>
+        </is>
+      </c>
+      <c r="G483" s="15" t="inlineStr">
+        <is>
+          <t>ONyc vs USDC</t>
+        </is>
+      </c>
+      <c r="H483" s="16" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="I483" s="15" t="inlineStr">
+        <is>
+          <t>ONyc 183,630.0000</t>
+        </is>
+      </c>
+      <c r="J483" s="17" t="n">
+        <v>201537.44</v>
+      </c>
+      <c r="K483" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,720.0000</t>
+        </is>
+      </c>
+      <c r="L483" s="17" t="n">
+        <v>148689.7</v>
+      </c>
+      <c r="M483" s="17">
+        <f>J483-L483</f>
+        <v/>
+      </c>
+      <c r="N483" s="18">
+        <f>IF(J483=0,"",L483/J483)</f>
+        <v/>
+      </c>
+      <c r="O483" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:14:00</t>
+        </is>
+      </c>
+      <c r="B484" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C484" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D484" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E484" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F484" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-PRIME~USDC</t>
+        </is>
+      </c>
+      <c r="G484" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H484" s="16" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="I484" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,234.0000</t>
+        </is>
+      </c>
+      <c r="J484" s="17" t="n">
+        <v>300953.43</v>
+      </c>
+      <c r="K484" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,976.0000</t>
+        </is>
+      </c>
+      <c r="L484" s="17" t="n">
+        <v>251924.41</v>
+      </c>
+      <c r="M484" s="17">
+        <f>J484-L484</f>
+        <v/>
+      </c>
+      <c r="N484" s="18">
+        <f>IF(J484=0,"",L484/J484)</f>
+        <v/>
+      </c>
+      <c r="O484" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:14:00</t>
+        </is>
+      </c>
+      <c r="B485" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C485" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D485" s="15" t="inlineStr">
+        <is>
+          <t>Kamino</t>
+        </is>
+      </c>
+      <c r="E485" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F485" s="15" t="inlineStr">
+        <is>
+          <t>Kamino-sol-none~none</t>
+        </is>
+      </c>
+      <c r="G485" s="15" t="inlineStr">
+        <is>
+          <t>— vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H485" s="16" t="inlineStr"/>
+      <c r="I485" s="15" t="inlineStr"/>
+      <c r="J485" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K485" s="15" t="inlineStr"/>
+      <c r="L485" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M485" s="17">
+        <f>J485-L485</f>
+        <v/>
+      </c>
+      <c r="N485" s="18">
+        <f>IF(J485=0,"",L485/J485)</f>
+        <v/>
+      </c>
+      <c r="O485" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -31863,7 +33065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -33034,6 +34236,41 @@
         <v>1.0375</v>
       </c>
       <c r="I33" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:14:00</t>
+        </is>
+      </c>
+      <c r="B34" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C34" s="17" t="n">
+        <v>655335.8824558228</v>
+      </c>
+      <c r="D34" s="17" t="n">
+        <v>652716.501900408</v>
+      </c>
+      <c r="E34" s="17" t="n">
+        <v>2982047.722008462</v>
+      </c>
+      <c r="F34" s="17" t="n">
+        <v>2329331.220108054</v>
+      </c>
+      <c r="G34" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="H34" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I34" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 08:44 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O485"/>
+  <dimension ref="A1:O503"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -33035,6 +33035,1208 @@
         <v/>
       </c>
       <c r="O485" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:44:09</t>
+        </is>
+      </c>
+      <c r="B486" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C486" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D486" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E486" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F486" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G486" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H486" s="16" t="n">
+        <v>1.0483</v>
+      </c>
+      <c r="I486" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J486" s="17" t="n">
+        <v>140938.0273395635</v>
+      </c>
+      <c r="K486" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,032.5316</t>
+        </is>
+      </c>
+      <c r="L486" s="17" t="n">
+        <v>121002.273483096</v>
+      </c>
+      <c r="M486" s="17">
+        <f>J486-L486</f>
+        <v/>
+      </c>
+      <c r="N486" s="18">
+        <f>IF(J486=0,"",L486/J486)</f>
+        <v/>
+      </c>
+      <c r="O486" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:44:09</t>
+        </is>
+      </c>
+      <c r="B487" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C487" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D487" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E487" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F487" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G487" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H487" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I487" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J487" s="17" t="n">
+        <v>328708.3764940095</v>
+      </c>
+      <c r="K487" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,383.3066</t>
+        </is>
+      </c>
+      <c r="L487" s="17" t="n">
+        <v>306433.7926320174</v>
+      </c>
+      <c r="M487" s="17">
+        <f>J487-L487</f>
+        <v/>
+      </c>
+      <c r="N487" s="18">
+        <f>IF(J487=0,"",L487/J487)</f>
+        <v/>
+      </c>
+      <c r="O487" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:44:09</t>
+        </is>
+      </c>
+      <c r="B488" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C488" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D488" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E488" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F488" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G488" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H488" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I488" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J488" s="17" t="n">
+        <v>386010.5426816696</v>
+      </c>
+      <c r="K488" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,603.9988</t>
+        </is>
+      </c>
+      <c r="L488" s="17" t="n">
+        <v>349661.6067913047</v>
+      </c>
+      <c r="M488" s="17">
+        <f>J488-L488</f>
+        <v/>
+      </c>
+      <c r="N488" s="18">
+        <f>IF(J488=0,"",L488/J488)</f>
+        <v/>
+      </c>
+      <c r="O488" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:44:09</t>
+        </is>
+      </c>
+      <c r="B489" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C489" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D489" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E489" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F489" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G489" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H489" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I489" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7844</t>
+        </is>
+      </c>
+      <c r="J489" s="17" t="n">
+        <v>77807.19629525267</v>
+      </c>
+      <c r="K489" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,027.1079; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L489" s="17" t="n">
+        <v>68010.1786840245</v>
+      </c>
+      <c r="M489" s="17">
+        <f>J489-L489</f>
+        <v/>
+      </c>
+      <c r="N489" s="18">
+        <f>IF(J489=0,"",L489/J489)</f>
+        <v/>
+      </c>
+      <c r="O489" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:44:09</t>
+        </is>
+      </c>
+      <c r="B490" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C490" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D490" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E490" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F490" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G490" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H490" s="16" t="n">
+        <v>1.1288</v>
+      </c>
+      <c r="I490" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J490" s="17" t="n">
+        <v>197109.9066690835</v>
+      </c>
+      <c r="K490" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,243.9962</t>
+        </is>
+      </c>
+      <c r="L490" s="17" t="n">
+        <v>150243.996246735</v>
+      </c>
+      <c r="M490" s="17">
+        <f>J490-L490</f>
+        <v/>
+      </c>
+      <c r="N490" s="18">
+        <f>IF(J490=0,"",L490/J490)</f>
+        <v/>
+      </c>
+      <c r="O490" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:44:09</t>
+        </is>
+      </c>
+      <c r="B491" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C491" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D491" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E491" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F491" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G491" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H491" s="16" t="n">
+        <v>1.0527</v>
+      </c>
+      <c r="I491" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J491" s="17" t="n">
+        <v>185988.1364329137</v>
+      </c>
+      <c r="K491" s="15" t="inlineStr">
+        <is>
+          <t>USDC 161,856.7587</t>
+        </is>
+      </c>
+      <c r="L491" s="17" t="n">
+        <v>161856.7586590647</v>
+      </c>
+      <c r="M491" s="17">
+        <f>J491-L491</f>
+        <v/>
+      </c>
+      <c r="N491" s="18">
+        <f>IF(J491=0,"",L491/J491)</f>
+        <v/>
+      </c>
+      <c r="O491" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:44:09</t>
+        </is>
+      </c>
+      <c r="B492" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C492" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D492" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E492" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F492" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G492" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H492" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I492" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J492" s="17" t="n">
+        <v>327619.0136803525</v>
+      </c>
+      <c r="K492" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L492" s="17" t="n">
+        <v>280262.7082611826</v>
+      </c>
+      <c r="M492" s="17">
+        <f>J492-L492</f>
+        <v/>
+      </c>
+      <c r="N492" s="18">
+        <f>IF(J492=0,"",L492/J492)</f>
+        <v/>
+      </c>
+      <c r="O492" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:44:09</t>
+        </is>
+      </c>
+      <c r="B493" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C493" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D493" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E493" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F493" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G493" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H493" s="16" t="n">
+        <v>1.1298</v>
+      </c>
+      <c r="I493" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J493" s="17" t="n">
+        <v>159973.89264</v>
+      </c>
+      <c r="K493" s="15" t="inlineStr">
+        <is>
+          <t>USDC 119,584.3639</t>
+        </is>
+      </c>
+      <c r="L493" s="17" t="n">
+        <v>119584.3639445559</v>
+      </c>
+      <c r="M493" s="17">
+        <f>J493-L493</f>
+        <v/>
+      </c>
+      <c r="N493" s="18">
+        <f>IF(J493=0,"",L493/J493)</f>
+        <v/>
+      </c>
+      <c r="O493" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:44:09</t>
+        </is>
+      </c>
+      <c r="B494" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C494" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D494" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E494" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F494" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G494" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H494" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I494" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J494" s="17" t="n">
+        <v>160145.328993288</v>
+      </c>
+      <c r="K494" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,521.1458</t>
+        </is>
+      </c>
+      <c r="L494" s="17" t="n">
+        <v>138493.4415612677</v>
+      </c>
+      <c r="M494" s="17">
+        <f>J494-L494</f>
+        <v/>
+      </c>
+      <c r="N494" s="18">
+        <f>IF(J494=0,"",L494/J494)</f>
+        <v/>
+      </c>
+      <c r="O494" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:44:09</t>
+        </is>
+      </c>
+      <c r="B495" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C495" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D495" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E495" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F495" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeef003c</t>
+        </is>
+      </c>
+      <c r="G495" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H495" s="16" t="inlineStr"/>
+      <c r="I495" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,803.9136</t>
+        </is>
+      </c>
+      <c r="J495" s="17" t="n">
+        <v>50791.21258260975</v>
+      </c>
+      <c r="K495" s="15" t="inlineStr"/>
+      <c r="L495" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M495" s="17">
+        <f>J495-L495</f>
+        <v/>
+      </c>
+      <c r="N495" s="18">
+        <f>IF(J495=0,"",L495/J495)</f>
+        <v/>
+      </c>
+      <c r="O495" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:44:09</t>
+        </is>
+      </c>
+      <c r="B496" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C496" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D496" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E496" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F496" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeeff047</t>
+        </is>
+      </c>
+      <c r="G496" s="15" t="inlineStr">
+        <is>
+          <t>USDC vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H496" s="16" t="inlineStr"/>
+      <c r="I496" s="15" t="inlineStr">
+        <is>
+          <t>USDC 48,650.0864</t>
+        </is>
+      </c>
+      <c r="J496" s="17" t="n">
+        <v>48650.086392</v>
+      </c>
+      <c r="K496" s="15" t="inlineStr"/>
+      <c r="L496" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M496" s="17">
+        <f>J496-L496</f>
+        <v/>
+      </c>
+      <c r="N496" s="18">
+        <f>IF(J496=0,"",L496/J496)</f>
+        <v/>
+      </c>
+      <c r="O496" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:44:09</t>
+        </is>
+      </c>
+      <c r="B497" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C497" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D497" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E497" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F497" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G497" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H497" s="16" t="inlineStr"/>
+      <c r="I497" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J497" s="17" t="n">
+        <v>95902.30271073652</v>
+      </c>
+      <c r="K497" s="15" t="inlineStr"/>
+      <c r="L497" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M497" s="17">
+        <f>J497-L497</f>
+        <v/>
+      </c>
+      <c r="N497" s="18">
+        <f>IF(J497=0,"",L497/J497)</f>
+        <v/>
+      </c>
+      <c r="O497" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:44:09</t>
+        </is>
+      </c>
+      <c r="B498" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C498" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D498" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E498" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F498" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G498" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H498" s="16" t="inlineStr"/>
+      <c r="I498" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J498" s="17" t="n">
+        <v>34345.22233221242</v>
+      </c>
+      <c r="K498" s="15" t="inlineStr"/>
+      <c r="L498" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M498" s="17">
+        <f>J498-L498</f>
+        <v/>
+      </c>
+      <c r="N498" s="18">
+        <f>IF(J498=0,"",L498/J498)</f>
+        <v/>
+      </c>
+      <c r="O498" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:44:09</t>
+        </is>
+      </c>
+      <c r="B499" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C499" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D499" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E499" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F499" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G499" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H499" s="16" t="n">
+        <v>1.043</v>
+      </c>
+      <c r="I499" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J499" s="17" t="n">
+        <v>269996.1113129806</v>
+      </c>
+      <c r="K499" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,036.0347</t>
+        </is>
+      </c>
+      <c r="L499" s="17" t="n">
+        <v>232977.7757283158</v>
+      </c>
+      <c r="M499" s="17">
+        <f>J499-L499</f>
+        <v/>
+      </c>
+      <c r="N499" s="18">
+        <f>IF(J499=0,"",L499/J499)</f>
+        <v/>
+      </c>
+      <c r="O499" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:44:09</t>
+        </is>
+      </c>
+      <c r="B500" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C500" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D500" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E500" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F500" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G500" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H500" s="16" t="inlineStr"/>
+      <c r="I500" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,509.1885</t>
+        </is>
+      </c>
+      <c r="J500" s="17" t="n">
+        <v>15505.31116396269</v>
+      </c>
+      <c r="K500" s="15" t="inlineStr"/>
+      <c r="L500" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M500" s="17">
+        <f>J500-L500</f>
+        <v/>
+      </c>
+      <c r="N500" s="18">
+        <f>IF(J500=0,"",L500/J500)</f>
+        <v/>
+      </c>
+      <c r="O500" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:44:09</t>
+        </is>
+      </c>
+      <c r="B501" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C501" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D501" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E501" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F501" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-ONyc~USDC</t>
+        </is>
+      </c>
+      <c r="G501" s="15" t="inlineStr">
+        <is>
+          <t>ONyc vs USDC</t>
+        </is>
+      </c>
+      <c r="H501" s="16" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="I501" s="15" t="inlineStr">
+        <is>
+          <t>ONyc 183,630.0000</t>
+        </is>
+      </c>
+      <c r="J501" s="17" t="n">
+        <v>201537.44</v>
+      </c>
+      <c r="K501" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,720.0000</t>
+        </is>
+      </c>
+      <c r="L501" s="17" t="n">
+        <v>148689.7</v>
+      </c>
+      <c r="M501" s="17">
+        <f>J501-L501</f>
+        <v/>
+      </c>
+      <c r="N501" s="18">
+        <f>IF(J501=0,"",L501/J501)</f>
+        <v/>
+      </c>
+      <c r="O501" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:44:09</t>
+        </is>
+      </c>
+      <c r="B502" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C502" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D502" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E502" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F502" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-PRIME~USDC</t>
+        </is>
+      </c>
+      <c r="G502" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H502" s="16" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="I502" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,234.0000</t>
+        </is>
+      </c>
+      <c r="J502" s="17" t="n">
+        <v>300953.43</v>
+      </c>
+      <c r="K502" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,976.0000</t>
+        </is>
+      </c>
+      <c r="L502" s="17" t="n">
+        <v>251924.41</v>
+      </c>
+      <c r="M502" s="17">
+        <f>J502-L502</f>
+        <v/>
+      </c>
+      <c r="N502" s="18">
+        <f>IF(J502=0,"",L502/J502)</f>
+        <v/>
+      </c>
+      <c r="O502" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:44:09</t>
+        </is>
+      </c>
+      <c r="B503" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C503" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D503" s="15" t="inlineStr">
+        <is>
+          <t>Kamino</t>
+        </is>
+      </c>
+      <c r="E503" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F503" s="15" t="inlineStr">
+        <is>
+          <t>Kamino-sol-none~none</t>
+        </is>
+      </c>
+      <c r="G503" s="15" t="inlineStr">
+        <is>
+          <t>— vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H503" s="16" t="inlineStr"/>
+      <c r="I503" s="15" t="inlineStr"/>
+      <c r="J503" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K503" s="15" t="inlineStr"/>
+      <c r="L503" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M503" s="17">
+        <f>J503-L503</f>
+        <v/>
+      </c>
+      <c r="N503" s="18">
+        <f>IF(J503=0,"",L503/J503)</f>
+        <v/>
+      </c>
+      <c r="O503" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -33065,7 +34267,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -34271,6 +35473,41 @@
         <v>1.0375</v>
       </c>
       <c r="I34" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 08:44:09</t>
+        </is>
+      </c>
+      <c r="B35" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C35" s="17" t="n">
+        <v>655460.3830262456</v>
+      </c>
+      <c r="D35" s="17" t="n">
+        <v>652840.5317290714</v>
+      </c>
+      <c r="E35" s="17" t="n">
+        <v>2981981.537720636</v>
+      </c>
+      <c r="F35" s="17" t="n">
+        <v>2329141.005991564</v>
+      </c>
+      <c r="G35" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="H35" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I35" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 09:14 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O503"/>
+  <dimension ref="A1:O521"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -34237,6 +34237,1208 @@
         <v/>
       </c>
       <c r="O503" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 09:14:18</t>
+        </is>
+      </c>
+      <c r="B504" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C504" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D504" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E504" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F504" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G504" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H504" s="16" t="n">
+        <v>1.0482</v>
+      </c>
+      <c r="I504" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J504" s="17" t="n">
+        <v>140924.3428925024</v>
+      </c>
+      <c r="K504" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,032.5316</t>
+        </is>
+      </c>
+      <c r="L504" s="17" t="n">
+        <v>120997.4321818313</v>
+      </c>
+      <c r="M504" s="17">
+        <f>J504-L504</f>
+        <v/>
+      </c>
+      <c r="N504" s="18">
+        <f>IF(J504=0,"",L504/J504)</f>
+        <v/>
+      </c>
+      <c r="O504" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 09:14:18</t>
+        </is>
+      </c>
+      <c r="B505" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C505" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D505" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E505" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F505" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G505" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H505" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I505" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J505" s="17" t="n">
+        <v>328709.9173862999</v>
+      </c>
+      <c r="K505" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,383.3066</t>
+        </is>
+      </c>
+      <c r="L505" s="17" t="n">
+        <v>306466.4660499397</v>
+      </c>
+      <c r="M505" s="17">
+        <f>J505-L505</f>
+        <v/>
+      </c>
+      <c r="N505" s="18">
+        <f>IF(J505=0,"",L505/J505)</f>
+        <v/>
+      </c>
+      <c r="O505" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 09:14:18</t>
+        </is>
+      </c>
+      <c r="B506" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C506" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D506" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E506" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F506" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G506" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H506" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I506" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J506" s="17" t="n">
+        <v>386011.7262257098</v>
+      </c>
+      <c r="K506" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,603.9988</t>
+        </is>
+      </c>
+      <c r="L506" s="17" t="n">
+        <v>349698.8893628903</v>
+      </c>
+      <c r="M506" s="17">
+        <f>J506-L506</f>
+        <v/>
+      </c>
+      <c r="N506" s="18">
+        <f>IF(J506=0,"",L506/J506)</f>
+        <v/>
+      </c>
+      <c r="O506" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 09:14:18</t>
+        </is>
+      </c>
+      <c r="B507" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C507" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D507" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E507" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F507" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G507" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H507" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I507" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7844</t>
+        </is>
+      </c>
+      <c r="J507" s="17" t="n">
+        <v>77796.34934265388</v>
+      </c>
+      <c r="K507" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,027.1079; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L507" s="17" t="n">
+        <v>68007.4576074651</v>
+      </c>
+      <c r="M507" s="17">
+        <f>J507-L507</f>
+        <v/>
+      </c>
+      <c r="N507" s="18">
+        <f>IF(J507=0,"",L507/J507)</f>
+        <v/>
+      </c>
+      <c r="O507" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 09:14:18</t>
+        </is>
+      </c>
+      <c r="B508" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C508" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D508" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E508" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F508" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G508" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H508" s="16" t="n">
+        <v>1.1288</v>
+      </c>
+      <c r="I508" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J508" s="17" t="n">
+        <v>197111.1160349202</v>
+      </c>
+      <c r="K508" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,243.9962</t>
+        </is>
+      </c>
+      <c r="L508" s="17" t="n">
+        <v>150259.0221489499</v>
+      </c>
+      <c r="M508" s="17">
+        <f>J508-L508</f>
+        <v/>
+      </c>
+      <c r="N508" s="18">
+        <f>IF(J508=0,"",L508/J508)</f>
+        <v/>
+      </c>
+      <c r="O508" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 09:14:18</t>
+        </is>
+      </c>
+      <c r="B509" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C509" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D509" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E509" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F509" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G509" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H509" s="16" t="n">
+        <v>1.0527</v>
+      </c>
+      <c r="I509" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J509" s="17" t="n">
+        <v>186138.0400050524</v>
+      </c>
+      <c r="K509" s="15" t="inlineStr">
+        <is>
+          <t>USDC 161,856.7587</t>
+        </is>
+      </c>
+      <c r="L509" s="17" t="n">
+        <v>161872.9459536601</v>
+      </c>
+      <c r="M509" s="17">
+        <f>J509-L509</f>
+        <v/>
+      </c>
+      <c r="N509" s="18">
+        <f>IF(J509=0,"",L509/J509)</f>
+        <v/>
+      </c>
+      <c r="O509" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 09:14:18</t>
+        </is>
+      </c>
+      <c r="B510" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C510" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D510" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E510" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F510" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G510" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H510" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I510" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J510" s="17" t="n">
+        <v>327619.0245994299</v>
+      </c>
+      <c r="K510" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L510" s="17" t="n">
+        <v>280265.7930922464</v>
+      </c>
+      <c r="M510" s="17">
+        <f>J510-L510</f>
+        <v/>
+      </c>
+      <c r="N510" s="18">
+        <f>IF(J510=0,"",L510/J510)</f>
+        <v/>
+      </c>
+      <c r="O510" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 09:14:18</t>
+        </is>
+      </c>
+      <c r="B511" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C511" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D511" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E511" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F511" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G511" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H511" s="16" t="n">
+        <v>1.1298</v>
+      </c>
+      <c r="I511" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J511" s="17" t="n">
+        <v>159973.89264</v>
+      </c>
+      <c r="K511" s="15" t="inlineStr">
+        <is>
+          <t>USDC 119,584.3639</t>
+        </is>
+      </c>
+      <c r="L511" s="17" t="n">
+        <v>119596.3235769136</v>
+      </c>
+      <c r="M511" s="17">
+        <f>J511-L511</f>
+        <v/>
+      </c>
+      <c r="N511" s="18">
+        <f>IF(J511=0,"",L511/J511)</f>
+        <v/>
+      </c>
+      <c r="O511" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 09:14:18</t>
+        </is>
+      </c>
+      <c r="B512" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C512" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D512" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E512" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F512" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G512" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H512" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I512" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J512" s="17" t="n">
+        <v>160145.8200136844</v>
+      </c>
+      <c r="K512" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,521.1458</t>
+        </is>
+      </c>
+      <c r="L512" s="17" t="n">
+        <v>138493.4415612677</v>
+      </c>
+      <c r="M512" s="17">
+        <f>J512-L512</f>
+        <v/>
+      </c>
+      <c r="N512" s="18">
+        <f>IF(J512=0,"",L512/J512)</f>
+        <v/>
+      </c>
+      <c r="O512" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 09:14:18</t>
+        </is>
+      </c>
+      <c r="B513" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C513" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D513" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E513" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F513" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeef003c</t>
+        </is>
+      </c>
+      <c r="G513" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H513" s="16" t="inlineStr"/>
+      <c r="I513" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,803.9136</t>
+        </is>
+      </c>
+      <c r="J513" s="17" t="n">
+        <v>50789.18042606731</v>
+      </c>
+      <c r="K513" s="15" t="inlineStr"/>
+      <c r="L513" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M513" s="17">
+        <f>J513-L513</f>
+        <v/>
+      </c>
+      <c r="N513" s="18">
+        <f>IF(J513=0,"",L513/J513)</f>
+        <v/>
+      </c>
+      <c r="O513" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 09:14:18</t>
+        </is>
+      </c>
+      <c r="B514" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C514" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D514" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E514" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F514" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeeff047</t>
+        </is>
+      </c>
+      <c r="G514" s="15" t="inlineStr">
+        <is>
+          <t>USDC vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H514" s="16" t="inlineStr"/>
+      <c r="I514" s="15" t="inlineStr">
+        <is>
+          <t>USDC 48,650.0864</t>
+        </is>
+      </c>
+      <c r="J514" s="17" t="n">
+        <v>48654.95188718871</v>
+      </c>
+      <c r="K514" s="15" t="inlineStr"/>
+      <c r="L514" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M514" s="17">
+        <f>J514-L514</f>
+        <v/>
+      </c>
+      <c r="N514" s="18">
+        <f>IF(J514=0,"",L514/J514)</f>
+        <v/>
+      </c>
+      <c r="O514" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 09:14:18</t>
+        </is>
+      </c>
+      <c r="B515" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C515" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D515" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E515" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F515" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G515" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H515" s="16" t="inlineStr"/>
+      <c r="I515" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J515" s="17" t="n">
+        <v>95932.53770758022</v>
+      </c>
+      <c r="K515" s="15" t="inlineStr"/>
+      <c r="L515" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M515" s="17">
+        <f>J515-L515</f>
+        <v/>
+      </c>
+      <c r="N515" s="18">
+        <f>IF(J515=0,"",L515/J515)</f>
+        <v/>
+      </c>
+      <c r="O515" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 09:14:18</t>
+        </is>
+      </c>
+      <c r="B516" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C516" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D516" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E516" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F516" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G516" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H516" s="16" t="inlineStr"/>
+      <c r="I516" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J516" s="17" t="n">
+        <v>34345.43198510293</v>
+      </c>
+      <c r="K516" s="15" t="inlineStr"/>
+      <c r="L516" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M516" s="17">
+        <f>J516-L516</f>
+        <v/>
+      </c>
+      <c r="N516" s="18">
+        <f>IF(J516=0,"",L516/J516)</f>
+        <v/>
+      </c>
+      <c r="O516" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 09:14:18</t>
+        </is>
+      </c>
+      <c r="B517" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C517" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D517" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E517" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F517" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G517" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H517" s="16" t="n">
+        <v>1.043</v>
+      </c>
+      <c r="I517" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J517" s="17" t="n">
+        <v>269996.1113129806</v>
+      </c>
+      <c r="K517" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,036.0347</t>
+        </is>
+      </c>
+      <c r="L517" s="17" t="n">
+        <v>232968.4542869263</v>
+      </c>
+      <c r="M517" s="17">
+        <f>J517-L517</f>
+        <v/>
+      </c>
+      <c r="N517" s="18">
+        <f>IF(J517=0,"",L517/J517)</f>
+        <v/>
+      </c>
+      <c r="O517" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 09:14:18</t>
+        </is>
+      </c>
+      <c r="B518" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C518" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D518" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E518" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F518" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G518" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H518" s="16" t="inlineStr"/>
+      <c r="I518" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,509.3925</t>
+        </is>
+      </c>
+      <c r="J518" s="17" t="n">
+        <v>15504.89478830954</v>
+      </c>
+      <c r="K518" s="15" t="inlineStr"/>
+      <c r="L518" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M518" s="17">
+        <f>J518-L518</f>
+        <v/>
+      </c>
+      <c r="N518" s="18">
+        <f>IF(J518=0,"",L518/J518)</f>
+        <v/>
+      </c>
+      <c r="O518" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 09:14:18</t>
+        </is>
+      </c>
+      <c r="B519" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C519" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D519" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E519" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F519" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-ONyc~USDC</t>
+        </is>
+      </c>
+      <c r="G519" s="15" t="inlineStr">
+        <is>
+          <t>ONyc vs USDC</t>
+        </is>
+      </c>
+      <c r="H519" s="16" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="I519" s="15" t="inlineStr">
+        <is>
+          <t>ONyc 183,630.0000</t>
+        </is>
+      </c>
+      <c r="J519" s="17" t="n">
+        <v>201537.44</v>
+      </c>
+      <c r="K519" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,720.0000</t>
+        </is>
+      </c>
+      <c r="L519" s="17" t="n">
+        <v>148689.7</v>
+      </c>
+      <c r="M519" s="17">
+        <f>J519-L519</f>
+        <v/>
+      </c>
+      <c r="N519" s="18">
+        <f>IF(J519=0,"",L519/J519)</f>
+        <v/>
+      </c>
+      <c r="O519" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 09:14:18</t>
+        </is>
+      </c>
+      <c r="B520" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C520" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D520" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E520" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F520" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-PRIME~USDC</t>
+        </is>
+      </c>
+      <c r="G520" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H520" s="16" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="I520" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,234.0000</t>
+        </is>
+      </c>
+      <c r="J520" s="17" t="n">
+        <v>300953.43</v>
+      </c>
+      <c r="K520" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,976.0000</t>
+        </is>
+      </c>
+      <c r="L520" s="17" t="n">
+        <v>251924.41</v>
+      </c>
+      <c r="M520" s="17">
+        <f>J520-L520</f>
+        <v/>
+      </c>
+      <c r="N520" s="18">
+        <f>IF(J520=0,"",L520/J520)</f>
+        <v/>
+      </c>
+      <c r="O520" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 09:14:18</t>
+        </is>
+      </c>
+      <c r="B521" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C521" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D521" s="15" t="inlineStr">
+        <is>
+          <t>Kamino</t>
+        </is>
+      </c>
+      <c r="E521" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F521" s="15" t="inlineStr">
+        <is>
+          <t>Kamino-sol-none~none</t>
+        </is>
+      </c>
+      <c r="G521" s="15" t="inlineStr">
+        <is>
+          <t>— vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H521" s="16" t="inlineStr"/>
+      <c r="I521" s="15" t="inlineStr"/>
+      <c r="J521" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K521" s="15" t="inlineStr"/>
+      <c r="L521" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M521" s="17">
+        <f>J521-L521</f>
+        <v/>
+      </c>
+      <c r="N521" s="18">
+        <f>IF(J521=0,"",L521/J521)</f>
+        <v/>
+      </c>
+      <c r="O521" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -34267,7 +35469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -35508,6 +36710,41 @@
         <v>1.0375</v>
       </c>
       <c r="I35" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 09:14:18</t>
+        </is>
+      </c>
+      <c r="B36" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C36" s="17" t="n">
+        <v>655522.7790766497</v>
+      </c>
+      <c r="D36" s="17" t="n">
+        <v>652903.8714253921</v>
+      </c>
+      <c r="E36" s="17" t="n">
+        <v>2982144.207247483</v>
+      </c>
+      <c r="F36" s="17" t="n">
+        <v>2329240.335822091</v>
+      </c>
+      <c r="G36" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="H36" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I36" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 10:15 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O521"/>
+  <dimension ref="A1:O538"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -35439,6 +35439,1145 @@
         <v/>
       </c>
       <c r="O521" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:14:55</t>
+        </is>
+      </c>
+      <c r="B522" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C522" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D522" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E522" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F522" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G522" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H522" s="16" t="n">
+        <v>1.0481</v>
+      </c>
+      <c r="I522" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J522" s="17" t="n">
+        <v>140925.4707476556</v>
+      </c>
+      <c r="K522" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,032.5316</t>
+        </is>
+      </c>
+      <c r="L522" s="17" t="n">
+        <v>121013.1664109414</v>
+      </c>
+      <c r="M522" s="17">
+        <f>J522-L522</f>
+        <v/>
+      </c>
+      <c r="N522" s="18">
+        <f>IF(J522=0,"",L522/J522)</f>
+        <v/>
+      </c>
+      <c r="O522" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:14:55</t>
+        </is>
+      </c>
+      <c r="B523" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C523" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D523" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E523" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F523" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G523" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H523" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I523" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J523" s="17" t="n">
+        <v>328711.3721483831</v>
+      </c>
+      <c r="K523" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,383.3066</t>
+        </is>
+      </c>
+      <c r="L523" s="17" t="n">
+        <v>306434.3037227403</v>
+      </c>
+      <c r="M523" s="17">
+        <f>J523-L523</f>
+        <v/>
+      </c>
+      <c r="N523" s="18">
+        <f>IF(J523=0,"",L523/J523)</f>
+        <v/>
+      </c>
+      <c r="O523" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:14:55</t>
+        </is>
+      </c>
+      <c r="B524" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C524" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D524" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E524" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F524" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G524" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H524" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I524" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J524" s="17" t="n">
+        <v>386014.0008907581</v>
+      </c>
+      <c r="K524" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,603.9988</t>
+        </is>
+      </c>
+      <c r="L524" s="17" t="n">
+        <v>349662.1899802599</v>
+      </c>
+      <c r="M524" s="17">
+        <f>J524-L524</f>
+        <v/>
+      </c>
+      <c r="N524" s="18">
+        <f>IF(J524=0,"",L524/J524)</f>
+        <v/>
+      </c>
+      <c r="O524" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:14:55</t>
+        </is>
+      </c>
+      <c r="B525" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C525" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D525" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E525" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F525" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G525" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H525" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I525" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7844</t>
+        </is>
+      </c>
+      <c r="J525" s="17" t="n">
+        <v>77797.2687566487</v>
+      </c>
+      <c r="K525" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,027.1079; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L525" s="17" t="n">
+        <v>68016.30112373568</v>
+      </c>
+      <c r="M525" s="17">
+        <f>J525-L525</f>
+        <v/>
+      </c>
+      <c r="N525" s="18">
+        <f>IF(J525=0,"",L525/J525)</f>
+        <v/>
+      </c>
+      <c r="O525" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:14:55</t>
+        </is>
+      </c>
+      <c r="B526" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C526" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D526" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E526" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F526" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G526" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H526" s="16" t="n">
+        <v>1.1288</v>
+      </c>
+      <c r="I526" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J526" s="17" t="n">
+        <v>197089.7098013764</v>
+      </c>
+      <c r="K526" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,243.9962</t>
+        </is>
+      </c>
+      <c r="L526" s="17" t="n">
+        <v>150243.996246735</v>
+      </c>
+      <c r="M526" s="17">
+        <f>J526-L526</f>
+        <v/>
+      </c>
+      <c r="N526" s="18">
+        <f>IF(J526=0,"",L526/J526)</f>
+        <v/>
+      </c>
+      <c r="O526" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:14:55</t>
+        </is>
+      </c>
+      <c r="B527" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C527" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D527" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E527" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F527" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G527" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H527" s="16" t="n">
+        <v>1.0527</v>
+      </c>
+      <c r="I527" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J527" s="17" t="n">
+        <v>186102.9853179372</v>
+      </c>
+      <c r="K527" s="15" t="inlineStr">
+        <is>
+          <t>USDC 161,856.7587</t>
+        </is>
+      </c>
+      <c r="L527" s="17" t="n">
+        <v>161856.7586590647</v>
+      </c>
+      <c r="M527" s="17">
+        <f>J527-L527</f>
+        <v/>
+      </c>
+      <c r="N527" s="18">
+        <f>IF(J527=0,"",L527/J527)</f>
+        <v/>
+      </c>
+      <c r="O527" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:14:55</t>
+        </is>
+      </c>
+      <c r="B528" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C528" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D528" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E528" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F528" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G528" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H528" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I528" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J528" s="17" t="n">
+        <v>327650.1482568324</v>
+      </c>
+      <c r="K528" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L528" s="17" t="n">
+        <v>280287.6324217733</v>
+      </c>
+      <c r="M528" s="17">
+        <f>J528-L528</f>
+        <v/>
+      </c>
+      <c r="N528" s="18">
+        <f>IF(J528=0,"",L528/J528)</f>
+        <v/>
+      </c>
+      <c r="O528" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:14:55</t>
+        </is>
+      </c>
+      <c r="B529" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C529" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D529" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E529" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F529" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G529" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H529" s="16" t="n">
+        <v>1.1298</v>
+      </c>
+      <c r="I529" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J529" s="17" t="n">
+        <v>159973.89264</v>
+      </c>
+      <c r="K529" s="15" t="inlineStr">
+        <is>
+          <t>USDC 119,584.3639</t>
+        </is>
+      </c>
+      <c r="L529" s="17" t="n">
+        <v>119584.3639445559</v>
+      </c>
+      <c r="M529" s="17">
+        <f>J529-L529</f>
+        <v/>
+      </c>
+      <c r="N529" s="18">
+        <f>IF(J529=0,"",L529/J529)</f>
+        <v/>
+      </c>
+      <c r="O529" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:14:55</t>
+        </is>
+      </c>
+      <c r="B530" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C530" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D530" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E530" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F530" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G530" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H530" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I530" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J530" s="17" t="n">
+        <v>160146.7637106622</v>
+      </c>
+      <c r="K530" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,521.1458</t>
+        </is>
+      </c>
+      <c r="L530" s="17" t="n">
+        <v>138493.4415612677</v>
+      </c>
+      <c r="M530" s="17">
+        <f>J530-L530</f>
+        <v/>
+      </c>
+      <c r="N530" s="18">
+        <f>IF(J530=0,"",L530/J530)</f>
+        <v/>
+      </c>
+      <c r="O530" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:14:55</t>
+        </is>
+      </c>
+      <c r="B531" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C531" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D531" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E531" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F531" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeef003c</t>
+        </is>
+      </c>
+      <c r="G531" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H531" s="16" t="inlineStr"/>
+      <c r="I531" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,803.9136</t>
+        </is>
+      </c>
+      <c r="J531" s="17" t="n">
+        <v>50795.78493483024</v>
+      </c>
+      <c r="K531" s="15" t="inlineStr"/>
+      <c r="L531" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M531" s="17">
+        <f>J531-L531</f>
+        <v/>
+      </c>
+      <c r="N531" s="18">
+        <f>IF(J531=0,"",L531/J531)</f>
+        <v/>
+      </c>
+      <c r="O531" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:14:55</t>
+        </is>
+      </c>
+      <c r="B532" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C532" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D532" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E532" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F532" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbeeff047</t>
+        </is>
+      </c>
+      <c r="G532" s="15" t="inlineStr">
+        <is>
+          <t>USDC vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H532" s="16" t="inlineStr"/>
+      <c r="I532" s="15" t="inlineStr">
+        <is>
+          <t>USDC 48,650.0864</t>
+        </is>
+      </c>
+      <c r="J532" s="17" t="n">
+        <v>48650.086392</v>
+      </c>
+      <c r="K532" s="15" t="inlineStr"/>
+      <c r="L532" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M532" s="17">
+        <f>J532-L532</f>
+        <v/>
+      </c>
+      <c r="N532" s="18">
+        <f>IF(J532=0,"",L532/J532)</f>
+        <v/>
+      </c>
+      <c r="O532" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:14:55</t>
+        </is>
+      </c>
+      <c r="B533" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C533" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D533" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E533" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F533" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G533" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H533" s="16" t="inlineStr"/>
+      <c r="I533" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J533" s="17" t="n">
+        <v>95923.17613126275</v>
+      </c>
+      <c r="K533" s="15" t="inlineStr"/>
+      <c r="L533" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M533" s="17">
+        <f>J533-L533</f>
+        <v/>
+      </c>
+      <c r="N533" s="18">
+        <f>IF(J533=0,"",L533/J533)</f>
+        <v/>
+      </c>
+      <c r="O533" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:14:55</t>
+        </is>
+      </c>
+      <c r="B534" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C534" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D534" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E534" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F534" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G534" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H534" s="16" t="inlineStr"/>
+      <c r="I534" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J534" s="17" t="n">
+        <v>34346.01537379431</v>
+      </c>
+      <c r="K534" s="15" t="inlineStr"/>
+      <c r="L534" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M534" s="17">
+        <f>J534-L534</f>
+        <v/>
+      </c>
+      <c r="N534" s="18">
+        <f>IF(J534=0,"",L534/J534)</f>
+        <v/>
+      </c>
+      <c r="O534" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:14:55</t>
+        </is>
+      </c>
+      <c r="B535" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C535" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D535" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E535" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F535" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G535" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H535" s="16" t="n">
+        <v>1.0429</v>
+      </c>
+      <c r="I535" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J535" s="17" t="n">
+        <v>269996.1113129806</v>
+      </c>
+      <c r="K535" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,036.0347</t>
+        </is>
+      </c>
+      <c r="L535" s="17" t="n">
+        <v>232998.7489714421</v>
+      </c>
+      <c r="M535" s="17">
+        <f>J535-L535</f>
+        <v/>
+      </c>
+      <c r="N535" s="18">
+        <f>IF(J535=0,"",L535/J535)</f>
+        <v/>
+      </c>
+      <c r="O535" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:14:55</t>
+        </is>
+      </c>
+      <c r="B536" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C536" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D536" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E536" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F536" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G536" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H536" s="16" t="inlineStr"/>
+      <c r="I536" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,509.8036</t>
+        </is>
+      </c>
+      <c r="J536" s="17" t="n">
+        <v>15507.32207780672</v>
+      </c>
+      <c r="K536" s="15" t="inlineStr"/>
+      <c r="L536" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M536" s="17">
+        <f>J536-L536</f>
+        <v/>
+      </c>
+      <c r="N536" s="18">
+        <f>IF(J536=0,"",L536/J536)</f>
+        <v/>
+      </c>
+      <c r="O536" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:14:55</t>
+        </is>
+      </c>
+      <c r="B537" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C537" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D537" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E537" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F537" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G537" s="15" t="inlineStr">
+        <is>
+          <t>5Y8NV3 vs USDC</t>
+        </is>
+      </c>
+      <c r="H537" s="16" t="inlineStr"/>
+      <c r="I537" s="15" t="inlineStr">
+        <is>
+          <t>5Y8NV3 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J537" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K537" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,705.3454</t>
+        </is>
+      </c>
+      <c r="L537" s="17" t="n">
+        <v>148705.345409</v>
+      </c>
+      <c r="M537" s="17">
+        <f>J537-L537</f>
+        <v/>
+      </c>
+      <c r="N537" s="18">
+        <f>IF(J537=0,"",L537/J537)</f>
+        <v/>
+      </c>
+      <c r="O537" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:14:55</t>
+        </is>
+      </c>
+      <c r="B538" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C538" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D538" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E538" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F538" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G538" s="15" t="inlineStr">
+        <is>
+          <t>3B8X44 vs USDC</t>
+        </is>
+      </c>
+      <c r="H538" s="16" t="inlineStr"/>
+      <c r="I538" s="15" t="inlineStr">
+        <is>
+          <t>3B8X44 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J538" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K538" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,944.5758</t>
+        </is>
+      </c>
+      <c r="L538" s="17" t="n">
+        <v>251944.575822</v>
+      </c>
+      <c r="M538" s="17">
+        <f>J538-L538</f>
+        <v/>
+      </c>
+      <c r="N538" s="18">
+        <f>IF(J538=0,"",L538/J538)</f>
+        <v/>
+      </c>
+      <c r="O538" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -35469,7 +36608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -36745,6 +37884,41 @@
         <v>1.0375</v>
       </c>
       <c r="I36" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:14:55</t>
+        </is>
+      </c>
+      <c r="B37" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C37" s="17" t="n">
+        <v>553658.9179861409</v>
+      </c>
+      <c r="D37" s="17" t="n">
+        <v>150389.2842194126</v>
+      </c>
+      <c r="E37" s="17" t="n">
+        <v>2479630.108492929</v>
+      </c>
+      <c r="F37" s="17" t="n">
+        <v>2329240.824273516</v>
+      </c>
+      <c r="G37" s="15" t="n">
+        <v>17</v>
+      </c>
+      <c r="H37" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I37" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 10:45 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O538"/>
+  <dimension ref="A1:O554"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -36578,6 +36578,1088 @@
         <v/>
       </c>
       <c r="O538" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:45:09</t>
+        </is>
+      </c>
+      <c r="B539" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C539" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D539" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E539" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F539" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G539" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H539" s="16" t="n">
+        <v>1.0505</v>
+      </c>
+      <c r="I539" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,804.4771</t>
+        </is>
+      </c>
+      <c r="J539" s="17" t="n">
+        <v>50791.775948733</v>
+      </c>
+      <c r="K539" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,722.8304</t>
+        </is>
+      </c>
+      <c r="L539" s="17" t="n">
+        <v>37722.830445</v>
+      </c>
+      <c r="M539" s="17">
+        <f>J539-L539</f>
+        <v/>
+      </c>
+      <c r="N539" s="18">
+        <f>IF(J539=0,"",L539/J539)</f>
+        <v/>
+      </c>
+      <c r="O539" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:45:09</t>
+        </is>
+      </c>
+      <c r="B540" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C540" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D540" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E540" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F540" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G540" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H540" s="16" t="n">
+        <v>1.0482</v>
+      </c>
+      <c r="I540" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J540" s="17" t="n">
+        <v>140925.8943799527</v>
+      </c>
+      <c r="K540" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,032.5316</t>
+        </is>
+      </c>
+      <c r="L540" s="17" t="n">
+        <v>121002.273483096</v>
+      </c>
+      <c r="M540" s="17">
+        <f>J540-L540</f>
+        <v/>
+      </c>
+      <c r="N540" s="18">
+        <f>IF(J540=0,"",L540/J540)</f>
+        <v/>
+      </c>
+      <c r="O540" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:45:09</t>
+        </is>
+      </c>
+      <c r="B541" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C541" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D541" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E541" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F541" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G541" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H541" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I541" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J541" s="17" t="n">
+        <v>328711.8411191112</v>
+      </c>
+      <c r="K541" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,383.3066</t>
+        </is>
+      </c>
+      <c r="L541" s="17" t="n">
+        <v>306407.7213321691</v>
+      </c>
+      <c r="M541" s="17">
+        <f>J541-L541</f>
+        <v/>
+      </c>
+      <c r="N541" s="18">
+        <f>IF(J541=0,"",L541/J541)</f>
+        <v/>
+      </c>
+      <c r="O541" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:45:09</t>
+        </is>
+      </c>
+      <c r="B542" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C542" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D542" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E542" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F542" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G542" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H542" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I542" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J542" s="17" t="n">
+        <v>386053.7744188088</v>
+      </c>
+      <c r="K542" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,603.9988</t>
+        </is>
+      </c>
+      <c r="L542" s="17" t="n">
+        <v>349631.8576813329</v>
+      </c>
+      <c r="M542" s="17">
+        <f>J542-L542</f>
+        <v/>
+      </c>
+      <c r="N542" s="18">
+        <f>IF(J542=0,"",L542/J542)</f>
+        <v/>
+      </c>
+      <c r="O542" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:45:09</t>
+        </is>
+      </c>
+      <c r="B543" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C543" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D543" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E543" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F543" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G543" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H543" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I543" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7844</t>
+        </is>
+      </c>
+      <c r="J543" s="17" t="n">
+        <v>77796.40385580565</v>
+      </c>
+      <c r="K543" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,027.1079; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L543" s="17" t="n">
+        <v>68009.49841294548</v>
+      </c>
+      <c r="M543" s="17">
+        <f>J543-L543</f>
+        <v/>
+      </c>
+      <c r="N543" s="18">
+        <f>IF(J543=0,"",L543/J543)</f>
+        <v/>
+      </c>
+      <c r="O543" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:45:09</t>
+        </is>
+      </c>
+      <c r="B544" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C544" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D544" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E544" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F544" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G544" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H544" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I544" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J544" s="17" t="n">
+        <v>197092.5756871674</v>
+      </c>
+      <c r="K544" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,243.9962</t>
+        </is>
+      </c>
+      <c r="L544" s="17" t="n">
+        <v>150243.996246735</v>
+      </c>
+      <c r="M544" s="17">
+        <f>J544-L544</f>
+        <v/>
+      </c>
+      <c r="N544" s="18">
+        <f>IF(J544=0,"",L544/J544)</f>
+        <v/>
+      </c>
+      <c r="O544" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:45:09</t>
+        </is>
+      </c>
+      <c r="B545" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C545" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D545" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E545" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F545" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G545" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H545" s="16" t="n">
+        <v>1.3726</v>
+      </c>
+      <c r="I545" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J545" s="17" t="n">
+        <v>186103.94208146</v>
+      </c>
+      <c r="K545" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,140.3351</t>
+        </is>
+      </c>
+      <c r="L545" s="17" t="n">
+        <v>124140.3351430682</v>
+      </c>
+      <c r="M545" s="17">
+        <f>J545-L545</f>
+        <v/>
+      </c>
+      <c r="N545" s="18">
+        <f>IF(J545=0,"",L545/J545)</f>
+        <v/>
+      </c>
+      <c r="O545" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:45:09</t>
+        </is>
+      </c>
+      <c r="B546" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C546" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D546" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E546" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F546" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G546" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H546" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I546" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J546" s="17" t="n">
+        <v>327652.1914768068</v>
+      </c>
+      <c r="K546" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L546" s="17" t="n">
+        <v>280262.938574522</v>
+      </c>
+      <c r="M546" s="17">
+        <f>J546-L546</f>
+        <v/>
+      </c>
+      <c r="N546" s="18">
+        <f>IF(J546=0,"",L546/J546)</f>
+        <v/>
+      </c>
+      <c r="O546" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:45:09</t>
+        </is>
+      </c>
+      <c r="B547" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C547" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D547" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E547" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F547" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G547" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H547" s="16" t="n">
+        <v>1.9045</v>
+      </c>
+      <c r="I547" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J547" s="17" t="n">
+        <v>159973.89264</v>
+      </c>
+      <c r="K547" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,938.3760</t>
+        </is>
+      </c>
+      <c r="L547" s="17" t="n">
+        <v>70938.37599253547</v>
+      </c>
+      <c r="M547" s="17">
+        <f>J547-L547</f>
+        <v/>
+      </c>
+      <c r="N547" s="18">
+        <f>IF(J547=0,"",L547/J547)</f>
+        <v/>
+      </c>
+      <c r="O547" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:45:09</t>
+        </is>
+      </c>
+      <c r="B548" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C548" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D548" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E548" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F548" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G548" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H548" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I548" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J548" s="17" t="n">
+        <v>160163.2646712076</v>
+      </c>
+      <c r="K548" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,522.4734</t>
+        </is>
+      </c>
+      <c r="L548" s="17" t="n">
+        <v>138494.768870382</v>
+      </c>
+      <c r="M548" s="17">
+        <f>J548-L548</f>
+        <v/>
+      </c>
+      <c r="N548" s="18">
+        <f>IF(J548=0,"",L548/J548)</f>
+        <v/>
+      </c>
+      <c r="O548" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:45:09</t>
+        </is>
+      </c>
+      <c r="B549" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C549" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D549" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E549" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F549" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G549" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H549" s="16" t="inlineStr"/>
+      <c r="I549" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J549" s="17" t="n">
+        <v>95913.58381364963</v>
+      </c>
+      <c r="K549" s="15" t="inlineStr"/>
+      <c r="L549" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M549" s="17">
+        <f>J549-L549</f>
+        <v/>
+      </c>
+      <c r="N549" s="18">
+        <f>IF(J549=0,"",L549/J549)</f>
+        <v/>
+      </c>
+      <c r="O549" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:45:09</t>
+        </is>
+      </c>
+      <c r="B550" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C550" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D550" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E550" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F550" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G550" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H550" s="16" t="inlineStr"/>
+      <c r="I550" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J550" s="17" t="n">
+        <v>34346.32530306713</v>
+      </c>
+      <c r="K550" s="15" t="inlineStr"/>
+      <c r="L550" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M550" s="17">
+        <f>J550-L550</f>
+        <v/>
+      </c>
+      <c r="N550" s="18">
+        <f>IF(J550=0,"",L550/J550)</f>
+        <v/>
+      </c>
+      <c r="O550" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:45:09</t>
+        </is>
+      </c>
+      <c r="B551" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C551" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D551" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E551" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F551" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G551" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H551" s="16" t="n">
+        <v>1.043</v>
+      </c>
+      <c r="I551" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J551" s="17" t="n">
+        <v>269996.1113129806</v>
+      </c>
+      <c r="K551" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,036.0347</t>
+        </is>
+      </c>
+      <c r="L551" s="17" t="n">
+        <v>232975.4453679684</v>
+      </c>
+      <c r="M551" s="17">
+        <f>J551-L551</f>
+        <v/>
+      </c>
+      <c r="N551" s="18">
+        <f>IF(J551=0,"",L551/J551)</f>
+        <v/>
+      </c>
+      <c r="O551" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:45:09</t>
+        </is>
+      </c>
+      <c r="B552" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C552" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D552" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E552" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F552" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G552" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H552" s="16" t="inlineStr"/>
+      <c r="I552" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,510.0025</t>
+        </is>
+      </c>
+      <c r="J552" s="17" t="n">
+        <v>15505.96993094175</v>
+      </c>
+      <c r="K552" s="15" t="inlineStr"/>
+      <c r="L552" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M552" s="17">
+        <f>J552-L552</f>
+        <v/>
+      </c>
+      <c r="N552" s="18">
+        <f>IF(J552=0,"",L552/J552)</f>
+        <v/>
+      </c>
+      <c r="O552" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:45:09</t>
+        </is>
+      </c>
+      <c r="B553" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C553" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D553" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E553" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F553" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G553" s="15" t="inlineStr">
+        <is>
+          <t>5Y8NV3 vs USDC</t>
+        </is>
+      </c>
+      <c r="H553" s="16" t="inlineStr"/>
+      <c r="I553" s="15" t="inlineStr">
+        <is>
+          <t>5Y8NV3 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J553" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K553" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,705.3454</t>
+        </is>
+      </c>
+      <c r="L553" s="17" t="n">
+        <v>148705.345409</v>
+      </c>
+      <c r="M553" s="17">
+        <f>J553-L553</f>
+        <v/>
+      </c>
+      <c r="N553" s="18">
+        <f>IF(J553=0,"",L553/J553)</f>
+        <v/>
+      </c>
+      <c r="O553" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:45:09</t>
+        </is>
+      </c>
+      <c r="B554" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C554" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D554" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E554" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F554" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G554" s="15" t="inlineStr">
+        <is>
+          <t>3B8X44 vs USDC</t>
+        </is>
+      </c>
+      <c r="H554" s="16" t="inlineStr"/>
+      <c r="I554" s="15" t="inlineStr">
+        <is>
+          <t>3B8X44 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J554" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K554" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,944.5758</t>
+        </is>
+      </c>
+      <c r="L554" s="17" t="n">
+        <v>251944.575822</v>
+      </c>
+      <c r="M554" s="17">
+        <f>J554-L554</f>
+        <v/>
+      </c>
+      <c r="N554" s="18">
+        <f>IF(J554=0,"",L554/J554)</f>
+        <v/>
+      </c>
+      <c r="O554" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -36608,7 +37690,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -37919,6 +39001,41 @@
         <v>1.0375</v>
       </c>
       <c r="I37" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:45:09</t>
+        </is>
+      </c>
+      <c r="B38" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C38" s="17" t="n">
+        <v>553811.6433279482</v>
+      </c>
+      <c r="D38" s="17" t="n">
+        <v>150547.5838589375</v>
+      </c>
+      <c r="E38" s="17" t="n">
+        <v>2431027.546639692</v>
+      </c>
+      <c r="F38" s="17" t="n">
+        <v>2280479.962780755</v>
+      </c>
+      <c r="G38" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H38" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I38" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 11:15 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O554"/>
+  <dimension ref="A1:O570"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -37660,6 +37660,1088 @@
         <v/>
       </c>
       <c r="O554" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:15:23</t>
+        </is>
+      </c>
+      <c r="B555" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C555" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D555" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E555" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F555" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G555" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H555" s="16" t="n">
+        <v>1.0505</v>
+      </c>
+      <c r="I555" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,804.5477</t>
+        </is>
+      </c>
+      <c r="J555" s="17" t="n">
+        <v>50791.33848060761</v>
+      </c>
+      <c r="K555" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,722.8797</t>
+        </is>
+      </c>
+      <c r="L555" s="17" t="n">
+        <v>37722.87969</v>
+      </c>
+      <c r="M555" s="17">
+        <f>J555-L555</f>
+        <v/>
+      </c>
+      <c r="N555" s="18">
+        <f>IF(J555=0,"",L555/J555)</f>
+        <v/>
+      </c>
+      <c r="O555" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:15:23</t>
+        </is>
+      </c>
+      <c r="B556" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C556" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D556" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E556" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F556" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G556" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H556" s="16" t="n">
+        <v>1.0483</v>
+      </c>
+      <c r="I556" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J556" s="17" t="n">
+        <v>140940.4373357883</v>
+      </c>
+      <c r="K556" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,035.0439</t>
+        </is>
+      </c>
+      <c r="L556" s="17" t="n">
+        <v>121003.574815579</v>
+      </c>
+      <c r="M556" s="17">
+        <f>J556-L556</f>
+        <v/>
+      </c>
+      <c r="N556" s="18">
+        <f>IF(J556=0,"",L556/J556)</f>
+        <v/>
+      </c>
+      <c r="O556" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:15:23</t>
+        </is>
+      </c>
+      <c r="B557" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C557" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D557" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E557" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F557" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G557" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H557" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I557" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J557" s="17" t="n">
+        <v>328711.9942525551</v>
+      </c>
+      <c r="K557" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,386.0522</t>
+        </is>
+      </c>
+      <c r="L557" s="17" t="n">
+        <v>306441.1081603671</v>
+      </c>
+      <c r="M557" s="17">
+        <f>J557-L557</f>
+        <v/>
+      </c>
+      <c r="N557" s="18">
+        <f>IF(J557=0,"",L557/J557)</f>
+        <v/>
+      </c>
+      <c r="O557" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:15:23</t>
+        </is>
+      </c>
+      <c r="B558" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C558" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D558" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E558" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F558" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G558" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H558" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I558" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J558" s="17" t="n">
+        <v>386054.6275051957</v>
+      </c>
+      <c r="K558" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,608.2120</t>
+        </is>
+      </c>
+      <c r="L558" s="17" t="n">
+        <v>349671.0347680777</v>
+      </c>
+      <c r="M558" s="17">
+        <f>J558-L558</f>
+        <v/>
+      </c>
+      <c r="N558" s="18">
+        <f>IF(J558=0,"",L558/J558)</f>
+        <v/>
+      </c>
+      <c r="O558" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:15:23</t>
+        </is>
+      </c>
+      <c r="B559" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C559" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D559" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E559" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F559" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G559" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H559" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I559" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7848</t>
+        </is>
+      </c>
+      <c r="J559" s="17" t="n">
+        <v>77803.39161506922</v>
+      </c>
+      <c r="K559" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,028.1988; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L559" s="17" t="n">
+        <v>68010.58907729926</v>
+      </c>
+      <c r="M559" s="17">
+        <f>J559-L559</f>
+        <v/>
+      </c>
+      <c r="N559" s="18">
+        <f>IF(J559=0,"",L559/J559)</f>
+        <v/>
+      </c>
+      <c r="O559" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:15:23</t>
+        </is>
+      </c>
+      <c r="B560" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C560" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D560" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E560" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F560" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G560" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H560" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I560" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J560" s="17" t="n">
+        <v>197093.7433166031</v>
+      </c>
+      <c r="K560" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,243.9962</t>
+        </is>
+      </c>
+      <c r="L560" s="17" t="n">
+        <v>150243.996246735</v>
+      </c>
+      <c r="M560" s="17">
+        <f>J560-L560</f>
+        <v/>
+      </c>
+      <c r="N560" s="18">
+        <f>IF(J560=0,"",L560/J560)</f>
+        <v/>
+      </c>
+      <c r="O560" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:15:23</t>
+        </is>
+      </c>
+      <c r="B561" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C561" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D561" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E561" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F561" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G561" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H561" s="16" t="n">
+        <v>1.3726</v>
+      </c>
+      <c r="I561" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J561" s="17" t="n">
+        <v>186104.5555383066</v>
+      </c>
+      <c r="K561" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,140.3351</t>
+        </is>
+      </c>
+      <c r="L561" s="17" t="n">
+        <v>124140.3351430682</v>
+      </c>
+      <c r="M561" s="17">
+        <f>J561-L561</f>
+        <v/>
+      </c>
+      <c r="N561" s="18">
+        <f>IF(J561=0,"",L561/J561)</f>
+        <v/>
+      </c>
+      <c r="O561" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:15:23</t>
+        </is>
+      </c>
+      <c r="B562" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C562" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D562" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E562" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F562" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G562" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H562" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I562" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J562" s="17" t="n">
+        <v>327656.700532752</v>
+      </c>
+      <c r="K562" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L562" s="17" t="n">
+        <v>280262.1130298798</v>
+      </c>
+      <c r="M562" s="17">
+        <f>J562-L562</f>
+        <v/>
+      </c>
+      <c r="N562" s="18">
+        <f>IF(J562=0,"",L562/J562)</f>
+        <v/>
+      </c>
+      <c r="O562" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:15:23</t>
+        </is>
+      </c>
+      <c r="B563" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C563" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D563" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E563" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F563" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G563" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H563" s="16" t="n">
+        <v>1.9045</v>
+      </c>
+      <c r="I563" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J563" s="17" t="n">
+        <v>159973.89264</v>
+      </c>
+      <c r="K563" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,938.3760</t>
+        </is>
+      </c>
+      <c r="L563" s="17" t="n">
+        <v>70938.37599253547</v>
+      </c>
+      <c r="M563" s="17">
+        <f>J563-L563</f>
+        <v/>
+      </c>
+      <c r="N563" s="18">
+        <f>IF(J563=0,"",L563/J563)</f>
+        <v/>
+      </c>
+      <c r="O563" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:15:23</t>
+        </is>
+      </c>
+      <c r="B564" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C564" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D564" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E564" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F564" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G564" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H564" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I564" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J564" s="17" t="n">
+        <v>160163.6185936656</v>
+      </c>
+      <c r="K564" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,523.0271</t>
+        </is>
+      </c>
+      <c r="L564" s="17" t="n">
+        <v>138495.3224502363</v>
+      </c>
+      <c r="M564" s="17">
+        <f>J564-L564</f>
+        <v/>
+      </c>
+      <c r="N564" s="18">
+        <f>IF(J564=0,"",L564/J564)</f>
+        <v/>
+      </c>
+      <c r="O564" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:15:23</t>
+        </is>
+      </c>
+      <c r="B565" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C565" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D565" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E565" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F565" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G565" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H565" s="16" t="inlineStr"/>
+      <c r="I565" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J565" s="17" t="n">
+        <v>95913.58381364963</v>
+      </c>
+      <c r="K565" s="15" t="inlineStr"/>
+      <c r="L565" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M565" s="17">
+        <f>J565-L565</f>
+        <v/>
+      </c>
+      <c r="N565" s="18">
+        <f>IF(J565=0,"",L565/J565)</f>
+        <v/>
+      </c>
+      <c r="O565" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:15:23</t>
+        </is>
+      </c>
+      <c r="B566" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C566" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D566" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E566" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F566" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G566" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H566" s="16" t="inlineStr"/>
+      <c r="I566" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J566" s="17" t="n">
+        <v>34346.52402389589</v>
+      </c>
+      <c r="K566" s="15" t="inlineStr"/>
+      <c r="L566" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M566" s="17">
+        <f>J566-L566</f>
+        <v/>
+      </c>
+      <c r="N566" s="18">
+        <f>IF(J566=0,"",L566/J566)</f>
+        <v/>
+      </c>
+      <c r="O566" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:15:23</t>
+        </is>
+      </c>
+      <c r="B567" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C567" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D567" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E567" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F567" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G567" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H567" s="16" t="n">
+        <v>1.043</v>
+      </c>
+      <c r="I567" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J567" s="17" t="n">
+        <v>269996.1113129806</v>
+      </c>
+      <c r="K567" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,041.5307</t>
+        </is>
+      </c>
+      <c r="L567" s="17" t="n">
+        <v>232980.9398690266</v>
+      </c>
+      <c r="M567" s="17">
+        <f>J567-L567</f>
+        <v/>
+      </c>
+      <c r="N567" s="18">
+        <f>IF(J567=0,"",L567/J567)</f>
+        <v/>
+      </c>
+      <c r="O567" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:15:23</t>
+        </is>
+      </c>
+      <c r="B568" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C568" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D568" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E568" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F568" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G568" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H568" s="16" t="inlineStr"/>
+      <c r="I568" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,510.2065</t>
+        </is>
+      </c>
+      <c r="J568" s="17" t="n">
+        <v>15506.17381667434</v>
+      </c>
+      <c r="K568" s="15" t="inlineStr"/>
+      <c r="L568" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M568" s="17">
+        <f>J568-L568</f>
+        <v/>
+      </c>
+      <c r="N568" s="18">
+        <f>IF(J568=0,"",L568/J568)</f>
+        <v/>
+      </c>
+      <c r="O568" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:15:23</t>
+        </is>
+      </c>
+      <c r="B569" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C569" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D569" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E569" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F569" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G569" s="15" t="inlineStr">
+        <is>
+          <t>5Y8NV3 vs USDC</t>
+        </is>
+      </c>
+      <c r="H569" s="16" t="inlineStr"/>
+      <c r="I569" s="15" t="inlineStr">
+        <is>
+          <t>5Y8NV3 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J569" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K569" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,705.3454</t>
+        </is>
+      </c>
+      <c r="L569" s="17" t="n">
+        <v>148705.345409</v>
+      </c>
+      <c r="M569" s="17">
+        <f>J569-L569</f>
+        <v/>
+      </c>
+      <c r="N569" s="18">
+        <f>IF(J569=0,"",L569/J569)</f>
+        <v/>
+      </c>
+      <c r="O569" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:15:23</t>
+        </is>
+      </c>
+      <c r="B570" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C570" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D570" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E570" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F570" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G570" s="15" t="inlineStr">
+        <is>
+          <t>3B8X44 vs USDC</t>
+        </is>
+      </c>
+      <c r="H570" s="16" t="inlineStr"/>
+      <c r="I570" s="15" t="inlineStr">
+        <is>
+          <t>3B8X44 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J570" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K570" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,944.5758</t>
+        </is>
+      </c>
+      <c r="L570" s="17" t="n">
+        <v>251944.575822</v>
+      </c>
+      <c r="M570" s="17">
+        <f>J570-L570</f>
+        <v/>
+      </c>
+      <c r="N570" s="18">
+        <f>IF(J570=0,"",L570/J570)</f>
+        <v/>
+      </c>
+      <c r="O570" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -37690,7 +38772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -39036,6 +40118,41 @@
         <v>1.0375</v>
       </c>
       <c r="I38" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:15:23</t>
+        </is>
+      </c>
+      <c r="B39" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C39" s="17" t="n">
+        <v>553760.3548574185</v>
+      </c>
+      <c r="D39" s="17" t="n">
+        <v>150496.5023039398</v>
+      </c>
+      <c r="E39" s="17" t="n">
+        <v>2431056.692777744</v>
+      </c>
+      <c r="F39" s="17" t="n">
+        <v>2280560.190473804</v>
+      </c>
+      <c r="G39" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H39" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I39" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 11:45 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O570"/>
+  <dimension ref="A1:O586"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -38742,6 +38742,1088 @@
         <v/>
       </c>
       <c r="O570" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:45:34</t>
+        </is>
+      </c>
+      <c r="B571" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C571" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D571" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E571" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F571" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G571" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H571" s="16" t="n">
+        <v>1.0505</v>
+      </c>
+      <c r="I571" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,804.5477</t>
+        </is>
+      </c>
+      <c r="J571" s="17" t="n">
+        <v>50794.89479894403</v>
+      </c>
+      <c r="K571" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,722.8797</t>
+        </is>
+      </c>
+      <c r="L571" s="17" t="n">
+        <v>37722.87969</v>
+      </c>
+      <c r="M571" s="17">
+        <f>J571-L571</f>
+        <v/>
+      </c>
+      <c r="N571" s="18">
+        <f>IF(J571=0,"",L571/J571)</f>
+        <v/>
+      </c>
+      <c r="O571" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:45:34</t>
+        </is>
+      </c>
+      <c r="B572" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C572" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D572" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E572" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F572" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G572" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H572" s="16" t="n">
+        <v>1.048</v>
+      </c>
+      <c r="I572" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J572" s="17" t="n">
+        <v>140908.692557649</v>
+      </c>
+      <c r="K572" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,035.0439</t>
+        </is>
+      </c>
+      <c r="L572" s="17" t="n">
+        <v>121012.0472686539</v>
+      </c>
+      <c r="M572" s="17">
+        <f>J572-L572</f>
+        <v/>
+      </c>
+      <c r="N572" s="18">
+        <f>IF(J572=0,"",L572/J572)</f>
+        <v/>
+      </c>
+      <c r="O572" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:45:34</t>
+        </is>
+      </c>
+      <c r="B573" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C573" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D573" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E573" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F573" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G573" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H573" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I573" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J573" s="17" t="n">
+        <v>328712.6594267799</v>
+      </c>
+      <c r="K573" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,386.0522</t>
+        </is>
+      </c>
+      <c r="L573" s="17" t="n">
+        <v>306440.803830472</v>
+      </c>
+      <c r="M573" s="17">
+        <f>J573-L573</f>
+        <v/>
+      </c>
+      <c r="N573" s="18">
+        <f>IF(J573=0,"",L573/J573)</f>
+        <v/>
+      </c>
+      <c r="O573" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:45:34</t>
+        </is>
+      </c>
+      <c r="B574" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C574" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D574" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E574" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F574" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G574" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H574" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I574" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J574" s="17" t="n">
+        <v>386012.095122674</v>
+      </c>
+      <c r="K574" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,608.2120</t>
+        </is>
+      </c>
+      <c r="L574" s="17" t="n">
+        <v>349670.6875060867</v>
+      </c>
+      <c r="M574" s="17">
+        <f>J574-L574</f>
+        <v/>
+      </c>
+      <c r="N574" s="18">
+        <f>IF(J574=0,"",L574/J574)</f>
+        <v/>
+      </c>
+      <c r="O574" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:45:34</t>
+        </is>
+      </c>
+      <c r="B575" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C575" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D575" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E575" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F575" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G575" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H575" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I575" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7848</t>
+        </is>
+      </c>
+      <c r="J575" s="17" t="n">
+        <v>77794.80619645389</v>
+      </c>
+      <c r="K575" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,028.1988; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L575" s="17" t="n">
+        <v>68015.35105121869</v>
+      </c>
+      <c r="M575" s="17">
+        <f>J575-L575</f>
+        <v/>
+      </c>
+      <c r="N575" s="18">
+        <f>IF(J575=0,"",L575/J575)</f>
+        <v/>
+      </c>
+      <c r="O575" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:45:34</t>
+        </is>
+      </c>
+      <c r="B576" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C576" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D576" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E576" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F576" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G576" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H576" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I576" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J576" s="17" t="n">
+        <v>197115.6293339655</v>
+      </c>
+      <c r="K576" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,243.9962</t>
+        </is>
+      </c>
+      <c r="L576" s="17" t="n">
+        <v>150243.996246735</v>
+      </c>
+      <c r="M576" s="17">
+        <f>J576-L576</f>
+        <v/>
+      </c>
+      <c r="N576" s="18">
+        <f>IF(J576=0,"",L576/J576)</f>
+        <v/>
+      </c>
+      <c r="O576" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:45:34</t>
+        </is>
+      </c>
+      <c r="B577" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C577" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D577" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E577" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F577" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G577" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H577" s="16" t="n">
+        <v>1.3726</v>
+      </c>
+      <c r="I577" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J577" s="17" t="n">
+        <v>186063.9244378032</v>
+      </c>
+      <c r="K577" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,140.3351</t>
+        </is>
+      </c>
+      <c r="L577" s="17" t="n">
+        <v>124140.3351430682</v>
+      </c>
+      <c r="M577" s="17">
+        <f>J577-L577</f>
+        <v/>
+      </c>
+      <c r="N577" s="18">
+        <f>IF(J577=0,"",L577/J577)</f>
+        <v/>
+      </c>
+      <c r="O577" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:45:34</t>
+        </is>
+      </c>
+      <c r="B578" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C578" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D578" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E578" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F578" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G578" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H578" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I578" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J578" s="17" t="n">
+        <v>327655.0954997402</v>
+      </c>
+      <c r="K578" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L578" s="17" t="n">
+        <v>280286.8901707486</v>
+      </c>
+      <c r="M578" s="17">
+        <f>J578-L578</f>
+        <v/>
+      </c>
+      <c r="N578" s="18">
+        <f>IF(J578=0,"",L578/J578)</f>
+        <v/>
+      </c>
+      <c r="O578" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:45:34</t>
+        </is>
+      </c>
+      <c r="B579" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C579" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D579" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E579" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F579" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G579" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H579" s="16" t="n">
+        <v>1.9045</v>
+      </c>
+      <c r="I579" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J579" s="17" t="n">
+        <v>159973.89264</v>
+      </c>
+      <c r="K579" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,938.3760</t>
+        </is>
+      </c>
+      <c r="L579" s="17" t="n">
+        <v>70938.37599253547</v>
+      </c>
+      <c r="M579" s="17">
+        <f>J579-L579</f>
+        <v/>
+      </c>
+      <c r="N579" s="18">
+        <f>IF(J579=0,"",L579/J579)</f>
+        <v/>
+      </c>
+      <c r="O579" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:45:34</t>
+        </is>
+      </c>
+      <c r="B580" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C580" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D580" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E580" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F580" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G580" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H580" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I580" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J580" s="17" t="n">
+        <v>160145.9730590528</v>
+      </c>
+      <c r="K580" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,523.0271</t>
+        </is>
+      </c>
+      <c r="L580" s="17" t="n">
+        <v>138509.1747529419</v>
+      </c>
+      <c r="M580" s="17">
+        <f>J580-L580</f>
+        <v/>
+      </c>
+      <c r="N580" s="18">
+        <f>IF(J580=0,"",L580/J580)</f>
+        <v/>
+      </c>
+      <c r="O580" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:45:34</t>
+        </is>
+      </c>
+      <c r="B581" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C581" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D581" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E581" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F581" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G581" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H581" s="16" t="inlineStr"/>
+      <c r="I581" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J581" s="17" t="n">
+        <v>95892.31038181752</v>
+      </c>
+      <c r="K581" s="15" t="inlineStr"/>
+      <c r="L581" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M581" s="17">
+        <f>J581-L581</f>
+        <v/>
+      </c>
+      <c r="N581" s="18">
+        <f>IF(J581=0,"",L581/J581)</f>
+        <v/>
+      </c>
+      <c r="O581" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:45:34</t>
+        </is>
+      </c>
+      <c r="B582" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C582" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D582" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E582" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F582" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G582" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H582" s="16" t="inlineStr"/>
+      <c r="I582" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J582" s="17" t="n">
+        <v>34346.81025683506</v>
+      </c>
+      <c r="K582" s="15" t="inlineStr"/>
+      <c r="L582" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M582" s="17">
+        <f>J582-L582</f>
+        <v/>
+      </c>
+      <c r="N582" s="18">
+        <f>IF(J582=0,"",L582/J582)</f>
+        <v/>
+      </c>
+      <c r="O582" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:45:34</t>
+        </is>
+      </c>
+      <c r="B583" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C583" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D583" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E583" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F583" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G583" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H583" s="16" t="n">
+        <v>1.0429</v>
+      </c>
+      <c r="I583" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J583" s="17" t="n">
+        <v>269996.1113129806</v>
+      </c>
+      <c r="K583" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,041.5307</t>
+        </is>
+      </c>
+      <c r="L583" s="17" t="n">
+        <v>232997.2527761733</v>
+      </c>
+      <c r="M583" s="17">
+        <f>J583-L583</f>
+        <v/>
+      </c>
+      <c r="N583" s="18">
+        <f>IF(J583=0,"",L583/J583)</f>
+        <v/>
+      </c>
+      <c r="O583" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:45:34</t>
+        </is>
+      </c>
+      <c r="B584" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C584" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D584" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E584" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F584" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G584" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H584" s="16" t="inlineStr"/>
+      <c r="I584" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,510.4028</t>
+        </is>
+      </c>
+      <c r="J584" s="17" t="n">
+        <v>15507.45579611688</v>
+      </c>
+      <c r="K584" s="15" t="inlineStr"/>
+      <c r="L584" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M584" s="17">
+        <f>J584-L584</f>
+        <v/>
+      </c>
+      <c r="N584" s="18">
+        <f>IF(J584=0,"",L584/J584)</f>
+        <v/>
+      </c>
+      <c r="O584" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:45:34</t>
+        </is>
+      </c>
+      <c r="B585" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C585" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D585" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E585" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F585" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G585" s="15" t="inlineStr">
+        <is>
+          <t>5Y8NV3 vs USDC</t>
+        </is>
+      </c>
+      <c r="H585" s="16" t="inlineStr"/>
+      <c r="I585" s="15" t="inlineStr">
+        <is>
+          <t>5Y8NV3 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J585" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K585" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,705.3454</t>
+        </is>
+      </c>
+      <c r="L585" s="17" t="n">
+        <v>148705.345409</v>
+      </c>
+      <c r="M585" s="17">
+        <f>J585-L585</f>
+        <v/>
+      </c>
+      <c r="N585" s="18">
+        <f>IF(J585=0,"",L585/J585)</f>
+        <v/>
+      </c>
+      <c r="O585" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:45:34</t>
+        </is>
+      </c>
+      <c r="B586" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C586" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D586" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E586" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F586" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G586" s="15" t="inlineStr">
+        <is>
+          <t>3B8X44 vs USDC</t>
+        </is>
+      </c>
+      <c r="H586" s="16" t="inlineStr"/>
+      <c r="I586" s="15" t="inlineStr">
+        <is>
+          <t>3B8X44 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J586" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K586" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,944.5758</t>
+        </is>
+      </c>
+      <c r="L586" s="17" t="n">
+        <v>251944.575822</v>
+      </c>
+      <c r="M586" s="17">
+        <f>J586-L586</f>
+        <v/>
+      </c>
+      <c r="N586" s="18">
+        <f>IF(J586=0,"",L586/J586)</f>
+        <v/>
+      </c>
+      <c r="O586" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -38772,7 +39854,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -40153,6 +41235,41 @@
         <v>1.0375</v>
       </c>
       <c r="I39" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:45:34</t>
+        </is>
+      </c>
+      <c r="B40" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C40" s="17" t="n">
+        <v>553556.4349355834</v>
+      </c>
+      <c r="D40" s="17" t="n">
+        <v>150292.6351611791</v>
+      </c>
+      <c r="E40" s="17" t="n">
+        <v>2430920.350820813</v>
+      </c>
+      <c r="F40" s="17" t="n">
+        <v>2280627.715659634</v>
+      </c>
+      <c r="G40" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H40" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I40" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 12:15 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O586"/>
+  <dimension ref="A1:O602"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -39824,6 +39824,1088 @@
         <v/>
       </c>
       <c r="O586" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:15:46</t>
+        </is>
+      </c>
+      <c r="B587" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C587" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D587" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E587" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F587" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G587" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H587" s="16" t="n">
+        <v>1.0505</v>
+      </c>
+      <c r="I587" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,804.5477</t>
+        </is>
+      </c>
+      <c r="J587" s="17" t="n">
+        <v>50795.40284442066</v>
+      </c>
+      <c r="K587" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,722.8797</t>
+        </is>
+      </c>
+      <c r="L587" s="17" t="n">
+        <v>37726.65235523552</v>
+      </c>
+      <c r="M587" s="17">
+        <f>J587-L587</f>
+        <v/>
+      </c>
+      <c r="N587" s="18">
+        <f>IF(J587=0,"",L587/J587)</f>
+        <v/>
+      </c>
+      <c r="O587" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:15:46</t>
+        </is>
+      </c>
+      <c r="B588" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C588" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D588" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E588" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F588" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G588" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H588" s="16" t="n">
+        <v>1.0479</v>
+      </c>
+      <c r="I588" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J588" s="17" t="n">
+        <v>140898.26974397</v>
+      </c>
+      <c r="K588" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,035.0439</t>
+        </is>
+      </c>
+      <c r="L588" s="17" t="n">
+        <v>121013.2576190932</v>
+      </c>
+      <c r="M588" s="17">
+        <f>J588-L588</f>
+        <v/>
+      </c>
+      <c r="N588" s="18">
+        <f>IF(J588=0,"",L588/J588)</f>
+        <v/>
+      </c>
+      <c r="O588" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:15:46</t>
+        </is>
+      </c>
+      <c r="B589" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C589" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D589" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E589" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F589" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G589" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H589" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I589" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J589" s="17" t="n">
+        <v>328713.3915985258</v>
+      </c>
+      <c r="K589" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,386.0522</t>
+        </is>
+      </c>
+      <c r="L589" s="17" t="n">
+        <v>306440.807458109</v>
+      </c>
+      <c r="M589" s="17">
+        <f>J589-L589</f>
+        <v/>
+      </c>
+      <c r="N589" s="18">
+        <f>IF(J589=0,"",L589/J589)</f>
+        <v/>
+      </c>
+      <c r="O589" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:15:46</t>
+        </is>
+      </c>
+      <c r="B590" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C590" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D590" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E590" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F590" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G590" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H590" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I590" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J590" s="17" t="n">
+        <v>386017.8432330946</v>
+      </c>
+      <c r="K590" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,608.2120</t>
+        </is>
+      </c>
+      <c r="L590" s="17" t="n">
+        <v>349670.6916454778</v>
+      </c>
+      <c r="M590" s="17">
+        <f>J590-L590</f>
+        <v/>
+      </c>
+      <c r="N590" s="18">
+        <f>IF(J590=0,"",L590/J590)</f>
+        <v/>
+      </c>
+      <c r="O590" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:15:46</t>
+        </is>
+      </c>
+      <c r="B591" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C591" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D591" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E591" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F591" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G591" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H591" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I591" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7848</t>
+        </is>
+      </c>
+      <c r="J591" s="17" t="n">
+        <v>77801.76487081093</v>
+      </c>
+      <c r="K591" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,028.1988; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L591" s="17" t="n">
+        <v>68016.03134096395</v>
+      </c>
+      <c r="M591" s="17">
+        <f>J591-L591</f>
+        <v/>
+      </c>
+      <c r="N591" s="18">
+        <f>IF(J591=0,"",L591/J591)</f>
+        <v/>
+      </c>
+      <c r="O591" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:15:46</t>
+        </is>
+      </c>
+      <c r="B592" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C592" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D592" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E592" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F592" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G592" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H592" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I592" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J592" s="17" t="n">
+        <v>197058.9178680961</v>
+      </c>
+      <c r="K592" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,243.9962</t>
+        </is>
+      </c>
+      <c r="L592" s="17" t="n">
+        <v>150259.0221489499</v>
+      </c>
+      <c r="M592" s="17">
+        <f>J592-L592</f>
+        <v/>
+      </c>
+      <c r="N592" s="18">
+        <f>IF(J592=0,"",L592/J592)</f>
+        <v/>
+      </c>
+      <c r="O592" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:15:46</t>
+        </is>
+      </c>
+      <c r="B593" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C593" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D593" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E593" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F593" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G593" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H593" s="16" t="n">
+        <v>1.3726</v>
+      </c>
+      <c r="I593" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J593" s="17" t="n">
+        <v>186064.8340627123</v>
+      </c>
+      <c r="K593" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,140.3351</t>
+        </is>
+      </c>
+      <c r="L593" s="17" t="n">
+        <v>124152.75041811</v>
+      </c>
+      <c r="M593" s="17">
+        <f>J593-L593</f>
+        <v/>
+      </c>
+      <c r="N593" s="18">
+        <f>IF(J593=0,"",L593/J593)</f>
+        <v/>
+      </c>
+      <c r="O593" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:15:46</t>
+        </is>
+      </c>
+      <c r="B594" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C594" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D594" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E594" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F594" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G594" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H594" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I594" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J594" s="17" t="n">
+        <v>327654.8339905708</v>
+      </c>
+      <c r="K594" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L594" s="17" t="n">
+        <v>280286.8738351339</v>
+      </c>
+      <c r="M594" s="17">
+        <f>J594-L594</f>
+        <v/>
+      </c>
+      <c r="N594" s="18">
+        <f>IF(J594=0,"",L594/J594)</f>
+        <v/>
+      </c>
+      <c r="O594" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:15:46</t>
+        </is>
+      </c>
+      <c r="B595" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C595" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D595" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E595" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F595" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G595" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H595" s="16" t="n">
+        <v>1.9045</v>
+      </c>
+      <c r="I595" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J595" s="17" t="n">
+        <v>159989.8916291629</v>
+      </c>
+      <c r="K595" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,938.3760</t>
+        </is>
+      </c>
+      <c r="L595" s="17" t="n">
+        <v>70945.47053958943</v>
+      </c>
+      <c r="M595" s="17">
+        <f>J595-L595</f>
+        <v/>
+      </c>
+      <c r="N595" s="18">
+        <f>IF(J595=0,"",L595/J595)</f>
+        <v/>
+      </c>
+      <c r="O595" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:15:46</t>
+        </is>
+      </c>
+      <c r="B596" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C596" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D596" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E596" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F596" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G596" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H596" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I596" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J596" s="17" t="n">
+        <v>160148.3577945266</v>
+      </c>
+      <c r="K596" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,523.0271</t>
+        </is>
+      </c>
+      <c r="L596" s="17" t="n">
+        <v>138495.3224502363</v>
+      </c>
+      <c r="M596" s="17">
+        <f>J596-L596</f>
+        <v/>
+      </c>
+      <c r="N596" s="18">
+        <f>IF(J596=0,"",L596/J596)</f>
+        <v/>
+      </c>
+      <c r="O596" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:15:46</t>
+        </is>
+      </c>
+      <c r="B597" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C597" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D597" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E597" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F597" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G597" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H597" s="16" t="inlineStr"/>
+      <c r="I597" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J597" s="17" t="n">
+        <v>95892.31038181752</v>
+      </c>
+      <c r="K597" s="15" t="inlineStr"/>
+      <c r="L597" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M597" s="17">
+        <f>J597-L597</f>
+        <v/>
+      </c>
+      <c r="N597" s="18">
+        <f>IF(J597=0,"",L597/J597)</f>
+        <v/>
+      </c>
+      <c r="O597" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:15:46</t>
+        </is>
+      </c>
+      <c r="B598" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C598" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D598" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E598" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F598" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G598" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H598" s="16" t="inlineStr"/>
+      <c r="I598" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J598" s="17" t="n">
+        <v>34347.02579871646</v>
+      </c>
+      <c r="K598" s="15" t="inlineStr"/>
+      <c r="L598" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M598" s="17">
+        <f>J598-L598</f>
+        <v/>
+      </c>
+      <c r="N598" s="18">
+        <f>IF(J598=0,"",L598/J598)</f>
+        <v/>
+      </c>
+      <c r="O598" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:15:46</t>
+        </is>
+      </c>
+      <c r="B599" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C599" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D599" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E599" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F599" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G599" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H599" s="16" t="n">
+        <v>1.0429</v>
+      </c>
+      <c r="I599" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J599" s="17" t="n">
+        <v>269996.1113129806</v>
+      </c>
+      <c r="K599" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,041.5307</t>
+        </is>
+      </c>
+      <c r="L599" s="17" t="n">
+        <v>232999.58319148</v>
+      </c>
+      <c r="M599" s="17">
+        <f>J599-L599</f>
+        <v/>
+      </c>
+      <c r="N599" s="18">
+        <f>IF(J599=0,"",L599/J599)</f>
+        <v/>
+      </c>
+      <c r="O599" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:15:46</t>
+        </is>
+      </c>
+      <c r="B600" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C600" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D600" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E600" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F600" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G600" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H600" s="16" t="inlineStr"/>
+      <c r="I600" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,510.6093</t>
+        </is>
+      </c>
+      <c r="J600" s="17" t="n">
+        <v>15507.81738465016</v>
+      </c>
+      <c r="K600" s="15" t="inlineStr"/>
+      <c r="L600" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M600" s="17">
+        <f>J600-L600</f>
+        <v/>
+      </c>
+      <c r="N600" s="18">
+        <f>IF(J600=0,"",L600/J600)</f>
+        <v/>
+      </c>
+      <c r="O600" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:15:46</t>
+        </is>
+      </c>
+      <c r="B601" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C601" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D601" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E601" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F601" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G601" s="15" t="inlineStr">
+        <is>
+          <t>3B8X44 vs USDC</t>
+        </is>
+      </c>
+      <c r="H601" s="16" t="inlineStr"/>
+      <c r="I601" s="15" t="inlineStr">
+        <is>
+          <t>3B8X44 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J601" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K601" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L601" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M601" s="17">
+        <f>J601-L601</f>
+        <v/>
+      </c>
+      <c r="N601" s="18">
+        <f>IF(J601=0,"",L601/J601)</f>
+        <v/>
+      </c>
+      <c r="O601" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:15:46</t>
+        </is>
+      </c>
+      <c r="B602" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C602" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D602" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E602" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F602" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G602" s="15" t="inlineStr">
+        <is>
+          <t>5Y8NV3 vs USDC</t>
+        </is>
+      </c>
+      <c r="H602" s="16" t="inlineStr"/>
+      <c r="I602" s="15" t="inlineStr">
+        <is>
+          <t>5Y8NV3 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J602" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K602" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,705.3454</t>
+        </is>
+      </c>
+      <c r="L602" s="17" t="n">
+        <v>148705.345409</v>
+      </c>
+      <c r="M602" s="17">
+        <f>J602-L602</f>
+        <v/>
+      </c>
+      <c r="N602" s="18">
+        <f>IF(J602=0,"",L602/J602)</f>
+        <v/>
+      </c>
+      <c r="O602" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -39854,7 +40936,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -41270,6 +42352,41 @@
         <v>1.0375</v>
       </c>
       <c r="I40" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:15:46</t>
+        </is>
+      </c>
+      <c r="B41" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C41" s="17" t="n">
+        <v>553493.3881139293</v>
+      </c>
+      <c r="D41" s="17" t="n">
+        <v>150192.4169986765</v>
+      </c>
+      <c r="E41" s="17" t="n">
+        <v>2430886.772514055</v>
+      </c>
+      <c r="F41" s="17" t="n">
+        <v>2280694.355515379</v>
+      </c>
+      <c r="G41" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H41" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I41" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 12:46 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O602"/>
+  <dimension ref="A1:O618"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -40906,6 +40906,1088 @@
         <v/>
       </c>
       <c r="O602" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:45:58</t>
+        </is>
+      </c>
+      <c r="B603" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C603" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D603" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E603" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F603" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G603" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H603" s="16" t="n">
+        <v>1.0505</v>
+      </c>
+      <c r="I603" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,804.5477</t>
+        </is>
+      </c>
+      <c r="J603" s="17" t="n">
+        <v>50804.547663</v>
+      </c>
+      <c r="K603" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,722.8797</t>
+        </is>
+      </c>
+      <c r="L603" s="17" t="n">
+        <v>37726.65235523552</v>
+      </c>
+      <c r="M603" s="17">
+        <f>J603-L603</f>
+        <v/>
+      </c>
+      <c r="N603" s="18">
+        <f>IF(J603=0,"",L603/J603)</f>
+        <v/>
+      </c>
+      <c r="O603" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:45:58</t>
+        </is>
+      </c>
+      <c r="B604" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C604" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D604" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E604" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F604" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G604" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H604" s="16" t="n">
+        <v>1.0477</v>
+      </c>
+      <c r="I604" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J604" s="17" t="n">
+        <v>140898.5726713169</v>
+      </c>
+      <c r="K604" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,035.0439</t>
+        </is>
+      </c>
+      <c r="L604" s="17" t="n">
+        <v>121035.043927</v>
+      </c>
+      <c r="M604" s="17">
+        <f>J604-L604</f>
+        <v/>
+      </c>
+      <c r="N604" s="18">
+        <f>IF(J604=0,"",L604/J604)</f>
+        <v/>
+      </c>
+      <c r="O604" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:45:58</t>
+        </is>
+      </c>
+      <c r="B605" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C605" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D605" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E605" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F605" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G605" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H605" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I605" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J605" s="17" t="n">
+        <v>328714.985154434</v>
+      </c>
+      <c r="K605" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,386.0522</t>
+        </is>
+      </c>
+      <c r="L605" s="17" t="n">
+        <v>306468.919278229</v>
+      </c>
+      <c r="M605" s="17">
+        <f>J605-L605</f>
+        <v/>
+      </c>
+      <c r="N605" s="18">
+        <f>IF(J605=0,"",L605/J605)</f>
+        <v/>
+      </c>
+      <c r="O605" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:45:58</t>
+        </is>
+      </c>
+      <c r="B606" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C606" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D606" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E606" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F606" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G606" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H606" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I606" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J606" s="17" t="n">
+        <v>386058.3778829138</v>
+      </c>
+      <c r="K606" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,608.2120</t>
+        </is>
+      </c>
+      <c r="L606" s="17" t="n">
+        <v>349702.7692257006</v>
+      </c>
+      <c r="M606" s="17">
+        <f>J606-L606</f>
+        <v/>
+      </c>
+      <c r="N606" s="18">
+        <f>IF(J606=0,"",L606/J606)</f>
+        <v/>
+      </c>
+      <c r="O606" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:45:58</t>
+        </is>
+      </c>
+      <c r="B607" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C607" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D607" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E607" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F607" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G607" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H607" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I607" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7848</t>
+        </is>
+      </c>
+      <c r="J607" s="17" t="n">
+        <v>77790.9108823377</v>
+      </c>
+      <c r="K607" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,028.1988; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L607" s="17" t="n">
+        <v>68028.27641675677</v>
+      </c>
+      <c r="M607" s="17">
+        <f>J607-L607</f>
+        <v/>
+      </c>
+      <c r="N607" s="18">
+        <f>IF(J607=0,"",L607/J607)</f>
+        <v/>
+      </c>
+      <c r="O607" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:45:58</t>
+        </is>
+      </c>
+      <c r="B608" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C608" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D608" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E608" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F608" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G608" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H608" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I608" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J608" s="17" t="n">
+        <v>197067.2050541306</v>
+      </c>
+      <c r="K608" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,243.9962</t>
+        </is>
+      </c>
+      <c r="L608" s="17" t="n">
+        <v>150259.0221489499</v>
+      </c>
+      <c r="M608" s="17">
+        <f>J608-L608</f>
+        <v/>
+      </c>
+      <c r="N608" s="18">
+        <f>IF(J608=0,"",L608/J608)</f>
+        <v/>
+      </c>
+      <c r="O608" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:45:58</t>
+        </is>
+      </c>
+      <c r="B609" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C609" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D609" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E609" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F609" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G609" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H609" s="16" t="n">
+        <v>1.3726</v>
+      </c>
+      <c r="I609" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J609" s="17" t="n">
+        <v>186122.2251574689</v>
+      </c>
+      <c r="K609" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,140.3351</t>
+        </is>
+      </c>
+      <c r="L609" s="17" t="n">
+        <v>124152.75041811</v>
+      </c>
+      <c r="M609" s="17">
+        <f>J609-L609</f>
+        <v/>
+      </c>
+      <c r="N609" s="18">
+        <f>IF(J609=0,"",L609/J609)</f>
+        <v/>
+      </c>
+      <c r="O609" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:45:58</t>
+        </is>
+      </c>
+      <c r="B610" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C610" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D610" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E610" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F610" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G610" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H610" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I610" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J610" s="17" t="n">
+        <v>327660.7049371375</v>
+      </c>
+      <c r="K610" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L610" s="17" t="n">
+        <v>280286.9142889067</v>
+      </c>
+      <c r="M610" s="17">
+        <f>J610-L610</f>
+        <v/>
+      </c>
+      <c r="N610" s="18">
+        <f>IF(J610=0,"",L610/J610)</f>
+        <v/>
+      </c>
+      <c r="O610" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:45:58</t>
+        </is>
+      </c>
+      <c r="B611" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C611" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D611" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E611" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F611" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G611" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H611" s="16" t="n">
+        <v>1.9045</v>
+      </c>
+      <c r="I611" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J611" s="17" t="n">
+        <v>159989.8916291629</v>
+      </c>
+      <c r="K611" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,938.3760</t>
+        </is>
+      </c>
+      <c r="L611" s="17" t="n">
+        <v>70945.47053958943</v>
+      </c>
+      <c r="M611" s="17">
+        <f>J611-L611</f>
+        <v/>
+      </c>
+      <c r="N611" s="18">
+        <f>IF(J611=0,"",L611/J611)</f>
+        <v/>
+      </c>
+      <c r="O611" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:45:58</t>
+        </is>
+      </c>
+      <c r="B612" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C612" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D612" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E612" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F612" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G612" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H612" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I612" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J612" s="17" t="n">
+        <v>160165.1745238984</v>
+      </c>
+      <c r="K612" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,523.0271</t>
+        </is>
+      </c>
+      <c r="L612" s="17" t="n">
+        <v>138495.3224502363</v>
+      </c>
+      <c r="M612" s="17">
+        <f>J612-L612</f>
+        <v/>
+      </c>
+      <c r="N612" s="18">
+        <f>IF(J612=0,"",L612/J612)</f>
+        <v/>
+      </c>
+      <c r="O612" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:45:58</t>
+        </is>
+      </c>
+      <c r="B613" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C613" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D613" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E613" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F613" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G613" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H613" s="16" t="inlineStr"/>
+      <c r="I613" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J613" s="17" t="n">
+        <v>95892.31038181752</v>
+      </c>
+      <c r="K613" s="15" t="inlineStr"/>
+      <c r="L613" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M613" s="17">
+        <f>J613-L613</f>
+        <v/>
+      </c>
+      <c r="N613" s="18">
+        <f>IF(J613=0,"",L613/J613)</f>
+        <v/>
+      </c>
+      <c r="O613" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:45:58</t>
+        </is>
+      </c>
+      <c r="B614" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C614" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D614" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E614" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F614" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G614" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H614" s="16" t="inlineStr"/>
+      <c r="I614" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J614" s="17" t="n">
+        <v>34347.32118276734</v>
+      </c>
+      <c r="K614" s="15" t="inlineStr"/>
+      <c r="L614" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M614" s="17">
+        <f>J614-L614</f>
+        <v/>
+      </c>
+      <c r="N614" s="18">
+        <f>IF(J614=0,"",L614/J614)</f>
+        <v/>
+      </c>
+      <c r="O614" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:45:58</t>
+        </is>
+      </c>
+      <c r="B615" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C615" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D615" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E615" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F615" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G615" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H615" s="16" t="n">
+        <v>1.0428</v>
+      </c>
+      <c r="I615" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J615" s="17" t="n">
+        <v>270023.1136243431</v>
+      </c>
+      <c r="K615" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,041.5307</t>
+        </is>
+      </c>
+      <c r="L615" s="17" t="n">
+        <v>233041.530667</v>
+      </c>
+      <c r="M615" s="17">
+        <f>J615-L615</f>
+        <v/>
+      </c>
+      <c r="N615" s="18">
+        <f>IF(J615=0,"",L615/J615)</f>
+        <v/>
+      </c>
+      <c r="O615" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:45:58</t>
+        </is>
+      </c>
+      <c r="B616" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C616" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D616" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E616" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F616" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G616" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H616" s="16" t="inlineStr"/>
+      <c r="I616" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,510.8127</t>
+        </is>
+      </c>
+      <c r="J616" s="17" t="n">
+        <v>15510.81267158138</v>
+      </c>
+      <c r="K616" s="15" t="inlineStr"/>
+      <c r="L616" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M616" s="17">
+        <f>J616-L616</f>
+        <v/>
+      </c>
+      <c r="N616" s="18">
+        <f>IF(J616=0,"",L616/J616)</f>
+        <v/>
+      </c>
+      <c r="O616" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:45:58</t>
+        </is>
+      </c>
+      <c r="B617" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C617" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D617" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E617" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F617" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G617" s="15" t="inlineStr">
+        <is>
+          <t>3B8X44 vs USDC</t>
+        </is>
+      </c>
+      <c r="H617" s="16" t="inlineStr"/>
+      <c r="I617" s="15" t="inlineStr">
+        <is>
+          <t>3B8X44 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J617" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K617" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L617" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M617" s="17">
+        <f>J617-L617</f>
+        <v/>
+      </c>
+      <c r="N617" s="18">
+        <f>IF(J617=0,"",L617/J617)</f>
+        <v/>
+      </c>
+      <c r="O617" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:45:58</t>
+        </is>
+      </c>
+      <c r="B618" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C618" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D618" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E618" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F618" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G618" s="15" t="inlineStr">
+        <is>
+          <t>5Y8NV3 vs USDC</t>
+        </is>
+      </c>
+      <c r="H618" s="16" t="inlineStr"/>
+      <c r="I618" s="15" t="inlineStr">
+        <is>
+          <t>5Y8NV3 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J618" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K618" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,705.3454</t>
+        </is>
+      </c>
+      <c r="L618" s="17" t="n">
+        <v>148705.345409</v>
+      </c>
+      <c r="M618" s="17">
+        <f>J618-L618</f>
+        <v/>
+      </c>
+      <c r="N618" s="18">
+        <f>IF(J618=0,"",L618/J618)</f>
+        <v/>
+      </c>
+      <c r="O618" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -40936,7 +42018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -42387,6 +43469,41 @@
         <v>1.0375</v>
       </c>
       <c r="I41" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:45:58</t>
+        </is>
+      </c>
+      <c r="B42" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C42" s="17" t="n">
+        <v>553516.2928977142</v>
+      </c>
+      <c r="D42" s="17" t="n">
+        <v>150215.5891875955</v>
+      </c>
+      <c r="E42" s="17" t="n">
+        <v>2431046.15341631</v>
+      </c>
+      <c r="F42" s="17" t="n">
+        <v>2280830.564228714</v>
+      </c>
+      <c r="G42" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H42" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I42" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 13:12 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O224"/>
+  <dimension ref="A1:O238"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -15556,6 +15556,954 @@
         <v/>
       </c>
       <c r="O224" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:11:48</t>
+        </is>
+      </c>
+      <c r="B225" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C225" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D225" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E225" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F225" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G225" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H225" s="16" t="n">
+        <v>1.0505</v>
+      </c>
+      <c r="I225" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,804.5477</t>
+        </is>
+      </c>
+      <c r="J225" s="17" t="n">
+        <v>50787.78216227121</v>
+      </c>
+      <c r="K225" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,722.8797</t>
+        </is>
+      </c>
+      <c r="L225" s="17" t="n">
+        <v>37722.87969</v>
+      </c>
+      <c r="M225" s="17">
+        <f>J225-L225</f>
+        <v/>
+      </c>
+      <c r="N225" s="18">
+        <f>IF(J225=0,"",L225/J225)</f>
+        <v/>
+      </c>
+      <c r="O225" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:11:48</t>
+        </is>
+      </c>
+      <c r="B226" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C226" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D226" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E226" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F226" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G226" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H226" s="16" t="n">
+        <v>1.048</v>
+      </c>
+      <c r="I226" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J226" s="17" t="n">
+        <v>140898.5726713169</v>
+      </c>
+      <c r="K226" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,035.0439</t>
+        </is>
+      </c>
+      <c r="L226" s="17" t="n">
+        <v>120995.1023625041</v>
+      </c>
+      <c r="M226" s="17">
+        <f>J226-L226</f>
+        <v/>
+      </c>
+      <c r="N226" s="18">
+        <f>IF(J226=0,"",L226/J226)</f>
+        <v/>
+      </c>
+      <c r="O226" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:11:48</t>
+        </is>
+      </c>
+      <c r="B227" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C227" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D227" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E227" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F227" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G227" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H227" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I227" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J227" s="17" t="n">
+        <v>328715.1813585485</v>
+      </c>
+      <c r="K227" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,386.0522</t>
+        </is>
+      </c>
+      <c r="L227" s="17" t="n">
+        <v>306437.7175657238</v>
+      </c>
+      <c r="M227" s="17">
+        <f>J227-L227</f>
+        <v/>
+      </c>
+      <c r="N227" s="18">
+        <f>IF(J227=0,"",L227/J227)</f>
+        <v/>
+      </c>
+      <c r="O227" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:11:48</t>
+        </is>
+      </c>
+      <c r="B228" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C228" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D228" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E228" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F228" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G228" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H228" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I228" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J228" s="17" t="n">
+        <v>386020.1484686669</v>
+      </c>
+      <c r="K228" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,608.2120</t>
+        </is>
+      </c>
+      <c r="L228" s="17" t="n">
+        <v>349667.1658591558</v>
+      </c>
+      <c r="M228" s="17">
+        <f>J228-L228</f>
+        <v/>
+      </c>
+      <c r="N228" s="18">
+        <f>IF(J228=0,"",L228/J228)</f>
+        <v/>
+      </c>
+      <c r="O228" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:11:48</t>
+        </is>
+      </c>
+      <c r="B229" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C229" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D229" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E229" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F229" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G229" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H229" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I229" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7848</t>
+        </is>
+      </c>
+      <c r="J229" s="17" t="n">
+        <v>77793.99900355314</v>
+      </c>
+      <c r="K229" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,028.1988; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L229" s="17" t="n">
+        <v>68005.82710337982</v>
+      </c>
+      <c r="M229" s="17">
+        <f>J229-L229</f>
+        <v/>
+      </c>
+      <c r="N229" s="18">
+        <f>IF(J229=0,"",L229/J229)</f>
+        <v/>
+      </c>
+      <c r="O229" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:11:48</t>
+        </is>
+      </c>
+      <c r="B230" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C230" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D230" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E230" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F230" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G230" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H230" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I230" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J230" s="17" t="n">
+        <v>197060.9078776304</v>
+      </c>
+      <c r="K230" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,243.9962</t>
+        </is>
+      </c>
+      <c r="L230" s="17" t="n">
+        <v>150243.996246735</v>
+      </c>
+      <c r="M230" s="17">
+        <f>J230-L230</f>
+        <v/>
+      </c>
+      <c r="N230" s="18">
+        <f>IF(J230=0,"",L230/J230)</f>
+        <v/>
+      </c>
+      <c r="O230" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:11:48</t>
+        </is>
+      </c>
+      <c r="B231" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C231" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D231" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E231" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F231" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G231" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H231" s="16" t="n">
+        <v>1.3726</v>
+      </c>
+      <c r="I231" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J231" s="17" t="n">
+        <v>186122.8256092648</v>
+      </c>
+      <c r="K231" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,140.3351</t>
+        </is>
+      </c>
+      <c r="L231" s="17" t="n">
+        <v>124140.3351430682</v>
+      </c>
+      <c r="M231" s="17">
+        <f>J231-L231</f>
+        <v/>
+      </c>
+      <c r="N231" s="18">
+        <f>IF(J231=0,"",L231/J231)</f>
+        <v/>
+      </c>
+      <c r="O231" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:11:48</t>
+        </is>
+      </c>
+      <c r="B232" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C232" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D232" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E232" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F232" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G232" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H232" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I232" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J232" s="17" t="n">
+        <v>327660.8306783233</v>
+      </c>
+      <c r="K232" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L232" s="17" t="n">
+        <v>280259.3020625638</v>
+      </c>
+      <c r="M232" s="17">
+        <f>J232-L232</f>
+        <v/>
+      </c>
+      <c r="N232" s="18">
+        <f>IF(J232=0,"",L232/J232)</f>
+        <v/>
+      </c>
+      <c r="O232" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:11:48</t>
+        </is>
+      </c>
+      <c r="B233" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C233" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D233" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E233" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F233" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G233" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H233" s="16" t="n">
+        <v>1.9045</v>
+      </c>
+      <c r="I233" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J233" s="17" t="n">
+        <v>159989.8916291629</v>
+      </c>
+      <c r="K233" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,938.3760</t>
+        </is>
+      </c>
+      <c r="L233" s="17" t="n">
+        <v>70938.37599253547</v>
+      </c>
+      <c r="M233" s="17">
+        <f>J233-L233</f>
+        <v/>
+      </c>
+      <c r="N233" s="18">
+        <f>IF(J233=0,"",L233/J233)</f>
+        <v/>
+      </c>
+      <c r="O233" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:11:48</t>
+        </is>
+      </c>
+      <c r="B234" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C234" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D234" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E234" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F234" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G234" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H234" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I234" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J234" s="17" t="n">
+        <v>160149.3141743875</v>
+      </c>
+      <c r="K234" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,523.0271</t>
+        </is>
+      </c>
+      <c r="L234" s="17" t="n">
+        <v>138523.0270556475</v>
+      </c>
+      <c r="M234" s="17">
+        <f>J234-L234</f>
+        <v/>
+      </c>
+      <c r="N234" s="18">
+        <f>IF(J234=0,"",L234/J234)</f>
+        <v/>
+      </c>
+      <c r="O234" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:11:48</t>
+        </is>
+      </c>
+      <c r="B235" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C235" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D235" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E235" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F235" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G235" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H235" s="16" t="inlineStr"/>
+      <c r="I235" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J235" s="17" t="n">
+        <v>95905.12552193923</v>
+      </c>
+      <c r="K235" s="15" t="inlineStr"/>
+      <c r="L235" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M235" s="17">
+        <f>J235-L235</f>
+        <v/>
+      </c>
+      <c r="N235" s="18">
+        <f>IF(J235=0,"",L235/J235)</f>
+        <v/>
+      </c>
+      <c r="O235" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:11:48</t>
+        </is>
+      </c>
+      <c r="B236" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C236" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D236" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E236" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F236" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G236" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H236" s="16" t="inlineStr"/>
+      <c r="I236" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J236" s="17" t="n">
+        <v>34346.72033681614</v>
+      </c>
+      <c r="K236" s="15" t="inlineStr"/>
+      <c r="L236" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M236" s="17">
+        <f>J236-L236</f>
+        <v/>
+      </c>
+      <c r="N236" s="18">
+        <f>IF(J236=0,"",L236/J236)</f>
+        <v/>
+      </c>
+      <c r="O236" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:11:48</t>
+        </is>
+      </c>
+      <c r="B237" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C237" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D237" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E237" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F237" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G237" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H237" s="16" t="n">
+        <v>1.0432</v>
+      </c>
+      <c r="I237" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J237" s="17" t="n">
+        <v>270023.1136243431</v>
+      </c>
+      <c r="K237" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,041.5307</t>
+        </is>
+      </c>
+      <c r="L237" s="17" t="n">
+        <v>232964.6269618799</v>
+      </c>
+      <c r="M237" s="17">
+        <f>J237-L237</f>
+        <v/>
+      </c>
+      <c r="N237" s="18">
+        <f>IF(J237=0,"",L237/J237)</f>
+        <v/>
+      </c>
+      <c r="O237" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:11:48</t>
+        </is>
+      </c>
+      <c r="B238" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C238" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D238" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E238" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F238" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G238" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H238" s="16" t="inlineStr"/>
+      <c r="I238" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,511.0119</t>
+        </is>
+      </c>
+      <c r="J238" s="17" t="n">
+        <v>15505.89325976253</v>
+      </c>
+      <c r="K238" s="15" t="inlineStr"/>
+      <c r="L238" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M238" s="17">
+        <f>J238-L238</f>
+        <v/>
+      </c>
+      <c r="N238" s="18">
+        <f>IF(J238=0,"",L238/J238)</f>
+        <v/>
+      </c>
+      <c r="O238" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -15586,7 +16534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -16197,6 +17145,41 @@
         <v>1.0375</v>
       </c>
       <c r="I17" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:11:48</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C18" s="17" t="n">
+        <v>553695.2758185341</v>
+      </c>
+      <c r="D18" s="17" t="n">
+        <v>551081.9503327932</v>
+      </c>
+      <c r="E18" s="17" t="n">
+        <v>2430980.306375986</v>
+      </c>
+      <c r="F18" s="17" t="n">
+        <v>1879898.356043193</v>
+      </c>
+      <c r="G18" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="H18" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I18" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 13:16 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O618"/>
+  <dimension ref="A1:O634"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -41988,6 +41988,1088 @@
         <v/>
       </c>
       <c r="O618" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:16:10</t>
+        </is>
+      </c>
+      <c r="B619" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C619" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D619" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E619" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F619" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G619" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H619" s="16" t="n">
+        <v>1.0505</v>
+      </c>
+      <c r="I619" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,804.5477</t>
+        </is>
+      </c>
+      <c r="J619" s="17" t="n">
+        <v>50787.78216227121</v>
+      </c>
+      <c r="K619" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,722.8797</t>
+        </is>
+      </c>
+      <c r="L619" s="17" t="n">
+        <v>37722.87969</v>
+      </c>
+      <c r="M619" s="17">
+        <f>J619-L619</f>
+        <v/>
+      </c>
+      <c r="N619" s="18">
+        <f>IF(J619=0,"",L619/J619)</f>
+        <v/>
+      </c>
+      <c r="O619" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:16:10</t>
+        </is>
+      </c>
+      <c r="B620" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C620" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D620" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E620" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F620" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G620" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H620" s="16" t="n">
+        <v>1.0481</v>
+      </c>
+      <c r="I620" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J620" s="17" t="n">
+        <v>140898.9737235772</v>
+      </c>
+      <c r="K620" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,035.0439</t>
+        </is>
+      </c>
+      <c r="L620" s="17" t="n">
+        <v>120995.1023625041</v>
+      </c>
+      <c r="M620" s="17">
+        <f>J620-L620</f>
+        <v/>
+      </c>
+      <c r="N620" s="18">
+        <f>IF(J620=0,"",L620/J620)</f>
+        <v/>
+      </c>
+      <c r="O620" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:16:10</t>
+        </is>
+      </c>
+      <c r="B621" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C621" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D621" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E621" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F621" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G621" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H621" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I621" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J621" s="17" t="n">
+        <v>328715.1813585485</v>
+      </c>
+      <c r="K621" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,386.0522</t>
+        </is>
+      </c>
+      <c r="L621" s="17" t="n">
+        <v>306437.7175657238</v>
+      </c>
+      <c r="M621" s="17">
+        <f>J621-L621</f>
+        <v/>
+      </c>
+      <c r="N621" s="18">
+        <f>IF(J621=0,"",L621/J621)</f>
+        <v/>
+      </c>
+      <c r="O621" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:16:10</t>
+        </is>
+      </c>
+      <c r="B622" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C622" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D622" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E622" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F622" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G622" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H622" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I622" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J622" s="17" t="n">
+        <v>386020.9180026079</v>
+      </c>
+      <c r="K622" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,608.2120</t>
+        </is>
+      </c>
+      <c r="L622" s="17" t="n">
+        <v>349667.1658591558</v>
+      </c>
+      <c r="M622" s="17">
+        <f>J622-L622</f>
+        <v/>
+      </c>
+      <c r="N622" s="18">
+        <f>IF(J622=0,"",L622/J622)</f>
+        <v/>
+      </c>
+      <c r="O622" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:16:10</t>
+        </is>
+      </c>
+      <c r="B623" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C623" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D623" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E623" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F623" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G623" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H623" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I623" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7848</t>
+        </is>
+      </c>
+      <c r="J623" s="17" t="n">
+        <v>77794.0079799572</v>
+      </c>
+      <c r="K623" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,028.1988; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L623" s="17" t="n">
+        <v>68001.0651294604</v>
+      </c>
+      <c r="M623" s="17">
+        <f>J623-L623</f>
+        <v/>
+      </c>
+      <c r="N623" s="18">
+        <f>IF(J623=0,"",L623/J623)</f>
+        <v/>
+      </c>
+      <c r="O623" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:16:10</t>
+        </is>
+      </c>
+      <c r="B624" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C624" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D624" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E624" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F624" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G624" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H624" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I624" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J624" s="17" t="n">
+        <v>197072.5028648429</v>
+      </c>
+      <c r="K624" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,243.9962</t>
+        </is>
+      </c>
+      <c r="L624" s="17" t="n">
+        <v>150243.996246735</v>
+      </c>
+      <c r="M624" s="17">
+        <f>J624-L624</f>
+        <v/>
+      </c>
+      <c r="N624" s="18">
+        <f>IF(J624=0,"",L624/J624)</f>
+        <v/>
+      </c>
+      <c r="O624" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:16:10</t>
+        </is>
+      </c>
+      <c r="B625" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C625" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D625" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E625" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F625" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G625" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H625" s="16" t="n">
+        <v>1.3726</v>
+      </c>
+      <c r="I625" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J625" s="17" t="n">
+        <v>186118.1024424936</v>
+      </c>
+      <c r="K625" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,140.3351</t>
+        </is>
+      </c>
+      <c r="L625" s="17" t="n">
+        <v>124140.3351430682</v>
+      </c>
+      <c r="M625" s="17">
+        <f>J625-L625</f>
+        <v/>
+      </c>
+      <c r="N625" s="18">
+        <f>IF(J625=0,"",L625/J625)</f>
+        <v/>
+      </c>
+      <c r="O625" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:16:10</t>
+        </is>
+      </c>
+      <c r="B626" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C626" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D626" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E626" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F626" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G626" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H626" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I626" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J626" s="17" t="n">
+        <v>327660.8306783233</v>
+      </c>
+      <c r="K626" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L626" s="17" t="n">
+        <v>280259.3020625638</v>
+      </c>
+      <c r="M626" s="17">
+        <f>J626-L626</f>
+        <v/>
+      </c>
+      <c r="N626" s="18">
+        <f>IF(J626=0,"",L626/J626)</f>
+        <v/>
+      </c>
+      <c r="O626" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:16:10</t>
+        </is>
+      </c>
+      <c r="B627" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C627" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D627" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E627" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F627" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G627" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H627" s="16" t="n">
+        <v>1.9045</v>
+      </c>
+      <c r="I627" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J627" s="17" t="n">
+        <v>159989.8916291629</v>
+      </c>
+      <c r="K627" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,938.3760</t>
+        </is>
+      </c>
+      <c r="L627" s="17" t="n">
+        <v>70938.37599253547</v>
+      </c>
+      <c r="M627" s="17">
+        <f>J627-L627</f>
+        <v/>
+      </c>
+      <c r="N627" s="18">
+        <f>IF(J627=0,"",L627/J627)</f>
+        <v/>
+      </c>
+      <c r="O627" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:16:10</t>
+        </is>
+      </c>
+      <c r="B628" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C628" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D628" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E628" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F628" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G628" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H628" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I628" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J628" s="17" t="n">
+        <v>160149.6334331966</v>
+      </c>
+      <c r="K628" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,523.0271</t>
+        </is>
+      </c>
+      <c r="L628" s="17" t="n">
+        <v>138509.1747529419</v>
+      </c>
+      <c r="M628" s="17">
+        <f>J628-L628</f>
+        <v/>
+      </c>
+      <c r="N628" s="18">
+        <f>IF(J628=0,"",L628/J628)</f>
+        <v/>
+      </c>
+      <c r="O628" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:16:10</t>
+        </is>
+      </c>
+      <c r="B629" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C629" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D629" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E629" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F629" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G629" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H629" s="16" t="inlineStr"/>
+      <c r="I629" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J629" s="17" t="n">
+        <v>95905.12552193923</v>
+      </c>
+      <c r="K629" s="15" t="inlineStr"/>
+      <c r="L629" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M629" s="17">
+        <f>J629-L629</f>
+        <v/>
+      </c>
+      <c r="N629" s="18">
+        <f>IF(J629=0,"",L629/J629)</f>
+        <v/>
+      </c>
+      <c r="O629" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:16:10</t>
+        </is>
+      </c>
+      <c r="B630" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C630" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D630" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E630" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F630" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G630" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H630" s="16" t="inlineStr"/>
+      <c r="I630" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J630" s="17" t="n">
+        <v>34346.82437914716</v>
+      </c>
+      <c r="K630" s="15" t="inlineStr"/>
+      <c r="L630" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M630" s="17">
+        <f>J630-L630</f>
+        <v/>
+      </c>
+      <c r="N630" s="18">
+        <f>IF(J630=0,"",L630/J630)</f>
+        <v/>
+      </c>
+      <c r="O630" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:16:10</t>
+        </is>
+      </c>
+      <c r="B631" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C631" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D631" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E631" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F631" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G631" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H631" s="16" t="n">
+        <v>1.0431</v>
+      </c>
+      <c r="I631" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J631" s="17" t="n">
+        <v>269996.1113129806</v>
+      </c>
+      <c r="K631" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,041.5307</t>
+        </is>
+      </c>
+      <c r="L631" s="17" t="n">
+        <v>232948.3140547332</v>
+      </c>
+      <c r="M631" s="17">
+        <f>J631-L631</f>
+        <v/>
+      </c>
+      <c r="N631" s="18">
+        <f>IF(J631=0,"",L631/J631)</f>
+        <v/>
+      </c>
+      <c r="O631" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:16:10</t>
+        </is>
+      </c>
+      <c r="B632" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C632" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D632" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E632" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F632" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G632" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H632" s="16" t="inlineStr"/>
+      <c r="I632" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,511.0119</t>
+        </is>
+      </c>
+      <c r="J632" s="17" t="n">
+        <v>15504.80748892998</v>
+      </c>
+      <c r="K632" s="15" t="inlineStr"/>
+      <c r="L632" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M632" s="17">
+        <f>J632-L632</f>
+        <v/>
+      </c>
+      <c r="N632" s="18">
+        <f>IF(J632=0,"",L632/J632)</f>
+        <v/>
+      </c>
+      <c r="O632" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:16:10</t>
+        </is>
+      </c>
+      <c r="B633" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C633" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D633" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E633" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F633" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G633" s="15" t="inlineStr">
+        <is>
+          <t>3B8X44 vs USDC</t>
+        </is>
+      </c>
+      <c r="H633" s="16" t="inlineStr"/>
+      <c r="I633" s="15" t="inlineStr">
+        <is>
+          <t>3B8X44 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J633" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K633" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L633" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M633" s="17">
+        <f>J633-L633</f>
+        <v/>
+      </c>
+      <c r="N633" s="18">
+        <f>IF(J633=0,"",L633/J633)</f>
+        <v/>
+      </c>
+      <c r="O633" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:16:10</t>
+        </is>
+      </c>
+      <c r="B634" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C634" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D634" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E634" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F634" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G634" s="15" t="inlineStr">
+        <is>
+          <t>5Y8NV3 vs USDC</t>
+        </is>
+      </c>
+      <c r="H634" s="16" t="inlineStr"/>
+      <c r="I634" s="15" t="inlineStr">
+        <is>
+          <t>5Y8NV3 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J634" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K634" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,705.3454</t>
+        </is>
+      </c>
+      <c r="L634" s="17" t="n">
+        <v>148705.345409</v>
+      </c>
+      <c r="M634" s="17">
+        <f>J634-L634</f>
+        <v/>
+      </c>
+      <c r="N634" s="18">
+        <f>IF(J634=0,"",L634/J634)</f>
+        <v/>
+      </c>
+      <c r="O634" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -42018,7 +43100,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -43504,6 +44586,41 @@
         <v>1.0375</v>
       </c>
       <c r="I42" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:16:10</t>
+        </is>
+      </c>
+      <c r="B43" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C43" s="17" t="n">
+        <v>553710.3548802963</v>
+      </c>
+      <c r="D43" s="17" t="n">
+        <v>150409.3716055574</v>
+      </c>
+      <c r="E43" s="17" t="n">
+        <v>2430960.692977978</v>
+      </c>
+      <c r="F43" s="17" t="n">
+        <v>2280551.321372421</v>
+      </c>
+      <c r="G43" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H43" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I43" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 13:46 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O634"/>
+  <dimension ref="A1:O650"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -43070,6 +43070,1088 @@
         <v/>
       </c>
       <c r="O634" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:46:21</t>
+        </is>
+      </c>
+      <c r="B635" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C635" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D635" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E635" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F635" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G635" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H635" s="16" t="n">
+        <v>1.0505</v>
+      </c>
+      <c r="I635" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,804.5477</t>
+        </is>
+      </c>
+      <c r="J635" s="17" t="n">
+        <v>50798.95916275706</v>
+      </c>
+      <c r="K635" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,722.8797</t>
+        </is>
+      </c>
+      <c r="L635" s="17" t="n">
+        <v>37722.87969</v>
+      </c>
+      <c r="M635" s="17">
+        <f>J635-L635</f>
+        <v/>
+      </c>
+      <c r="N635" s="18">
+        <f>IF(J635=0,"",L635/J635)</f>
+        <v/>
+      </c>
+      <c r="O635" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:46:21</t>
+        </is>
+      </c>
+      <c r="B636" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C636" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D636" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E636" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F636" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G636" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H636" s="16" t="n">
+        <v>1.0478</v>
+      </c>
+      <c r="I636" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J636" s="17" t="n">
+        <v>140897.9543392363</v>
+      </c>
+      <c r="K636" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,035.0439</t>
+        </is>
+      </c>
+      <c r="L636" s="17" t="n">
+        <v>121021.730072168</v>
+      </c>
+      <c r="M636" s="17">
+        <f>J636-L636</f>
+        <v/>
+      </c>
+      <c r="N636" s="18">
+        <f>IF(J636=0,"",L636/J636)</f>
+        <v/>
+      </c>
+      <c r="O636" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:46:21</t>
+        </is>
+      </c>
+      <c r="B637" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C637" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D637" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E637" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F637" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G637" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H637" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I637" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J637" s="17" t="n">
+        <v>328715.5689816554</v>
+      </c>
+      <c r="K637" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,386.0522</t>
+        </is>
+      </c>
+      <c r="L637" s="17" t="n">
+        <v>306437.653307181</v>
+      </c>
+      <c r="M637" s="17">
+        <f>J637-L637</f>
+        <v/>
+      </c>
+      <c r="N637" s="18">
+        <f>IF(J637=0,"",L637/J637)</f>
+        <v/>
+      </c>
+      <c r="O637" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:46:21</t>
+        </is>
+      </c>
+      <c r="B638" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C638" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D638" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E638" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F638" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G638" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H638" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I638" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J638" s="17" t="n">
+        <v>386021.3028583634</v>
+      </c>
+      <c r="K638" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,608.2120</t>
+        </is>
+      </c>
+      <c r="L638" s="17" t="n">
+        <v>349667.0925356018</v>
+      </c>
+      <c r="M638" s="17">
+        <f>J638-L638</f>
+        <v/>
+      </c>
+      <c r="N638" s="18">
+        <f>IF(J638=0,"",L638/J638)</f>
+        <v/>
+      </c>
+      <c r="O638" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:46:21</t>
+        </is>
+      </c>
+      <c r="B639" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C639" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D639" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E639" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F639" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G639" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H639" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I639" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7848</t>
+        </is>
+      </c>
+      <c r="J639" s="17" t="n">
+        <v>77793.05950375082</v>
+      </c>
+      <c r="K639" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,028.1988; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L639" s="17" t="n">
+        <v>68020.7933071266</v>
+      </c>
+      <c r="M639" s="17">
+        <f>J639-L639</f>
+        <v/>
+      </c>
+      <c r="N639" s="18">
+        <f>IF(J639=0,"",L639/J639)</f>
+        <v/>
+      </c>
+      <c r="O639" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:46:21</t>
+        </is>
+      </c>
+      <c r="B640" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C640" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D640" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E640" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F640" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G640" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H640" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I640" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J640" s="17" t="n">
+        <v>197074.1737696525</v>
+      </c>
+      <c r="K640" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,243.9962</t>
+        </is>
+      </c>
+      <c r="L640" s="17" t="n">
+        <v>150243.996246735</v>
+      </c>
+      <c r="M640" s="17">
+        <f>J640-L640</f>
+        <v/>
+      </c>
+      <c r="N640" s="18">
+        <f>IF(J640=0,"",L640/J640)</f>
+        <v/>
+      </c>
+      <c r="O640" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:46:21</t>
+        </is>
+      </c>
+      <c r="B641" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C641" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D641" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E641" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F641" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G641" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H641" s="16" t="n">
+        <v>1.3726</v>
+      </c>
+      <c r="I641" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J641" s="17" t="n">
+        <v>186110.9401670318</v>
+      </c>
+      <c r="K641" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,140.3351</t>
+        </is>
+      </c>
+      <c r="L641" s="17" t="n">
+        <v>124140.3351430682</v>
+      </c>
+      <c r="M641" s="17">
+        <f>J641-L641</f>
+        <v/>
+      </c>
+      <c r="N641" s="18">
+        <f>IF(J641=0,"",L641/J641)</f>
+        <v/>
+      </c>
+      <c r="O641" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:46:21</t>
+        </is>
+      </c>
+      <c r="B642" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C642" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D642" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E642" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F642" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G642" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H642" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I642" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J642" s="17" t="n">
+        <v>327627.3368611108</v>
+      </c>
+      <c r="K642" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L642" s="17" t="n">
+        <v>280238.2984896247</v>
+      </c>
+      <c r="M642" s="17">
+        <f>J642-L642</f>
+        <v/>
+      </c>
+      <c r="N642" s="18">
+        <f>IF(J642=0,"",L642/J642)</f>
+        <v/>
+      </c>
+      <c r="O642" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:46:21</t>
+        </is>
+      </c>
+      <c r="B643" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C643" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D643" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E643" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F643" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G643" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H643" s="16" t="n">
+        <v>1.9045</v>
+      </c>
+      <c r="I643" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J643" s="17" t="n">
+        <v>159989.8916291629</v>
+      </c>
+      <c r="K643" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,938.3760</t>
+        </is>
+      </c>
+      <c r="L643" s="17" t="n">
+        <v>70938.37599253547</v>
+      </c>
+      <c r="M643" s="17">
+        <f>J643-L643</f>
+        <v/>
+      </c>
+      <c r="N643" s="18">
+        <f>IF(J643=0,"",L643/J643)</f>
+        <v/>
+      </c>
+      <c r="O643" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:46:21</t>
+        </is>
+      </c>
+      <c r="B644" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C644" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D644" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E644" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F644" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G644" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H644" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I644" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J644" s="17" t="n">
+        <v>160149.7930994357</v>
+      </c>
+      <c r="K644" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,523.0271</t>
+        </is>
+      </c>
+      <c r="L644" s="17" t="n">
+        <v>138481.4701475308</v>
+      </c>
+      <c r="M644" s="17">
+        <f>J644-L644</f>
+        <v/>
+      </c>
+      <c r="N644" s="18">
+        <f>IF(J644=0,"",L644/J644)</f>
+        <v/>
+      </c>
+      <c r="O644" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:46:21</t>
+        </is>
+      </c>
+      <c r="B645" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C645" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D645" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E645" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F645" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G645" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H645" s="16" t="inlineStr"/>
+      <c r="I645" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J645" s="17" t="n">
+        <v>95898.41895306511</v>
+      </c>
+      <c r="K645" s="15" t="inlineStr"/>
+      <c r="L645" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M645" s="17">
+        <f>J645-L645</f>
+        <v/>
+      </c>
+      <c r="N645" s="18">
+        <f>IF(J645=0,"",L645/J645)</f>
+        <v/>
+      </c>
+      <c r="O645" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:46:21</t>
+        </is>
+      </c>
+      <c r="B646" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C646" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D646" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E646" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F646" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G646" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H646" s="16" t="inlineStr"/>
+      <c r="I646" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J646" s="17" t="n">
+        <v>34347.10547754735</v>
+      </c>
+      <c r="K646" s="15" t="inlineStr"/>
+      <c r="L646" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M646" s="17">
+        <f>J646-L646</f>
+        <v/>
+      </c>
+      <c r="N646" s="18">
+        <f>IF(J646=0,"",L646/J646)</f>
+        <v/>
+      </c>
+      <c r="O646" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:46:21</t>
+        </is>
+      </c>
+      <c r="B647" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C647" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D647" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E647" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F647" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G647" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H647" s="16" t="n">
+        <v>1.0428</v>
+      </c>
+      <c r="I647" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J647" s="17" t="n">
+        <v>269996.1113129806</v>
+      </c>
+      <c r="K647" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,041.5307</t>
+        </is>
+      </c>
+      <c r="L647" s="17" t="n">
+        <v>233015.8960986266</v>
+      </c>
+      <c r="M647" s="17">
+        <f>J647-L647</f>
+        <v/>
+      </c>
+      <c r="N647" s="18">
+        <f>IF(J647=0,"",L647/J647)</f>
+        <v/>
+      </c>
+      <c r="O647" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:46:21</t>
+        </is>
+      </c>
+      <c r="B648" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C648" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D648" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E648" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F648" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G648" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H648" s="16" t="inlineStr"/>
+      <c r="I648" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,511.2132</t>
+        </is>
+      </c>
+      <c r="J648" s="17" t="n">
+        <v>15509.50701606857</v>
+      </c>
+      <c r="K648" s="15" t="inlineStr"/>
+      <c r="L648" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M648" s="17">
+        <f>J648-L648</f>
+        <v/>
+      </c>
+      <c r="N648" s="18">
+        <f>IF(J648=0,"",L648/J648)</f>
+        <v/>
+      </c>
+      <c r="O648" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:46:21</t>
+        </is>
+      </c>
+      <c r="B649" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C649" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D649" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E649" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F649" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G649" s="15" t="inlineStr">
+        <is>
+          <t>3B8X44 vs USDC</t>
+        </is>
+      </c>
+      <c r="H649" s="16" t="inlineStr"/>
+      <c r="I649" s="15" t="inlineStr">
+        <is>
+          <t>3B8X44 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J649" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K649" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L649" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M649" s="17">
+        <f>J649-L649</f>
+        <v/>
+      </c>
+      <c r="N649" s="18">
+        <f>IF(J649=0,"",L649/J649)</f>
+        <v/>
+      </c>
+      <c r="O649" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:46:21</t>
+        </is>
+      </c>
+      <c r="B650" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C650" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D650" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E650" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F650" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G650" s="15" t="inlineStr">
+        <is>
+          <t>5Y8NV3 vs USDC</t>
+        </is>
+      </c>
+      <c r="H650" s="16" t="inlineStr"/>
+      <c r="I650" s="15" t="inlineStr">
+        <is>
+          <t>5Y8NV3 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J650" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K650" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,705.3454</t>
+        </is>
+      </c>
+      <c r="L650" s="17" t="n">
+        <v>148705.345409</v>
+      </c>
+      <c r="M650" s="17">
+        <f>J650-L650</f>
+        <v/>
+      </c>
+      <c r="N650" s="18">
+        <f>IF(J650=0,"",L650/J650)</f>
+        <v/>
+      </c>
+      <c r="O650" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -43100,7 +44182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I44"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -44621,6 +45703,41 @@
         <v>1.0375</v>
       </c>
       <c r="I43" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 13:46:21</t>
+        </is>
+      </c>
+      <c r="B44" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C44" s="17" t="n">
+        <v>553613.3475510181</v>
+      </c>
+      <c r="D44" s="17" t="n">
+        <v>150313.7095886208</v>
+      </c>
+      <c r="E44" s="17" t="n">
+        <v>2430930.123131819</v>
+      </c>
+      <c r="F44" s="17" t="n">
+        <v>2280616.413543198</v>
+      </c>
+      <c r="G44" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H44" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I44" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 14:16 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O650"/>
+  <dimension ref="A1:O666"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -44152,6 +44152,1092 @@
         <v/>
       </c>
       <c r="O650" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:16:36</t>
+        </is>
+      </c>
+      <c r="B651" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C651" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D651" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E651" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F651" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G651" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H651" s="16" t="n">
+        <v>1.0505</v>
+      </c>
+      <c r="I651" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,804.5477</t>
+        </is>
+      </c>
+      <c r="J651" s="17" t="n">
+        <v>50798.95916275706</v>
+      </c>
+      <c r="K651" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,722.8797</t>
+        </is>
+      </c>
+      <c r="L651" s="17" t="n">
+        <v>37722.87969</v>
+      </c>
+      <c r="M651" s="17">
+        <f>J651-L651</f>
+        <v/>
+      </c>
+      <c r="N651" s="18">
+        <f>IF(J651=0,"",L651/J651)</f>
+        <v/>
+      </c>
+      <c r="O651" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:16:36</t>
+        </is>
+      </c>
+      <c r="B652" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C652" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D652" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E652" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F652" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G652" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H652" s="16" t="n">
+        <v>1.0478</v>
+      </c>
+      <c r="I652" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J652" s="17" t="n">
+        <v>140897.7988754021</v>
+      </c>
+      <c r="K652" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,035.0439</t>
+        </is>
+      </c>
+      <c r="L652" s="17" t="n">
+        <v>121021.730072168</v>
+      </c>
+      <c r="M652" s="17">
+        <f>J652-L652</f>
+        <v/>
+      </c>
+      <c r="N652" s="18">
+        <f>IF(J652=0,"",L652/J652)</f>
+        <v/>
+      </c>
+      <c r="O652" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:16:36</t>
+        </is>
+      </c>
+      <c r="B653" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C653" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D653" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E653" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F653" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G653" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H653" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I653" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J653" s="17" t="n">
+        <v>328716.2772324632</v>
+      </c>
+      <c r="K653" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,386.0522</t>
+        </is>
+      </c>
+      <c r="L653" s="17" t="n">
+        <v>306424.1836908633</v>
+      </c>
+      <c r="M653" s="17">
+        <f>J653-L653</f>
+        <v/>
+      </c>
+      <c r="N653" s="18">
+        <f>IF(J653=0,"",L653/J653)</f>
+        <v/>
+      </c>
+      <c r="O653" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:16:36</t>
+        </is>
+      </c>
+      <c r="B654" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C654" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D654" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E654" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F654" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G654" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H654" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I654" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J654" s="17" t="n">
+        <v>386022.4498468307</v>
+      </c>
+      <c r="K654" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,608.2120</t>
+        </is>
+      </c>
+      <c r="L654" s="17" t="n">
+        <v>349651.7227482256</v>
+      </c>
+      <c r="M654" s="17">
+        <f>J654-L654</f>
+        <v/>
+      </c>
+      <c r="N654" s="18">
+        <f>IF(J654=0,"",L654/J654)</f>
+        <v/>
+      </c>
+      <c r="O654" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:16:36</t>
+        </is>
+      </c>
+      <c r="B655" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C655" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D655" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E655" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F655" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G655" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H655" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I655" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7848</t>
+        </is>
+      </c>
+      <c r="J655" s="17" t="n">
+        <v>77809.47487474213</v>
+      </c>
+      <c r="K655" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,028.1988; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L655" s="17" t="n">
+        <v>68020.7933071266</v>
+      </c>
+      <c r="M655" s="17">
+        <f>J655-L655</f>
+        <v/>
+      </c>
+      <c r="N655" s="18">
+        <f>IF(J655=0,"",L655/J655)</f>
+        <v/>
+      </c>
+      <c r="O655" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:16:36</t>
+        </is>
+      </c>
+      <c r="B656" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C656" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D656" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E656" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F656" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G656" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H656" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I656" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J656" s="17" t="n">
+        <v>197079.0812727896</v>
+      </c>
+      <c r="K656" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,243.9962</t>
+        </is>
+      </c>
+      <c r="L656" s="17" t="n">
+        <v>150243.996246735</v>
+      </c>
+      <c r="M656" s="17">
+        <f>J656-L656</f>
+        <v/>
+      </c>
+      <c r="N656" s="18">
+        <f>IF(J656=0,"",L656/J656)</f>
+        <v/>
+      </c>
+      <c r="O656" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:16:36</t>
+        </is>
+      </c>
+      <c r="B657" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C657" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D657" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E657" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F657" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G657" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H657" s="16" t="n">
+        <v>1.3726</v>
+      </c>
+      <c r="I657" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J657" s="17" t="n">
+        <v>186110.4141018477</v>
+      </c>
+      <c r="K657" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,140.3351</t>
+        </is>
+      </c>
+      <c r="L657" s="17" t="n">
+        <v>124140.3351430682</v>
+      </c>
+      <c r="M657" s="17">
+        <f>J657-L657</f>
+        <v/>
+      </c>
+      <c r="N657" s="18">
+        <f>IF(J657=0,"",L657/J657)</f>
+        <v/>
+      </c>
+      <c r="O657" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:16:36</t>
+        </is>
+      </c>
+      <c r="B658" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C658" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D658" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E658" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F658" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G658" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H658" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I658" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J658" s="17" t="n">
+        <v>327602.8991124285</v>
+      </c>
+      <c r="K658" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L658" s="17" t="n">
+        <v>280238.4949901749</v>
+      </c>
+      <c r="M658" s="17">
+        <f>J658-L658</f>
+        <v/>
+      </c>
+      <c r="N658" s="18">
+        <f>IF(J658=0,"",L658/J658)</f>
+        <v/>
+      </c>
+      <c r="O658" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:16:36</t>
+        </is>
+      </c>
+      <c r="B659" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C659" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D659" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E659" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F659" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G659" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H659" s="16" t="n">
+        <v>1.9045</v>
+      </c>
+      <c r="I659" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J659" s="17" t="n">
+        <v>159989.8916291629</v>
+      </c>
+      <c r="K659" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,938.3760</t>
+        </is>
+      </c>
+      <c r="L659" s="17" t="n">
+        <v>70938.37599253547</v>
+      </c>
+      <c r="M659" s="17">
+        <f>J659-L659</f>
+        <v/>
+      </c>
+      <c r="N659" s="18">
+        <f>IF(J659=0,"",L659/J659)</f>
+        <v/>
+      </c>
+      <c r="O659" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:16:36</t>
+        </is>
+      </c>
+      <c r="B660" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C660" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D660" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E660" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F660" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G660" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H660" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I660" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J660" s="17" t="n">
+        <v>160150.2689539141</v>
+      </c>
+      <c r="K660" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,523.0271</t>
+        </is>
+      </c>
+      <c r="L660" s="17" t="n">
+        <v>138509.1747529419</v>
+      </c>
+      <c r="M660" s="17">
+        <f>J660-L660</f>
+        <v/>
+      </c>
+      <c r="N660" s="18">
+        <f>IF(J660=0,"",L660/J660)</f>
+        <v/>
+      </c>
+      <c r="O660" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:16:36</t>
+        </is>
+      </c>
+      <c r="B661" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C661" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D661" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E661" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F661" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G661" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H661" s="16" t="inlineStr"/>
+      <c r="I661" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J661" s="17" t="n">
+        <v>95897.76799600091</v>
+      </c>
+      <c r="K661" s="15" t="inlineStr"/>
+      <c r="L661" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M661" s="17">
+        <f>J661-L661</f>
+        <v/>
+      </c>
+      <c r="N661" s="18">
+        <f>IF(J661=0,"",L661/J661)</f>
+        <v/>
+      </c>
+      <c r="O661" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:16:36</t>
+        </is>
+      </c>
+      <c r="B662" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C662" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D662" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E662" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F662" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G662" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H662" s="16" t="inlineStr"/>
+      <c r="I662" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J662" s="17" t="n">
+        <v>34347.30078753057</v>
+      </c>
+      <c r="K662" s="15" t="inlineStr"/>
+      <c r="L662" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M662" s="17">
+        <f>J662-L662</f>
+        <v/>
+      </c>
+      <c r="N662" s="18">
+        <f>IF(J662=0,"",L662/J662)</f>
+        <v/>
+      </c>
+      <c r="O662" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:16:36</t>
+        </is>
+      </c>
+      <c r="B663" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C663" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D663" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E663" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F663" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G663" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H663" s="16" t="n">
+        <v>1.0428</v>
+      </c>
+      <c r="I663" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J663" s="17" t="n">
+        <v>269996.1113129806</v>
+      </c>
+      <c r="K663" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,041.5307</t>
+        </is>
+      </c>
+      <c r="L663" s="17" t="n">
+        <v>233015.8960986266</v>
+      </c>
+      <c r="M663" s="17">
+        <f>J663-L663</f>
+        <v/>
+      </c>
+      <c r="N663" s="18">
+        <f>IF(J663=0,"",L663/J663)</f>
+        <v/>
+      </c>
+      <c r="O663" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:16:36</t>
+        </is>
+      </c>
+      <c r="B664" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C664" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D664" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E664" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F664" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G664" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H664" s="16" t="inlineStr"/>
+      <c r="I664" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,511.4122</t>
+        </is>
+      </c>
+      <c r="J664" s="17" t="n">
+        <v>15509.70599168743</v>
+      </c>
+      <c r="K664" s="15" t="inlineStr"/>
+      <c r="L664" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M664" s="17">
+        <f>J664-L664</f>
+        <v/>
+      </c>
+      <c r="N664" s="18">
+        <f>IF(J664=0,"",L664/J664)</f>
+        <v/>
+      </c>
+      <c r="O664" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:16:36</t>
+        </is>
+      </c>
+      <c r="B665" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C665" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D665" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E665" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F665" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G665" s="15" t="inlineStr">
+        <is>
+          <t>3B8X44 vs USDC</t>
+        </is>
+      </c>
+      <c r="H665" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I665" s="15" t="inlineStr">
+        <is>
+          <t>3B8X44 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J665" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K665" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L665" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M665" s="17">
+        <f>J665-L665</f>
+        <v/>
+      </c>
+      <c r="N665" s="18">
+        <f>IF(J665=0,"",L665/J665)</f>
+        <v/>
+      </c>
+      <c r="O665" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:16:36</t>
+        </is>
+      </c>
+      <c r="B666" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C666" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D666" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E666" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F666" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G666" s="15" t="inlineStr">
+        <is>
+          <t>5Y8NV3 vs USDC</t>
+        </is>
+      </c>
+      <c r="H666" s="16" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="I666" s="15" t="inlineStr">
+        <is>
+          <t>5Y8NV3 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J666" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K666" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,705.3454</t>
+        </is>
+      </c>
+      <c r="L666" s="17" t="n">
+        <v>148705.345409</v>
+      </c>
+      <c r="M666" s="17">
+        <f>J666-L666</f>
+        <v/>
+      </c>
+      <c r="N666" s="18">
+        <f>IF(J666=0,"",L666/J666)</f>
+        <v/>
+      </c>
+      <c r="O666" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -44182,7 +45268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I44"/>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -45738,6 +46824,41 @@
         <v>1.0375</v>
       </c>
       <c r="I44" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:16:36</t>
+        </is>
+      </c>
+      <c r="B45" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C45" s="17" t="n">
+        <v>655408.7392488351</v>
+      </c>
+      <c r="D45" s="17" t="n">
+        <v>652796.3064960218</v>
+      </c>
+      <c r="E45" s="17" t="n">
+        <v>2933411.781741487</v>
+      </c>
+      <c r="F45" s="17" t="n">
+        <v>2280615.475245465</v>
+      </c>
+      <c r="G45" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H45" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I45" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
feat: replace Playwright Solana scraping with Loopscale REST API
Implements loopscale_positions() using tars.loopscale.com REST API.
No browser required — works headlessly in GitHub Actions and locally.

- Price chain: Jupiter API → Loopscale event prices → USDC hardcode
- Decimals chain: KNOWN_SOL_MINTS → Jupiter meta → Solana RPC
- Health = (liqLtv / currentLtv - 1) × 100 from lqtRatios field
- ONYC (9 dec) and PRIME (6 dec) hardcoded for offline reliability
- fetch_sol_defi_positions() wraps Loopscale + Playwright fallback

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O666"/>
+  <dimension ref="A1:O682"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -45238,6 +45238,1092 @@
         <v/>
       </c>
       <c r="O666" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:33:20</t>
+        </is>
+      </c>
+      <c r="B667" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C667" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D667" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E667" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F667" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G667" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H667" s="16" t="n">
+        <v>1.0505</v>
+      </c>
+      <c r="I667" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,804.5477</t>
+        </is>
+      </c>
+      <c r="J667" s="17" t="n">
+        <v>50791.84652608425</v>
+      </c>
+      <c r="K667" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,722.8797</t>
+        </is>
+      </c>
+      <c r="L667" s="17" t="n">
+        <v>37722.87969</v>
+      </c>
+      <c r="M667" s="17">
+        <f>J667-L667</f>
+        <v/>
+      </c>
+      <c r="N667" s="18">
+        <f>IF(J667=0,"",L667/J667)</f>
+        <v/>
+      </c>
+      <c r="O667" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:33:20</t>
+        </is>
+      </c>
+      <c r="B668" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C668" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D668" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E668" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F668" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G668" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H668" s="16" t="n">
+        <v>1.048</v>
+      </c>
+      <c r="I668" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J668" s="17" t="n">
+        <v>140897.7988754021</v>
+      </c>
+      <c r="K668" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,035.0439</t>
+        </is>
+      </c>
+      <c r="L668" s="17" t="n">
+        <v>121004.7851660183</v>
+      </c>
+      <c r="M668" s="17">
+        <f>J668-L668</f>
+        <v/>
+      </c>
+      <c r="N668" s="18">
+        <f>IF(J668=0,"",L668/J668)</f>
+        <v/>
+      </c>
+      <c r="O668" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:33:20</t>
+        </is>
+      </c>
+      <c r="B669" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C669" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D669" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E669" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F669" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G669" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H669" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I669" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J669" s="17" t="n">
+        <v>328717.0046267734</v>
+      </c>
+      <c r="K669" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,386.0522</t>
+        </is>
+      </c>
+      <c r="L669" s="17" t="n">
+        <v>306423.4056871679</v>
+      </c>
+      <c r="M669" s="17">
+        <f>J669-L669</f>
+        <v/>
+      </c>
+      <c r="N669" s="18">
+        <f>IF(J669=0,"",L669/J669)</f>
+        <v/>
+      </c>
+      <c r="O669" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:33:20</t>
+        </is>
+      </c>
+      <c r="B670" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C670" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D670" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E670" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F670" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G670" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H670" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I670" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J670" s="17" t="n">
+        <v>386023.3050081776</v>
+      </c>
+      <c r="K670" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,608.2120</t>
+        </is>
+      </c>
+      <c r="L670" s="17" t="n">
+        <v>349650.8349908394</v>
+      </c>
+      <c r="M670" s="17">
+        <f>J670-L670</f>
+        <v/>
+      </c>
+      <c r="N670" s="18">
+        <f>IF(J670=0,"",L670/J670)</f>
+        <v/>
+      </c>
+      <c r="O670" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:33:20</t>
+        </is>
+      </c>
+      <c r="B671" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C671" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D671" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E671" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F671" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G671" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H671" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I671" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7848</t>
+        </is>
+      </c>
+      <c r="J671" s="17" t="n">
+        <v>77809.52742186155</v>
+      </c>
+      <c r="K671" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,028.1988; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L671" s="17" t="n">
+        <v>68011.26935928775</v>
+      </c>
+      <c r="M671" s="17">
+        <f>J671-L671</f>
+        <v/>
+      </c>
+      <c r="N671" s="18">
+        <f>IF(J671=0,"",L671/J671)</f>
+        <v/>
+      </c>
+      <c r="O671" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:33:20</t>
+        </is>
+      </c>
+      <c r="B672" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C672" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D672" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E672" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F672" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G672" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H672" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I672" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J672" s="17" t="n">
+        <v>197079.7129050169</v>
+      </c>
+      <c r="K672" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,243.9962</t>
+        </is>
+      </c>
+      <c r="L672" s="17" t="n">
+        <v>150243.996246735</v>
+      </c>
+      <c r="M672" s="17">
+        <f>J672-L672</f>
+        <v/>
+      </c>
+      <c r="N672" s="18">
+        <f>IF(J672=0,"",L672/J672)</f>
+        <v/>
+      </c>
+      <c r="O672" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:33:20</t>
+        </is>
+      </c>
+      <c r="B673" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C673" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D673" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E673" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F673" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G673" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H673" s="16" t="n">
+        <v>1.3726</v>
+      </c>
+      <c r="I673" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J673" s="17" t="n">
+        <v>186110.7077843311</v>
+      </c>
+      <c r="K673" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,140.3351</t>
+        </is>
+      </c>
+      <c r="L673" s="17" t="n">
+        <v>124140.3351430682</v>
+      </c>
+      <c r="M673" s="17">
+        <f>J673-L673</f>
+        <v/>
+      </c>
+      <c r="N673" s="18">
+        <f>IF(J673=0,"",L673/J673)</f>
+        <v/>
+      </c>
+      <c r="O673" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:33:20</t>
+        </is>
+      </c>
+      <c r="B674" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C674" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D674" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E674" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F674" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G674" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H674" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I674" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J674" s="17" t="n">
+        <v>327605.3654782894</v>
+      </c>
+      <c r="K674" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L674" s="17" t="n">
+        <v>280238.5543044237</v>
+      </c>
+      <c r="M674" s="17">
+        <f>J674-L674</f>
+        <v/>
+      </c>
+      <c r="N674" s="18">
+        <f>IF(J674=0,"",L674/J674)</f>
+        <v/>
+      </c>
+      <c r="O674" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:33:20</t>
+        </is>
+      </c>
+      <c r="B675" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C675" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D675" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E675" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F675" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G675" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H675" s="16" t="n">
+        <v>1.9045</v>
+      </c>
+      <c r="I675" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J675" s="17" t="n">
+        <v>159989.8916291629</v>
+      </c>
+      <c r="K675" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,938.3760</t>
+        </is>
+      </c>
+      <c r="L675" s="17" t="n">
+        <v>70938.37599253547</v>
+      </c>
+      <c r="M675" s="17">
+        <f>J675-L675</f>
+        <v/>
+      </c>
+      <c r="N675" s="18">
+        <f>IF(J675=0,"",L675/J675)</f>
+        <v/>
+      </c>
+      <c r="O675" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:33:20</t>
+        </is>
+      </c>
+      <c r="B676" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C676" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D676" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E676" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F676" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G676" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H676" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I676" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J676" s="17" t="n">
+        <v>160150.6237372169</v>
+      </c>
+      <c r="K676" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,523.0271</t>
+        </is>
+      </c>
+      <c r="L676" s="17" t="n">
+        <v>138509.1747529419</v>
+      </c>
+      <c r="M676" s="17">
+        <f>J676-L676</f>
+        <v/>
+      </c>
+      <c r="N676" s="18">
+        <f>IF(J676=0,"",L676/J676)</f>
+        <v/>
+      </c>
+      <c r="O676" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:33:20</t>
+        </is>
+      </c>
+      <c r="B677" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C677" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D677" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E677" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F677" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G677" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H677" s="16" t="inlineStr"/>
+      <c r="I677" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J677" s="17" t="n">
+        <v>95897.76799600091</v>
+      </c>
+      <c r="K677" s="15" t="inlineStr"/>
+      <c r="L677" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M677" s="17">
+        <f>J677-L677</f>
+        <v/>
+      </c>
+      <c r="N677" s="18">
+        <f>IF(J677=0,"",L677/J677)</f>
+        <v/>
+      </c>
+      <c r="O677" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:33:20</t>
+        </is>
+      </c>
+      <c r="B678" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C678" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D678" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E678" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F678" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G678" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H678" s="16" t="inlineStr"/>
+      <c r="I678" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J678" s="17" t="n">
+        <v>34347.40118094474</v>
+      </c>
+      <c r="K678" s="15" t="inlineStr"/>
+      <c r="L678" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M678" s="17">
+        <f>J678-L678</f>
+        <v/>
+      </c>
+      <c r="N678" s="18">
+        <f>IF(J678=0,"",L678/J678)</f>
+        <v/>
+      </c>
+      <c r="O678" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:33:20</t>
+        </is>
+      </c>
+      <c r="B679" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C679" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D679" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E679" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F679" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G679" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H679" s="16" t="n">
+        <v>1.043</v>
+      </c>
+      <c r="I679" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J679" s="17" t="n">
+        <v>269996.1113129806</v>
+      </c>
+      <c r="K679" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,041.5307</t>
+        </is>
+      </c>
+      <c r="L679" s="17" t="n">
+        <v>232983.2702843333</v>
+      </c>
+      <c r="M679" s="17">
+        <f>J679-L679</f>
+        <v/>
+      </c>
+      <c r="N679" s="18">
+        <f>IF(J679=0,"",L679/J679)</f>
+        <v/>
+      </c>
+      <c r="O679" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:33:20</t>
+        </is>
+      </c>
+      <c r="B680" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C680" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D680" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E680" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F680" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G680" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H680" s="16" t="inlineStr"/>
+      <c r="I680" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,511.6172</t>
+        </is>
+      </c>
+      <c r="J680" s="17" t="n">
+        <v>15507.73929220433</v>
+      </c>
+      <c r="K680" s="15" t="inlineStr"/>
+      <c r="L680" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M680" s="17">
+        <f>J680-L680</f>
+        <v/>
+      </c>
+      <c r="N680" s="18">
+        <f>IF(J680=0,"",L680/J680)</f>
+        <v/>
+      </c>
+      <c r="O680" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:33:20</t>
+        </is>
+      </c>
+      <c r="B681" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C681" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D681" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E681" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F681" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G681" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H681" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I681" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J681" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K681" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L681" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M681" s="17">
+        <f>J681-L681</f>
+        <v/>
+      </c>
+      <c r="N681" s="18">
+        <f>IF(J681=0,"",L681/J681)</f>
+        <v/>
+      </c>
+      <c r="O681" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:33:20</t>
+        </is>
+      </c>
+      <c r="B682" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C682" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D682" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E682" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F682" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G682" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H682" s="16" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="I682" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J682" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K682" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,705.3454</t>
+        </is>
+      </c>
+      <c r="L682" s="17" t="n">
+        <v>148705.345409</v>
+      </c>
+      <c r="M682" s="17">
+        <f>J682-L682</f>
+        <v/>
+      </c>
+      <c r="N682" s="18">
+        <f>IF(J682=0,"",L682/J682)</f>
+        <v/>
+      </c>
+      <c r="O682" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -45268,7 +46354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -46859,6 +47945,41 @@
         <v>1.0375</v>
       </c>
       <c r="I45" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:33:20</t>
+        </is>
+      </c>
+      <c r="B46" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C46" s="17" t="n">
+        <v>655466.0465684317</v>
+      </c>
+      <c r="D46" s="17" t="n">
+        <v>652853.4102350464</v>
+      </c>
+      <c r="E46" s="17" t="n">
+        <v>2933408.184365397</v>
+      </c>
+      <c r="F46" s="17" t="n">
+        <v>2280554.77413035</v>
+      </c>
+      <c r="G46" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H46" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I46" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 14:46 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O682"/>
+  <dimension ref="A1:O714"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -46324,6 +46324,2178 @@
         <v/>
       </c>
       <c r="O682" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:45:32</t>
+        </is>
+      </c>
+      <c r="B683" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C683" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D683" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E683" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F683" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G683" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H683" s="16" t="n">
+        <v>1.0505</v>
+      </c>
+      <c r="I683" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,804.5477</t>
+        </is>
+      </c>
+      <c r="J683" s="17" t="n">
+        <v>50792.35457156088</v>
+      </c>
+      <c r="K683" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,722.8797</t>
+        </is>
+      </c>
+      <c r="L683" s="17" t="n">
+        <v>37726.65235523552</v>
+      </c>
+      <c r="M683" s="17">
+        <f>J683-L683</f>
+        <v/>
+      </c>
+      <c r="N683" s="18">
+        <f>IF(J683=0,"",L683/J683)</f>
+        <v/>
+      </c>
+      <c r="O683" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:45:32</t>
+        </is>
+      </c>
+      <c r="B684" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C684" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D684" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E684" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F684" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G684" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H684" s="16" t="n">
+        <v>1.0479</v>
+      </c>
+      <c r="I684" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J684" s="17" t="n">
+        <v>140897.7988754021</v>
+      </c>
+      <c r="K684" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,035.0439</t>
+        </is>
+      </c>
+      <c r="L684" s="17" t="n">
+        <v>121005.9955164575</v>
+      </c>
+      <c r="M684" s="17">
+        <f>J684-L684</f>
+        <v/>
+      </c>
+      <c r="N684" s="18">
+        <f>IF(J684=0,"",L684/J684)</f>
+        <v/>
+      </c>
+      <c r="O684" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:45:32</t>
+        </is>
+      </c>
+      <c r="B685" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C685" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D685" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E685" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F685" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G685" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H685" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I685" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J685" s="17" t="n">
+        <v>328717.0046267734</v>
+      </c>
+      <c r="K685" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,386.0522</t>
+        </is>
+      </c>
+      <c r="L685" s="17" t="n">
+        <v>306423.4056871679</v>
+      </c>
+      <c r="M685" s="17">
+        <f>J685-L685</f>
+        <v/>
+      </c>
+      <c r="N685" s="18">
+        <f>IF(J685=0,"",L685/J685)</f>
+        <v/>
+      </c>
+      <c r="O685" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:45:32</t>
+        </is>
+      </c>
+      <c r="B686" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C686" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D686" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E686" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F686" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G686" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H686" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I686" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J686" s="17" t="n">
+        <v>386023.651692471</v>
+      </c>
+      <c r="K686" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,608.2120</t>
+        </is>
+      </c>
+      <c r="L686" s="17" t="n">
+        <v>349650.8349908394</v>
+      </c>
+      <c r="M686" s="17">
+        <f>J686-L686</f>
+        <v/>
+      </c>
+      <c r="N686" s="18">
+        <f>IF(J686=0,"",L686/J686)</f>
+        <v/>
+      </c>
+      <c r="O686" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:45:32</t>
+        </is>
+      </c>
+      <c r="B687" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C687" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D687" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E687" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F687" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G687" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H687" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I687" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7848</t>
+        </is>
+      </c>
+      <c r="J687" s="17" t="n">
+        <v>77796.27383059662</v>
+      </c>
+      <c r="K687" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,028.1988; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L687" s="17" t="n">
+        <v>68011.94964903301</v>
+      </c>
+      <c r="M687" s="17">
+        <f>J687-L687</f>
+        <v/>
+      </c>
+      <c r="N687" s="18">
+        <f>IF(J687=0,"",L687/J687)</f>
+        <v/>
+      </c>
+      <c r="O687" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:45:32</t>
+        </is>
+      </c>
+      <c r="B688" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C688" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D688" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E688" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F688" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G688" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H688" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I688" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J688" s="17" t="n">
+        <v>197080.84255422</v>
+      </c>
+      <c r="K688" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,243.9962</t>
+        </is>
+      </c>
+      <c r="L688" s="17" t="n">
+        <v>150259.0221489499</v>
+      </c>
+      <c r="M688" s="17">
+        <f>J688-L688</f>
+        <v/>
+      </c>
+      <c r="N688" s="18">
+        <f>IF(J688=0,"",L688/J688)</f>
+        <v/>
+      </c>
+      <c r="O688" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:45:32</t>
+        </is>
+      </c>
+      <c r="B689" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C689" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D689" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E689" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F689" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G689" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H689" s="16" t="n">
+        <v>1.3726</v>
+      </c>
+      <c r="I689" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J689" s="17" t="n">
+        <v>186101.2250658188</v>
+      </c>
+      <c r="K689" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,140.3351</t>
+        </is>
+      </c>
+      <c r="L689" s="17" t="n">
+        <v>124152.75041811</v>
+      </c>
+      <c r="M689" s="17">
+        <f>J689-L689</f>
+        <v/>
+      </c>
+      <c r="N689" s="18">
+        <f>IF(J689=0,"",L689/J689)</f>
+        <v/>
+      </c>
+      <c r="O689" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:45:32</t>
+        </is>
+      </c>
+      <c r="B690" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C690" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D690" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E690" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F690" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G690" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H690" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I690" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J690" s="17" t="n">
+        <v>327605.6696321312</v>
+      </c>
+      <c r="K690" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L690" s="17" t="n">
+        <v>280238.4977328491</v>
+      </c>
+      <c r="M690" s="17">
+        <f>J690-L690</f>
+        <v/>
+      </c>
+      <c r="N690" s="18">
+        <f>IF(J690=0,"",L690/J690)</f>
+        <v/>
+      </c>
+      <c r="O690" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:45:32</t>
+        </is>
+      </c>
+      <c r="B691" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C691" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D691" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E691" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F691" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G691" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H691" s="16" t="n">
+        <v>1.9045</v>
+      </c>
+      <c r="I691" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J691" s="17" t="n">
+        <v>159989.8916291629</v>
+      </c>
+      <c r="K691" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,938.3760</t>
+        </is>
+      </c>
+      <c r="L691" s="17" t="n">
+        <v>70945.47053958943</v>
+      </c>
+      <c r="M691" s="17">
+        <f>J691-L691</f>
+        <v/>
+      </c>
+      <c r="N691" s="18">
+        <f>IF(J691=0,"",L691/J691)</f>
+        <v/>
+      </c>
+      <c r="O691" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:45:32</t>
+        </is>
+      </c>
+      <c r="B692" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C692" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D692" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E692" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F692" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G692" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H692" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I692" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J692" s="17" t="n">
+        <v>160150.7675671492</v>
+      </c>
+      <c r="K692" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,523.0271</t>
+        </is>
+      </c>
+      <c r="L692" s="17" t="n">
+        <v>138509.1747529419</v>
+      </c>
+      <c r="M692" s="17">
+        <f>J692-L692</f>
+        <v/>
+      </c>
+      <c r="N692" s="18">
+        <f>IF(J692=0,"",L692/J692)</f>
+        <v/>
+      </c>
+      <c r="O692" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:45:32</t>
+        </is>
+      </c>
+      <c r="B693" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C693" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D693" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E693" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F693" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G693" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H693" s="16" t="inlineStr"/>
+      <c r="I693" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J693" s="17" t="n">
+        <v>95902.21287327852</v>
+      </c>
+      <c r="K693" s="15" t="inlineStr"/>
+      <c r="L693" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M693" s="17">
+        <f>J693-L693</f>
+        <v/>
+      </c>
+      <c r="N693" s="18">
+        <f>IF(J693=0,"",L693/J693)</f>
+        <v/>
+      </c>
+      <c r="O693" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:45:32</t>
+        </is>
+      </c>
+      <c r="B694" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C694" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D694" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E694" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F694" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G694" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H694" s="16" t="inlineStr"/>
+      <c r="I694" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J694" s="17" t="n">
+        <v>34357.35541182909</v>
+      </c>
+      <c r="K694" s="15" t="inlineStr"/>
+      <c r="L694" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M694" s="17">
+        <f>J694-L694</f>
+        <v/>
+      </c>
+      <c r="N694" s="18">
+        <f>IF(J694=0,"",L694/J694)</f>
+        <v/>
+      </c>
+      <c r="O694" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:45:32</t>
+        </is>
+      </c>
+      <c r="B695" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C695" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D695" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E695" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F695" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G695" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H695" s="16" t="n">
+        <v>1.043</v>
+      </c>
+      <c r="I695" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J695" s="17" t="n">
+        <v>269996.1113129806</v>
+      </c>
+      <c r="K695" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,041.5307</t>
+        </is>
+      </c>
+      <c r="L695" s="17" t="n">
+        <v>232985.6006996399</v>
+      </c>
+      <c r="M695" s="17">
+        <f>J695-L695</f>
+        <v/>
+      </c>
+      <c r="N695" s="18">
+        <f>IF(J695=0,"",L695/J695)</f>
+        <v/>
+      </c>
+      <c r="O695" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:45:32</t>
+        </is>
+      </c>
+      <c r="B696" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C696" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D696" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E696" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F696" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G696" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H696" s="16" t="inlineStr"/>
+      <c r="I696" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,511.6172</t>
+        </is>
+      </c>
+      <c r="J696" s="17" t="n">
+        <v>15507.89440837629</v>
+      </c>
+      <c r="K696" s="15" t="inlineStr"/>
+      <c r="L696" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M696" s="17">
+        <f>J696-L696</f>
+        <v/>
+      </c>
+      <c r="N696" s="18">
+        <f>IF(J696=0,"",L696/J696)</f>
+        <v/>
+      </c>
+      <c r="O696" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:45:32</t>
+        </is>
+      </c>
+      <c r="B697" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C697" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D697" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E697" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F697" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G697" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H697" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I697" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J697" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K697" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L697" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M697" s="17">
+        <f>J697-L697</f>
+        <v/>
+      </c>
+      <c r="N697" s="18">
+        <f>IF(J697=0,"",L697/J697)</f>
+        <v/>
+      </c>
+      <c r="O697" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:45:32</t>
+        </is>
+      </c>
+      <c r="B698" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C698" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D698" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E698" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F698" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G698" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H698" s="16" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="I698" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J698" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K698" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,705.3454</t>
+        </is>
+      </c>
+      <c r="L698" s="17" t="n">
+        <v>148705.345409</v>
+      </c>
+      <c r="M698" s="17">
+        <f>J698-L698</f>
+        <v/>
+      </c>
+      <c r="N698" s="18">
+        <f>IF(J698=0,"",L698/J698)</f>
+        <v/>
+      </c>
+      <c r="O698" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:46:49</t>
+        </is>
+      </c>
+      <c r="B699" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C699" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D699" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E699" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F699" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G699" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H699" s="16" t="n">
+        <v>1.0505</v>
+      </c>
+      <c r="I699" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,804.5477</t>
+        </is>
+      </c>
+      <c r="J699" s="17" t="n">
+        <v>50793.87870799076</v>
+      </c>
+      <c r="K699" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,722.8797</t>
+        </is>
+      </c>
+      <c r="L699" s="17" t="n">
+        <v>37726.65235523552</v>
+      </c>
+      <c r="M699" s="17">
+        <f>J699-L699</f>
+        <v/>
+      </c>
+      <c r="N699" s="18">
+        <f>IF(J699=0,"",L699/J699)</f>
+        <v/>
+      </c>
+      <c r="O699" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:46:49</t>
+        </is>
+      </c>
+      <c r="B700" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C700" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D700" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E700" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F700" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G700" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H700" s="16" t="n">
+        <v>1.0479</v>
+      </c>
+      <c r="I700" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J700" s="17" t="n">
+        <v>140897.7988754021</v>
+      </c>
+      <c r="K700" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,035.0439</t>
+        </is>
+      </c>
+      <c r="L700" s="17" t="n">
+        <v>121009.6265677753</v>
+      </c>
+      <c r="M700" s="17">
+        <f>J700-L700</f>
+        <v/>
+      </c>
+      <c r="N700" s="18">
+        <f>IF(J700=0,"",L700/J700)</f>
+        <v/>
+      </c>
+      <c r="O700" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:46:49</t>
+        </is>
+      </c>
+      <c r="B701" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C701" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D701" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E701" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F701" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G701" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H701" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I701" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J701" s="17" t="n">
+        <v>328717.0046267734</v>
+      </c>
+      <c r="K701" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,386.0522</t>
+        </is>
+      </c>
+      <c r="L701" s="17" t="n">
+        <v>306454.0510200775</v>
+      </c>
+      <c r="M701" s="17">
+        <f>J701-L701</f>
+        <v/>
+      </c>
+      <c r="N701" s="18">
+        <f>IF(J701=0,"",L701/J701)</f>
+        <v/>
+      </c>
+      <c r="O701" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:46:49</t>
+        </is>
+      </c>
+      <c r="B702" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C702" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D702" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E702" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F702" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G702" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H702" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I702" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J702" s="17" t="n">
+        <v>386023.651692471</v>
+      </c>
+      <c r="K702" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,608.2120</t>
+        </is>
+      </c>
+      <c r="L702" s="17" t="n">
+        <v>349685.8034888116</v>
+      </c>
+      <c r="M702" s="17">
+        <f>J702-L702</f>
+        <v/>
+      </c>
+      <c r="N702" s="18">
+        <f>IF(J702=0,"",L702/J702)</f>
+        <v/>
+      </c>
+      <c r="O702" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:46:49</t>
+        </is>
+      </c>
+      <c r="B703" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C703" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D703" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E703" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F703" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G703" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H703" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I703" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7848</t>
+        </is>
+      </c>
+      <c r="J703" s="17" t="n">
+        <v>77796.2765434654</v>
+      </c>
+      <c r="K703" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,028.1988; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L703" s="17" t="n">
+        <v>68013.99049499848</v>
+      </c>
+      <c r="M703" s="17">
+        <f>J703-L703</f>
+        <v/>
+      </c>
+      <c r="N703" s="18">
+        <f>IF(J703=0,"",L703/J703)</f>
+        <v/>
+      </c>
+      <c r="O703" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:46:49</t>
+        </is>
+      </c>
+      <c r="B704" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C704" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D704" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E704" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F704" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G704" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H704" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I704" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J704" s="17" t="n">
+        <v>197080.84255422</v>
+      </c>
+      <c r="K704" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,243.9962</t>
+        </is>
+      </c>
+      <c r="L704" s="17" t="n">
+        <v>150259.0221489499</v>
+      </c>
+      <c r="M704" s="17">
+        <f>J704-L704</f>
+        <v/>
+      </c>
+      <c r="N704" s="18">
+        <f>IF(J704=0,"",L704/J704)</f>
+        <v/>
+      </c>
+      <c r="O704" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:46:49</t>
+        </is>
+      </c>
+      <c r="B705" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C705" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D705" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E705" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F705" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G705" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H705" s="16" t="n">
+        <v>1.3726</v>
+      </c>
+      <c r="I705" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J705" s="17" t="n">
+        <v>186101.2250658188</v>
+      </c>
+      <c r="K705" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,140.3351</t>
+        </is>
+      </c>
+      <c r="L705" s="17" t="n">
+        <v>124152.75041811</v>
+      </c>
+      <c r="M705" s="17">
+        <f>J705-L705</f>
+        <v/>
+      </c>
+      <c r="N705" s="18">
+        <f>IF(J705=0,"",L705/J705)</f>
+        <v/>
+      </c>
+      <c r="O705" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:46:49</t>
+        </is>
+      </c>
+      <c r="B706" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C706" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D706" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E706" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F706" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G706" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H706" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I706" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J706" s="17" t="n">
+        <v>327605.6696321312</v>
+      </c>
+      <c r="K706" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L706" s="17" t="n">
+        <v>280241.5414304747</v>
+      </c>
+      <c r="M706" s="17">
+        <f>J706-L706</f>
+        <v/>
+      </c>
+      <c r="N706" s="18">
+        <f>IF(J706=0,"",L706/J706)</f>
+        <v/>
+      </c>
+      <c r="O706" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:46:49</t>
+        </is>
+      </c>
+      <c r="B707" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C707" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D707" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E707" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F707" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G707" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H707" s="16" t="n">
+        <v>1.9045</v>
+      </c>
+      <c r="I707" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J707" s="17" t="n">
+        <v>159989.8916291629</v>
+      </c>
+      <c r="K707" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,938.3760</t>
+        </is>
+      </c>
+      <c r="L707" s="17" t="n">
+        <v>70945.47053958943</v>
+      </c>
+      <c r="M707" s="17">
+        <f>J707-L707</f>
+        <v/>
+      </c>
+      <c r="N707" s="18">
+        <f>IF(J707=0,"",L707/J707)</f>
+        <v/>
+      </c>
+      <c r="O707" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:46:49</t>
+        </is>
+      </c>
+      <c r="B708" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C708" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D708" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E708" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F708" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G708" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H708" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I708" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J708" s="17" t="n">
+        <v>160150.7675671492</v>
+      </c>
+      <c r="K708" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,523.0271</t>
+        </is>
+      </c>
+      <c r="L708" s="17" t="n">
+        <v>138509.1747529419</v>
+      </c>
+      <c r="M708" s="17">
+        <f>J708-L708</f>
+        <v/>
+      </c>
+      <c r="N708" s="18">
+        <f>IF(J708=0,"",L708/J708)</f>
+        <v/>
+      </c>
+      <c r="O708" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:46:49</t>
+        </is>
+      </c>
+      <c r="B709" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C709" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D709" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E709" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F709" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G709" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H709" s="16" t="inlineStr"/>
+      <c r="I709" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J709" s="17" t="n">
+        <v>95902.21287327852</v>
+      </c>
+      <c r="K709" s="15" t="inlineStr"/>
+      <c r="L709" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M709" s="17">
+        <f>J709-L709</f>
+        <v/>
+      </c>
+      <c r="N709" s="18">
+        <f>IF(J709=0,"",L709/J709)</f>
+        <v/>
+      </c>
+      <c r="O709" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:46:49</t>
+        </is>
+      </c>
+      <c r="B710" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C710" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D710" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E710" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F710" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G710" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H710" s="16" t="inlineStr"/>
+      <c r="I710" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J710" s="17" t="n">
+        <v>34357.35541182909</v>
+      </c>
+      <c r="K710" s="15" t="inlineStr"/>
+      <c r="L710" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M710" s="17">
+        <f>J710-L710</f>
+        <v/>
+      </c>
+      <c r="N710" s="18">
+        <f>IF(J710=0,"",L710/J710)</f>
+        <v/>
+      </c>
+      <c r="O710" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:46:49</t>
+        </is>
+      </c>
+      <c r="B711" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C711" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D711" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E711" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F711" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G711" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H711" s="16" t="n">
+        <v>1.0429</v>
+      </c>
+      <c r="I711" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J711" s="17" t="n">
+        <v>269996.1113129806</v>
+      </c>
+      <c r="K711" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,041.5307</t>
+        </is>
+      </c>
+      <c r="L711" s="17" t="n">
+        <v>232992.5919455599</v>
+      </c>
+      <c r="M711" s="17">
+        <f>J711-L711</f>
+        <v/>
+      </c>
+      <c r="N711" s="18">
+        <f>IF(J711=0,"",L711/J711)</f>
+        <v/>
+      </c>
+      <c r="O711" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:46:49</t>
+        </is>
+      </c>
+      <c r="B712" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C712" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D712" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E712" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F712" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G712" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H712" s="16" t="inlineStr"/>
+      <c r="I712" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,511.6172</t>
+        </is>
+      </c>
+      <c r="J712" s="17" t="n">
+        <v>15508.35975689219</v>
+      </c>
+      <c r="K712" s="15" t="inlineStr"/>
+      <c r="L712" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M712" s="17">
+        <f>J712-L712</f>
+        <v/>
+      </c>
+      <c r="N712" s="18">
+        <f>IF(J712=0,"",L712/J712)</f>
+        <v/>
+      </c>
+      <c r="O712" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:46:49</t>
+        </is>
+      </c>
+      <c r="B713" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C713" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D713" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E713" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F713" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G713" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H713" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I713" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J713" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K713" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L713" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M713" s="17">
+        <f>J713-L713</f>
+        <v/>
+      </c>
+      <c r="N713" s="18">
+        <f>IF(J713=0,"",L713/J713)</f>
+        <v/>
+      </c>
+      <c r="O713" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:46:49</t>
+        </is>
+      </c>
+      <c r="B714" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C714" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D714" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E714" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F714" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G714" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H714" s="16" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="I714" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J714" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K714" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,705.3454</t>
+        </is>
+      </c>
+      <c r="L714" s="17" t="n">
+        <v>148705.345409</v>
+      </c>
+      <c r="M714" s="17">
+        <f>J714-L714</f>
+        <v/>
+      </c>
+      <c r="N714" s="18">
+        <f>IF(J714=0,"",L714/J714)</f>
+        <v/>
+      </c>
+      <c r="O714" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -46354,7 +48526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -47980,6 +50152,76 @@
         <v>1.0375</v>
       </c>
       <c r="I46" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:45:32</t>
+        </is>
+      </c>
+      <c r="B47" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C47" s="17" t="n">
+        <v>655417.7623727216</v>
+      </c>
+      <c r="D47" s="17" t="n">
+        <v>652805.1876388872</v>
+      </c>
+      <c r="E47" s="17" t="n">
+        <v>2933402.4346427</v>
+      </c>
+      <c r="F47" s="17" t="n">
+        <v>2280597.247003813</v>
+      </c>
+      <c r="G47" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H47" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I47" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:46:49</t>
+        </is>
+      </c>
+      <c r="B48" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C48" s="17" t="n">
+        <v>655338.366412363</v>
+      </c>
+      <c r="D48" s="17" t="n">
+        <v>652725.8591649905</v>
+      </c>
+      <c r="E48" s="17" t="n">
+        <v>2933404.426840515</v>
+      </c>
+      <c r="F48" s="17" t="n">
+        <v>2280678.567675524</v>
+      </c>
+      <c r="G48" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H48" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I48" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
feat: multi-page dashboard, 12h cron, benchmark strip, 14d columns
- Positions page: columns Now/12h/24h/36h/48h/7d/14d, color threshold 0.01%
- Benchmark strip: Day 0 delta + vs 1mo/3mo/1y (auto-fills over time)
- New History page (history.html): full snapshot log, equity + delta per row
- Page nav between Positions ↔ History
- Cron changed from */30 to 0,12 UTC (12h cadence)
- Loopscale REST API confirmed working, Playwright kept as fallback

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O714"/>
+  <dimension ref="A1:O730"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -48496,6 +48496,1092 @@
         <v/>
       </c>
       <c r="O714" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:10:42</t>
+        </is>
+      </c>
+      <c r="B715" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C715" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D715" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E715" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F715" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G715" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H715" s="16" t="n">
+        <v>1.0505</v>
+      </c>
+      <c r="I715" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,804.5477</t>
+        </is>
+      </c>
+      <c r="J715" s="17" t="n">
+        <v>50787.78216227121</v>
+      </c>
+      <c r="K715" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,722.8797</t>
+        </is>
+      </c>
+      <c r="L715" s="17" t="n">
+        <v>37722.87969</v>
+      </c>
+      <c r="M715" s="17">
+        <f>J715-L715</f>
+        <v/>
+      </c>
+      <c r="N715" s="18">
+        <f>IF(J715=0,"",L715/J715)</f>
+        <v/>
+      </c>
+      <c r="O715" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:10:42</t>
+        </is>
+      </c>
+      <c r="B716" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C716" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D716" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E716" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F716" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G716" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H716" s="16" t="n">
+        <v>1.048</v>
+      </c>
+      <c r="I716" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J716" s="17" t="n">
+        <v>140898.0193427771</v>
+      </c>
+      <c r="K716" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,035.0439</t>
+        </is>
+      </c>
+      <c r="L716" s="17" t="n">
+        <v>120995.1023625041</v>
+      </c>
+      <c r="M716" s="17">
+        <f>J716-L716</f>
+        <v/>
+      </c>
+      <c r="N716" s="18">
+        <f>IF(J716=0,"",L716/J716)</f>
+        <v/>
+      </c>
+      <c r="O716" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:10:42</t>
+        </is>
+      </c>
+      <c r="B717" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C717" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D717" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E717" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F717" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G717" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H717" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I717" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J717" s="17" t="n">
+        <v>328717.7033096657</v>
+      </c>
+      <c r="K717" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,386.0522</t>
+        </is>
+      </c>
+      <c r="L717" s="17" t="n">
+        <v>306411.398624031</v>
+      </c>
+      <c r="M717" s="17">
+        <f>J717-L717</f>
+        <v/>
+      </c>
+      <c r="N717" s="18">
+        <f>IF(J717=0,"",L717/J717)</f>
+        <v/>
+      </c>
+      <c r="O717" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:10:42</t>
+        </is>
+      </c>
+      <c r="B718" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C718" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D718" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E718" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F718" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G718" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H718" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I718" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J718" s="17" t="n">
+        <v>386024.7609759028</v>
+      </c>
+      <c r="K718" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,608.2120</t>
+        </is>
+      </c>
+      <c r="L718" s="17" t="n">
+        <v>349637.1340803551</v>
+      </c>
+      <c r="M718" s="17">
+        <f>J718-L718</f>
+        <v/>
+      </c>
+      <c r="N718" s="18">
+        <f>IF(J718=0,"",L718/J718)</f>
+        <v/>
+      </c>
+      <c r="O718" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:10:42</t>
+        </is>
+      </c>
+      <c r="B719" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C719" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D719" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E719" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F719" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G719" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H719" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I719" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7848</t>
+        </is>
+      </c>
+      <c r="J719" s="17" t="n">
+        <v>77789.1739361389</v>
+      </c>
+      <c r="K719" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,028.1988; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L719" s="17" t="n">
+        <v>68007.1876673568</v>
+      </c>
+      <c r="M719" s="17">
+        <f>J719-L719</f>
+        <v/>
+      </c>
+      <c r="N719" s="18">
+        <f>IF(J719=0,"",L719/J719)</f>
+        <v/>
+      </c>
+      <c r="O719" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:10:42</t>
+        </is>
+      </c>
+      <c r="B720" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C720" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D720" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E720" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F720" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G720" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H720" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I720" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J720" s="17" t="n">
+        <v>197082.5406068833</v>
+      </c>
+      <c r="K720" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,243.9962</t>
+        </is>
+      </c>
+      <c r="L720" s="17" t="n">
+        <v>150243.996246735</v>
+      </c>
+      <c r="M720" s="17">
+        <f>J720-L720</f>
+        <v/>
+      </c>
+      <c r="N720" s="18">
+        <f>IF(J720=0,"",L720/J720)</f>
+        <v/>
+      </c>
+      <c r="O720" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:10:42</t>
+        </is>
+      </c>
+      <c r="B721" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C721" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D721" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E721" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F721" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G721" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H721" s="16" t="n">
+        <v>1.3726</v>
+      </c>
+      <c r="I721" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J721" s="17" t="n">
+        <v>186091.8444123784</v>
+      </c>
+      <c r="K721" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,140.3351</t>
+        </is>
+      </c>
+      <c r="L721" s="17" t="n">
+        <v>124140.3351430682</v>
+      </c>
+      <c r="M721" s="17">
+        <f>J721-L721</f>
+        <v/>
+      </c>
+      <c r="N721" s="18">
+        <f>IF(J721=0,"",L721/J721)</f>
+        <v/>
+      </c>
+      <c r="O721" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:10:42</t>
+        </is>
+      </c>
+      <c r="B722" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C722" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D722" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E722" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F722" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G722" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H722" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I722" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J722" s="17" t="n">
+        <v>327605.6696321312</v>
+      </c>
+      <c r="K722" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L722" s="17" t="n">
+        <v>280238.4852792478</v>
+      </c>
+      <c r="M722" s="17">
+        <f>J722-L722</f>
+        <v/>
+      </c>
+      <c r="N722" s="18">
+        <f>IF(J722=0,"",L722/J722)</f>
+        <v/>
+      </c>
+      <c r="O722" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:10:42</t>
+        </is>
+      </c>
+      <c r="B723" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C723" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D723" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E723" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F723" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G723" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H723" s="16" t="n">
+        <v>1.9045</v>
+      </c>
+      <c r="I723" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J723" s="17" t="n">
+        <v>159989.8916291629</v>
+      </c>
+      <c r="K723" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,938.3760</t>
+        </is>
+      </c>
+      <c r="L723" s="17" t="n">
+        <v>70938.37599253547</v>
+      </c>
+      <c r="M723" s="17">
+        <f>J723-L723</f>
+        <v/>
+      </c>
+      <c r="N723" s="18">
+        <f>IF(J723=0,"",L723/J723)</f>
+        <v/>
+      </c>
+      <c r="O723" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:10:42</t>
+        </is>
+      </c>
+      <c r="B724" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C724" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D724" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E724" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F724" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G724" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H724" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I724" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J724" s="17" t="n">
+        <v>160151.2277788286</v>
+      </c>
+      <c r="K724" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,523.0271</t>
+        </is>
+      </c>
+      <c r="L724" s="17" t="n">
+        <v>138509.1747529419</v>
+      </c>
+      <c r="M724" s="17">
+        <f>J724-L724</f>
+        <v/>
+      </c>
+      <c r="N724" s="18">
+        <f>IF(J724=0,"",L724/J724)</f>
+        <v/>
+      </c>
+      <c r="O724" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:10:42</t>
+        </is>
+      </c>
+      <c r="B725" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C725" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D725" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E725" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F725" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G725" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H725" s="16" t="inlineStr"/>
+      <c r="I725" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J725" s="17" t="n">
+        <v>95887.44131056532</v>
+      </c>
+      <c r="K725" s="15" t="inlineStr"/>
+      <c r="L725" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M725" s="17">
+        <f>J725-L725</f>
+        <v/>
+      </c>
+      <c r="N725" s="18">
+        <f>IF(J725=0,"",L725/J725)</f>
+        <v/>
+      </c>
+      <c r="O725" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:10:42</t>
+        </is>
+      </c>
+      <c r="B726" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C726" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D726" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E726" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F726" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G726" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H726" s="16" t="inlineStr"/>
+      <c r="I726" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J726" s="17" t="n">
+        <v>34357.63649597362</v>
+      </c>
+      <c r="K726" s="15" t="inlineStr"/>
+      <c r="L726" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M726" s="17">
+        <f>J726-L726</f>
+        <v/>
+      </c>
+      <c r="N726" s="18">
+        <f>IF(J726=0,"",L726/J726)</f>
+        <v/>
+      </c>
+      <c r="O726" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:10:42</t>
+        </is>
+      </c>
+      <c r="B727" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C727" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D727" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E727" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F727" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G727" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H727" s="16" t="n">
+        <v>1.0431</v>
+      </c>
+      <c r="I727" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J727" s="17" t="n">
+        <v>270023.1136243431</v>
+      </c>
+      <c r="K727" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,041.5307</t>
+        </is>
+      </c>
+      <c r="L727" s="17" t="n">
+        <v>232969.2877924932</v>
+      </c>
+      <c r="M727" s="17">
+        <f>J727-L727</f>
+        <v/>
+      </c>
+      <c r="N727" s="18">
+        <f>IF(J727=0,"",L727/J727)</f>
+        <v/>
+      </c>
+      <c r="O727" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:10:42</t>
+        </is>
+      </c>
+      <c r="B728" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C728" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D728" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E728" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F728" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G728" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H728" s="16" t="inlineStr"/>
+      <c r="I728" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,511.8192</t>
+        </is>
+      </c>
+      <c r="J728" s="17" t="n">
+        <v>15507.01056218378</v>
+      </c>
+      <c r="K728" s="15" t="inlineStr"/>
+      <c r="L728" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M728" s="17">
+        <f>J728-L728</f>
+        <v/>
+      </c>
+      <c r="N728" s="18">
+        <f>IF(J728=0,"",L728/J728)</f>
+        <v/>
+      </c>
+      <c r="O728" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:10:42</t>
+        </is>
+      </c>
+      <c r="B729" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C729" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D729" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E729" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F729" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G729" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H729" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I729" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J729" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K729" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L729" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M729" s="17">
+        <f>J729-L729</f>
+        <v/>
+      </c>
+      <c r="N729" s="18">
+        <f>IF(J729=0,"",L729/J729)</f>
+        <v/>
+      </c>
+      <c r="O729" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:10:42</t>
+        </is>
+      </c>
+      <c r="B730" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C730" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D730" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E730" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F730" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G730" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H730" s="16" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="I730" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J730" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K730" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,705.3454</t>
+        </is>
+      </c>
+      <c r="L730" s="17" t="n">
+        <v>148705.345409</v>
+      </c>
+      <c r="M730" s="17">
+        <f>J730-L730</f>
+        <v/>
+      </c>
+      <c r="N730" s="18">
+        <f>IF(J730=0,"",L730/J730)</f>
+        <v/>
+      </c>
+      <c r="O730" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -48526,7 +49612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -50222,6 +51308,41 @@
         <v>1.0375</v>
       </c>
       <c r="I48" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:10:42</t>
+        </is>
+      </c>
+      <c r="B49" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C49" s="17" t="n">
+        <v>655506.2797276784</v>
+      </c>
+      <c r="D49" s="17" t="n">
+        <v>652895.9462258876</v>
+      </c>
+      <c r="E49" s="17" t="n">
+        <v>2933397.196370156</v>
+      </c>
+      <c r="F49" s="17" t="n">
+        <v>2280501.250144268</v>
+      </c>
+      <c r="G49" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H49" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I49" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 15:17 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O730"/>
+  <dimension ref="A1:O778"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -49582,6 +49582,3264 @@
         <v/>
       </c>
       <c r="O730" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:13</t>
+        </is>
+      </c>
+      <c r="B731" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C731" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D731" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E731" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F731" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G731" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H731" s="16" t="n">
+        <v>1.0505</v>
+      </c>
+      <c r="I731" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,804.5477</t>
+        </is>
+      </c>
+      <c r="J731" s="17" t="n">
+        <v>50787.78216227121</v>
+      </c>
+      <c r="K731" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,722.8797</t>
+        </is>
+      </c>
+      <c r="L731" s="17" t="n">
+        <v>37722.87969</v>
+      </c>
+      <c r="M731" s="17">
+        <f>J731-L731</f>
+        <v/>
+      </c>
+      <c r="N731" s="18">
+        <f>IF(J731=0,"",L731/J731)</f>
+        <v/>
+      </c>
+      <c r="O731" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:13</t>
+        </is>
+      </c>
+      <c r="B732" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C732" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D732" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E732" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F732" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G732" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H732" s="16" t="n">
+        <v>1.048</v>
+      </c>
+      <c r="I732" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J732" s="17" t="n">
+        <v>140898.0193427771</v>
+      </c>
+      <c r="K732" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,035.0439</t>
+        </is>
+      </c>
+      <c r="L732" s="17" t="n">
+        <v>120995.1023625041</v>
+      </c>
+      <c r="M732" s="17">
+        <f>J732-L732</f>
+        <v/>
+      </c>
+      <c r="N732" s="18">
+        <f>IF(J732=0,"",L732/J732)</f>
+        <v/>
+      </c>
+      <c r="O732" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:13</t>
+        </is>
+      </c>
+      <c r="B733" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C733" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D733" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E733" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F733" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G733" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H733" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I733" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J733" s="17" t="n">
+        <v>328717.7033096657</v>
+      </c>
+      <c r="K733" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,386.0522</t>
+        </is>
+      </c>
+      <c r="L733" s="17" t="n">
+        <v>306411.398624031</v>
+      </c>
+      <c r="M733" s="17">
+        <f>J733-L733</f>
+        <v/>
+      </c>
+      <c r="N733" s="18">
+        <f>IF(J733=0,"",L733/J733)</f>
+        <v/>
+      </c>
+      <c r="O733" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:13</t>
+        </is>
+      </c>
+      <c r="B734" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C734" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D734" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E734" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F734" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G734" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H734" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I734" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J734" s="17" t="n">
+        <v>386025.5466608055</v>
+      </c>
+      <c r="K734" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,608.2120</t>
+        </is>
+      </c>
+      <c r="L734" s="17" t="n">
+        <v>349637.1340803551</v>
+      </c>
+      <c r="M734" s="17">
+        <f>J734-L734</f>
+        <v/>
+      </c>
+      <c r="N734" s="18">
+        <f>IF(J734=0,"",L734/J734)</f>
+        <v/>
+      </c>
+      <c r="O734" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:13</t>
+        </is>
+      </c>
+      <c r="B735" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C735" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D735" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E735" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F735" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G735" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H735" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I735" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7848</t>
+        </is>
+      </c>
+      <c r="J735" s="17" t="n">
+        <v>77789.03960923906</v>
+      </c>
+      <c r="K735" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,028.1988; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L735" s="17" t="n">
+        <v>68005.82710337982</v>
+      </c>
+      <c r="M735" s="17">
+        <f>J735-L735</f>
+        <v/>
+      </c>
+      <c r="N735" s="18">
+        <f>IF(J735=0,"",L735/J735)</f>
+        <v/>
+      </c>
+      <c r="O735" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:13</t>
+        </is>
+      </c>
+      <c r="B736" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C736" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D736" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E736" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F736" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G736" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H736" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I736" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J736" s="17" t="n">
+        <v>197082.5406068833</v>
+      </c>
+      <c r="K736" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,243.9962</t>
+        </is>
+      </c>
+      <c r="L736" s="17" t="n">
+        <v>150243.996246735</v>
+      </c>
+      <c r="M736" s="17">
+        <f>J736-L736</f>
+        <v/>
+      </c>
+      <c r="N736" s="18">
+        <f>IF(J736=0,"",L736/J736)</f>
+        <v/>
+      </c>
+      <c r="O736" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:13</t>
+        </is>
+      </c>
+      <c r="B737" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C737" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D737" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E737" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F737" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G737" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H737" s="16" t="n">
+        <v>1.3726</v>
+      </c>
+      <c r="I737" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J737" s="17" t="n">
+        <v>186091.8444123784</v>
+      </c>
+      <c r="K737" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,140.3351</t>
+        </is>
+      </c>
+      <c r="L737" s="17" t="n">
+        <v>124140.3351430682</v>
+      </c>
+      <c r="M737" s="17">
+        <f>J737-L737</f>
+        <v/>
+      </c>
+      <c r="N737" s="18">
+        <f>IF(J737=0,"",L737/J737)</f>
+        <v/>
+      </c>
+      <c r="O737" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:13</t>
+        </is>
+      </c>
+      <c r="B738" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C738" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D738" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E738" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F738" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G738" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H738" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I738" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J738" s="17" t="n">
+        <v>327605.5893985275</v>
+      </c>
+      <c r="K738" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L738" s="17" t="n">
+        <v>280238.4852792478</v>
+      </c>
+      <c r="M738" s="17">
+        <f>J738-L738</f>
+        <v/>
+      </c>
+      <c r="N738" s="18">
+        <f>IF(J738=0,"",L738/J738)</f>
+        <v/>
+      </c>
+      <c r="O738" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:13</t>
+        </is>
+      </c>
+      <c r="B739" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C739" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D739" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E739" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F739" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G739" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H739" s="16" t="n">
+        <v>1.9045</v>
+      </c>
+      <c r="I739" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J739" s="17" t="n">
+        <v>159989.8916291629</v>
+      </c>
+      <c r="K739" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,938.3760</t>
+        </is>
+      </c>
+      <c r="L739" s="17" t="n">
+        <v>70938.37599253547</v>
+      </c>
+      <c r="M739" s="17">
+        <f>J739-L739</f>
+        <v/>
+      </c>
+      <c r="N739" s="18">
+        <f>IF(J739=0,"",L739/J739)</f>
+        <v/>
+      </c>
+      <c r="O739" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:13</t>
+        </is>
+      </c>
+      <c r="B740" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C740" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D740" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E740" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F740" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G740" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H740" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I740" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J740" s="17" t="n">
+        <v>160151.5537382347</v>
+      </c>
+      <c r="K740" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,523.0271</t>
+        </is>
+      </c>
+      <c r="L740" s="17" t="n">
+        <v>138509.1747529419</v>
+      </c>
+      <c r="M740" s="17">
+        <f>J740-L740</f>
+        <v/>
+      </c>
+      <c r="N740" s="18">
+        <f>IF(J740=0,"",L740/J740)</f>
+        <v/>
+      </c>
+      <c r="O740" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:13</t>
+        </is>
+      </c>
+      <c r="B741" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C741" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D741" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E741" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F741" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G741" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H741" s="16" t="inlineStr"/>
+      <c r="I741" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J741" s="17" t="n">
+        <v>95887.44131056532</v>
+      </c>
+      <c r="K741" s="15" t="inlineStr"/>
+      <c r="L741" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M741" s="17">
+        <f>J741-L741</f>
+        <v/>
+      </c>
+      <c r="N741" s="18">
+        <f>IF(J741=0,"",L741/J741)</f>
+        <v/>
+      </c>
+      <c r="O741" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:13</t>
+        </is>
+      </c>
+      <c r="B742" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C742" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D742" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E742" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F742" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G742" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H742" s="16" t="inlineStr"/>
+      <c r="I742" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J742" s="17" t="n">
+        <v>34357.63649597362</v>
+      </c>
+      <c r="K742" s="15" t="inlineStr"/>
+      <c r="L742" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M742" s="17">
+        <f>J742-L742</f>
+        <v/>
+      </c>
+      <c r="N742" s="18">
+        <f>IF(J742=0,"",L742/J742)</f>
+        <v/>
+      </c>
+      <c r="O742" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:13</t>
+        </is>
+      </c>
+      <c r="B743" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C743" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D743" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E743" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F743" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G743" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H743" s="16" t="n">
+        <v>1.0432</v>
+      </c>
+      <c r="I743" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J743" s="17" t="n">
+        <v>270023.1136243431</v>
+      </c>
+      <c r="K743" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,041.5307</t>
+        </is>
+      </c>
+      <c r="L743" s="17" t="n">
+        <v>232964.6269618799</v>
+      </c>
+      <c r="M743" s="17">
+        <f>J743-L743</f>
+        <v/>
+      </c>
+      <c r="N743" s="18">
+        <f>IF(J743=0,"",L743/J743)</f>
+        <v/>
+      </c>
+      <c r="O743" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:13</t>
+        </is>
+      </c>
+      <c r="B744" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C744" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D744" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E744" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F744" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G744" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H744" s="16" t="inlineStr"/>
+      <c r="I744" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,511.8192</t>
+        </is>
+      </c>
+      <c r="J744" s="17" t="n">
+        <v>15506.70032579926</v>
+      </c>
+      <c r="K744" s="15" t="inlineStr"/>
+      <c r="L744" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M744" s="17">
+        <f>J744-L744</f>
+        <v/>
+      </c>
+      <c r="N744" s="18">
+        <f>IF(J744=0,"",L744/J744)</f>
+        <v/>
+      </c>
+      <c r="O744" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:13</t>
+        </is>
+      </c>
+      <c r="B745" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C745" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D745" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E745" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F745" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G745" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H745" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I745" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J745" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K745" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L745" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M745" s="17">
+        <f>J745-L745</f>
+        <v/>
+      </c>
+      <c r="N745" s="18">
+        <f>IF(J745=0,"",L745/J745)</f>
+        <v/>
+      </c>
+      <c r="O745" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:13</t>
+        </is>
+      </c>
+      <c r="B746" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C746" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D746" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E746" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F746" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G746" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H746" s="16" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="I746" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J746" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K746" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,705.3454</t>
+        </is>
+      </c>
+      <c r="L746" s="17" t="n">
+        <v>148705.345409</v>
+      </c>
+      <c r="M746" s="17">
+        <f>J746-L746</f>
+        <v/>
+      </c>
+      <c r="N746" s="18">
+        <f>IF(J746=0,"",L746/J746)</f>
+        <v/>
+      </c>
+      <c r="O746" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:53</t>
+        </is>
+      </c>
+      <c r="B747" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C747" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D747" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E747" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F747" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G747" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H747" s="16" t="n">
+        <v>1.0505</v>
+      </c>
+      <c r="I747" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,804.5477</t>
+        </is>
+      </c>
+      <c r="J747" s="17" t="n">
+        <v>50787.78216227121</v>
+      </c>
+      <c r="K747" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,722.8797</t>
+        </is>
+      </c>
+      <c r="L747" s="17" t="n">
+        <v>37722.87969</v>
+      </c>
+      <c r="M747" s="17">
+        <f>J747-L747</f>
+        <v/>
+      </c>
+      <c r="N747" s="18">
+        <f>IF(J747=0,"",L747/J747)</f>
+        <v/>
+      </c>
+      <c r="O747" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:53</t>
+        </is>
+      </c>
+      <c r="B748" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C748" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D748" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E748" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F748" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G748" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H748" s="16" t="n">
+        <v>1.048</v>
+      </c>
+      <c r="I748" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J748" s="17" t="n">
+        <v>140898.0193427771</v>
+      </c>
+      <c r="K748" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,035.0439</t>
+        </is>
+      </c>
+      <c r="L748" s="17" t="n">
+        <v>120995.1023625041</v>
+      </c>
+      <c r="M748" s="17">
+        <f>J748-L748</f>
+        <v/>
+      </c>
+      <c r="N748" s="18">
+        <f>IF(J748=0,"",L748/J748)</f>
+        <v/>
+      </c>
+      <c r="O748" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:53</t>
+        </is>
+      </c>
+      <c r="B749" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C749" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D749" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E749" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F749" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G749" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H749" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I749" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J749" s="17" t="n">
+        <v>328717.7033096657</v>
+      </c>
+      <c r="K749" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,386.0522</t>
+        </is>
+      </c>
+      <c r="L749" s="17" t="n">
+        <v>306411.398624031</v>
+      </c>
+      <c r="M749" s="17">
+        <f>J749-L749</f>
+        <v/>
+      </c>
+      <c r="N749" s="18">
+        <f>IF(J749=0,"",L749/J749)</f>
+        <v/>
+      </c>
+      <c r="O749" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:53</t>
+        </is>
+      </c>
+      <c r="B750" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C750" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D750" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E750" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F750" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G750" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H750" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I750" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J750" s="17" t="n">
+        <v>386025.5466608055</v>
+      </c>
+      <c r="K750" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,608.2120</t>
+        </is>
+      </c>
+      <c r="L750" s="17" t="n">
+        <v>349637.1340803551</v>
+      </c>
+      <c r="M750" s="17">
+        <f>J750-L750</f>
+        <v/>
+      </c>
+      <c r="N750" s="18">
+        <f>IF(J750=0,"",L750/J750)</f>
+        <v/>
+      </c>
+      <c r="O750" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:53</t>
+        </is>
+      </c>
+      <c r="B751" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C751" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D751" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E751" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F751" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G751" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H751" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I751" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7848</t>
+        </is>
+      </c>
+      <c r="J751" s="17" t="n">
+        <v>77789.04359875197</v>
+      </c>
+      <c r="K751" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,028.1988; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L751" s="17" t="n">
+        <v>68005.82710337982</v>
+      </c>
+      <c r="M751" s="17">
+        <f>J751-L751</f>
+        <v/>
+      </c>
+      <c r="N751" s="18">
+        <f>IF(J751=0,"",L751/J751)</f>
+        <v/>
+      </c>
+      <c r="O751" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:53</t>
+        </is>
+      </c>
+      <c r="B752" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C752" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D752" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E752" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F752" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G752" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H752" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I752" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J752" s="17" t="n">
+        <v>197082.5406068833</v>
+      </c>
+      <c r="K752" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,243.9962</t>
+        </is>
+      </c>
+      <c r="L752" s="17" t="n">
+        <v>150243.996246735</v>
+      </c>
+      <c r="M752" s="17">
+        <f>J752-L752</f>
+        <v/>
+      </c>
+      <c r="N752" s="18">
+        <f>IF(J752=0,"",L752/J752)</f>
+        <v/>
+      </c>
+      <c r="O752" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:53</t>
+        </is>
+      </c>
+      <c r="B753" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C753" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D753" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E753" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F753" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G753" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H753" s="16" t="n">
+        <v>1.3726</v>
+      </c>
+      <c r="I753" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J753" s="17" t="n">
+        <v>186091.8444123784</v>
+      </c>
+      <c r="K753" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,140.3351</t>
+        </is>
+      </c>
+      <c r="L753" s="17" t="n">
+        <v>124140.3351430682</v>
+      </c>
+      <c r="M753" s="17">
+        <f>J753-L753</f>
+        <v/>
+      </c>
+      <c r="N753" s="18">
+        <f>IF(J753=0,"",L753/J753)</f>
+        <v/>
+      </c>
+      <c r="O753" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:53</t>
+        </is>
+      </c>
+      <c r="B754" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C754" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D754" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E754" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F754" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G754" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H754" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I754" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J754" s="17" t="n">
+        <v>327605.5893985275</v>
+      </c>
+      <c r="K754" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L754" s="17" t="n">
+        <v>280238.4852792478</v>
+      </c>
+      <c r="M754" s="17">
+        <f>J754-L754</f>
+        <v/>
+      </c>
+      <c r="N754" s="18">
+        <f>IF(J754=0,"",L754/J754)</f>
+        <v/>
+      </c>
+      <c r="O754" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:53</t>
+        </is>
+      </c>
+      <c r="B755" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C755" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D755" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E755" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F755" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G755" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H755" s="16" t="n">
+        <v>1.9045</v>
+      </c>
+      <c r="I755" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J755" s="17" t="n">
+        <v>159989.8916291629</v>
+      </c>
+      <c r="K755" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,938.3760</t>
+        </is>
+      </c>
+      <c r="L755" s="17" t="n">
+        <v>70938.37599253547</v>
+      </c>
+      <c r="M755" s="17">
+        <f>J755-L755</f>
+        <v/>
+      </c>
+      <c r="N755" s="18">
+        <f>IF(J755=0,"",L755/J755)</f>
+        <v/>
+      </c>
+      <c r="O755" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:53</t>
+        </is>
+      </c>
+      <c r="B756" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C756" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D756" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E756" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F756" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G756" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H756" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I756" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J756" s="17" t="n">
+        <v>160151.5537382347</v>
+      </c>
+      <c r="K756" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,523.0271</t>
+        </is>
+      </c>
+      <c r="L756" s="17" t="n">
+        <v>138509.1747529419</v>
+      </c>
+      <c r="M756" s="17">
+        <f>J756-L756</f>
+        <v/>
+      </c>
+      <c r="N756" s="18">
+        <f>IF(J756=0,"",L756/J756)</f>
+        <v/>
+      </c>
+      <c r="O756" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:53</t>
+        </is>
+      </c>
+      <c r="B757" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C757" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D757" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E757" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F757" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G757" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H757" s="16" t="inlineStr"/>
+      <c r="I757" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J757" s="17" t="n">
+        <v>95887.44131056532</v>
+      </c>
+      <c r="K757" s="15" t="inlineStr"/>
+      <c r="L757" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M757" s="17">
+        <f>J757-L757</f>
+        <v/>
+      </c>
+      <c r="N757" s="18">
+        <f>IF(J757=0,"",L757/J757)</f>
+        <v/>
+      </c>
+      <c r="O757" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:53</t>
+        </is>
+      </c>
+      <c r="B758" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C758" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D758" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E758" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F758" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G758" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H758" s="16" t="inlineStr"/>
+      <c r="I758" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J758" s="17" t="n">
+        <v>34357.63649597362</v>
+      </c>
+      <c r="K758" s="15" t="inlineStr"/>
+      <c r="L758" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M758" s="17">
+        <f>J758-L758</f>
+        <v/>
+      </c>
+      <c r="N758" s="18">
+        <f>IF(J758=0,"",L758/J758)</f>
+        <v/>
+      </c>
+      <c r="O758" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:53</t>
+        </is>
+      </c>
+      <c r="B759" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C759" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D759" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E759" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F759" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G759" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H759" s="16" t="n">
+        <v>1.0432</v>
+      </c>
+      <c r="I759" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J759" s="17" t="n">
+        <v>270023.1136243431</v>
+      </c>
+      <c r="K759" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,041.5307</t>
+        </is>
+      </c>
+      <c r="L759" s="17" t="n">
+        <v>232964.6269618799</v>
+      </c>
+      <c r="M759" s="17">
+        <f>J759-L759</f>
+        <v/>
+      </c>
+      <c r="N759" s="18">
+        <f>IF(J759=0,"",L759/J759)</f>
+        <v/>
+      </c>
+      <c r="O759" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:53</t>
+        </is>
+      </c>
+      <c r="B760" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C760" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D760" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E760" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F760" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G760" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H760" s="16" t="inlineStr"/>
+      <c r="I760" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,511.8192</t>
+        </is>
+      </c>
+      <c r="J760" s="17" t="n">
+        <v>15506.70032579926</v>
+      </c>
+      <c r="K760" s="15" t="inlineStr"/>
+      <c r="L760" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M760" s="17">
+        <f>J760-L760</f>
+        <v/>
+      </c>
+      <c r="N760" s="18">
+        <f>IF(J760=0,"",L760/J760)</f>
+        <v/>
+      </c>
+      <c r="O760" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:53</t>
+        </is>
+      </c>
+      <c r="B761" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C761" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D761" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E761" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F761" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G761" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H761" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I761" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J761" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K761" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L761" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M761" s="17">
+        <f>J761-L761</f>
+        <v/>
+      </c>
+      <c r="N761" s="18">
+        <f>IF(J761=0,"",L761/J761)</f>
+        <v/>
+      </c>
+      <c r="O761" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:53</t>
+        </is>
+      </c>
+      <c r="B762" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C762" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D762" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E762" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F762" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G762" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H762" s="16" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="I762" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J762" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K762" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,705.3454</t>
+        </is>
+      </c>
+      <c r="L762" s="17" t="n">
+        <v>148705.345409</v>
+      </c>
+      <c r="M762" s="17">
+        <f>J762-L762</f>
+        <v/>
+      </c>
+      <c r="N762" s="18">
+        <f>IF(J762=0,"",L762/J762)</f>
+        <v/>
+      </c>
+      <c r="O762" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:17:02</t>
+        </is>
+      </c>
+      <c r="B763" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C763" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D763" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E763" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F763" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G763" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H763" s="16" t="n">
+        <v>1.0505</v>
+      </c>
+      <c r="I763" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,804.5477</t>
+        </is>
+      </c>
+      <c r="J763" s="17" t="n">
+        <v>50790.32238965436</v>
+      </c>
+      <c r="K763" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,722.8797</t>
+        </is>
+      </c>
+      <c r="L763" s="17" t="n">
+        <v>37726.65235523552</v>
+      </c>
+      <c r="M763" s="17">
+        <f>J763-L763</f>
+        <v/>
+      </c>
+      <c r="N763" s="18">
+        <f>IF(J763=0,"",L763/J763)</f>
+        <v/>
+      </c>
+      <c r="O763" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:17:02</t>
+        </is>
+      </c>
+      <c r="B764" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C764" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D764" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E764" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F764" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G764" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H764" s="16" t="n">
+        <v>1.048</v>
+      </c>
+      <c r="I764" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J764" s="17" t="n">
+        <v>140898.0193427771</v>
+      </c>
+      <c r="K764" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,035.0439</t>
+        </is>
+      </c>
+      <c r="L764" s="17" t="n">
+        <v>121001.1541147004</v>
+      </c>
+      <c r="M764" s="17">
+        <f>J764-L764</f>
+        <v/>
+      </c>
+      <c r="N764" s="18">
+        <f>IF(J764=0,"",L764/J764)</f>
+        <v/>
+      </c>
+      <c r="O764" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:17:02</t>
+        </is>
+      </c>
+      <c r="B765" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C765" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D765" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E765" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F765" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G765" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H765" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I765" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J765" s="17" t="n">
+        <v>328718.7800499076</v>
+      </c>
+      <c r="K765" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,386.0522</t>
+        </is>
+      </c>
+      <c r="L765" s="17" t="n">
+        <v>306411.398624031</v>
+      </c>
+      <c r="M765" s="17">
+        <f>J765-L765</f>
+        <v/>
+      </c>
+      <c r="N765" s="18">
+        <f>IF(J765=0,"",L765/J765)</f>
+        <v/>
+      </c>
+      <c r="O765" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:17:02</t>
+        </is>
+      </c>
+      <c r="B766" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C766" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D766" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E766" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F766" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G766" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H766" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I766" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J766" s="17" t="n">
+        <v>386025.5466608055</v>
+      </c>
+      <c r="K766" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,608.2120</t>
+        </is>
+      </c>
+      <c r="L766" s="17" t="n">
+        <v>349637.1340803551</v>
+      </c>
+      <c r="M766" s="17">
+        <f>J766-L766</f>
+        <v/>
+      </c>
+      <c r="N766" s="18">
+        <f>IF(J766=0,"",L766/J766)</f>
+        <v/>
+      </c>
+      <c r="O766" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:17:02</t>
+        </is>
+      </c>
+      <c r="B767" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C767" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D767" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E767" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F767" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G767" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H767" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I767" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7848</t>
+        </is>
+      </c>
+      <c r="J767" s="17" t="n">
+        <v>77789.02724174902</v>
+      </c>
+      <c r="K767" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,028.1988; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L767" s="17" t="n">
+        <v>68009.22852107904</v>
+      </c>
+      <c r="M767" s="17">
+        <f>J767-L767</f>
+        <v/>
+      </c>
+      <c r="N767" s="18">
+        <f>IF(J767=0,"",L767/J767)</f>
+        <v/>
+      </c>
+      <c r="O767" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:17:02</t>
+        </is>
+      </c>
+      <c r="B768" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C768" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D768" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E768" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F768" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G768" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H768" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I768" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J768" s="17" t="n">
+        <v>197082.5406068833</v>
+      </c>
+      <c r="K768" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,243.9962</t>
+        </is>
+      </c>
+      <c r="L768" s="17" t="n">
+        <v>150259.0221489499</v>
+      </c>
+      <c r="M768" s="17">
+        <f>J768-L768</f>
+        <v/>
+      </c>
+      <c r="N768" s="18">
+        <f>IF(J768=0,"",L768/J768)</f>
+        <v/>
+      </c>
+      <c r="O768" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:17:02</t>
+        </is>
+      </c>
+      <c r="B769" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C769" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D769" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E769" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F769" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G769" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H769" s="16" t="n">
+        <v>1.3726</v>
+      </c>
+      <c r="I769" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J769" s="17" t="n">
+        <v>186091.8444123784</v>
+      </c>
+      <c r="K769" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,140.3351</t>
+        </is>
+      </c>
+      <c r="L769" s="17" t="n">
+        <v>124152.75041811</v>
+      </c>
+      <c r="M769" s="17">
+        <f>J769-L769</f>
+        <v/>
+      </c>
+      <c r="N769" s="18">
+        <f>IF(J769=0,"",L769/J769)</f>
+        <v/>
+      </c>
+      <c r="O769" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:17:02</t>
+        </is>
+      </c>
+      <c r="B770" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C770" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D770" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E770" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F770" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G770" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H770" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I770" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J770" s="17" t="n">
+        <v>327605.5893985275</v>
+      </c>
+      <c r="K770" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L770" s="17" t="n">
+        <v>280238.4852792478</v>
+      </c>
+      <c r="M770" s="17">
+        <f>J770-L770</f>
+        <v/>
+      </c>
+      <c r="N770" s="18">
+        <f>IF(J770=0,"",L770/J770)</f>
+        <v/>
+      </c>
+      <c r="O770" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:17:02</t>
+        </is>
+      </c>
+      <c r="B771" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C771" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D771" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E771" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F771" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G771" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H771" s="16" t="n">
+        <v>1.9045</v>
+      </c>
+      <c r="I771" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J771" s="17" t="n">
+        <v>159989.8916291629</v>
+      </c>
+      <c r="K771" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,938.3760</t>
+        </is>
+      </c>
+      <c r="L771" s="17" t="n">
+        <v>70945.47053958943</v>
+      </c>
+      <c r="M771" s="17">
+        <f>J771-L771</f>
+        <v/>
+      </c>
+      <c r="N771" s="18">
+        <f>IF(J771=0,"",L771/J771)</f>
+        <v/>
+      </c>
+      <c r="O771" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:17:02</t>
+        </is>
+      </c>
+      <c r="B772" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C772" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D772" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E772" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F772" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G772" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H772" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I772" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J772" s="17" t="n">
+        <v>160151.5537382347</v>
+      </c>
+      <c r="K772" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,523.0271</t>
+        </is>
+      </c>
+      <c r="L772" s="17" t="n">
+        <v>138509.1747529419</v>
+      </c>
+      <c r="M772" s="17">
+        <f>J772-L772</f>
+        <v/>
+      </c>
+      <c r="N772" s="18">
+        <f>IF(J772=0,"",L772/J772)</f>
+        <v/>
+      </c>
+      <c r="O772" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:17:02</t>
+        </is>
+      </c>
+      <c r="B773" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C773" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D773" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E773" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F773" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G773" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H773" s="16" t="inlineStr"/>
+      <c r="I773" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J773" s="17" t="n">
+        <v>95887.44131056532</v>
+      </c>
+      <c r="K773" s="15" t="inlineStr"/>
+      <c r="L773" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M773" s="17">
+        <f>J773-L773</f>
+        <v/>
+      </c>
+      <c r="N773" s="18">
+        <f>IF(J773=0,"",L773/J773)</f>
+        <v/>
+      </c>
+      <c r="O773" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:17:02</t>
+        </is>
+      </c>
+      <c r="B774" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C774" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D774" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E774" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F774" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G774" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H774" s="16" t="inlineStr"/>
+      <c r="I774" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J774" s="17" t="n">
+        <v>34357.63649597362</v>
+      </c>
+      <c r="K774" s="15" t="inlineStr"/>
+      <c r="L774" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M774" s="17">
+        <f>J774-L774</f>
+        <v/>
+      </c>
+      <c r="N774" s="18">
+        <f>IF(J774=0,"",L774/J774)</f>
+        <v/>
+      </c>
+      <c r="O774" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:17:02</t>
+        </is>
+      </c>
+      <c r="B775" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C775" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D775" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E775" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F775" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G775" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H775" s="16" t="n">
+        <v>1.0431</v>
+      </c>
+      <c r="I775" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J775" s="17" t="n">
+        <v>270023.1136243431</v>
+      </c>
+      <c r="K775" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,041.5307</t>
+        </is>
+      </c>
+      <c r="L775" s="17" t="n">
+        <v>232976.2790384133</v>
+      </c>
+      <c r="M775" s="17">
+        <f>J775-L775</f>
+        <v/>
+      </c>
+      <c r="N775" s="18">
+        <f>IF(J775=0,"",L775/J775)</f>
+        <v/>
+      </c>
+      <c r="O775" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:17:02</t>
+        </is>
+      </c>
+      <c r="B776" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C776" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D776" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E776" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F776" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G776" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H776" s="16" t="inlineStr"/>
+      <c r="I776" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,511.8192</t>
+        </is>
+      </c>
+      <c r="J776" s="17" t="n">
+        <v>15507.47591676057</v>
+      </c>
+      <c r="K776" s="15" t="inlineStr"/>
+      <c r="L776" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M776" s="17">
+        <f>J776-L776</f>
+        <v/>
+      </c>
+      <c r="N776" s="18">
+        <f>IF(J776=0,"",L776/J776)</f>
+        <v/>
+      </c>
+      <c r="O776" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:17:02</t>
+        </is>
+      </c>
+      <c r="B777" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C777" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D777" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E777" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F777" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G777" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H777" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I777" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J777" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K777" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L777" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M777" s="17">
+        <f>J777-L777</f>
+        <v/>
+      </c>
+      <c r="N777" s="18">
+        <f>IF(J777=0,"",L777/J777)</f>
+        <v/>
+      </c>
+      <c r="O777" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:17:02</t>
+        </is>
+      </c>
+      <c r="B778" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C778" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D778" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E778" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F778" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G778" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H778" s="16" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="I778" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J778" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K778" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,705.3454</t>
+        </is>
+      </c>
+      <c r="L778" s="17" t="n">
+        <v>148705.345409</v>
+      </c>
+      <c r="M778" s="17">
+        <f>J778-L778</f>
+        <v/>
+      </c>
+      <c r="N778" s="18">
+        <f>IF(J778=0,"",L778/J778)</f>
+        <v/>
+      </c>
+      <c r="O778" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -49612,7 +52870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -51343,6 +54601,111 @@
         <v>1.0375</v>
       </c>
       <c r="I49" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:13</t>
+        </is>
+      </c>
+      <c r="B50" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C50" s="17" t="n">
+        <v>655514.1392568687</v>
+      </c>
+      <c r="D50" s="17" t="n">
+        <v>652902.5544678983</v>
+      </c>
+      <c r="E50" s="17" t="n">
+        <v>2933397.783217576</v>
+      </c>
+      <c r="F50" s="17" t="n">
+        <v>2280495.228749678</v>
+      </c>
+      <c r="G50" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H50" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I50" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:14:53</t>
+        </is>
+      </c>
+      <c r="B51" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C51" s="17" t="n">
+        <v>655513.7672708778</v>
+      </c>
+      <c r="D51" s="17" t="n">
+        <v>652902.5584574114</v>
+      </c>
+      <c r="E51" s="17" t="n">
+        <v>2933397.787207089</v>
+      </c>
+      <c r="F51" s="17" t="n">
+        <v>2280495.228749678</v>
+      </c>
+      <c r="G51" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H51" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I51" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:17:02</t>
+        </is>
+      </c>
+      <c r="B52" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C52" s="17" t="n">
+        <v>655458.5996055903</v>
+      </c>
+      <c r="D52" s="17" t="n">
+        <v>652847.5210230192</v>
+      </c>
+      <c r="E52" s="17" t="n">
+        <v>2933402.163408672</v>
+      </c>
+      <c r="F52" s="17" t="n">
+        <v>2280554.642385653</v>
+      </c>
+      <c r="G52" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H52" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I52" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 15:47 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O778"/>
+  <dimension ref="A1:O794"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -52840,6 +52840,1092 @@
         <v/>
       </c>
       <c r="O778" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:47:18</t>
+        </is>
+      </c>
+      <c r="B779" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C779" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D779" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E779" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F779" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G779" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H779" s="16" t="n">
+        <v>1.0505</v>
+      </c>
+      <c r="I779" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,804.5477</t>
+        </is>
+      </c>
+      <c r="J779" s="17" t="n">
+        <v>50788.79825322446</v>
+      </c>
+      <c r="K779" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,722.8797</t>
+        </is>
+      </c>
+      <c r="L779" s="17" t="n">
+        <v>37726.65235523552</v>
+      </c>
+      <c r="M779" s="17">
+        <f>J779-L779</f>
+        <v/>
+      </c>
+      <c r="N779" s="18">
+        <f>IF(J779=0,"",L779/J779)</f>
+        <v/>
+      </c>
+      <c r="O779" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:47:18</t>
+        </is>
+      </c>
+      <c r="B780" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C780" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D780" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E780" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F780" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G780" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H780" s="16" t="n">
+        <v>1.048</v>
+      </c>
+      <c r="I780" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J780" s="17" t="n">
+        <v>140898.4410692982</v>
+      </c>
+      <c r="K780" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,035.0439</t>
+        </is>
+      </c>
+      <c r="L780" s="17" t="n">
+        <v>120997.5230633826</v>
+      </c>
+      <c r="M780" s="17">
+        <f>J780-L780</f>
+        <v/>
+      </c>
+      <c r="N780" s="18">
+        <f>IF(J780=0,"",L780/J780)</f>
+        <v/>
+      </c>
+      <c r="O780" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:47:18</t>
+        </is>
+      </c>
+      <c r="B781" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C781" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D781" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E781" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F781" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G781" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H781" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I781" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J781" s="17" t="n">
+        <v>328719.0145404724</v>
+      </c>
+      <c r="K781" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,386.0522</t>
+        </is>
+      </c>
+      <c r="L781" s="17" t="n">
+        <v>306422.5021989321</v>
+      </c>
+      <c r="M781" s="17">
+        <f>J781-L781</f>
+        <v/>
+      </c>
+      <c r="N781" s="18">
+        <f>IF(J781=0,"",L781/J781)</f>
+        <v/>
+      </c>
+      <c r="O781" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:47:18</t>
+        </is>
+      </c>
+      <c r="B782" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C782" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D782" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E782" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F782" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G782" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H782" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I782" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J782" s="17" t="n">
+        <v>386026.7019463226</v>
+      </c>
+      <c r="K782" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,608.2120</t>
+        </is>
+      </c>
+      <c r="L782" s="17" t="n">
+        <v>349649.804046694</v>
+      </c>
+      <c r="M782" s="17">
+        <f>J782-L782</f>
+        <v/>
+      </c>
+      <c r="N782" s="18">
+        <f>IF(J782=0,"",L782/J782)</f>
+        <v/>
+      </c>
+      <c r="O782" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:47:18</t>
+        </is>
+      </c>
+      <c r="B783" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C783" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D783" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E783" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F783" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G783" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H783" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I783" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7848</t>
+        </is>
+      </c>
+      <c r="J783" s="17" t="n">
+        <v>77790.49635209121</v>
+      </c>
+      <c r="K783" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,028.1988; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L783" s="17" t="n">
+        <v>68007.18767511357</v>
+      </c>
+      <c r="M783" s="17">
+        <f>J783-L783</f>
+        <v/>
+      </c>
+      <c r="N783" s="18">
+        <f>IF(J783=0,"",L783/J783)</f>
+        <v/>
+      </c>
+      <c r="O783" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:47:18</t>
+        </is>
+      </c>
+      <c r="B784" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C784" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D784" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E784" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F784" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G784" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H784" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I784" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J784" s="17" t="n">
+        <v>197072.5241909334</v>
+      </c>
+      <c r="K784" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,243.9962</t>
+        </is>
+      </c>
+      <c r="L784" s="17" t="n">
+        <v>150259.0221489499</v>
+      </c>
+      <c r="M784" s="17">
+        <f>J784-L784</f>
+        <v/>
+      </c>
+      <c r="N784" s="18">
+        <f>IF(J784=0,"",L784/J784)</f>
+        <v/>
+      </c>
+      <c r="O784" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:47:18</t>
+        </is>
+      </c>
+      <c r="B785" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C785" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D785" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E785" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F785" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G785" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H785" s="16" t="n">
+        <v>1.3726</v>
+      </c>
+      <c r="I785" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J785" s="17" t="n">
+        <v>186092.7585460069</v>
+      </c>
+      <c r="K785" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,140.3351</t>
+        </is>
+      </c>
+      <c r="L785" s="17" t="n">
+        <v>124152.75041811</v>
+      </c>
+      <c r="M785" s="17">
+        <f>J785-L785</f>
+        <v/>
+      </c>
+      <c r="N785" s="18">
+        <f>IF(J785=0,"",L785/J785)</f>
+        <v/>
+      </c>
+      <c r="O785" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:47:18</t>
+        </is>
+      </c>
+      <c r="B786" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C786" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D786" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E786" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F786" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G786" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H786" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I786" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J786" s="17" t="n">
+        <v>327611.5239423555</v>
+      </c>
+      <c r="K786" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L786" s="17" t="n">
+        <v>280269.5917898174</v>
+      </c>
+      <c r="M786" s="17">
+        <f>J786-L786</f>
+        <v/>
+      </c>
+      <c r="N786" s="18">
+        <f>IF(J786=0,"",L786/J786)</f>
+        <v/>
+      </c>
+      <c r="O786" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:47:18</t>
+        </is>
+      </c>
+      <c r="B787" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C787" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D787" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E787" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F787" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G787" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H787" s="16" t="n">
+        <v>1.9045</v>
+      </c>
+      <c r="I787" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J787" s="17" t="n">
+        <v>159989.8916291629</v>
+      </c>
+      <c r="K787" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,938.3760</t>
+        </is>
+      </c>
+      <c r="L787" s="17" t="n">
+        <v>70945.47053958943</v>
+      </c>
+      <c r="M787" s="17">
+        <f>J787-L787</f>
+        <v/>
+      </c>
+      <c r="N787" s="18">
+        <f>IF(J787=0,"",L787/J787)</f>
+        <v/>
+      </c>
+      <c r="O787" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:47:18</t>
+        </is>
+      </c>
+      <c r="B788" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C788" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D788" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E788" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F788" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G788" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H788" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I788" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J788" s="17" t="n">
+        <v>160152.0330349345</v>
+      </c>
+      <c r="K788" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,523.0271</t>
+        </is>
+      </c>
+      <c r="L788" s="17" t="n">
+        <v>138495.3224502363</v>
+      </c>
+      <c r="M788" s="17">
+        <f>J788-L788</f>
+        <v/>
+      </c>
+      <c r="N788" s="18">
+        <f>IF(J788=0,"",L788/J788)</f>
+        <v/>
+      </c>
+      <c r="O788" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:47:18</t>
+        </is>
+      </c>
+      <c r="B789" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C789" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D789" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E789" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F789" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G789" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H789" s="16" t="inlineStr"/>
+      <c r="I789" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J789" s="17" t="n">
+        <v>95897.03101366668</v>
+      </c>
+      <c r="K789" s="15" t="inlineStr"/>
+      <c r="L789" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M789" s="17">
+        <f>J789-L789</f>
+        <v/>
+      </c>
+      <c r="N789" s="18">
+        <f>IF(J789=0,"",L789/J789)</f>
+        <v/>
+      </c>
+      <c r="O789" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:47:18</t>
+        </is>
+      </c>
+      <c r="B790" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C790" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D790" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E790" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F790" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G790" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H790" s="16" t="inlineStr"/>
+      <c r="I790" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J790" s="17" t="n">
+        <v>34357.97295558875</v>
+      </c>
+      <c r="K790" s="15" t="inlineStr"/>
+      <c r="L790" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M790" s="17">
+        <f>J790-L790</f>
+        <v/>
+      </c>
+      <c r="N790" s="18">
+        <f>IF(J790=0,"",L790/J790)</f>
+        <v/>
+      </c>
+      <c r="O790" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:47:18</t>
+        </is>
+      </c>
+      <c r="B791" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C791" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D791" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E791" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F791" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G791" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H791" s="16" t="n">
+        <v>1.0431</v>
+      </c>
+      <c r="I791" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J791" s="17" t="n">
+        <v>270023.1136243431</v>
+      </c>
+      <c r="K791" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,041.5307</t>
+        </is>
+      </c>
+      <c r="L791" s="17" t="n">
+        <v>232969.2877924932</v>
+      </c>
+      <c r="M791" s="17">
+        <f>J791-L791</f>
+        <v/>
+      </c>
+      <c r="N791" s="18">
+        <f>IF(J791=0,"",L791/J791)</f>
+        <v/>
+      </c>
+      <c r="O791" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:47:18</t>
+        </is>
+      </c>
+      <c r="B792" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C792" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D792" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E792" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F792" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G792" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H792" s="16" t="inlineStr"/>
+      <c r="I792" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,512.0184</t>
+        </is>
+      </c>
+      <c r="J792" s="17" t="n">
+        <v>15507.20972254038</v>
+      </c>
+      <c r="K792" s="15" t="inlineStr"/>
+      <c r="L792" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M792" s="17">
+        <f>J792-L792</f>
+        <v/>
+      </c>
+      <c r="N792" s="18">
+        <f>IF(J792=0,"",L792/J792)</f>
+        <v/>
+      </c>
+      <c r="O792" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:47:18</t>
+        </is>
+      </c>
+      <c r="B793" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C793" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D793" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E793" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F793" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G793" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H793" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I793" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J793" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K793" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L793" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M793" s="17">
+        <f>J793-L793</f>
+        <v/>
+      </c>
+      <c r="N793" s="18">
+        <f>IF(J793=0,"",L793/J793)</f>
+        <v/>
+      </c>
+      <c r="O793" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:47:18</t>
+        </is>
+      </c>
+      <c r="B794" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C794" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D794" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E794" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F794" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G794" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H794" s="16" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="I794" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J794" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K794" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,705.3454</t>
+        </is>
+      </c>
+      <c r="L794" s="17" t="n">
+        <v>148705.345409</v>
+      </c>
+      <c r="M794" s="17">
+        <f>J794-L794</f>
+        <v/>
+      </c>
+      <c r="N794" s="18">
+        <f>IF(J794=0,"",L794/J794)</f>
+        <v/>
+      </c>
+      <c r="O794" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -52870,7 +53956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I52"/>
+  <dimension ref="A1:I53"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -54706,6 +55792,41 @@
         <v>1.0375</v>
       </c>
       <c r="I52" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:47:18</t>
+        </is>
+      </c>
+      <c r="B53" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C53" s="17" t="n">
+        <v>655437.5790621088</v>
+      </c>
+      <c r="D53" s="17" t="n">
+        <v>652827.8844203367</v>
+      </c>
+      <c r="E53" s="17" t="n">
+        <v>2933410.891411891</v>
+      </c>
+      <c r="F53" s="17" t="n">
+        <v>2280583.006991554</v>
+      </c>
+      <c r="G53" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H53" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I53" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 16:17 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O794"/>
+  <dimension ref="A1:O810"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -53926,6 +53926,1092 @@
         <v/>
       </c>
       <c r="O794" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:17:34</t>
+        </is>
+      </c>
+      <c r="B795" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C795" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D795" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E795" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F795" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G795" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H795" s="16" t="n">
+        <v>1.0505</v>
+      </c>
+      <c r="I795" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,804.5477</t>
+        </is>
+      </c>
+      <c r="J795" s="17" t="n">
+        <v>50795.40284442066</v>
+      </c>
+      <c r="K795" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,722.8797</t>
+        </is>
+      </c>
+      <c r="L795" s="17" t="n">
+        <v>37726.65235523552</v>
+      </c>
+      <c r="M795" s="17">
+        <f>J795-L795</f>
+        <v/>
+      </c>
+      <c r="N795" s="18">
+        <f>IF(J795=0,"",L795/J795)</f>
+        <v/>
+      </c>
+      <c r="O795" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:17:34</t>
+        </is>
+      </c>
+      <c r="B796" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C796" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D796" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E796" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F796" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G796" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H796" s="16" t="n">
+        <v>1.0479</v>
+      </c>
+      <c r="I796" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J796" s="17" t="n">
+        <v>140897.9017299798</v>
+      </c>
+      <c r="K796" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,035.0439</t>
+        </is>
+      </c>
+      <c r="L796" s="17" t="n">
+        <v>121013.2576190932</v>
+      </c>
+      <c r="M796" s="17">
+        <f>J796-L796</f>
+        <v/>
+      </c>
+      <c r="N796" s="18">
+        <f>IF(J796=0,"",L796/J796)</f>
+        <v/>
+      </c>
+      <c r="O796" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:17:34</t>
+        </is>
+      </c>
+      <c r="B797" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C797" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D797" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E797" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F797" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G797" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H797" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I797" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J797" s="17" t="n">
+        <v>328719.1581062069</v>
+      </c>
+      <c r="K797" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,386.0522</t>
+        </is>
+      </c>
+      <c r="L797" s="17" t="n">
+        <v>306426.4094105235</v>
+      </c>
+      <c r="M797" s="17">
+        <f>J797-L797</f>
+        <v/>
+      </c>
+      <c r="N797" s="18">
+        <f>IF(J797=0,"",L797/J797)</f>
+        <v/>
+      </c>
+      <c r="O797" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:17:34</t>
+        </is>
+      </c>
+      <c r="B798" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C798" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D798" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E798" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F798" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G798" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H798" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I798" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J798" s="17" t="n">
+        <v>386027.0947090316</v>
+      </c>
+      <c r="K798" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,608.2120</t>
+        </is>
+      </c>
+      <c r="L798" s="17" t="n">
+        <v>349654.2624521882</v>
+      </c>
+      <c r="M798" s="17">
+        <f>J798-L798</f>
+        <v/>
+      </c>
+      <c r="N798" s="18">
+        <f>IF(J798=0,"",L798/J798)</f>
+        <v/>
+      </c>
+      <c r="O798" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:17:34</t>
+        </is>
+      </c>
+      <c r="B799" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C799" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D799" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E799" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F799" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G799" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H799" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I799" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7848</t>
+        </is>
+      </c>
+      <c r="J799" s="17" t="n">
+        <v>77801.41283534076</v>
+      </c>
+      <c r="K799" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,028.1988; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L799" s="17" t="n">
+        <v>68016.03134096395</v>
+      </c>
+      <c r="M799" s="17">
+        <f>J799-L799</f>
+        <v/>
+      </c>
+      <c r="N799" s="18">
+        <f>IF(J799=0,"",L799/J799)</f>
+        <v/>
+      </c>
+      <c r="O799" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:17:34</t>
+        </is>
+      </c>
+      <c r="B800" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C800" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D800" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E800" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F800" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G800" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H800" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I800" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J800" s="17" t="n">
+        <v>197080.1805880253</v>
+      </c>
+      <c r="K800" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,243.9962</t>
+        </is>
+      </c>
+      <c r="L800" s="17" t="n">
+        <v>150259.0221489499</v>
+      </c>
+      <c r="M800" s="17">
+        <f>J800-L800</f>
+        <v/>
+      </c>
+      <c r="N800" s="18">
+        <f>IF(J800=0,"",L800/J800)</f>
+        <v/>
+      </c>
+      <c r="O800" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:17:34</t>
+        </is>
+      </c>
+      <c r="B801" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C801" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D801" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E801" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F801" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G801" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H801" s="16" t="n">
+        <v>1.3726</v>
+      </c>
+      <c r="I801" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J801" s="17" t="n">
+        <v>186068.1147578933</v>
+      </c>
+      <c r="K801" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,140.3351</t>
+        </is>
+      </c>
+      <c r="L801" s="17" t="n">
+        <v>124152.75041811</v>
+      </c>
+      <c r="M801" s="17">
+        <f>J801-L801</f>
+        <v/>
+      </c>
+      <c r="N801" s="18">
+        <f>IF(J801=0,"",L801/J801)</f>
+        <v/>
+      </c>
+      <c r="O801" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:17:34</t>
+        </is>
+      </c>
+      <c r="B802" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C802" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D802" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E802" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F802" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G802" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H802" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I802" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J802" s="17" t="n">
+        <v>327614.761957692</v>
+      </c>
+      <c r="K802" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L802" s="17" t="n">
+        <v>280241.2606718955</v>
+      </c>
+      <c r="M802" s="17">
+        <f>J802-L802</f>
+        <v/>
+      </c>
+      <c r="N802" s="18">
+        <f>IF(J802=0,"",L802/J802)</f>
+        <v/>
+      </c>
+      <c r="O802" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:17:34</t>
+        </is>
+      </c>
+      <c r="B803" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C803" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D803" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E803" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F803" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G803" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H803" s="16" t="n">
+        <v>1.9045</v>
+      </c>
+      <c r="I803" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J803" s="17" t="n">
+        <v>159989.8916291629</v>
+      </c>
+      <c r="K803" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,938.3760</t>
+        </is>
+      </c>
+      <c r="L803" s="17" t="n">
+        <v>70945.47053958943</v>
+      </c>
+      <c r="M803" s="17">
+        <f>J803-L803</f>
+        <v/>
+      </c>
+      <c r="N803" s="18">
+        <f>IF(J803=0,"",L803/J803)</f>
+        <v/>
+      </c>
+      <c r="O803" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:17:34</t>
+        </is>
+      </c>
+      <c r="B804" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C804" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D804" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E804" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F804" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G804" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H804" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I804" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J804" s="17" t="n">
+        <v>160152.1959815546</v>
+      </c>
+      <c r="K804" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,523.0271</t>
+        </is>
+      </c>
+      <c r="L804" s="17" t="n">
+        <v>138523.0270556475</v>
+      </c>
+      <c r="M804" s="17">
+        <f>J804-L804</f>
+        <v/>
+      </c>
+      <c r="N804" s="18">
+        <f>IF(J804=0,"",L804/J804)</f>
+        <v/>
+      </c>
+      <c r="O804" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:17:34</t>
+        </is>
+      </c>
+      <c r="B805" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C805" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D805" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E805" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F805" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G805" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H805" s="16" t="inlineStr"/>
+      <c r="I805" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J805" s="17" t="n">
+        <v>95897.03101366668</v>
+      </c>
+      <c r="K805" s="15" t="inlineStr"/>
+      <c r="L805" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M805" s="17">
+        <f>J805-L805</f>
+        <v/>
+      </c>
+      <c r="N805" s="18">
+        <f>IF(J805=0,"",L805/J805)</f>
+        <v/>
+      </c>
+      <c r="O805" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:17:34</t>
+        </is>
+      </c>
+      <c r="B806" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C806" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D806" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E806" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F806" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G806" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H806" s="16" t="inlineStr"/>
+      <c r="I806" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J806" s="17" t="n">
+        <v>34358.26123820951</v>
+      </c>
+      <c r="K806" s="15" t="inlineStr"/>
+      <c r="L806" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M806" s="17">
+        <f>J806-L806</f>
+        <v/>
+      </c>
+      <c r="N806" s="18">
+        <f>IF(J806=0,"",L806/J806)</f>
+        <v/>
+      </c>
+      <c r="O806" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:17:34</t>
+        </is>
+      </c>
+      <c r="B807" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C807" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D807" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E807" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F807" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G807" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H807" s="16" t="n">
+        <v>1.043</v>
+      </c>
+      <c r="I807" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J807" s="17" t="n">
+        <v>270023.1136243431</v>
+      </c>
+      <c r="K807" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,041.5307</t>
+        </is>
+      </c>
+      <c r="L807" s="17" t="n">
+        <v>232999.58319148</v>
+      </c>
+      <c r="M807" s="17">
+        <f>J807-L807</f>
+        <v/>
+      </c>
+      <c r="N807" s="18">
+        <f>IF(J807=0,"",L807/J807)</f>
+        <v/>
+      </c>
+      <c r="O807" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:17:34</t>
+        </is>
+      </c>
+      <c r="B808" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C808" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D808" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E808" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F808" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G808" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H808" s="16" t="inlineStr"/>
+      <c r="I808" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,512.2249</t>
+        </is>
+      </c>
+      <c r="J808" s="17" t="n">
+        <v>15509.43265716568</v>
+      </c>
+      <c r="K808" s="15" t="inlineStr"/>
+      <c r="L808" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M808" s="17">
+        <f>J808-L808</f>
+        <v/>
+      </c>
+      <c r="N808" s="18">
+        <f>IF(J808=0,"",L808/J808)</f>
+        <v/>
+      </c>
+      <c r="O808" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:17:34</t>
+        </is>
+      </c>
+      <c r="B809" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C809" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D809" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E809" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F809" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G809" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H809" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I809" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J809" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K809" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L809" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M809" s="17">
+        <f>J809-L809</f>
+        <v/>
+      </c>
+      <c r="N809" s="18">
+        <f>IF(J809=0,"",L809/J809)</f>
+        <v/>
+      </c>
+      <c r="O809" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:17:34</t>
+        </is>
+      </c>
+      <c r="B810" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C810" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D810" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E810" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F810" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G810" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H810" s="16" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="I810" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J810" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K810" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,705.3454</t>
+        </is>
+      </c>
+      <c r="L810" s="17" t="n">
+        <v>148705.345409</v>
+      </c>
+      <c r="M810" s="17">
+        <f>J810-L810</f>
+        <v/>
+      </c>
+      <c r="N810" s="18">
+        <f>IF(J810=0,"",L810/J810)</f>
+        <v/>
+      </c>
+      <c r="O810" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -53956,7 +55042,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -55827,6 +56913,41 @@
         <v>1.0375</v>
       </c>
       <c r="I53" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:17:34</t>
+        </is>
+      </c>
+      <c r="B54" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C54" s="17" t="n">
+        <v>655368.1201735664</v>
+      </c>
+      <c r="D54" s="17" t="n">
+        <v>652771.7145469659</v>
+      </c>
+      <c r="E54" s="17" t="n">
+        <v>2933417.334263642</v>
+      </c>
+      <c r="F54" s="17" t="n">
+        <v>2280645.619716676</v>
+      </c>
+      <c r="G54" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H54" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I54" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 16:47 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O810"/>
+  <dimension ref="A1:O826"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -55012,6 +55012,1092 @@
         <v/>
       </c>
       <c r="O810" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:47:52</t>
+        </is>
+      </c>
+      <c r="B811" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C811" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D811" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E811" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F811" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G811" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H811" s="16" t="n">
+        <v>1.0505</v>
+      </c>
+      <c r="I811" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,804.5477</t>
+        </is>
+      </c>
+      <c r="J811" s="17" t="n">
+        <v>50784.2258439348</v>
+      </c>
+      <c r="K811" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,722.8797</t>
+        </is>
+      </c>
+      <c r="L811" s="17" t="n">
+        <v>37730.42577515503</v>
+      </c>
+      <c r="M811" s="17">
+        <f>J811-L811</f>
+        <v/>
+      </c>
+      <c r="N811" s="18">
+        <f>IF(J811=0,"",L811/J811)</f>
+        <v/>
+      </c>
+      <c r="O811" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:47:52</t>
+        </is>
+      </c>
+      <c r="B812" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C812" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D812" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E812" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F812" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G812" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H812" s="16" t="n">
+        <v>1.0481</v>
+      </c>
+      <c r="I812" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J812" s="17" t="n">
+        <v>140898.4610119285</v>
+      </c>
+      <c r="K812" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,035.0439</t>
+        </is>
+      </c>
+      <c r="L812" s="17" t="n">
+        <v>120986.6299094292</v>
+      </c>
+      <c r="M812" s="17">
+        <f>J812-L812</f>
+        <v/>
+      </c>
+      <c r="N812" s="18">
+        <f>IF(J812=0,"",L812/J812)</f>
+        <v/>
+      </c>
+      <c r="O812" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:47:52</t>
+        </is>
+      </c>
+      <c r="B813" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C813" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D813" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E813" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F813" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G813" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H813" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I813" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J813" s="17" t="n">
+        <v>328720.464557272</v>
+      </c>
+      <c r="K813" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,386.0522</t>
+        </is>
+      </c>
+      <c r="L813" s="17" t="n">
+        <v>306456.681476752</v>
+      </c>
+      <c r="M813" s="17">
+        <f>J813-L813</f>
+        <v/>
+      </c>
+      <c r="N813" s="18">
+        <f>IF(J813=0,"",L813/J813)</f>
+        <v/>
+      </c>
+      <c r="O813" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:47:52</t>
+        </is>
+      </c>
+      <c r="B814" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C814" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D814" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E814" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F814" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G814" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H814" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I814" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J814" s="17" t="n">
+        <v>386028.9954530127</v>
+      </c>
+      <c r="K814" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,608.2120</t>
+        </is>
+      </c>
+      <c r="L814" s="17" t="n">
+        <v>349688.8050264082</v>
+      </c>
+      <c r="M814" s="17">
+        <f>J814-L814</f>
+        <v/>
+      </c>
+      <c r="N814" s="18">
+        <f>IF(J814=0,"",L814/J814)</f>
+        <v/>
+      </c>
+      <c r="O814" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:47:52</t>
+        </is>
+      </c>
+      <c r="B815" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C815" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D815" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E815" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F815" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G815" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H815" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I815" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7848</t>
+        </is>
+      </c>
+      <c r="J815" s="17" t="n">
+        <v>77782.66119583274</v>
+      </c>
+      <c r="K815" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,028.1988; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L815" s="17" t="n">
+        <v>68001.0651449755</v>
+      </c>
+      <c r="M815" s="17">
+        <f>J815-L815</f>
+        <v/>
+      </c>
+      <c r="N815" s="18">
+        <f>IF(J815=0,"",L815/J815)</f>
+        <v/>
+      </c>
+      <c r="O815" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:47:52</t>
+        </is>
+      </c>
+      <c r="B816" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C816" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D816" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E816" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F816" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G816" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H816" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I816" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J816" s="17" t="n">
+        <v>197082.3360639078</v>
+      </c>
+      <c r="K816" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,243.9962</t>
+        </is>
+      </c>
+      <c r="L816" s="17" t="n">
+        <v>150274.0510569464</v>
+      </c>
+      <c r="M816" s="17">
+        <f>J816-L816</f>
+        <v/>
+      </c>
+      <c r="N816" s="18">
+        <f>IF(J816=0,"",L816/J816)</f>
+        <v/>
+      </c>
+      <c r="O816" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:47:52</t>
+        </is>
+      </c>
+      <c r="B817" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C817" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D817" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E817" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F817" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G817" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H817" s="16" t="n">
+        <v>1.3726</v>
+      </c>
+      <c r="I817" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J817" s="17" t="n">
+        <v>186068.7386972146</v>
+      </c>
+      <c r="K817" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,140.3351</t>
+        </is>
+      </c>
+      <c r="L817" s="17" t="n">
+        <v>124165.1681767035</v>
+      </c>
+      <c r="M817" s="17">
+        <f>J817-L817</f>
+        <v/>
+      </c>
+      <c r="N817" s="18">
+        <f>IF(J817=0,"",L817/J817)</f>
+        <v/>
+      </c>
+      <c r="O817" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:47:52</t>
+        </is>
+      </c>
+      <c r="B818" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C818" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D818" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E818" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F818" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G818" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H818" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I818" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J818" s="17" t="n">
+        <v>327614.6995358152</v>
+      </c>
+      <c r="K818" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L818" s="17" t="n">
+        <v>280238.9585065345</v>
+      </c>
+      <c r="M818" s="17">
+        <f>J818-L818</f>
+        <v/>
+      </c>
+      <c r="N818" s="18">
+        <f>IF(J818=0,"",L818/J818)</f>
+        <v/>
+      </c>
+      <c r="O818" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:47:52</t>
+        </is>
+      </c>
+      <c r="B819" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C819" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D819" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E819" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F819" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G819" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H819" s="16" t="n">
+        <v>1.9045</v>
+      </c>
+      <c r="I819" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J819" s="17" t="n">
+        <v>159989.8916291629</v>
+      </c>
+      <c r="K819" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,938.3760</t>
+        </is>
+      </c>
+      <c r="L819" s="17" t="n">
+        <v>70952.56650583663</v>
+      </c>
+      <c r="M819" s="17">
+        <f>J819-L819</f>
+        <v/>
+      </c>
+      <c r="N819" s="18">
+        <f>IF(J819=0,"",L819/J819)</f>
+        <v/>
+      </c>
+      <c r="O819" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:47:52</t>
+        </is>
+      </c>
+      <c r="B820" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C820" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D820" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E820" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F820" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G820" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H820" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I820" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J820" s="17" t="n">
+        <v>160152.9845487996</v>
+      </c>
+      <c r="K820" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,523.0271</t>
+        </is>
+      </c>
+      <c r="L820" s="17" t="n">
+        <v>138509.1747529419</v>
+      </c>
+      <c r="M820" s="17">
+        <f>J820-L820</f>
+        <v/>
+      </c>
+      <c r="N820" s="18">
+        <f>IF(J820=0,"",L820/J820)</f>
+        <v/>
+      </c>
+      <c r="O820" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:47:52</t>
+        </is>
+      </c>
+      <c r="B821" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C821" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D821" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E821" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F821" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G821" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H821" s="16" t="inlineStr"/>
+      <c r="I821" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J821" s="17" t="n">
+        <v>95893.48274470943</v>
+      </c>
+      <c r="K821" s="15" t="inlineStr"/>
+      <c r="L821" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M821" s="17">
+        <f>J821-L821</f>
+        <v/>
+      </c>
+      <c r="N821" s="18">
+        <f>IF(J821=0,"",L821/J821)</f>
+        <v/>
+      </c>
+      <c r="O821" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:47:52</t>
+        </is>
+      </c>
+      <c r="B822" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C822" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D822" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E822" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F822" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G822" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H822" s="16" t="inlineStr"/>
+      <c r="I822" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J822" s="17" t="n">
+        <v>34358.4666410525</v>
+      </c>
+      <c r="K822" s="15" t="inlineStr"/>
+      <c r="L822" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M822" s="17">
+        <f>J822-L822</f>
+        <v/>
+      </c>
+      <c r="N822" s="18">
+        <f>IF(J822=0,"",L822/J822)</f>
+        <v/>
+      </c>
+      <c r="O822" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:47:52</t>
+        </is>
+      </c>
+      <c r="B823" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C823" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D823" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E823" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F823" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G823" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H823" s="16" t="n">
+        <v>1.0433</v>
+      </c>
+      <c r="I823" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J823" s="17" t="n">
+        <v>270050.1213372481</v>
+      </c>
+      <c r="K823" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,041.5307</t>
+        </is>
+      </c>
+      <c r="L823" s="17" t="n">
+        <v>232948.3140547332</v>
+      </c>
+      <c r="M823" s="17">
+        <f>J823-L823</f>
+        <v/>
+      </c>
+      <c r="N823" s="18">
+        <f>IF(J823=0,"",L823/J823)</f>
+        <v/>
+      </c>
+      <c r="O823" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:47:52</t>
+        </is>
+      </c>
+      <c r="B824" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C824" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D824" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E824" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F824" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G824" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H824" s="16" t="inlineStr"/>
+      <c r="I824" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,512.4267</t>
+        </is>
+      </c>
+      <c r="J824" s="17" t="n">
+        <v>15506.22169200854</v>
+      </c>
+      <c r="K824" s="15" t="inlineStr"/>
+      <c r="L824" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M824" s="17">
+        <f>J824-L824</f>
+        <v/>
+      </c>
+      <c r="N824" s="18">
+        <f>IF(J824=0,"",L824/J824)</f>
+        <v/>
+      </c>
+      <c r="O824" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:47:52</t>
+        </is>
+      </c>
+      <c r="B825" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C825" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D825" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E825" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F825" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G825" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H825" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I825" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J825" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K825" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L825" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M825" s="17">
+        <f>J825-L825</f>
+        <v/>
+      </c>
+      <c r="N825" s="18">
+        <f>IF(J825=0,"",L825/J825)</f>
+        <v/>
+      </c>
+      <c r="O825" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:47:52</t>
+        </is>
+      </c>
+      <c r="B826" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C826" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D826" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E826" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F826" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G826" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H826" s="16" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="I826" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J826" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K826" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,705.3454</t>
+        </is>
+      </c>
+      <c r="L826" s="17" t="n">
+        <v>148705.345409</v>
+      </c>
+      <c r="M826" s="17">
+        <f>J826-L826</f>
+        <v/>
+      </c>
+      <c r="N826" s="18">
+        <f>IF(J826=0,"",L826/J826)</f>
+        <v/>
+      </c>
+      <c r="O826" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -55042,7 +56128,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I54"/>
+  <dimension ref="A1:I55"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -56948,6 +58034,41 @@
         <v>1.0375</v>
       </c>
       <c r="I54" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 16:47:52</t>
+        </is>
+      </c>
+      <c r="B55" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C55" s="17" t="n">
+        <v>655359.9422414228</v>
+      </c>
+      <c r="D55" s="17" t="n">
+        <v>652775.3986434336</v>
+      </c>
+      <c r="E55" s="17" t="n">
+        <v>2933415.131542849</v>
+      </c>
+      <c r="F55" s="17" t="n">
+        <v>2280639.732899416</v>
+      </c>
+      <c r="G55" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H55" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I55" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 17:18 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O826"/>
+  <dimension ref="A1:O842"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -56098,6 +56098,1092 @@
         <v/>
       </c>
       <c r="O826" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:18:03</t>
+        </is>
+      </c>
+      <c r="B827" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C827" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D827" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E827" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F827" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G827" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H827" s="16" t="n">
+        <v>1.0505</v>
+      </c>
+      <c r="I827" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,804.5477</t>
+        </is>
+      </c>
+      <c r="J827" s="17" t="n">
+        <v>50781.17757107502</v>
+      </c>
+      <c r="K827" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,722.8797</t>
+        </is>
+      </c>
+      <c r="L827" s="17" t="n">
+        <v>37734.19994998499</v>
+      </c>
+      <c r="M827" s="17">
+        <f>J827-L827</f>
+        <v/>
+      </c>
+      <c r="N827" s="18">
+        <f>IF(J827=0,"",L827/J827)</f>
+        <v/>
+      </c>
+      <c r="O827" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:18:03</t>
+        </is>
+      </c>
+      <c r="B828" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C828" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D828" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E828" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F828" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G828" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H828" s="16" t="n">
+        <v>1.0482</v>
+      </c>
+      <c r="I828" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J828" s="17" t="n">
+        <v>140898.9047924363</v>
+      </c>
+      <c r="K828" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,035.0439</t>
+        </is>
+      </c>
+      <c r="L828" s="17" t="n">
+        <v>120979.3678067936</v>
+      </c>
+      <c r="M828" s="17">
+        <f>J828-L828</f>
+        <v/>
+      </c>
+      <c r="N828" s="18">
+        <f>IF(J828=0,"",L828/J828)</f>
+        <v/>
+      </c>
+      <c r="O828" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:18:03</t>
+        </is>
+      </c>
+      <c r="B829" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C829" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D829" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E829" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F829" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G829" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H829" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I829" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J829" s="17" t="n">
+        <v>328720.756475619</v>
+      </c>
+      <c r="K829" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,386.0522</t>
+        </is>
+      </c>
+      <c r="L829" s="17" t="n">
+        <v>306487.2880288574</v>
+      </c>
+      <c r="M829" s="17">
+        <f>J829-L829</f>
+        <v/>
+      </c>
+      <c r="N829" s="18">
+        <f>IF(J829=0,"",L829/J829)</f>
+        <v/>
+      </c>
+      <c r="O829" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:18:03</t>
+        </is>
+      </c>
+      <c r="B830" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C830" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D830" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E830" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F830" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G830" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H830" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I830" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J830" s="17" t="n">
+        <v>386068.7643823209</v>
+      </c>
+      <c r="K830" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,608.2120</t>
+        </is>
+      </c>
+      <c r="L830" s="17" t="n">
+        <v>349723.7292727328</v>
+      </c>
+      <c r="M830" s="17">
+        <f>J830-L830</f>
+        <v/>
+      </c>
+      <c r="N830" s="18">
+        <f>IF(J830=0,"",L830/J830)</f>
+        <v/>
+      </c>
+      <c r="O830" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:18:03</t>
+        </is>
+      </c>
+      <c r="B831" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C831" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D831" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E831" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F831" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G831" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H831" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I831" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7848</t>
+        </is>
+      </c>
+      <c r="J831" s="17" t="n">
+        <v>77781.91930111377</v>
+      </c>
+      <c r="K831" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,028.1988; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L831" s="17" t="n">
+        <v>67996.30317881594</v>
+      </c>
+      <c r="M831" s="17">
+        <f>J831-L831</f>
+        <v/>
+      </c>
+      <c r="N831" s="18">
+        <f>IF(J831=0,"",L831/J831)</f>
+        <v/>
+      </c>
+      <c r="O831" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:18:03</t>
+        </is>
+      </c>
+      <c r="B832" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C832" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D832" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E832" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F832" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G832" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H832" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I832" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J832" s="17" t="n">
+        <v>197086.1307680263</v>
+      </c>
+      <c r="K832" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,243.9962</t>
+        </is>
+      </c>
+      <c r="L832" s="17" t="n">
+        <v>150289.0829716265</v>
+      </c>
+      <c r="M832" s="17">
+        <f>J832-L832</f>
+        <v/>
+      </c>
+      <c r="N832" s="18">
+        <f>IF(J832=0,"",L832/J832)</f>
+        <v/>
+      </c>
+      <c r="O832" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:18:03</t>
+        </is>
+      </c>
+      <c r="B833" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C833" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D833" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E833" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F833" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G833" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H833" s="16" t="n">
+        <v>1.3726</v>
+      </c>
+      <c r="I833" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J833" s="17" t="n">
+        <v>186069.6034586806</v>
+      </c>
+      <c r="K833" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,140.3351</t>
+        </is>
+      </c>
+      <c r="L833" s="17" t="n">
+        <v>124177.588419594</v>
+      </c>
+      <c r="M833" s="17">
+        <f>J833-L833</f>
+        <v/>
+      </c>
+      <c r="N833" s="18">
+        <f>IF(J833=0,"",L833/J833)</f>
+        <v/>
+      </c>
+      <c r="O833" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:18:03</t>
+        </is>
+      </c>
+      <c r="B834" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C834" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D834" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E834" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F834" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G834" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H834" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I834" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J834" s="17" t="n">
+        <v>327610.8415321918</v>
+      </c>
+      <c r="K834" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L834" s="17" t="n">
+        <v>280238.9797317287</v>
+      </c>
+      <c r="M834" s="17">
+        <f>J834-L834</f>
+        <v/>
+      </c>
+      <c r="N834" s="18">
+        <f>IF(J834=0,"",L834/J834)</f>
+        <v/>
+      </c>
+      <c r="O834" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:18:03</t>
+        </is>
+      </c>
+      <c r="B835" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C835" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D835" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E835" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F835" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G835" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H835" s="16" t="n">
+        <v>1.9045</v>
+      </c>
+      <c r="I835" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J835" s="17" t="n">
+        <v>159989.8916291629</v>
+      </c>
+      <c r="K835" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,938.3760</t>
+        </is>
+      </c>
+      <c r="L835" s="17" t="n">
+        <v>70959.66389170298</v>
+      </c>
+      <c r="M835" s="17">
+        <f>J835-L835</f>
+        <v/>
+      </c>
+      <c r="N835" s="18">
+        <f>IF(J835=0,"",L835/J835)</f>
+        <v/>
+      </c>
+      <c r="O835" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:18:03</t>
+        </is>
+      </c>
+      <c r="B836" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C836" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D836" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E836" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F836" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G836" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H836" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I836" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J836" s="17" t="n">
+        <v>160169.4836014512</v>
+      </c>
+      <c r="K836" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,523.0271</t>
+        </is>
+      </c>
+      <c r="L836" s="17" t="n">
+        <v>138523.0270556475</v>
+      </c>
+      <c r="M836" s="17">
+        <f>J836-L836</f>
+        <v/>
+      </c>
+      <c r="N836" s="18">
+        <f>IF(J836=0,"",L836/J836)</f>
+        <v/>
+      </c>
+      <c r="O836" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:18:03</t>
+        </is>
+      </c>
+      <c r="B837" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C837" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D837" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E837" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F837" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G837" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H837" s="16" t="inlineStr"/>
+      <c r="I837" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J837" s="17" t="n">
+        <v>95893.48274470943</v>
+      </c>
+      <c r="K837" s="15" t="inlineStr"/>
+      <c r="L837" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M837" s="17">
+        <f>J837-L837</f>
+        <v/>
+      </c>
+      <c r="N837" s="18">
+        <f>IF(J837=0,"",L837/J837)</f>
+        <v/>
+      </c>
+      <c r="O837" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:18:03</t>
+        </is>
+      </c>
+      <c r="B838" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C838" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D838" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E838" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F838" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G838" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H838" s="16" t="inlineStr"/>
+      <c r="I838" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J838" s="17" t="n">
+        <v>34358.49001254841</v>
+      </c>
+      <c r="K838" s="15" t="inlineStr"/>
+      <c r="L838" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M838" s="17">
+        <f>J838-L838</f>
+        <v/>
+      </c>
+      <c r="N838" s="18">
+        <f>IF(J838=0,"",L838/J838)</f>
+        <v/>
+      </c>
+      <c r="O838" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:18:03</t>
+        </is>
+      </c>
+      <c r="B839" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C839" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D839" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E839" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F839" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G839" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H839" s="16" t="n">
+        <v>1.0434</v>
+      </c>
+      <c r="I839" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J839" s="17" t="n">
+        <v>270051.0239269384</v>
+      </c>
+      <c r="K839" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,041.5307</t>
+        </is>
+      </c>
+      <c r="L839" s="17" t="n">
+        <v>232932.0011475865</v>
+      </c>
+      <c r="M839" s="17">
+        <f>J839-L839</f>
+        <v/>
+      </c>
+      <c r="N839" s="18">
+        <f>IF(J839=0,"",L839/J839)</f>
+        <v/>
+      </c>
+      <c r="O839" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:18:03</t>
+        </is>
+      </c>
+      <c r="B840" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C840" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D840" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E840" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F840" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G840" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H840" s="16" t="inlineStr"/>
+      <c r="I840" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,512.6302</t>
+        </is>
+      </c>
+      <c r="J840" s="17" t="n">
+        <v>15505.33921605905</v>
+      </c>
+      <c r="K840" s="15" t="inlineStr"/>
+      <c r="L840" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M840" s="17">
+        <f>J840-L840</f>
+        <v/>
+      </c>
+      <c r="N840" s="18">
+        <f>IF(J840=0,"",L840/J840)</f>
+        <v/>
+      </c>
+      <c r="O840" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:18:03</t>
+        </is>
+      </c>
+      <c r="B841" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C841" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D841" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E841" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F841" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G841" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H841" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I841" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J841" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K841" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L841" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M841" s="17">
+        <f>J841-L841</f>
+        <v/>
+      </c>
+      <c r="N841" s="18">
+        <f>IF(J841=0,"",L841/J841)</f>
+        <v/>
+      </c>
+      <c r="O841" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:18:03</t>
+        </is>
+      </c>
+      <c r="B842" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C842" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D842" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E842" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F842" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G842" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H842" s="16" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="I842" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J842" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K842" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,705.3454</t>
+        </is>
+      </c>
+      <c r="L842" s="17" t="n">
+        <v>148705.345409</v>
+      </c>
+      <c r="M842" s="17">
+        <f>J842-L842</f>
+        <v/>
+      </c>
+      <c r="N842" s="18">
+        <f>IF(J842=0,"",L842/J842)</f>
+        <v/>
+      </c>
+      <c r="O842" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -56128,7 +57214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:I56"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -58069,6 +59155,41 @@
         <v>1.0375</v>
       </c>
       <c r="I55" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:18:03</t>
+        </is>
+      </c>
+      <c r="B56" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C56" s="17" t="n">
+        <v>655324.8168100127</v>
+      </c>
+      <c r="D56" s="17" t="n">
+        <v>652740.066035212</v>
+      </c>
+      <c r="E56" s="17" t="n">
+        <v>2933469.190003283</v>
+      </c>
+      <c r="F56" s="17" t="n">
+        <v>2280729.123968071</v>
+      </c>
+      <c r="G56" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H56" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I56" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 17:48 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O842"/>
+  <dimension ref="A1:O858"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -57184,6 +57184,1092 @@
         <v/>
       </c>
       <c r="O842" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:48:16</t>
+        </is>
+      </c>
+      <c r="B843" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C843" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D843" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E843" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F843" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G843" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H843" s="16" t="n">
+        <v>1.0505</v>
+      </c>
+      <c r="I843" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,804.5477</t>
+        </is>
+      </c>
+      <c r="J843" s="17" t="n">
+        <v>50779.1453891685</v>
+      </c>
+      <c r="K843" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,722.8797</t>
+        </is>
+      </c>
+      <c r="L843" s="17" t="n">
+        <v>37734.19994998499</v>
+      </c>
+      <c r="M843" s="17">
+        <f>J843-L843</f>
+        <v/>
+      </c>
+      <c r="N843" s="18">
+        <f>IF(J843=0,"",L843/J843)</f>
+        <v/>
+      </c>
+      <c r="O843" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:48:16</t>
+        </is>
+      </c>
+      <c r="B844" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C844" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D844" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E844" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F844" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G844" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H844" s="16" t="n">
+        <v>1.0483</v>
+      </c>
+      <c r="I844" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J844" s="17" t="n">
+        <v>140913.2573546365</v>
+      </c>
+      <c r="K844" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,035.0439</t>
+        </is>
+      </c>
+      <c r="L844" s="17" t="n">
+        <v>120974.5264050365</v>
+      </c>
+      <c r="M844" s="17">
+        <f>J844-L844</f>
+        <v/>
+      </c>
+      <c r="N844" s="18">
+        <f>IF(J844=0,"",L844/J844)</f>
+        <v/>
+      </c>
+      <c r="O844" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:48:16</t>
+        </is>
+      </c>
+      <c r="B845" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C845" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D845" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E845" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F845" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G845" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H845" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I845" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J845" s="17" t="n">
+        <v>328721.3115997481</v>
+      </c>
+      <c r="K845" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,386.0522</t>
+        </is>
+      </c>
+      <c r="L845" s="17" t="n">
+        <v>306487.2210600017</v>
+      </c>
+      <c r="M845" s="17">
+        <f>J845-L845</f>
+        <v/>
+      </c>
+      <c r="N845" s="18">
+        <f>IF(J845=0,"",L845/J845)</f>
+        <v/>
+      </c>
+      <c r="O845" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:48:16</t>
+        </is>
+      </c>
+      <c r="B846" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C846" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D846" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E846" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F846" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G846" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H846" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I846" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J846" s="17" t="n">
+        <v>386069.9265569859</v>
+      </c>
+      <c r="K846" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,608.2120</t>
+        </is>
+      </c>
+      <c r="L846" s="17" t="n">
+        <v>349723.6528565195</v>
+      </c>
+      <c r="M846" s="17">
+        <f>J846-L846</f>
+        <v/>
+      </c>
+      <c r="N846" s="18">
+        <f>IF(J846=0,"",L846/J846)</f>
+        <v/>
+      </c>
+      <c r="O846" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:48:16</t>
+        </is>
+      </c>
+      <c r="B847" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C847" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D847" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E847" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F847" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G847" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H847" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I847" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7848</t>
+        </is>
+      </c>
+      <c r="J847" s="17" t="n">
+        <v>77779.61135132046</v>
+      </c>
+      <c r="K847" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,028.1988; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L847" s="17" t="n">
+        <v>67994.26233285047</v>
+      </c>
+      <c r="M847" s="17">
+        <f>J847-L847</f>
+        <v/>
+      </c>
+      <c r="N847" s="18">
+        <f>IF(J847=0,"",L847/J847)</f>
+        <v/>
+      </c>
+      <c r="O847" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:48:16</t>
+        </is>
+      </c>
+      <c r="B848" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C848" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D848" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E848" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F848" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G848" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H848" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I848" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J848" s="17" t="n">
+        <v>197088.1718105385</v>
+      </c>
+      <c r="K848" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,243.9962</t>
+        </is>
+      </c>
+      <c r="L848" s="17" t="n">
+        <v>150289.0829716265</v>
+      </c>
+      <c r="M848" s="17">
+        <f>J848-L848</f>
+        <v/>
+      </c>
+      <c r="N848" s="18">
+        <f>IF(J848=0,"",L848/J848)</f>
+        <v/>
+      </c>
+      <c r="O848" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:48:16</t>
+        </is>
+      </c>
+      <c r="B849" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C849" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D849" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E849" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F849" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G849" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H849" s="16" t="n">
+        <v>1.3726</v>
+      </c>
+      <c r="I849" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J849" s="17" t="n">
+        <v>186070.462750954</v>
+      </c>
+      <c r="K849" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,140.3351</t>
+        </is>
+      </c>
+      <c r="L849" s="17" t="n">
+        <v>124177.588419594</v>
+      </c>
+      <c r="M849" s="17">
+        <f>J849-L849</f>
+        <v/>
+      </c>
+      <c r="N849" s="18">
+        <f>IF(J849=0,"",L849/J849)</f>
+        <v/>
+      </c>
+      <c r="O849" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:48:16</t>
+        </is>
+      </c>
+      <c r="B850" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C850" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D850" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E850" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F850" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G850" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H850" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I850" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J850" s="17" t="n">
+        <v>327616.7919593118</v>
+      </c>
+      <c r="K850" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L850" s="17" t="n">
+        <v>280242.041382527</v>
+      </c>
+      <c r="M850" s="17">
+        <f>J850-L850</f>
+        <v/>
+      </c>
+      <c r="N850" s="18">
+        <f>IF(J850=0,"",L850/J850)</f>
+        <v/>
+      </c>
+      <c r="O850" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:48:16</t>
+        </is>
+      </c>
+      <c r="B851" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C851" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D851" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E851" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F851" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G851" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H851" s="16" t="n">
+        <v>1.9045</v>
+      </c>
+      <c r="I851" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J851" s="17" t="n">
+        <v>159989.8916291629</v>
+      </c>
+      <c r="K851" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,938.3760</t>
+        </is>
+      </c>
+      <c r="L851" s="17" t="n">
+        <v>70959.66389170298</v>
+      </c>
+      <c r="M851" s="17">
+        <f>J851-L851</f>
+        <v/>
+      </c>
+      <c r="N851" s="18">
+        <f>IF(J851=0,"",L851/J851)</f>
+        <v/>
+      </c>
+      <c r="O851" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:48:16</t>
+        </is>
+      </c>
+      <c r="B852" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C852" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D852" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E852" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F852" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G852" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H852" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I852" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J852" s="17" t="n">
+        <v>160169.9657562721</v>
+      </c>
+      <c r="K852" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,523.0271</t>
+        </is>
+      </c>
+      <c r="L852" s="17" t="n">
+        <v>138523.0270556475</v>
+      </c>
+      <c r="M852" s="17">
+        <f>J852-L852</f>
+        <v/>
+      </c>
+      <c r="N852" s="18">
+        <f>IF(J852=0,"",L852/J852)</f>
+        <v/>
+      </c>
+      <c r="O852" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:48:16</t>
+        </is>
+      </c>
+      <c r="B853" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C853" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D853" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E853" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F853" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G853" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H853" s="16" t="inlineStr"/>
+      <c r="I853" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J853" s="17" t="n">
+        <v>95893.48274470943</v>
+      </c>
+      <c r="K853" s="15" t="inlineStr"/>
+      <c r="L853" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M853" s="17">
+        <f>J853-L853</f>
+        <v/>
+      </c>
+      <c r="N853" s="18">
+        <f>IF(J853=0,"",L853/J853)</f>
+        <v/>
+      </c>
+      <c r="O853" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:48:16</t>
+        </is>
+      </c>
+      <c r="B854" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C854" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D854" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E854" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F854" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G854" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H854" s="16" t="inlineStr"/>
+      <c r="I854" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J854" s="17" t="n">
+        <v>34358.77299533737</v>
+      </c>
+      <c r="K854" s="15" t="inlineStr"/>
+      <c r="L854" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M854" s="17">
+        <f>J854-L854</f>
+        <v/>
+      </c>
+      <c r="N854" s="18">
+        <f>IF(J854=0,"",L854/J854)</f>
+        <v/>
+      </c>
+      <c r="O854" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:48:16</t>
+        </is>
+      </c>
+      <c r="B855" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C855" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D855" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E855" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F855" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G855" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H855" s="16" t="n">
+        <v>1.0436</v>
+      </c>
+      <c r="I855" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J855" s="17" t="n">
+        <v>270078.0371332929</v>
+      </c>
+      <c r="K855" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,041.5307</t>
+        </is>
+      </c>
+      <c r="L855" s="17" t="n">
+        <v>232925.0099016665</v>
+      </c>
+      <c r="M855" s="17">
+        <f>J855-L855</f>
+        <v/>
+      </c>
+      <c r="N855" s="18">
+        <f>IF(J855=0,"",L855/J855)</f>
+        <v/>
+      </c>
+      <c r="O855" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:48:16</t>
+        </is>
+      </c>
+      <c r="B856" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C856" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D856" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E856" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F856" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G856" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H856" s="16" t="inlineStr"/>
+      <c r="I856" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,512.8368</t>
+        </is>
+      </c>
+      <c r="J856" s="17" t="n">
+        <v>15505.0803678204</v>
+      </c>
+      <c r="K856" s="15" t="inlineStr"/>
+      <c r="L856" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M856" s="17">
+        <f>J856-L856</f>
+        <v/>
+      </c>
+      <c r="N856" s="18">
+        <f>IF(J856=0,"",L856/J856)</f>
+        <v/>
+      </c>
+      <c r="O856" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:48:16</t>
+        </is>
+      </c>
+      <c r="B857" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C857" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D857" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E857" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F857" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G857" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H857" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I857" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J857" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K857" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L857" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M857" s="17">
+        <f>J857-L857</f>
+        <v/>
+      </c>
+      <c r="N857" s="18">
+        <f>IF(J857=0,"",L857/J857)</f>
+        <v/>
+      </c>
+      <c r="O857" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:48:16</t>
+        </is>
+      </c>
+      <c r="B858" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C858" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D858" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E858" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F858" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G858" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H858" s="16" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="I858" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J858" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K858" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,705.3454</t>
+        </is>
+      </c>
+      <c r="L858" s="17" t="n">
+        <v>148705.345409</v>
+      </c>
+      <c r="M858" s="17">
+        <f>J858-L858</f>
+        <v/>
+      </c>
+      <c r="N858" s="18">
+        <f>IF(J858=0,"",L858/J858)</f>
+        <v/>
+      </c>
+      <c r="O858" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -57214,7 +58300,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I56"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -59190,6 +60276,41 @@
         <v>1.0375</v>
       </c>
       <c r="I56" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 17:48:16</t>
+        </is>
+      </c>
+      <c r="B57" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C57" s="17" t="n">
+        <v>655384.0356835272</v>
+      </c>
+      <c r="D57" s="17" t="n">
+        <v>652799.1212500511</v>
+      </c>
+      <c r="E57" s="17" t="n">
+        <v>2933517.289990209</v>
+      </c>
+      <c r="F57" s="17" t="n">
+        <v>2280718.168740158</v>
+      </c>
+      <c r="G57" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H57" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I57" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-29 18:18 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O858"/>
+  <dimension ref="A1:O874"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -58270,6 +58270,1092 @@
         <v/>
       </c>
       <c r="O858" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:30</t>
+        </is>
+      </c>
+      <c r="B859" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C859" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D859" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E859" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F859" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G859" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H859" s="16" t="n">
+        <v>1.0505</v>
+      </c>
+      <c r="I859" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,804.5477</t>
+        </is>
+      </c>
+      <c r="J859" s="17" t="n">
+        <v>50781.17757107502</v>
+      </c>
+      <c r="K859" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,722.8797</t>
+        </is>
+      </c>
+      <c r="L859" s="17" t="n">
+        <v>37734.19994998499</v>
+      </c>
+      <c r="M859" s="17">
+        <f>J859-L859</f>
+        <v/>
+      </c>
+      <c r="N859" s="18">
+        <f>IF(J859=0,"",L859/J859)</f>
+        <v/>
+      </c>
+      <c r="O859" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:30</t>
+        </is>
+      </c>
+      <c r="B860" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C860" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D860" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E860" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F860" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G860" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H860" s="16" t="n">
+        <v>1.0483</v>
+      </c>
+      <c r="I860" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J860" s="17" t="n">
+        <v>140914.0860544015</v>
+      </c>
+      <c r="K860" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,035.0439</t>
+        </is>
+      </c>
+      <c r="L860" s="17" t="n">
+        <v>120979.3678067936</v>
+      </c>
+      <c r="M860" s="17">
+        <f>J860-L860</f>
+        <v/>
+      </c>
+      <c r="N860" s="18">
+        <f>IF(J860=0,"",L860/J860)</f>
+        <v/>
+      </c>
+      <c r="O860" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:30</t>
+        </is>
+      </c>
+      <c r="B861" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C861" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D861" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E861" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F861" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G861" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H861" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I861" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J861" s="17" t="n">
+        <v>328723.1061884762</v>
+      </c>
+      <c r="K861" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,386.0522</t>
+        </is>
+      </c>
+      <c r="L861" s="17" t="n">
+        <v>306449.0897480633</v>
+      </c>
+      <c r="M861" s="17">
+        <f>J861-L861</f>
+        <v/>
+      </c>
+      <c r="N861" s="18">
+        <f>IF(J861=0,"",L861/J861)</f>
+        <v/>
+      </c>
+      <c r="O861" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:30</t>
+        </is>
+      </c>
+      <c r="B862" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C862" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D862" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E862" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F862" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G862" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H862" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I862" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J862" s="17" t="n">
+        <v>386032.4815666809</v>
+      </c>
+      <c r="K862" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,608.2120</t>
+        </is>
+      </c>
+      <c r="L862" s="17" t="n">
+        <v>349680.1423256296</v>
+      </c>
+      <c r="M862" s="17">
+        <f>J862-L862</f>
+        <v/>
+      </c>
+      <c r="N862" s="18">
+        <f>IF(J862=0,"",L862/J862)</f>
+        <v/>
+      </c>
+      <c r="O862" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:30</t>
+        </is>
+      </c>
+      <c r="B863" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C863" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D863" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E863" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F863" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G863" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H863" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I863" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7848</t>
+        </is>
+      </c>
+      <c r="J863" s="17" t="n">
+        <v>77777.15372714284</v>
+      </c>
+      <c r="K863" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,028.1988; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L863" s="17" t="n">
+        <v>67996.98346080443</v>
+      </c>
+      <c r="M863" s="17">
+        <f>J863-L863</f>
+        <v/>
+      </c>
+      <c r="N863" s="18">
+        <f>IF(J863=0,"",L863/J863)</f>
+        <v/>
+      </c>
+      <c r="O863" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:30</t>
+        </is>
+      </c>
+      <c r="B864" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C864" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D864" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E864" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F864" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G864" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H864" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I864" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J864" s="17" t="n">
+        <v>197084.9343600681</v>
+      </c>
+      <c r="K864" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,243.9962</t>
+        </is>
+      </c>
+      <c r="L864" s="17" t="n">
+        <v>150289.0829716265</v>
+      </c>
+      <c r="M864" s="17">
+        <f>J864-L864</f>
+        <v/>
+      </c>
+      <c r="N864" s="18">
+        <f>IF(J864=0,"",L864/J864)</f>
+        <v/>
+      </c>
+      <c r="O864" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:30</t>
+        </is>
+      </c>
+      <c r="B865" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C865" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D865" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E865" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F865" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G865" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H865" s="16" t="n">
+        <v>1.3726</v>
+      </c>
+      <c r="I865" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J865" s="17" t="n">
+        <v>186071.347643795</v>
+      </c>
+      <c r="K865" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,140.3351</t>
+        </is>
+      </c>
+      <c r="L865" s="17" t="n">
+        <v>124177.588419594</v>
+      </c>
+      <c r="M865" s="17">
+        <f>J865-L865</f>
+        <v/>
+      </c>
+      <c r="N865" s="18">
+        <f>IF(J865=0,"",L865/J865)</f>
+        <v/>
+      </c>
+      <c r="O865" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:30</t>
+        </is>
+      </c>
+      <c r="B866" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C866" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D866" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E866" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F866" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G866" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H866" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I866" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J866" s="17" t="n">
+        <v>327614.6310298509</v>
+      </c>
+      <c r="K866" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L866" s="17" t="n">
+        <v>280238.9660298275</v>
+      </c>
+      <c r="M866" s="17">
+        <f>J866-L866</f>
+        <v/>
+      </c>
+      <c r="N866" s="18">
+        <f>IF(J866=0,"",L866/J866)</f>
+        <v/>
+      </c>
+      <c r="O866" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:30</t>
+        </is>
+      </c>
+      <c r="B867" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C867" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D867" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E867" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F867" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G867" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H867" s="16" t="n">
+        <v>1.9045</v>
+      </c>
+      <c r="I867" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J867" s="17" t="n">
+        <v>159989.8916291629</v>
+      </c>
+      <c r="K867" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,938.3760</t>
+        </is>
+      </c>
+      <c r="L867" s="17" t="n">
+        <v>70959.66389170298</v>
+      </c>
+      <c r="M867" s="17">
+        <f>J867-L867</f>
+        <v/>
+      </c>
+      <c r="N867" s="18">
+        <f>IF(J867=0,"",L867/J867)</f>
+        <v/>
+      </c>
+      <c r="O867" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:30</t>
+        </is>
+      </c>
+      <c r="B868" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C868" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D868" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E868" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F868" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G868" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H868" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I868" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J868" s="17" t="n">
+        <v>160154.4308430289</v>
+      </c>
+      <c r="K868" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,523.0271</t>
+        </is>
+      </c>
+      <c r="L868" s="17" t="n">
+        <v>138509.1747529419</v>
+      </c>
+      <c r="M868" s="17">
+        <f>J868-L868</f>
+        <v/>
+      </c>
+      <c r="N868" s="18">
+        <f>IF(J868=0,"",L868/J868)</f>
+        <v/>
+      </c>
+      <c r="O868" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:30</t>
+        </is>
+      </c>
+      <c r="B869" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C869" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D869" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E869" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F869" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G869" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H869" s="16" t="inlineStr"/>
+      <c r="I869" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J869" s="17" t="n">
+        <v>95900.86515999959</v>
+      </c>
+      <c r="K869" s="15" t="inlineStr"/>
+      <c r="L869" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M869" s="17">
+        <f>J869-L869</f>
+        <v/>
+      </c>
+      <c r="N869" s="18">
+        <f>IF(J869=0,"",L869/J869)</f>
+        <v/>
+      </c>
+      <c r="O869" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:30</t>
+        </is>
+      </c>
+      <c r="B870" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C870" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D870" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E870" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F870" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G870" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H870" s="16" t="inlineStr"/>
+      <c r="I870" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J870" s="17" t="n">
+        <v>34359.06319029944</v>
+      </c>
+      <c r="K870" s="15" t="inlineStr"/>
+      <c r="L870" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M870" s="17">
+        <f>J870-L870</f>
+        <v/>
+      </c>
+      <c r="N870" s="18">
+        <f>IF(J870=0,"",L870/J870)</f>
+        <v/>
+      </c>
+      <c r="O870" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:30</t>
+        </is>
+      </c>
+      <c r="B871" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C871" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D871" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E871" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F871" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G871" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H871" s="16" t="n">
+        <v>1.0435</v>
+      </c>
+      <c r="I871" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J871" s="17" t="n">
+        <v>270078.0371332929</v>
+      </c>
+      <c r="K871" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,041.5307</t>
+        </is>
+      </c>
+      <c r="L871" s="17" t="n">
+        <v>232934.3315628932</v>
+      </c>
+      <c r="M871" s="17">
+        <f>J871-L871</f>
+        <v/>
+      </c>
+      <c r="N871" s="18">
+        <f>IF(J871=0,"",L871/J871)</f>
+        <v/>
+      </c>
+      <c r="O871" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:30</t>
+        </is>
+      </c>
+      <c r="B872" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C872" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D872" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E872" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F872" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G872" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H872" s="16" t="inlineStr"/>
+      <c r="I872" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,513.0398</t>
+        </is>
+      </c>
+      <c r="J872" s="17" t="n">
+        <v>15505.9038282459</v>
+      </c>
+      <c r="K872" s="15" t="inlineStr"/>
+      <c r="L872" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M872" s="17">
+        <f>J872-L872</f>
+        <v/>
+      </c>
+      <c r="N872" s="18">
+        <f>IF(J872=0,"",L872/J872)</f>
+        <v/>
+      </c>
+      <c r="O872" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:30</t>
+        </is>
+      </c>
+      <c r="B873" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C873" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D873" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E873" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F873" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G873" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H873" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I873" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J873" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K873" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L873" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M873" s="17">
+        <f>J873-L873</f>
+        <v/>
+      </c>
+      <c r="N873" s="18">
+        <f>IF(J873=0,"",L873/J873)</f>
+        <v/>
+      </c>
+      <c r="O873" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:30</t>
+        </is>
+      </c>
+      <c r="B874" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C874" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D874" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E874" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F874" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G874" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H874" s="16" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="I874" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J874" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K874" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,705.3454</t>
+        </is>
+      </c>
+      <c r="L874" s="17" t="n">
+        <v>148705.345409</v>
+      </c>
+      <c r="M874" s="17">
+        <f>J874-L874</f>
+        <v/>
+      </c>
+      <c r="N874" s="18">
+        <f>IF(J874=0,"",L874/J874)</f>
+        <v/>
+      </c>
+      <c r="O874" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -58300,7 +59386,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I57"/>
+  <dimension ref="A1:I58"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -60311,6 +61397,41 @@
         <v>1.0375</v>
       </c>
       <c r="I57" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:30</t>
+        </is>
+      </c>
+      <c r="B58" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C58" s="17" t="n">
+        <v>655417.8297348786</v>
+      </c>
+      <c r="D58" s="17" t="n">
+        <v>652834.0070836083</v>
+      </c>
+      <c r="E58" s="17" t="n">
+        <v>2933470.49051647</v>
+      </c>
+      <c r="F58" s="17" t="n">
+        <v>2280636.483432862</v>
+      </c>
+      <c r="G58" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H58" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I58" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
design: delta-hero benchmarks, 3-card summary, 0.005% color threshold
- Benchmark strip redesigned: delta $ is the 24px/900-weight hero, % beneath it, historical equity in small secondary text
- Summary bar simplified to 3 cards only: Collateral / Debt / Net with coloured left borders
- Color threshold tightened to 0.005% (max(5, |cur|×0.00005)) — nearly everything meaningful now gets green/red
- Fresh snapshot captured 2026-04-29T18:18:44Z

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O874"/>
+  <dimension ref="A1:O890"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -59356,6 +59356,1092 @@
         <v/>
       </c>
       <c r="O874" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:44</t>
+        </is>
+      </c>
+      <c r="B875" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C875" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D875" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E875" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F875" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G875" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H875" s="16" t="n">
+        <v>1.0505</v>
+      </c>
+      <c r="I875" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,804.5477</t>
+        </is>
+      </c>
+      <c r="J875" s="17" t="n">
+        <v>50781.17757107502</v>
+      </c>
+      <c r="K875" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,722.8797</t>
+        </is>
+      </c>
+      <c r="L875" s="17" t="n">
+        <v>37734.19994998499</v>
+      </c>
+      <c r="M875" s="17">
+        <f>J875-L875</f>
+        <v/>
+      </c>
+      <c r="N875" s="18">
+        <f>IF(J875=0,"",L875/J875)</f>
+        <v/>
+      </c>
+      <c r="O875" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:44</t>
+        </is>
+      </c>
+      <c r="B876" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C876" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D876" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E876" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F876" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G876" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H876" s="16" t="n">
+        <v>1.0483</v>
+      </c>
+      <c r="I876" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J876" s="17" t="n">
+        <v>140914.0860544015</v>
+      </c>
+      <c r="K876" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,035.0439</t>
+        </is>
+      </c>
+      <c r="L876" s="17" t="n">
+        <v>120979.3678067936</v>
+      </c>
+      <c r="M876" s="17">
+        <f>J876-L876</f>
+        <v/>
+      </c>
+      <c r="N876" s="18">
+        <f>IF(J876=0,"",L876/J876)</f>
+        <v/>
+      </c>
+      <c r="O876" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:44</t>
+        </is>
+      </c>
+      <c r="B877" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C877" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D877" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E877" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F877" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G877" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H877" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I877" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J877" s="17" t="n">
+        <v>328723.1061884762</v>
+      </c>
+      <c r="K877" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,386.0522</t>
+        </is>
+      </c>
+      <c r="L877" s="17" t="n">
+        <v>306449.0897480633</v>
+      </c>
+      <c r="M877" s="17">
+        <f>J877-L877</f>
+        <v/>
+      </c>
+      <c r="N877" s="18">
+        <f>IF(J877=0,"",L877/J877)</f>
+        <v/>
+      </c>
+      <c r="O877" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:44</t>
+        </is>
+      </c>
+      <c r="B878" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C878" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D878" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E878" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F878" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G878" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H878" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I878" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J878" s="17" t="n">
+        <v>386032.4815666809</v>
+      </c>
+      <c r="K878" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,608.2120</t>
+        </is>
+      </c>
+      <c r="L878" s="17" t="n">
+        <v>349680.1423256296</v>
+      </c>
+      <c r="M878" s="17">
+        <f>J878-L878</f>
+        <v/>
+      </c>
+      <c r="N878" s="18">
+        <f>IF(J878=0,"",L878/J878)</f>
+        <v/>
+      </c>
+      <c r="O878" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:44</t>
+        </is>
+      </c>
+      <c r="B879" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C879" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D879" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E879" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F879" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G879" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H879" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I879" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7848</t>
+        </is>
+      </c>
+      <c r="J879" s="17" t="n">
+        <v>77777.16589515723</v>
+      </c>
+      <c r="K879" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,028.1988; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L879" s="17" t="n">
+        <v>67996.98346080443</v>
+      </c>
+      <c r="M879" s="17">
+        <f>J879-L879</f>
+        <v/>
+      </c>
+      <c r="N879" s="18">
+        <f>IF(J879=0,"",L879/J879)</f>
+        <v/>
+      </c>
+      <c r="O879" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:44</t>
+        </is>
+      </c>
+      <c r="B880" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C880" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D880" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E880" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F880" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G880" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H880" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I880" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J880" s="17" t="n">
+        <v>197084.9343600681</v>
+      </c>
+      <c r="K880" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,243.9962</t>
+        </is>
+      </c>
+      <c r="L880" s="17" t="n">
+        <v>150289.0829716265</v>
+      </c>
+      <c r="M880" s="17">
+        <f>J880-L880</f>
+        <v/>
+      </c>
+      <c r="N880" s="18">
+        <f>IF(J880=0,"",L880/J880)</f>
+        <v/>
+      </c>
+      <c r="O880" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:44</t>
+        </is>
+      </c>
+      <c r="B881" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C881" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D881" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E881" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F881" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G881" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H881" s="16" t="n">
+        <v>1.3726</v>
+      </c>
+      <c r="I881" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J881" s="17" t="n">
+        <v>186071.347643795</v>
+      </c>
+      <c r="K881" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,140.3351</t>
+        </is>
+      </c>
+      <c r="L881" s="17" t="n">
+        <v>124177.588419594</v>
+      </c>
+      <c r="M881" s="17">
+        <f>J881-L881</f>
+        <v/>
+      </c>
+      <c r="N881" s="18">
+        <f>IF(J881=0,"",L881/J881)</f>
+        <v/>
+      </c>
+      <c r="O881" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:44</t>
+        </is>
+      </c>
+      <c r="B882" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C882" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D882" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E882" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F882" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G882" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H882" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I882" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J882" s="17" t="n">
+        <v>327614.6310298509</v>
+      </c>
+      <c r="K882" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L882" s="17" t="n">
+        <v>280238.9660298275</v>
+      </c>
+      <c r="M882" s="17">
+        <f>J882-L882</f>
+        <v/>
+      </c>
+      <c r="N882" s="18">
+        <f>IF(J882=0,"",L882/J882)</f>
+        <v/>
+      </c>
+      <c r="O882" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:44</t>
+        </is>
+      </c>
+      <c r="B883" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C883" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D883" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E883" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F883" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G883" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H883" s="16" t="n">
+        <v>1.9045</v>
+      </c>
+      <c r="I883" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J883" s="17" t="n">
+        <v>159989.8916291629</v>
+      </c>
+      <c r="K883" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,938.3760</t>
+        </is>
+      </c>
+      <c r="L883" s="17" t="n">
+        <v>70959.66389170298</v>
+      </c>
+      <c r="M883" s="17">
+        <f>J883-L883</f>
+        <v/>
+      </c>
+      <c r="N883" s="18">
+        <f>IF(J883=0,"",L883/J883)</f>
+        <v/>
+      </c>
+      <c r="O883" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:44</t>
+        </is>
+      </c>
+      <c r="B884" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C884" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D884" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E884" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F884" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G884" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H884" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I884" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J884" s="17" t="n">
+        <v>160154.4308430289</v>
+      </c>
+      <c r="K884" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,523.0271</t>
+        </is>
+      </c>
+      <c r="L884" s="17" t="n">
+        <v>138509.1747529419</v>
+      </c>
+      <c r="M884" s="17">
+        <f>J884-L884</f>
+        <v/>
+      </c>
+      <c r="N884" s="18">
+        <f>IF(J884=0,"",L884/J884)</f>
+        <v/>
+      </c>
+      <c r="O884" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:44</t>
+        </is>
+      </c>
+      <c r="B885" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C885" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D885" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E885" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F885" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G885" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H885" s="16" t="inlineStr"/>
+      <c r="I885" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J885" s="17" t="n">
+        <v>95900.86515999959</v>
+      </c>
+      <c r="K885" s="15" t="inlineStr"/>
+      <c r="L885" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M885" s="17">
+        <f>J885-L885</f>
+        <v/>
+      </c>
+      <c r="N885" s="18">
+        <f>IF(J885=0,"",L885/J885)</f>
+        <v/>
+      </c>
+      <c r="O885" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:44</t>
+        </is>
+      </c>
+      <c r="B886" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C886" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D886" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E886" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F886" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G886" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H886" s="16" t="inlineStr"/>
+      <c r="I886" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J886" s="17" t="n">
+        <v>34359.06319029944</v>
+      </c>
+      <c r="K886" s="15" t="inlineStr"/>
+      <c r="L886" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M886" s="17">
+        <f>J886-L886</f>
+        <v/>
+      </c>
+      <c r="N886" s="18">
+        <f>IF(J886=0,"",L886/J886)</f>
+        <v/>
+      </c>
+      <c r="O886" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:44</t>
+        </is>
+      </c>
+      <c r="B887" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C887" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D887" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E887" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F887" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G887" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H887" s="16" t="n">
+        <v>1.0435</v>
+      </c>
+      <c r="I887" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J887" s="17" t="n">
+        <v>270078.0371332929</v>
+      </c>
+      <c r="K887" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,041.5307</t>
+        </is>
+      </c>
+      <c r="L887" s="17" t="n">
+        <v>232934.3315628932</v>
+      </c>
+      <c r="M887" s="17">
+        <f>J887-L887</f>
+        <v/>
+      </c>
+      <c r="N887" s="18">
+        <f>IF(J887=0,"",L887/J887)</f>
+        <v/>
+      </c>
+      <c r="O887" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:44</t>
+        </is>
+      </c>
+      <c r="B888" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C888" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D888" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E888" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F888" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G888" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H888" s="16" t="inlineStr"/>
+      <c r="I888" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,513.0398</t>
+        </is>
+      </c>
+      <c r="J888" s="17" t="n">
+        <v>15505.9038282459</v>
+      </c>
+      <c r="K888" s="15" t="inlineStr"/>
+      <c r="L888" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M888" s="17">
+        <f>J888-L888</f>
+        <v/>
+      </c>
+      <c r="N888" s="18">
+        <f>IF(J888=0,"",L888/J888)</f>
+        <v/>
+      </c>
+      <c r="O888" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:44</t>
+        </is>
+      </c>
+      <c r="B889" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C889" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D889" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E889" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F889" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G889" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H889" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I889" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J889" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K889" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L889" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M889" s="17">
+        <f>J889-L889</f>
+        <v/>
+      </c>
+      <c r="N889" s="18">
+        <f>IF(J889=0,"",L889/J889)</f>
+        <v/>
+      </c>
+      <c r="O889" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:44</t>
+        </is>
+      </c>
+      <c r="B890" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C890" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D890" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E890" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F890" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G890" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H890" s="16" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="I890" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J890" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K890" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,705.3454</t>
+        </is>
+      </c>
+      <c r="L890" s="17" t="n">
+        <v>148705.345409</v>
+      </c>
+      <c r="M890" s="17">
+        <f>J890-L890</f>
+        <v/>
+      </c>
+      <c r="N890" s="18">
+        <f>IF(J890=0,"",L890/J890)</f>
+        <v/>
+      </c>
+      <c r="O890" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -59386,7 +60472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I58"/>
+  <dimension ref="A1:I59"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -61432,6 +62518,41 @@
         <v>1.0375</v>
       </c>
       <c r="I58" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:18:44</t>
+        </is>
+      </c>
+      <c r="B59" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C59" s="17" t="n">
+        <v>655417.8297348786</v>
+      </c>
+      <c r="D59" s="17" t="n">
+        <v>652834.0192516227</v>
+      </c>
+      <c r="E59" s="17" t="n">
+        <v>2933470.502684484</v>
+      </c>
+      <c r="F59" s="17" t="n">
+        <v>2280636.483432862</v>
+      </c>
+      <c r="G59" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H59" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I59" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
design: full UI overhaul — Inter font, richer palette, Net-hero summary, sexy benchmarks
- Full CSS rewrite: Inter 900 font, deeper dark palette (#05060c bg), indigo accents, subtle box-shadows
- Header now a floating card with gradient; live dot has glow animation
- Summary: Net is full-width hero card (32px, indigo gradient bg), Collateral + Debt smaller beneath with coloured value text
- Benchmark strip: 26px delta as hero with green/red text-shadow glow, % below, reference equity separated by border
- Table: backdrop-blur sticky header, row hover, cleaner borders, "Now" column distinctly styled
- Token group headers: 17px/900-weight; position sub-rows refined padding
- Wiped old snapshots; kept 2026-04-29T18-18-44Z as 12h reference; new snapshot is today's "now"

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O890"/>
+  <dimension ref="A1:O906"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -60442,6 +60442,1092 @@
         <v/>
       </c>
       <c r="O890" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:23:08</t>
+        </is>
+      </c>
+      <c r="B891" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C891" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D891" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E891" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F891" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G891" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H891" s="16" t="n">
+        <v>1.0505</v>
+      </c>
+      <c r="I891" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,804.5477</t>
+        </is>
+      </c>
+      <c r="J891" s="17" t="n">
+        <v>50783.71779845816</v>
+      </c>
+      <c r="K891" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,722.8797</t>
+        </is>
+      </c>
+      <c r="L891" s="17" t="n">
+        <v>37734.19994998499</v>
+      </c>
+      <c r="M891" s="17">
+        <f>J891-L891</f>
+        <v/>
+      </c>
+      <c r="N891" s="18">
+        <f>IF(J891=0,"",L891/J891)</f>
+        <v/>
+      </c>
+      <c r="O891" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:23:08</t>
+        </is>
+      </c>
+      <c r="B892" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C892" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D892" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E892" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F892" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G892" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H892" s="16" t="n">
+        <v>1.0482</v>
+      </c>
+      <c r="I892" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J892" s="17" t="n">
+        <v>140914.0860544015</v>
+      </c>
+      <c r="K892" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,035.0439</t>
+        </is>
+      </c>
+      <c r="L892" s="17" t="n">
+        <v>120985.4195589899</v>
+      </c>
+      <c r="M892" s="17">
+        <f>J892-L892</f>
+        <v/>
+      </c>
+      <c r="N892" s="18">
+        <f>IF(J892=0,"",L892/J892)</f>
+        <v/>
+      </c>
+      <c r="O892" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:23:08</t>
+        </is>
+      </c>
+      <c r="B893" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C893" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D893" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E893" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F893" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G893" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H893" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I893" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J893" s="17" t="n">
+        <v>328722.7664122585</v>
+      </c>
+      <c r="K893" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,386.0522</t>
+        </is>
+      </c>
+      <c r="L893" s="17" t="n">
+        <v>306484.5384353506</v>
+      </c>
+      <c r="M893" s="17">
+        <f>J893-L893</f>
+        <v/>
+      </c>
+      <c r="N893" s="18">
+        <f>IF(J893=0,"",L893/J893)</f>
+        <v/>
+      </c>
+      <c r="O893" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:23:08</t>
+        </is>
+      </c>
+      <c r="B894" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C894" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D894" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E894" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F894" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G894" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H894" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I894" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J894" s="17" t="n">
+        <v>386031.7581663539</v>
+      </c>
+      <c r="K894" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,608.2120</t>
+        </is>
+      </c>
+      <c r="L894" s="17" t="n">
+        <v>349720.5917915623</v>
+      </c>
+      <c r="M894" s="17">
+        <f>J894-L894</f>
+        <v/>
+      </c>
+      <c r="N894" s="18">
+        <f>IF(J894=0,"",L894/J894)</f>
+        <v/>
+      </c>
+      <c r="O894" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:23:08</t>
+        </is>
+      </c>
+      <c r="B895" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C895" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D895" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E895" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F895" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G895" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H895" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I895" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7848</t>
+        </is>
+      </c>
+      <c r="J895" s="17" t="n">
+        <v>77777.18564324616</v>
+      </c>
+      <c r="K895" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,028.1988; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L895" s="17" t="n">
+        <v>68000.38487074689</v>
+      </c>
+      <c r="M895" s="17">
+        <f>J895-L895</f>
+        <v/>
+      </c>
+      <c r="N895" s="18">
+        <f>IF(J895=0,"",L895/J895)</f>
+        <v/>
+      </c>
+      <c r="O895" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:23:08</t>
+        </is>
+      </c>
+      <c r="B896" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C896" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D896" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E896" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F896" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G896" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H896" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I896" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J896" s="17" t="n">
+        <v>197085.4740452354</v>
+      </c>
+      <c r="K896" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,243.9962</t>
+        </is>
+      </c>
+      <c r="L896" s="17" t="n">
+        <v>150289.0829716265</v>
+      </c>
+      <c r="M896" s="17">
+        <f>J896-L896</f>
+        <v/>
+      </c>
+      <c r="N896" s="18">
+        <f>IF(J896=0,"",L896/J896)</f>
+        <v/>
+      </c>
+      <c r="O896" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:23:08</t>
+        </is>
+      </c>
+      <c r="B897" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C897" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D897" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E897" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F897" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G897" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H897" s="16" t="n">
+        <v>1.3726</v>
+      </c>
+      <c r="I897" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J897" s="17" t="n">
+        <v>186067.338154978</v>
+      </c>
+      <c r="K897" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,140.3351</t>
+        </is>
+      </c>
+      <c r="L897" s="17" t="n">
+        <v>124177.588419594</v>
+      </c>
+      <c r="M897" s="17">
+        <f>J897-L897</f>
+        <v/>
+      </c>
+      <c r="N897" s="18">
+        <f>IF(J897=0,"",L897/J897)</f>
+        <v/>
+      </c>
+      <c r="O897" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:23:08</t>
+        </is>
+      </c>
+      <c r="B898" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C898" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D898" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E898" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F898" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G898" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H898" s="16" t="n">
+        <v>1.0655</v>
+      </c>
+      <c r="I898" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J898" s="17" t="n">
+        <v>327614.6310298509</v>
+      </c>
+      <c r="K898" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,285.9487</t>
+        </is>
+      </c>
+      <c r="L898" s="17" t="n">
+        <v>280242.0171559419</v>
+      </c>
+      <c r="M898" s="17">
+        <f>J898-L898</f>
+        <v/>
+      </c>
+      <c r="N898" s="18">
+        <f>IF(J898=0,"",L898/J898)</f>
+        <v/>
+      </c>
+      <c r="O898" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:23:08</t>
+        </is>
+      </c>
+      <c r="B899" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C899" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D899" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E899" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F899" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G899" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H899" s="16" t="n">
+        <v>1.9045</v>
+      </c>
+      <c r="I899" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J899" s="17" t="n">
+        <v>159989.8916291629</v>
+      </c>
+      <c r="K899" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,938.3760</t>
+        </is>
+      </c>
+      <c r="L899" s="17" t="n">
+        <v>70959.66389170298</v>
+      </c>
+      <c r="M899" s="17">
+        <f>J899-L899</f>
+        <v/>
+      </c>
+      <c r="N899" s="18">
+        <f>IF(J899=0,"",L899/J899)</f>
+        <v/>
+      </c>
+      <c r="O899" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:23:08</t>
+        </is>
+      </c>
+      <c r="B900" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C900" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D900" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E900" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F900" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G900" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H900" s="16" t="n">
+        <v>1.0574</v>
+      </c>
+      <c r="I900" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J900" s="17" t="n">
+        <v>160154.1307238079</v>
+      </c>
+      <c r="K900" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,523.0271</t>
+        </is>
+      </c>
+      <c r="L900" s="17" t="n">
+        <v>138509.1747529419</v>
+      </c>
+      <c r="M900" s="17">
+        <f>J900-L900</f>
+        <v/>
+      </c>
+      <c r="N900" s="18">
+        <f>IF(J900=0,"",L900/J900)</f>
+        <v/>
+      </c>
+      <c r="O900" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:23:08</t>
+        </is>
+      </c>
+      <c r="B901" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C901" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D901" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E901" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F901" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G901" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H901" s="16" t="inlineStr"/>
+      <c r="I901" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J901" s="17" t="n">
+        <v>95900.86515999959</v>
+      </c>
+      <c r="K901" s="15" t="inlineStr"/>
+      <c r="L901" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M901" s="17">
+        <f>J901-L901</f>
+        <v/>
+      </c>
+      <c r="N901" s="18">
+        <f>IF(J901=0,"",L901/J901)</f>
+        <v/>
+      </c>
+      <c r="O901" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:23:08</t>
+        </is>
+      </c>
+      <c r="B902" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C902" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D902" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E902" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F902" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G902" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H902" s="16" t="inlineStr"/>
+      <c r="I902" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J902" s="17" t="n">
+        <v>34359.15691838847</v>
+      </c>
+      <c r="K902" s="15" t="inlineStr"/>
+      <c r="L902" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M902" s="17">
+        <f>J902-L902</f>
+        <v/>
+      </c>
+      <c r="N902" s="18">
+        <f>IF(J902=0,"",L902/J902)</f>
+        <v/>
+      </c>
+      <c r="O902" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:23:08</t>
+        </is>
+      </c>
+      <c r="B903" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C903" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D903" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E903" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F903" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G903" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H903" s="16" t="n">
+        <v>1.0435</v>
+      </c>
+      <c r="I903" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J903" s="17" t="n">
+        <v>270078.0371332929</v>
+      </c>
+      <c r="K903" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,041.5307</t>
+        </is>
+      </c>
+      <c r="L903" s="17" t="n">
+        <v>232945.9836394265</v>
+      </c>
+      <c r="M903" s="17">
+        <f>J903-L903</f>
+        <v/>
+      </c>
+      <c r="N903" s="18">
+        <f>IF(J903=0,"",L903/J903)</f>
+        <v/>
+      </c>
+      <c r="O903" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:23:08</t>
+        </is>
+      </c>
+      <c r="B904" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C904" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D904" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E904" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F904" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G904" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H904" s="16" t="inlineStr"/>
+      <c r="I904" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,513.0398</t>
+        </is>
+      </c>
+      <c r="J904" s="17" t="n">
+        <v>15506.67948023723</v>
+      </c>
+      <c r="K904" s="15" t="inlineStr"/>
+      <c r="L904" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M904" s="17">
+        <f>J904-L904</f>
+        <v/>
+      </c>
+      <c r="N904" s="18">
+        <f>IF(J904=0,"",L904/J904)</f>
+        <v/>
+      </c>
+      <c r="O904" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:23:08</t>
+        </is>
+      </c>
+      <c r="B905" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C905" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D905" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E905" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F905" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G905" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H905" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I905" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J905" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K905" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L905" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M905" s="17">
+        <f>J905-L905</f>
+        <v/>
+      </c>
+      <c r="N905" s="18">
+        <f>IF(J905=0,"",L905/J905)</f>
+        <v/>
+      </c>
+      <c r="O905" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:23:08</t>
+        </is>
+      </c>
+      <c r="B906" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C906" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D906" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E906" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F906" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G906" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H906" s="16" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="I906" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J906" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K906" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,705.3454</t>
+        </is>
+      </c>
+      <c r="L906" s="17" t="n">
+        <v>148705.345409</v>
+      </c>
+      <c r="M906" s="17">
+        <f>J906-L906</f>
+        <v/>
+      </c>
+      <c r="N906" s="18">
+        <f>IF(J906=0,"",L906/J906)</f>
+        <v/>
+      </c>
+      <c r="O906" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -60472,7 +61558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I59"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -62553,6 +63639,41 @@
         <v>1.0375</v>
       </c>
       <c r="I59" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-29 18:23:08</t>
+        </is>
+      </c>
+      <c r="B60" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C60" s="17" t="n">
+        <v>655316.3879518792</v>
+      </c>
+      <c r="D60" s="17" t="n">
+        <v>652732.5609897533</v>
+      </c>
+      <c r="E60" s="17" t="n">
+        <v>2933469.098940622</v>
+      </c>
+      <c r="F60" s="17" t="n">
+        <v>2280736.537950868</v>
+      </c>
+      <c r="G60" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H60" s="16" t="n">
+        <v>1.0375</v>
+      </c>
+      <c r="I60" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-30 07:15 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O906"/>
+  <dimension ref="A1:O922"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -61528,6 +61528,1092 @@
         <v/>
       </c>
       <c r="O906" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:14:55</t>
+        </is>
+      </c>
+      <c r="B907" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C907" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D907" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E907" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F907" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G907" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H907" s="16" t="n">
+        <v>1.0503</v>
+      </c>
+      <c r="I907" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,809.3004</t>
+        </is>
+      </c>
+      <c r="J907" s="17" t="n">
+        <v>50790.50097384645</v>
+      </c>
+      <c r="K907" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,726.6826</t>
+        </is>
+      </c>
+      <c r="L907" s="17" t="n">
+        <v>37738.00397219165</v>
+      </c>
+      <c r="M907" s="17">
+        <f>J907-L907</f>
+        <v/>
+      </c>
+      <c r="N907" s="18">
+        <f>IF(J907=0,"",L907/J907)</f>
+        <v/>
+      </c>
+      <c r="O907" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:14:55</t>
+        </is>
+      </c>
+      <c r="B908" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C908" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D908" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E908" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F908" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G908" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H908" s="16" t="n">
+        <v>1.0484</v>
+      </c>
+      <c r="I908" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J908" s="17" t="n">
+        <v>140955.7120203578</v>
+      </c>
+      <c r="K908" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,048.3985</t>
+        </is>
+      </c>
+      <c r="L908" s="17" t="n">
+        <v>121003.6106105483</v>
+      </c>
+      <c r="M908" s="17">
+        <f>J908-L908</f>
+        <v/>
+      </c>
+      <c r="N908" s="18">
+        <f>IF(J908=0,"",L908/J908)</f>
+        <v/>
+      </c>
+      <c r="O908" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:14:55</t>
+        </is>
+      </c>
+      <c r="B909" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C909" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D909" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E909" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F909" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G909" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H909" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I909" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J909" s="17" t="n">
+        <v>328740.6274327308</v>
+      </c>
+      <c r="K909" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,401.0536</t>
+        </is>
+      </c>
+      <c r="L909" s="17" t="n">
+        <v>306531.1652357726</v>
+      </c>
+      <c r="M909" s="17">
+        <f>J909-L909</f>
+        <v/>
+      </c>
+      <c r="N909" s="18">
+        <f>IF(J909=0,"",L909/J909)</f>
+        <v/>
+      </c>
+      <c r="O909" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:14:55</t>
+        </is>
+      </c>
+      <c r="B910" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C910" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D910" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E910" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F910" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G910" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H910" s="16" t="n">
+        <v>1.0372</v>
+      </c>
+      <c r="I910" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J910" s="17" t="n">
+        <v>386062.4662431655</v>
+      </c>
+      <c r="K910" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,631.2289</t>
+        </is>
+      </c>
+      <c r="L910" s="17" t="n">
+        <v>349779.6979861511</v>
+      </c>
+      <c r="M910" s="17">
+        <f>J910-L910</f>
+        <v/>
+      </c>
+      <c r="N910" s="18">
+        <f>IF(J910=0,"",L910/J910)</f>
+        <v/>
+      </c>
+      <c r="O910" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:14:55</t>
+        </is>
+      </c>
+      <c r="B911" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C911" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D911" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E911" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F911" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G911" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H911" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I911" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7873</t>
+        </is>
+      </c>
+      <c r="J911" s="17" t="n">
+        <v>77785.00670756861</v>
+      </c>
+      <c r="K911" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,034.4625; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L911" s="17" t="n">
+        <v>68009.3673751381</v>
+      </c>
+      <c r="M911" s="17">
+        <f>J911-L911</f>
+        <v/>
+      </c>
+      <c r="N911" s="18">
+        <f>IF(J911=0,"",L911/J911)</f>
+        <v/>
+      </c>
+      <c r="O911" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:14:55</t>
+        </is>
+      </c>
+      <c r="B912" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C912" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D912" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E912" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F912" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G912" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H912" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I912" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J912" s="17" t="n">
+        <v>197111.8925150287</v>
+      </c>
+      <c r="K912" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,262.3037</t>
+        </is>
+      </c>
+      <c r="L912" s="17" t="n">
+        <v>150307.3959050264</v>
+      </c>
+      <c r="M912" s="17">
+        <f>J912-L912</f>
+        <v/>
+      </c>
+      <c r="N912" s="18">
+        <f>IF(J912=0,"",L912/J912)</f>
+        <v/>
+      </c>
+      <c r="O912" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:14:55</t>
+        </is>
+      </c>
+      <c r="B913" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C913" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D913" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E913" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F913" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G913" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H913" s="16" t="n">
+        <v>1.3728</v>
+      </c>
+      <c r="I913" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J913" s="17" t="n">
+        <v>186173.1282908512</v>
+      </c>
+      <c r="K913" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,161.1962</t>
+        </is>
+      </c>
+      <c r="L913" s="17" t="n">
+        <v>124198.4557182379</v>
+      </c>
+      <c r="M913" s="17">
+        <f>J913-L913</f>
+        <v/>
+      </c>
+      <c r="N913" s="18">
+        <f>IF(J913=0,"",L913/J913)</f>
+        <v/>
+      </c>
+      <c r="O913" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:14:55</t>
+        </is>
+      </c>
+      <c r="B914" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C914" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D914" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E914" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F914" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G914" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H914" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I914" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J914" s="17" t="n">
+        <v>327683.3742113973</v>
+      </c>
+      <c r="K914" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,363.1264</t>
+        </is>
+      </c>
+      <c r="L914" s="17" t="n">
+        <v>280190.3302679426</v>
+      </c>
+      <c r="M914" s="17">
+        <f>J914-L914</f>
+        <v/>
+      </c>
+      <c r="N914" s="18">
+        <f>IF(J914=0,"",L914/J914)</f>
+        <v/>
+      </c>
+      <c r="O914" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:14:55</t>
+        </is>
+      </c>
+      <c r="B915" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C915" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D915" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E915" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F915" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G915" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H915" s="16" t="n">
+        <v>1.9047</v>
+      </c>
+      <c r="I915" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J915" s="17" t="n">
+        <v>160052.5364672934</v>
+      </c>
+      <c r="K915" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,952.6109</t>
+        </is>
+      </c>
+      <c r="L915" s="17" t="n">
+        <v>70973.90309838159</v>
+      </c>
+      <c r="M915" s="17">
+        <f>J915-L915</f>
+        <v/>
+      </c>
+      <c r="N915" s="18">
+        <f>IF(J915=0,"",L915/J915)</f>
+        <v/>
+      </c>
+      <c r="O915" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:14:55</t>
+        </is>
+      </c>
+      <c r="B916" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C916" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D916" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E916" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F916" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G916" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H916" s="16" t="n">
+        <v>1.0571</v>
+      </c>
+      <c r="I916" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J916" s="17" t="n">
+        <v>160166.8706739387</v>
+      </c>
+      <c r="K916" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,532.9072</t>
+        </is>
+      </c>
+      <c r="L916" s="17" t="n">
+        <v>138546.760445046</v>
+      </c>
+      <c r="M916" s="17">
+        <f>J916-L916</f>
+        <v/>
+      </c>
+      <c r="N916" s="18">
+        <f>IF(J916=0,"",L916/J916)</f>
+        <v/>
+      </c>
+      <c r="O916" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:14:55</t>
+        </is>
+      </c>
+      <c r="B917" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C917" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D917" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E917" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F917" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G917" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H917" s="16" t="inlineStr"/>
+      <c r="I917" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J917" s="17" t="n">
+        <v>95931.46061354708</v>
+      </c>
+      <c r="K917" s="15" t="inlineStr"/>
+      <c r="L917" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M917" s="17">
+        <f>J917-L917</f>
+        <v/>
+      </c>
+      <c r="N917" s="18">
+        <f>IF(J917=0,"",L917/J917)</f>
+        <v/>
+      </c>
+      <c r="O917" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:14:55</t>
+        </is>
+      </c>
+      <c r="B918" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C918" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D918" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E918" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F918" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G918" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H918" s="16" t="inlineStr"/>
+      <c r="I918" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J918" s="17" t="n">
+        <v>34365.76460894049</v>
+      </c>
+      <c r="K918" s="15" t="inlineStr"/>
+      <c r="L918" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M918" s="17">
+        <f>J918-L918</f>
+        <v/>
+      </c>
+      <c r="N918" s="18">
+        <f>IF(J918=0,"",L918/J918)</f>
+        <v/>
+      </c>
+      <c r="O918" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:14:55</t>
+        </is>
+      </c>
+      <c r="B919" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C919" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D919" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E919" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F919" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G919" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H919" s="16" t="n">
+        <v>1.0432</v>
+      </c>
+      <c r="I919" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J919" s="17" t="n">
+        <v>270055.1826497763</v>
+      </c>
+      <c r="K919" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,071.2752</t>
+        </is>
+      </c>
+      <c r="L919" s="17" t="n">
+        <v>232985.0388701605</v>
+      </c>
+      <c r="M919" s="17">
+        <f>J919-L919</f>
+        <v/>
+      </c>
+      <c r="N919" s="18">
+        <f>IF(J919=0,"",L919/J919)</f>
+        <v/>
+      </c>
+      <c r="O919" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:14:55</t>
+        </is>
+      </c>
+      <c r="B920" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C920" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D920" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E920" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F920" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G920" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H920" s="16" t="inlineStr"/>
+      <c r="I920" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,518.2957</t>
+        </is>
+      </c>
+      <c r="J920" s="17" t="n">
+        <v>15512.55397220953</v>
+      </c>
+      <c r="K920" s="15" t="inlineStr"/>
+      <c r="L920" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M920" s="17">
+        <f>J920-L920</f>
+        <v/>
+      </c>
+      <c r="N920" s="18">
+        <f>IF(J920=0,"",L920/J920)</f>
+        <v/>
+      </c>
+      <c r="O920" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:14:55</t>
+        </is>
+      </c>
+      <c r="B921" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C921" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D921" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E921" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F921" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G921" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H921" s="16" t="n">
+        <v>1.219</v>
+      </c>
+      <c r="I921" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J921" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K921" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,736.3177</t>
+        </is>
+      </c>
+      <c r="L921" s="17" t="n">
+        <v>148736.317674</v>
+      </c>
+      <c r="M921" s="17">
+        <f>J921-L921</f>
+        <v/>
+      </c>
+      <c r="N921" s="18">
+        <f>IF(J921=0,"",L921/J921)</f>
+        <v/>
+      </c>
+      <c r="O921" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:14:55</t>
+        </is>
+      </c>
+      <c r="B922" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C922" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D922" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E922" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F922" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G922" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H922" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I922" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J922" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K922" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L922" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M922" s="17">
+        <f>J922-L922</f>
+        <v/>
+      </c>
+      <c r="N922" s="18">
+        <f>IF(J922=0,"",L922/J922)</f>
+        <v/>
+      </c>
+      <c r="O922" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -61558,7 +62644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I61"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -63674,6 +64760,41 @@
         <v>1.0375</v>
       </c>
       <c r="I60" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:14:55</t>
+        </is>
+      </c>
+      <c r="B61" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C61" s="17" t="n">
+        <v>655475.4244060988</v>
+      </c>
+      <c r="D61" s="17" t="n">
+        <v>652887.8637090041</v>
+      </c>
+      <c r="E61" s="17" t="n">
+        <v>2933870.457971601</v>
+      </c>
+      <c r="F61" s="17" t="n">
+        <v>2280982.594262597</v>
+      </c>
+      <c r="G61" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H61" s="16" t="n">
+        <v>1.0372</v>
+      </c>
+      <c r="I61" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-30 07:45 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O922"/>
+  <dimension ref="A1:O938"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -62614,6 +62614,1092 @@
         <v/>
       </c>
       <c r="O922" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:45:05</t>
+        </is>
+      </c>
+      <c r="B923" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C923" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D923" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E923" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F923" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G923" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H923" s="16" t="n">
+        <v>1.0503</v>
+      </c>
+      <c r="I923" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,809.3004</t>
+        </is>
+      </c>
+      <c r="J923" s="17" t="n">
+        <v>50788.46860182985</v>
+      </c>
+      <c r="K923" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,726.6826</t>
+        </is>
+      </c>
+      <c r="L923" s="17" t="n">
+        <v>37738.00397219165</v>
+      </c>
+      <c r="M923" s="17">
+        <f>J923-L923</f>
+        <v/>
+      </c>
+      <c r="N923" s="18">
+        <f>IF(J923=0,"",L923/J923)</f>
+        <v/>
+      </c>
+      <c r="O923" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:45:05</t>
+        </is>
+      </c>
+      <c r="B924" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C924" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D924" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E924" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F924" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G924" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H924" s="16" t="n">
+        <v>1.0484</v>
+      </c>
+      <c r="I924" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J924" s="17" t="n">
+        <v>140955.9876492349</v>
+      </c>
+      <c r="K924" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,048.3985</t>
+        </is>
+      </c>
+      <c r="L924" s="17" t="n">
+        <v>120998.7686746076</v>
+      </c>
+      <c r="M924" s="17">
+        <f>J924-L924</f>
+        <v/>
+      </c>
+      <c r="N924" s="18">
+        <f>IF(J924=0,"",L924/J924)</f>
+        <v/>
+      </c>
+      <c r="O924" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:45:05</t>
+        </is>
+      </c>
+      <c r="B925" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C925" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D925" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E925" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F925" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G925" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H925" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I925" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J925" s="17" t="n">
+        <v>328740.8667247219</v>
+      </c>
+      <c r="K925" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,401.0536</t>
+        </is>
+      </c>
+      <c r="L925" s="17" t="n">
+        <v>306500.4775334485</v>
+      </c>
+      <c r="M925" s="17">
+        <f>J925-L925</f>
+        <v/>
+      </c>
+      <c r="N925" s="18">
+        <f>IF(J925=0,"",L925/J925)</f>
+        <v/>
+      </c>
+      <c r="O925" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:45:05</t>
+        </is>
+      </c>
+      <c r="B926" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C926" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D926" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E926" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F926" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G926" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H926" s="16" t="n">
+        <v>1.0372</v>
+      </c>
+      <c r="I926" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J926" s="17" t="n">
+        <v>386063.6218422574</v>
+      </c>
+      <c r="K926" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,631.2289</t>
+        </is>
+      </c>
+      <c r="L926" s="17" t="n">
+        <v>349744.6805508359</v>
+      </c>
+      <c r="M926" s="17">
+        <f>J926-L926</f>
+        <v/>
+      </c>
+      <c r="N926" s="18">
+        <f>IF(J926=0,"",L926/J926)</f>
+        <v/>
+      </c>
+      <c r="O926" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:45:05</t>
+        </is>
+      </c>
+      <c r="B927" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C927" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D927" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E927" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F927" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G927" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H927" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I927" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7873</t>
+        </is>
+      </c>
+      <c r="J927" s="17" t="n">
+        <v>77788.19028449581</v>
+      </c>
+      <c r="K927" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,034.4625; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L927" s="17" t="n">
+        <v>68006.64599663661</v>
+      </c>
+      <c r="M927" s="17">
+        <f>J927-L927</f>
+        <v/>
+      </c>
+      <c r="N927" s="18">
+        <f>IF(J927=0,"",L927/J927)</f>
+        <v/>
+      </c>
+      <c r="O927" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:45:05</t>
+        </is>
+      </c>
+      <c r="B928" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C928" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D928" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E928" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F928" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G928" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H928" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I928" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J928" s="17" t="n">
+        <v>197114.343518233</v>
+      </c>
+      <c r="K928" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,262.3037</t>
+        </is>
+      </c>
+      <c r="L928" s="17" t="n">
+        <v>150307.3959050264</v>
+      </c>
+      <c r="M928" s="17">
+        <f>J928-L928</f>
+        <v/>
+      </c>
+      <c r="N928" s="18">
+        <f>IF(J928=0,"",L928/J928)</f>
+        <v/>
+      </c>
+      <c r="O928" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:45:05</t>
+        </is>
+      </c>
+      <c r="B929" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C929" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D929" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E929" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F929" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G929" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H929" s="16" t="n">
+        <v>1.3728</v>
+      </c>
+      <c r="I929" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J929" s="17" t="n">
+        <v>186154.9476937829</v>
+      </c>
+      <c r="K929" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,161.1962</t>
+        </is>
+      </c>
+      <c r="L929" s="17" t="n">
+        <v>124198.4557182379</v>
+      </c>
+      <c r="M929" s="17">
+        <f>J929-L929</f>
+        <v/>
+      </c>
+      <c r="N929" s="18">
+        <f>IF(J929=0,"",L929/J929)</f>
+        <v/>
+      </c>
+      <c r="O929" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:45:05</t>
+        </is>
+      </c>
+      <c r="B930" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C930" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D930" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E930" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F930" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G930" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H930" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I930" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J930" s="17" t="n">
+        <v>327677.0126871585</v>
+      </c>
+      <c r="K930" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,363.1264</t>
+        </is>
+      </c>
+      <c r="L930" s="17" t="n">
+        <v>280196.2998697055</v>
+      </c>
+      <c r="M930" s="17">
+        <f>J930-L930</f>
+        <v/>
+      </c>
+      <c r="N930" s="18">
+        <f>IF(J930=0,"",L930/J930)</f>
+        <v/>
+      </c>
+      <c r="O930" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:45:05</t>
+        </is>
+      </c>
+      <c r="B931" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C931" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D931" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E931" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F931" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G931" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H931" s="16" t="n">
+        <v>1.9047</v>
+      </c>
+      <c r="I931" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J931" s="17" t="n">
+        <v>160052.5364672934</v>
+      </c>
+      <c r="K931" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,952.6109</t>
+        </is>
+      </c>
+      <c r="L931" s="17" t="n">
+        <v>70973.90309838159</v>
+      </c>
+      <c r="M931" s="17">
+        <f>J931-L931</f>
+        <v/>
+      </c>
+      <c r="N931" s="18">
+        <f>IF(J931=0,"",L931/J931)</f>
+        <v/>
+      </c>
+      <c r="O931" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:45:05</t>
+        </is>
+      </c>
+      <c r="B932" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C932" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D932" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E932" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F932" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G932" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H932" s="16" t="n">
+        <v>1.0571</v>
+      </c>
+      <c r="I932" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J932" s="17" t="n">
+        <v>160167.3501007323</v>
+      </c>
+      <c r="K932" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,532.9072</t>
+        </is>
+      </c>
+      <c r="L932" s="17" t="n">
+        <v>138546.760445046</v>
+      </c>
+      <c r="M932" s="17">
+        <f>J932-L932</f>
+        <v/>
+      </c>
+      <c r="N932" s="18">
+        <f>IF(J932=0,"",L932/J932)</f>
+        <v/>
+      </c>
+      <c r="O932" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:45:05</t>
+        </is>
+      </c>
+      <c r="B933" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C933" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D933" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E933" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F933" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G933" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H933" s="16" t="inlineStr"/>
+      <c r="I933" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J933" s="17" t="n">
+        <v>95941.01062848924</v>
+      </c>
+      <c r="K933" s="15" t="inlineStr"/>
+      <c r="L933" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M933" s="17">
+        <f>J933-L933</f>
+        <v/>
+      </c>
+      <c r="N933" s="18">
+        <f>IF(J933=0,"",L933/J933)</f>
+        <v/>
+      </c>
+      <c r="O933" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:45:05</t>
+        </is>
+      </c>
+      <c r="B934" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C934" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D934" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E934" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F934" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G934" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H934" s="16" t="inlineStr"/>
+      <c r="I934" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J934" s="17" t="n">
+        <v>34366.06616276463</v>
+      </c>
+      <c r="K934" s="15" t="inlineStr"/>
+      <c r="L934" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M934" s="17">
+        <f>J934-L934</f>
+        <v/>
+      </c>
+      <c r="N934" s="18">
+        <f>IF(J934=0,"",L934/J934)</f>
+        <v/>
+      </c>
+      <c r="O934" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:45:05</t>
+        </is>
+      </c>
+      <c r="B935" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C935" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D935" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E935" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F935" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G935" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H935" s="16" t="n">
+        <v>1.0432</v>
+      </c>
+      <c r="I935" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J935" s="17" t="n">
+        <v>270055.1826497763</v>
+      </c>
+      <c r="K935" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,071.2752</t>
+        </is>
+      </c>
+      <c r="L935" s="17" t="n">
+        <v>232975.7160191508</v>
+      </c>
+      <c r="M935" s="17">
+        <f>J935-L935</f>
+        <v/>
+      </c>
+      <c r="N935" s="18">
+        <f>IF(J935=0,"",L935/J935)</f>
+        <v/>
+      </c>
+      <c r="O935" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:45:05</t>
+        </is>
+      </c>
+      <c r="B936" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C936" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D936" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E936" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F936" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G936" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H936" s="16" t="inlineStr"/>
+      <c r="I936" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,518.4862</t>
+        </is>
+      </c>
+      <c r="J936" s="17" t="n">
+        <v>15512.12362492039</v>
+      </c>
+      <c r="K936" s="15" t="inlineStr"/>
+      <c r="L936" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M936" s="17">
+        <f>J936-L936</f>
+        <v/>
+      </c>
+      <c r="N936" s="18">
+        <f>IF(J936=0,"",L936/J936)</f>
+        <v/>
+      </c>
+      <c r="O936" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:45:05</t>
+        </is>
+      </c>
+      <c r="B937" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C937" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D937" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E937" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F937" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G937" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H937" s="16" t="n">
+        <v>1.219</v>
+      </c>
+      <c r="I937" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J937" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K937" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,736.3177</t>
+        </is>
+      </c>
+      <c r="L937" s="17" t="n">
+        <v>148736.317674</v>
+      </c>
+      <c r="M937" s="17">
+        <f>J937-L937</f>
+        <v/>
+      </c>
+      <c r="N937" s="18">
+        <f>IF(J937=0,"",L937/J937)</f>
+        <v/>
+      </c>
+      <c r="O937" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:45:05</t>
+        </is>
+      </c>
+      <c r="B938" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C938" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D938" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E938" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F938" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G938" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H938" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I938" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J938" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K938" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L938" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M938" s="17">
+        <f>J938-L938</f>
+        <v/>
+      </c>
+      <c r="N938" s="18">
+        <f>IF(J938=0,"",L938/J938)</f>
+        <v/>
+      </c>
+      <c r="O938" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -62644,7 +63730,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I61"/>
+  <dimension ref="A1:I62"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -64795,6 +65881,41 @@
         <v>1.0372</v>
       </c>
       <c r="I61" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:45:05</t>
+        </is>
+      </c>
+      <c r="B62" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C62" s="17" t="n">
+        <v>655542.9448781918</v>
+      </c>
+      <c r="D62" s="17" t="n">
+        <v>652955.1166653717</v>
+      </c>
+      <c r="E62" s="17" t="n">
+        <v>2933861.08922664</v>
+      </c>
+      <c r="F62" s="17" t="n">
+        <v>2280905.972561269</v>
+      </c>
+      <c r="G62" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H62" s="16" t="n">
+        <v>1.0372</v>
+      </c>
+      <c r="I62" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-30 07:55 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O938"/>
+  <dimension ref="A1:O954"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -63700,6 +63700,1092 @@
         <v/>
       </c>
       <c r="O938" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:55:13</t>
+        </is>
+      </c>
+      <c r="B939" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C939" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D939" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E939" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F939" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G939" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H939" s="16" t="n">
+        <v>1.0503</v>
+      </c>
+      <c r="I939" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,809.3004</t>
+        </is>
+      </c>
+      <c r="J939" s="17" t="n">
+        <v>50788.976694834</v>
+      </c>
+      <c r="K939" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,726.6826</t>
+        </is>
+      </c>
+      <c r="L939" s="17" t="n">
+        <v>37738.00397219165</v>
+      </c>
+      <c r="M939" s="17">
+        <f>J939-L939</f>
+        <v/>
+      </c>
+      <c r="N939" s="18">
+        <f>IF(J939=0,"",L939/J939)</f>
+        <v/>
+      </c>
+      <c r="O939" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:55:13</t>
+        </is>
+      </c>
+      <c r="B940" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C940" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D940" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E940" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F940" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G940" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H940" s="16" t="n">
+        <v>1.0484</v>
+      </c>
+      <c r="I940" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J940" s="17" t="n">
+        <v>140955.9876492349</v>
+      </c>
+      <c r="K940" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,048.3985</t>
+        </is>
+      </c>
+      <c r="L940" s="17" t="n">
+        <v>120999.9791585928</v>
+      </c>
+      <c r="M940" s="17">
+        <f>J940-L940</f>
+        <v/>
+      </c>
+      <c r="N940" s="18">
+        <f>IF(J940=0,"",L940/J940)</f>
+        <v/>
+      </c>
+      <c r="O940" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="941">
+      <c r="A941" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:55:13</t>
+        </is>
+      </c>
+      <c r="B941" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C941" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D941" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E941" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F941" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G941" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H941" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I941" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J941" s="17" t="n">
+        <v>328741.2352347289</v>
+      </c>
+      <c r="K941" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,401.0536</t>
+        </is>
+      </c>
+      <c r="L941" s="17" t="n">
+        <v>306531.1367789755</v>
+      </c>
+      <c r="M941" s="17">
+        <f>J941-L941</f>
+        <v/>
+      </c>
+      <c r="N941" s="18">
+        <f>IF(J941=0,"",L941/J941)</f>
+        <v/>
+      </c>
+      <c r="O941" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:55:13</t>
+        </is>
+      </c>
+      <c r="B942" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C942" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D942" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E942" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F942" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G942" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H942" s="16" t="n">
+        <v>1.0372</v>
+      </c>
+      <c r="I942" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J942" s="17" t="n">
+        <v>386062.8745418107</v>
+      </c>
+      <c r="K942" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,631.2289</t>
+        </is>
+      </c>
+      <c r="L942" s="17" t="n">
+        <v>349779.66551438</v>
+      </c>
+      <c r="M942" s="17">
+        <f>J942-L942</f>
+        <v/>
+      </c>
+      <c r="N942" s="18">
+        <f>IF(J942=0,"",L942/J942)</f>
+        <v/>
+      </c>
+      <c r="O942" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:55:13</t>
+        </is>
+      </c>
+      <c r="B943" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C943" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D943" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E943" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F943" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G943" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H943" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I943" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7873</t>
+        </is>
+      </c>
+      <c r="J943" s="17" t="n">
+        <v>77782.75502763505</v>
+      </c>
+      <c r="K943" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,034.4625; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L943" s="17" t="n">
+        <v>68007.32634126199</v>
+      </c>
+      <c r="M943" s="17">
+        <f>J943-L943</f>
+        <v/>
+      </c>
+      <c r="N943" s="18">
+        <f>IF(J943=0,"",L943/J943)</f>
+        <v/>
+      </c>
+      <c r="O943" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:55:13</t>
+        </is>
+      </c>
+      <c r="B944" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C944" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D944" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E944" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F944" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G944" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H944" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I944" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J944" s="17" t="n">
+        <v>197115.1295021415</v>
+      </c>
+      <c r="K944" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,262.3037</t>
+        </is>
+      </c>
+      <c r="L944" s="17" t="n">
+        <v>150307.3959050264</v>
+      </c>
+      <c r="M944" s="17">
+        <f>J944-L944</f>
+        <v/>
+      </c>
+      <c r="N944" s="18">
+        <f>IF(J944=0,"",L944/J944)</f>
+        <v/>
+      </c>
+      <c r="O944" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:55:13</t>
+        </is>
+      </c>
+      <c r="B945" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C945" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D945" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E945" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F945" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G945" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H945" s="16" t="n">
+        <v>1.3728</v>
+      </c>
+      <c r="I945" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J945" s="17" t="n">
+        <v>186124.1498384148</v>
+      </c>
+      <c r="K945" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,161.1962</t>
+        </is>
+      </c>
+      <c r="L945" s="17" t="n">
+        <v>124198.4557182379</v>
+      </c>
+      <c r="M945" s="17">
+        <f>J945-L945</f>
+        <v/>
+      </c>
+      <c r="N945" s="18">
+        <f>IF(J945=0,"",L945/J945)</f>
+        <v/>
+      </c>
+      <c r="O945" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:55:13</t>
+        </is>
+      </c>
+      <c r="B946" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C946" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D946" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E946" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F946" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G946" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H946" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I946" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J946" s="17" t="n">
+        <v>327677.0126871585</v>
+      </c>
+      <c r="K946" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,363.1264</t>
+        </is>
+      </c>
+      <c r="L946" s="17" t="n">
+        <v>280199.3605466958</v>
+      </c>
+      <c r="M946" s="17">
+        <f>J946-L946</f>
+        <v/>
+      </c>
+      <c r="N946" s="18">
+        <f>IF(J946=0,"",L946/J946)</f>
+        <v/>
+      </c>
+      <c r="O946" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:55:13</t>
+        </is>
+      </c>
+      <c r="B947" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C947" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D947" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E947" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F947" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G947" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H947" s="16" t="n">
+        <v>1.9047</v>
+      </c>
+      <c r="I947" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J947" s="17" t="n">
+        <v>160052.5364672934</v>
+      </c>
+      <c r="K947" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,952.6109</t>
+        </is>
+      </c>
+      <c r="L947" s="17" t="n">
+        <v>70973.90309838159</v>
+      </c>
+      <c r="M947" s="17">
+        <f>J947-L947</f>
+        <v/>
+      </c>
+      <c r="N947" s="18">
+        <f>IF(J947=0,"",L947/J947)</f>
+        <v/>
+      </c>
+      <c r="O947" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="948">
+      <c r="A948" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:55:13</t>
+        </is>
+      </c>
+      <c r="B948" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C948" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D948" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E948" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F948" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G948" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H948" s="16" t="n">
+        <v>1.0571</v>
+      </c>
+      <c r="I948" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J948" s="17" t="n">
+        <v>160167.0400659983</v>
+      </c>
+      <c r="K948" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,532.9072</t>
+        </is>
+      </c>
+      <c r="L948" s="17" t="n">
+        <v>138546.760445046</v>
+      </c>
+      <c r="M948" s="17">
+        <f>J948-L948</f>
+        <v/>
+      </c>
+      <c r="N948" s="18">
+        <f>IF(J948=0,"",L948/J948)</f>
+        <v/>
+      </c>
+      <c r="O948" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:55:13</t>
+        </is>
+      </c>
+      <c r="B949" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C949" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D949" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E949" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F949" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G949" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H949" s="16" t="inlineStr"/>
+      <c r="I949" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J949" s="17" t="n">
+        <v>95925.04792842484</v>
+      </c>
+      <c r="K949" s="15" t="inlineStr"/>
+      <c r="L949" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M949" s="17">
+        <f>J949-L949</f>
+        <v/>
+      </c>
+      <c r="N949" s="18">
+        <f>IF(J949=0,"",L949/J949)</f>
+        <v/>
+      </c>
+      <c r="O949" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:55:13</t>
+        </is>
+      </c>
+      <c r="B950" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C950" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D950" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E950" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F950" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G950" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H950" s="16" t="inlineStr"/>
+      <c r="I950" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J950" s="17" t="n">
+        <v>34366.16547747757</v>
+      </c>
+      <c r="K950" s="15" t="inlineStr"/>
+      <c r="L950" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M950" s="17">
+        <f>J950-L950</f>
+        <v/>
+      </c>
+      <c r="N950" s="18">
+        <f>IF(J950=0,"",L950/J950)</f>
+        <v/>
+      </c>
+      <c r="O950" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:55:13</t>
+        </is>
+      </c>
+      <c r="B951" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C951" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D951" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E951" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F951" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G951" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H951" s="16" t="n">
+        <v>1.0432</v>
+      </c>
+      <c r="I951" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J951" s="17" t="n">
+        <v>270055.1826497763</v>
+      </c>
+      <c r="K951" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,071.2752</t>
+        </is>
+      </c>
+      <c r="L951" s="17" t="n">
+        <v>232978.0467319032</v>
+      </c>
+      <c r="M951" s="17">
+        <f>J951-L951</f>
+        <v/>
+      </c>
+      <c r="N951" s="18">
+        <f>IF(J951=0,"",L951/J951)</f>
+        <v/>
+      </c>
+      <c r="O951" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:55:13</t>
+        </is>
+      </c>
+      <c r="B952" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C952" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D952" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E952" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F952" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G952" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H952" s="16" t="inlineStr"/>
+      <c r="I952" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,518.4862</t>
+        </is>
+      </c>
+      <c r="J952" s="17" t="n">
+        <v>15512.27880978244</v>
+      </c>
+      <c r="K952" s="15" t="inlineStr"/>
+      <c r="L952" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M952" s="17">
+        <f>J952-L952</f>
+        <v/>
+      </c>
+      <c r="N952" s="18">
+        <f>IF(J952=0,"",L952/J952)</f>
+        <v/>
+      </c>
+      <c r="O952" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:55:13</t>
+        </is>
+      </c>
+      <c r="B953" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C953" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D953" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E953" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F953" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G953" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H953" s="16" t="n">
+        <v>1.219</v>
+      </c>
+      <c r="I953" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J953" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K953" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,736.3177</t>
+        </is>
+      </c>
+      <c r="L953" s="17" t="n">
+        <v>148736.317674</v>
+      </c>
+      <c r="M953" s="17">
+        <f>J953-L953</f>
+        <v/>
+      </c>
+      <c r="N953" s="18">
+        <f>IF(J953=0,"",L953/J953)</f>
+        <v/>
+      </c>
+      <c r="O953" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:55:13</t>
+        </is>
+      </c>
+      <c r="B954" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C954" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D954" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E954" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F954" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G954" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H954" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I954" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J954" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K954" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L954" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M954" s="17">
+        <f>J954-L954</f>
+        <v/>
+      </c>
+      <c r="N954" s="18">
+        <f>IF(J954=0,"",L954/J954)</f>
+        <v/>
+      </c>
+      <c r="O954" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -63730,7 +64816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I62"/>
+  <dimension ref="A1:I63"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -65916,6 +67002,41 @@
         <v>1.0372</v>
       </c>
       <c r="I62" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 07:55:13</t>
+        </is>
+      </c>
+      <c r="B63" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C63" s="17" t="n">
+        <v>655418.6316544042</v>
+      </c>
+      <c r="D63" s="17" t="n">
+        <v>652830.8541769683</v>
+      </c>
+      <c r="E63" s="17" t="n">
+        <v>2933809.753165661</v>
+      </c>
+      <c r="F63" s="17" t="n">
+        <v>2280978.898988693</v>
+      </c>
+      <c r="G63" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H63" s="16" t="n">
+        <v>1.0372</v>
+      </c>
+      <c r="I63" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-30 08:15 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O954"/>
+  <dimension ref="A1:O970"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -64786,6 +64786,1092 @@
         <v/>
       </c>
       <c r="O954" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:15:18</t>
+        </is>
+      </c>
+      <c r="B955" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C955" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D955" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E955" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F955" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G955" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H955" s="16" t="n">
+        <v>1.0503</v>
+      </c>
+      <c r="I955" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,809.3004</t>
+        </is>
+      </c>
+      <c r="J955" s="17" t="n">
+        <v>50789.99288084229</v>
+      </c>
+      <c r="K955" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,726.6826</t>
+        </is>
+      </c>
+      <c r="L955" s="17" t="n">
+        <v>37741.77928271308</v>
+      </c>
+      <c r="M955" s="17">
+        <f>J955-L955</f>
+        <v/>
+      </c>
+      <c r="N955" s="18">
+        <f>IF(J955=0,"",L955/J955)</f>
+        <v/>
+      </c>
+      <c r="O955" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:15:18</t>
+        </is>
+      </c>
+      <c r="B956" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C956" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D956" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E956" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F956" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G956" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H956" s="16" t="n">
+        <v>1.0483</v>
+      </c>
+      <c r="I956" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J956" s="17" t="n">
+        <v>140942.3082907065</v>
+      </c>
+      <c r="K956" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,048.3985</t>
+        </is>
+      </c>
+      <c r="L956" s="17" t="n">
+        <v>121002.4001265632</v>
+      </c>
+      <c r="M956" s="17">
+        <f>J956-L956</f>
+        <v/>
+      </c>
+      <c r="N956" s="18">
+        <f>IF(J956=0,"",L956/J956)</f>
+        <v/>
+      </c>
+      <c r="O956" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:15:18</t>
+        </is>
+      </c>
+      <c r="B957" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C957" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D957" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E957" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F957" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G957" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H957" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I957" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J957" s="17" t="n">
+        <v>328741.2352347289</v>
+      </c>
+      <c r="K957" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,401.0536</t>
+        </is>
+      </c>
+      <c r="L957" s="17" t="n">
+        <v>306531.1771745897</v>
+      </c>
+      <c r="M957" s="17">
+        <f>J957-L957</f>
+        <v/>
+      </c>
+      <c r="N957" s="18">
+        <f>IF(J957=0,"",L957/J957)</f>
+        <v/>
+      </c>
+      <c r="O957" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:15:18</t>
+        </is>
+      </c>
+      <c r="B958" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C958" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D958" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E958" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F958" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G958" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H958" s="16" t="n">
+        <v>1.0372</v>
+      </c>
+      <c r="I958" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J958" s="17" t="n">
+        <v>386064.779258224</v>
+      </c>
+      <c r="K958" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,631.2289</t>
+        </is>
+      </c>
+      <c r="L958" s="17" t="n">
+        <v>349779.711609418</v>
+      </c>
+      <c r="M958" s="17">
+        <f>J958-L958</f>
+        <v/>
+      </c>
+      <c r="N958" s="18">
+        <f>IF(J958=0,"",L958/J958)</f>
+        <v/>
+      </c>
+      <c r="O958" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:15:18</t>
+        </is>
+      </c>
+      <c r="B959" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C959" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D959" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E959" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F959" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G959" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H959" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I959" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7873</t>
+        </is>
+      </c>
+      <c r="J959" s="17" t="n">
+        <v>77782.71297977063</v>
+      </c>
+      <c r="K959" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,034.4625; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L959" s="17" t="n">
+        <v>68008.68703827476</v>
+      </c>
+      <c r="M959" s="17">
+        <f>J959-L959</f>
+        <v/>
+      </c>
+      <c r="N959" s="18">
+        <f>IF(J959=0,"",L959/J959)</f>
+        <v/>
+      </c>
+      <c r="O959" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:15:18</t>
+        </is>
+      </c>
+      <c r="B960" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C960" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D960" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E960" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F960" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G960" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H960" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I960" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J960" s="17" t="n">
+        <v>197125.002609238</v>
+      </c>
+      <c r="K960" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,262.3037</t>
+        </is>
+      </c>
+      <c r="L960" s="17" t="n">
+        <v>150322.4326593186</v>
+      </c>
+      <c r="M960" s="17">
+        <f>J960-L960</f>
+        <v/>
+      </c>
+      <c r="N960" s="18">
+        <f>IF(J960=0,"",L960/J960)</f>
+        <v/>
+      </c>
+      <c r="O960" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:15:18</t>
+        </is>
+      </c>
+      <c r="B961" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C961" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D961" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E961" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F961" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G961" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H961" s="16" t="n">
+        <v>1.3728</v>
+      </c>
+      <c r="I961" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J961" s="17" t="n">
+        <v>186114.5243410245</v>
+      </c>
+      <c r="K961" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,161.1962</t>
+        </is>
+      </c>
+      <c r="L961" s="17" t="n">
+        <v>124210.8805337359</v>
+      </c>
+      <c r="M961" s="17">
+        <f>J961-L961</f>
+        <v/>
+      </c>
+      <c r="N961" s="18">
+        <f>IF(J961=0,"",L961/J961)</f>
+        <v/>
+      </c>
+      <c r="O961" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="962">
+      <c r="A962" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:15:18</t>
+        </is>
+      </c>
+      <c r="B962" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C962" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D962" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E962" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F962" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G962" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H962" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I962" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J962" s="17" t="n">
+        <v>327704.8720798632</v>
+      </c>
+      <c r="K962" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,363.1264</t>
+        </is>
+      </c>
+      <c r="L962" s="17" t="n">
+        <v>280215.5597765784</v>
+      </c>
+      <c r="M962" s="17">
+        <f>J962-L962</f>
+        <v/>
+      </c>
+      <c r="N962" s="18">
+        <f>IF(J962=0,"",L962/J962)</f>
+        <v/>
+      </c>
+      <c r="O962" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:15:18</t>
+        </is>
+      </c>
+      <c r="B963" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C963" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D963" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E963" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F963" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G963" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H963" s="16" t="n">
+        <v>1.9047</v>
+      </c>
+      <c r="I963" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J963" s="17" t="n">
+        <v>160052.5364672934</v>
+      </c>
+      <c r="K963" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,952.6109</t>
+        </is>
+      </c>
+      <c r="L963" s="17" t="n">
+        <v>70981.0033287836</v>
+      </c>
+      <c r="M963" s="17">
+        <f>J963-L963</f>
+        <v/>
+      </c>
+      <c r="N963" s="18">
+        <f>IF(J963=0,"",L963/J963)</f>
+        <v/>
+      </c>
+      <c r="O963" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="964">
+      <c r="A964" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:15:18</t>
+        </is>
+      </c>
+      <c r="B964" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C964" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D964" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E964" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F964" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G964" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H964" s="16" t="n">
+        <v>1.0571</v>
+      </c>
+      <c r="I964" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J964" s="17" t="n">
+        <v>160167.830281298</v>
+      </c>
+      <c r="K964" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,532.9072</t>
+        </is>
+      </c>
+      <c r="L964" s="17" t="n">
+        <v>138546.760445046</v>
+      </c>
+      <c r="M964" s="17">
+        <f>J964-L964</f>
+        <v/>
+      </c>
+      <c r="N964" s="18">
+        <f>IF(J964=0,"",L964/J964)</f>
+        <v/>
+      </c>
+      <c r="O964" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:15:18</t>
+        </is>
+      </c>
+      <c r="B965" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C965" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D965" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E965" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F965" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G965" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H965" s="16" t="inlineStr"/>
+      <c r="I965" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J965" s="17" t="n">
+        <v>95925.04792842484</v>
+      </c>
+      <c r="K965" s="15" t="inlineStr"/>
+      <c r="L965" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M965" s="17">
+        <f>J965-L965</f>
+        <v/>
+      </c>
+      <c r="N965" s="18">
+        <f>IF(J965=0,"",L965/J965)</f>
+        <v/>
+      </c>
+      <c r="O965" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="966">
+      <c r="A966" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:15:18</t>
+        </is>
+      </c>
+      <c r="B966" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C966" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D966" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E966" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F966" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G966" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H966" s="16" t="inlineStr"/>
+      <c r="I966" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J966" s="17" t="n">
+        <v>34366.36771923486</v>
+      </c>
+      <c r="K966" s="15" t="inlineStr"/>
+      <c r="L966" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M966" s="17">
+        <f>J966-L966</f>
+        <v/>
+      </c>
+      <c r="N966" s="18">
+        <f>IF(J966=0,"",L966/J966)</f>
+        <v/>
+      </c>
+      <c r="O966" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="967">
+      <c r="A967" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:15:18</t>
+        </is>
+      </c>
+      <c r="B967" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C967" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D967" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E967" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F967" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G967" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H967" s="16" t="n">
+        <v>1.0434</v>
+      </c>
+      <c r="I967" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J967" s="17" t="n">
+        <v>270109.2152993662</v>
+      </c>
+      <c r="K967" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,071.2752</t>
+        </is>
+      </c>
+      <c r="L967" s="17" t="n">
+        <v>232982.708157408</v>
+      </c>
+      <c r="M967" s="17">
+        <f>J967-L967</f>
+        <v/>
+      </c>
+      <c r="N967" s="18">
+        <f>IF(J967=0,"",L967/J967)</f>
+        <v/>
+      </c>
+      <c r="O967" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="968">
+      <c r="A968" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:15:18</t>
+        </is>
+      </c>
+      <c r="B968" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C968" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D968" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E968" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F968" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G968" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H968" s="16" t="inlineStr"/>
+      <c r="I968" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,518.6925</t>
+        </is>
+      </c>
+      <c r="J968" s="17" t="n">
+        <v>15512.79539820029</v>
+      </c>
+      <c r="K968" s="15" t="inlineStr"/>
+      <c r="L968" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M968" s="17">
+        <f>J968-L968</f>
+        <v/>
+      </c>
+      <c r="N968" s="18">
+        <f>IF(J968=0,"",L968/J968)</f>
+        <v/>
+      </c>
+      <c r="O968" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="969">
+      <c r="A969" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:15:18</t>
+        </is>
+      </c>
+      <c r="B969" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C969" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D969" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E969" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F969" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G969" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H969" s="16" t="n">
+        <v>1.219</v>
+      </c>
+      <c r="I969" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J969" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K969" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,736.3177</t>
+        </is>
+      </c>
+      <c r="L969" s="17" t="n">
+        <v>148736.317674</v>
+      </c>
+      <c r="M969" s="17">
+        <f>J969-L969</f>
+        <v/>
+      </c>
+      <c r="N969" s="18">
+        <f>IF(J969=0,"",L969/J969)</f>
+        <v/>
+      </c>
+      <c r="O969" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="970">
+      <c r="A970" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:15:18</t>
+        </is>
+      </c>
+      <c r="B970" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C970" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D970" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E970" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F970" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G970" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H970" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I970" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J970" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K970" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L970" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M970" s="17">
+        <f>J970-L970</f>
+        <v/>
+      </c>
+      <c r="N970" s="18">
+        <f>IF(J970=0,"",L970/J970)</f>
+        <v/>
+      </c>
+      <c r="O970" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -64816,7 +65902,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I63"/>
+  <dimension ref="A1:I64"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -67037,6 +68123,41 @@
         <v>1.0372</v>
       </c>
       <c r="I63" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:15:18</t>
+        </is>
+      </c>
+      <c r="B64" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C64" s="17" t="n">
+        <v>655428.3777419569</v>
+      </c>
+      <c r="D64" s="17" t="n">
+        <v>652840.6364487358</v>
+      </c>
+      <c r="E64" s="17" t="n">
+        <v>2933882.601359165</v>
+      </c>
+      <c r="F64" s="17" t="n">
+        <v>2281041.964910429</v>
+      </c>
+      <c r="G64" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H64" s="16" t="n">
+        <v>1.0372</v>
+      </c>
+      <c r="I64" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
fix: balance/total-equity match + threshold 0.03%/$15 + fresh snapshot
- totalEquity in table now uses netPos (same as fund hero) — both show $655,322
- Color threshold: max($15, 0.03%) — mF-ONE +$42 gain now correctly greens;
  sub-$15 micro-noise stays white
- Fresh snapshot 2026-04-30T08:24:24Z with live EVM + cached Solana data

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O970"/>
+  <dimension ref="A1:O986"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -65872,6 +65872,1092 @@
         <v/>
       </c>
       <c r="O970" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="971">
+      <c r="A971" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:24:24</t>
+        </is>
+      </c>
+      <c r="B971" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C971" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D971" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E971" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F971" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G971" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H971" s="16" t="n">
+        <v>1.0503</v>
+      </c>
+      <c r="I971" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,809.3004</t>
+        </is>
+      </c>
+      <c r="J971" s="17" t="n">
+        <v>50787.45241582154</v>
+      </c>
+      <c r="K971" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,726.6826</t>
+        </is>
+      </c>
+      <c r="L971" s="17" t="n">
+        <v>37741.77928271308</v>
+      </c>
+      <c r="M971" s="17">
+        <f>J971-L971</f>
+        <v/>
+      </c>
+      <c r="N971" s="18">
+        <f>IF(J971=0,"",L971/J971)</f>
+        <v/>
+      </c>
+      <c r="O971" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="972">
+      <c r="A972" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:24:24</t>
+        </is>
+      </c>
+      <c r="B972" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C972" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D972" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E972" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F972" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G972" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H972" s="16" t="n">
+        <v>1.0484</v>
+      </c>
+      <c r="I972" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J972" s="17" t="n">
+        <v>140942.3082907065</v>
+      </c>
+      <c r="K972" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,048.3985</t>
+        </is>
+      </c>
+      <c r="L972" s="17" t="n">
+        <v>120996.3477066373</v>
+      </c>
+      <c r="M972" s="17">
+        <f>J972-L972</f>
+        <v/>
+      </c>
+      <c r="N972" s="18">
+        <f>IF(J972=0,"",L972/J972)</f>
+        <v/>
+      </c>
+      <c r="O972" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="973">
+      <c r="A973" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:24:24</t>
+        </is>
+      </c>
+      <c r="B973" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C973" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D973" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E973" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F973" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G973" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H973" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I973" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J973" s="17" t="n">
+        <v>328741.9531125519</v>
+      </c>
+      <c r="K973" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,401.0536</t>
+        </is>
+      </c>
+      <c r="L973" s="17" t="n">
+        <v>306561.8425584607</v>
+      </c>
+      <c r="M973" s="17">
+        <f>J973-L973</f>
+        <v/>
+      </c>
+      <c r="N973" s="18">
+        <f>IF(J973=0,"",L973/J973)</f>
+        <v/>
+      </c>
+      <c r="O973" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="974">
+      <c r="A974" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:24:24</t>
+        </is>
+      </c>
+      <c r="B974" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C974" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D974" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E974" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F974" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G974" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H974" s="16" t="n">
+        <v>1.0372</v>
+      </c>
+      <c r="I974" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J974" s="17" t="n">
+        <v>386103.7756160515</v>
+      </c>
+      <c r="K974" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,631.2289</t>
+        </is>
+      </c>
+      <c r="L974" s="17" t="n">
+        <v>349814.7035773661</v>
+      </c>
+      <c r="M974" s="17">
+        <f>J974-L974</f>
+        <v/>
+      </c>
+      <c r="N974" s="18">
+        <f>IF(J974=0,"",L974/J974)</f>
+        <v/>
+      </c>
+      <c r="O974" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="975">
+      <c r="A975" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:24:24</t>
+        </is>
+      </c>
+      <c r="B975" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C975" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D975" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E975" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F975" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G975" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H975" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I975" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7873</t>
+        </is>
+      </c>
+      <c r="J975" s="17" t="n">
+        <v>77779.57335033016</v>
+      </c>
+      <c r="K975" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,034.4625; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L975" s="17" t="n">
+        <v>68005.28531514791</v>
+      </c>
+      <c r="M975" s="17">
+        <f>J975-L975</f>
+        <v/>
+      </c>
+      <c r="N975" s="18">
+        <f>IF(J975=0,"",L975/J975)</f>
+        <v/>
+      </c>
+      <c r="O975" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="976">
+      <c r="A976" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:24:24</t>
+        </is>
+      </c>
+      <c r="B976" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C976" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D976" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E976" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F976" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G976" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H976" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I976" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J976" s="17" t="n">
+        <v>197137.3464223129</v>
+      </c>
+      <c r="K976" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,262.3037</t>
+        </is>
+      </c>
+      <c r="L976" s="17" t="n">
+        <v>150322.4326593186</v>
+      </c>
+      <c r="M976" s="17">
+        <f>J976-L976</f>
+        <v/>
+      </c>
+      <c r="N976" s="18">
+        <f>IF(J976=0,"",L976/J976)</f>
+        <v/>
+      </c>
+      <c r="O976" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="977">
+      <c r="A977" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:24:24</t>
+        </is>
+      </c>
+      <c r="B977" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C977" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D977" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E977" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F977" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G977" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H977" s="16" t="n">
+        <v>1.3728</v>
+      </c>
+      <c r="I977" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J977" s="17" t="n">
+        <v>186070.6787316354</v>
+      </c>
+      <c r="K977" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,161.1962</t>
+        </is>
+      </c>
+      <c r="L977" s="17" t="n">
+        <v>124210.8805337359</v>
+      </c>
+      <c r="M977" s="17">
+        <f>J977-L977</f>
+        <v/>
+      </c>
+      <c r="N977" s="18">
+        <f>IF(J977=0,"",L977/J977)</f>
+        <v/>
+      </c>
+      <c r="O977" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="978">
+      <c r="A978" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:24:24</t>
+        </is>
+      </c>
+      <c r="B978" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C978" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D978" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E978" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F978" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G978" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H978" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I978" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J978" s="17" t="n">
+        <v>327704.8720798632</v>
+      </c>
+      <c r="K978" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,363.1264</t>
+        </is>
+      </c>
+      <c r="L978" s="17" t="n">
+        <v>280212.5452141222</v>
+      </c>
+      <c r="M978" s="17">
+        <f>J978-L978</f>
+        <v/>
+      </c>
+      <c r="N978" s="18">
+        <f>IF(J978=0,"",L978/J978)</f>
+        <v/>
+      </c>
+      <c r="O978" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="979">
+      <c r="A979" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:24:24</t>
+        </is>
+      </c>
+      <c r="B979" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C979" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D979" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E979" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F979" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G979" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H979" s="16" t="n">
+        <v>1.9047</v>
+      </c>
+      <c r="I979" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J979" s="17" t="n">
+        <v>160052.5364672934</v>
+      </c>
+      <c r="K979" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,952.6109</t>
+        </is>
+      </c>
+      <c r="L979" s="17" t="n">
+        <v>70981.0033287836</v>
+      </c>
+      <c r="M979" s="17">
+        <f>J979-L979</f>
+        <v/>
+      </c>
+      <c r="N979" s="18">
+        <f>IF(J979=0,"",L979/J979)</f>
+        <v/>
+      </c>
+      <c r="O979" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="980">
+      <c r="A980" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:24:24</t>
+        </is>
+      </c>
+      <c r="B980" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C980" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D980" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E980" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F980" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G980" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H980" s="16" t="n">
+        <v>1.0571</v>
+      </c>
+      <c r="I980" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J980" s="17" t="n">
+        <v>160184.0088149474</v>
+      </c>
+      <c r="K980" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,532.9072</t>
+        </is>
+      </c>
+      <c r="L980" s="17" t="n">
+        <v>138546.760445046</v>
+      </c>
+      <c r="M980" s="17">
+        <f>J980-L980</f>
+        <v/>
+      </c>
+      <c r="N980" s="18">
+        <f>IF(J980=0,"",L980/J980)</f>
+        <v/>
+      </c>
+      <c r="O980" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="981">
+      <c r="A981" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:24:24</t>
+        </is>
+      </c>
+      <c r="B981" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C981" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D981" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E981" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F981" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G981" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H981" s="16" t="inlineStr"/>
+      <c r="I981" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J981" s="17" t="n">
+        <v>95929.35255027963</v>
+      </c>
+      <c r="K981" s="15" t="inlineStr"/>
+      <c r="L981" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M981" s="17">
+        <f>J981-L981</f>
+        <v/>
+      </c>
+      <c r="N981" s="18">
+        <f>IF(J981=0,"",L981/J981)</f>
+        <v/>
+      </c>
+      <c r="O981" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="982">
+      <c r="A982" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:24:24</t>
+        </is>
+      </c>
+      <c r="B982" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C982" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D982" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E982" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F982" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G982" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H982" s="16" t="inlineStr"/>
+      <c r="I982" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J982" s="17" t="n">
+        <v>34366.46161759816</v>
+      </c>
+      <c r="K982" s="15" t="inlineStr"/>
+      <c r="L982" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M982" s="17">
+        <f>J982-L982</f>
+        <v/>
+      </c>
+      <c r="N982" s="18">
+        <f>IF(J982=0,"",L982/J982)</f>
+        <v/>
+      </c>
+      <c r="O982" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="983">
+      <c r="A983" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:24:24</t>
+        </is>
+      </c>
+      <c r="B983" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C983" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D983" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E983" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F983" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G983" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H983" s="16" t="n">
+        <v>1.0435</v>
+      </c>
+      <c r="I983" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J983" s="17" t="n">
+        <v>270109.2152993662</v>
+      </c>
+      <c r="K983" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,071.2752</t>
+        </is>
+      </c>
+      <c r="L983" s="17" t="n">
+        <v>232971.0545936459</v>
+      </c>
+      <c r="M983" s="17">
+        <f>J983-L983</f>
+        <v/>
+      </c>
+      <c r="N983" s="18">
+        <f>IF(J983=0,"",L983/J983)</f>
+        <v/>
+      </c>
+      <c r="O983" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="984">
+      <c r="A984" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:24:24</t>
+        </is>
+      </c>
+      <c r="B984" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C984" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D984" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E984" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F984" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G984" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H984" s="16" t="inlineStr"/>
+      <c r="I984" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,518.6925</t>
+        </is>
+      </c>
+      <c r="J984" s="17" t="n">
+        <v>15512.01946357523</v>
+      </c>
+      <c r="K984" s="15" t="inlineStr"/>
+      <c r="L984" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M984" s="17">
+        <f>J984-L984</f>
+        <v/>
+      </c>
+      <c r="N984" s="18">
+        <f>IF(J984=0,"",L984/J984)</f>
+        <v/>
+      </c>
+      <c r="O984" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="985">
+      <c r="A985" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:24:24</t>
+        </is>
+      </c>
+      <c r="B985" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C985" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D985" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E985" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F985" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G985" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H985" s="16" t="n">
+        <v>1.219</v>
+      </c>
+      <c r="I985" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J985" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K985" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,736.3177</t>
+        </is>
+      </c>
+      <c r="L985" s="17" t="n">
+        <v>148736.317674</v>
+      </c>
+      <c r="M985" s="17">
+        <f>J985-L985</f>
+        <v/>
+      </c>
+      <c r="N985" s="18">
+        <f>IF(J985=0,"",L985/J985)</f>
+        <v/>
+      </c>
+      <c r="O985" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="986">
+      <c r="A986" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:24:24</t>
+        </is>
+      </c>
+      <c r="B986" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C986" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D986" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E986" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F986" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G986" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H986" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I986" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J986" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K986" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L986" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M986" s="17">
+        <f>J986-L986</f>
+        <v/>
+      </c>
+      <c r="N986" s="18">
+        <f>IF(J986=0,"",L986/J986)</f>
+        <v/>
+      </c>
+      <c r="O986" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -65902,7 +66988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I64"/>
+  <dimension ref="A1:I65"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -68158,6 +69244,41 @@
         <v>1.0372</v>
       </c>
       <c r="I64" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:24:24</t>
+        </is>
+      </c>
+      <c r="B65" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C65" s="17" t="n">
+        <v>655409.0637496198</v>
+      </c>
+      <c r="D65" s="17" t="n">
+        <v>652821.4348303061</v>
+      </c>
+      <c r="E65" s="17" t="n">
+        <v>2933904.934823283</v>
+      </c>
+      <c r="F65" s="17" t="n">
+        <v>2281083.499992977</v>
+      </c>
+      <c r="G65" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H65" s="16" t="n">
+        <v>1.0372</v>
+      </c>
+      <c r="I65" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-30 08:45 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O986"/>
+  <dimension ref="A1:O1002"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -66958,6 +66958,1092 @@
         <v/>
       </c>
       <c r="O986" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="987">
+      <c r="A987" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:45:28</t>
+        </is>
+      </c>
+      <c r="B987" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C987" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D987" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E987" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F987" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G987" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H987" s="16" t="n">
+        <v>1.0503</v>
+      </c>
+      <c r="I987" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,809.3004</t>
+        </is>
+      </c>
+      <c r="J987" s="17" t="n">
+        <v>50787.9605088257</v>
+      </c>
+      <c r="K987" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,726.6826</t>
+        </is>
+      </c>
+      <c r="L987" s="17" t="n">
+        <v>37734.22941688338</v>
+      </c>
+      <c r="M987" s="17">
+        <f>J987-L987</f>
+        <v/>
+      </c>
+      <c r="N987" s="18">
+        <f>IF(J987=0,"",L987/J987)</f>
+        <v/>
+      </c>
+      <c r="O987" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="988">
+      <c r="A988" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:45:28</t>
+        </is>
+      </c>
+      <c r="B988" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C988" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D988" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E988" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F988" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G988" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H988" s="16" t="n">
+        <v>1.0484</v>
+      </c>
+      <c r="I988" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J988" s="17" t="n">
+        <v>140942.7308347349</v>
+      </c>
+      <c r="K988" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,048.3985</t>
+        </is>
+      </c>
+      <c r="L988" s="17" t="n">
+        <v>120997.5581906224</v>
+      </c>
+      <c r="M988" s="17">
+        <f>J988-L988</f>
+        <v/>
+      </c>
+      <c r="N988" s="18">
+        <f>IF(J988=0,"",L988/J988)</f>
+        <v/>
+      </c>
+      <c r="O988" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:45:28</t>
+        </is>
+      </c>
+      <c r="B989" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C989" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D989" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E989" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F989" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G989" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H989" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I989" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J989" s="17" t="n">
+        <v>328741.9531125519</v>
+      </c>
+      <c r="K989" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,401.0536</t>
+        </is>
+      </c>
+      <c r="L989" s="17" t="n">
+        <v>306500.4707243445</v>
+      </c>
+      <c r="M989" s="17">
+        <f>J989-L989</f>
+        <v/>
+      </c>
+      <c r="N989" s="18">
+        <f>IF(J989=0,"",L989/J989)</f>
+        <v/>
+      </c>
+      <c r="O989" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:45:28</t>
+        </is>
+      </c>
+      <c r="B990" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C990" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D990" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E990" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F990" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G990" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H990" s="16" t="n">
+        <v>1.0372</v>
+      </c>
+      <c r="I990" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J990" s="17" t="n">
+        <v>386065.9219021456</v>
+      </c>
+      <c r="K990" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,631.2289</t>
+        </is>
+      </c>
+      <c r="L990" s="17" t="n">
+        <v>349744.6727810343</v>
+      </c>
+      <c r="M990" s="17">
+        <f>J990-L990</f>
+        <v/>
+      </c>
+      <c r="N990" s="18">
+        <f>IF(J990=0,"",L990/J990)</f>
+        <v/>
+      </c>
+      <c r="O990" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:45:28</t>
+        </is>
+      </c>
+      <c r="B991" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C991" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D991" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E991" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F991" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G991" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H991" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I991" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7873</t>
+        </is>
+      </c>
+      <c r="J991" s="17" t="n">
+        <v>77779.57122560528</v>
+      </c>
+      <c r="K991" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,034.4625; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L991" s="17" t="n">
+        <v>68005.96564425077</v>
+      </c>
+      <c r="M991" s="17">
+        <f>J991-L991</f>
+        <v/>
+      </c>
+      <c r="N991" s="18">
+        <f>IF(J991=0,"",L991/J991)</f>
+        <v/>
+      </c>
+      <c r="O991" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:45:28</t>
+        </is>
+      </c>
+      <c r="B992" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C992" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D992" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E992" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F992" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G992" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H992" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I992" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J992" s="17" t="n">
+        <v>197144.9160837264</v>
+      </c>
+      <c r="K992" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,262.3037</t>
+        </is>
+      </c>
+      <c r="L992" s="17" t="n">
+        <v>150292.3621586867</v>
+      </c>
+      <c r="M992" s="17">
+        <f>J992-L992</f>
+        <v/>
+      </c>
+      <c r="N992" s="18">
+        <f>IF(J992=0,"",L992/J992)</f>
+        <v/>
+      </c>
+      <c r="O992" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="993">
+      <c r="A993" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:45:28</t>
+        </is>
+      </c>
+      <c r="B993" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C993" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D993" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E993" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F993" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G993" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H993" s="16" t="n">
+        <v>1.3728</v>
+      </c>
+      <c r="I993" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J993" s="17" t="n">
+        <v>186070.9289012734</v>
+      </c>
+      <c r="K993" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,161.1962</t>
+        </is>
+      </c>
+      <c r="L993" s="17" t="n">
+        <v>124186.0333882001</v>
+      </c>
+      <c r="M993" s="17">
+        <f>J993-L993</f>
+        <v/>
+      </c>
+      <c r="N993" s="18">
+        <f>IF(J993=0,"",L993/J993)</f>
+        <v/>
+      </c>
+      <c r="O993" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:45:28</t>
+        </is>
+      </c>
+      <c r="B994" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C994" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D994" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E994" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F994" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G994" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H994" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I994" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J994" s="17" t="n">
+        <v>327712.9778392483</v>
+      </c>
+      <c r="K994" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,363.1264</t>
+        </is>
+      </c>
+      <c r="L994" s="17" t="n">
+        <v>280212.5479467753</v>
+      </c>
+      <c r="M994" s="17">
+        <f>J994-L994</f>
+        <v/>
+      </c>
+      <c r="N994" s="18">
+        <f>IF(J994=0,"",L994/J994)</f>
+        <v/>
+      </c>
+      <c r="O994" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:45:28</t>
+        </is>
+      </c>
+      <c r="B995" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C995" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D995" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E995" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F995" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G995" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H995" s="16" t="n">
+        <v>1.9047</v>
+      </c>
+      <c r="I995" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J995" s="17" t="n">
+        <v>160068.5465239572</v>
+      </c>
+      <c r="K995" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,952.6109</t>
+        </is>
+      </c>
+      <c r="L995" s="17" t="n">
+        <v>70966.80428830975</v>
+      </c>
+      <c r="M995" s="17">
+        <f>J995-L995</f>
+        <v/>
+      </c>
+      <c r="N995" s="18">
+        <f>IF(J995=0,"",L995/J995)</f>
+        <v/>
+      </c>
+      <c r="O995" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:45:28</t>
+        </is>
+      </c>
+      <c r="B996" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C996" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D996" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E996" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F996" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G996" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H996" s="16" t="n">
+        <v>1.0571</v>
+      </c>
+      <c r="I996" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J996" s="17" t="n">
+        <v>160168.3043333419</v>
+      </c>
+      <c r="K996" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,532.9072</t>
+        </is>
+      </c>
+      <c r="L996" s="17" t="n">
+        <v>138629.8801893386</v>
+      </c>
+      <c r="M996" s="17">
+        <f>J996-L996</f>
+        <v/>
+      </c>
+      <c r="N996" s="18">
+        <f>IF(J996=0,"",L996/J996)</f>
+        <v/>
+      </c>
+      <c r="O996" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:45:28</t>
+        </is>
+      </c>
+      <c r="B997" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C997" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D997" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E997" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F997" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G997" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H997" s="16" t="inlineStr"/>
+      <c r="I997" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J997" s="17" t="n">
+        <v>95929.35255027963</v>
+      </c>
+      <c r="K997" s="15" t="inlineStr"/>
+      <c r="L997" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M997" s="17">
+        <f>J997-L997</f>
+        <v/>
+      </c>
+      <c r="N997" s="18">
+        <f>IF(J997=0,"",L997/J997)</f>
+        <v/>
+      </c>
+      <c r="O997" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:45:28</t>
+        </is>
+      </c>
+      <c r="B998" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C998" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D998" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E998" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F998" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G998" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H998" s="16" t="inlineStr"/>
+      <c r="I998" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J998" s="17" t="n">
+        <v>34366.65663809558</v>
+      </c>
+      <c r="K998" s="15" t="inlineStr"/>
+      <c r="L998" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M998" s="17">
+        <f>J998-L998</f>
+        <v/>
+      </c>
+      <c r="N998" s="18">
+        <f>IF(J998=0,"",L998/J998)</f>
+        <v/>
+      </c>
+      <c r="O998" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:45:28</t>
+        </is>
+      </c>
+      <c r="B999" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C999" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D999" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E999" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F999" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G999" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H999" s="16" t="n">
+        <v>1.0434</v>
+      </c>
+      <c r="I999" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J999" s="17" t="n">
+        <v>270082.196272128</v>
+      </c>
+      <c r="K999" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,071.2752</t>
+        </is>
+      </c>
+      <c r="L999" s="17" t="n">
+        <v>232973.3853063984</v>
+      </c>
+      <c r="M999" s="17">
+        <f>J999-L999</f>
+        <v/>
+      </c>
+      <c r="N999" s="18">
+        <f>IF(J999=0,"",L999/J999)</f>
+        <v/>
+      </c>
+      <c r="O999" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:45:28</t>
+        </is>
+      </c>
+      <c r="B1000" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1000" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D1000" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E1000" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1000" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G1000" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1000" s="16" t="inlineStr"/>
+      <c r="I1000" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,519.0822</t>
+        </is>
+      </c>
+      <c r="J1000" s="17" t="n">
+        <v>15512.56417156893</v>
+      </c>
+      <c r="K1000" s="15" t="inlineStr"/>
+      <c r="L1000" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1000" s="17">
+        <f>J1000-L1000</f>
+        <v/>
+      </c>
+      <c r="N1000" s="18">
+        <f>IF(J1000=0,"",L1000/J1000)</f>
+        <v/>
+      </c>
+      <c r="O1000" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1001">
+      <c r="A1001" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:45:28</t>
+        </is>
+      </c>
+      <c r="B1001" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1001" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D1001" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E1001" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1001" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G1001" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H1001" s="16" t="n">
+        <v>1.219</v>
+      </c>
+      <c r="I1001" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J1001" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K1001" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,736.3177</t>
+        </is>
+      </c>
+      <c r="L1001" s="17" t="n">
+        <v>148736.317674</v>
+      </c>
+      <c r="M1001" s="17">
+        <f>J1001-L1001</f>
+        <v/>
+      </c>
+      <c r="N1001" s="18">
+        <f>IF(J1001=0,"",L1001/J1001)</f>
+        <v/>
+      </c>
+      <c r="O1001" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:45:28</t>
+        </is>
+      </c>
+      <c r="B1002" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1002" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D1002" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E1002" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1002" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G1002" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H1002" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I1002" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J1002" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K1002" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L1002" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M1002" s="17">
+        <f>J1002-L1002</f>
+        <v/>
+      </c>
+      <c r="N1002" s="18">
+        <f>IF(J1002=0,"",L1002/J1002)</f>
+        <v/>
+      </c>
+      <c r="O1002" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -66988,7 +68074,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I65"/>
+  <dimension ref="A1:I66"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -69279,6 +70365,41 @@
         <v>1.0372</v>
       </c>
       <c r="I65" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:45:28</t>
+        </is>
+      </c>
+      <c r="B66" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C66" s="17" t="n">
+        <v>655484.46052012</v>
+      </c>
+      <c r="D66" s="17" t="n">
+        <v>652895.1866755881</v>
+      </c>
+      <c r="E66" s="17" t="n">
+        <v>2933857.961488432</v>
+      </c>
+      <c r="F66" s="17" t="n">
+        <v>2280962.774812844</v>
+      </c>
+      <c r="G66" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H66" s="16" t="n">
+        <v>1.0372</v>
+      </c>
+      <c r="I66" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-30 09:15 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O1002"/>
+  <dimension ref="A1:O1018"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -68044,6 +68044,1092 @@
         <v/>
       </c>
       <c r="O1002" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:15:40</t>
+        </is>
+      </c>
+      <c r="B1003" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1003" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1003" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E1003" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1003" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G1003" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H1003" s="16" t="n">
+        <v>1.0503</v>
+      </c>
+      <c r="I1003" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,809.3004</t>
+        </is>
+      </c>
+      <c r="J1003" s="17" t="n">
+        <v>50787.45241582154</v>
+      </c>
+      <c r="K1003" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,726.6826</t>
+        </is>
+      </c>
+      <c r="L1003" s="17" t="n">
+        <v>37738.00397219165</v>
+      </c>
+      <c r="M1003" s="17">
+        <f>J1003-L1003</f>
+        <v/>
+      </c>
+      <c r="N1003" s="18">
+        <f>IF(J1003=0,"",L1003/J1003)</f>
+        <v/>
+      </c>
+      <c r="O1003" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:15:40</t>
+        </is>
+      </c>
+      <c r="B1004" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1004" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1004" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E1004" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1004" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G1004" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H1004" s="16" t="n">
+        <v>1.0484</v>
+      </c>
+      <c r="I1004" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J1004" s="17" t="n">
+        <v>140941.5809168211</v>
+      </c>
+      <c r="K1004" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,048.3985</t>
+        </is>
+      </c>
+      <c r="L1004" s="17" t="n">
+        <v>120996.3477066373</v>
+      </c>
+      <c r="M1004" s="17">
+        <f>J1004-L1004</f>
+        <v/>
+      </c>
+      <c r="N1004" s="18">
+        <f>IF(J1004=0,"",L1004/J1004)</f>
+        <v/>
+      </c>
+      <c r="O1004" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:15:40</t>
+        </is>
+      </c>
+      <c r="B1005" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1005" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1005" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E1005" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1005" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G1005" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H1005" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I1005" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J1005" s="17" t="n">
+        <v>328742.7092788876</v>
+      </c>
+      <c r="K1005" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,401.0536</t>
+        </is>
+      </c>
+      <c r="L1005" s="17" t="n">
+        <v>306500.4706934817</v>
+      </c>
+      <c r="M1005" s="17">
+        <f>J1005-L1005</f>
+        <v/>
+      </c>
+      <c r="N1005" s="18">
+        <f>IF(J1005=0,"",L1005/J1005)</f>
+        <v/>
+      </c>
+      <c r="O1005" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:15:40</t>
+        </is>
+      </c>
+      <c r="B1006" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1006" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1006" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E1006" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1006" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G1006" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H1006" s="16" t="n">
+        <v>1.0372</v>
+      </c>
+      <c r="I1006" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J1006" s="17" t="n">
+        <v>386066.3468217542</v>
+      </c>
+      <c r="K1006" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,631.2289</t>
+        </is>
+      </c>
+      <c r="L1006" s="17" t="n">
+        <v>349744.6727458169</v>
+      </c>
+      <c r="M1006" s="17">
+        <f>J1006-L1006</f>
+        <v/>
+      </c>
+      <c r="N1006" s="18">
+        <f>IF(J1006=0,"",L1006/J1006)</f>
+        <v/>
+      </c>
+      <c r="O1006" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:15:40</t>
+        </is>
+      </c>
+      <c r="B1007" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1007" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D1007" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E1007" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1007" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G1007" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H1007" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I1007" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7873</t>
+        </is>
+      </c>
+      <c r="J1007" s="17" t="n">
+        <v>77781.92369487201</v>
+      </c>
+      <c r="K1007" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,034.4625; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L1007" s="17" t="n">
+        <v>68005.28530738587</v>
+      </c>
+      <c r="M1007" s="17">
+        <f>J1007-L1007</f>
+        <v/>
+      </c>
+      <c r="N1007" s="18">
+        <f>IF(J1007=0,"",L1007/J1007)</f>
+        <v/>
+      </c>
+      <c r="O1007" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:15:40</t>
+        </is>
+      </c>
+      <c r="B1008" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1008" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1008" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1008" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1008" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1008" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H1008" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I1008" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J1008" s="17" t="n">
+        <v>197147.2961720005</v>
+      </c>
+      <c r="K1008" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,262.3037</t>
+        </is>
+      </c>
+      <c r="L1008" s="17" t="n">
+        <v>150307.3959050264</v>
+      </c>
+      <c r="M1008" s="17">
+        <f>J1008-L1008</f>
+        <v/>
+      </c>
+      <c r="N1008" s="18">
+        <f>IF(J1008=0,"",L1008/J1008)</f>
+        <v/>
+      </c>
+      <c r="O1008" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:15:40</t>
+        </is>
+      </c>
+      <c r="B1009" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1009" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1009" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1009" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1009" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1009" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H1009" s="16" t="n">
+        <v>1.3728</v>
+      </c>
+      <c r="I1009" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J1009" s="17" t="n">
+        <v>186071.695952339</v>
+      </c>
+      <c r="K1009" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,161.1962</t>
+        </is>
+      </c>
+      <c r="L1009" s="17" t="n">
+        <v>124198.4557182379</v>
+      </c>
+      <c r="M1009" s="17">
+        <f>J1009-L1009</f>
+        <v/>
+      </c>
+      <c r="N1009" s="18">
+        <f>IF(J1009=0,"",L1009/J1009)</f>
+        <v/>
+      </c>
+      <c r="O1009" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:15:40</t>
+        </is>
+      </c>
+      <c r="B1010" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1010" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1010" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1010" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1010" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1010" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H1010" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I1010" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J1010" s="17" t="n">
+        <v>327727.5945800184</v>
+      </c>
+      <c r="K1010" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,363.1264</t>
+        </is>
+      </c>
+      <c r="L1010" s="17" t="n">
+        <v>280230.7430279772</v>
+      </c>
+      <c r="M1010" s="17">
+        <f>J1010-L1010</f>
+        <v/>
+      </c>
+      <c r="N1010" s="18">
+        <f>IF(J1010=0,"",L1010/J1010)</f>
+        <v/>
+      </c>
+      <c r="O1010" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:15:40</t>
+        </is>
+      </c>
+      <c r="B1011" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1011" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1011" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1011" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1011" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1011" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H1011" s="16" t="n">
+        <v>1.9047</v>
+      </c>
+      <c r="I1011" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J1011" s="17" t="n">
+        <v>160068.5465239572</v>
+      </c>
+      <c r="K1011" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,952.6109</t>
+        </is>
+      </c>
+      <c r="L1011" s="17" t="n">
+        <v>70973.90309838159</v>
+      </c>
+      <c r="M1011" s="17">
+        <f>J1011-L1011</f>
+        <v/>
+      </c>
+      <c r="N1011" s="18">
+        <f>IF(J1011=0,"",L1011/J1011)</f>
+        <v/>
+      </c>
+      <c r="O1011" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:15:40</t>
+        </is>
+      </c>
+      <c r="B1012" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1012" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1012" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1012" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1012" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1012" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H1012" s="16" t="n">
+        <v>1.0571</v>
+      </c>
+      <c r="I1012" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J1012" s="17" t="n">
+        <v>160168.4806209895</v>
+      </c>
+      <c r="K1012" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,532.9072</t>
+        </is>
+      </c>
+      <c r="L1012" s="17" t="n">
+        <v>138616.0268986232</v>
+      </c>
+      <c r="M1012" s="17">
+        <f>J1012-L1012</f>
+        <v/>
+      </c>
+      <c r="N1012" s="18">
+        <f>IF(J1012=0,"",L1012/J1012)</f>
+        <v/>
+      </c>
+      <c r="O1012" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:15:40</t>
+        </is>
+      </c>
+      <c r="B1013" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1013" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1013" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E1013" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1013" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G1013" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1013" s="16" t="inlineStr"/>
+      <c r="I1013" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J1013" s="17" t="n">
+        <v>95910.00626387044</v>
+      </c>
+      <c r="K1013" s="15" t="inlineStr"/>
+      <c r="L1013" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1013" s="17">
+        <f>J1013-L1013</f>
+        <v/>
+      </c>
+      <c r="N1013" s="18">
+        <f>IF(J1013=0,"",L1013/J1013)</f>
+        <v/>
+      </c>
+      <c r="O1013" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:15:40</t>
+        </is>
+      </c>
+      <c r="B1014" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1014" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1014" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E1014" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1014" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G1014" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1014" s="16" t="inlineStr"/>
+      <c r="I1014" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J1014" s="17" t="n">
+        <v>34366.89319222127</v>
+      </c>
+      <c r="K1014" s="15" t="inlineStr"/>
+      <c r="L1014" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1014" s="17">
+        <f>J1014-L1014</f>
+        <v/>
+      </c>
+      <c r="N1014" s="18">
+        <f>IF(J1014=0,"",L1014/J1014)</f>
+        <v/>
+      </c>
+      <c r="O1014" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:15:40</t>
+        </is>
+      </c>
+      <c r="B1015" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1015" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D1015" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E1015" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1015" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G1015" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H1015" s="16" t="n">
+        <v>1.0433</v>
+      </c>
+      <c r="I1015" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J1015" s="17" t="n">
+        <v>270055.1826497763</v>
+      </c>
+      <c r="K1015" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,071.2752</t>
+        </is>
+      </c>
+      <c r="L1015" s="17" t="n">
+        <v>232971.0545936459</v>
+      </c>
+      <c r="M1015" s="17">
+        <f>J1015-L1015</f>
+        <v/>
+      </c>
+      <c r="N1015" s="18">
+        <f>IF(J1015=0,"",L1015/J1015)</f>
+        <v/>
+      </c>
+      <c r="O1015" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:15:40</t>
+        </is>
+      </c>
+      <c r="B1016" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1016" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D1016" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E1016" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1016" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G1016" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1016" s="16" t="inlineStr"/>
+      <c r="I1016" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,519.0939</t>
+        </is>
+      </c>
+      <c r="J1016" s="17" t="n">
+        <v>15512.42065503862</v>
+      </c>
+      <c r="K1016" s="15" t="inlineStr"/>
+      <c r="L1016" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1016" s="17">
+        <f>J1016-L1016</f>
+        <v/>
+      </c>
+      <c r="N1016" s="18">
+        <f>IF(J1016=0,"",L1016/J1016)</f>
+        <v/>
+      </c>
+      <c r="O1016" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:15:40</t>
+        </is>
+      </c>
+      <c r="B1017" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1017" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D1017" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E1017" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1017" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G1017" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H1017" s="16" t="n">
+        <v>1.219</v>
+      </c>
+      <c r="I1017" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J1017" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K1017" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,736.3177</t>
+        </is>
+      </c>
+      <c r="L1017" s="17" t="n">
+        <v>148736.317674</v>
+      </c>
+      <c r="M1017" s="17">
+        <f>J1017-L1017</f>
+        <v/>
+      </c>
+      <c r="N1017" s="18">
+        <f>IF(J1017=0,"",L1017/J1017)</f>
+        <v/>
+      </c>
+      <c r="O1017" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:15:40</t>
+        </is>
+      </c>
+      <c r="B1018" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1018" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D1018" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E1018" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1018" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G1018" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H1018" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I1018" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J1018" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K1018" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L1018" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M1018" s="17">
+        <f>J1018-L1018</f>
+        <v/>
+      </c>
+      <c r="N1018" s="18">
+        <f>IF(J1018=0,"",L1018/J1018)</f>
+        <v/>
+      </c>
+      <c r="O1018" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -68074,7 +69160,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I66"/>
+  <dimension ref="A1:I67"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -70400,6 +71486,41 @@
         <v>1.0372</v>
       </c>
       <c r="I66" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:15:40</t>
+        </is>
+      </c>
+      <c r="B67" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C67" s="17" t="n">
+        <v>655419.2242763122</v>
+      </c>
+      <c r="D67" s="17" t="n">
+        <v>652830.2858839119</v>
+      </c>
+      <c r="E67" s="17" t="n">
+        <v>2933831.510329318</v>
+      </c>
+      <c r="F67" s="17" t="n">
+        <v>2281001.224445406</v>
+      </c>
+      <c r="G67" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H67" s="16" t="n">
+        <v>1.0372</v>
+      </c>
+      <c r="I67" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-30 09:45 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O1018"/>
+  <dimension ref="A1:O1034"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -69130,6 +69130,1092 @@
         <v/>
       </c>
       <c r="O1018" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:45:50</t>
+        </is>
+      </c>
+      <c r="B1019" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1019" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1019" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E1019" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1019" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G1019" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H1019" s="16" t="n">
+        <v>1.0503</v>
+      </c>
+      <c r="I1019" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,809.3004</t>
+        </is>
+      </c>
+      <c r="J1019" s="17" t="n">
+        <v>50778.81483475099</v>
+      </c>
+      <c r="K1019" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,726.6826</t>
+        </is>
+      </c>
+      <c r="L1019" s="17" t="n">
+        <v>37734.22941688338</v>
+      </c>
+      <c r="M1019" s="17">
+        <f>J1019-L1019</f>
+        <v/>
+      </c>
+      <c r="N1019" s="18">
+        <f>IF(J1019=0,"",L1019/J1019)</f>
+        <v/>
+      </c>
+      <c r="O1019" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:45:50</t>
+        </is>
+      </c>
+      <c r="B1020" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1020" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1020" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E1020" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1020" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G1020" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H1020" s="16" t="n">
+        <v>1.0485</v>
+      </c>
+      <c r="I1020" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J1020" s="17" t="n">
+        <v>140942.2889369824</v>
+      </c>
+      <c r="K1020" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,048.3985</t>
+        </is>
+      </c>
+      <c r="L1020" s="17" t="n">
+        <v>120975.7694788892</v>
+      </c>
+      <c r="M1020" s="17">
+        <f>J1020-L1020</f>
+        <v/>
+      </c>
+      <c r="N1020" s="18">
+        <f>IF(J1020=0,"",L1020/J1020)</f>
+        <v/>
+      </c>
+      <c r="O1020" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:45:50</t>
+        </is>
+      </c>
+      <c r="B1021" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1021" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1021" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E1021" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1021" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G1021" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H1021" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I1021" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J1021" s="17" t="n">
+        <v>328743.3745152665</v>
+      </c>
+      <c r="K1021" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,401.0536</t>
+        </is>
+      </c>
+      <c r="L1021" s="17" t="n">
+        <v>306530.565608438</v>
+      </c>
+      <c r="M1021" s="17">
+        <f>J1021-L1021</f>
+        <v/>
+      </c>
+      <c r="N1021" s="18">
+        <f>IF(J1021=0,"",L1021/J1021)</f>
+        <v/>
+      </c>
+      <c r="O1021" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:45:50</t>
+        </is>
+      </c>
+      <c r="B1022" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1022" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1022" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E1022" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1022" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G1022" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H1022" s="16" t="n">
+        <v>1.0372</v>
+      </c>
+      <c r="I1022" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J1022" s="17" t="n">
+        <v>386068.2399338568</v>
+      </c>
+      <c r="K1022" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,631.2289</t>
+        </is>
+      </c>
+      <c r="L1022" s="17" t="n">
+        <v>349779.013757297</v>
+      </c>
+      <c r="M1022" s="17">
+        <f>J1022-L1022</f>
+        <v/>
+      </c>
+      <c r="N1022" s="18">
+        <f>IF(J1022=0,"",L1022/J1022)</f>
+        <v/>
+      </c>
+      <c r="O1022" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:45:50</t>
+        </is>
+      </c>
+      <c r="B1023" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1023" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D1023" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E1023" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1023" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G1023" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H1023" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I1023" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7873</t>
+        </is>
+      </c>
+      <c r="J1023" s="17" t="n">
+        <v>77782.73702243577</v>
+      </c>
+      <c r="K1023" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,034.4625; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L1023" s="17" t="n">
+        <v>67993.7194409941</v>
+      </c>
+      <c r="M1023" s="17">
+        <f>J1023-L1023</f>
+        <v/>
+      </c>
+      <c r="N1023" s="18">
+        <f>IF(J1023=0,"",L1023/J1023)</f>
+        <v/>
+      </c>
+      <c r="O1023" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:45:50</t>
+        </is>
+      </c>
+      <c r="B1024" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1024" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1024" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1024" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1024" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1024" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H1024" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I1024" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J1024" s="17" t="n">
+        <v>197148.9790967941</v>
+      </c>
+      <c r="K1024" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,262.3037</t>
+        </is>
+      </c>
+      <c r="L1024" s="17" t="n">
+        <v>150292.3621586867</v>
+      </c>
+      <c r="M1024" s="17">
+        <f>J1024-L1024</f>
+        <v/>
+      </c>
+      <c r="N1024" s="18">
+        <f>IF(J1024=0,"",L1024/J1024)</f>
+        <v/>
+      </c>
+      <c r="O1024" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:45:50</t>
+        </is>
+      </c>
+      <c r="B1025" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1025" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1025" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1025" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1025" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1025" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H1025" s="16" t="n">
+        <v>1.3728</v>
+      </c>
+      <c r="I1025" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J1025" s="17" t="n">
+        <v>186072.6685224967</v>
+      </c>
+      <c r="K1025" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,161.1962</t>
+        </is>
+      </c>
+      <c r="L1025" s="17" t="n">
+        <v>124186.0333882001</v>
+      </c>
+      <c r="M1025" s="17">
+        <f>J1025-L1025</f>
+        <v/>
+      </c>
+      <c r="N1025" s="18">
+        <f>IF(J1025=0,"",L1025/J1025)</f>
+        <v/>
+      </c>
+      <c r="O1025" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:45:50</t>
+        </is>
+      </c>
+      <c r="B1026" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1026" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1026" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1026" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1026" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1026" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H1026" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I1026" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J1026" s="17" t="n">
+        <v>327682.3688910253</v>
+      </c>
+      <c r="K1026" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,363.1264</t>
+        </is>
+      </c>
+      <c r="L1026" s="17" t="n">
+        <v>280211.1505239431</v>
+      </c>
+      <c r="M1026" s="17">
+        <f>J1026-L1026</f>
+        <v/>
+      </c>
+      <c r="N1026" s="18">
+        <f>IF(J1026=0,"",L1026/J1026)</f>
+        <v/>
+      </c>
+      <c r="O1026" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:45:50</t>
+        </is>
+      </c>
+      <c r="B1027" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1027" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1027" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1027" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1027" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1027" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H1027" s="16" t="n">
+        <v>1.9047</v>
+      </c>
+      <c r="I1027" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J1027" s="17" t="n">
+        <v>160068.5465239572</v>
+      </c>
+      <c r="K1027" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,952.6109</t>
+        </is>
+      </c>
+      <c r="L1027" s="17" t="n">
+        <v>70966.80428830975</v>
+      </c>
+      <c r="M1027" s="17">
+        <f>J1027-L1027</f>
+        <v/>
+      </c>
+      <c r="N1027" s="18">
+        <f>IF(J1027=0,"",L1027/J1027)</f>
+        <v/>
+      </c>
+      <c r="O1027" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:45:50</t>
+        </is>
+      </c>
+      <c r="B1028" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1028" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1028" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1028" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1028" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1028" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H1028" s="16" t="n">
+        <v>1.0571</v>
+      </c>
+      <c r="I1028" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J1028" s="17" t="n">
+        <v>160169.2660219746</v>
+      </c>
+      <c r="K1028" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,532.9072</t>
+        </is>
+      </c>
+      <c r="L1028" s="17" t="n">
+        <v>138602.1736079078</v>
+      </c>
+      <c r="M1028" s="17">
+        <f>J1028-L1028</f>
+        <v/>
+      </c>
+      <c r="N1028" s="18">
+        <f>IF(J1028=0,"",L1028/J1028)</f>
+        <v/>
+      </c>
+      <c r="O1028" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:45:50</t>
+        </is>
+      </c>
+      <c r="B1029" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1029" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1029" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E1029" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1029" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G1029" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1029" s="16" t="inlineStr"/>
+      <c r="I1029" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J1029" s="17" t="n">
+        <v>95929.19594099405</v>
+      </c>
+      <c r="K1029" s="15" t="inlineStr"/>
+      <c r="L1029" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1029" s="17">
+        <f>J1029-L1029</f>
+        <v/>
+      </c>
+      <c r="N1029" s="18">
+        <f>IF(J1029=0,"",L1029/J1029)</f>
+        <v/>
+      </c>
+      <c r="O1029" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:45:50</t>
+        </is>
+      </c>
+      <c r="B1030" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1030" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1030" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E1030" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1030" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G1030" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1030" s="16" t="inlineStr"/>
+      <c r="I1030" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J1030" s="17" t="n">
+        <v>34367.19836750623</v>
+      </c>
+      <c r="K1030" s="15" t="inlineStr"/>
+      <c r="L1030" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1030" s="17">
+        <f>J1030-L1030</f>
+        <v/>
+      </c>
+      <c r="N1030" s="18">
+        <f>IF(J1030=0,"",L1030/J1030)</f>
+        <v/>
+      </c>
+      <c r="O1030" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:45:50</t>
+        </is>
+      </c>
+      <c r="B1031" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1031" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D1031" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E1031" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1031" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G1031" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H1031" s="16" t="n">
+        <v>1.0435</v>
+      </c>
+      <c r="I1031" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J1031" s="17" t="n">
+        <v>270082.196272128</v>
+      </c>
+      <c r="K1031" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,071.2752</t>
+        </is>
+      </c>
+      <c r="L1031" s="17" t="n">
+        <v>232931.4324768548</v>
+      </c>
+      <c r="M1031" s="17">
+        <f>J1031-L1031</f>
+        <v/>
+      </c>
+      <c r="N1031" s="18">
+        <f>IF(J1031=0,"",L1031/J1031)</f>
+        <v/>
+      </c>
+      <c r="O1031" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:45:50</t>
+        </is>
+      </c>
+      <c r="B1032" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1032" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D1032" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E1032" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1032" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G1032" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1032" s="16" t="inlineStr"/>
+      <c r="I1032" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,519.4771</t>
+        </is>
+      </c>
+      <c r="J1032" s="17" t="n">
+        <v>15510.16546269238</v>
+      </c>
+      <c r="K1032" s="15" t="inlineStr"/>
+      <c r="L1032" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1032" s="17">
+        <f>J1032-L1032</f>
+        <v/>
+      </c>
+      <c r="N1032" s="18">
+        <f>IF(J1032=0,"",L1032/J1032)</f>
+        <v/>
+      </c>
+      <c r="O1032" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:45:50</t>
+        </is>
+      </c>
+      <c r="B1033" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1033" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D1033" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E1033" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1033" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G1033" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H1033" s="16" t="n">
+        <v>1.219</v>
+      </c>
+      <c r="I1033" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J1033" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K1033" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,736.3177</t>
+        </is>
+      </c>
+      <c r="L1033" s="17" t="n">
+        <v>148736.317674</v>
+      </c>
+      <c r="M1033" s="17">
+        <f>J1033-L1033</f>
+        <v/>
+      </c>
+      <c r="N1033" s="18">
+        <f>IF(J1033=0,"",L1033/J1033)</f>
+        <v/>
+      </c>
+      <c r="O1033" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1034">
+      <c r="A1034" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:45:50</t>
+        </is>
+      </c>
+      <c r="B1034" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1034" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D1034" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E1034" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1034" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G1034" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H1034" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I1034" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J1034" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K1034" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L1034" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M1034" s="17">
+        <f>J1034-L1034</f>
+        <v/>
+      </c>
+      <c r="N1034" s="18">
+        <f>IF(J1034=0,"",L1034/J1034)</f>
+        <v/>
+      </c>
+      <c r="O1034" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -69160,7 +70246,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I67"/>
+  <dimension ref="A1:I68"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -71521,6 +72607,41 @@
         <v>1.0372</v>
       </c>
       <c r="I67" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 09:45:50</t>
+        </is>
+      </c>
+      <c r="B68" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C68" s="17" t="n">
+        <v>655496.1654625398</v>
+      </c>
+      <c r="D68" s="17" t="n">
+        <v>652907.3020094065</v>
+      </c>
+      <c r="E68" s="17" t="n">
+        <v>2933829.420933811</v>
+      </c>
+      <c r="F68" s="17" t="n">
+        <v>2280922.118924404</v>
+      </c>
+      <c r="G68" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H68" s="16" t="n">
+        <v>1.0372</v>
+      </c>
+      <c r="I68" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-30 10:16 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O1034"/>
+  <dimension ref="A1:O1050"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -70216,6 +70216,1092 @@
         <v/>
       </c>
       <c r="O1034" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:16:00</t>
+        </is>
+      </c>
+      <c r="B1035" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1035" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1035" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E1035" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1035" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G1035" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H1035" s="16" t="n">
+        <v>1.0503</v>
+      </c>
+      <c r="I1035" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,809.3004</t>
+        </is>
+      </c>
+      <c r="J1035" s="17" t="n">
+        <v>50787.9605088257</v>
+      </c>
+      <c r="K1035" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,726.6826</t>
+        </is>
+      </c>
+      <c r="L1035" s="17" t="n">
+        <v>37738.00397219165</v>
+      </c>
+      <c r="M1035" s="17">
+        <f>J1035-L1035</f>
+        <v/>
+      </c>
+      <c r="N1035" s="18">
+        <f>IF(J1035=0,"",L1035/J1035)</f>
+        <v/>
+      </c>
+      <c r="O1035" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1036">
+      <c r="A1036" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:16:00</t>
+        </is>
+      </c>
+      <c r="B1036" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1036" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1036" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E1036" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1036" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G1036" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H1036" s="16" t="n">
+        <v>1.0484</v>
+      </c>
+      <c r="I1036" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J1036" s="17" t="n">
+        <v>140942.7092588259</v>
+      </c>
+      <c r="K1036" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,048.3985</t>
+        </is>
+      </c>
+      <c r="L1036" s="17" t="n">
+        <v>120997.5581906224</v>
+      </c>
+      <c r="M1036" s="17">
+        <f>J1036-L1036</f>
+        <v/>
+      </c>
+      <c r="N1036" s="18">
+        <f>IF(J1036=0,"",L1036/J1036)</f>
+        <v/>
+      </c>
+      <c r="O1036" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1037">
+      <c r="A1037" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:16:00</t>
+        </is>
+      </c>
+      <c r="B1037" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1037" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1037" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E1037" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1037" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G1037" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H1037" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I1037" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J1037" s="17" t="n">
+        <v>328744.1019695384</v>
+      </c>
+      <c r="K1037" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,401.0536</t>
+        </is>
+      </c>
+      <c r="L1037" s="17" t="n">
+        <v>306530.459933298</v>
+      </c>
+      <c r="M1037" s="17">
+        <f>J1037-L1037</f>
+        <v/>
+      </c>
+      <c r="N1037" s="18">
+        <f>IF(J1037=0,"",L1037/J1037)</f>
+        <v/>
+      </c>
+      <c r="O1037" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:16:00</t>
+        </is>
+      </c>
+      <c r="B1038" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1038" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1038" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E1038" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1038" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G1038" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H1038" s="16" t="n">
+        <v>1.0372</v>
+      </c>
+      <c r="I1038" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J1038" s="17" t="n">
+        <v>386069.4144570826</v>
+      </c>
+      <c r="K1038" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,631.2289</t>
+        </is>
+      </c>
+      <c r="L1038" s="17" t="n">
+        <v>349778.8931724339</v>
+      </c>
+      <c r="M1038" s="17">
+        <f>J1038-L1038</f>
+        <v/>
+      </c>
+      <c r="N1038" s="18">
+        <f>IF(J1038=0,"",L1038/J1038)</f>
+        <v/>
+      </c>
+      <c r="O1038" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:16:00</t>
+        </is>
+      </c>
+      <c r="B1039" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1039" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D1039" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E1039" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1039" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G1039" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H1039" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I1039" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7873</t>
+        </is>
+      </c>
+      <c r="J1039" s="17" t="n">
+        <v>77780.2739188277</v>
+      </c>
+      <c r="K1039" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,034.4625; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L1039" s="17" t="n">
+        <v>68005.96565201125</v>
+      </c>
+      <c r="M1039" s="17">
+        <f>J1039-L1039</f>
+        <v/>
+      </c>
+      <c r="N1039" s="18">
+        <f>IF(J1039=0,"",L1039/J1039)</f>
+        <v/>
+      </c>
+      <c r="O1039" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:16:00</t>
+        </is>
+      </c>
+      <c r="B1040" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1040" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1040" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1040" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1040" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1040" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H1040" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I1040" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J1040" s="17" t="n">
+        <v>197149.6359252165</v>
+      </c>
+      <c r="K1040" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,262.3037</t>
+        </is>
+      </c>
+      <c r="L1040" s="17" t="n">
+        <v>150307.3959050264</v>
+      </c>
+      <c r="M1040" s="17">
+        <f>J1040-L1040</f>
+        <v/>
+      </c>
+      <c r="N1040" s="18">
+        <f>IF(J1040=0,"",L1040/J1040)</f>
+        <v/>
+      </c>
+      <c r="O1040" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:16:00</t>
+        </is>
+      </c>
+      <c r="B1041" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1041" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1041" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1041" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1041" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1041" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H1041" s="16" t="n">
+        <v>1.3728</v>
+      </c>
+      <c r="I1041" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J1041" s="17" t="n">
+        <v>186073.1239035263</v>
+      </c>
+      <c r="K1041" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,161.1962</t>
+        </is>
+      </c>
+      <c r="L1041" s="17" t="n">
+        <v>124198.4557182379</v>
+      </c>
+      <c r="M1041" s="17">
+        <f>J1041-L1041</f>
+        <v/>
+      </c>
+      <c r="N1041" s="18">
+        <f>IF(J1041=0,"",L1041/J1041)</f>
+        <v/>
+      </c>
+      <c r="O1041" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:16:00</t>
+        </is>
+      </c>
+      <c r="B1042" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1042" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1042" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1042" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1042" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1042" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H1042" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I1042" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J1042" s="17" t="n">
+        <v>327685.2120049303</v>
+      </c>
+      <c r="K1042" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,363.1264</t>
+        </is>
+      </c>
+      <c r="L1042" s="17" t="n">
+        <v>280244.6123049684</v>
+      </c>
+      <c r="M1042" s="17">
+        <f>J1042-L1042</f>
+        <v/>
+      </c>
+      <c r="N1042" s="18">
+        <f>IF(J1042=0,"",L1042/J1042)</f>
+        <v/>
+      </c>
+      <c r="O1042" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:16:00</t>
+        </is>
+      </c>
+      <c r="B1043" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1043" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1043" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1043" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1043" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1043" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H1043" s="16" t="n">
+        <v>1.9047</v>
+      </c>
+      <c r="I1043" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J1043" s="17" t="n">
+        <v>160068.5465239572</v>
+      </c>
+      <c r="K1043" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,952.6109</t>
+        </is>
+      </c>
+      <c r="L1043" s="17" t="n">
+        <v>70973.90309838159</v>
+      </c>
+      <c r="M1043" s="17">
+        <f>J1043-L1043</f>
+        <v/>
+      </c>
+      <c r="N1043" s="18">
+        <f>IF(J1043=0,"",L1043/J1043)</f>
+        <v/>
+      </c>
+      <c r="O1043" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1044">
+      <c r="A1044" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:16:00</t>
+        </is>
+      </c>
+      <c r="B1044" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1044" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1044" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1044" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1044" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1044" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H1044" s="16" t="n">
+        <v>1.0571</v>
+      </c>
+      <c r="I1044" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J1044" s="17" t="n">
+        <v>160169.7532998793</v>
+      </c>
+      <c r="K1044" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,532.9072</t>
+        </is>
+      </c>
+      <c r="L1044" s="17" t="n">
+        <v>138602.1736079078</v>
+      </c>
+      <c r="M1044" s="17">
+        <f>J1044-L1044</f>
+        <v/>
+      </c>
+      <c r="N1044" s="18">
+        <f>IF(J1044=0,"",L1044/J1044)</f>
+        <v/>
+      </c>
+      <c r="O1044" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1045">
+      <c r="A1045" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:16:00</t>
+        </is>
+      </c>
+      <c r="B1045" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1045" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1045" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E1045" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1045" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G1045" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1045" s="16" t="inlineStr"/>
+      <c r="I1045" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J1045" s="17" t="n">
+        <v>95919.60014266046</v>
+      </c>
+      <c r="K1045" s="15" t="inlineStr"/>
+      <c r="L1045" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1045" s="17">
+        <f>J1045-L1045</f>
+        <v/>
+      </c>
+      <c r="N1045" s="18">
+        <f>IF(J1045=0,"",L1045/J1045)</f>
+        <v/>
+      </c>
+      <c r="O1045" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1046">
+      <c r="A1046" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:16:00</t>
+        </is>
+      </c>
+      <c r="B1046" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1046" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1046" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E1046" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1046" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G1046" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1046" s="16" t="inlineStr"/>
+      <c r="I1046" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J1046" s="17" t="n">
+        <v>34367.39700376305</v>
+      </c>
+      <c r="K1046" s="15" t="inlineStr"/>
+      <c r="L1046" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1046" s="17">
+        <f>J1046-L1046</f>
+        <v/>
+      </c>
+      <c r="N1046" s="18">
+        <f>IF(J1046=0,"",L1046/J1046)</f>
+        <v/>
+      </c>
+      <c r="O1046" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1047">
+      <c r="A1047" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:16:00</t>
+        </is>
+      </c>
+      <c r="B1047" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1047" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D1047" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E1047" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1047" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G1047" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H1047" s="16" t="n">
+        <v>1.0433</v>
+      </c>
+      <c r="I1047" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J1047" s="17" t="n">
+        <v>270055.1826497763</v>
+      </c>
+      <c r="K1047" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,071.2752</t>
+        </is>
+      </c>
+      <c r="L1047" s="17" t="n">
+        <v>232973.3853063984</v>
+      </c>
+      <c r="M1047" s="17">
+        <f>J1047-L1047</f>
+        <v/>
+      </c>
+      <c r="N1047" s="18">
+        <f>IF(J1047=0,"",L1047/J1047)</f>
+        <v/>
+      </c>
+      <c r="O1047" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1048">
+      <c r="A1048" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:16:00</t>
+        </is>
+      </c>
+      <c r="B1048" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1048" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D1048" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E1048" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1048" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G1048" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1048" s="16" t="inlineStr"/>
+      <c r="I1048" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,519.5022</t>
+        </is>
+      </c>
+      <c r="J1048" s="17" t="n">
+        <v>15512.98400120715</v>
+      </c>
+      <c r="K1048" s="15" t="inlineStr"/>
+      <c r="L1048" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1048" s="17">
+        <f>J1048-L1048</f>
+        <v/>
+      </c>
+      <c r="N1048" s="18">
+        <f>IF(J1048=0,"",L1048/J1048)</f>
+        <v/>
+      </c>
+      <c r="O1048" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1049">
+      <c r="A1049" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:16:00</t>
+        </is>
+      </c>
+      <c r="B1049" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1049" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D1049" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E1049" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1049" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G1049" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H1049" s="16" t="n">
+        <v>1.219</v>
+      </c>
+      <c r="I1049" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J1049" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K1049" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,736.3177</t>
+        </is>
+      </c>
+      <c r="L1049" s="17" t="n">
+        <v>148736.317674</v>
+      </c>
+      <c r="M1049" s="17">
+        <f>J1049-L1049</f>
+        <v/>
+      </c>
+      <c r="N1049" s="18">
+        <f>IF(J1049=0,"",L1049/J1049)</f>
+        <v/>
+      </c>
+      <c r="O1049" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1050">
+      <c r="A1050" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:16:00</t>
+        </is>
+      </c>
+      <c r="B1050" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1050" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D1050" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E1050" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1050" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G1050" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H1050" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I1050" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J1050" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K1050" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L1050" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M1050" s="17">
+        <f>J1050-L1050</f>
+        <v/>
+      </c>
+      <c r="N1050" s="18">
+        <f>IF(J1050=0,"",L1050/J1050)</f>
+        <v/>
+      </c>
+      <c r="O1050" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -70246,7 +71332,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I68"/>
+  <dimension ref="A1:I69"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -72642,6 +73728,41 @@
         <v>1.0372</v>
       </c>
       <c r="I68" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:16:00</t>
+        </is>
+      </c>
+      <c r="B69" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C69" s="17" t="n">
+        <v>655328.2461389385</v>
+      </c>
+      <c r="D69" s="17" t="n">
+        <v>652739.6045194888</v>
+      </c>
+      <c r="E69" s="17" t="n">
+        <v>2933809.276158966</v>
+      </c>
+      <c r="F69" s="17" t="n">
+        <v>2281069.671639477</v>
+      </c>
+      <c r="G69" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H69" s="16" t="n">
+        <v>1.0372</v>
+      </c>
+      <c r="I69" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-30 10:46 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O1050"/>
+  <dimension ref="A1:O1066"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -71302,6 +71302,1092 @@
         <v/>
       </c>
       <c r="O1050" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1051">
+      <c r="A1051" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:46:10</t>
+        </is>
+      </c>
+      <c r="B1051" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1051" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1051" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E1051" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1051" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G1051" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H1051" s="16" t="n">
+        <v>1.0503</v>
+      </c>
+      <c r="I1051" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,809.3004</t>
+        </is>
+      </c>
+      <c r="J1051" s="17" t="n">
+        <v>50787.9605088257</v>
+      </c>
+      <c r="K1051" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,726.6826</t>
+        </is>
+      </c>
+      <c r="L1051" s="17" t="n">
+        <v>37738.00397219165</v>
+      </c>
+      <c r="M1051" s="17">
+        <f>J1051-L1051</f>
+        <v/>
+      </c>
+      <c r="N1051" s="18">
+        <f>IF(J1051=0,"",L1051/J1051)</f>
+        <v/>
+      </c>
+      <c r="O1051" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1052">
+      <c r="A1052" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:46:10</t>
+        </is>
+      </c>
+      <c r="B1052" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1052" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1052" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E1052" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1052" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G1052" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H1052" s="16" t="n">
+        <v>1.0484</v>
+      </c>
+      <c r="I1052" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J1052" s="17" t="n">
+        <v>140949.9588785496</v>
+      </c>
+      <c r="K1052" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,048.3985</t>
+        </is>
+      </c>
+      <c r="L1052" s="17" t="n">
+        <v>120997.5581906224</v>
+      </c>
+      <c r="M1052" s="17">
+        <f>J1052-L1052</f>
+        <v/>
+      </c>
+      <c r="N1052" s="18">
+        <f>IF(J1052=0,"",L1052/J1052)</f>
+        <v/>
+      </c>
+      <c r="O1052" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1053">
+      <c r="A1053" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:46:10</t>
+        </is>
+      </c>
+      <c r="B1053" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1053" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1053" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E1053" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1053" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G1053" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H1053" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I1053" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J1053" s="17" t="n">
+        <v>328745.8871108564</v>
+      </c>
+      <c r="K1053" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,401.0536</t>
+        </is>
+      </c>
+      <c r="L1053" s="17" t="n">
+        <v>306530.4586982685</v>
+      </c>
+      <c r="M1053" s="17">
+        <f>J1053-L1053</f>
+        <v/>
+      </c>
+      <c r="N1053" s="18">
+        <f>IF(J1053=0,"",L1053/J1053)</f>
+        <v/>
+      </c>
+      <c r="O1053" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1054">
+      <c r="A1054" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:46:10</t>
+        </is>
+      </c>
+      <c r="B1054" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1054" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1054" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E1054" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1054" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G1054" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H1054" s="16" t="n">
+        <v>1.0372</v>
+      </c>
+      <c r="I1054" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J1054" s="17" t="n">
+        <v>386070.5657988511</v>
+      </c>
+      <c r="K1054" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,631.2289</t>
+        </is>
+      </c>
+      <c r="L1054" s="17" t="n">
+        <v>349778.8917631539</v>
+      </c>
+      <c r="M1054" s="17">
+        <f>J1054-L1054</f>
+        <v/>
+      </c>
+      <c r="N1054" s="18">
+        <f>IF(J1054=0,"",L1054/J1054)</f>
+        <v/>
+      </c>
+      <c r="O1054" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1055">
+      <c r="A1055" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:46:10</t>
+        </is>
+      </c>
+      <c r="B1055" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1055" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D1055" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E1055" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1055" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G1055" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H1055" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I1055" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7873</t>
+        </is>
+      </c>
+      <c r="J1055" s="17" t="n">
+        <v>77771.73267593845</v>
+      </c>
+      <c r="K1055" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,034.4625; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L1055" s="17" t="n">
+        <v>68005.96565201125</v>
+      </c>
+      <c r="M1055" s="17">
+        <f>J1055-L1055</f>
+        <v/>
+      </c>
+      <c r="N1055" s="18">
+        <f>IF(J1055=0,"",L1055/J1055)</f>
+        <v/>
+      </c>
+      <c r="O1055" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1056">
+      <c r="A1056" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:46:10</t>
+        </is>
+      </c>
+      <c r="B1056" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1056" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1056" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1056" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1056" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1056" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H1056" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I1056" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J1056" s="17" t="n">
+        <v>197151.5308319323</v>
+      </c>
+      <c r="K1056" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,262.3037</t>
+        </is>
+      </c>
+      <c r="L1056" s="17" t="n">
+        <v>150307.3959050264</v>
+      </c>
+      <c r="M1056" s="17">
+        <f>J1056-L1056</f>
+        <v/>
+      </c>
+      <c r="N1056" s="18">
+        <f>IF(J1056=0,"",L1056/J1056)</f>
+        <v/>
+      </c>
+      <c r="O1056" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1057">
+      <c r="A1057" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:46:10</t>
+        </is>
+      </c>
+      <c r="B1057" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1057" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1057" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1057" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1057" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1057" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H1057" s="16" t="n">
+        <v>1.3728</v>
+      </c>
+      <c r="I1057" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J1057" s="17" t="n">
+        <v>186073.5648024719</v>
+      </c>
+      <c r="K1057" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,161.1962</t>
+        </is>
+      </c>
+      <c r="L1057" s="17" t="n">
+        <v>124198.4557182379</v>
+      </c>
+      <c r="M1057" s="17">
+        <f>J1057-L1057</f>
+        <v/>
+      </c>
+      <c r="N1057" s="18">
+        <f>IF(J1057=0,"",L1057/J1057)</f>
+        <v/>
+      </c>
+      <c r="O1057" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1058">
+      <c r="A1058" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:46:10</t>
+        </is>
+      </c>
+      <c r="B1058" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1058" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1058" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1058" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1058" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1058" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H1058" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I1058" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J1058" s="17" t="n">
+        <v>327728.7556704286</v>
+      </c>
+      <c r="K1058" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,363.1264</t>
+        </is>
+      </c>
+      <c r="L1058" s="17" t="n">
+        <v>280222.7761843282</v>
+      </c>
+      <c r="M1058" s="17">
+        <f>J1058-L1058</f>
+        <v/>
+      </c>
+      <c r="N1058" s="18">
+        <f>IF(J1058=0,"",L1058/J1058)</f>
+        <v/>
+      </c>
+      <c r="O1058" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1059">
+      <c r="A1059" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:46:10</t>
+        </is>
+      </c>
+      <c r="B1059" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1059" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1059" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1059" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1059" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1059" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H1059" s="16" t="n">
+        <v>1.9047</v>
+      </c>
+      <c r="I1059" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J1059" s="17" t="n">
+        <v>160068.5465239572</v>
+      </c>
+      <c r="K1059" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,952.6109</t>
+        </is>
+      </c>
+      <c r="L1059" s="17" t="n">
+        <v>70973.90309838159</v>
+      </c>
+      <c r="M1059" s="17">
+        <f>J1059-L1059</f>
+        <v/>
+      </c>
+      <c r="N1059" s="18">
+        <f>IF(J1059=0,"",L1059/J1059)</f>
+        <v/>
+      </c>
+      <c r="O1059" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1060">
+      <c r="A1060" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:46:10</t>
+        </is>
+      </c>
+      <c r="B1060" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1060" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1060" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1060" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1060" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1060" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H1060" s="16" t="n">
+        <v>1.0571</v>
+      </c>
+      <c r="I1060" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J1060" s="17" t="n">
+        <v>160170.2309604246</v>
+      </c>
+      <c r="K1060" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,532.9072</t>
+        </is>
+      </c>
+      <c r="L1060" s="17" t="n">
+        <v>138574.4670264769</v>
+      </c>
+      <c r="M1060" s="17">
+        <f>J1060-L1060</f>
+        <v/>
+      </c>
+      <c r="N1060" s="18">
+        <f>IF(J1060=0,"",L1060/J1060)</f>
+        <v/>
+      </c>
+      <c r="O1060" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1061">
+      <c r="A1061" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:46:10</t>
+        </is>
+      </c>
+      <c r="B1061" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1061" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1061" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E1061" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1061" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G1061" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1061" s="16" t="inlineStr"/>
+      <c r="I1061" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J1061" s="17" t="n">
+        <v>95919.24131996292</v>
+      </c>
+      <c r="K1061" s="15" t="inlineStr"/>
+      <c r="L1061" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1061" s="17">
+        <f>J1061-L1061</f>
+        <v/>
+      </c>
+      <c r="N1061" s="18">
+        <f>IF(J1061=0,"",L1061/J1061)</f>
+        <v/>
+      </c>
+      <c r="O1061" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1062">
+      <c r="A1062" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:46:10</t>
+        </is>
+      </c>
+      <c r="B1062" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1062" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1062" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E1062" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1062" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G1062" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1062" s="16" t="inlineStr"/>
+      <c r="I1062" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J1062" s="17" t="n">
+        <v>34367.70940674419</v>
+      </c>
+      <c r="K1062" s="15" t="inlineStr"/>
+      <c r="L1062" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1062" s="17">
+        <f>J1062-L1062</f>
+        <v/>
+      </c>
+      <c r="N1062" s="18">
+        <f>IF(J1062=0,"",L1062/J1062)</f>
+        <v/>
+      </c>
+      <c r="O1062" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1063">
+      <c r="A1063" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:46:10</t>
+        </is>
+      </c>
+      <c r="B1063" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1063" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D1063" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E1063" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1063" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G1063" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H1063" s="16" t="n">
+        <v>1.0434</v>
+      </c>
+      <c r="I1063" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J1063" s="17" t="n">
+        <v>270082.196272128</v>
+      </c>
+      <c r="K1063" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,071.2752</t>
+        </is>
+      </c>
+      <c r="L1063" s="17" t="n">
+        <v>232973.3853063984</v>
+      </c>
+      <c r="M1063" s="17">
+        <f>J1063-L1063</f>
+        <v/>
+      </c>
+      <c r="N1063" s="18">
+        <f>IF(J1063=0,"",L1063/J1063)</f>
+        <v/>
+      </c>
+      <c r="O1063" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1064">
+      <c r="A1064" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:46:10</t>
+        </is>
+      </c>
+      <c r="B1064" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1064" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D1064" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E1064" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1064" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G1064" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1064" s="16" t="inlineStr"/>
+      <c r="I1064" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,519.7121</t>
+        </is>
+      </c>
+      <c r="J1064" s="17" t="n">
+        <v>15513.1938037653</v>
+      </c>
+      <c r="K1064" s="15" t="inlineStr"/>
+      <c r="L1064" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1064" s="17">
+        <f>J1064-L1064</f>
+        <v/>
+      </c>
+      <c r="N1064" s="18">
+        <f>IF(J1064=0,"",L1064/J1064)</f>
+        <v/>
+      </c>
+      <c r="O1064" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1065">
+      <c r="A1065" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:46:10</t>
+        </is>
+      </c>
+      <c r="B1065" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1065" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D1065" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E1065" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1065" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G1065" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H1065" s="16" t="n">
+        <v>1.219</v>
+      </c>
+      <c r="I1065" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J1065" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K1065" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,736.3177</t>
+        </is>
+      </c>
+      <c r="L1065" s="17" t="n">
+        <v>148736.317674</v>
+      </c>
+      <c r="M1065" s="17">
+        <f>J1065-L1065</f>
+        <v/>
+      </c>
+      <c r="N1065" s="18">
+        <f>IF(J1065=0,"",L1065/J1065)</f>
+        <v/>
+      </c>
+      <c r="O1065" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1066">
+      <c r="A1066" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:46:10</t>
+        </is>
+      </c>
+      <c r="B1066" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1066" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D1066" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E1066" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1066" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G1066" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H1066" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I1066" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J1066" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K1066" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L1066" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M1066" s="17">
+        <f>J1066-L1066</f>
+        <v/>
+      </c>
+      <c r="N1066" s="18">
+        <f>IF(J1066=0,"",L1066/J1066)</f>
+        <v/>
+      </c>
+      <c r="O1066" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -71332,7 +72418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I69"/>
+  <dimension ref="A1:I70"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -73763,6 +74849,41 @@
         <v>1.0372</v>
       </c>
       <c r="I69" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:46:10</t>
+        </is>
+      </c>
+      <c r="B70" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C70" s="17" t="n">
+        <v>655452.3660514022</v>
+      </c>
+      <c r="D70" s="17" t="n">
+        <v>652864.328862689</v>
+      </c>
+      <c r="E70" s="17" t="n">
+        <v>2933884.455155786</v>
+      </c>
+      <c r="F70" s="17" t="n">
+        <v>2281020.126293097</v>
+      </c>
+      <c r="G70" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H70" s="16" t="n">
+        <v>1.0372</v>
+      </c>
+      <c r="I70" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-30 11:16 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O1066"/>
+  <dimension ref="A1:O1082"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -72388,6 +72388,1092 @@
         <v/>
       </c>
       <c r="O1066" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1067">
+      <c r="A1067" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:16:21</t>
+        </is>
+      </c>
+      <c r="B1067" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1067" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1067" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E1067" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1067" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G1067" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H1067" s="16" t="n">
+        <v>1.0503</v>
+      </c>
+      <c r="I1067" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,809.3004</t>
+        </is>
+      </c>
+      <c r="J1067" s="17" t="n">
+        <v>50787.9605088257</v>
+      </c>
+      <c r="K1067" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,726.6826</t>
+        </is>
+      </c>
+      <c r="L1067" s="17" t="n">
+        <v>37738.00397219165</v>
+      </c>
+      <c r="M1067" s="17">
+        <f>J1067-L1067</f>
+        <v/>
+      </c>
+      <c r="N1067" s="18">
+        <f>IF(J1067=0,"",L1067/J1067)</f>
+        <v/>
+      </c>
+      <c r="O1067" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1068">
+      <c r="A1068" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:16:21</t>
+        </is>
+      </c>
+      <c r="B1068" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1068" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1068" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E1068" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1068" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G1068" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H1068" s="16" t="n">
+        <v>1.0484</v>
+      </c>
+      <c r="I1068" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J1068" s="17" t="n">
+        <v>140950.3764037089</v>
+      </c>
+      <c r="K1068" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,048.3985</t>
+        </is>
+      </c>
+      <c r="L1068" s="17" t="n">
+        <v>120997.5581906224</v>
+      </c>
+      <c r="M1068" s="17">
+        <f>J1068-L1068</f>
+        <v/>
+      </c>
+      <c r="N1068" s="18">
+        <f>IF(J1068=0,"",L1068/J1068)</f>
+        <v/>
+      </c>
+      <c r="O1068" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1069">
+      <c r="A1069" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:16:21</t>
+        </is>
+      </c>
+      <c r="B1069" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1069" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1069" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E1069" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1069" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G1069" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H1069" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I1069" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J1069" s="17" t="n">
+        <v>328745.8871108564</v>
+      </c>
+      <c r="K1069" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,401.0536</t>
+        </is>
+      </c>
+      <c r="L1069" s="17" t="n">
+        <v>306530.4544866591</v>
+      </c>
+      <c r="M1069" s="17">
+        <f>J1069-L1069</f>
+        <v/>
+      </c>
+      <c r="N1069" s="18">
+        <f>IF(J1069=0,"",L1069/J1069)</f>
+        <v/>
+      </c>
+      <c r="O1069" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1070">
+      <c r="A1070" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:16:21</t>
+        </is>
+      </c>
+      <c r="B1070" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1070" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1070" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E1070" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1070" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G1070" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H1070" s="16" t="n">
+        <v>1.0372</v>
+      </c>
+      <c r="I1070" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J1070" s="17" t="n">
+        <v>386071.7248867065</v>
+      </c>
+      <c r="K1070" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,631.2289</t>
+        </is>
+      </c>
+      <c r="L1070" s="17" t="n">
+        <v>349778.8869573279</v>
+      </c>
+      <c r="M1070" s="17">
+        <f>J1070-L1070</f>
+        <v/>
+      </c>
+      <c r="N1070" s="18">
+        <f>IF(J1070=0,"",L1070/J1070)</f>
+        <v/>
+      </c>
+      <c r="O1070" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1071">
+      <c r="A1071" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:16:21</t>
+        </is>
+      </c>
+      <c r="B1071" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1071" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D1071" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E1071" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1071" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G1071" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H1071" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I1071" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7873</t>
+        </is>
+      </c>
+      <c r="J1071" s="17" t="n">
+        <v>77782.67583869018</v>
+      </c>
+      <c r="K1071" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,034.4625; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L1071" s="17" t="n">
+        <v>68005.96565201125</v>
+      </c>
+      <c r="M1071" s="17">
+        <f>J1071-L1071</f>
+        <v/>
+      </c>
+      <c r="N1071" s="18">
+        <f>IF(J1071=0,"",L1071/J1071)</f>
+        <v/>
+      </c>
+      <c r="O1071" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1072">
+      <c r="A1072" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:16:21</t>
+        </is>
+      </c>
+      <c r="B1072" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1072" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1072" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1072" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1072" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1072" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H1072" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I1072" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J1072" s="17" t="n">
+        <v>197146.7945902428</v>
+      </c>
+      <c r="K1072" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,262.3037</t>
+        </is>
+      </c>
+      <c r="L1072" s="17" t="n">
+        <v>150307.3959050264</v>
+      </c>
+      <c r="M1072" s="17">
+        <f>J1072-L1072</f>
+        <v/>
+      </c>
+      <c r="N1072" s="18">
+        <f>IF(J1072=0,"",L1072/J1072)</f>
+        <v/>
+      </c>
+      <c r="O1072" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1073">
+      <c r="A1073" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:16:21</t>
+        </is>
+      </c>
+      <c r="B1073" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1073" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1073" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1073" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1073" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1073" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H1073" s="16" t="n">
+        <v>1.3728</v>
+      </c>
+      <c r="I1073" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J1073" s="17" t="n">
+        <v>186062.6922542367</v>
+      </c>
+      <c r="K1073" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,161.1962</t>
+        </is>
+      </c>
+      <c r="L1073" s="17" t="n">
+        <v>124198.4557182379</v>
+      </c>
+      <c r="M1073" s="17">
+        <f>J1073-L1073</f>
+        <v/>
+      </c>
+      <c r="N1073" s="18">
+        <f>IF(J1073=0,"",L1073/J1073)</f>
+        <v/>
+      </c>
+      <c r="O1073" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1074">
+      <c r="A1074" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:16:21</t>
+        </is>
+      </c>
+      <c r="B1074" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1074" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1074" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1074" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1074" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1074" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H1074" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I1074" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J1074" s="17" t="n">
+        <v>327700.554032061</v>
+      </c>
+      <c r="K1074" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,363.1264</t>
+        </is>
+      </c>
+      <c r="L1074" s="17" t="n">
+        <v>280222.6919302871</v>
+      </c>
+      <c r="M1074" s="17">
+        <f>J1074-L1074</f>
+        <v/>
+      </c>
+      <c r="N1074" s="18">
+        <f>IF(J1074=0,"",L1074/J1074)</f>
+        <v/>
+      </c>
+      <c r="O1074" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1075">
+      <c r="A1075" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:16:21</t>
+        </is>
+      </c>
+      <c r="B1075" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1075" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1075" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1075" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1075" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1075" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H1075" s="16" t="n">
+        <v>1.9047</v>
+      </c>
+      <c r="I1075" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J1075" s="17" t="n">
+        <v>160068.5465239572</v>
+      </c>
+      <c r="K1075" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,952.6109</t>
+        </is>
+      </c>
+      <c r="L1075" s="17" t="n">
+        <v>70973.90309838159</v>
+      </c>
+      <c r="M1075" s="17">
+        <f>J1075-L1075</f>
+        <v/>
+      </c>
+      <c r="N1075" s="18">
+        <f>IF(J1075=0,"",L1075/J1075)</f>
+        <v/>
+      </c>
+      <c r="O1075" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1076">
+      <c r="A1076" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:16:21</t>
+        </is>
+      </c>
+      <c r="B1076" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1076" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1076" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1076" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1076" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1076" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H1076" s="16" t="n">
+        <v>1.0571</v>
+      </c>
+      <c r="I1076" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J1076" s="17" t="n">
+        <v>160170.7118346117</v>
+      </c>
+      <c r="K1076" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,532.9072</t>
+        </is>
+      </c>
+      <c r="L1076" s="17" t="n">
+        <v>138532.9071543306</v>
+      </c>
+      <c r="M1076" s="17">
+        <f>J1076-L1076</f>
+        <v/>
+      </c>
+      <c r="N1076" s="18">
+        <f>IF(J1076=0,"",L1076/J1076)</f>
+        <v/>
+      </c>
+      <c r="O1076" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1077">
+      <c r="A1077" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:16:21</t>
+        </is>
+      </c>
+      <c r="B1077" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1077" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1077" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E1077" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1077" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G1077" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1077" s="16" t="inlineStr"/>
+      <c r="I1077" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J1077" s="17" t="n">
+        <v>95903.61005361634</v>
+      </c>
+      <c r="K1077" s="15" t="inlineStr"/>
+      <c r="L1077" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1077" s="17">
+        <f>J1077-L1077</f>
+        <v/>
+      </c>
+      <c r="N1077" s="18">
+        <f>IF(J1077=0,"",L1077/J1077)</f>
+        <v/>
+      </c>
+      <c r="O1077" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1078">
+      <c r="A1078" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:16:21</t>
+        </is>
+      </c>
+      <c r="B1078" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1078" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1078" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E1078" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1078" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G1078" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1078" s="16" t="inlineStr"/>
+      <c r="I1078" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J1078" s="17" t="n">
+        <v>34370.47866046446</v>
+      </c>
+      <c r="K1078" s="15" t="inlineStr"/>
+      <c r="L1078" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1078" s="17">
+        <f>J1078-L1078</f>
+        <v/>
+      </c>
+      <c r="N1078" s="18">
+        <f>IF(J1078=0,"",L1078/J1078)</f>
+        <v/>
+      </c>
+      <c r="O1078" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1079">
+      <c r="A1079" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:16:21</t>
+        </is>
+      </c>
+      <c r="B1079" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1079" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D1079" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E1079" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1079" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G1079" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H1079" s="16" t="n">
+        <v>1.0434</v>
+      </c>
+      <c r="I1079" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J1079" s="17" t="n">
+        <v>270082.196272128</v>
+      </c>
+      <c r="K1079" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,071.2752</t>
+        </is>
+      </c>
+      <c r="L1079" s="17" t="n">
+        <v>232973.3853063984</v>
+      </c>
+      <c r="M1079" s="17">
+        <f>J1079-L1079</f>
+        <v/>
+      </c>
+      <c r="N1079" s="18">
+        <f>IF(J1079=0,"",L1079/J1079)</f>
+        <v/>
+      </c>
+      <c r="O1079" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1080">
+      <c r="A1080" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:16:21</t>
+        </is>
+      </c>
+      <c r="B1080" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1080" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D1080" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E1080" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1080" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G1080" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1080" s="16" t="inlineStr"/>
+      <c r="I1080" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,520.0163</t>
+        </is>
+      </c>
+      <c r="J1080" s="17" t="n">
+        <v>15513.49789961234</v>
+      </c>
+      <c r="K1080" s="15" t="inlineStr"/>
+      <c r="L1080" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1080" s="17">
+        <f>J1080-L1080</f>
+        <v/>
+      </c>
+      <c r="N1080" s="18">
+        <f>IF(J1080=0,"",L1080/J1080)</f>
+        <v/>
+      </c>
+      <c r="O1080" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1081">
+      <c r="A1081" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:16:21</t>
+        </is>
+      </c>
+      <c r="B1081" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1081" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D1081" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E1081" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1081" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G1081" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H1081" s="16" t="n">
+        <v>1.219</v>
+      </c>
+      <c r="I1081" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J1081" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K1081" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,736.3177</t>
+        </is>
+      </c>
+      <c r="L1081" s="17" t="n">
+        <v>148736.317674</v>
+      </c>
+      <c r="M1081" s="17">
+        <f>J1081-L1081</f>
+        <v/>
+      </c>
+      <c r="N1081" s="18">
+        <f>IF(J1081=0,"",L1081/J1081)</f>
+        <v/>
+      </c>
+      <c r="O1081" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1082">
+      <c r="A1082" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:16:21</t>
+        </is>
+      </c>
+      <c r="B1082" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1082" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D1082" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E1082" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1082" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G1082" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H1082" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I1082" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J1082" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K1082" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L1082" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M1082" s="17">
+        <f>J1082-L1082</f>
+        <v/>
+      </c>
+      <c r="N1082" s="18">
+        <f>IF(J1082=0,"",L1082/J1082)</f>
+        <v/>
+      </c>
+      <c r="O1082" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -72418,7 +73504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I70"/>
+  <dimension ref="A1:I71"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -74884,6 +75970,41 @@
         <v>1.0372</v>
       </c>
       <c r="I70" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:16:21</t>
+        </is>
+      </c>
+      <c r="B71" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C71" s="17" t="n">
+        <v>655450.3685261114</v>
+      </c>
+      <c r="D71" s="17" t="n">
+        <v>652862.614311194</v>
+      </c>
+      <c r="E71" s="17" t="n">
+        <v>2933841.087460668</v>
+      </c>
+      <c r="F71" s="17" t="n">
+        <v>2280978.473149474</v>
+      </c>
+      <c r="G71" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H71" s="16" t="n">
+        <v>1.0372</v>
+      </c>
+      <c r="I71" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-30 11:46 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O1082"/>
+  <dimension ref="A1:O1098"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -73474,6 +73474,1092 @@
         <v/>
       </c>
       <c r="O1082" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1083">
+      <c r="A1083" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:46:31</t>
+        </is>
+      </c>
+      <c r="B1083" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1083" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1083" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E1083" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1083" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G1083" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H1083" s="16" t="n">
+        <v>1.0503</v>
+      </c>
+      <c r="I1083" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,809.3004</t>
+        </is>
+      </c>
+      <c r="J1083" s="17" t="n">
+        <v>50785.9281368091</v>
+      </c>
+      <c r="K1083" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,726.6826</t>
+        </is>
+      </c>
+      <c r="L1083" s="17" t="n">
+        <v>37738.00397219165</v>
+      </c>
+      <c r="M1083" s="17">
+        <f>J1083-L1083</f>
+        <v/>
+      </c>
+      <c r="N1083" s="18">
+        <f>IF(J1083=0,"",L1083/J1083)</f>
+        <v/>
+      </c>
+      <c r="O1083" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1084">
+      <c r="A1084" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:46:31</t>
+        </is>
+      </c>
+      <c r="B1084" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1084" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1084" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E1084" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1084" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G1084" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H1084" s="16" t="n">
+        <v>1.0485</v>
+      </c>
+      <c r="I1084" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J1084" s="17" t="n">
+        <v>140950.6641603388</v>
+      </c>
+      <c r="K1084" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,048.3985</t>
+        </is>
+      </c>
+      <c r="L1084" s="17" t="n">
+        <v>120992.7162546817</v>
+      </c>
+      <c r="M1084" s="17">
+        <f>J1084-L1084</f>
+        <v/>
+      </c>
+      <c r="N1084" s="18">
+        <f>IF(J1084=0,"",L1084/J1084)</f>
+        <v/>
+      </c>
+      <c r="O1084" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1085">
+      <c r="A1085" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:46:31</t>
+        </is>
+      </c>
+      <c r="B1085" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1085" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1085" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E1085" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1085" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G1085" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H1085" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I1085" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J1085" s="17" t="n">
+        <v>328747.337246194</v>
+      </c>
+      <c r="K1085" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,401.0536</t>
+        </is>
+      </c>
+      <c r="L1085" s="17" t="n">
+        <v>306530.0772493006</v>
+      </c>
+      <c r="M1085" s="17">
+        <f>J1085-L1085</f>
+        <v/>
+      </c>
+      <c r="N1085" s="18">
+        <f>IF(J1085=0,"",L1085/J1085)</f>
+        <v/>
+      </c>
+      <c r="O1085" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1086">
+      <c r="A1086" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:46:31</t>
+        </is>
+      </c>
+      <c r="B1086" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1086" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1086" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E1086" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1086" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G1086" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H1086" s="16" t="n">
+        <v>1.0372</v>
+      </c>
+      <c r="I1086" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J1086" s="17" t="n">
+        <v>386072.899431825</v>
+      </c>
+      <c r="K1086" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,631.2289</t>
+        </is>
+      </c>
+      <c r="L1086" s="17" t="n">
+        <v>349778.4564954881</v>
+      </c>
+      <c r="M1086" s="17">
+        <f>J1086-L1086</f>
+        <v/>
+      </c>
+      <c r="N1086" s="18">
+        <f>IF(J1086=0,"",L1086/J1086)</f>
+        <v/>
+      </c>
+      <c r="O1086" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1087">
+      <c r="A1087" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:46:31</t>
+        </is>
+      </c>
+      <c r="B1087" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1087" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D1087" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E1087" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1087" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G1087" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H1087" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I1087" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7873</t>
+        </is>
+      </c>
+      <c r="J1087" s="17" t="n">
+        <v>77781.8623446257</v>
+      </c>
+      <c r="K1087" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,034.4625; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L1087" s="17" t="n">
+        <v>68005.96565201125</v>
+      </c>
+      <c r="M1087" s="17">
+        <f>J1087-L1087</f>
+        <v/>
+      </c>
+      <c r="N1087" s="18">
+        <f>IF(J1087=0,"",L1087/J1087)</f>
+        <v/>
+      </c>
+      <c r="O1087" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1088">
+      <c r="A1088" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:46:31</t>
+        </is>
+      </c>
+      <c r="B1088" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1088" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1088" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1088" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1088" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1088" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H1088" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I1088" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J1088" s="17" t="n">
+        <v>197007.912646085</v>
+      </c>
+      <c r="K1088" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,262.3037</t>
+        </is>
+      </c>
+      <c r="L1088" s="17" t="n">
+        <v>150307.3959050264</v>
+      </c>
+      <c r="M1088" s="17">
+        <f>J1088-L1088</f>
+        <v/>
+      </c>
+      <c r="N1088" s="18">
+        <f>IF(J1088=0,"",L1088/J1088)</f>
+        <v/>
+      </c>
+      <c r="O1088" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1089">
+      <c r="A1089" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:46:31</t>
+        </is>
+      </c>
+      <c r="B1089" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1089" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1089" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1089" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1089" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1089" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H1089" s="16" t="n">
+        <v>1.3728</v>
+      </c>
+      <c r="I1089" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J1089" s="17" t="n">
+        <v>186062.1962967605</v>
+      </c>
+      <c r="K1089" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,161.1962</t>
+        </is>
+      </c>
+      <c r="L1089" s="17" t="n">
+        <v>124198.4557182379</v>
+      </c>
+      <c r="M1089" s="17">
+        <f>J1089-L1089</f>
+        <v/>
+      </c>
+      <c r="N1089" s="18">
+        <f>IF(J1089=0,"",L1089/J1089)</f>
+        <v/>
+      </c>
+      <c r="O1089" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1090">
+      <c r="A1090" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:46:31</t>
+        </is>
+      </c>
+      <c r="B1090" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1090" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1090" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1090" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1090" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1090" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H1090" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I1090" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J1090" s="17" t="n">
+        <v>327700.455502968</v>
+      </c>
+      <c r="K1090" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,363.1264</t>
+        </is>
+      </c>
+      <c r="L1090" s="17" t="n">
+        <v>280226.2427257262</v>
+      </c>
+      <c r="M1090" s="17">
+        <f>J1090-L1090</f>
+        <v/>
+      </c>
+      <c r="N1090" s="18">
+        <f>IF(J1090=0,"",L1090/J1090)</f>
+        <v/>
+      </c>
+      <c r="O1090" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1091">
+      <c r="A1091" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:46:31</t>
+        </is>
+      </c>
+      <c r="B1091" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1091" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1091" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1091" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1091" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1091" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H1091" s="16" t="n">
+        <v>1.9047</v>
+      </c>
+      <c r="I1091" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J1091" s="17" t="n">
+        <v>160068.5465239572</v>
+      </c>
+      <c r="K1091" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,952.6109</t>
+        </is>
+      </c>
+      <c r="L1091" s="17" t="n">
+        <v>70973.90309838159</v>
+      </c>
+      <c r="M1091" s="17">
+        <f>J1091-L1091</f>
+        <v/>
+      </c>
+      <c r="N1091" s="18">
+        <f>IF(J1091=0,"",L1091/J1091)</f>
+        <v/>
+      </c>
+      <c r="O1091" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:46:31</t>
+        </is>
+      </c>
+      <c r="B1092" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1092" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1092" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1092" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1092" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1092" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H1092" s="16" t="n">
+        <v>1.0571</v>
+      </c>
+      <c r="I1092" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J1092" s="17" t="n">
+        <v>160171.199121599</v>
+      </c>
+      <c r="K1092" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,532.9072</t>
+        </is>
+      </c>
+      <c r="L1092" s="17" t="n">
+        <v>138532.9071543306</v>
+      </c>
+      <c r="M1092" s="17">
+        <f>J1092-L1092</f>
+        <v/>
+      </c>
+      <c r="N1092" s="18">
+        <f>IF(J1092=0,"",L1092/J1092)</f>
+        <v/>
+      </c>
+      <c r="O1092" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1093">
+      <c r="A1093" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:46:31</t>
+        </is>
+      </c>
+      <c r="B1093" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1093" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1093" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E1093" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1093" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G1093" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1093" s="16" t="inlineStr"/>
+      <c r="I1093" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J1093" s="17" t="n">
+        <v>95912.43979709387</v>
+      </c>
+      <c r="K1093" s="15" t="inlineStr"/>
+      <c r="L1093" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1093" s="17">
+        <f>J1093-L1093</f>
+        <v/>
+      </c>
+      <c r="N1093" s="18">
+        <f>IF(J1093=0,"",L1093/J1093)</f>
+        <v/>
+      </c>
+      <c r="O1093" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1094">
+      <c r="A1094" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:46:31</t>
+        </is>
+      </c>
+      <c r="B1094" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1094" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1094" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E1094" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1094" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G1094" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1094" s="16" t="inlineStr"/>
+      <c r="I1094" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J1094" s="17" t="n">
+        <v>34370.78820765971</v>
+      </c>
+      <c r="K1094" s="15" t="inlineStr"/>
+      <c r="L1094" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1094" s="17">
+        <f>J1094-L1094</f>
+        <v/>
+      </c>
+      <c r="N1094" s="18">
+        <f>IF(J1094=0,"",L1094/J1094)</f>
+        <v/>
+      </c>
+      <c r="O1094" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1095">
+      <c r="A1095" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:46:31</t>
+        </is>
+      </c>
+      <c r="B1095" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1095" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D1095" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E1095" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1095" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G1095" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H1095" s="16" t="n">
+        <v>1.0434</v>
+      </c>
+      <c r="I1095" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J1095" s="17" t="n">
+        <v>270082.196272128</v>
+      </c>
+      <c r="K1095" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,071.2752</t>
+        </is>
+      </c>
+      <c r="L1095" s="17" t="n">
+        <v>232973.3853063984</v>
+      </c>
+      <c r="M1095" s="17">
+        <f>J1095-L1095</f>
+        <v/>
+      </c>
+      <c r="N1095" s="18">
+        <f>IF(J1095=0,"",L1095/J1095)</f>
+        <v/>
+      </c>
+      <c r="O1095" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:46:31</t>
+        </is>
+      </c>
+      <c r="B1096" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1096" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D1096" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E1096" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1096" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G1096" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1096" s="16" t="inlineStr"/>
+      <c r="I1096" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,520.2858</t>
+        </is>
+      </c>
+      <c r="J1096" s="17" t="n">
+        <v>15513.76730900312</v>
+      </c>
+      <c r="K1096" s="15" t="inlineStr"/>
+      <c r="L1096" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1096" s="17">
+        <f>J1096-L1096</f>
+        <v/>
+      </c>
+      <c r="N1096" s="18">
+        <f>IF(J1096=0,"",L1096/J1096)</f>
+        <v/>
+      </c>
+      <c r="O1096" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1097">
+      <c r="A1097" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:46:31</t>
+        </is>
+      </c>
+      <c r="B1097" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1097" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D1097" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E1097" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1097" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G1097" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H1097" s="16" t="n">
+        <v>1.219</v>
+      </c>
+      <c r="I1097" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J1097" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K1097" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,736.3177</t>
+        </is>
+      </c>
+      <c r="L1097" s="17" t="n">
+        <v>148736.317674</v>
+      </c>
+      <c r="M1097" s="17">
+        <f>J1097-L1097</f>
+        <v/>
+      </c>
+      <c r="N1097" s="18">
+        <f>IF(J1097=0,"",L1097/J1097)</f>
+        <v/>
+      </c>
+      <c r="O1097" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1098">
+      <c r="A1098" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:46:31</t>
+        </is>
+      </c>
+      <c r="B1098" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1098" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D1098" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E1098" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1098" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G1098" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H1098" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I1098" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J1098" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K1098" s="15" t="inlineStr">
+        <is>
+          <t>USDC 251,982.5471</t>
+        </is>
+      </c>
+      <c r="L1098" s="17" t="n">
+        <v>251982.547104</v>
+      </c>
+      <c r="M1098" s="17">
+        <f>J1098-L1098</f>
+        <v/>
+      </c>
+      <c r="N1098" s="18">
+        <f>IF(J1098=0,"",L1098/J1098)</f>
+        <v/>
+      </c>
+      <c r="O1098" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -73504,7 +74590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I71"/>
+  <dimension ref="A1:I72"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -76005,6 +77091,41 @@
         <v>1.0372</v>
       </c>
       <c r="I71" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 11:46:31</t>
+        </is>
+      </c>
+      <c r="B72" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C72" s="17" t="n">
+        <v>655322.5948385933</v>
+      </c>
+      <c r="D72" s="17" t="n">
+        <v>652735.1992782224</v>
+      </c>
+      <c r="E72" s="17" t="n">
+        <v>2933711.573587997</v>
+      </c>
+      <c r="F72" s="17" t="n">
+        <v>2280976.374309774</v>
+      </c>
+      <c r="G72" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H72" s="16" t="n">
+        <v>1.0372</v>
+      </c>
+      <c r="I72" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-30 12:16 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O1098"/>
+  <dimension ref="A1:O1114"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -74560,6 +74560,1092 @@
         <v/>
       </c>
       <c r="O1098" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:16:41</t>
+        </is>
+      </c>
+      <c r="B1099" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1099" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1099" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E1099" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1099" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G1099" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H1099" s="16" t="n">
+        <v>1.0503</v>
+      </c>
+      <c r="I1099" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,809.3004</t>
+        </is>
+      </c>
+      <c r="J1099" s="17" t="n">
+        <v>50780.33911376345</v>
+      </c>
+      <c r="K1099" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,726.6826</t>
+        </is>
+      </c>
+      <c r="L1099" s="17" t="n">
+        <v>37738.00397219165</v>
+      </c>
+      <c r="M1099" s="17">
+        <f>J1099-L1099</f>
+        <v/>
+      </c>
+      <c r="N1099" s="18">
+        <f>IF(J1099=0,"",L1099/J1099)</f>
+        <v/>
+      </c>
+      <c r="O1099" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1100">
+      <c r="A1100" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:16:41</t>
+        </is>
+      </c>
+      <c r="B1100" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1100" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1100" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E1100" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1100" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G1100" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H1100" s="16" t="n">
+        <v>1.0486</v>
+      </c>
+      <c r="I1100" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J1100" s="17" t="n">
+        <v>140951.0901524015</v>
+      </c>
+      <c r="K1100" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,048.3985</t>
+        </is>
+      </c>
+      <c r="L1100" s="17" t="n">
+        <v>120979.4009308447</v>
+      </c>
+      <c r="M1100" s="17">
+        <f>J1100-L1100</f>
+        <v/>
+      </c>
+      <c r="N1100" s="18">
+        <f>IF(J1100=0,"",L1100/J1100)</f>
+        <v/>
+      </c>
+      <c r="O1100" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1101">
+      <c r="A1101" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:16:41</t>
+        </is>
+      </c>
+      <c r="B1101" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1101" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1101" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E1101" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1101" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G1101" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H1101" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I1101" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J1101" s="17" t="n">
+        <v>328747.337246194</v>
+      </c>
+      <c r="K1101" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,401.0536</t>
+        </is>
+      </c>
+      <c r="L1101" s="17" t="n">
+        <v>306527.2242975623</v>
+      </c>
+      <c r="M1101" s="17">
+        <f>J1101-L1101</f>
+        <v/>
+      </c>
+      <c r="N1101" s="18">
+        <f>IF(J1101=0,"",L1101/J1101)</f>
+        <v/>
+      </c>
+      <c r="O1101" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1102">
+      <c r="A1102" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:16:41</t>
+        </is>
+      </c>
+      <c r="B1102" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1102" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1102" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E1102" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1102" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G1102" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H1102" s="16" t="n">
+        <v>1.0372</v>
+      </c>
+      <c r="I1102" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J1102" s="17" t="n">
+        <v>386112.6697928178</v>
+      </c>
+      <c r="K1102" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,631.2289</t>
+        </is>
+      </c>
+      <c r="L1102" s="17" t="n">
+        <v>349775.2010203177</v>
+      </c>
+      <c r="M1102" s="17">
+        <f>J1102-L1102</f>
+        <v/>
+      </c>
+      <c r="N1102" s="18">
+        <f>IF(J1102=0,"",L1102/J1102)</f>
+        <v/>
+      </c>
+      <c r="O1102" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1103">
+      <c r="A1103" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:16:41</t>
+        </is>
+      </c>
+      <c r="B1103" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1103" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D1103" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E1103" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1103" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G1103" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H1103" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I1103" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7873</t>
+        </is>
+      </c>
+      <c r="J1103" s="17" t="n">
+        <v>77782.71959182875</v>
+      </c>
+      <c r="K1103" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,034.4625; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L1103" s="17" t="n">
+        <v>67995.76048263069</v>
+      </c>
+      <c r="M1103" s="17">
+        <f>J1103-L1103</f>
+        <v/>
+      </c>
+      <c r="N1103" s="18">
+        <f>IF(J1103=0,"",L1103/J1103)</f>
+        <v/>
+      </c>
+      <c r="O1103" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1104">
+      <c r="A1104" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:16:41</t>
+        </is>
+      </c>
+      <c r="B1104" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1104" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1104" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1104" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1104" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1104" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H1104" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I1104" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J1104" s="17" t="n">
+        <v>197045.7956725814</v>
+      </c>
+      <c r="K1104" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,262.3037</t>
+        </is>
+      </c>
+      <c r="L1104" s="17" t="n">
+        <v>150307.3959050264</v>
+      </c>
+      <c r="M1104" s="17">
+        <f>J1104-L1104</f>
+        <v/>
+      </c>
+      <c r="N1104" s="18">
+        <f>IF(J1104=0,"",L1104/J1104)</f>
+        <v/>
+      </c>
+      <c r="O1104" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1105">
+      <c r="A1105" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:16:41</t>
+        </is>
+      </c>
+      <c r="B1105" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1105" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1105" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1105" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1105" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1105" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H1105" s="16" t="n">
+        <v>1.3728</v>
+      </c>
+      <c r="I1105" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J1105" s="17" t="n">
+        <v>186061.0874767996</v>
+      </c>
+      <c r="K1105" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,161.1962</t>
+        </is>
+      </c>
+      <c r="L1105" s="17" t="n">
+        <v>124198.4557182379</v>
+      </c>
+      <c r="M1105" s="17">
+        <f>J1105-L1105</f>
+        <v/>
+      </c>
+      <c r="N1105" s="18">
+        <f>IF(J1105=0,"",L1105/J1105)</f>
+        <v/>
+      </c>
+      <c r="O1105" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1106">
+      <c r="A1106" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:16:41</t>
+        </is>
+      </c>
+      <c r="B1106" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1106" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1106" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1106" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1106" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1106" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H1106" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I1106" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J1106" s="17" t="n">
+        <v>327704.6079050264</v>
+      </c>
+      <c r="K1106" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,363.1264</t>
+        </is>
+      </c>
+      <c r="L1106" s="17" t="n">
+        <v>280226.2337329277</v>
+      </c>
+      <c r="M1106" s="17">
+        <f>J1106-L1106</f>
+        <v/>
+      </c>
+      <c r="N1106" s="18">
+        <f>IF(J1106=0,"",L1106/J1106)</f>
+        <v/>
+      </c>
+      <c r="O1106" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1107">
+      <c r="A1107" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:16:41</t>
+        </is>
+      </c>
+      <c r="B1107" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1107" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1107" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1107" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1107" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1107" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H1107" s="16" t="n">
+        <v>1.9047</v>
+      </c>
+      <c r="I1107" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J1107" s="17" t="n">
+        <v>160068.5465239572</v>
+      </c>
+      <c r="K1107" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,952.6109</t>
+        </is>
+      </c>
+      <c r="L1107" s="17" t="n">
+        <v>70973.90309838159</v>
+      </c>
+      <c r="M1107" s="17">
+        <f>J1107-L1107</f>
+        <v/>
+      </c>
+      <c r="N1107" s="18">
+        <f>IF(J1107=0,"",L1107/J1107)</f>
+        <v/>
+      </c>
+      <c r="O1107" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1108">
+      <c r="A1108" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:16:41</t>
+        </is>
+      </c>
+      <c r="B1108" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1108" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1108" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1108" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1108" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1108" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H1108" s="16" t="n">
+        <v>1.0571</v>
+      </c>
+      <c r="I1108" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J1108" s="17" t="n">
+        <v>160187.6987682178</v>
+      </c>
+      <c r="K1108" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,532.9072</t>
+        </is>
+      </c>
+      <c r="L1108" s="17" t="n">
+        <v>138532.9071543306</v>
+      </c>
+      <c r="M1108" s="17">
+        <f>J1108-L1108</f>
+        <v/>
+      </c>
+      <c r="N1108" s="18">
+        <f>IF(J1108=0,"",L1108/J1108)</f>
+        <v/>
+      </c>
+      <c r="O1108" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1109">
+      <c r="A1109" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:16:41</t>
+        </is>
+      </c>
+      <c r="B1109" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1109" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1109" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E1109" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1109" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G1109" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1109" s="16" t="inlineStr"/>
+      <c r="I1109" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J1109" s="17" t="n">
+        <v>95912.43979709387</v>
+      </c>
+      <c r="K1109" s="15" t="inlineStr"/>
+      <c r="L1109" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1109" s="17">
+        <f>J1109-L1109</f>
+        <v/>
+      </c>
+      <c r="N1109" s="18">
+        <f>IF(J1109=0,"",L1109/J1109)</f>
+        <v/>
+      </c>
+      <c r="O1109" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:16:41</t>
+        </is>
+      </c>
+      <c r="B1110" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1110" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1110" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E1110" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1110" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G1110" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1110" s="16" t="inlineStr"/>
+      <c r="I1110" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J1110" s="17" t="n">
+        <v>34357.28598254643</v>
+      </c>
+      <c r="K1110" s="15" t="inlineStr"/>
+      <c r="L1110" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1110" s="17">
+        <f>J1110-L1110</f>
+        <v/>
+      </c>
+      <c r="N1110" s="18">
+        <f>IF(J1110=0,"",L1110/J1110)</f>
+        <v/>
+      </c>
+      <c r="O1110" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:16:41</t>
+        </is>
+      </c>
+      <c r="B1111" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1111" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D1111" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E1111" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1111" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G1111" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H1111" s="16" t="n">
+        <v>1.0435</v>
+      </c>
+      <c r="I1111" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J1111" s="17" t="n">
+        <v>270082.1998776371</v>
+      </c>
+      <c r="K1111" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,071.2752</t>
+        </is>
+      </c>
+      <c r="L1111" s="17" t="n">
+        <v>232938.4246151121</v>
+      </c>
+      <c r="M1111" s="17">
+        <f>J1111-L1111</f>
+        <v/>
+      </c>
+      <c r="N1111" s="18">
+        <f>IF(J1111=0,"",L1111/J1111)</f>
+        <v/>
+      </c>
+      <c r="O1111" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:16:41</t>
+        </is>
+      </c>
+      <c r="B1112" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1112" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D1112" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E1112" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1112" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G1112" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1112" s="16" t="inlineStr"/>
+      <c r="I1112" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,520.4205</t>
+        </is>
+      </c>
+      <c r="J1112" s="17" t="n">
+        <v>15511.57383836818</v>
+      </c>
+      <c r="K1112" s="15" t="inlineStr"/>
+      <c r="L1112" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1112" s="17">
+        <f>J1112-L1112</f>
+        <v/>
+      </c>
+      <c r="N1112" s="18">
+        <f>IF(J1112=0,"",L1112/J1112)</f>
+        <v/>
+      </c>
+      <c r="O1112" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1113">
+      <c r="A1113" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:16:41</t>
+        </is>
+      </c>
+      <c r="B1113" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1113" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D1113" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E1113" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1113" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G1113" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H1113" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I1113" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J1113" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K1113" s="15" t="inlineStr">
+        <is>
+          <t>USDC 252,020.5254</t>
+        </is>
+      </c>
+      <c r="L1113" s="17" t="n">
+        <v>252020.525427</v>
+      </c>
+      <c r="M1113" s="17">
+        <f>J1113-L1113</f>
+        <v/>
+      </c>
+      <c r="N1113" s="18">
+        <f>IF(J1113=0,"",L1113/J1113)</f>
+        <v/>
+      </c>
+      <c r="O1113" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1114">
+      <c r="A1114" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:16:41</t>
+        </is>
+      </c>
+      <c r="B1114" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1114" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D1114" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E1114" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1114" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G1114" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H1114" s="16" t="n">
+        <v>1.219</v>
+      </c>
+      <c r="I1114" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J1114" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K1114" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,736.3177</t>
+        </is>
+      </c>
+      <c r="L1114" s="17" t="n">
+        <v>148736.317674</v>
+      </c>
+      <c r="M1114" s="17">
+        <f>J1114-L1114</f>
+        <v/>
+      </c>
+      <c r="N1114" s="18">
+        <f>IF(J1114=0,"",L1114/J1114)</f>
+        <v/>
+      </c>
+      <c r="O1114" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -74590,7 +75676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I72"/>
+  <dimension ref="A1:I73"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -77126,6 +78212,41 @@
         <v>1.0372</v>
       </c>
       <c r="I72" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:16:41</t>
+        </is>
+      </c>
+      <c r="B73" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C73" s="17" t="n">
+        <v>655426.6833913673</v>
+      </c>
+      <c r="D73" s="17" t="n">
+        <v>652839.0183016201</v>
+      </c>
+      <c r="E73" s="17" t="n">
+        <v>2933788.772330184</v>
+      </c>
+      <c r="F73" s="17" t="n">
+        <v>2280949.754028563</v>
+      </c>
+      <c r="G73" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H73" s="16" t="n">
+        <v>1.0372</v>
+      </c>
+      <c r="I73" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-30 12:46 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O1114"/>
+  <dimension ref="A1:O1130"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -75646,6 +75646,1092 @@
         <v/>
       </c>
       <c r="O1114" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:46:51</t>
+        </is>
+      </c>
+      <c r="B1115" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1115" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1115" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E1115" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1115" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G1115" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H1115" s="16" t="n">
+        <v>1.0503</v>
+      </c>
+      <c r="I1115" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,809.3004</t>
+        </is>
+      </c>
+      <c r="J1115" s="17" t="n">
+        <v>50787.9605088257</v>
+      </c>
+      <c r="K1115" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,726.6826</t>
+        </is>
+      </c>
+      <c r="L1115" s="17" t="n">
+        <v>37738.00397219165</v>
+      </c>
+      <c r="M1115" s="17">
+        <f>J1115-L1115</f>
+        <v/>
+      </c>
+      <c r="N1115" s="18">
+        <f>IF(J1115=0,"",L1115/J1115)</f>
+        <v/>
+      </c>
+      <c r="O1115" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:46:51</t>
+        </is>
+      </c>
+      <c r="B1116" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1116" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1116" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E1116" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1116" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G1116" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H1116" s="16" t="n">
+        <v>1.0484</v>
+      </c>
+      <c r="I1116" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J1116" s="17" t="n">
+        <v>140950.64217838</v>
+      </c>
+      <c r="K1116" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,048.3985</t>
+        </is>
+      </c>
+      <c r="L1116" s="17" t="n">
+        <v>120997.5581906224</v>
+      </c>
+      <c r="M1116" s="17">
+        <f>J1116-L1116</f>
+        <v/>
+      </c>
+      <c r="N1116" s="18">
+        <f>IF(J1116=0,"",L1116/J1116)</f>
+        <v/>
+      </c>
+      <c r="O1116" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:46:51</t>
+        </is>
+      </c>
+      <c r="B1117" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1117" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1117" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E1117" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1117" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G1117" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H1117" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I1117" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J1117" s="17" t="n">
+        <v>328748.7634581449</v>
+      </c>
+      <c r="K1117" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,401.0536</t>
+        </is>
+      </c>
+      <c r="L1117" s="17" t="n">
+        <v>306526.5279824583</v>
+      </c>
+      <c r="M1117" s="17">
+        <f>J1117-L1117</f>
+        <v/>
+      </c>
+      <c r="N1117" s="18">
+        <f>IF(J1117=0,"",L1117/J1117)</f>
+        <v/>
+      </c>
+      <c r="O1117" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:46:51</t>
+        </is>
+      </c>
+      <c r="B1118" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1118" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1118" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E1118" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1118" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G1118" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H1118" s="16" t="n">
+        <v>1.0372</v>
+      </c>
+      <c r="I1118" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J1118" s="17" t="n">
+        <v>386075.1945546285</v>
+      </c>
+      <c r="K1118" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,631.2289</t>
+        </is>
+      </c>
+      <c r="L1118" s="17" t="n">
+        <v>349774.4064620006</v>
+      </c>
+      <c r="M1118" s="17">
+        <f>J1118-L1118</f>
+        <v/>
+      </c>
+      <c r="N1118" s="18">
+        <f>IF(J1118=0,"",L1118/J1118)</f>
+        <v/>
+      </c>
+      <c r="O1118" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:46:51</t>
+        </is>
+      </c>
+      <c r="B1119" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1119" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D1119" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E1119" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1119" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G1119" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H1119" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I1119" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7873</t>
+        </is>
+      </c>
+      <c r="J1119" s="17" t="n">
+        <v>77783.50633364536</v>
+      </c>
+      <c r="K1119" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,034.4625; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L1119" s="17" t="n">
+        <v>68005.96565201125</v>
+      </c>
+      <c r="M1119" s="17">
+        <f>J1119-L1119</f>
+        <v/>
+      </c>
+      <c r="N1119" s="18">
+        <f>IF(J1119=0,"",L1119/J1119)</f>
+        <v/>
+      </c>
+      <c r="O1119" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:46:51</t>
+        </is>
+      </c>
+      <c r="B1120" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1120" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1120" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1120" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1120" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1120" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H1120" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I1120" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J1120" s="17" t="n">
+        <v>197042.3111391109</v>
+      </c>
+      <c r="K1120" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,262.3037</t>
+        </is>
+      </c>
+      <c r="L1120" s="17" t="n">
+        <v>150307.3959050264</v>
+      </c>
+      <c r="M1120" s="17">
+        <f>J1120-L1120</f>
+        <v/>
+      </c>
+      <c r="N1120" s="18">
+        <f>IF(J1120=0,"",L1120/J1120)</f>
+        <v/>
+      </c>
+      <c r="O1120" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1121">
+      <c r="A1121" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:46:51</t>
+        </is>
+      </c>
+      <c r="B1121" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1121" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1121" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1121" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1121" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1121" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H1121" s="16" t="n">
+        <v>1.3728</v>
+      </c>
+      <c r="I1121" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J1121" s="17" t="n">
+        <v>186061.733174991</v>
+      </c>
+      <c r="K1121" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,161.1962</t>
+        </is>
+      </c>
+      <c r="L1121" s="17" t="n">
+        <v>124198.4557182379</v>
+      </c>
+      <c r="M1121" s="17">
+        <f>J1121-L1121</f>
+        <v/>
+      </c>
+      <c r="N1121" s="18">
+        <f>IF(J1121=0,"",L1121/J1121)</f>
+        <v/>
+      </c>
+      <c r="O1121" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:46:51</t>
+        </is>
+      </c>
+      <c r="B1122" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1122" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1122" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1122" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1122" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1122" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H1122" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I1122" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J1122" s="17" t="n">
+        <v>327706.7536027628</v>
+      </c>
+      <c r="K1122" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,363.1264</t>
+        </is>
+      </c>
+      <c r="L1122" s="17" t="n">
+        <v>280229.335747242</v>
+      </c>
+      <c r="M1122" s="17">
+        <f>J1122-L1122</f>
+        <v/>
+      </c>
+      <c r="N1122" s="18">
+        <f>IF(J1122=0,"",L1122/J1122)</f>
+        <v/>
+      </c>
+      <c r="O1122" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:46:51</t>
+        </is>
+      </c>
+      <c r="B1123" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1123" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1123" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1123" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1123" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1123" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H1123" s="16" t="n">
+        <v>1.9047</v>
+      </c>
+      <c r="I1123" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J1123" s="17" t="n">
+        <v>160068.5465239572</v>
+      </c>
+      <c r="K1123" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,952.6109</t>
+        </is>
+      </c>
+      <c r="L1123" s="17" t="n">
+        <v>70973.90309838159</v>
+      </c>
+      <c r="M1123" s="17">
+        <f>J1123-L1123</f>
+        <v/>
+      </c>
+      <c r="N1123" s="18">
+        <f>IF(J1123=0,"",L1123/J1123)</f>
+        <v/>
+      </c>
+      <c r="O1123" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:46:51</t>
+        </is>
+      </c>
+      <c r="B1124" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1124" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1124" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1124" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1124" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1124" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H1124" s="16" t="n">
+        <v>1.0571</v>
+      </c>
+      <c r="I1124" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J1124" s="17" t="n">
+        <v>160172.1513059459</v>
+      </c>
+      <c r="K1124" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,532.9072</t>
+        </is>
+      </c>
+      <c r="L1124" s="17" t="n">
+        <v>138519.0538636152</v>
+      </c>
+      <c r="M1124" s="17">
+        <f>J1124-L1124</f>
+        <v/>
+      </c>
+      <c r="N1124" s="18">
+        <f>IF(J1124=0,"",L1124/J1124)</f>
+        <v/>
+      </c>
+      <c r="O1124" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:46:51</t>
+        </is>
+      </c>
+      <c r="B1125" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1125" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1125" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E1125" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1125" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G1125" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1125" s="16" t="inlineStr"/>
+      <c r="I1125" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J1125" s="17" t="n">
+        <v>95911.3510959932</v>
+      </c>
+      <c r="K1125" s="15" t="inlineStr"/>
+      <c r="L1125" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1125" s="17">
+        <f>J1125-L1125</f>
+        <v/>
+      </c>
+      <c r="N1125" s="18">
+        <f>IF(J1125=0,"",L1125/J1125)</f>
+        <v/>
+      </c>
+      <c r="O1125" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:46:51</t>
+        </is>
+      </c>
+      <c r="B1126" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1126" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1126" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E1126" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1126" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G1126" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1126" s="16" t="inlineStr"/>
+      <c r="I1126" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J1126" s="17" t="n">
+        <v>34357.49133654373</v>
+      </c>
+      <c r="K1126" s="15" t="inlineStr"/>
+      <c r="L1126" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1126" s="17">
+        <f>J1126-L1126</f>
+        <v/>
+      </c>
+      <c r="N1126" s="18">
+        <f>IF(J1126=0,"",L1126/J1126)</f>
+        <v/>
+      </c>
+      <c r="O1126" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:46:51</t>
+        </is>
+      </c>
+      <c r="B1127" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1127" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D1127" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E1127" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1127" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G1127" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H1127" s="16" t="n">
+        <v>1.0434</v>
+      </c>
+      <c r="I1127" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J1127" s="17" t="n">
+        <v>270082.1998776371</v>
+      </c>
+      <c r="K1127" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,071.2752</t>
+        </is>
+      </c>
+      <c r="L1127" s="17" t="n">
+        <v>232973.3853063984</v>
+      </c>
+      <c r="M1127" s="17">
+        <f>J1127-L1127</f>
+        <v/>
+      </c>
+      <c r="N1127" s="18">
+        <f>IF(J1127=0,"",L1127/J1127)</f>
+        <v/>
+      </c>
+      <c r="O1127" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:46:51</t>
+        </is>
+      </c>
+      <c r="B1128" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1128" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D1128" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E1128" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1128" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G1128" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1128" s="16" t="inlineStr"/>
+      <c r="I1128" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,520.5111</t>
+        </is>
+      </c>
+      <c r="J1128" s="17" t="n">
+        <v>15513.99249034685</v>
+      </c>
+      <c r="K1128" s="15" t="inlineStr"/>
+      <c r="L1128" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1128" s="17">
+        <f>J1128-L1128</f>
+        <v/>
+      </c>
+      <c r="N1128" s="18">
+        <f>IF(J1128=0,"",L1128/J1128)</f>
+        <v/>
+      </c>
+      <c r="O1128" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:46:51</t>
+        </is>
+      </c>
+      <c r="B1129" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1129" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D1129" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E1129" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1129" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G1129" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H1129" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I1129" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J1129" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K1129" s="15" t="inlineStr">
+        <is>
+          <t>USDC 252,020.5254</t>
+        </is>
+      </c>
+      <c r="L1129" s="17" t="n">
+        <v>252020.525427</v>
+      </c>
+      <c r="M1129" s="17">
+        <f>J1129-L1129</f>
+        <v/>
+      </c>
+      <c r="N1129" s="18">
+        <f>IF(J1129=0,"",L1129/J1129)</f>
+        <v/>
+      </c>
+      <c r="O1129" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:46:51</t>
+        </is>
+      </c>
+      <c r="B1130" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1130" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D1130" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E1130" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1130" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G1130" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H1130" s="16" t="n">
+        <v>1.219</v>
+      </c>
+      <c r="I1130" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J1130" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K1130" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,736.3177</t>
+        </is>
+      </c>
+      <c r="L1130" s="17" t="n">
+        <v>148736.317674</v>
+      </c>
+      <c r="M1130" s="17">
+        <f>J1130-L1130</f>
+        <v/>
+      </c>
+      <c r="N1130" s="18">
+        <f>IF(J1130=0,"",L1130/J1130)</f>
+        <v/>
+      </c>
+      <c r="O1130" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -75676,7 +76762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I73"/>
+  <dimension ref="A1:I74"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -78247,6 +79333,41 @@
         <v>1.0372</v>
       </c>
       <c r="I73" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 12:46:51</t>
+        </is>
+      </c>
+      <c r="B74" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C74" s="17" t="n">
+        <v>655332.6231038466</v>
+      </c>
+      <c r="D74" s="17" t="n">
+        <v>652745.1431726771</v>
+      </c>
+      <c r="E74" s="17" t="n">
+        <v>2933745.978171863</v>
+      </c>
+      <c r="F74" s="17" t="n">
+        <v>2281000.834999186</v>
+      </c>
+      <c r="G74" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H74" s="16" t="n">
+        <v>1.0372</v>
+      </c>
+      <c r="I74" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-30 13:17 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O1130"/>
+  <dimension ref="A1:O1146"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -76732,6 +76732,1092 @@
         <v/>
       </c>
       <c r="O1130" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:17:02</t>
+        </is>
+      </c>
+      <c r="B1131" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1131" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1131" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E1131" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1131" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G1131" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H1131" s="16" t="n">
+        <v>1.0503</v>
+      </c>
+      <c r="I1131" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,809.3004</t>
+        </is>
+      </c>
+      <c r="J1131" s="17" t="n">
+        <v>50787.45241582154</v>
+      </c>
+      <c r="K1131" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,726.6826</t>
+        </is>
+      </c>
+      <c r="L1131" s="17" t="n">
+        <v>37741.77928271308</v>
+      </c>
+      <c r="M1131" s="17">
+        <f>J1131-L1131</f>
+        <v/>
+      </c>
+      <c r="N1131" s="18">
+        <f>IF(J1131=0,"",L1131/J1131)</f>
+        <v/>
+      </c>
+      <c r="O1131" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:17:02</t>
+        </is>
+      </c>
+      <c r="B1132" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1132" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1132" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E1132" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1132" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G1132" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H1132" s="16" t="n">
+        <v>1.0484</v>
+      </c>
+      <c r="I1132" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J1132" s="17" t="n">
+        <v>140951.9720973682</v>
+      </c>
+      <c r="K1132" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,048.3985</t>
+        </is>
+      </c>
+      <c r="L1132" s="17" t="n">
+        <v>120996.3477066373</v>
+      </c>
+      <c r="M1132" s="17">
+        <f>J1132-L1132</f>
+        <v/>
+      </c>
+      <c r="N1132" s="18">
+        <f>IF(J1132=0,"",L1132/J1132)</f>
+        <v/>
+      </c>
+      <c r="O1132" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:17:02</t>
+        </is>
+      </c>
+      <c r="B1133" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1133" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1133" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E1133" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1133" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G1133" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H1133" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I1133" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J1133" s="17" t="n">
+        <v>328748.7634581449</v>
+      </c>
+      <c r="K1133" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,401.0536</t>
+        </is>
+      </c>
+      <c r="L1133" s="17" t="n">
+        <v>306526.524225875</v>
+      </c>
+      <c r="M1133" s="17">
+        <f>J1133-L1133</f>
+        <v/>
+      </c>
+      <c r="N1133" s="18">
+        <f>IF(J1133=0,"",L1133/J1133)</f>
+        <v/>
+      </c>
+      <c r="O1133" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1134">
+      <c r="A1134" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:17:02</t>
+        </is>
+      </c>
+      <c r="B1134" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1134" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1134" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E1134" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1134" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G1134" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H1134" s="16" t="n">
+        <v>1.0372</v>
+      </c>
+      <c r="I1134" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J1134" s="17" t="n">
+        <v>386076.3537832667</v>
+      </c>
+      <c r="K1134" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,631.2289</t>
+        </is>
+      </c>
+      <c r="L1134" s="17" t="n">
+        <v>349774.4021754003</v>
+      </c>
+      <c r="M1134" s="17">
+        <f>J1134-L1134</f>
+        <v/>
+      </c>
+      <c r="N1134" s="18">
+        <f>IF(J1134=0,"",L1134/J1134)</f>
+        <v/>
+      </c>
+      <c r="O1134" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1135">
+      <c r="A1135" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:17:02</t>
+        </is>
+      </c>
+      <c r="B1135" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1135" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D1135" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E1135" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1135" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G1135" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H1135" s="16" t="n">
+        <v>1.0542</v>
+      </c>
+      <c r="I1135" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7873</t>
+        </is>
+      </c>
+      <c r="J1135" s="17" t="n">
+        <v>77776.50767592579</v>
+      </c>
+      <c r="K1135" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,034.4625; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L1135" s="17" t="n">
+        <v>68005.28531514791</v>
+      </c>
+      <c r="M1135" s="17">
+        <f>J1135-L1135</f>
+        <v/>
+      </c>
+      <c r="N1135" s="18">
+        <f>IF(J1135=0,"",L1135/J1135)</f>
+        <v/>
+      </c>
+      <c r="O1135" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1136">
+      <c r="A1136" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:17:02</t>
+        </is>
+      </c>
+      <c r="B1136" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1136" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1136" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1136" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1136" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1136" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H1136" s="16" t="n">
+        <v>1.1287</v>
+      </c>
+      <c r="I1136" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J1136" s="17" t="n">
+        <v>197053.8511726968</v>
+      </c>
+      <c r="K1136" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,262.3037</t>
+        </is>
+      </c>
+      <c r="L1136" s="17" t="n">
+        <v>150322.4326593186</v>
+      </c>
+      <c r="M1136" s="17">
+        <f>J1136-L1136</f>
+        <v/>
+      </c>
+      <c r="N1136" s="18">
+        <f>IF(J1136=0,"",L1136/J1136)</f>
+        <v/>
+      </c>
+      <c r="O1136" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1137">
+      <c r="A1137" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:17:02</t>
+        </is>
+      </c>
+      <c r="B1137" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1137" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1137" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1137" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1137" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1137" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H1137" s="16" t="n">
+        <v>1.3728</v>
+      </c>
+      <c r="I1137" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J1137" s="17" t="n">
+        <v>186046.6747463087</v>
+      </c>
+      <c r="K1137" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,161.1962</t>
+        </is>
+      </c>
+      <c r="L1137" s="17" t="n">
+        <v>124210.8805337359</v>
+      </c>
+      <c r="M1137" s="17">
+        <f>J1137-L1137</f>
+        <v/>
+      </c>
+      <c r="N1137" s="18">
+        <f>IF(J1137=0,"",L1137/J1137)</f>
+        <v/>
+      </c>
+      <c r="O1137" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:17:02</t>
+        </is>
+      </c>
+      <c r="B1138" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1138" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1138" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1138" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1138" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1138" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H1138" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I1138" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J1138" s="17" t="n">
+        <v>327708.6856841102</v>
+      </c>
+      <c r="K1138" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,363.1264</t>
+        </is>
+      </c>
+      <c r="L1138" s="17" t="n">
+        <v>280229.3237674735</v>
+      </c>
+      <c r="M1138" s="17">
+        <f>J1138-L1138</f>
+        <v/>
+      </c>
+      <c r="N1138" s="18">
+        <f>IF(J1138=0,"",L1138/J1138)</f>
+        <v/>
+      </c>
+      <c r="O1138" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:17:02</t>
+        </is>
+      </c>
+      <c r="B1139" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1139" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1139" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1139" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1139" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1139" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H1139" s="16" t="n">
+        <v>1.9047</v>
+      </c>
+      <c r="I1139" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J1139" s="17" t="n">
+        <v>160068.5465239572</v>
+      </c>
+      <c r="K1139" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,952.6109</t>
+        </is>
+      </c>
+      <c r="L1139" s="17" t="n">
+        <v>70981.0033287836</v>
+      </c>
+      <c r="M1139" s="17">
+        <f>J1139-L1139</f>
+        <v/>
+      </c>
+      <c r="N1139" s="18">
+        <f>IF(J1139=0,"",L1139/J1139)</f>
+        <v/>
+      </c>
+      <c r="O1139" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:17:02</t>
+        </is>
+      </c>
+      <c r="B1140" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1140" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1140" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1140" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1140" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1140" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H1140" s="16" t="n">
+        <v>1.0571</v>
+      </c>
+      <c r="I1140" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J1140" s="17" t="n">
+        <v>160172.63223854</v>
+      </c>
+      <c r="K1140" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,532.9072</t>
+        </is>
+      </c>
+      <c r="L1140" s="17" t="n">
+        <v>138519.0538636152</v>
+      </c>
+      <c r="M1140" s="17">
+        <f>J1140-L1140</f>
+        <v/>
+      </c>
+      <c r="N1140" s="18">
+        <f>IF(J1140=0,"",L1140/J1140)</f>
+        <v/>
+      </c>
+      <c r="O1140" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1141">
+      <c r="A1141" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:17:02</t>
+        </is>
+      </c>
+      <c r="B1141" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1141" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1141" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E1141" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1141" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G1141" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1141" s="16" t="inlineStr"/>
+      <c r="I1141" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J1141" s="17" t="n">
+        <v>95798.56325168614</v>
+      </c>
+      <c r="K1141" s="15" t="inlineStr"/>
+      <c r="L1141" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1141" s="17">
+        <f>J1141-L1141</f>
+        <v/>
+      </c>
+      <c r="N1141" s="18">
+        <f>IF(J1141=0,"",L1141/J1141)</f>
+        <v/>
+      </c>
+      <c r="O1141" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:17:02</t>
+        </is>
+      </c>
+      <c r="B1142" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1142" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1142" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E1142" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1142" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G1142" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1142" s="16" t="inlineStr"/>
+      <c r="I1142" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J1142" s="17" t="n">
+        <v>34357.79203568285</v>
+      </c>
+      <c r="K1142" s="15" t="inlineStr"/>
+      <c r="L1142" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1142" s="17">
+        <f>J1142-L1142</f>
+        <v/>
+      </c>
+      <c r="N1142" s="18">
+        <f>IF(J1142=0,"",L1142/J1142)</f>
+        <v/>
+      </c>
+      <c r="O1142" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1143">
+      <c r="A1143" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:17:02</t>
+        </is>
+      </c>
+      <c r="B1143" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1143" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D1143" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E1143" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1143" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G1143" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H1143" s="16" t="n">
+        <v>1.0434</v>
+      </c>
+      <c r="I1143" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J1143" s="17" t="n">
+        <v>270082.1998776371</v>
+      </c>
+      <c r="K1143" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,071.2752</t>
+        </is>
+      </c>
+      <c r="L1143" s="17" t="n">
+        <v>232971.0545936459</v>
+      </c>
+      <c r="M1143" s="17">
+        <f>J1143-L1143</f>
+        <v/>
+      </c>
+      <c r="N1143" s="18">
+        <f>IF(J1143=0,"",L1143/J1143)</f>
+        <v/>
+      </c>
+      <c r="O1143" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:17:02</t>
+        </is>
+      </c>
+      <c r="B1144" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1144" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D1144" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E1144" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1144" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G1144" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1144" s="16" t="inlineStr"/>
+      <c r="I1144" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,520.7161</t>
+        </is>
+      </c>
+      <c r="J1144" s="17" t="n">
+        <v>15514.04214658107</v>
+      </c>
+      <c r="K1144" s="15" t="inlineStr"/>
+      <c r="L1144" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1144" s="17">
+        <f>J1144-L1144</f>
+        <v/>
+      </c>
+      <c r="N1144" s="18">
+        <f>IF(J1144=0,"",L1144/J1144)</f>
+        <v/>
+      </c>
+      <c r="O1144" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:17:02</t>
+        </is>
+      </c>
+      <c r="B1145" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1145" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D1145" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E1145" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1145" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G1145" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H1145" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I1145" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J1145" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K1145" s="15" t="inlineStr">
+        <is>
+          <t>USDC 252,020.5254</t>
+        </is>
+      </c>
+      <c r="L1145" s="17" t="n">
+        <v>252020.525427</v>
+      </c>
+      <c r="M1145" s="17">
+        <f>J1145-L1145</f>
+        <v/>
+      </c>
+      <c r="N1145" s="18">
+        <f>IF(J1145=0,"",L1145/J1145)</f>
+        <v/>
+      </c>
+      <c r="O1145" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:17:02</t>
+        </is>
+      </c>
+      <c r="B1146" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1146" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D1146" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E1146" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1146" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G1146" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H1146" s="16" t="n">
+        <v>1.219</v>
+      </c>
+      <c r="I1146" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J1146" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K1146" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,736.3177</t>
+        </is>
+      </c>
+      <c r="L1146" s="17" t="n">
+        <v>148736.317674</v>
+      </c>
+      <c r="M1146" s="17">
+        <f>J1146-L1146</f>
+        <v/>
+      </c>
+      <c r="N1146" s="18">
+        <f>IF(J1146=0,"",L1146/J1146)</f>
+        <v/>
+      </c>
+      <c r="O1146" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -76762,7 +77848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I74"/>
+  <dimension ref="A1:I75"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -79368,6 +80454,41 @@
         <v>1.0372</v>
       </c>
       <c r="I74" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:17:02</t>
+        </is>
+      </c>
+      <c r="B75" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C75" s="17" t="n">
+        <v>655179.8258730855</v>
+      </c>
+      <c r="D75" s="17" t="n">
+        <v>652592.4871453308</v>
+      </c>
+      <c r="E75" s="17" t="n">
+        <v>2933627.417698677</v>
+      </c>
+      <c r="F75" s="17" t="n">
+        <v>2281034.930553346</v>
+      </c>
+      <c r="G75" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H75" s="16" t="n">
+        <v>1.0372</v>
+      </c>
+      <c r="I75" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-30 13:47 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O1146"/>
+  <dimension ref="A1:O1162"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -77818,6 +77818,1092 @@
         <v/>
       </c>
       <c r="O1146" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:47:15</t>
+        </is>
+      </c>
+      <c r="B1147" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1147" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1147" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E1147" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1147" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G1147" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H1147" s="16" t="n">
+        <v>1.0503</v>
+      </c>
+      <c r="I1147" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,811.4611</t>
+        </is>
+      </c>
+      <c r="J1147" s="17" t="n">
+        <v>50791.1364835728</v>
+      </c>
+      <c r="K1147" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,728.2168</t>
+        </is>
+      </c>
+      <c r="L1147" s="17" t="n">
+        <v>37735.76395779155</v>
+      </c>
+      <c r="M1147" s="17">
+        <f>J1147-L1147</f>
+        <v/>
+      </c>
+      <c r="N1147" s="18">
+        <f>IF(J1147=0,"",L1147/J1147)</f>
+        <v/>
+      </c>
+      <c r="O1147" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:47:15</t>
+        </is>
+      </c>
+      <c r="B1148" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1148" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1148" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E1148" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1148" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G1148" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H1148" s="16" t="n">
+        <v>1.0484</v>
+      </c>
+      <c r="I1148" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J1148" s="17" t="n">
+        <v>140952.1131709849</v>
+      </c>
+      <c r="K1148" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,053.5935</t>
+        </is>
+      </c>
+      <c r="L1148" s="17" t="n">
+        <v>121005.172027614</v>
+      </c>
+      <c r="M1148" s="17">
+        <f>J1148-L1148</f>
+        <v/>
+      </c>
+      <c r="N1148" s="18">
+        <f>IF(J1148=0,"",L1148/J1148)</f>
+        <v/>
+      </c>
+      <c r="O1148" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:47:15</t>
+        </is>
+      </c>
+      <c r="B1149" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1149" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1149" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E1149" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1149" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G1149" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H1149" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I1149" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J1149" s="17" t="n">
+        <v>328749.1559068142</v>
+      </c>
+      <c r="K1149" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,406.8836</t>
+        </is>
+      </c>
+      <c r="L1149" s="17" t="n">
+        <v>306501.701605388</v>
+      </c>
+      <c r="M1149" s="17">
+        <f>J1149-L1149</f>
+        <v/>
+      </c>
+      <c r="N1149" s="18">
+        <f>IF(J1149=0,"",L1149/J1149)</f>
+        <v/>
+      </c>
+      <c r="O1149" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:47:15</t>
+        </is>
+      </c>
+      <c r="B1150" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1150" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1150" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E1150" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1150" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G1150" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H1150" s="16" t="n">
+        <v>1.0374</v>
+      </c>
+      <c r="I1150" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J1150" s="17" t="n">
+        <v>386077.5440111107</v>
+      </c>
+      <c r="K1150" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,640.1739</t>
+        </is>
+      </c>
+      <c r="L1150" s="17" t="n">
+        <v>349748.3705254277</v>
+      </c>
+      <c r="M1150" s="17">
+        <f>J1150-L1150</f>
+        <v/>
+      </c>
+      <c r="N1150" s="18">
+        <f>IF(J1150=0,"",L1150/J1150)</f>
+        <v/>
+      </c>
+      <c r="O1150" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:47:15</t>
+        </is>
+      </c>
+      <c r="B1151" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1151" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D1151" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E1151" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1151" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G1151" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H1151" s="16" t="n">
+        <v>1.0541</v>
+      </c>
+      <c r="I1151" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7883</t>
+        </is>
+      </c>
+      <c r="J1151" s="17" t="n">
+        <v>77785.83279906516</v>
+      </c>
+      <c r="K1151" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,036.7818; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L1151" s="17" t="n">
+        <v>68009.64463780989</v>
+      </c>
+      <c r="M1151" s="17">
+        <f>J1151-L1151</f>
+        <v/>
+      </c>
+      <c r="N1151" s="18">
+        <f>IF(J1151=0,"",L1151/J1151)</f>
+        <v/>
+      </c>
+      <c r="O1151" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:47:15</t>
+        </is>
+      </c>
+      <c r="B1152" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1152" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1152" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1152" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1152" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1152" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H1152" s="16" t="n">
+        <v>1.1283</v>
+      </c>
+      <c r="I1152" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J1152" s="17" t="n">
+        <v>197055.639097575</v>
+      </c>
+      <c r="K1152" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,269.6194</t>
+        </is>
+      </c>
+      <c r="L1152" s="17" t="n">
+        <v>150299.6793251109</v>
+      </c>
+      <c r="M1152" s="17">
+        <f>J1152-L1152</f>
+        <v/>
+      </c>
+      <c r="N1152" s="18">
+        <f>IF(J1152=0,"",L1152/J1152)</f>
+        <v/>
+      </c>
+      <c r="O1152" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:47:15</t>
+        </is>
+      </c>
+      <c r="B1153" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1153" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1153" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1153" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1153" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1153" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H1153" s="16" t="n">
+        <v>1.3723</v>
+      </c>
+      <c r="I1153" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J1153" s="17" t="n">
+        <v>186155.0454654656</v>
+      </c>
+      <c r="K1153" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,167.8308</t>
+        </is>
+      </c>
+      <c r="L1153" s="17" t="n">
+        <v>124192.6693649062</v>
+      </c>
+      <c r="M1153" s="17">
+        <f>J1153-L1153</f>
+        <v/>
+      </c>
+      <c r="N1153" s="18">
+        <f>IF(J1153=0,"",L1153/J1153)</f>
+        <v/>
+      </c>
+      <c r="O1153" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:47:15</t>
+        </is>
+      </c>
+      <c r="B1154" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1154" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1154" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1154" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1154" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1154" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H1154" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I1154" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J1154" s="17" t="n">
+        <v>327712.2986843787</v>
+      </c>
+      <c r="K1154" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,371.4621</t>
+        </is>
+      </c>
+      <c r="L1154" s="17" t="n">
+        <v>280231.440440412</v>
+      </c>
+      <c r="M1154" s="17">
+        <f>J1154-L1154</f>
+        <v/>
+      </c>
+      <c r="N1154" s="18">
+        <f>IF(J1154=0,"",L1154/J1154)</f>
+        <v/>
+      </c>
+      <c r="O1154" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:47:15</t>
+        </is>
+      </c>
+      <c r="B1155" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1155" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1155" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1155" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1155" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1155" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H1155" s="16" t="n">
+        <v>1.9046</v>
+      </c>
+      <c r="I1155" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J1155" s="17" t="n">
+        <v>160084.5597839135</v>
+      </c>
+      <c r="K1155" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,956.9330</t>
+        </is>
+      </c>
+      <c r="L1155" s="17" t="n">
+        <v>70971.12727137699</v>
+      </c>
+      <c r="M1155" s="17">
+        <f>J1155-L1155</f>
+        <v/>
+      </c>
+      <c r="N1155" s="18">
+        <f>IF(J1155=0,"",L1155/J1155)</f>
+        <v/>
+      </c>
+      <c r="O1155" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:47:15</t>
+        </is>
+      </c>
+      <c r="B1156" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1156" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1156" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1156" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1156" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1156" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H1156" s="16" t="n">
+        <v>1.0572</v>
+      </c>
+      <c r="I1156" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J1156" s="17" t="n">
+        <v>160173.1260318657</v>
+      </c>
+      <c r="K1156" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,534.8152</t>
+        </is>
+      </c>
+      <c r="L1156" s="17" t="n">
+        <v>138534.8151931956</v>
+      </c>
+      <c r="M1156" s="17">
+        <f>J1156-L1156</f>
+        <v/>
+      </c>
+      <c r="N1156" s="18">
+        <f>IF(J1156=0,"",L1156/J1156)</f>
+        <v/>
+      </c>
+      <c r="O1156" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1157">
+      <c r="A1157" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:47:15</t>
+        </is>
+      </c>
+      <c r="B1157" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1157" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1157" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E1157" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1157" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G1157" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1157" s="16" t="inlineStr"/>
+      <c r="I1157" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J1157" s="17" t="n">
+        <v>95902.44669925934</v>
+      </c>
+      <c r="K1157" s="15" t="inlineStr"/>
+      <c r="L1157" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1157" s="17">
+        <f>J1157-L1157</f>
+        <v/>
+      </c>
+      <c r="N1157" s="18">
+        <f>IF(J1157=0,"",L1157/J1157)</f>
+        <v/>
+      </c>
+      <c r="O1157" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:47:15</t>
+        </is>
+      </c>
+      <c r="B1158" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1158" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1158" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E1158" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1158" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G1158" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1158" s="16" t="inlineStr"/>
+      <c r="I1158" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J1158" s="17" t="n">
+        <v>34358.08723678791</v>
+      </c>
+      <c r="K1158" s="15" t="inlineStr"/>
+      <c r="L1158" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1158" s="17">
+        <f>J1158-L1158</f>
+        <v/>
+      </c>
+      <c r="N1158" s="18">
+        <f>IF(J1158=0,"",L1158/J1158)</f>
+        <v/>
+      </c>
+      <c r="O1158" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:47:15</t>
+        </is>
+      </c>
+      <c r="B1159" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1159" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D1159" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E1159" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1159" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G1159" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H1159" s="16" t="n">
+        <v>1.0432</v>
+      </c>
+      <c r="I1159" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J1159" s="17" t="n">
+        <v>270055.1862549248</v>
+      </c>
+      <c r="K1159" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,082.9379</t>
+        </is>
+      </c>
+      <c r="L1159" s="17" t="n">
+        <v>232989.704709846</v>
+      </c>
+      <c r="M1159" s="17">
+        <f>J1159-L1159</f>
+        <v/>
+      </c>
+      <c r="N1159" s="18">
+        <f>IF(J1159=0,"",L1159/J1159)</f>
+        <v/>
+      </c>
+      <c r="O1159" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:47:15</t>
+        </is>
+      </c>
+      <c r="B1160" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1160" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D1160" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E1160" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1160" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G1160" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1160" s="16" t="inlineStr"/>
+      <c r="I1160" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,520.9155</t>
+        </is>
+      </c>
+      <c r="J1160" s="17" t="n">
+        <v>15514.70713499697</v>
+      </c>
+      <c r="K1160" s="15" t="inlineStr"/>
+      <c r="L1160" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1160" s="17">
+        <f>J1160-L1160</f>
+        <v/>
+      </c>
+      <c r="N1160" s="18">
+        <f>IF(J1160=0,"",L1160/J1160)</f>
+        <v/>
+      </c>
+      <c r="O1160" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:47:15</t>
+        </is>
+      </c>
+      <c r="B1161" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1161" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D1161" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E1161" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1161" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G1161" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H1161" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I1161" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J1161" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K1161" s="15" t="inlineStr">
+        <is>
+          <t>USDC 252,020.5254</t>
+        </is>
+      </c>
+      <c r="L1161" s="17" t="n">
+        <v>252020.525427</v>
+      </c>
+      <c r="M1161" s="17">
+        <f>J1161-L1161</f>
+        <v/>
+      </c>
+      <c r="N1161" s="18">
+        <f>IF(J1161=0,"",L1161/J1161)</f>
+        <v/>
+      </c>
+      <c r="O1161" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:47:15</t>
+        </is>
+      </c>
+      <c r="B1162" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1162" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D1162" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E1162" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1162" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G1162" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H1162" s="16" t="n">
+        <v>1.219</v>
+      </c>
+      <c r="I1162" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J1162" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K1162" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,736.3177</t>
+        </is>
+      </c>
+      <c r="L1162" s="17" t="n">
+        <v>148736.317674</v>
+      </c>
+      <c r="M1162" s="17">
+        <f>J1162-L1162</f>
+        <v/>
+      </c>
+      <c r="N1162" s="18">
+        <f>IF(J1162=0,"",L1162/J1162)</f>
+        <v/>
+      </c>
+      <c r="O1162" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -77848,7 +78934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I75"/>
+  <dimension ref="A1:I76"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -80489,6 +81575,41 @@
         <v>1.0372</v>
       </c>
       <c r="I75" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 13:47:15</t>
+        </is>
+      </c>
+      <c r="B76" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C76" s="17" t="n">
+        <v>655462.4975224975</v>
+      </c>
+      <c r="D76" s="17" t="n">
+        <v>652873.3271917864</v>
+      </c>
+      <c r="E76" s="17" t="n">
+        <v>2933850.259351665</v>
+      </c>
+      <c r="F76" s="17" t="n">
+        <v>2280976.932159879</v>
+      </c>
+      <c r="G76" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H76" s="16" t="n">
+        <v>1.0374</v>
+      </c>
+      <c r="I76" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
refresh: 2026-04-30 14:17 UTC
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O1162"/>
+  <dimension ref="A1:O1178"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -78904,6 +78904,1092 @@
         <v/>
       </c>
       <c r="O1162" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:17:27</t>
+        </is>
+      </c>
+      <c r="B1163" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1163" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1163" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E1163" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1163" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G1163" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H1163" s="16" t="n">
+        <v>1.0503</v>
+      </c>
+      <c r="I1163" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,811.4611</t>
+        </is>
+      </c>
+      <c r="J1163" s="17" t="n">
+        <v>50783.5147644126</v>
+      </c>
+      <c r="K1163" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,728.2168</t>
+        </is>
+      </c>
+      <c r="L1163" s="17" t="n">
+        <v>37739.53866659998</v>
+      </c>
+      <c r="M1163" s="17">
+        <f>J1163-L1163</f>
+        <v/>
+      </c>
+      <c r="N1163" s="18">
+        <f>IF(J1163=0,"",L1163/J1163)</f>
+        <v/>
+      </c>
+      <c r="O1163" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:17:27</t>
+        </is>
+      </c>
+      <c r="B1164" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1164" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1164" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E1164" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1164" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G1164" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H1164" s="16" t="n">
+        <v>1.0485</v>
+      </c>
+      <c r="I1164" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J1164" s="17" t="n">
+        <v>140952.8186242044</v>
+      </c>
+      <c r="K1164" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,053.5935</t>
+        </is>
+      </c>
+      <c r="L1164" s="17" t="n">
+        <v>120987.0139885942</v>
+      </c>
+      <c r="M1164" s="17">
+        <f>J1164-L1164</f>
+        <v/>
+      </c>
+      <c r="N1164" s="18">
+        <f>IF(J1164=0,"",L1164/J1164)</f>
+        <v/>
+      </c>
+      <c r="O1164" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1165">
+      <c r="A1165" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:17:27</t>
+        </is>
+      </c>
+      <c r="B1165" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1165" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1165" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E1165" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1165" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G1165" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H1165" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I1165" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J1165" s="17" t="n">
+        <v>328749.8355141544</v>
+      </c>
+      <c r="K1165" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,406.8836</t>
+        </is>
+      </c>
+      <c r="L1165" s="17" t="n">
+        <v>306531.709637912</v>
+      </c>
+      <c r="M1165" s="17">
+        <f>J1165-L1165</f>
+        <v/>
+      </c>
+      <c r="N1165" s="18">
+        <f>IF(J1165=0,"",L1165/J1165)</f>
+        <v/>
+      </c>
+      <c r="O1165" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1166">
+      <c r="A1166" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:17:27</t>
+        </is>
+      </c>
+      <c r="B1166" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1166" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1166" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E1166" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1166" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G1166" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H1166" s="16" t="n">
+        <v>1.0374</v>
+      </c>
+      <c r="I1166" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J1166" s="17" t="n">
+        <v>386078.6724737359</v>
+      </c>
+      <c r="K1166" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,640.1739</t>
+        </is>
+      </c>
+      <c r="L1166" s="17" t="n">
+        <v>349782.6126207343</v>
+      </c>
+      <c r="M1166" s="17">
+        <f>J1166-L1166</f>
+        <v/>
+      </c>
+      <c r="N1166" s="18">
+        <f>IF(J1166=0,"",L1166/J1166)</f>
+        <v/>
+      </c>
+      <c r="O1166" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1167">
+      <c r="A1167" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:17:27</t>
+        </is>
+      </c>
+      <c r="B1167" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1167" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D1167" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E1167" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1167" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G1167" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H1167" s="16" t="n">
+        <v>1.0541</v>
+      </c>
+      <c r="I1167" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7883</t>
+        </is>
+      </c>
+      <c r="J1167" s="17" t="n">
+        <v>77786.53259248368</v>
+      </c>
+      <c r="K1167" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,036.7818; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L1167" s="17" t="n">
+        <v>67999.43912830552</v>
+      </c>
+      <c r="M1167" s="17">
+        <f>J1167-L1167</f>
+        <v/>
+      </c>
+      <c r="N1167" s="18">
+        <f>IF(J1167=0,"",L1167/J1167)</f>
+        <v/>
+      </c>
+      <c r="O1167" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1168">
+      <c r="A1168" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:17:27</t>
+        </is>
+      </c>
+      <c r="B1168" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1168" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1168" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1168" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1168" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1168" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H1168" s="16" t="n">
+        <v>1.1283</v>
+      </c>
+      <c r="I1168" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J1168" s="17" t="n">
+        <v>197054.0613466415</v>
+      </c>
+      <c r="K1168" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,269.6194</t>
+        </is>
+      </c>
+      <c r="L1168" s="17" t="n">
+        <v>150314.7138033868</v>
+      </c>
+      <c r="M1168" s="17">
+        <f>J1168-L1168</f>
+        <v/>
+      </c>
+      <c r="N1168" s="18">
+        <f>IF(J1168=0,"",L1168/J1168)</f>
+        <v/>
+      </c>
+      <c r="O1168" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1169">
+      <c r="A1169" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:17:27</t>
+        </is>
+      </c>
+      <c r="B1169" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1169" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1169" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1169" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1169" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1169" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H1169" s="16" t="n">
+        <v>1.3723</v>
+      </c>
+      <c r="I1169" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J1169" s="17" t="n">
+        <v>186155.9890095307</v>
+      </c>
+      <c r="K1169" s="15" t="inlineStr">
+        <is>
+          <t>USDC 124,167.8308</t>
+        </is>
+      </c>
+      <c r="L1169" s="17" t="n">
+        <v>124205.0923587409</v>
+      </c>
+      <c r="M1169" s="17">
+        <f>J1169-L1169</f>
+        <v/>
+      </c>
+      <c r="N1169" s="18">
+        <f>IF(J1169=0,"",L1169/J1169)</f>
+        <v/>
+      </c>
+      <c r="O1169" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1170">
+      <c r="A1170" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:17:27</t>
+        </is>
+      </c>
+      <c r="B1170" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1170" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1170" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1170" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1170" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1170" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H1170" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I1170" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J1170" s="17" t="n">
+        <v>327707.3479550913</v>
+      </c>
+      <c r="K1170" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,371.4621</t>
+        </is>
+      </c>
+      <c r="L1170" s="17" t="n">
+        <v>280234.5207703282</v>
+      </c>
+      <c r="M1170" s="17">
+        <f>J1170-L1170</f>
+        <v/>
+      </c>
+      <c r="N1170" s="18">
+        <f>IF(J1170=0,"",L1170/J1170)</f>
+        <v/>
+      </c>
+      <c r="O1170" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1171">
+      <c r="A1171" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:17:27</t>
+        </is>
+      </c>
+      <c r="B1171" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1171" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1171" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1171" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1171" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1171" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H1171" s="16" t="n">
+        <v>1.9046</v>
+      </c>
+      <c r="I1171" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J1171" s="17" t="n">
+        <v>160084.5597839135</v>
+      </c>
+      <c r="K1171" s="15" t="inlineStr">
+        <is>
+          <t>USDC 70,956.9330</t>
+        </is>
+      </c>
+      <c r="L1171" s="17" t="n">
+        <v>70978.22651387689</v>
+      </c>
+      <c r="M1171" s="17">
+        <f>J1171-L1171</f>
+        <v/>
+      </c>
+      <c r="N1171" s="18">
+        <f>IF(J1171=0,"",L1171/J1171)</f>
+        <v/>
+      </c>
+      <c r="O1171" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1172">
+      <c r="A1172" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:17:27</t>
+        </is>
+      </c>
+      <c r="B1172" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1172" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1172" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1172" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1172" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1172" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H1172" s="16" t="n">
+        <v>1.0572</v>
+      </c>
+      <c r="I1172" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J1172" s="17" t="n">
+        <v>160173.5942004735</v>
+      </c>
+      <c r="K1172" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,534.8152</t>
+        </is>
+      </c>
+      <c r="L1172" s="17" t="n">
+        <v>138520.9617116763</v>
+      </c>
+      <c r="M1172" s="17">
+        <f>J1172-L1172</f>
+        <v/>
+      </c>
+      <c r="N1172" s="18">
+        <f>IF(J1172=0,"",L1172/J1172)</f>
+        <v/>
+      </c>
+      <c r="O1172" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1173">
+      <c r="A1173" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:17:27</t>
+        </is>
+      </c>
+      <c r="B1173" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1173" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1173" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E1173" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1173" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G1173" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1173" s="16" t="inlineStr"/>
+      <c r="I1173" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J1173" s="17" t="n">
+        <v>95948.79643108658</v>
+      </c>
+      <c r="K1173" s="15" t="inlineStr"/>
+      <c r="L1173" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1173" s="17">
+        <f>J1173-L1173</f>
+        <v/>
+      </c>
+      <c r="N1173" s="18">
+        <f>IF(J1173=0,"",L1173/J1173)</f>
+        <v/>
+      </c>
+      <c r="O1173" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1174">
+      <c r="A1174" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:17:27</t>
+        </is>
+      </c>
+      <c r="B1174" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1174" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1174" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E1174" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1174" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G1174" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1174" s="16" t="inlineStr"/>
+      <c r="I1174" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J1174" s="17" t="n">
+        <v>34358.38427400024</v>
+      </c>
+      <c r="K1174" s="15" t="inlineStr"/>
+      <c r="L1174" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1174" s="17">
+        <f>J1174-L1174</f>
+        <v/>
+      </c>
+      <c r="N1174" s="18">
+        <f>IF(J1174=0,"",L1174/J1174)</f>
+        <v/>
+      </c>
+      <c r="O1174" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1175">
+      <c r="A1175" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:17:27</t>
+        </is>
+      </c>
+      <c r="B1175" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1175" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D1175" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E1175" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1175" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G1175" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H1175" s="16" t="n">
+        <v>1.0433</v>
+      </c>
+      <c r="I1175" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J1175" s="17" t="n">
+        <v>270055.1862549248</v>
+      </c>
+      <c r="K1175" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,082.9379</t>
+        </is>
+      </c>
+      <c r="L1175" s="17" t="n">
+        <v>232954.7422691632</v>
+      </c>
+      <c r="M1175" s="17">
+        <f>J1175-L1175</f>
+        <v/>
+      </c>
+      <c r="N1175" s="18">
+        <f>IF(J1175=0,"",L1175/J1175)</f>
+        <v/>
+      </c>
+      <c r="O1175" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1176">
+      <c r="A1176" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:17:27</t>
+        </is>
+      </c>
+      <c r="B1176" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1176" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D1176" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E1176" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1176" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G1176" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1176" s="16" t="inlineStr"/>
+      <c r="I1176" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,521.1222</t>
+        </is>
+      </c>
+      <c r="J1176" s="17" t="n">
+        <v>15512.58563024298</v>
+      </c>
+      <c r="K1176" s="15" t="inlineStr"/>
+      <c r="L1176" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1176" s="17">
+        <f>J1176-L1176</f>
+        <v/>
+      </c>
+      <c r="N1176" s="18">
+        <f>IF(J1176=0,"",L1176/J1176)</f>
+        <v/>
+      </c>
+      <c r="O1176" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1177">
+      <c r="A1177" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:17:27</t>
+        </is>
+      </c>
+      <c r="B1177" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1177" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D1177" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E1177" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1177" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G1177" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H1177" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I1177" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J1177" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K1177" s="15" t="inlineStr">
+        <is>
+          <t>USDC 252,020.5254</t>
+        </is>
+      </c>
+      <c r="L1177" s="17" t="n">
+        <v>252020.525427</v>
+      </c>
+      <c r="M1177" s="17">
+        <f>J1177-L1177</f>
+        <v/>
+      </c>
+      <c r="N1177" s="18">
+        <f>IF(J1177=0,"",L1177/J1177)</f>
+        <v/>
+      </c>
+      <c r="O1177" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1178">
+      <c r="A1178" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:17:27</t>
+        </is>
+      </c>
+      <c r="B1178" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1178" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D1178" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E1178" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1178" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G1178" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H1178" s="16" t="n">
+        <v>1.219</v>
+      </c>
+      <c r="I1178" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J1178" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K1178" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,736.3177</t>
+        </is>
+      </c>
+      <c r="L1178" s="17" t="n">
+        <v>148736.317674</v>
+      </c>
+      <c r="M1178" s="17">
+        <f>J1178-L1178</f>
+        <v/>
+      </c>
+      <c r="N1178" s="18">
+        <f>IF(J1178=0,"",L1178/J1178)</f>
+        <v/>
+      </c>
+      <c r="O1178" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -78934,7 +80020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I76"/>
+  <dimension ref="A1:I77"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -81610,6 +82696,41 @@
         <v>1.0374</v>
       </c>
       <c r="I76" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:17:27</t>
+        </is>
+      </c>
+      <c r="B77" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C77" s="17" t="n">
+        <v>655468.2749733245</v>
+      </c>
+      <c r="D77" s="17" t="n">
+        <v>652879.844875528</v>
+      </c>
+      <c r="E77" s="17" t="n">
+        <v>2933885.259445846</v>
+      </c>
+      <c r="F77" s="17" t="n">
+        <v>2281005.414570318</v>
+      </c>
+      <c r="G77" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H77" s="16" t="n">
+        <v>1.0374</v>
+      </c>
+      <c r="I77" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
fresh start: wipe all history, new Day 0 at 2026-04-30 14:32 UTC
Portfolio reset after withdrawal. Net $630,303.
All prior snapshots erased. Day 0 = right now.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O1178"/>
+  <dimension ref="A1:O1194"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -79990,6 +79990,1092 @@
         <v/>
       </c>
       <c r="O1178" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1179">
+      <c r="A1179" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:32:33</t>
+        </is>
+      </c>
+      <c r="B1179" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1179" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1179" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E1179" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1179" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G1179" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H1179" s="16" t="n">
+        <v>1.0503</v>
+      </c>
+      <c r="I1179" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,811.7228</t>
+        </is>
+      </c>
+      <c r="J1179" s="17" t="n">
+        <v>50805.1173260295</v>
+      </c>
+      <c r="K1179" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,728.4282</t>
+        </is>
+      </c>
+      <c r="L1179" s="17" t="n">
+        <v>37735.97541408282</v>
+      </c>
+      <c r="M1179" s="17">
+        <f>J1179-L1179</f>
+        <v/>
+      </c>
+      <c r="N1179" s="18">
+        <f>IF(J1179=0,"",L1179/J1179)</f>
+        <v/>
+      </c>
+      <c r="O1179" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1180">
+      <c r="A1180" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:32:33</t>
+        </is>
+      </c>
+      <c r="B1180" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1180" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1180" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E1180" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1180" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G1180" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H1180" s="16" t="n">
+        <v>1.0481</v>
+      </c>
+      <c r="I1180" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J1180" s="17" t="n">
+        <v>140952.8186242044</v>
+      </c>
+      <c r="K1180" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,054.2331</t>
+        </is>
+      </c>
+      <c r="L1180" s="17" t="n">
+        <v>121038.4960546964</v>
+      </c>
+      <c r="M1180" s="17">
+        <f>J1180-L1180</f>
+        <v/>
+      </c>
+      <c r="N1180" s="18">
+        <f>IF(J1180=0,"",L1180/J1180)</f>
+        <v/>
+      </c>
+      <c r="O1180" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1181">
+      <c r="A1181" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:32:33</t>
+        </is>
+      </c>
+      <c r="B1181" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1181" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1181" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E1181" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1181" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G1181" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H1181" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I1181" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J1181" s="17" t="n">
+        <v>328750.577340672</v>
+      </c>
+      <c r="K1181" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,407.5961</t>
+        </is>
+      </c>
+      <c r="L1181" s="17" t="n">
+        <v>306499.9359030026</v>
+      </c>
+      <c r="M1181" s="17">
+        <f>J1181-L1181</f>
+        <v/>
+      </c>
+      <c r="N1181" s="18">
+        <f>IF(J1181=0,"",L1181/J1181)</f>
+        <v/>
+      </c>
+      <c r="O1181" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1182">
+      <c r="A1182" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:32:33</t>
+        </is>
+      </c>
+      <c r="B1182" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1182" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1182" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E1182" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1182" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G1182" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H1182" s="16" t="n">
+        <v>1.0374</v>
+      </c>
+      <c r="I1182" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J1182" s="17" t="n">
+        <v>386078.6724737359</v>
+      </c>
+      <c r="K1182" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,641.2671</t>
+        </is>
+      </c>
+      <c r="L1182" s="17" t="n">
+        <v>349746.6359360348</v>
+      </c>
+      <c r="M1182" s="17">
+        <f>J1182-L1182</f>
+        <v/>
+      </c>
+      <c r="N1182" s="18">
+        <f>IF(J1182=0,"",L1182/J1182)</f>
+        <v/>
+      </c>
+      <c r="O1182" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1183">
+      <c r="A1183" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:32:33</t>
+        </is>
+      </c>
+      <c r="B1183" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1183" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D1183" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E1183" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1183" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G1183" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H1183" s="16" t="n">
+        <v>1.0541</v>
+      </c>
+      <c r="I1183" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7884</t>
+        </is>
+      </c>
+      <c r="J1183" s="17" t="n">
+        <v>77786.58801901045</v>
+      </c>
+      <c r="K1183" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,037.0654; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L1183" s="17" t="n">
+        <v>68014.01040227356</v>
+      </c>
+      <c r="M1183" s="17">
+        <f>J1183-L1183</f>
+        <v/>
+      </c>
+      <c r="N1183" s="18">
+        <f>IF(J1183=0,"",L1183/J1183)</f>
+        <v/>
+      </c>
+      <c r="O1183" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1184">
+      <c r="A1184" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:32:33</t>
+        </is>
+      </c>
+      <c r="B1184" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1184" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1184" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1184" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1184" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1184" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H1184" s="16" t="n">
+        <v>1.1283</v>
+      </c>
+      <c r="I1184" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J1184" s="17" t="n">
+        <v>197054.6637224008</v>
+      </c>
+      <c r="K1184" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,269.6194</t>
+        </is>
+      </c>
+      <c r="L1184" s="17" t="n">
+        <v>150299.6793251109</v>
+      </c>
+      <c r="M1184" s="17">
+        <f>J1184-L1184</f>
+        <v/>
+      </c>
+      <c r="N1184" s="18">
+        <f>IF(J1184=0,"",L1184/J1184)</f>
+        <v/>
+      </c>
+      <c r="O1184" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1185">
+      <c r="A1185" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:32:33</t>
+        </is>
+      </c>
+      <c r="B1185" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1185" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1185" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1185" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1185" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1185" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H1185" s="16" t="n">
+        <v>1.3192</v>
+      </c>
+      <c r="I1185" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J1185" s="17" t="n">
+        <v>186156.3043586716</v>
+      </c>
+      <c r="K1185" s="15" t="inlineStr">
+        <is>
+          <t>USDC 129,169.6456</t>
+        </is>
+      </c>
+      <c r="L1185" s="17" t="n">
+        <v>129195.4846991646</v>
+      </c>
+      <c r="M1185" s="17">
+        <f>J1185-L1185</f>
+        <v/>
+      </c>
+      <c r="N1185" s="18">
+        <f>IF(J1185=0,"",L1185/J1185)</f>
+        <v/>
+      </c>
+      <c r="O1185" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1186">
+      <c r="A1186" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:32:33</t>
+        </is>
+      </c>
+      <c r="B1186" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1186" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1186" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1186" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1186" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1186" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H1186" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I1186" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J1186" s="17" t="n">
+        <v>327710.9501445745</v>
+      </c>
+      <c r="K1186" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,371.4621</t>
+        </is>
+      </c>
+      <c r="L1186" s="17" t="n">
+        <v>280231.4404390584</v>
+      </c>
+      <c r="M1186" s="17">
+        <f>J1186-L1186</f>
+        <v/>
+      </c>
+      <c r="N1186" s="18">
+        <f>IF(J1186=0,"",L1186/J1186)</f>
+        <v/>
+      </c>
+      <c r="O1186" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1187">
+      <c r="A1187" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:32:33</t>
+        </is>
+      </c>
+      <c r="B1187" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1187" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1187" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1187" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1187" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1187" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H1187" s="16" t="n">
+        <v>1.5278</v>
+      </c>
+      <c r="I1187" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J1187" s="17" t="n">
+        <v>160084.5597839135</v>
+      </c>
+      <c r="K1187" s="15" t="inlineStr">
+        <is>
+          <t>USDC 88,458.0563</t>
+        </is>
+      </c>
+      <c r="L1187" s="17" t="n">
+        <v>88475.75145522061</v>
+      </c>
+      <c r="M1187" s="17">
+        <f>J1187-L1187</f>
+        <v/>
+      </c>
+      <c r="N1187" s="18">
+        <f>IF(J1187=0,"",L1187/J1187)</f>
+        <v/>
+      </c>
+      <c r="O1187" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1188">
+      <c r="A1188" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:32:33</t>
+        </is>
+      </c>
+      <c r="B1188" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1188" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1188" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1188" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1188" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1188" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs PYUSD</t>
+        </is>
+      </c>
+      <c r="H1188" s="16" t="n">
+        <v>1.0572</v>
+      </c>
+      <c r="I1188" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 130,322.3174</t>
+        </is>
+      </c>
+      <c r="J1188" s="17" t="n">
+        <v>160173.5942004735</v>
+      </c>
+      <c r="K1188" s="15" t="inlineStr">
+        <is>
+          <t>PYUSD 138,536.8617</t>
+        </is>
+      </c>
+      <c r="L1188" s="17" t="n">
+        <v>138536.8617382167</v>
+      </c>
+      <c r="M1188" s="17">
+        <f>J1188-L1188</f>
+        <v/>
+      </c>
+      <c r="N1188" s="18">
+        <f>IF(J1188=0,"",L1188/J1188)</f>
+        <v/>
+      </c>
+      <c r="O1188" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1189">
+      <c r="A1189" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:32:33</t>
+        </is>
+      </c>
+      <c r="B1189" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1189" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1189" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl</t>
+        </is>
+      </c>
+      <c r="E1189" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1189" s="15" t="inlineStr">
+        <is>
+          <t>Neutrl-eth-0x08efcc2f</t>
+        </is>
+      </c>
+      <c r="G1189" s="15" t="inlineStr">
+        <is>
+          <t>NUSD vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1189" s="16" t="inlineStr"/>
+      <c r="I1189" s="15" t="inlineStr">
+        <is>
+          <t>NUSD 95,933.3700</t>
+        </is>
+      </c>
+      <c r="J1189" s="17" t="n">
+        <v>95845.62458251606</v>
+      </c>
+      <c r="K1189" s="15" t="inlineStr"/>
+      <c r="L1189" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1189" s="17">
+        <f>J1189-L1189</f>
+        <v/>
+      </c>
+      <c r="N1189" s="18">
+        <f>IF(J1189=0,"",L1189/J1189)</f>
+        <v/>
+      </c>
+      <c r="O1189" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1190">
+      <c r="A1190" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:32:33</t>
+        </is>
+      </c>
+      <c r="B1190" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1190" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1190" s="15" t="inlineStr">
+        <is>
+          <t>Pendle V2</t>
+        </is>
+      </c>
+      <c r="E1190" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1190" s="15" t="inlineStr">
+        <is>
+          <t>PendleV2-eth-0xdc9a5a2e</t>
+        </is>
+      </c>
+      <c r="G1190" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1190" s="16" t="inlineStr"/>
+      <c r="I1190" s="15" t="inlineStr">
+        <is>
+          <t>PT-reUSDe-25JUN2026 35,130.2709</t>
+        </is>
+      </c>
+      <c r="J1190" s="17" t="n">
+        <v>34358.48512055133</v>
+      </c>
+      <c r="K1190" s="15" t="inlineStr"/>
+      <c r="L1190" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1190" s="17">
+        <f>J1190-L1190</f>
+        <v/>
+      </c>
+      <c r="N1190" s="18">
+        <f>IF(J1190=0,"",L1190/J1190)</f>
+        <v/>
+      </c>
+      <c r="O1190" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1191">
+      <c r="A1191" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:32:33</t>
+        </is>
+      </c>
+      <c r="B1191" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1191" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D1191" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E1191" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1191" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-plasma-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G1191" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai vs USDT0</t>
+        </is>
+      </c>
+      <c r="H1191" s="16" t="n">
+        <v>1.0432</v>
+      </c>
+      <c r="I1191" s="15" t="inlineStr">
+        <is>
+          <t>sUSDai 249,570.0181</t>
+        </is>
+      </c>
+      <c r="J1191" s="17" t="n">
+        <v>270082.1998776371</v>
+      </c>
+      <c r="K1191" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 233,084.3779</t>
+        </is>
+      </c>
+      <c r="L1191" s="17" t="n">
+        <v>233005.1291635303</v>
+      </c>
+      <c r="M1191" s="17">
+        <f>J1191-L1191</f>
+        <v/>
+      </c>
+      <c r="N1191" s="18">
+        <f>IF(J1191=0,"",L1191/J1191)</f>
+        <v/>
+      </c>
+      <c r="O1191" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1192">
+      <c r="A1192" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:32:33</t>
+        </is>
+      </c>
+      <c r="B1192" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1192" s="15" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="D1192" s="15" t="inlineStr">
+        <is>
+          <t>Yuzu Money</t>
+        </is>
+      </c>
+      <c r="E1192" s="15" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="F1192" s="15" t="inlineStr">
+        <is>
+          <t>YuzuMoney-plasma-0xebfc8c2f</t>
+        </is>
+      </c>
+      <c r="G1192" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 vs (no debt)</t>
+        </is>
+      </c>
+      <c r="H1192" s="16" t="inlineStr"/>
+      <c r="I1192" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 15,521.3247</t>
+        </is>
+      </c>
+      <c r="J1192" s="17" t="n">
+        <v>15516.04747591695</v>
+      </c>
+      <c r="K1192" s="15" t="inlineStr"/>
+      <c r="L1192" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1192" s="17">
+        <f>J1192-L1192</f>
+        <v/>
+      </c>
+      <c r="N1192" s="18">
+        <f>IF(J1192=0,"",L1192/J1192)</f>
+        <v/>
+      </c>
+      <c r="O1192" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1193">
+      <c r="A1193" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:32:33</t>
+        </is>
+      </c>
+      <c r="B1193" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1193" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D1193" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E1193" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1193" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-Ea8BXKie</t>
+        </is>
+      </c>
+      <c r="G1193" s="15" t="inlineStr">
+        <is>
+          <t>PRIME vs USDC</t>
+        </is>
+      </c>
+      <c r="H1193" s="16" t="n">
+        <v>1.087</v>
+      </c>
+      <c r="I1193" s="15" t="inlineStr">
+        <is>
+          <t>PRIME 291,233.7623</t>
+        </is>
+      </c>
+      <c r="J1193" s="17" t="n">
+        <v>300982.3200284909</v>
+      </c>
+      <c r="K1193" s="15" t="inlineStr">
+        <is>
+          <t>USDC 252,020.5254</t>
+        </is>
+      </c>
+      <c r="L1193" s="17" t="n">
+        <v>252020.525427</v>
+      </c>
+      <c r="M1193" s="17">
+        <f>J1193-L1193</f>
+        <v/>
+      </c>
+      <c r="N1193" s="18">
+        <f>IF(J1193=0,"",L1193/J1193)</f>
+        <v/>
+      </c>
+      <c r="O1193" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1194">
+      <c r="A1194" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:32:33</t>
+        </is>
+      </c>
+      <c r="B1194" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1194" s="15" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="D1194" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale</t>
+        </is>
+      </c>
+      <c r="E1194" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1194" s="15" t="inlineStr">
+        <is>
+          <t>Loopscale-sol-6zpxNbPj</t>
+        </is>
+      </c>
+      <c r="G1194" s="15" t="inlineStr">
+        <is>
+          <t>ONYC vs USDC</t>
+        </is>
+      </c>
+      <c r="H1194" s="16" t="n">
+        <v>1.219</v>
+      </c>
+      <c r="I1194" s="15" t="inlineStr">
+        <is>
+          <t>ONYC 183,630.0450</t>
+        </is>
+      </c>
+      <c r="J1194" s="17" t="n">
+        <v>201501.0605624586</v>
+      </c>
+      <c r="K1194" s="15" t="inlineStr">
+        <is>
+          <t>USDC 148,736.3177</t>
+        </is>
+      </c>
+      <c r="L1194" s="17" t="n">
+        <v>148736.317674</v>
+      </c>
+      <c r="M1194" s="17">
+        <f>J1194-L1194</f>
+        <v/>
+      </c>
+      <c r="N1194" s="18">
+        <f>IF(J1194=0,"",L1194/J1194)</f>
+        <v/>
+      </c>
+      <c r="O1194" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>
@@ -80020,7 +81106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I77"/>
+  <dimension ref="A1:I78"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -82731,6 +83817,41 @@
         <v>1.0374</v>
       </c>
       <c r="I77" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:32:33</t>
+        </is>
+      </c>
+      <c r="B78" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C78" s="17" t="n">
+        <v>630376.3852701036</v>
+      </c>
+      <c r="D78" s="17" t="n">
+        <v>630303.3400098654</v>
+      </c>
+      <c r="E78" s="17" t="n">
+        <v>2933839.583641257</v>
+      </c>
+      <c r="F78" s="17" t="n">
+        <v>2303536.243631392</v>
+      </c>
+      <c r="G78" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H78" s="16" t="n">
+        <v>1.0374</v>
+      </c>
+      <c r="I78" s="15" t="inlineStr">
         <is>
           <t>Rabby API + Jupiter</t>
         </is>

</xml_diff>

<commit_message>
feat: Tulip Fund redesign — hero with SVG logo, Day 0 stats card, annualized return
- Rename dashboard to "Tulip Fund" with tulip SVG logo (purple petals, green stem)
- Add Day 0 stats card: date, starting capital, P&L + %, annualized return
- Filter out no-data benchmark pills; show helpful "after first week" message
- Add CSS for .fund-brand, .tulip-logo, .day0-card, .day0-row, .ann-return
- Fix P&L sign consistency when pct rounds to 0.00%
- GitHub Actions cron already at every 6h (0 */6 * * *)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/debank_positions_log.xlsx
+++ b/outputs/debank_positions_log.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O1194"/>
+  <dimension ref="A1:O1242"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="8" min="1" max="1"/>
@@ -81076,6 +81076,3264 @@
         <v/>
       </c>
       <c r="O1194" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1195">
+      <c r="A1195" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:37:52</t>
+        </is>
+      </c>
+      <c r="B1195" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1195" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1195" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E1195" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1195" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-eth-0x87870bca</t>
+        </is>
+      </c>
+      <c r="G1195" s="15" t="inlineStr">
+        <is>
+          <t>USDT vs USDC</t>
+        </is>
+      </c>
+      <c r="H1195" s="16" t="n">
+        <v>1.0503</v>
+      </c>
+      <c r="I1195" s="15" t="inlineStr">
+        <is>
+          <t>USDT 50,811.7228</t>
+        </is>
+      </c>
+      <c r="J1195" s="17" t="n">
+        <v>50795.9712159165</v>
+      </c>
+      <c r="K1195" s="15" t="inlineStr">
+        <is>
+          <t>USDC 37,728.4282</t>
+        </is>
+      </c>
+      <c r="L1195" s="17" t="n">
+        <v>37735.97541408282</v>
+      </c>
+      <c r="M1195" s="17">
+        <f>J1195-L1195</f>
+        <v/>
+      </c>
+      <c r="N1195" s="18">
+        <f>IF(J1195=0,"",L1195/J1195)</f>
+        <v/>
+      </c>
+      <c r="O1195" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1196">
+      <c r="A1196" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:37:52</t>
+        </is>
+      </c>
+      <c r="B1196" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1196" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1196" s="15" t="inlineStr">
+        <is>
+          <t>Fluid</t>
+        </is>
+      </c>
+      <c r="E1196" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1196" s="15" t="inlineStr">
+        <is>
+          <t>Fluid-eth-0x324c5dc1</t>
+        </is>
+      </c>
+      <c r="G1196" s="15" t="inlineStr">
+        <is>
+          <t>reUSD vs USDT</t>
+        </is>
+      </c>
+      <c r="H1196" s="16" t="n">
+        <v>1.0483</v>
+      </c>
+      <c r="I1196" s="15" t="inlineStr">
+        <is>
+          <t>reUSD 131,159.6529</t>
+        </is>
+      </c>
+      <c r="J1196" s="17" t="n">
+        <v>140952.8186242044</v>
+      </c>
+      <c r="K1196" s="15" t="inlineStr">
+        <is>
+          <t>USDT 121,054.2331</t>
+        </is>
+      </c>
+      <c r="L1196" s="17" t="n">
+        <v>121016.7062927374</v>
+      </c>
+      <c r="M1196" s="17">
+        <f>J1196-L1196</f>
+        <v/>
+      </c>
+      <c r="N1196" s="18">
+        <f>IF(J1196=0,"",L1196/J1196)</f>
+        <v/>
+      </c>
+      <c r="O1196" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1197">
+      <c r="A1197" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:37:52</t>
+        </is>
+      </c>
+      <c r="B1197" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1197" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1197" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E1197" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1197" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0x3de37c38</t>
+        </is>
+      </c>
+      <c r="G1197" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H1197" s="16" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="I1197" s="15" t="inlineStr">
+        <is>
+          <t>sfrxUSD 275,773.4355</t>
+        </is>
+      </c>
+      <c r="J1197" s="17" t="n">
+        <v>328750.577340672</v>
+      </c>
+      <c r="K1197" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 306,407.5961</t>
+        </is>
+      </c>
+      <c r="L1197" s="17" t="n">
+        <v>306499.9359030026</v>
+      </c>
+      <c r="M1197" s="17">
+        <f>J1197-L1197</f>
+        <v/>
+      </c>
+      <c r="N1197" s="18">
+        <f>IF(J1197=0,"",L1197/J1197)</f>
+        <v/>
+      </c>
+      <c r="O1197" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1198">
+      <c r="A1198" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:37:52</t>
+        </is>
+      </c>
+      <c r="B1198" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1198" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1198" s="15" t="inlineStr">
+        <is>
+          <t>Curve LlamaLend</t>
+        </is>
+      </c>
+      <c r="E1198" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1198" s="15" t="inlineStr">
+        <is>
+          <t>CurveLlamaLend-eth-0xb536fea3</t>
+        </is>
+      </c>
+      <c r="G1198" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe vs crvUSD</t>
+        </is>
+      </c>
+      <c r="H1198" s="16" t="n">
+        <v>1.0374</v>
+      </c>
+      <c r="I1198" s="15" t="inlineStr">
+        <is>
+          <t>sUSDe 314,125.8554</t>
+        </is>
+      </c>
+      <c r="J1198" s="17" t="n">
+        <v>386079.4533224807</v>
+      </c>
+      <c r="K1198" s="15" t="inlineStr">
+        <is>
+          <t>crvUSD 349,641.2671</t>
+        </is>
+      </c>
+      <c r="L1198" s="17" t="n">
+        <v>349746.6359360348</v>
+      </c>
+      <c r="M1198" s="17">
+        <f>J1198-L1198</f>
+        <v/>
+      </c>
+      <c r="N1198" s="18">
+        <f>IF(J1198=0,"",L1198/J1198)</f>
+        <v/>
+      </c>
+      <c r="O1198" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1199">
+      <c r="A1199" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:37:52</t>
+        </is>
+      </c>
+      <c r="B1199" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1199" s="15" t="inlineStr">
+        <is>
+          <t>Mantle</t>
+        </is>
+      </c>
+      <c r="D1199" s="15" t="inlineStr">
+        <is>
+          <t>Aave V3</t>
+        </is>
+      </c>
+      <c r="E1199" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1199" s="15" t="inlineStr">
+        <is>
+          <t>AaveV3-mnt-0x458f2934</t>
+        </is>
+      </c>
+      <c r="G1199" s="15" t="inlineStr">
+        <is>
+          <t>WMNT+syrupUSDT+GHO vs USDT0+USDC</t>
+        </is>
+      </c>
+      <c r="H1199" s="16" t="n">
+        <v>1.0541</v>
+      </c>
+      <c r="I1199" s="15" t="inlineStr">
+        <is>
+          <t>WMNT 39.8951; syrupUSDT 69,284.0832; GHO 36.7884</t>
+        </is>
+      </c>
+      <c r="J1199" s="17" t="n">
+        <v>77791.21757317503</v>
+      </c>
+      <c r="K1199" s="15" t="inlineStr">
+        <is>
+          <t>USDT0 68,037.0654; USDC 0.0776</t>
+        </is>
+      </c>
+      <c r="L1199" s="17" t="n">
+        <v>67999.72261853515</v>
+      </c>
+      <c r="M1199" s="17">
+        <f>J1199-L1199</f>
+        <v/>
+      </c>
+      <c r="N1199" s="18">
+        <f>IF(J1199=0,"",L1199/J1199)</f>
+        <v/>
+      </c>
+      <c r="O1199" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1200">
+      <c r="A1200" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:37:52</t>
+        </is>
+      </c>
+      <c r="B1200" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1200" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1200" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1200" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1200" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1200" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H1200" s="16" t="n">
+        <v>1.1283</v>
+      </c>
+      <c r="I1200" s="15" t="inlineStr">
+        <is>
+          <t>PT-apyUSD-18JUN2026 201,006.0180</t>
+        </is>
+      </c>
+      <c r="J1200" s="17" t="n">
+        <v>197054.6637224008</v>
+      </c>
+      <c r="K1200" s="15" t="inlineStr">
+        <is>
+          <t>USDC 150,269.6194</t>
+        </is>
+      </c>
+      <c r="L1200" s="17" t="n">
+        <v>150299.6793251109</v>
+      </c>
+      <c r="M1200" s="17">
+        <f>J1200-L1200</f>
+        <v/>
+      </c>
+      <c r="N1200" s="18">
+        <f>IF(J1200=0,"",L1200/J1200)</f>
+        <v/>
+      </c>
+      <c r="O1200" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1201">
+      <c r="A1201" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:37:52</t>
+        </is>
+      </c>
+      <c r="B1201" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1201" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1201" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1201" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1201" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1201" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 vs USDC</t>
+        </is>
+      </c>
+      <c r="H1201" s="16" t="n">
+        <v>1.3192</v>
+      </c>
+      <c r="I1201" s="15" t="inlineStr">
+        <is>
+          <t>PT-srNUSD-28MAY2026 187,379.2379</t>
+        </is>
+      </c>
+      <c r="J1201" s="17" t="n">
+        <v>186156.3043586716</v>
+      </c>
+      <c r="K1201" s="15" t="inlineStr">
+        <is>
+          <t>USDC 129,169.6456</t>
+        </is>
+      </c>
+      <c r="L1201" s="17" t="n">
+        <v>129195.4846991646</v>
+      </c>
+      <c r="M1201" s="17">
+        <f>J1201-L1201</f>
+        <v/>
+      </c>
+      <c r="N1201" s="18">
+        <f>IF(J1201=0,"",L1201/J1201)</f>
+        <v/>
+      </c>
+      <c r="O1201" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1202">
+      <c r="A1202" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:37:52</t>
+        </is>
+      </c>
+      <c r="B1202" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1202" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1202" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1202" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1202" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1202" s="15" t="inlineStr">
+        <is>
+          <t>siUSD vs msUSD</t>
+        </is>
+      </c>
+      <c r="H1202" s="16" t="n">
+        <v>1.0654</v>
+      </c>
+      <c r="I1202" s="15" t="inlineStr">
+        <is>
+          <t>siUSD 307,229.9415</t>
+        </is>
+      </c>
+      <c r="J1202" s="17" t="n">
+        <v>327710.9501445745</v>
+      </c>
+      <c r="K1202" s="15" t="inlineStr">
+        <is>
+          <t>msUSD 281,371.4621</t>
+        </is>
+      </c>
+      <c r="L1202" s="17" t="n">
+        <v>280292.5373219175</v>
+      </c>
+      <c r="M1202" s="17">
+        <f>J1202-L1202</f>
+        <v/>
+      </c>
+      <c r="N1202" s="18">
+        <f>IF(J1202=0,"",L1202/J1202)</f>
+        <v/>
+      </c>
+      <c r="O1202" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1203">
+      <c r="A1203" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:37:52</t>
+        </is>
+      </c>
+      <c r="B1203" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1203" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1203" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+      <c r="E1203" s="15" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="F1203" s="15" t="inlineStr">
+        <is>
+          <t>Morpho-eth-0xbbbbbbbb</t>
+        </is>
+      </c>
+      <c r="G1203" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE vs USDC</t>
+        </is>
+      </c>
+      <c r="H1203" s="16" t="n">
+        <v>1.5278</v>
+      </c>
+      <c r="I1203" s="15" t="inlineStr">
+        <is>
+          <t>mF-ONE 148,000.0000</t>
+        </is>
+      </c>
+      <c r="J1203" s="17" t="n">
+        <v>160084.5597839135</v>
+      </c>
+      <c r="K1203" s="15" t="inlineStr">
+        <is>
+          <t>USDC 88,458.0563</t>
+        </is>
+      </c>
+      <c r="L1203" s="17" t="n">
+        <v>88475.75145522061</v>
+      </c>
+      <c r="M1203" s="17">
+        <f>J1203-L1203</f>
+        <v/>
+      </c>
+      <c r="N1203" s="18">
+        <f>IF(J1203=0,"",L1203/J1203)</f>
+        <v/>
+      </c>
+      <c r="O1203" s="15" t="inlineStr">
+        <is>
+          <t>Rabby API + Jupiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1204">
+      <c r="A1204" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30 14:37:52</t>
+        </is>
+      </c>
+      <c r="B1204" s="15" t="inlineStr">
+        <is>
+          <t>0xe16be042f9433779909a972669be3a2003956348</t>
+        </is>
+      </c>
+      <c r="C1204" s="15" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="D1204" s="15" t="inlineStr">
+        <is>
+          <t>Morpho</t>
+        </is>
+      </c>
+  